<commit_message>
📊 Dados atualizados - 2026-06-01 06:04
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -833,7 +833,7 @@
         <v>1046280835</v>
       </c>
       <c r="I2" t="n">
-        <v>33000</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
         <v>152359482</v>
@@ -1770,7 +1770,7 @@
         <v>7.62</v>
       </c>
       <c r="H6" t="n">
-        <v>480705330</v>
+        <v>480705400</v>
       </c>
       <c r="I6" t="n">
         <v>400</v>
@@ -1788,7 +1788,7 @@
         <v>13.39</v>
       </c>
       <c r="N6" t="n">
-        <v>5.929744418362787</v>
+        <v>5.929745281848342</v>
       </c>
       <c r="O6" t="n">
         <v>1.24</v>
@@ -1866,7 +1866,7 @@
         <v>34696585</v>
       </c>
       <c r="AN6" t="n">
-        <v>51577825.10729614</v>
+        <v>51577832.61802575</v>
       </c>
       <c r="AO6" t="n">
         <v>0</v>
@@ -4358,7 +4358,7 @@
         <v>10735948032</v>
       </c>
       <c r="I17" t="n">
-        <v>1636500</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -6238,7 +6238,7 @@
         <v>1264703498</v>
       </c>
       <c r="I25" t="n">
-        <v>935100</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
         <v>346494097</v>
@@ -8804,7 +8804,7 @@
         <v>25.18</v>
       </c>
       <c r="H36" t="n">
-        <v>221626877</v>
+        <v>221627000</v>
       </c>
       <c r="I36" t="n">
         <v>300</v>
@@ -8822,7 +8822,7 @@
         <v>10.3</v>
       </c>
       <c r="N36" t="n">
-        <v>2.024579828765792</v>
+        <v>2.024580952380952</v>
       </c>
       <c r="O36" t="n">
         <v>0.85</v>
@@ -8900,7 +8900,7 @@
         <v>12348000</v>
       </c>
       <c r="AN36" t="n">
-        <v>39647026.29695886</v>
+        <v>39647048.30053668</v>
       </c>
       <c r="AO36" t="n">
         <v>0</v>
@@ -9039,7 +9039,7 @@
         <v>20.05</v>
       </c>
       <c r="H37" t="n">
-        <v>221626877</v>
+        <v>221627000</v>
       </c>
       <c r="I37" t="n">
         <v>500</v>
@@ -9057,7 +9057,7 @@
         <v>7.41</v>
       </c>
       <c r="N37" t="n">
-        <v>2.024579828765792</v>
+        <v>2.024580952380952</v>
       </c>
       <c r="O37" t="n">
         <v>0.61</v>
@@ -9135,7 +9135,7 @@
         <v>12348000</v>
       </c>
       <c r="AN37" t="n">
-        <v>55131063.93034826</v>
+        <v>55131094.52736319</v>
       </c>
       <c r="AO37" t="n">
         <v>0</v>
@@ -11859,7 +11859,7 @@
         <v>51.5</v>
       </c>
       <c r="H49" t="n">
-        <v>971368795</v>
+        <v>961354500</v>
       </c>
       <c r="I49" t="n">
         <v>6400</v>
@@ -11877,7 +11877,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="N49" t="n">
-        <v>1.060650217744008</v>
+        <v>1.049715478819949</v>
       </c>
       <c r="O49" t="n">
         <v>0.08</v>
@@ -11955,7 +11955,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN49" t="n">
-        <v>177581132.5411335</v>
+        <v>175750365.630713</v>
       </c>
       <c r="AO49" t="n">
         <v>2.4346</v>
@@ -12094,7 +12094,7 @@
         <v>31.8</v>
       </c>
       <c r="H50" t="n">
-        <v>971368795</v>
+        <v>961354500</v>
       </c>
       <c r="I50" t="n">
         <v>400</v>
@@ -12112,7 +12112,7 @@
         <v>5.78</v>
       </c>
       <c r="N50" t="n">
-        <v>1.060650217744008</v>
+        <v>1.049715478819949</v>
       </c>
       <c r="O50" t="n">
         <v>0.06</v>
@@ -12190,7 +12190,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN50" t="n">
-        <v>254952439.6325459</v>
+        <v>252324015.7480315</v>
       </c>
       <c r="AO50" t="n">
         <v>3.526</v>
@@ -14428,7 +14428,7 @@
         <v>371.99</v>
       </c>
       <c r="H60" t="n">
-        <v>169162448</v>
+        <v>169162400</v>
       </c>
       <c r="I60" t="n">
         <v>22</v>
@@ -14446,7 +14446,7 @@
         <v>2.87</v>
       </c>
       <c r="N60" t="n">
-        <v>11.95409020350892</v>
+        <v>11.95408681152484</v>
       </c>
       <c r="O60" t="n">
         <v>0.64</v>
@@ -14524,7 +14524,7 @@
         <v>59731412.5</v>
       </c>
       <c r="AN60" t="n">
-        <v>21305094.20654912</v>
+        <v>21305088.16120907</v>
       </c>
       <c r="AO60" t="n">
         <v>0</v>
@@ -17016,7 +17016,7 @@
         <v>1677831237</v>
       </c>
       <c r="I71" t="n">
-        <v>334200</v>
+        <v>0</v>
       </c>
       <c r="J71" t="n">
         <v>0</v>
@@ -19598,7 +19598,7 @@
         <v>9.970000000000001</v>
       </c>
       <c r="H82" t="n">
-        <v>418946000</v>
+        <v>421482500</v>
       </c>
       <c r="I82" t="n">
         <v>5400</v>
@@ -19616,7 +19616,7 @@
         <v>6.04</v>
       </c>
       <c r="N82" t="n">
-        <v>1.065324891165197</v>
+        <v>1.071774878959425</v>
       </c>
       <c r="O82" t="n">
         <v>1.01</v>
@@ -19694,7 +19694,7 @@
         <v>65949124.8</v>
       </c>
       <c r="AN82" t="n">
-        <v>74545551.60142349</v>
+        <v>74996886.12099645</v>
       </c>
       <c r="AO82" t="n">
         <v>0</v>
@@ -21948,7 +21948,7 @@
         <v>10</v>
       </c>
       <c r="H92" t="n">
-        <v>79882570</v>
+        <v>78978720</v>
       </c>
       <c r="I92" t="n">
         <v>0</v>
@@ -21966,7 +21966,7 @@
         <v>3.42</v>
       </c>
       <c r="N92" t="n">
-        <v>0.147499383147723</v>
+        <v>0.145830466919088</v>
       </c>
       <c r="O92" t="n">
         <v>0.15</v>
@@ -22044,7 +22044,7 @@
         <v>23342055.36</v>
       </c>
       <c r="AN92" t="n">
-        <v>56654304.96453901</v>
+        <v>56013276.59574468</v>
       </c>
       <c r="AO92" t="n">
         <v>0</v>
@@ -22183,7 +22183,7 @@
         <v>5.09</v>
       </c>
       <c r="H93" t="n">
-        <v>79882570</v>
+        <v>78978720</v>
       </c>
       <c r="I93" t="n">
         <v>16200</v>
@@ -22201,7 +22201,7 @@
         <v>2.3</v>
       </c>
       <c r="N93" t="n">
-        <v>0.1960900798807849</v>
+        <v>0.1938713728624674</v>
       </c>
       <c r="O93" t="n">
         <v>0.1</v>
@@ -22279,7 +22279,7 @@
         <v>17557944.64</v>
       </c>
       <c r="AN93" t="n">
-        <v>84086915.78947368</v>
+        <v>83135494.73684211</v>
       </c>
       <c r="AO93" t="n">
         <v>0</v>
@@ -22418,7 +22418,7 @@
         <v>48.25</v>
       </c>
       <c r="H94" t="n">
-        <v>8466620000</v>
+        <v>8504620000</v>
       </c>
       <c r="I94" t="n">
         <v>700</v>
@@ -22436,7 +22436,7 @@
         <v>5.78</v>
       </c>
       <c r="N94" t="n">
-        <v>0.794947733512501</v>
+        <v>0.7985156288324132</v>
       </c>
       <c r="O94" t="n">
         <v>0.36</v>
@@ -22514,7 +22514,7 @@
         <v>1209900967.64</v>
       </c>
       <c r="AN94" t="n">
-        <v>3045546762.589928</v>
+        <v>3059215827.33813</v>
       </c>
       <c r="AO94" t="n">
         <v>0</v>
@@ -22653,7 +22653,7 @@
         <v>43.01</v>
       </c>
       <c r="H95" t="n">
-        <v>8466620000</v>
+        <v>8504620000</v>
       </c>
       <c r="I95" t="n">
         <v>0</v>
@@ -22671,7 +22671,7 @@
         <v>4.65</v>
       </c>
       <c r="N95" t="n">
-        <v>4.439009863416192</v>
+        <v>4.458933088364261</v>
       </c>
       <c r="O95" t="n">
         <v>0.29</v>
@@ -22749,7 +22749,7 @@
         <v>216671749.24</v>
       </c>
       <c r="AN95" t="n">
-        <v>3779741071.428571</v>
+        <v>3796705357.142857</v>
       </c>
       <c r="AO95" t="n">
         <v>0</v>
@@ -23358,7 +23358,7 @@
         <v>39</v>
       </c>
       <c r="H98" t="n">
-        <v>10125870300</v>
+        <v>10125870000</v>
       </c>
       <c r="I98" t="n">
         <v>300</v>
@@ -23376,7 +23376,7 @@
         <v>24.76</v>
       </c>
       <c r="N98" t="n">
-        <v>2.055405152079463</v>
+        <v>2.055405091183804</v>
       </c>
       <c r="O98" t="n">
         <v>3.06</v>
@@ -23454,7 +23454,7 @@
         <v>576395765.0400001</v>
       </c>
       <c r="AN98" t="n">
-        <v>703674100.0694927</v>
+        <v>703674079.2216817</v>
       </c>
       <c r="AO98" t="n">
         <v>0</v>
@@ -23593,7 +23593,7 @@
         <v>123.99</v>
       </c>
       <c r="H99" t="n">
-        <v>16430174995</v>
+        <v>16431230000</v>
       </c>
       <c r="I99" t="n">
         <v>0</v>
@@ -23611,7 +23611,7 @@
         <v>10.65</v>
       </c>
       <c r="N99" t="n">
-        <v>1.623404683832894</v>
+        <v>1.623508924965991</v>
       </c>
       <c r="O99" t="n">
         <v>1.16</v>
@@ -23689,7 +23689,7 @@
         <v>1267125769.6</v>
       </c>
       <c r="AN99" t="n">
-        <v>2827913080.034424</v>
+        <v>2828094664.371773</v>
       </c>
       <c r="AO99" t="n">
         <v>0</v>
@@ -23828,7 +23828,7 @@
         <v>123.99</v>
       </c>
       <c r="H100" t="n">
-        <v>16430174995</v>
+        <v>16431230000</v>
       </c>
       <c r="I100" t="n">
         <v>400</v>
@@ -23846,7 +23846,7 @@
         <v>10.81</v>
       </c>
       <c r="N100" t="n">
-        <v>5.883605589352394</v>
+        <v>5.883983384069533</v>
       </c>
       <c r="O100" t="n">
         <v>1.18</v>
@@ -23924,7 +23924,7 @@
         <v>349625391.8</v>
       </c>
       <c r="AN100" t="n">
-        <v>2784775422.881356</v>
+        <v>2784954237.288136</v>
       </c>
       <c r="AO100" t="n">
         <v>0</v>
@@ -25708,7 +25708,7 @@
         <v>33.32</v>
       </c>
       <c r="H108" t="n">
-        <v>2810987237</v>
+        <v>2823659000</v>
       </c>
       <c r="I108" t="n">
         <v>0</v>
@@ -25726,7 +25726,7 @@
         <v>11.44</v>
       </c>
       <c r="N108" t="n">
-        <v>0.5140330116231125</v>
+        <v>0.5163502418160237</v>
       </c>
       <c r="O108" t="n">
         <v>0.21</v>
@@ -25804,7 +25804,7 @@
         <v>182100901.84</v>
       </c>
       <c r="AN108" t="n">
-        <v>989784238.3802817</v>
+        <v>994246126.7605634</v>
       </c>
       <c r="AO108" t="n">
         <v>0</v>
@@ -25943,7 +25943,7 @@
         <v>33.46</v>
       </c>
       <c r="H109" t="n">
-        <v>2810987237</v>
+        <v>2823659000</v>
       </c>
       <c r="I109" t="n">
         <v>700</v>
@@ -25961,7 +25961,7 @@
         <v>8.92</v>
       </c>
       <c r="N109" t="n">
-        <v>0.8795242277486919</v>
+        <v>0.8834890705697799</v>
       </c>
       <c r="O109" t="n">
         <v>0.17</v>
@@ -26039,7 +26039,7 @@
         <v>106427852.74</v>
       </c>
       <c r="AN109" t="n">
-        <v>1271939926.244344</v>
+        <v>1277673755.656109</v>
       </c>
       <c r="AO109" t="n">
         <v>0</v>
@@ -28763,7 +28763,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="H121" t="n">
-        <v>14957796</v>
+        <v>14957800</v>
       </c>
       <c r="I121" t="n">
         <v>3200</v>
@@ -28781,7 +28781,7 @@
         <v>0.19</v>
       </c>
       <c r="N121" t="n">
-        <v>0.03453912267618955</v>
+        <v>0.03453913191260986</v>
       </c>
       <c r="O121" t="n">
         <v>0.02</v>
@@ -28859,7 +28859,7 @@
         <v>129011019.48</v>
       </c>
       <c r="AN121" t="n">
-        <v>5002607.357859531</v>
+        <v>5002608.695652174</v>
       </c>
       <c r="AO121" t="n">
         <v>0</v>
@@ -31116,7 +31116,7 @@
         <v>2109342135</v>
       </c>
       <c r="I131" t="n">
-        <v>808700</v>
+        <v>0</v>
       </c>
       <c r="J131" t="n">
         <v>116217243</v>
@@ -31351,7 +31351,7 @@
         <v>828180636</v>
       </c>
       <c r="I132" t="n">
-        <v>46100</v>
+        <v>0</v>
       </c>
       <c r="J132" t="n">
         <v>116481187</v>
@@ -32758,7 +32758,7 @@
         <v>4.05</v>
       </c>
       <c r="H138" t="n">
-        <v>53953981</v>
+        <v>53954010</v>
       </c>
       <c r="I138" t="n">
         <v>17900</v>
@@ -32776,7 +32776,7 @@
         <v>15.76</v>
       </c>
       <c r="N138" t="n">
-        <v>0.2873569836108065</v>
+        <v>0.2873571380637749</v>
       </c>
       <c r="O138" t="n">
         <v>0.2</v>
@@ -32854,7 +32854,7 @@
         <v>2797615.38</v>
       </c>
       <c r="AN138" t="n">
-        <v>28101031.77083334</v>
+        <v>28101046.875</v>
       </c>
       <c r="AO138" t="n">
         <v>0</v>
@@ -33463,7 +33463,7 @@
         <v>13.49</v>
       </c>
       <c r="H141" t="n">
-        <v>295067662</v>
+        <v>295393500</v>
       </c>
       <c r="I141" t="n">
         <v>400</v>
@@ -33481,7 +33481,7 @@
         <v>2.98</v>
       </c>
       <c r="N141" t="n">
-        <v>1.174552095674234</v>
+        <v>1.17584913277805</v>
       </c>
       <c r="O141" t="n">
         <v>0.5</v>
@@ -33559,7 +33559,7 @@
         <v>45922500</v>
       </c>
       <c r="AN141" t="n">
-        <v>76640951.16883117</v>
+        <v>76725584.41558442</v>
       </c>
       <c r="AO141" t="n">
         <v>0</v>
@@ -33698,7 +33698,7 @@
         <v>12.4</v>
       </c>
       <c r="H142" t="n">
-        <v>295067662</v>
+        <v>295393500</v>
       </c>
       <c r="I142" t="n">
         <v>2100</v>
@@ -33716,7 +33716,7 @@
         <v>3.05</v>
       </c>
       <c r="N142" t="n">
-        <v>0.8981868966920612</v>
+        <v>0.8991787485949795</v>
       </c>
       <c r="O142" t="n">
         <v>0.51</v>
@@ -33794,7 +33794,7 @@
         <v>60052500</v>
       </c>
       <c r="AN142" t="n">
-        <v>74700673.92405063</v>
+        <v>74783164.55696203</v>
       </c>
       <c r="AO142" t="n">
         <v>0</v>
@@ -40748,10 +40748,10 @@
         <v>4.05</v>
       </c>
       <c r="H172" t="n">
-        <v>218121994</v>
+        <v>218122000</v>
       </c>
       <c r="I172" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="J172" t="n">
         <v>53857284</v>
@@ -40766,7 +40766,7 @@
         <v>0.38</v>
       </c>
       <c r="N172" t="n">
-        <v>0.04829369610626934</v>
+        <v>0.04829369743471023</v>
       </c>
       <c r="O172" t="n">
         <v>0.08</v>
@@ -40844,7 +40844,7 @@
         <v>640901679.6</v>
       </c>
       <c r="AN172" t="n">
-        <v>218121994</v>
+        <v>218122000</v>
       </c>
       <c r="AO172" t="n">
         <v>0</v>
@@ -42158,7 +42158,7 @@
         <v>205</v>
       </c>
       <c r="H178" t="n">
-        <v>1308387080</v>
+        <v>1308387000</v>
       </c>
       <c r="I178" t="n">
         <v>200</v>
@@ -42176,7 +42176,7 @@
         <v>52.85</v>
       </c>
       <c r="N178" t="n">
-        <v>0.5314813982081992</v>
+        <v>0.5314813657113086</v>
       </c>
       <c r="O178" t="n">
         <v>0.67</v>
@@ -42254,7 +42254,7 @@
         <v>24125385.06</v>
       </c>
       <c r="AN178" t="n">
-        <v>196454516.5165165</v>
+        <v>196454504.5045045</v>
       </c>
       <c r="AO178" t="n">
         <v>0</v>
@@ -42628,7 +42628,7 @@
         <v>35.22</v>
       </c>
       <c r="H180" t="n">
-        <v>3406523000</v>
+        <v>3521732000</v>
       </c>
       <c r="I180" t="n">
         <v>0</v>
@@ -42646,7 +42646,7 @@
         <v>12.71</v>
       </c>
       <c r="N180" t="n">
-        <v>8.322440323038641</v>
+        <v>8.603906212796895</v>
       </c>
       <c r="O180" t="n">
         <v>0.8</v>
@@ -42724,7 +42724,7 @@
         <v>84360399.48</v>
       </c>
       <c r="AN180" t="n">
-        <v>441831776.9130999</v>
+        <v>456774578.4695201</v>
       </c>
       <c r="AO180" t="n">
         <v>4.0605</v>
@@ -42863,7 +42863,7 @@
         <v>38.33</v>
       </c>
       <c r="H181" t="n">
-        <v>3406523000</v>
+        <v>3521732000</v>
       </c>
       <c r="I181" t="n">
         <v>100</v>
@@ -42881,7 +42881,7 @@
         <v>13.08</v>
       </c>
       <c r="N181" t="n">
-        <v>4.161220161519321</v>
+        <v>4.301953106398448</v>
       </c>
       <c r="O181" t="n">
         <v>0.83</v>
@@ -42959,7 +42959,7 @@
         <v>168720798.96</v>
       </c>
       <c r="AN181" t="n">
-        <v>429033123.4256927</v>
+        <v>443543073.0478589</v>
       </c>
       <c r="AO181" t="n">
         <v>4.0605</v>
@@ -43101,7 +43101,7 @@
         <v>27703023</v>
       </c>
       <c r="I182" t="n">
-        <v>401300</v>
+        <v>0</v>
       </c>
       <c r="J182" t="n">
         <v>24515924</v>
@@ -46391,7 +46391,7 @@
         <v>285833251</v>
       </c>
       <c r="I196" t="n">
-        <v>288700</v>
+        <v>0</v>
       </c>
       <c r="J196" t="n">
         <v>103188981</v>
@@ -46626,7 +46626,7 @@
         <v>4394033885</v>
       </c>
       <c r="I197" t="n">
-        <v>6893500</v>
+        <v>0</v>
       </c>
       <c r="J197" t="n">
         <v>1360382643</v>
@@ -48006,7 +48006,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>IBOVESPA</t>
+          <t>Brazil Stock Exchange Index</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
@@ -52955,7 +52955,7 @@
         <v>1265228793</v>
       </c>
       <c r="I224" t="n">
-        <v>791500</v>
+        <v>0</v>
       </c>
       <c r="J224" t="n">
         <v>179720130</v>
@@ -54130,7 +54130,7 @@
         <v>2290490048</v>
       </c>
       <c r="I229" t="n">
-        <v>406800</v>
+        <v>0</v>
       </c>
       <c r="J229" t="n">
         <v>195434352</v>
@@ -54835,7 +54835,7 @@
         <v>291753245</v>
       </c>
       <c r="I232" t="n">
-        <v>2103000</v>
+        <v>0</v>
       </c>
       <c r="J232" t="n">
         <v>206917263</v>
@@ -55070,7 +55070,7 @@
         <v>2389769219</v>
       </c>
       <c r="I233" t="n">
-        <v>495900</v>
+        <v>0</v>
       </c>
       <c r="J233" t="n">
         <v>87859154</v>
@@ -56242,7 +56242,7 @@
         <v>3.33</v>
       </c>
       <c r="H238" t="n">
-        <v>138421436</v>
+        <v>138421400</v>
       </c>
       <c r="I238" t="n">
         <v>4100</v>
@@ -56260,7 +56260,7 @@
         <v>4.2</v>
       </c>
       <c r="N238" t="n">
-        <v>1.616230276276742</v>
+        <v>1.616229855935128</v>
       </c>
       <c r="O238" t="n">
         <v>0.75</v>
@@ -56338,7 +56338,7 @@
         <v>23184000</v>
       </c>
       <c r="AN238" t="n">
-        <v>20003097.68786127</v>
+        <v>20003092.48554913</v>
       </c>
       <c r="AO238" t="n">
         <v>0</v>
@@ -57185,7 +57185,7 @@
         <v>1711105382</v>
       </c>
       <c r="I242" t="n">
-        <v>156900</v>
+        <v>0</v>
       </c>
       <c r="J242" t="n">
         <v>333548825</v>
@@ -58833,7 +58833,7 @@
         <v>2137100</v>
       </c>
       <c r="J249" t="n">
-        <v>234178207</v>
+        <v>234238661</v>
       </c>
       <c r="K249" t="n">
         <v>3.08</v>
@@ -58845,7 +58845,7 @@
         <v>11.84</v>
       </c>
       <c r="N249" t="n">
-        <v>2.006438548217108</v>
+        <v>2.005920712111505</v>
       </c>
       <c r="O249" t="n">
         <v>0.79</v>
@@ -58917,10 +58917,10 @@
         <v>0</v>
       </c>
       <c r="AL249" t="n">
-        <v>1774500733.23389</v>
+        <v>1774958827.386635</v>
       </c>
       <c r="AM249" t="n">
-        <v>297406322.89</v>
+        <v>297483099.47</v>
       </c>
       <c r="AN249" t="n">
         <v>606546281.9420784</v>
@@ -59065,7 +59065,7 @@
         <v>1378506316</v>
       </c>
       <c r="I250" t="n">
-        <v>592800</v>
+        <v>0</v>
       </c>
       <c r="J250" t="n">
         <v>820539225</v>
@@ -62120,7 +62120,7 @@
         <v>388193524</v>
       </c>
       <c r="I263" t="n">
-        <v>308300</v>
+        <v>0</v>
       </c>
       <c r="J263" t="n">
         <v>105774820</v>
@@ -64232,7 +64232,7 @@
         <v>1.87</v>
       </c>
       <c r="H272" t="n">
-        <v>12382173</v>
+        <v>12382180</v>
       </c>
       <c r="I272" t="n">
         <v>400</v>
@@ -64250,7 +64250,7 @@
         <v>0.96</v>
       </c>
       <c r="N272" t="n">
-        <v>4.749079792220064</v>
+        <v>4.749082477012026</v>
       </c>
       <c r="O272" t="n">
         <v>1.87</v>
@@ -64328,7 +64328,7 @@
         <v>37941114.78</v>
       </c>
       <c r="AN272" t="n">
-        <v>10957675.22123894</v>
+        <v>10957681.4159292</v>
       </c>
       <c r="AO272" t="n">
         <v>0</v>
@@ -65645,7 +65645,7 @@
         <v>1521030017</v>
       </c>
       <c r="I278" t="n">
-        <v>18637400</v>
+        <v>0</v>
       </c>
       <c r="J278" t="n">
         <v>1135097787</v>
@@ -65880,7 +65880,7 @@
         <v>2129568598</v>
       </c>
       <c r="I279" t="n">
-        <v>866400</v>
+        <v>0</v>
       </c>
       <c r="J279" t="n">
         <v>199959554</v>
@@ -67287,7 +67287,7 @@
         <v>1.49</v>
       </c>
       <c r="H285" t="n">
-        <v>4898354</v>
+        <v>4898350</v>
       </c>
       <c r="I285" t="n">
         <v>8800</v>
@@ -67305,7 +67305,7 @@
         <v>0.05</v>
       </c>
       <c r="N285" t="n">
-        <v>0.04965387162591944</v>
+        <v>0.04965383107852606</v>
       </c>
       <c r="O285" t="n">
         <v>0.02</v>
@@ -67383,7 +67383,7 @@
         <v>178674864.1</v>
       </c>
       <c r="AN285" t="n">
-        <v>24491770</v>
+        <v>24491750</v>
       </c>
       <c r="AO285" t="n">
         <v>0</v>
@@ -71050,7 +71050,7 @@
         <v>577126024</v>
       </c>
       <c r="I301" t="n">
-        <v>864300</v>
+        <v>0</v>
       </c>
       <c r="J301" t="n">
         <v>141800000</v>
@@ -75283,7 +75283,7 @@
         <v>2583700</v>
       </c>
       <c r="J319" t="n">
-        <v>293472126</v>
+        <v>293482126</v>
       </c>
       <c r="K319" t="n">
         <v>17.88</v>
@@ -75295,7 +75295,7 @@
         <v>5.09</v>
       </c>
       <c r="N319" t="n">
-        <v>1.013600373806227</v>
+        <v>1.013565836766863</v>
       </c>
       <c r="O319" t="n">
         <v>0.4</v>
@@ -75367,10 +75367,10 @@
         <v>57.65</v>
       </c>
       <c r="AL319" t="n">
-        <v>3292005241.148325</v>
+        <v>3292117415.523658</v>
       </c>
       <c r="AM319" t="n">
-        <v>619226185.86</v>
+        <v>619247285.86</v>
       </c>
       <c r="AN319" t="n">
         <v>887440889.0957447</v>
@@ -75512,7 +75512,7 @@
         <v>5.88</v>
       </c>
       <c r="H320" t="n">
-        <v>15101033933</v>
+        <v>15101040000</v>
       </c>
       <c r="I320" t="n">
         <v>100</v>
@@ -75530,7 +75530,7 @@
         <v>11.35</v>
       </c>
       <c r="N320" t="n">
-        <v>0.7782978214383929</v>
+        <v>0.7782981341277692</v>
       </c>
       <c r="O320" t="n">
         <v>0.49</v>
@@ -75608,7 +75608,7 @@
         <v>1412512331.45</v>
       </c>
       <c r="AN320" t="n">
-        <v>3340936710.840708</v>
+        <v>3340938053.097345</v>
       </c>
       <c r="AO320" t="n">
         <v>0</v>
@@ -76687,7 +76687,7 @@
         <v>7.5</v>
       </c>
       <c r="H325" t="n">
-        <v>602601400</v>
+        <v>601026800</v>
       </c>
       <c r="I325" t="n">
         <v>0</v>
@@ -76783,7 +76783,7 @@
         <v>8742210.08</v>
       </c>
       <c r="AN325" t="n">
-        <v>6919294.982202319</v>
+        <v>6901214.835227924</v>
       </c>
       <c r="AO325" t="n">
         <v>0</v>
@@ -76922,7 +76922,7 @@
         <v>6.82</v>
       </c>
       <c r="H326" t="n">
-        <v>602601400</v>
+        <v>601026800</v>
       </c>
       <c r="I326" t="n">
         <v>100</v>
@@ -77018,7 +77018,7 @@
         <v>2719637.39</v>
       </c>
       <c r="AN326" t="n">
-        <v>5946919.964472516</v>
+        <v>5931380.637520971</v>
       </c>
       <c r="AO326" t="n">
         <v>0.4906</v>
@@ -77157,7 +77157,7 @@
         <v>6.5</v>
       </c>
       <c r="H327" t="n">
-        <v>602601400</v>
+        <v>601026800</v>
       </c>
       <c r="I327" t="n">
         <v>0</v>
@@ -77253,7 +77253,7 @@
         <v>4627783.64</v>
       </c>
       <c r="AN327" t="n">
-        <v>8743491.004062681</v>
+        <v>8720644.225188624</v>
       </c>
       <c r="AO327" t="n">
         <v>0</v>
@@ -77392,7 +77392,7 @@
         <v>1.87</v>
       </c>
       <c r="H328" t="n">
-        <v>126583385</v>
+        <v>126583400</v>
       </c>
       <c r="I328" t="n">
         <v>3500</v>
@@ -77410,7 +77410,7 @@
         <v>0.11</v>
       </c>
       <c r="N328" t="n">
-        <v>0.01464108975559552</v>
+        <v>0.01464109149054949</v>
       </c>
       <c r="O328" t="n">
         <v>0.02</v>
@@ -77488,7 +77488,7 @@
         <v>1659121826.79</v>
       </c>
       <c r="AN328" t="n">
-        <v>1265833850</v>
+        <v>1265834000</v>
       </c>
       <c r="AO328" t="n">
         <v>0</v>
@@ -79510,7 +79510,7 @@
         <v>2638794919</v>
       </c>
       <c r="I337" t="n">
-        <v>1853200</v>
+        <v>0</v>
       </c>
       <c r="J337" t="n">
         <v>230663994</v>
@@ -83035,7 +83035,7 @@
         <v>891148357</v>
       </c>
       <c r="I352" t="n">
-        <v>800800</v>
+        <v>0</v>
       </c>
       <c r="J352" t="n">
         <v>141902688</v>
@@ -83267,7 +83267,7 @@
         <v>38.66</v>
       </c>
       <c r="H353" t="n">
-        <v>144628152</v>
+        <v>144628200</v>
       </c>
       <c r="I353" t="n">
         <v>0</v>
@@ -83285,7 +83285,7 @@
         <v>3.42</v>
       </c>
       <c r="N353" t="n">
-        <v>1.882462610288645</v>
+        <v>1.882463235050865</v>
       </c>
       <c r="O353" t="n">
         <v>0.78</v>
@@ -83363,7 +83363,7 @@
         <v>9672800</v>
       </c>
       <c r="AN353" t="n">
-        <v>58317803.22580645</v>
+        <v>58317822.58064516</v>
       </c>
       <c r="AO353" t="n">
         <v>0</v>
@@ -83502,7 +83502,7 @@
         <v>76</v>
       </c>
       <c r="H354" t="n">
-        <v>144628152</v>
+        <v>144628200</v>
       </c>
       <c r="I354" t="n">
         <v>100</v>
@@ -83520,7 +83520,7 @@
         <v>6.19</v>
       </c>
       <c r="N354" t="n">
-        <v>2.053770066794647</v>
+        <v>2.053770748411343</v>
       </c>
       <c r="O354" t="n">
         <v>1.42</v>
@@ -83598,7 +83598,7 @@
         <v>8865980</v>
       </c>
       <c r="AN354" t="n">
-        <v>32139589.33333333</v>
+        <v>32139600</v>
       </c>
       <c r="AO354" t="n">
         <v>0</v>
@@ -83737,7 +83737,7 @@
         <v>70.20999999999999</v>
       </c>
       <c r="H355" t="n">
-        <v>144628152</v>
+        <v>144628200</v>
       </c>
       <c r="I355" t="n">
         <v>0</v>
@@ -83755,7 +83755,7 @@
         <v>6.02</v>
       </c>
       <c r="N355" t="n">
-        <v>1.971599161149002</v>
+        <v>1.971599815494359</v>
       </c>
       <c r="O355" t="n">
         <v>1.38</v>
@@ -83833,7 +83833,7 @@
         <v>9235490</v>
       </c>
       <c r="AN355" t="n">
-        <v>33095686.95652174</v>
+        <v>33095697.94050343</v>
       </c>
       <c r="AO355" t="n">
         <v>0</v>
@@ -85617,7 +85617,7 @@
         <v>1.13</v>
       </c>
       <c r="H363" t="n">
-        <v>102277576</v>
+        <v>102277600</v>
       </c>
       <c r="I363" t="n">
         <v>24000</v>
@@ -85635,7 +85635,7 @@
         <v>0.74</v>
       </c>
       <c r="N363" t="n">
-        <v>0.3617754986321123</v>
+        <v>0.3617755835247379</v>
       </c>
       <c r="O363" t="n">
         <v>0.11</v>
@@ -85713,7 +85713,7 @@
         <v>163434690.6</v>
       </c>
       <c r="AN363" t="n">
-        <v>96488279.24528301</v>
+        <v>96488301.88679245</v>
       </c>
       <c r="AO363" t="n">
         <v>0</v>
@@ -85855,7 +85855,7 @@
         <v>520748192</v>
       </c>
       <c r="I364" t="n">
-        <v>55900</v>
+        <v>0</v>
       </c>
       <c r="J364" t="n">
         <v>60906215</v>
@@ -86795,7 +86795,7 @@
         <v>971259108</v>
       </c>
       <c r="I368" t="n">
-        <v>2087000</v>
+        <v>0</v>
       </c>
       <c r="J368" t="n">
         <v>65492864</v>
@@ -89145,7 +89145,7 @@
         <v>7811506751</v>
       </c>
       <c r="I378" t="n">
-        <v>1138000</v>
+        <v>0</v>
       </c>
       <c r="J378" t="n">
         <v>500737647</v>
@@ -90082,7 +90082,7 @@
         <v>1.32</v>
       </c>
       <c r="H382" t="n">
-        <v>87233998</v>
+        <v>87234000</v>
       </c>
       <c r="I382" t="n">
         <v>6762700</v>
@@ -90100,7 +90100,7 @@
         <v>39.8</v>
       </c>
       <c r="N382" t="n">
-        <v>0.3233999908059702</v>
+        <v>0.3233999982205104</v>
       </c>
       <c r="O382" t="n">
         <v>0.24</v>
@@ -90178,7 +90178,7 @@
         <v>2643454.56</v>
       </c>
       <c r="AN382" t="n">
-        <v>8237393.57884797</v>
+        <v>8237393.767705383</v>
       </c>
       <c r="AO382" t="n">
         <v>0</v>
@@ -94550,7 +94550,7 @@
         <v>435807817</v>
       </c>
       <c r="I401" t="n">
-        <v>1255800</v>
+        <v>0</v>
       </c>
       <c r="J401" t="n">
         <v>322820608</v>
@@ -95017,10 +95017,10 @@
         <v>8.32</v>
       </c>
       <c r="H403" t="n">
-        <v>92429705</v>
+        <v>92429780</v>
       </c>
       <c r="I403" t="n">
-        <v>59800</v>
+        <v>0</v>
       </c>
       <c r="J403" t="n">
         <v>11109348</v>
@@ -95035,7 +95035,7 @@
         <v>5.91</v>
       </c>
       <c r="N403" t="n">
-        <v>0.6316733055609033</v>
+        <v>0.631673818117964</v>
       </c>
       <c r="O403" t="n">
         <v>0.23</v>
@@ -95113,7 +95113,7 @@
         <v>11442628.44</v>
       </c>
       <c r="AN403" t="n">
-        <v>39669401.28755365</v>
+        <v>39669433.47639485</v>
       </c>
       <c r="AO403" t="n">
         <v>0</v>
@@ -95252,7 +95252,7 @@
         <v>3.99</v>
       </c>
       <c r="H404" t="n">
-        <v>6030860251</v>
+        <v>6010339000</v>
       </c>
       <c r="I404" t="n">
         <v>800</v>
@@ -95270,7 +95270,7 @@
         <v>9.42</v>
       </c>
       <c r="N404" t="n">
-        <v>0.6798119474799617</v>
+        <v>0.6774987465390641</v>
       </c>
       <c r="O404" t="n">
         <v>0.66</v>
@@ -95348,7 +95348,7 @@
         <v>483489419.2399999</v>
       </c>
       <c r="AN404" t="n">
-        <v>1157554750.671785</v>
+        <v>1153615930.902111</v>
       </c>
       <c r="AO404" t="n">
         <v>0</v>
@@ -95487,7 +95487,7 @@
         <v>4.02</v>
       </c>
       <c r="H405" t="n">
-        <v>6030860251</v>
+        <v>6010339000</v>
       </c>
       <c r="I405" t="n">
         <v>13600</v>
@@ -95505,7 +95505,7 @@
         <v>9.92</v>
       </c>
       <c r="N405" t="n">
-        <v>1.475100432630107</v>
+        <v>1.470081097913606</v>
       </c>
       <c r="O405" t="n">
         <v>0.6899999999999999</v>
@@ -95583,7 +95583,7 @@
         <v>222820003.58</v>
       </c>
       <c r="AN405" t="n">
-        <v>1100521943.613139</v>
+        <v>1096777189.781022</v>
       </c>
       <c r="AO405" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-06-05 05:21
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1300,7 +1300,7 @@
         <v>16.07</v>
       </c>
       <c r="H4" t="n">
-        <v>252288710408</v>
+        <v>50125205609</v>
       </c>
       <c r="I4" t="n">
         <v>24645900</v>
@@ -1318,7 +1318,7 @@
         <v>15.16</v>
       </c>
       <c r="N4" t="n">
-        <v>2.781949145878039</v>
+        <v>0.552723000190566</v>
       </c>
       <c r="O4" t="n">
         <v>1.73</v>
@@ -1396,7 +1396,7 @@
         <v>16078938186.78</v>
       </c>
       <c r="AN4" t="n">
-        <v>24831565985.03937</v>
+        <v>4933583229.232284</v>
       </c>
       <c r="AO4" t="n">
         <v>0.269</v>
@@ -1770,7 +1770,7 @@
         <v>7.62</v>
       </c>
       <c r="H6" t="n">
-        <v>478744700</v>
+        <v>486371500</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -1788,7 +1788,7 @@
         <v>13.39</v>
       </c>
       <c r="N6" t="n">
-        <v>5.905559051416731</v>
+        <v>5.999639503426634</v>
       </c>
       <c r="O6" t="n">
         <v>1.24</v>
@@ -1866,7 +1866,7 @@
         <v>34696585</v>
       </c>
       <c r="AN6" t="n">
-        <v>51367457.08154506</v>
+        <v>52185783.26180258</v>
       </c>
       <c r="AO6" t="n">
         <v>0</v>
@@ -2005,7 +2005,7 @@
         <v>18.5</v>
       </c>
       <c r="H7" t="n">
-        <v>1899642900</v>
+        <v>383570205</v>
       </c>
       <c r="I7" t="n">
         <v>146400</v>
@@ -2023,7 +2023,7 @@
         <v>87.38</v>
       </c>
       <c r="N7" t="n">
-        <v>1.866086156900857</v>
+        <v>0.3767945279347628</v>
       </c>
       <c r="O7" t="n">
         <v>0.54</v>
@@ -2101,7 +2101,7 @@
         <v>23617192.12</v>
       </c>
       <c r="AN7" t="n">
-        <v>62059552.43384515</v>
+        <v>12530878.96112382</v>
       </c>
       <c r="AO7" t="n">
         <v>0</v>
@@ -2475,7 +2475,7 @@
         <v>23.9</v>
       </c>
       <c r="H9" t="n">
-        <v>208533200</v>
+        <v>211022600</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -2493,7 +2493,7 @@
         <v>2.59</v>
       </c>
       <c r="N9" t="n">
-        <v>0.3145196764442663</v>
+        <v>0.3182743077573635</v>
       </c>
       <c r="O9" t="n">
         <v>0.36</v>
@@ -2571,7 +2571,7 @@
         <v>81220091.82000001</v>
       </c>
       <c r="AN9" t="n">
-        <v>72659651.56794424</v>
+        <v>73527038.32752612</v>
       </c>
       <c r="AO9" t="n">
         <v>0</v>
@@ -2710,7 +2710,7 @@
         <v>58</v>
       </c>
       <c r="H10" t="n">
-        <v>208533200</v>
+        <v>211022600</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -2728,7 +2728,7 @@
         <v>6.01</v>
       </c>
       <c r="N10" t="n">
-        <v>58.73667881531669</v>
+        <v>59.43785775585398</v>
       </c>
       <c r="O10" t="n">
         <v>0.84</v>
@@ -2806,7 +2806,7 @@
         <v>434912.52</v>
       </c>
       <c r="AN10" t="n">
-        <v>31264347.82608696</v>
+        <v>31637571.2143928</v>
       </c>
       <c r="AO10" t="n">
         <v>0</v>
@@ -2945,7 +2945,7 @@
         <v>55</v>
       </c>
       <c r="H11" t="n">
-        <v>208533200</v>
+        <v>211022600</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -2963,7 +2963,7 @@
         <v>5.7</v>
       </c>
       <c r="N11" t="n">
-        <v>29.06140725999438</v>
+        <v>29.40833267634549</v>
       </c>
       <c r="O11" t="n">
         <v>0.79</v>
@@ -3041,7 +3041,7 @@
         <v>879011.7000000001</v>
       </c>
       <c r="AN11" t="n">
-        <v>32995759.49367088</v>
+        <v>33389651.89873417</v>
       </c>
       <c r="AO11" t="n">
         <v>0</v>
@@ -6470,7 +6470,7 @@
         <v>8.789999999999999</v>
       </c>
       <c r="H26" t="n">
-        <v>11849016638</v>
+        <v>2484807181</v>
       </c>
       <c r="I26" t="n">
         <v>14407900</v>
@@ -6488,7 +6488,7 @@
         <v>12.95</v>
       </c>
       <c r="N26" t="n">
-        <v>0.1544850122654682</v>
+        <v>0.03239639875287586</v>
       </c>
       <c r="O26" t="n">
         <v>0.26</v>
@@ -6566,7 +6566,7 @@
         <v>920401258.1600001</v>
       </c>
       <c r="AN26" t="n">
-        <v>4128577225.783972</v>
+        <v>865786474.2160279</v>
       </c>
       <c r="AO26" t="n">
         <v>0.1043</v>
@@ -6924,7 +6924,7 @@
         <v>108.98</v>
       </c>
       <c r="H28" t="n">
-        <v>5381781881</v>
+        <v>5602147300</v>
       </c>
       <c r="I28" t="n">
         <v>1303791</v>
@@ -6942,7 +6942,7 @@
         <v>97.38</v>
       </c>
       <c r="N28" t="n">
-        <v>3.195030783170264</v>
+        <v>3.325856281642601</v>
       </c>
       <c r="O28" t="n">
         <v>3.27</v>
@@ -7020,7 +7020,7 @@
         <v>98033392.08</v>
       </c>
       <c r="AN28" t="n">
-        <v>442945010.781893</v>
+        <v>461082082.3045267</v>
       </c>
       <c r="AO28" t="n">
         <v>0</v>
@@ -8804,7 +8804,7 @@
         <v>26</v>
       </c>
       <c r="H36" t="n">
-        <v>217718167</v>
+        <v>222603300</v>
       </c>
       <c r="I36" t="n">
         <v>200</v>
@@ -8822,7 +8822,7 @@
         <v>10.3</v>
       </c>
       <c r="N36" t="n">
-        <v>1.988873440038873</v>
+        <v>2.033499533527697</v>
       </c>
       <c r="O36" t="n">
         <v>0.85</v>
@@ -8900,7 +8900,7 @@
         <v>12348000</v>
       </c>
       <c r="AN36" t="n">
-        <v>38947793.73881932</v>
+        <v>39821699.46332737</v>
       </c>
       <c r="AO36" t="n">
         <v>0</v>
@@ -9039,7 +9039,7 @@
         <v>18.9</v>
       </c>
       <c r="H37" t="n">
-        <v>217718167</v>
+        <v>222603300</v>
       </c>
       <c r="I37" t="n">
         <v>100</v>
@@ -9057,7 +9057,7 @@
         <v>7.41</v>
       </c>
       <c r="N37" t="n">
-        <v>1.988873440038873</v>
+        <v>2.033499533527697</v>
       </c>
       <c r="O37" t="n">
         <v>0.61</v>
@@ -9135,7 +9135,7 @@
         <v>12348000</v>
       </c>
       <c r="AN37" t="n">
-        <v>54158748.00995026</v>
+        <v>55373955.2238806</v>
       </c>
       <c r="AO37" t="n">
         <v>0</v>
@@ -9274,7 +9274,7 @@
         <v>93.90000000000001</v>
       </c>
       <c r="H38" t="n">
-        <v>489276300</v>
+        <v>496146600</v>
       </c>
       <c r="I38" t="n">
         <v>400</v>
@@ -9292,7 +9292,7 @@
         <v>17.37</v>
       </c>
       <c r="N38" t="n">
-        <v>3.946454263501761</v>
+        <v>4.001869424069596</v>
       </c>
       <c r="O38" t="n">
         <v>2.37</v>
@@ -9370,7 +9370,7 @@
         <v>12707817.55</v>
       </c>
       <c r="AN38" t="n">
-        <v>21911164.35288849</v>
+        <v>22218835.64711151</v>
       </c>
       <c r="AO38" t="n">
         <v>0</v>
@@ -9979,7 +9979,7 @@
         <v>15.11</v>
       </c>
       <c r="H41" t="n">
-        <v>171240416273</v>
+        <v>34463147866</v>
       </c>
       <c r="I41" t="n">
         <v>5029500</v>
@@ -9997,7 +9997,7 @@
         <v>8.74</v>
       </c>
       <c r="N41" t="n">
-        <v>1.354743067791931</v>
+        <v>0.2726500652236111</v>
       </c>
       <c r="O41" t="n">
         <v>0.09</v>
@@ -10075,7 +10075,7 @@
         <v>10819896393.24</v>
       </c>
       <c r="AN41" t="n">
-        <v>16854371680.41339</v>
+        <v>3392042112.795276</v>
       </c>
       <c r="AO41" t="n">
         <v>0.5647</v>
@@ -10214,7 +10214,7 @@
         <v>17.37</v>
       </c>
       <c r="H42" t="n">
-        <v>171240416273</v>
+        <v>34463147866</v>
       </c>
       <c r="I42" t="n">
         <v>30635400</v>
@@ -10232,7 +10232,7 @@
         <v>10.11</v>
       </c>
       <c r="N42" t="n">
-        <v>1.358772740251641</v>
+        <v>0.2734610606699732</v>
       </c>
       <c r="O42" t="n">
         <v>0.1</v>
@@ -10310,7 +10310,7 @@
         <v>10787808143.88</v>
       </c>
       <c r="AN42" t="n">
-        <v>14561259887.15986</v>
+        <v>2930539784.523809</v>
       </c>
       <c r="AO42" t="n">
         <v>1.1139</v>
@@ -11389,7 +11389,7 @@
         <v>8.75</v>
       </c>
       <c r="H47" t="n">
-        <v>3041819375</v>
+        <v>3095401000</v>
       </c>
       <c r="I47" t="n">
         <v>8500</v>
@@ -11407,7 +11407,7 @@
         <v>8.390000000000001</v>
       </c>
       <c r="N47" t="n">
-        <v>0.8159581099878105</v>
+        <v>0.8303312058476117</v>
       </c>
       <c r="O47" t="n">
         <v>0.07000000000000001</v>
@@ -11485,7 +11485,7 @@
         <v>249024468</v>
       </c>
       <c r="AN47" t="n">
-        <v>462986206.240487</v>
+        <v>471141704.718417</v>
       </c>
       <c r="AO47" t="n">
         <v>0.3403</v>
@@ -11624,7 +11624,7 @@
         <v>8.949999999999999</v>
       </c>
       <c r="H48" t="n">
-        <v>3041819375</v>
+        <v>3095401000</v>
       </c>
       <c r="I48" t="n">
         <v>2400</v>
@@ -11642,7 +11642,7 @@
         <v>8.449999999999999</v>
       </c>
       <c r="N48" t="n">
-        <v>2.21997632648109</v>
+        <v>2.259081192474123</v>
       </c>
       <c r="O48" t="n">
         <v>0.07000000000000001</v>
@@ -11720,7 +11720,7 @@
         <v>91529595.08</v>
       </c>
       <c r="AN48" t="n">
-        <v>459489331.570997</v>
+        <v>467583232.6283988</v>
       </c>
       <c r="AO48" t="n">
         <v>0.3691</v>
@@ -11859,7 +11859,7 @@
         <v>52.6</v>
       </c>
       <c r="H49" t="n">
-        <v>972035000</v>
+        <v>975138100</v>
       </c>
       <c r="I49" t="n">
         <v>0</v>
@@ -11877,7 +11877,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="N49" t="n">
-        <v>1.061377655646017</v>
+        <v>1.064765970884908</v>
       </c>
       <c r="O49" t="n">
         <v>0.08</v>
@@ -11955,7 +11955,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN49" t="n">
-        <v>177702925.0457039</v>
+        <v>178270219.3784278</v>
       </c>
       <c r="AO49" t="n">
         <v>2.4346</v>
@@ -12094,7 +12094,7 @@
         <v>30.91</v>
       </c>
       <c r="H50" t="n">
-        <v>972035000</v>
+        <v>975138100</v>
       </c>
       <c r="I50" t="n">
         <v>200</v>
@@ -12112,7 +12112,7 @@
         <v>5.78</v>
       </c>
       <c r="N50" t="n">
-        <v>1.061377655646017</v>
+        <v>1.064765970884908</v>
       </c>
       <c r="O50" t="n">
         <v>0.06</v>
@@ -12190,7 +12190,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN50" t="n">
-        <v>255127296.5879265</v>
+        <v>255941758.5301837</v>
       </c>
       <c r="AO50" t="n">
         <v>3.526</v>
@@ -12548,7 +12548,7 @@
         <v>9.109999999999999</v>
       </c>
       <c r="H52" t="n">
-        <v>241638800</v>
+        <v>245488300</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
@@ -13958,7 +13958,7 @@
         <v>21.49</v>
       </c>
       <c r="H58" t="n">
-        <v>100696200</v>
+        <v>102300400</v>
       </c>
       <c r="I58" t="n">
         <v>0</v>
@@ -13976,7 +13976,7 @@
         <v>13.78</v>
       </c>
       <c r="N58" t="n">
-        <v>1.869697854855712</v>
+        <v>1.899484175479127</v>
       </c>
       <c r="O58" t="n">
         <v>0.17</v>
@@ -14054,7 +14054,7 @@
         <v>6872145.189999999</v>
       </c>
       <c r="AN58" t="n">
-        <v>14303437.5</v>
+        <v>14531306.81818182</v>
       </c>
       <c r="AO58" t="n">
         <v>0</v>
@@ -14193,7 +14193,7 @@
         <v>17.85</v>
       </c>
       <c r="H59" t="n">
-        <v>100696200</v>
+        <v>102300400</v>
       </c>
       <c r="I59" t="n">
         <v>100</v>
@@ -14211,7 +14211,7 @@
         <v>12.47</v>
       </c>
       <c r="N59" t="n">
-        <v>10.83431540620549</v>
+        <v>11.00691783583674</v>
       </c>
       <c r="O59" t="n">
         <v>0.15</v>
@@ -14289,7 +14289,7 @@
         <v>1185938.81</v>
       </c>
       <c r="AN59" t="n">
-        <v>15807880.69073783</v>
+        <v>16059717.42543171</v>
       </c>
       <c r="AO59" t="n">
         <v>0</v>
@@ -14428,7 +14428,7 @@
         <v>390</v>
       </c>
       <c r="H60" t="n">
-        <v>176629089</v>
+        <v>179443000</v>
       </c>
       <c r="I60" t="n">
         <v>98</v>
@@ -14446,7 +14446,7 @@
         <v>2.87</v>
       </c>
       <c r="N60" t="n">
-        <v>12.48173035702111</v>
+        <v>12.6805791341365</v>
       </c>
       <c r="O60" t="n">
         <v>0.64</v>
@@ -14524,7 +14524,7 @@
         <v>59731412.5</v>
       </c>
       <c r="AN60" t="n">
-        <v>22245477.20403023</v>
+        <v>22599874.05541562</v>
       </c>
       <c r="AO60" t="n">
         <v>0</v>
@@ -16073,7 +16073,7 @@
         <v>180</v>
       </c>
       <c r="H67" t="n">
-        <v>1679480000</v>
+        <v>1699276000</v>
       </c>
       <c r="I67" t="n">
         <v>0</v>
@@ -16091,7 +16091,7 @@
         <v>4.43</v>
       </c>
       <c r="N67" t="n">
-        <v>0.460772768697043</v>
+        <v>0.4662038888825329</v>
       </c>
       <c r="O67" t="n">
         <v>0.06</v>
@@ -16169,7 +16169,7 @@
         <v>252228482.01</v>
       </c>
       <c r="AN67" t="n">
-        <v>608507246.3768116</v>
+        <v>615679710.1449276</v>
       </c>
       <c r="AO67" t="n">
         <v>0</v>
@@ -17248,7 +17248,7 @@
         <v>7.22</v>
       </c>
       <c r="H72" t="n">
-        <v>6439290796</v>
+        <v>1288524924</v>
       </c>
       <c r="I72" t="n">
         <v>27800</v>
@@ -17266,7 +17266,7 @@
         <v>1.5</v>
       </c>
       <c r="N72" t="n">
-        <v>0.1540485788909728</v>
+        <v>0.03082566694007691</v>
       </c>
       <c r="O72" t="n">
         <v>0.08</v>
@@ -17344,7 +17344,7 @@
         <v>2691945165.92</v>
       </c>
       <c r="AN72" t="n">
-        <v>3597369159.776536</v>
+        <v>719846326.2569833</v>
       </c>
       <c r="AO72" t="n">
         <v>0</v>
@@ -17483,7 +17483,7 @@
         <v>9.43</v>
       </c>
       <c r="H73" t="n">
-        <v>6439290796</v>
+        <v>1288524924</v>
       </c>
       <c r="I73" t="n">
         <v>8515200</v>
@@ -17501,7 +17501,7 @@
         <v>1.57</v>
       </c>
       <c r="N73" t="n">
-        <v>0.2016427140968452</v>
+        <v>0.04034942217832264</v>
       </c>
       <c r="O73" t="n">
         <v>0.09</v>
@@ -17579,7 +17579,7 @@
         <v>2056559936.32</v>
       </c>
       <c r="AN73" t="n">
-        <v>3443471013.903743</v>
+        <v>689050761.4973261</v>
       </c>
       <c r="AO73" t="n">
         <v>0</v>
@@ -17718,7 +17718,7 @@
         <v>7.02</v>
       </c>
       <c r="H74" t="n">
-        <v>6439290796</v>
+        <v>1288524924</v>
       </c>
       <c r="I74" t="n">
         <v>0</v>
@@ -17736,7 +17736,7 @@
         <v>1.36</v>
       </c>
       <c r="N74" t="n">
-        <v>145.3224043321735</v>
+        <v>29.07952846514234</v>
       </c>
       <c r="O74" t="n">
         <v>0.07000000000000001</v>
@@ -17814,7 +17814,7 @@
         <v>2853588.4</v>
       </c>
       <c r="AN74" t="n">
-        <v>3974870861.728395</v>
+        <v>795385755.5555555</v>
       </c>
       <c r="AO74" t="n">
         <v>0</v>
@@ -18893,7 +18893,7 @@
         <v>3.35</v>
       </c>
       <c r="H79" t="n">
-        <v>7367671540</v>
+        <v>7518212000</v>
       </c>
       <c r="I79" t="n">
         <v>42700</v>
@@ -18911,7 +18911,7 @@
         <v>2.47</v>
       </c>
       <c r="N79" t="n">
-        <v>1.030140892164263</v>
+        <v>1.051189317427154</v>
       </c>
       <c r="O79" t="n">
         <v>0.03</v>
@@ -18989,7 +18989,7 @@
         <v>531401092.4</v>
       </c>
       <c r="AN79" t="n">
-        <v>4465255478.787879</v>
+        <v>4556492121.212121</v>
       </c>
       <c r="AO79" t="n">
         <v>0</v>
@@ -19128,7 +19128,7 @@
         <v>3.75</v>
       </c>
       <c r="H80" t="n">
-        <v>7367671540</v>
+        <v>7518212000</v>
       </c>
       <c r="I80" t="n">
         <v>10300</v>
@@ -19146,7 +19146,7 @@
         <v>3.36</v>
       </c>
       <c r="N80" t="n">
-        <v>1.985848380165031</v>
+        <v>2.026424364995145</v>
       </c>
       <c r="O80" t="n">
         <v>0.04</v>
@@ -19224,7 +19224,7 @@
         <v>275659512.02</v>
       </c>
       <c r="AN80" t="n">
-        <v>3274520684.444445</v>
+        <v>3341427555.555555</v>
       </c>
       <c r="AO80" t="n">
         <v>0</v>
@@ -19598,7 +19598,7 @@
         <v>9.56</v>
       </c>
       <c r="H82" t="n">
-        <v>407954500</v>
+        <v>408913500</v>
       </c>
       <c r="I82" t="n">
         <v>5800</v>
@@ -19616,7 +19616,7 @@
         <v>6.04</v>
       </c>
       <c r="N82" t="n">
-        <v>1.037374944056877</v>
+        <v>1.039813555645548</v>
       </c>
       <c r="O82" t="n">
         <v>1.01</v>
@@ -19694,7 +19694,7 @@
         <v>65949124.8</v>
       </c>
       <c r="AN82" t="n">
-        <v>72589768.68327402</v>
+        <v>72760409.25266904</v>
       </c>
       <c r="AO82" t="n">
         <v>0</v>
@@ -20773,7 +20773,7 @@
         <v>15.31</v>
       </c>
       <c r="H87" t="n">
-        <v>6910556032</v>
+        <v>6938858000</v>
       </c>
       <c r="I87" t="n">
         <v>100</v>
@@ -20791,7 +20791,7 @@
         <v>7.13</v>
       </c>
       <c r="N87" t="n">
-        <v>0.7373621269827751</v>
+        <v>0.740381970715413</v>
       </c>
       <c r="O87" t="n">
         <v>0.21</v>
@@ -20869,7 +20869,7 @@
         <v>580126647.04</v>
       </c>
       <c r="AN87" t="n">
-        <v>1258753375.591985</v>
+        <v>1263908561.020036</v>
       </c>
       <c r="AO87" t="n">
         <v>0</v>
@@ -21243,7 +21243,7 @@
         <v>27.6</v>
       </c>
       <c r="H89" t="n">
-        <v>1994288259</v>
+        <v>2031912000</v>
       </c>
       <c r="I89" t="n">
         <v>3500</v>
@@ -21261,7 +21261,7 @@
         <v>11.38</v>
       </c>
       <c r="N89" t="n">
-        <v>8.348628424617905</v>
+        <v>8.506131549923653</v>
       </c>
       <c r="O89" t="n">
         <v>1.53</v>
@@ -21339,7 +21339,7 @@
         <v>95908776.3</v>
       </c>
       <c r="AN89" t="n">
-        <v>217479635.6597601</v>
+        <v>221582551.7993457</v>
       </c>
       <c r="AO89" t="n">
         <v>0</v>
@@ -21478,7 +21478,7 @@
         <v>24.6</v>
       </c>
       <c r="H90" t="n">
-        <v>1994288259</v>
+        <v>2031912000</v>
       </c>
       <c r="I90" t="n">
         <v>3900</v>
@@ -21496,7 +21496,7 @@
         <v>10.59</v>
       </c>
       <c r="N90" t="n">
-        <v>45.68007715016017</v>
+        <v>46.54186600330191</v>
       </c>
       <c r="O90" t="n">
         <v>1.42</v>
@@ -21574,7 +21574,7 @@
         <v>17528576.7</v>
       </c>
       <c r="AN90" t="n">
-        <v>233796982.2977726</v>
+        <v>238207737.3974209</v>
       </c>
       <c r="AO90" t="n">
         <v>0</v>
@@ -21713,7 +21713,7 @@
         <v>28.9</v>
       </c>
       <c r="H91" t="n">
-        <v>1994288259</v>
+        <v>2031912000</v>
       </c>
       <c r="I91" t="n">
         <v>900</v>
@@ -21731,7 +21731,7 @@
         <v>11.3</v>
       </c>
       <c r="N91" t="n">
-        <v>10.1327885964233</v>
+        <v>10.32395123905489</v>
       </c>
       <c r="O91" t="n">
         <v>1.52</v>
@@ -21809,7 +21809,7 @@
         <v>79021360.05</v>
       </c>
       <c r="AN91" t="n">
-        <v>219152555.9340659</v>
+        <v>223287032.967033</v>
       </c>
       <c r="AO91" t="n">
         <v>0</v>
@@ -21948,7 +21948,7 @@
         <v>10</v>
       </c>
       <c r="H92" t="n">
-        <v>78056470</v>
+        <v>78472560</v>
       </c>
       <c r="I92" t="n">
         <v>0</v>
@@ -21966,7 +21966,7 @@
         <v>3.42</v>
       </c>
       <c r="N92" t="n">
-        <v>0.144127575961674</v>
+        <v>0.1448958664452418</v>
       </c>
       <c r="O92" t="n">
         <v>0.15</v>
@@ -22044,7 +22044,7 @@
         <v>23342055.36</v>
       </c>
       <c r="AN92" t="n">
-        <v>55359198.58156028</v>
+        <v>55654297.87234043</v>
       </c>
       <c r="AO92" t="n">
         <v>0</v>
@@ -22183,7 +22183,7 @@
         <v>4.76</v>
       </c>
       <c r="H93" t="n">
-        <v>78056470</v>
+        <v>78472560</v>
       </c>
       <c r="I93" t="n">
         <v>1000</v>
@@ -22201,7 +22201,7 @@
         <v>2.3</v>
       </c>
       <c r="N93" t="n">
-        <v>0.1916074988262408</v>
+        <v>0.1926288871132925</v>
       </c>
       <c r="O93" t="n">
         <v>0.1</v>
@@ -22279,7 +22279,7 @@
         <v>17557944.64</v>
       </c>
       <c r="AN93" t="n">
-        <v>82164705.2631579</v>
+        <v>82602694.73684211</v>
       </c>
       <c r="AO93" t="n">
         <v>0</v>
@@ -22418,7 +22418,7 @@
         <v>47.02</v>
       </c>
       <c r="H94" t="n">
-        <v>8462061000</v>
+        <v>8415703000</v>
       </c>
       <c r="I94" t="n">
         <v>400</v>
@@ -22436,7 +22436,7 @@
         <v>5.78</v>
       </c>
       <c r="N94" t="n">
-        <v>0.7945196799660937</v>
+        <v>0.790167035459765</v>
       </c>
       <c r="O94" t="n">
         <v>0.36</v>
@@ -22514,7 +22514,7 @@
         <v>1209900967.64</v>
       </c>
       <c r="AN94" t="n">
-        <v>3043906834.532374</v>
+        <v>3027231294.964029</v>
       </c>
       <c r="AO94" t="n">
         <v>0</v>
@@ -22653,7 +22653,7 @@
         <v>43.01</v>
       </c>
       <c r="H95" t="n">
-        <v>8462061000</v>
+        <v>8415703000</v>
       </c>
       <c r="I95" t="n">
         <v>0</v>
@@ -22671,7 +22671,7 @@
         <v>4.65</v>
       </c>
       <c r="N95" t="n">
-        <v>4.436619600717818</v>
+        <v>4.412314314871961</v>
       </c>
       <c r="O95" t="n">
         <v>0.29</v>
@@ -22749,7 +22749,7 @@
         <v>216671749.24</v>
       </c>
       <c r="AN95" t="n">
-        <v>3777705803.571428</v>
+        <v>3757010267.857142</v>
       </c>
       <c r="AO95" t="n">
         <v>0</v>
@@ -23358,7 +23358,7 @@
         <v>39</v>
       </c>
       <c r="H98" t="n">
-        <v>10084570000</v>
+        <v>10245230000</v>
       </c>
       <c r="I98" t="n">
         <v>0</v>
@@ -23376,7 +23376,7 @@
         <v>24.76</v>
       </c>
       <c r="N98" t="n">
-        <v>2.047021788784515</v>
+        <v>2.079633444074341</v>
       </c>
       <c r="O98" t="n">
         <v>3.06</v>
@@ -23454,7 +23454,7 @@
         <v>576395765.0400001</v>
       </c>
       <c r="AN98" t="n">
-        <v>700804030.5767894</v>
+        <v>711968728.2835302</v>
       </c>
       <c r="AO98" t="n">
         <v>0</v>
@@ -23593,7 +23593,7 @@
         <v>124</v>
       </c>
       <c r="H99" t="n">
-        <v>16704261000</v>
+        <v>16597250000</v>
       </c>
       <c r="I99" t="n">
         <v>300</v>
@@ -23611,7 +23611,7 @@
         <v>10.65</v>
       </c>
       <c r="N99" t="n">
-        <v>1.650486105937373</v>
+        <v>1.639912745722128</v>
       </c>
       <c r="O99" t="n">
         <v>1.16</v>
@@ -23689,7 +23689,7 @@
         <v>1267125769.6</v>
       </c>
       <c r="AN99" t="n">
-        <v>2875087951.807229</v>
+        <v>2856669535.283993</v>
       </c>
       <c r="AO99" t="n">
         <v>0</v>
@@ -23828,7 +23828,7 @@
         <v>123</v>
       </c>
       <c r="H100" t="n">
-        <v>16704261000</v>
+        <v>16597250000</v>
       </c>
       <c r="I100" t="n">
         <v>1400</v>
@@ -23846,7 +23846,7 @@
         <v>10.81</v>
       </c>
       <c r="N100" t="n">
-        <v>5.981755119194408</v>
+        <v>5.94343474111482</v>
       </c>
       <c r="O100" t="n">
         <v>1.18</v>
@@ -23924,7 +23924,7 @@
         <v>349625391.8</v>
       </c>
       <c r="AN100" t="n">
-        <v>2831230677.966102</v>
+        <v>2813093220.338983</v>
       </c>
       <c r="AO100" t="n">
         <v>0</v>
@@ -24063,7 +24063,7 @@
         <v>24.55</v>
       </c>
       <c r="H101" t="n">
-        <v>627899028</v>
+        <v>639332100</v>
       </c>
       <c r="I101" t="n">
         <v>600</v>
@@ -24081,7 +24081,7 @@
         <v>6.28</v>
       </c>
       <c r="N101" t="n">
-        <v>2.025059475604219</v>
+        <v>2.061932682531472</v>
       </c>
       <c r="O101" t="n">
         <v>0.49</v>
@@ -24159,7 +24159,7 @@
         <v>42633867</v>
       </c>
       <c r="AN101" t="n">
-        <v>64932681.28231645</v>
+        <v>66115005.17063082</v>
       </c>
       <c r="AO101" t="n">
         <v>0</v>
@@ -24298,7 +24298,7 @@
         <v>24.8</v>
       </c>
       <c r="H102" t="n">
-        <v>627899028</v>
+        <v>639332100</v>
       </c>
       <c r="I102" t="n">
         <v>13900</v>
@@ -24316,7 +24316,7 @@
         <v>6.32</v>
       </c>
       <c r="N102" t="n">
-        <v>1.452875322093296</v>
+        <v>1.479329938876866</v>
       </c>
       <c r="O102" t="n">
         <v>0.49</v>
@@ -24394,7 +24394,7 @@
         <v>59424311.94</v>
       </c>
       <c r="AN102" t="n">
-        <v>64532274.20349435</v>
+        <v>65707307.29701953</v>
       </c>
       <c r="AO102" t="n">
         <v>0</v>
@@ -25003,7 +25003,7 @@
         <v>15.5</v>
       </c>
       <c r="H105" t="n">
-        <v>35419910600</v>
+        <v>7062081279</v>
       </c>
       <c r="I105" t="n">
         <v>62400</v>
@@ -25021,7 +25021,7 @@
         <v>10.61</v>
       </c>
       <c r="N105" t="n">
-        <v>2.50459875228973</v>
+        <v>0.4993711068246475</v>
       </c>
       <c r="O105" t="n">
         <v>0.66</v>
@@ -25099,7 +25099,7 @@
         <v>1339242675.4</v>
       </c>
       <c r="AN105" t="n">
-        <v>4799445880.758807</v>
+        <v>956921582.5203252</v>
       </c>
       <c r="AO105" t="n">
         <v>0.2241</v>
@@ -25238,7 +25238,7 @@
         <v>10.86</v>
       </c>
       <c r="H106" t="n">
-        <v>35419910600</v>
+        <v>7062081279</v>
       </c>
       <c r="I106" t="n">
         <v>14788500</v>
@@ -25256,7 +25256,7 @@
         <v>8.08</v>
       </c>
       <c r="N106" t="n">
-        <v>1.257573548352255</v>
+        <v>0.2507371267273628</v>
       </c>
       <c r="O106" t="n">
         <v>0.5</v>
@@ -25334,7 +25334,7 @@
         <v>2667251977.6</v>
       </c>
       <c r="AN106" t="n">
-        <v>6302475195.729537</v>
+        <v>1256598092.348754</v>
       </c>
       <c r="AO106" t="n">
         <v>0.423</v>
@@ -27588,7 +27588,7 @@
         <v>3.58</v>
       </c>
       <c r="H116" t="n">
-        <v>14200316717</v>
+        <v>2856852129</v>
       </c>
       <c r="I116" t="n">
         <v>66785000</v>
@@ -27606,7 +27606,7 @@
         <v>1.73</v>
       </c>
       <c r="N116" t="n">
-        <v>0.3337031336458342</v>
+        <v>0.06713515809607086</v>
       </c>
       <c r="O116" t="n">
         <v>0.18</v>
@@ -27684,7 +27684,7 @@
         <v>13208681203.56</v>
       </c>
       <c r="AN116" t="n">
-        <v>1039554664.494876</v>
+        <v>209139980.1610542</v>
       </c>
       <c r="AO116" t="n">
         <v>0</v>
@@ -28293,7 +28293,7 @@
         <v>6.68</v>
       </c>
       <c r="H119" t="n">
-        <v>8822168893</v>
+        <v>1756205035</v>
       </c>
       <c r="I119" t="n">
         <v>25347200</v>
@@ -28311,7 +28311,7 @@
         <v>8.109999999999999</v>
       </c>
       <c r="N119" t="n">
-        <v>0.1944649424043814</v>
+        <v>0.03871160426916571</v>
       </c>
       <c r="O119" t="n">
         <v>0.13</v>
@@ -28389,7 +28389,7 @@
         <v>1551529917.99</v>
       </c>
       <c r="AN119" t="n">
-        <v>3886418014.537445</v>
+        <v>773658605.7268722</v>
       </c>
       <c r="AO119" t="n">
         <v>0</v>
@@ -28763,7 +28763,7 @@
         <v>0.52</v>
       </c>
       <c r="H121" t="n">
-        <v>13832727</v>
+        <v>14053100</v>
       </c>
       <c r="I121" t="n">
         <v>100</v>
@@ -28781,7 +28781,7 @@
         <v>0.19</v>
       </c>
       <c r="N121" t="n">
-        <v>0.03194122013692655</v>
+        <v>0.03245008454994033</v>
       </c>
       <c r="O121" t="n">
         <v>0.02</v>
@@ -28859,7 +28859,7 @@
         <v>129011019.48</v>
       </c>
       <c r="AN121" t="n">
-        <v>4626330.100334448</v>
+        <v>4700033.444816053</v>
       </c>
       <c r="AO121" t="n">
         <v>0</v>
@@ -32288,7 +32288,7 @@
         <v>6.51</v>
       </c>
       <c r="H136" t="n">
-        <v>431284400</v>
+        <v>436226700</v>
       </c>
       <c r="I136" t="n">
         <v>0</v>
@@ -32306,7 +32306,7 @@
         <v>89.8</v>
       </c>
       <c r="N136" t="n">
-        <v>1.006736286804628</v>
+        <v>1.01827297292236</v>
       </c>
       <c r="O136" t="n">
         <v>0.49</v>
@@ -32384,7 +32384,7 @@
         <v>3812747.4</v>
       </c>
       <c r="AN136" t="n">
-        <v>7291367.709213863</v>
+        <v>7374923.076923077</v>
       </c>
       <c r="AO136" t="n">
         <v>0</v>
@@ -32523,7 +32523,7 @@
         <v>3.7</v>
       </c>
       <c r="H137" t="n">
-        <v>431284400</v>
+        <v>436226700</v>
       </c>
       <c r="I137" t="n">
         <v>2200</v>
@@ -32541,7 +32541,7 @@
         <v>51.86</v>
       </c>
       <c r="N137" t="n">
-        <v>2.589296256995011</v>
+        <v>2.618968275948042</v>
       </c>
       <c r="O137" t="n">
         <v>0.29</v>
@@ -32619,7 +32619,7 @@
         <v>1482422.55</v>
       </c>
       <c r="AN137" t="n">
-        <v>12621726.66081358</v>
+        <v>12766365.23266023</v>
       </c>
       <c r="AO137" t="n">
         <v>0</v>
@@ -32993,7 +32993,7 @@
         <v>2.5</v>
       </c>
       <c r="H139" t="n">
-        <v>26592280</v>
+        <v>27015920</v>
       </c>
       <c r="I139" t="n">
         <v>0</v>
@@ -33011,7 +33011,7 @@
         <v>186.65</v>
       </c>
       <c r="N139" t="n">
-        <v>4.929809720091126</v>
+        <v>5.008346219775222</v>
       </c>
       <c r="O139" t="n">
         <v>4.19</v>
@@ -33089,7 +33089,7 @@
         <v>106804.76</v>
       </c>
       <c r="AN139" t="n">
-        <v>107722.1096978044</v>
+        <v>109438.2240946285</v>
       </c>
       <c r="AO139" t="n">
         <v>0</v>
@@ -34403,7 +34403,7 @@
         <v>51.52</v>
       </c>
       <c r="H145" t="n">
-        <v>8508092000</v>
+        <v>8643633000</v>
       </c>
       <c r="I145" t="n">
         <v>0</v>
@@ -34421,7 +34421,7 @@
         <v>10.18</v>
       </c>
       <c r="N145" t="n">
-        <v>1.838477248404962</v>
+        <v>1.867765723979281</v>
       </c>
       <c r="O145" t="n">
         <v>0.73</v>
@@ -34499,7 +34499,7 @@
         <v>441028665.6</v>
       </c>
       <c r="AN145" t="n">
-        <v>1955883218.390805</v>
+        <v>1987042068.965518</v>
       </c>
       <c r="AO145" t="n">
         <v>0</v>
@@ -34638,7 +34638,7 @@
         <v>37.39</v>
       </c>
       <c r="H146" t="n">
-        <v>8508092000</v>
+        <v>8643633000</v>
       </c>
       <c r="I146" t="n">
         <v>0</v>
@@ -34656,7 +34656,7 @@
         <v>8.16</v>
       </c>
       <c r="N146" t="n">
-        <v>1.658067401888382</v>
+        <v>1.684481798173631</v>
       </c>
       <c r="O146" t="n">
         <v>0.58</v>
@@ -34734,7 +34734,7 @@
         <v>489015806.4</v>
       </c>
       <c r="AN146" t="n">
-        <v>2437848710.601719</v>
+        <v>2476685673.352436</v>
       </c>
       <c r="AO146" t="n">
         <v>0</v>
@@ -37223,7 +37223,7 @@
         <v>5.93</v>
       </c>
       <c r="H157" t="n">
-        <v>54171330</v>
+        <v>55034330</v>
       </c>
       <c r="I157" t="n">
         <v>5000</v>
@@ -37241,7 +37241,7 @@
         <v>8.27</v>
       </c>
       <c r="N157" t="n">
-        <v>0.00453757852061481</v>
+        <v>0.004609866394353382</v>
       </c>
       <c r="O157" t="n">
         <v>0.62</v>
@@ -37319,7 +37319,7 @@
         <v>1653465426.75</v>
       </c>
       <c r="AN157" t="n">
-        <v>9058750.836120401</v>
+        <v>9203065.217391303</v>
       </c>
       <c r="AO157" t="n">
         <v>0</v>
@@ -37458,7 +37458,7 @@
         <v>16.4</v>
       </c>
       <c r="H158" t="n">
-        <v>54171330</v>
+        <v>55034330</v>
       </c>
       <c r="I158" t="n">
         <v>0</v>
@@ -37476,7 +37476,7 @@
         <v>14.74</v>
       </c>
       <c r="N158" t="n">
-        <v>4.616745925819266</v>
+        <v>4.690295010436204</v>
       </c>
       <c r="O158" t="n">
         <v>1.1</v>
@@ -37554,7 +37554,7 @@
         <v>1625112</v>
       </c>
       <c r="AN158" t="n">
-        <v>5086509.859154929</v>
+        <v>5167542.723004695</v>
       </c>
       <c r="AO158" t="n">
         <v>0</v>
@@ -37693,7 +37693,7 @@
         <v>6.59</v>
       </c>
       <c r="H159" t="n">
-        <v>54171330</v>
+        <v>55034330</v>
       </c>
       <c r="I159" t="n">
         <v>0</v>
@@ -37711,7 +37711,7 @@
         <v>8.83</v>
       </c>
       <c r="N159" t="n">
-        <v>9.216775191570086</v>
+        <v>9.363607048759579</v>
       </c>
       <c r="O159" t="n">
         <v>0.66</v>
@@ -37789,7 +37789,7 @@
         <v>814029.75</v>
       </c>
       <c r="AN159" t="n">
-        <v>8490804.07523511</v>
+        <v>8626070.532915361</v>
       </c>
       <c r="AO159" t="n">
         <v>0</v>
@@ -37928,7 +37928,7 @@
         <v>10</v>
       </c>
       <c r="H160" t="n">
-        <v>54171330</v>
+        <v>55034330</v>
       </c>
       <c r="I160" t="n">
         <v>0</v>
@@ -37946,7 +37946,7 @@
         <v>13.4</v>
       </c>
       <c r="N160" t="n">
-        <v>8.327698037625836</v>
+        <v>8.460366063433419</v>
       </c>
       <c r="O160" t="n">
         <v>1</v>
@@ -38024,7 +38024,7 @@
         <v>900936.75</v>
       </c>
       <c r="AN160" t="n">
-        <v>5596211.776859504</v>
+        <v>5685364.669421487</v>
       </c>
       <c r="AO160" t="n">
         <v>0</v>
@@ -38633,7 +38633,7 @@
         <v>3.01</v>
       </c>
       <c r="H163" t="n">
-        <v>29633360</v>
+        <v>30016120</v>
       </c>
       <c r="I163" t="n">
         <v>0</v>
@@ -38651,7 +38651,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="N163" t="n">
-        <v>0.5522843211827023</v>
+        <v>0.5594179147669563</v>
       </c>
       <c r="O163" t="n">
         <v>0.07000000000000001</v>
@@ -38729,7 +38729,7 @@
         <v>8649345</v>
       </c>
       <c r="AN163" t="n">
-        <v>7408340</v>
+        <v>7504030</v>
       </c>
       <c r="AO163" t="n">
         <v>0</v>
@@ -38868,7 +38868,7 @@
         <v>4</v>
       </c>
       <c r="H164" t="n">
-        <v>29633360</v>
+        <v>30016120</v>
       </c>
       <c r="I164" t="n">
         <v>3300</v>
@@ -38886,7 +38886,7 @@
         <v>1.51</v>
       </c>
       <c r="N164" t="n">
-        <v>0.02761421605913512</v>
+        <v>0.02797089573834782</v>
       </c>
       <c r="O164" t="n">
         <v>0.11</v>
@@ -38964,7 +38964,7 @@
         <v>172986900</v>
       </c>
       <c r="AN164" t="n">
-        <v>4615788.16199377</v>
+        <v>4675408.099688473</v>
       </c>
       <c r="AO164" t="n">
         <v>0</v>
@@ -40748,7 +40748,7 @@
         <v>3.96</v>
       </c>
       <c r="H172" t="n">
-        <v>212404898</v>
+        <v>215788700</v>
       </c>
       <c r="I172" t="n">
         <v>2700</v>
@@ -40766,7 +40766,7 @@
         <v>0.38</v>
       </c>
       <c r="N172" t="n">
-        <v>0.04702789208636675</v>
+        <v>0.047777088911845</v>
       </c>
       <c r="O172" t="n">
         <v>0.08</v>
@@ -40844,7 +40844,7 @@
         <v>640901679.6</v>
       </c>
       <c r="AN172" t="n">
-        <v>212404898</v>
+        <v>215788700</v>
       </c>
       <c r="AO172" t="n">
         <v>0</v>
@@ -42158,7 +42158,7 @@
         <v>205</v>
       </c>
       <c r="H178" t="n">
-        <v>1303051000</v>
+        <v>1323809000</v>
       </c>
       <c r="I178" t="n">
         <v>0</v>
@@ -42176,7 +42176,7 @@
         <v>52.85</v>
       </c>
       <c r="N178" t="n">
-        <v>0.5293138231054622</v>
+        <v>0.5377459538048923</v>
       </c>
       <c r="O178" t="n">
         <v>0.67</v>
@@ -42254,7 +42254,7 @@
         <v>24125385.06</v>
       </c>
       <c r="AN178" t="n">
-        <v>195653303.3033033</v>
+        <v>198770120.1201201</v>
       </c>
       <c r="AO178" t="n">
         <v>0</v>
@@ -42628,7 +42628,7 @@
         <v>36</v>
       </c>
       <c r="H180" t="n">
-        <v>3534561000</v>
+        <v>3586174000</v>
       </c>
       <c r="I180" t="n">
         <v>0</v>
@@ -42646,7 +42646,7 @@
         <v>12.71</v>
       </c>
       <c r="N180" t="n">
-        <v>8.635248607051759</v>
+        <v>8.76134378163094</v>
       </c>
       <c r="O180" t="n">
         <v>0.8</v>
@@ -42724,7 +42724,7 @@
         <v>84360399.48</v>
       </c>
       <c r="AN180" t="n">
-        <v>458438521.4007782</v>
+        <v>465132814.5265889</v>
       </c>
       <c r="AO180" t="n">
         <v>4.0605</v>
@@ -42863,7 +42863,7 @@
         <v>38.3</v>
       </c>
       <c r="H181" t="n">
-        <v>3534561000</v>
+        <v>3586174000</v>
       </c>
       <c r="I181" t="n">
         <v>0</v>
@@ -42881,7 +42881,7 @@
         <v>13.08</v>
       </c>
       <c r="N181" t="n">
-        <v>4.317624303525879</v>
+        <v>4.38067189081547</v>
       </c>
       <c r="O181" t="n">
         <v>0.83</v>
@@ -42959,7 +42959,7 @@
         <v>168720798.96</v>
       </c>
       <c r="AN181" t="n">
-        <v>445158816.1209068</v>
+        <v>451659193.9546599</v>
       </c>
       <c r="AO181" t="n">
         <v>4.0605</v>
@@ -43333,7 +43333,7 @@
         <v>20.64</v>
       </c>
       <c r="H183" t="n">
-        <v>45304362984</v>
+        <v>8993443632</v>
       </c>
       <c r="I183" t="n">
         <v>47700</v>
@@ -43351,7 +43351,7 @@
         <v>12.45</v>
       </c>
       <c r="N183" t="n">
-        <v>1.815192998321849</v>
+        <v>0.3603369485048055</v>
       </c>
       <c r="O183" t="n">
         <v>0.43</v>
@@ -43429,7 +43429,7 @@
         <v>1075708228.5</v>
       </c>
       <c r="AN183" t="n">
-        <v>6701828843.786983</v>
+        <v>1330391069.822485</v>
       </c>
       <c r="AO183" t="n">
         <v>0</v>
@@ -43568,7 +43568,7 @@
         <v>24.13</v>
       </c>
       <c r="H184" t="n">
-        <v>45304362984</v>
+        <v>8993443632</v>
       </c>
       <c r="I184" t="n">
         <v>13017800</v>
@@ -43586,7 +43586,7 @@
         <v>14.65</v>
       </c>
       <c r="N184" t="n">
-        <v>1.02659903163437</v>
+        <v>0.2037918627601091</v>
       </c>
       <c r="O184" t="n">
         <v>0.5</v>
@@ -43664,7 +43664,7 @@
         <v>1902025995</v>
       </c>
       <c r="AN184" t="n">
-        <v>5691502887.437186</v>
+        <v>1129829602.01005</v>
       </c>
       <c r="AO184" t="n">
         <v>0</v>
@@ -44743,7 +44743,7 @@
         <v>10</v>
       </c>
       <c r="H189" t="n">
-        <v>796765000</v>
+        <v>806156500</v>
       </c>
       <c r="I189" t="n">
         <v>0</v>
@@ -44761,7 +44761,7 @@
         <v>46.67</v>
       </c>
       <c r="N189" t="n">
-        <v>22.78648591451142</v>
+        <v>23.05507110897419</v>
       </c>
       <c r="O189" t="n">
         <v>1.77</v>
@@ -44839,7 +44839,7 @@
         <v>29480305.74</v>
       </c>
       <c r="AN189" t="n">
-        <v>63741200</v>
+        <v>64492520</v>
       </c>
       <c r="AO189" t="n">
         <v>0</v>
@@ -45213,7 +45213,7 @@
         <v>2.81</v>
       </c>
       <c r="H191" t="n">
-        <v>5397730</v>
+        <v>5483720</v>
       </c>
       <c r="I191" t="n">
         <v>0</v>
@@ -45231,7 +45231,7 @@
         <v>0.02</v>
       </c>
       <c r="N191" t="n">
-        <v>0.02848956560071868</v>
+        <v>0.02894342634329117</v>
       </c>
       <c r="O191" t="n">
         <v>0.01</v>
@@ -45309,7 +45309,7 @@
         <v>256931318.49</v>
       </c>
       <c r="AN191" t="n">
-        <v>89962166.66666667</v>
+        <v>91395333.33333334</v>
       </c>
       <c r="AO191" t="n">
         <v>0</v>
@@ -46858,7 +46858,7 @@
         <v>30</v>
       </c>
       <c r="H198" t="n">
-        <v>273278700</v>
+        <v>277240400</v>
       </c>
       <c r="I198" t="n">
         <v>0</v>
@@ -46876,7 +46876,7 @@
         <v>8.289999999999999</v>
       </c>
       <c r="N198" t="n">
-        <v>6.037400487786134</v>
+        <v>6.124924211780951</v>
       </c>
       <c r="O198" t="n">
         <v>0.2</v>
@@ -46954,7 +46954,7 @@
         <v>26538458.42</v>
       </c>
       <c r="AN198" t="n">
-        <v>13428928.74692875</v>
+        <v>13623606.87960688</v>
       </c>
       <c r="AO198" t="n">
         <v>0</v>
@@ -47093,7 +47093,7 @@
         <v>96</v>
       </c>
       <c r="H199" t="n">
-        <v>1656730</v>
+        <v>1683120</v>
       </c>
       <c r="I199" t="n">
         <v>0</v>
@@ -47111,7 +47111,7 @@
         <v>44.39</v>
       </c>
       <c r="N199" t="n">
-        <v>1.07122049874674</v>
+        <v>1.08828393633882</v>
       </c>
       <c r="O199" t="n">
         <v>3.9</v>
@@ -47189,7 +47189,7 @@
         <v>369787.6800000001</v>
       </c>
       <c r="AN199" t="n">
-        <v>136581.2036273702</v>
+        <v>138756.8013190437</v>
       </c>
       <c r="AO199" t="n">
         <v>0</v>
@@ -47328,7 +47328,7 @@
         <v>4.91</v>
       </c>
       <c r="H200" t="n">
-        <v>1656730</v>
+        <v>1683120</v>
       </c>
       <c r="I200" t="n">
         <v>0</v>
@@ -47346,7 +47346,7 @@
         <v>2.31</v>
       </c>
       <c r="N200" t="n">
-        <v>0.5412935822044339</v>
+        <v>0.5499158306301732</v>
       </c>
       <c r="O200" t="n">
         <v>0.2</v>
@@ -47424,7 +47424,7 @@
         <v>731810.16</v>
       </c>
       <c r="AN200" t="n">
-        <v>2629730.158730159</v>
+        <v>2671619.047619048</v>
       </c>
       <c r="AO200" t="n">
         <v>0</v>
@@ -48006,7 +48006,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>IBOVESPA</t>
+          <t>Brazil Stock Exchange Index</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
@@ -51072,7 +51072,7 @@
         <v>39.9</v>
       </c>
       <c r="H216" t="n">
-        <v>429249159132</v>
+        <v>87193179276</v>
       </c>
       <c r="I216" t="n">
         <v>4269800</v>
@@ -51090,7 +51090,7 @@
         <v>10.94</v>
       </c>
       <c r="N216" t="n">
-        <v>2.167182431367668</v>
+        <v>0.4402187453183333</v>
       </c>
       <c r="O216" t="n">
         <v>0.16</v>
@@ -51168,7 +51168,7 @@
         <v>22302439618.69</v>
       </c>
       <c r="AN216" t="n">
-        <v>44206916491.45211</v>
+        <v>8979730100.514933</v>
       </c>
       <c r="AO216" t="n">
         <v>0.4601</v>
@@ -51307,7 +51307,7 @@
         <v>38.72</v>
       </c>
       <c r="H217" t="n">
-        <v>429249159132</v>
+        <v>87193179276</v>
       </c>
       <c r="I217" t="n">
         <v>40844400</v>
@@ -51325,7 +51325,7 @@
         <v>11.77</v>
       </c>
       <c r="N217" t="n">
-        <v>2.250765354657841</v>
+        <v>0.4571969051115621</v>
       </c>
       <c r="O217" t="n">
         <v>0.17</v>
@@ -51403,7 +51403,7 @@
         <v>21474231073.55</v>
       </c>
       <c r="AN217" t="n">
-        <v>41076474558.08613</v>
+        <v>8343844906.794259</v>
       </c>
       <c r="AO217" t="n">
         <v>0.4601</v>
@@ -53187,7 +53187,7 @@
         <v>16.76</v>
       </c>
       <c r="H225" t="n">
-        <v>20946447253</v>
+        <v>4152070426</v>
       </c>
       <c r="I225" t="n">
         <v>5072400</v>
@@ -53277,13 +53277,13 @@
         <v>22.3</v>
       </c>
       <c r="AL225" t="n">
-        <v>100263012483.5459</v>
+        <v>19874448584.35249</v>
       </c>
       <c r="AM225" t="n">
-        <v>8913381809.787233</v>
+        <v>1766838479.148936</v>
       </c>
       <c r="AN225" t="n">
-        <v>4214576912.072435</v>
+        <v>835426645.0704225</v>
       </c>
       <c r="AO225" t="n">
         <v>0.9119</v>
@@ -53422,7 +53422,7 @@
         <v>3.37</v>
       </c>
       <c r="H226" t="n">
-        <v>20946447253</v>
+        <v>4152070426</v>
       </c>
       <c r="I226" t="n">
         <v>989400</v>
@@ -53440,7 +53440,7 @@
         <v>13.06</v>
       </c>
       <c r="N226" t="n">
-        <v>2.683815841085569</v>
+        <v>0.5319943877836241</v>
       </c>
       <c r="O226" t="n">
         <v>0.39</v>
@@ -53518,7 +53518,7 @@
         <v>693840140.6999999</v>
       </c>
       <c r="AN226" t="n">
-        <v>4206113906.224899</v>
+        <v>833749081.5261043</v>
       </c>
       <c r="AO226" t="n">
         <v>0.1824</v>
@@ -53657,7 +53657,7 @@
         <v>3.35</v>
       </c>
       <c r="H227" t="n">
-        <v>20946447253</v>
+        <v>4152070426</v>
       </c>
       <c r="I227" t="n">
         <v>6230100</v>
@@ -53675,7 +53675,7 @@
         <v>13.06</v>
       </c>
       <c r="N227" t="n">
-        <v>1.579953850636249</v>
+        <v>0.3131834042516227</v>
       </c>
       <c r="O227" t="n">
         <v>0.39</v>
@@ -53753,7 +53753,7 @@
         <v>1178603514.3</v>
       </c>
       <c r="AN227" t="n">
-        <v>4206113906.224899</v>
+        <v>833749081.5261043</v>
       </c>
       <c r="AO227" t="n">
         <v>0.1824</v>
@@ -56242,7 +56242,7 @@
         <v>3.25</v>
       </c>
       <c r="H238" t="n">
-        <v>134852315</v>
+        <v>136688400</v>
       </c>
       <c r="I238" t="n">
         <v>6100</v>
@@ -56260,7 +56260,7 @@
         <v>4.2</v>
       </c>
       <c r="N238" t="n">
-        <v>1.574556662806246</v>
+        <v>1.595995077639752</v>
       </c>
       <c r="O238" t="n">
         <v>0.75</v>
@@ -56338,7 +56338,7 @@
         <v>23184000</v>
       </c>
       <c r="AN238" t="n">
-        <v>19487328.75722544</v>
+        <v>19752658.95953757</v>
       </c>
       <c r="AO238" t="n">
         <v>0</v>
@@ -56712,7 +56712,7 @@
         <v>2.5</v>
       </c>
       <c r="H240" t="n">
-        <v>2519140</v>
+        <v>2559270</v>
       </c>
       <c r="I240" t="n">
         <v>0</v>
@@ -56808,7 +56808,7 @@
         <v>54534.6</v>
       </c>
       <c r="AN240" t="n">
-        <v>96852.74894271433</v>
+        <v>98395.61707035755</v>
       </c>
       <c r="AO240" t="n">
         <v>0</v>
@@ -56947,7 +56947,7 @@
         <v>3</v>
       </c>
       <c r="H241" t="n">
-        <v>2519140</v>
+        <v>2559270</v>
       </c>
       <c r="I241" t="n">
         <v>0</v>
@@ -57043,7 +57043,7 @@
         <v>55732.8</v>
       </c>
       <c r="AN241" t="n">
-        <v>75086.14008941878</v>
+        <v>76282.2652757079</v>
       </c>
       <c r="AO241" t="n">
         <v>0</v>
@@ -58357,7 +58357,7 @@
         <v>5.23</v>
       </c>
       <c r="H247" t="n">
-        <v>19434517</v>
+        <v>19663590</v>
       </c>
       <c r="I247" t="n">
         <v>2100</v>
@@ -58375,7 +58375,7 @@
         <v>4.4</v>
       </c>
       <c r="N247" t="n">
-        <v>0.02924670921706602</v>
+        <v>0.02959143769271998</v>
       </c>
       <c r="O247" t="n">
         <v>0.05</v>
@@ -58453,7 +58453,7 @@
         <v>5648272.88</v>
       </c>
       <c r="AN247" t="n">
-        <v>32939859.3220339</v>
+        <v>33328118.6440678</v>
       </c>
       <c r="AO247" t="n">
         <v>0</v>
@@ -59767,7 +59767,7 @@
         <v>18.47</v>
       </c>
       <c r="H253" t="n">
-        <v>182494158</v>
+        <v>185401500</v>
       </c>
       <c r="I253" t="n">
         <v>1800</v>
@@ -59785,7 +59785,7 @@
         <v>7.29</v>
       </c>
       <c r="N253" t="n">
-        <v>0.1824510995405084</v>
+        <v>0.1853577555696856</v>
       </c>
       <c r="O253" t="n">
         <v>0.12</v>
@@ -59863,7 +59863,7 @@
         <v>24405758.4</v>
       </c>
       <c r="AN253" t="n">
-        <v>125858040</v>
+        <v>127863103.4482759</v>
       </c>
       <c r="AO253" t="n">
         <v>0</v>
@@ -60002,7 +60002,7 @@
         <v>4.02</v>
       </c>
       <c r="H254" t="n">
-        <v>284259826</v>
+        <v>288788300</v>
       </c>
       <c r="I254" t="n">
         <v>4900</v>
@@ -60020,7 +60020,7 @@
         <v>0.59</v>
       </c>
       <c r="N254" t="n">
-        <v>0.664718282683527</v>
+        <v>0.6753077476206405</v>
       </c>
       <c r="O254" t="n">
         <v>0.6899999999999999</v>
@@ -60098,7 +60098,7 @@
         <v>520437330</v>
       </c>
       <c r="AN254" t="n">
-        <v>181057214.0127389</v>
+        <v>183941592.3566879</v>
       </c>
       <c r="AO254" t="n">
         <v>0</v>
@@ -61647,7 +61647,7 @@
         <v>47</v>
       </c>
       <c r="H261" t="n">
-        <v>296262200</v>
+        <v>299885200</v>
       </c>
       <c r="I261" t="n">
         <v>0</v>
@@ -61665,7 +61665,7 @@
         <v>22.68</v>
       </c>
       <c r="N261" t="n">
-        <v>1.890858310737324</v>
+        <v>1.913981678010642</v>
       </c>
       <c r="O261" t="n">
         <v>0.21</v>
@@ -61743,7 +61743,7 @@
         <v>11657091.15</v>
       </c>
       <c r="AN261" t="n">
-        <v>19175546.92556635</v>
+        <v>19410045.30744337</v>
       </c>
       <c r="AO261" t="n">
         <v>0</v>
@@ -61882,7 +61882,7 @@
         <v>41</v>
       </c>
       <c r="H262" t="n">
-        <v>296262200</v>
+        <v>299885200</v>
       </c>
       <c r="I262" t="n">
         <v>0</v>
@@ -61900,7 +61900,7 @@
         <v>19.78</v>
       </c>
       <c r="N262" t="n">
-        <v>13.76626957289186</v>
+        <v>13.93461772754199</v>
       </c>
       <c r="O262" t="n">
         <v>0.18</v>
@@ -61978,7 +61978,7 @@
         <v>1601153.28</v>
       </c>
       <c r="AN262" t="n">
-        <v>21977908.01186943</v>
+        <v>22246676.5578635</v>
       </c>
       <c r="AO262" t="n">
         <v>0</v>
@@ -62352,7 +62352,7 @@
         <v>76</v>
       </c>
       <c r="H264" t="n">
-        <v>409408700</v>
+        <v>415930900</v>
       </c>
       <c r="I264" t="n">
         <v>0</v>
@@ -62370,7 +62370,7 @@
         <v>16.17</v>
       </c>
       <c r="N264" t="n">
-        <v>1.569164686014143</v>
+        <v>1.594162703679917</v>
       </c>
       <c r="O264" t="n">
         <v>1.16</v>
@@ -62448,7 +62448,7 @@
         <v>19672515.1</v>
       </c>
       <c r="AN264" t="n">
-        <v>24413160.40548599</v>
+        <v>24802081.09719738</v>
       </c>
       <c r="AO264" t="n">
         <v>1.1</v>
@@ -62587,7 +62587,7 @@
         <v>44.99</v>
       </c>
       <c r="H265" t="n">
-        <v>409408700</v>
+        <v>415930900</v>
       </c>
       <c r="I265" t="n">
         <v>1200</v>
@@ -62605,7 +62605,7 @@
         <v>11.14</v>
       </c>
       <c r="N265" t="n">
-        <v>1.444147801008293</v>
+        <v>1.467154202161313</v>
       </c>
       <c r="O265" t="n">
         <v>0.8</v>
@@ -62683,7 +62683,7 @@
         <v>21375524</v>
       </c>
       <c r="AN265" t="n">
-        <v>35446640.69264069</v>
+        <v>36011333.33333333</v>
       </c>
       <c r="AO265" t="n">
         <v>1.21</v>
@@ -63057,7 +63057,7 @@
         <v>16</v>
       </c>
       <c r="H267" t="n">
-        <v>30060930</v>
+        <v>30410450</v>
       </c>
       <c r="I267" t="n">
         <v>0</v>
@@ -63075,7 +63075,7 @@
         <v>4.28</v>
       </c>
       <c r="N267" t="n">
-        <v>0.4018835050730777</v>
+        <v>0.4065562255342591</v>
       </c>
       <c r="O267" t="n">
         <v>0.1</v>
@@ -63153,7 +63153,7 @@
         <v>2565643.74</v>
       </c>
       <c r="AN267" t="n">
-        <v>46970203.125</v>
+        <v>47516328.125</v>
       </c>
       <c r="AO267" t="n">
         <v>0</v>
@@ -63292,7 +63292,7 @@
         <v>14</v>
       </c>
       <c r="H268" t="n">
-        <v>30060930</v>
+        <v>30410450</v>
       </c>
       <c r="I268" t="n">
         <v>0</v>
@@ -63310,7 +63310,7 @@
         <v>2.74</v>
       </c>
       <c r="N268" t="n">
-        <v>0.2009417525365389</v>
+        <v>0.2032781127671296</v>
       </c>
       <c r="O268" t="n">
         <v>0.07000000000000001</v>
@@ -63388,7 +63388,7 @@
         <v>5131287.48</v>
       </c>
       <c r="AN268" t="n">
-        <v>73319341.46341464</v>
+        <v>74171829.26829268</v>
       </c>
       <c r="AO268" t="n">
         <v>0</v>
@@ -63762,7 +63762,7 @@
         <v>2.53</v>
       </c>
       <c r="H270" t="n">
-        <v>6691190</v>
+        <v>6797780</v>
       </c>
       <c r="I270" t="n">
         <v>0</v>
@@ -63780,7 +63780,7 @@
         <v>0.12</v>
       </c>
       <c r="N270" t="n">
-        <v>0.07663989259102685</v>
+        <v>0.07786075855825803</v>
       </c>
       <c r="O270" t="n">
         <v>0.29</v>
@@ -63858,7 +63858,7 @@
         <v>63122875.13</v>
       </c>
       <c r="AN270" t="n">
-        <v>95588428.57142857</v>
+        <v>97111142.85714285</v>
       </c>
       <c r="AO270" t="n">
         <v>0</v>
@@ -64232,7 +64232,7 @@
         <v>1.86</v>
       </c>
       <c r="H272" t="n">
-        <v>12315960</v>
+        <v>12461130</v>
       </c>
       <c r="I272" t="n">
         <v>0</v>
@@ -64250,7 +64250,7 @@
         <v>0.96</v>
       </c>
       <c r="N272" t="n">
-        <v>4.723684345049178</v>
+        <v>4.779363094929073</v>
       </c>
       <c r="O272" t="n">
         <v>1.87</v>
@@ -64328,7 +64328,7 @@
         <v>37941114.78</v>
       </c>
       <c r="AN272" t="n">
-        <v>10899079.6460177</v>
+        <v>11027548.67256637</v>
       </c>
       <c r="AO272" t="n">
         <v>0</v>
@@ -66582,7 +66582,7 @@
         <v>29.01</v>
       </c>
       <c r="H282" t="n">
-        <v>688155498</v>
+        <v>703592200</v>
       </c>
       <c r="I282" t="n">
         <v>200</v>
@@ -66600,7 +66600,7 @@
         <v>17.82</v>
       </c>
       <c r="N282" t="n">
-        <v>0.3507509187914097</v>
+        <v>0.3586189623155046</v>
       </c>
       <c r="O282" t="n">
         <v>0.52</v>
@@ -66678,7 +66678,7 @@
         <v>42378103.55</v>
       </c>
       <c r="AN282" t="n">
-        <v>76803068.97321428</v>
+        <v>78525915.17857142</v>
       </c>
       <c r="AO282" t="n">
         <v>0</v>
@@ -66817,7 +66817,7 @@
         <v>30.1</v>
       </c>
       <c r="H283" t="n">
-        <v>688155498</v>
+        <v>703592200</v>
       </c>
       <c r="I283" t="n">
         <v>0</v>
@@ -66835,7 +66835,7 @@
         <v>18.34</v>
       </c>
       <c r="N283" t="n">
-        <v>7.836526012333223</v>
+        <v>8.012314939573089</v>
       </c>
       <c r="O283" t="n">
         <v>0.54</v>
@@ -66913,7 +66913,7 @@
         <v>1896779.1</v>
       </c>
       <c r="AN283" t="n">
-        <v>74556391.98266523</v>
+        <v>76228840.73672806</v>
       </c>
       <c r="AO283" t="n">
         <v>0</v>
@@ -67287,7 +67287,7 @@
         <v>1.5</v>
       </c>
       <c r="H285" t="n">
-        <v>4911109</v>
+        <v>4989350</v>
       </c>
       <c r="I285" t="n">
         <v>8500</v>
@@ -67305,7 +67305,7 @@
         <v>0.05</v>
       </c>
       <c r="N285" t="n">
-        <v>0.04978316712652813</v>
+        <v>0.05057628427769433</v>
       </c>
       <c r="O285" t="n">
         <v>0.02</v>
@@ -67383,7 +67383,7 @@
         <v>178674864.1</v>
       </c>
       <c r="AN285" t="n">
-        <v>24555545</v>
+        <v>24946750</v>
       </c>
       <c r="AO285" t="n">
         <v>0</v>
@@ -67757,7 +67757,7 @@
         <v>40</v>
       </c>
       <c r="H287" t="n">
-        <v>714455400</v>
+        <v>724292900</v>
       </c>
       <c r="I287" t="n">
         <v>0</v>
@@ -67775,7 +67775,7 @@
         <v>21.05</v>
       </c>
       <c r="N287" t="n">
-        <v>12.05287107138443</v>
+        <v>12.2188298130564</v>
       </c>
       <c r="O287" t="n">
         <v>0.54</v>
@@ -67853,7 +67853,7 @@
         <v>16864244.22</v>
       </c>
       <c r="AN287" t="n">
-        <v>30044381.83347351</v>
+        <v>30458069.80656013</v>
       </c>
       <c r="AO287" t="n">
         <v>0.3943</v>
@@ -67992,7 +67992,7 @@
         <v>38.9</v>
       </c>
       <c r="H288" t="n">
-        <v>714455400</v>
+        <v>724292900</v>
       </c>
       <c r="I288" t="n">
         <v>0</v>
@@ -68010,7 +68010,7 @@
         <v>21.15</v>
       </c>
       <c r="N288" t="n">
-        <v>12.72992788976894</v>
+        <v>12.90520918180705</v>
       </c>
       <c r="O288" t="n">
         <v>0.54</v>
@@ -68088,7 +68088,7 @@
         <v>15967298.72</v>
       </c>
       <c r="AN288" t="n">
-        <v>29893531.38075314</v>
+        <v>30305142.25941423</v>
       </c>
       <c r="AO288" t="n">
         <v>0.4337</v>
@@ -68227,7 +68227,7 @@
         <v>45.95</v>
       </c>
       <c r="H289" t="n">
-        <v>567846262500</v>
+        <v>112394149176</v>
       </c>
       <c r="I289" t="n">
         <v>10466400</v>
@@ -68245,7 +68245,7 @@
         <v>6.46</v>
       </c>
       <c r="N289" t="n">
-        <v>2.002095662258903</v>
+        <v>0.3962759876905058</v>
       </c>
       <c r="O289" t="n">
         <v>0.41</v>
@@ -68323,7 +68323,7 @@
         <v>44727810605.82</v>
       </c>
       <c r="AN289" t="n">
-        <v>147876630859.375</v>
+        <v>29269309681.25</v>
       </c>
       <c r="AO289" t="n">
         <v>0.9432</v>
@@ -68462,7 +68462,7 @@
         <v>41.25</v>
       </c>
       <c r="H290" t="n">
-        <v>567846262500</v>
+        <v>112394149176</v>
       </c>
       <c r="I290" t="n">
         <v>42895100</v>
@@ -68480,7 +68480,7 @@
         <v>6.09</v>
       </c>
       <c r="N290" t="n">
-        <v>2.735711997591562</v>
+        <v>0.5414811061821139</v>
       </c>
       <c r="O290" t="n">
         <v>0.39</v>
@@ -68558,7 +68558,7 @@
         <v>32733473287.79</v>
       </c>
       <c r="AN290" t="n">
-        <v>156863608425.4144</v>
+        <v>31048107507.18232</v>
       </c>
       <c r="AO290" t="n">
         <v>0.9432</v>
@@ -69637,7 +69637,7 @@
         <v>2.93</v>
       </c>
       <c r="H295" t="n">
-        <v>36257980</v>
+        <v>36835600</v>
       </c>
       <c r="I295" t="n">
         <v>0</v>
@@ -69655,7 +69655,7 @@
         <v>0.32</v>
       </c>
       <c r="N295" t="n">
-        <v>0.03101328135062323</v>
+        <v>0.03150734890688938</v>
       </c>
       <c r="O295" t="n">
         <v>0.09</v>
@@ -69733,7 +69733,7 @@
         <v>176068173.06</v>
       </c>
       <c r="AN295" t="n">
-        <v>15764339.13043478</v>
+        <v>16015478.26086957</v>
       </c>
       <c r="AO295" t="n">
         <v>0</v>
@@ -71282,7 +71282,7 @@
         <v>0.47</v>
       </c>
       <c r="H302" t="n">
-        <v>439169</v>
+        <v>65875496</v>
       </c>
       <c r="I302" t="n">
         <v>15</v>
@@ -71375,10 +71375,10 @@
         <v>0</v>
       </c>
       <c r="AM302" t="n">
-        <v>2889.459832883742</v>
+        <v>433419.9355220738</v>
       </c>
       <c r="AN302" t="n">
-        <v>1756676</v>
+        <v>263501984</v>
       </c>
       <c r="AO302" t="n">
         <v>0</v>
@@ -72457,7 +72457,7 @@
         <v>8.42</v>
       </c>
       <c r="H307" t="n">
-        <v>405453200</v>
+        <v>411912400</v>
       </c>
       <c r="I307" t="n">
         <v>0</v>
@@ -72475,7 +72475,7 @@
         <v>9.75</v>
       </c>
       <c r="N307" t="n">
-        <v>1.459973062330529</v>
+        <v>1.483231623378279</v>
       </c>
       <c r="O307" t="n">
         <v>0.39</v>
@@ -72553,7 +72553,7 @@
         <v>13774554.64</v>
       </c>
       <c r="AN307" t="n">
-        <v>40383784.86055777</v>
+        <v>41027131.47410359</v>
       </c>
       <c r="AO307" t="n">
         <v>0</v>
@@ -72692,7 +72692,7 @@
         <v>8.5</v>
       </c>
       <c r="H308" t="n">
-        <v>405453200</v>
+        <v>411912400</v>
       </c>
       <c r="I308" t="n">
         <v>0</v>
@@ -72710,7 +72710,7 @@
         <v>9.6</v>
       </c>
       <c r="N308" t="n">
-        <v>0.7300841679079787</v>
+        <v>0.741715003864758</v>
       </c>
       <c r="O308" t="n">
         <v>0.39</v>
@@ -72788,7 +72788,7 @@
         <v>27545425.04</v>
       </c>
       <c r="AN308" t="n">
-        <v>41037773.27935223</v>
+        <v>41691538.46153846</v>
       </c>
       <c r="AO308" t="n">
         <v>0</v>
@@ -75512,7 +75512,7 @@
         <v>5.91</v>
       </c>
       <c r="H320" t="n">
-        <v>15116180000</v>
+        <v>15356990000</v>
       </c>
       <c r="I320" t="n">
         <v>0</v>
@@ -75530,7 +75530,7 @@
         <v>11.35</v>
       </c>
       <c r="N320" t="n">
-        <v>0.7790784402358714</v>
+        <v>0.7914896366620319</v>
       </c>
       <c r="O320" t="n">
         <v>0.49</v>
@@ -75608,7 +75608,7 @@
         <v>1412512331.45</v>
       </c>
       <c r="AN320" t="n">
-        <v>3344287610.619469</v>
+        <v>3397564159.292036</v>
       </c>
       <c r="AO320" t="n">
         <v>0</v>
@@ -76687,7 +76687,7 @@
         <v>7.5</v>
       </c>
       <c r="H325" t="n">
-        <v>601265900</v>
+        <v>609559400</v>
       </c>
       <c r="I325" t="n">
         <v>0</v>
@@ -76783,7 +76783,7 @@
         <v>8742210.08</v>
       </c>
       <c r="AN325" t="n">
-        <v>6903960.27098404</v>
+        <v>6999189.344356413</v>
       </c>
       <c r="AO325" t="n">
         <v>0</v>
@@ -76922,7 +76922,7 @@
         <v>6.92</v>
       </c>
       <c r="H326" t="n">
-        <v>601265900</v>
+        <v>609559400</v>
       </c>
       <c r="I326" t="n">
         <v>200</v>
@@ -77018,7 +77018,7 @@
         <v>2719637.39</v>
       </c>
       <c r="AN326" t="n">
-        <v>5933740.254613639</v>
+        <v>6015586.69693082</v>
       </c>
       <c r="AO326" t="n">
         <v>0.4906</v>
@@ -77157,7 +77157,7 @@
         <v>6.5</v>
       </c>
       <c r="H327" t="n">
-        <v>601265900</v>
+        <v>609559400</v>
       </c>
       <c r="I327" t="n">
         <v>0</v>
@@ -77253,7 +77253,7 @@
         <v>4627783.64</v>
       </c>
       <c r="AN327" t="n">
-        <v>8724113.464886826</v>
+        <v>8844448.636099827</v>
       </c>
       <c r="AO327" t="n">
         <v>0</v>
@@ -77392,7 +77392,7 @@
         <v>1.47</v>
       </c>
       <c r="H328" t="n">
-        <v>99506683</v>
+        <v>100679600</v>
       </c>
       <c r="I328" t="n">
         <v>15500</v>
@@ -77410,7 +77410,7 @@
         <v>0.11</v>
       </c>
       <c r="N328" t="n">
-        <v>0.01150930098041375</v>
+        <v>0.01164496478078426</v>
       </c>
       <c r="O328" t="n">
         <v>0.02</v>
@@ -77488,7 +77488,7 @@
         <v>1659121826.79</v>
       </c>
       <c r="AN328" t="n">
-        <v>995066830</v>
+        <v>1006796000</v>
       </c>
       <c r="AO328" t="n">
         <v>0</v>
@@ -78097,7 +78097,7 @@
         <v>26.72</v>
       </c>
       <c r="H331" t="n">
-        <v>100864416928</v>
+        <v>20288419438</v>
       </c>
       <c r="I331" t="n">
         <v>3462700</v>
@@ -78115,7 +78115,7 @@
         <v>10.97</v>
       </c>
       <c r="N331" t="n">
-        <v>0.07642600000000002</v>
+        <v>0.07642600000000001</v>
       </c>
       <c r="O331" t="n">
         <v>0.1</v>
@@ -78187,13 +78187,13 @@
         <v>6.94</v>
       </c>
       <c r="AL331" t="n">
-        <v>1319765746316.698</v>
+        <v>265464886792.4528</v>
       </c>
       <c r="AM331" t="n">
-        <v>97926618376.69902</v>
+        <v>19697494600</v>
       </c>
       <c r="AN331" t="n">
-        <v>12529741233.29192</v>
+        <v>2520300551.304348</v>
       </c>
       <c r="AO331" t="n">
         <v>0.702</v>
@@ -78332,7 +78332,7 @@
         <v>12.97</v>
       </c>
       <c r="H332" t="n">
-        <v>100864416928</v>
+        <v>20288419438</v>
       </c>
       <c r="I332" t="n">
         <v>169300</v>
@@ -78350,7 +78350,7 @@
         <v>10.74</v>
       </c>
       <c r="N332" t="n">
-        <v>1.264431228435906</v>
+        <v>0.2543345997957371</v>
       </c>
       <c r="O332" t="n">
         <v>0.1</v>
@@ -78428,7 +78428,7 @@
         <v>5918977298.05</v>
       </c>
       <c r="AN332" t="n">
-        <v>12800052909.64467</v>
+        <v>2574672517.512691</v>
       </c>
       <c r="AO332" t="n">
         <v>0.3343</v>
@@ -78567,7 +78567,7 @@
         <v>13.88</v>
       </c>
       <c r="H333" t="n">
-        <v>100864416928</v>
+        <v>20288419438</v>
       </c>
       <c r="I333" t="n">
         <v>165700</v>
@@ -78585,7 +78585,7 @@
         <v>10.86</v>
       </c>
       <c r="N333" t="n">
-        <v>1.312144677867852</v>
+        <v>0.2639319434813714</v>
       </c>
       <c r="O333" t="n">
         <v>0.1</v>
@@ -78663,7 +78663,7 @@
         <v>5703745831</v>
       </c>
       <c r="AN333" t="n">
-        <v>12655510279.54831</v>
+        <v>2545598423.839398</v>
       </c>
       <c r="AO333" t="n">
         <v>0.3677</v>
@@ -79742,7 +79742,7 @@
         <v>27.23</v>
       </c>
       <c r="H338" t="n">
-        <v>95581600733</v>
+        <v>19493073177</v>
       </c>
       <c r="I338" t="n">
         <v>24893300</v>
@@ -79760,7 +79760,7 @@
         <v>14.04</v>
       </c>
       <c r="N338" t="n">
-        <v>0.55058047587875</v>
+        <v>0.1122863126776083</v>
       </c>
       <c r="O338" t="n">
         <v>1.05</v>
@@ -79838,7 +79838,7 @@
         <v>36126473756.25</v>
       </c>
       <c r="AN338" t="n">
-        <v>9915103810.477179</v>
+        <v>2022103026.659751</v>
       </c>
       <c r="AO338" t="n">
         <v>2.6439</v>
@@ -80682,7 +80682,7 @@
         <v>5.75</v>
       </c>
       <c r="H342" t="n">
-        <v>386041602</v>
+        <v>392191600</v>
       </c>
       <c r="I342" t="n">
         <v>46200</v>
@@ -80700,7 +80700,7 @@
         <v>0.62</v>
       </c>
       <c r="N342" t="n">
-        <v>2.611078327924297</v>
+        <v>2.652675208704462</v>
       </c>
       <c r="O342" t="n">
         <v>0.1</v>
@@ -80778,7 +80778,7 @@
         <v>61075833.72000001</v>
       </c>
       <c r="AN342" t="n">
-        <v>419610436.9565217</v>
+        <v>426295217.3913043</v>
       </c>
       <c r="AO342" t="n">
         <v>0</v>
@@ -83267,7 +83267,7 @@
         <v>38.66</v>
       </c>
       <c r="H353" t="n">
-        <v>152351900</v>
+        <v>154499700</v>
       </c>
       <c r="I353" t="n">
         <v>0</v>
@@ -83285,7 +83285,7 @@
         <v>3.42</v>
       </c>
       <c r="N353" t="n">
-        <v>1.982993984161773</v>
+        <v>2.010949490323382</v>
       </c>
       <c r="O353" t="n">
         <v>0.78</v>
@@ -83363,7 +83363,7 @@
         <v>9672800</v>
       </c>
       <c r="AN353" t="n">
-        <v>61432217.74193548</v>
+        <v>62298266.12903226</v>
       </c>
       <c r="AO353" t="n">
         <v>0</v>
@@ -83502,7 +83502,7 @@
         <v>76.09999999999999</v>
       </c>
       <c r="H354" t="n">
-        <v>152351900</v>
+        <v>154499700</v>
       </c>
       <c r="I354" t="n">
         <v>0</v>
@@ -83520,7 +83520,7 @@
         <v>6.19</v>
       </c>
       <c r="N354" t="n">
-        <v>2.163449975073258</v>
+        <v>2.193949482177943</v>
       </c>
       <c r="O354" t="n">
         <v>1.42</v>
@@ -83598,7 +83598,7 @@
         <v>8865980</v>
       </c>
       <c r="AN354" t="n">
-        <v>33855977.77777778</v>
+        <v>34333266.66666666</v>
       </c>
       <c r="AO354" t="n">
         <v>0</v>
@@ -83737,7 +83737,7 @@
         <v>79.98999999999999</v>
       </c>
       <c r="H355" t="n">
-        <v>152351900</v>
+        <v>154499700</v>
       </c>
       <c r="I355" t="n">
         <v>200</v>
@@ -83755,7 +83755,7 @@
         <v>6.02</v>
       </c>
       <c r="N355" t="n">
-        <v>2.076890799513615</v>
+        <v>2.106170027794952</v>
       </c>
       <c r="O355" t="n">
         <v>1.38</v>
@@ -83833,7 +83833,7 @@
         <v>9235490</v>
       </c>
       <c r="AN355" t="n">
-        <v>34863135.01144165</v>
+        <v>35354622.42562929</v>
       </c>
       <c r="AO355" t="n">
         <v>0</v>
@@ -86087,7 +86087,7 @@
         <v>11.9</v>
       </c>
       <c r="H365" t="n">
-        <v>1164414490</v>
+        <v>1152851000</v>
       </c>
       <c r="I365" t="n">
         <v>100</v>
@@ -86105,7 +86105,7 @@
         <v>20.34</v>
       </c>
       <c r="N365" t="n">
-        <v>3.080330827293003</v>
+        <v>3.049740882712277</v>
       </c>
       <c r="O365" t="n">
         <v>0.27</v>
@@ -86183,7 +86183,7 @@
         <v>45966751.6</v>
       </c>
       <c r="AN365" t="n">
-        <v>123873881.9148936</v>
+        <v>122643723.4042553</v>
       </c>
       <c r="AO365" t="n">
         <v>0</v>
@@ -86322,7 +86322,7 @@
         <v>7.87</v>
       </c>
       <c r="H366" t="n">
-        <v>1164414490</v>
+        <v>1152851000</v>
       </c>
       <c r="I366" t="n">
         <v>3300</v>
@@ -86340,7 +86340,7 @@
         <v>14.31</v>
       </c>
       <c r="N366" t="n">
-        <v>13.98568974732772</v>
+        <v>13.84680158943789</v>
       </c>
       <c r="O366" t="n">
         <v>0.19</v>
@@ -86418,7 +86418,7 @@
         <v>10124120.05</v>
       </c>
       <c r="AN366" t="n">
-        <v>176159529.5007564</v>
+        <v>174410136.1573374</v>
       </c>
       <c r="AO366" t="n">
         <v>0</v>
@@ -87262,7 +87262,7 @@
         <v>22.34</v>
       </c>
       <c r="H370" t="n">
-        <v>53222101483</v>
+        <v>10656839669</v>
       </c>
       <c r="I370" t="n">
         <v>4922500</v>
@@ -87280,7 +87280,7 @@
         <v>34.8</v>
       </c>
       <c r="N370" t="n">
-        <v>2.029828549282336</v>
+        <v>0.4064393701584706</v>
       </c>
       <c r="O370" t="n">
         <v>1.06</v>
@@ -87358,7 +87358,7 @@
         <v>1746251898.97</v>
       </c>
       <c r="AN370" t="n">
-        <v>5311586974.351297</v>
+        <v>1063556853.193613</v>
       </c>
       <c r="AO370" t="n">
         <v>0.3753</v>
@@ -87732,7 +87732,7 @@
         <v>0.14</v>
       </c>
       <c r="H372" t="n">
-        <v>30226378</v>
+        <v>120905512</v>
       </c>
       <c r="I372" t="n">
         <v>869400</v>
@@ -87750,7 +87750,7 @@
         <v>1.46</v>
       </c>
       <c r="N372" t="n">
-        <v>0.07920891104520003</v>
+        <v>0.3168356441808001</v>
       </c>
       <c r="O372" t="n">
         <v>68.65000000000001</v>
@@ -87828,7 +87828,7 @@
         <v>91050535.8</v>
       </c>
       <c r="AN372" t="n">
-        <v>13615485.58558558</v>
+        <v>54461942.34234234</v>
       </c>
       <c r="AO372" t="n">
         <v>0</v>
@@ -89377,7 +89377,7 @@
         <v>9.98</v>
       </c>
       <c r="H379" t="n">
-        <v>19083160</v>
+        <v>19387170</v>
       </c>
       <c r="I379" t="n">
         <v>0</v>
@@ -89395,7 +89395,7 @@
         <v>0.73</v>
       </c>
       <c r="N379" t="n">
-        <v>0.4943009148302772</v>
+        <v>0.5021755237062471</v>
       </c>
       <c r="O379" t="n">
         <v>0.24</v>
@@ -89473,7 +89473,7 @@
         <v>19824366.83</v>
       </c>
       <c r="AN379" t="n">
-        <v>4479615.023474178</v>
+        <v>4550978.873239437</v>
       </c>
       <c r="AO379" t="n">
         <v>0</v>
@@ -89612,7 +89612,7 @@
         <v>1.65</v>
       </c>
       <c r="H380" t="n">
-        <v>19083160</v>
+        <v>19387170</v>
       </c>
       <c r="I380" t="n">
         <v>0</v>
@@ -89630,7 +89630,7 @@
         <v>0.12</v>
       </c>
       <c r="N380" t="n">
-        <v>0.2568972231003798</v>
+        <v>0.2609898013104219</v>
       </c>
       <c r="O380" t="n">
         <v>0.04</v>
@@ -89708,7 +89708,7 @@
         <v>38144447.58</v>
       </c>
       <c r="AN380" t="n">
-        <v>28482328.35820895</v>
+        <v>28936074.62686567</v>
       </c>
       <c r="AO380" t="n">
         <v>0</v>
@@ -90082,7 +90082,7 @@
         <v>24.92</v>
       </c>
       <c r="H382" t="n">
-        <v>27806957165</v>
+        <v>5566619037</v>
       </c>
       <c r="I382" t="n">
         <v>6191100</v>
@@ -90100,7 +90100,7 @@
         <v>10.01</v>
       </c>
       <c r="N382" t="n">
-        <v>0.1995472129124867</v>
+        <v>0.03994695671258429</v>
       </c>
       <c r="O382" t="n">
         <v>0.65</v>
@@ -90178,7 +90178,7 @@
         <v>2968160662.18</v>
       </c>
       <c r="AN382" t="n">
-        <v>5399409158.252427</v>
+        <v>1080896900.38835</v>
       </c>
       <c r="AO382" t="n">
         <v>0</v>
@@ -91727,7 +91727,7 @@
         <v>81.79000000000001</v>
       </c>
       <c r="H389" t="n">
-        <v>361597847127</v>
+        <v>71226169037</v>
       </c>
       <c r="I389" t="n">
         <v>19308800</v>
@@ -91745,7 +91745,7 @@
         <v>12.88</v>
       </c>
       <c r="N389" t="n">
-        <v>1.695117173567411</v>
+        <v>0.3338977355681796</v>
       </c>
       <c r="O389" t="n">
         <v>0.8</v>
@@ -91823,7 +91823,7 @@
         <v>30184400327.2</v>
       </c>
       <c r="AN389" t="n">
-        <v>39562127694.42013</v>
+        <v>7792797487.636761</v>
       </c>
       <c r="AO389" t="n">
         <v>3.5818</v>
@@ -92902,7 +92902,7 @@
         <v>0.31</v>
       </c>
       <c r="H394" t="n">
-        <v>15128127</v>
+        <v>15306440</v>
       </c>
       <c r="I394" t="n">
         <v>159000</v>
@@ -92920,7 +92920,7 @@
         <v>1.29</v>
       </c>
       <c r="N394" t="n">
-        <v>0.2698978760869934</v>
+        <v>0.273079122514836</v>
       </c>
       <c r="O394" t="n">
         <v>0.13</v>
@@ -92998,7 +92998,7 @@
         <v>22936192.23</v>
       </c>
       <c r="AN394" t="n">
-        <v>9952715.131578946</v>
+        <v>10070026.31578947</v>
       </c>
       <c r="AO394" t="n">
         <v>0</v>
@@ -93137,7 +93137,7 @@
         <v>33.75</v>
       </c>
       <c r="H395" t="n">
-        <v>108451811250</v>
+        <v>21672914228</v>
       </c>
       <c r="I395" t="n">
         <v>7626900</v>
@@ -93155,7 +93155,7 @@
         <v>20.73</v>
       </c>
       <c r="N395" t="n">
-        <v>1.848679197157437</v>
+        <v>0.3694384189003669</v>
       </c>
       <c r="O395" t="n">
         <v>1.01</v>
@@ -93233,7 +93233,7 @@
         <v>6065907649.36</v>
       </c>
       <c r="AN395" t="n">
-        <v>8148145097.670924</v>
+        <v>1628318123.816679</v>
       </c>
       <c r="AO395" t="n">
         <v>0.1645</v>
@@ -94782,7 +94782,7 @@
         <v>8.050000000000001</v>
       </c>
       <c r="H402" t="n">
-        <v>89065443</v>
+        <v>90484380</v>
       </c>
       <c r="I402" t="n">
         <v>4000</v>
@@ -94800,7 +94800,7 @@
         <v>5.91</v>
       </c>
       <c r="N402" t="n">
-        <v>0.6086816223318706</v>
+        <v>0.6183787713725677</v>
       </c>
       <c r="O402" t="n">
         <v>0.23</v>
@@ -94878,7 +94878,7 @@
         <v>11442628.44</v>
       </c>
       <c r="AN402" t="n">
-        <v>38225512.01716738</v>
+        <v>38834497.85407725</v>
       </c>
       <c r="AO402" t="n">
         <v>0</v>
@@ -95017,7 +95017,7 @@
         <v>3.92</v>
       </c>
       <c r="H403" t="n">
-        <v>5816295064</v>
+        <v>5969951000</v>
       </c>
       <c r="I403" t="n">
         <v>1400</v>
@@ -95035,7 +95035,7 @@
         <v>9.42</v>
       </c>
       <c r="N403" t="n">
-        <v>0.6556256835698195</v>
+        <v>0.6729461215747784</v>
       </c>
       <c r="O403" t="n">
         <v>0.66</v>
@@ -95113,7 +95113,7 @@
         <v>483489419.2399999</v>
       </c>
       <c r="AN403" t="n">
-        <v>1116371413.435701</v>
+        <v>1145863915.547025</v>
       </c>
       <c r="AO403" t="n">
         <v>0</v>
@@ -95252,7 +95252,7 @@
         <v>3.94</v>
       </c>
       <c r="H404" t="n">
-        <v>5816295064</v>
+        <v>5969951000</v>
       </c>
       <c r="I404" t="n">
         <v>37200</v>
@@ -95270,7 +95270,7 @@
         <v>9.92</v>
       </c>
       <c r="N404" t="n">
-        <v>1.422619495085819</v>
+        <v>1.460202514462234</v>
       </c>
       <c r="O404" t="n">
         <v>0.6899999999999999</v>
@@ -95348,7 +95348,7 @@
         <v>222820003.58</v>
       </c>
       <c r="AN404" t="n">
-        <v>1061367712.408759</v>
+        <v>1089407116.788321</v>
       </c>
       <c r="AO404" t="n">
         <v>0</v>
@@ -95722,7 +95722,7 @@
         <v>20.5</v>
       </c>
       <c r="H406" t="n">
-        <v>713043537</v>
+        <v>724983000</v>
       </c>
       <c r="I406" t="n">
         <v>0</v>
@@ -95740,7 +95740,7 @@
         <v>6.94</v>
       </c>
       <c r="N406" t="n">
-        <v>0.5128847333279744</v>
+        <v>0.5214726637685165</v>
       </c>
       <c r="O406" t="n">
         <v>0.53</v>
@@ -95818,7 +95818,7 @@
         <v>53525040.6</v>
       </c>
       <c r="AN406" t="n">
-        <v>175626486.9458128</v>
+        <v>178567241.3793104</v>
       </c>
       <c r="AO406" t="n">
         <v>0.9505</v>
@@ -95957,7 +95957,7 @@
         <v>18.99</v>
       </c>
       <c r="H407" t="n">
-        <v>713043537</v>
+        <v>724983000</v>
       </c>
       <c r="I407" t="n">
         <v>800</v>
@@ -95975,7 +95975,7 @@
         <v>7.58</v>
       </c>
       <c r="N407" t="n">
-        <v>0.4283088752519947</v>
+        <v>0.4354806364464908</v>
       </c>
       <c r="O407" t="n">
         <v>0.58</v>
@@ -96053,7 +96053,7 @@
         <v>64094343.5</v>
       </c>
       <c r="AN407" t="n">
-        <v>160957909.0293454</v>
+        <v>163653047.4040632</v>
       </c>
       <c r="AO407" t="n">
         <v>0.7018</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-06-08 05:34
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -2475,7 +2475,7 @@
         <v>24</v>
       </c>
       <c r="H9" t="n">
-        <v>211905528</v>
+        <v>209405000</v>
       </c>
       <c r="I9" t="n">
         <v>300</v>
@@ -2493,7 +2493,7 @@
         <v>2.59</v>
       </c>
       <c r="N9" t="n">
-        <v>0.3196059817012898</v>
+        <v>0.3158345666100725</v>
       </c>
       <c r="O9" t="n">
         <v>0.36</v>
@@ -2571,7 +2571,7 @@
         <v>81220091.82000001</v>
       </c>
       <c r="AN9" t="n">
-        <v>73834678.7456446</v>
+        <v>72963414.63414633</v>
       </c>
       <c r="AO9" t="n">
         <v>0</v>
@@ -2710,7 +2710,7 @@
         <v>58</v>
       </c>
       <c r="H10" t="n">
-        <v>211905528</v>
+        <v>209405000</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -2728,7 +2728,7 @@
         <v>6.01</v>
       </c>
       <c r="N10" t="n">
-        <v>59.68654841208066</v>
+        <v>58.98223509408282</v>
       </c>
       <c r="O10" t="n">
         <v>0.84</v>
@@ -2806,7 +2806,7 @@
         <v>434912.52</v>
       </c>
       <c r="AN10" t="n">
-        <v>31769944.22788606</v>
+        <v>31395052.47376312</v>
       </c>
       <c r="AO10" t="n">
         <v>0</v>
@@ -2945,7 +2945,7 @@
         <v>55</v>
       </c>
       <c r="H11" t="n">
-        <v>211905528</v>
+        <v>209405000</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -2963,7 +2963,7 @@
         <v>5.7</v>
       </c>
       <c r="N11" t="n">
-        <v>29.53137845605468</v>
+        <v>29.18290222985655</v>
       </c>
       <c r="O11" t="n">
         <v>0.79</v>
@@ -3041,7 +3041,7 @@
         <v>879011.7000000001</v>
       </c>
       <c r="AN11" t="n">
-        <v>33529355.69620253</v>
+        <v>33133702.53164557</v>
       </c>
       <c r="AO11" t="n">
         <v>0</v>
@@ -8804,7 +8804,7 @@
         <v>26</v>
       </c>
       <c r="H36" t="n">
-        <v>222603250</v>
+        <v>220010000</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
@@ -8822,7 +8822,7 @@
         <v>10.3</v>
       </c>
       <c r="N36" t="n">
-        <v>2.033499076773567</v>
+        <v>2.009809523809524</v>
       </c>
       <c r="O36" t="n">
         <v>0.85</v>
@@ -8900,7 +8900,7 @@
         <v>12348000</v>
       </c>
       <c r="AN36" t="n">
-        <v>39821690.51878354</v>
+        <v>39357781.75313059</v>
       </c>
       <c r="AO36" t="n">
         <v>0</v>
@@ -9039,7 +9039,7 @@
         <v>18.9</v>
       </c>
       <c r="H37" t="n">
-        <v>222603250</v>
+        <v>220010000</v>
       </c>
       <c r="I37" t="n">
         <v>600</v>
@@ -9057,7 +9057,7 @@
         <v>7.41</v>
       </c>
       <c r="N37" t="n">
-        <v>2.033499076773567</v>
+        <v>2.009809523809524</v>
       </c>
       <c r="O37" t="n">
         <v>0.61</v>
@@ -9135,7 +9135,7 @@
         <v>12348000</v>
       </c>
       <c r="AN37" t="n">
-        <v>55373942.78606965</v>
+        <v>54728855.72139304</v>
       </c>
       <c r="AO37" t="n">
         <v>0</v>
@@ -10684,7 +10684,7 @@
         <v>7.9</v>
       </c>
       <c r="H44" t="n">
-        <v>7684038</v>
+        <v>8748190</v>
       </c>
       <c r="I44" t="n">
         <v>400</v>
@@ -10702,7 +10702,7 @@
         <v>0.75</v>
       </c>
       <c r="N44" t="n">
-        <v>0.3433787455387201</v>
+        <v>0.3909328022498555</v>
       </c>
       <c r="O44" t="n">
         <v>0.03</v>
@@ -10780,7 +10780,7 @@
         <v>5719748.64</v>
       </c>
       <c r="AN44" t="n">
-        <v>7684038</v>
+        <v>8748190</v>
       </c>
       <c r="AO44" t="n">
         <v>0</v>
@@ -10919,7 +10919,7 @@
         <v>3.98</v>
       </c>
       <c r="H45" t="n">
-        <v>7684038</v>
+        <v>8748190</v>
       </c>
       <c r="I45" t="n">
         <v>2200</v>
@@ -10937,7 +10937,7 @@
         <v>0.63</v>
       </c>
       <c r="N45" t="n">
-        <v>0.2100071990366179</v>
+        <v>0.2390908111776842</v>
       </c>
       <c r="O45" t="n">
         <v>0.02</v>
@@ -11015,7 +11015,7 @@
         <v>9352251.359999999</v>
       </c>
       <c r="AN45" t="n">
-        <v>9147664.285714285</v>
+        <v>10414511.9047619</v>
       </c>
       <c r="AO45" t="n">
         <v>0</v>
@@ -11859,7 +11859,7 @@
         <v>52.6</v>
       </c>
       <c r="H49" t="n">
-        <v>963682900</v>
+        <v>963778100</v>
       </c>
       <c r="I49" t="n">
         <v>0</v>
@@ -11877,7 +11877,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="N49" t="n">
-        <v>1.052257889055595</v>
+        <v>1.052361839173458</v>
       </c>
       <c r="O49" t="n">
         <v>0.08</v>
@@ -11955,7 +11955,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN49" t="n">
-        <v>176176032.9067642</v>
+        <v>176193436.928702</v>
       </c>
       <c r="AO49" t="n">
         <v>2.4346</v>
@@ -12094,7 +12094,7 @@
         <v>30.91</v>
       </c>
       <c r="H50" t="n">
-        <v>963682900</v>
+        <v>963778100</v>
       </c>
       <c r="I50" t="n">
         <v>800</v>
@@ -12112,7 +12112,7 @@
         <v>5.78</v>
       </c>
       <c r="N50" t="n">
-        <v>1.052257889055595</v>
+        <v>1.052361839173458</v>
       </c>
       <c r="O50" t="n">
         <v>0.06</v>
@@ -12190,7 +12190,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN50" t="n">
-        <v>252935144.3569554</v>
+        <v>252960131.2335958</v>
       </c>
       <c r="AO50" t="n">
         <v>3.526</v>
@@ -14428,7 +14428,7 @@
         <v>389.92</v>
       </c>
       <c r="H60" t="n">
-        <v>179406175</v>
+        <v>177316100</v>
       </c>
       <c r="I60" t="n">
         <v>49</v>
@@ -14446,7 +14446,7 @@
         <v>2.87</v>
       </c>
       <c r="N60" t="n">
-        <v>12.67797684635367</v>
+        <v>12.53027890642968</v>
       </c>
       <c r="O60" t="n">
         <v>0.64</v>
@@ -14524,7 +14524,7 @@
         <v>59731412.5</v>
       </c>
       <c r="AN60" t="n">
-        <v>22595236.14609572</v>
+        <v>22332002.51889168</v>
       </c>
       <c r="AO60" t="n">
         <v>0</v>
@@ -19598,7 +19598,7 @@
         <v>9.65</v>
       </c>
       <c r="H82" t="n">
-        <v>404149700</v>
+        <v>407954500</v>
       </c>
       <c r="I82" t="n">
         <v>6100</v>
@@ -19616,7 +19616,7 @@
         <v>6.04</v>
       </c>
       <c r="N82" t="n">
-        <v>1.027699835222074</v>
+        <v>1.037374944056877</v>
       </c>
       <c r="O82" t="n">
         <v>1.01</v>
@@ -19694,7 +19694,7 @@
         <v>65949124.8</v>
       </c>
       <c r="AN82" t="n">
-        <v>71912758.00711744</v>
+        <v>72589768.68327402</v>
       </c>
       <c r="AO82" t="n">
         <v>0</v>
@@ -20491,7 +20491,7 @@
         <v>0</v>
       </c>
       <c r="BR85" t="n">
-        <v>29</v>
+        <v>26.5</v>
       </c>
       <c r="BS85" t="n">
         <v>0</v>
@@ -20773,7 +20773,7 @@
         <v>15.31</v>
       </c>
       <c r="H87" t="n">
-        <v>6938858099</v>
+        <v>6938858000</v>
       </c>
       <c r="I87" t="n">
         <v>200</v>
@@ -20791,7 +20791,7 @@
         <v>7.13</v>
       </c>
       <c r="N87" t="n">
-        <v>0.7403819812787961</v>
+        <v>0.740381970715413</v>
       </c>
       <c r="O87" t="n">
         <v>0.21</v>
@@ -20869,7 +20869,7 @@
         <v>580126647.04</v>
       </c>
       <c r="AN87" t="n">
-        <v>1263908579.052823</v>
+        <v>1263908561.020036</v>
       </c>
       <c r="AO87" t="n">
         <v>0</v>
@@ -21243,7 +21243,7 @@
         <v>27.3</v>
       </c>
       <c r="H89" t="n">
-        <v>2009825943</v>
+        <v>1992196000</v>
       </c>
       <c r="I89" t="n">
         <v>1800</v>
@@ -21261,7 +21261,7 @@
         <v>11.38</v>
       </c>
       <c r="N89" t="n">
-        <v>8.413673359676679</v>
+        <v>8.33986966425303</v>
       </c>
       <c r="O89" t="n">
         <v>1.53</v>
@@ -21339,7 +21339,7 @@
         <v>95908776.3</v>
       </c>
       <c r="AN89" t="n">
-        <v>219174039.5856052</v>
+        <v>217251472.1919302</v>
       </c>
       <c r="AO89" t="n">
         <v>0</v>
@@ -21478,7 +21478,7 @@
         <v>25.15</v>
       </c>
       <c r="H90" t="n">
-        <v>2009825943</v>
+        <v>1992196000</v>
       </c>
       <c r="I90" t="n">
         <v>1100</v>
@@ -21496,7 +21496,7 @@
         <v>10.59</v>
       </c>
       <c r="N90" t="n">
-        <v>46.03597484982908</v>
+        <v>45.63215300874942</v>
       </c>
       <c r="O90" t="n">
         <v>1.42</v>
@@ -21574,7 +21574,7 @@
         <v>17528576.7</v>
       </c>
       <c r="AN90" t="n">
-        <v>235618516.1781946</v>
+        <v>233551699.8827667</v>
       </c>
       <c r="AO90" t="n">
         <v>0</v>
@@ -21713,7 +21713,7 @@
         <v>28.6</v>
       </c>
       <c r="H91" t="n">
-        <v>2009825943</v>
+        <v>1992196000</v>
       </c>
       <c r="I91" t="n">
         <v>1800</v>
@@ -21731,7 +21731,7 @@
         <v>11.3</v>
       </c>
       <c r="N91" t="n">
-        <v>10.21173408814925</v>
+        <v>10.12215802782807</v>
       </c>
       <c r="O91" t="n">
         <v>1.52</v>
@@ -21809,7 +21809,7 @@
         <v>79021360.05</v>
       </c>
       <c r="AN91" t="n">
-        <v>220859993.7362638</v>
+        <v>218922637.3626374</v>
       </c>
       <c r="AO91" t="n">
         <v>0</v>
@@ -21948,7 +21948,7 @@
         <v>10</v>
       </c>
       <c r="H92" t="n">
-        <v>77550720</v>
+        <v>77558380</v>
       </c>
       <c r="I92" t="n">
         <v>0</v>
@@ -21966,7 +21966,7 @@
         <v>3.42</v>
       </c>
       <c r="N92" t="n">
-        <v>0.1431937325334147</v>
+        <v>0.1432078763607217</v>
       </c>
       <c r="O92" t="n">
         <v>0.15</v>
@@ -22044,7 +22044,7 @@
         <v>23342055.36</v>
       </c>
       <c r="AN92" t="n">
-        <v>55000510.63829788</v>
+        <v>55005943.26241135</v>
       </c>
       <c r="AO92" t="n">
         <v>0</v>
@@ -22183,7 +22183,7 @@
         <v>4.76</v>
       </c>
       <c r="H93" t="n">
-        <v>77550720</v>
+        <v>77558380</v>
       </c>
       <c r="I93" t="n">
         <v>0</v>
@@ -22201,7 +22201,7 @@
         <v>2.3</v>
       </c>
       <c r="N93" t="n">
-        <v>0.190366019516052</v>
+        <v>0.1903848227419858</v>
       </c>
       <c r="O93" t="n">
         <v>0.1</v>
@@ -22279,7 +22279,7 @@
         <v>17557944.64</v>
       </c>
       <c r="AN93" t="n">
-        <v>81632336.84210527</v>
+        <v>81640400</v>
       </c>
       <c r="AO93" t="n">
         <v>0</v>
@@ -23593,7 +23593,7 @@
         <v>124</v>
       </c>
       <c r="H99" t="n">
-        <v>16529770250</v>
+        <v>16389570000</v>
       </c>
       <c r="I99" t="n">
         <v>0</v>
@@ -23611,7 +23611,7 @@
         <v>10.65</v>
       </c>
       <c r="N99" t="n">
-        <v>1.6332453217752</v>
+        <v>1.619392654801549</v>
       </c>
       <c r="O99" t="n">
         <v>1.16</v>
@@ -23689,7 +23689,7 @@
         <v>1267125769.6</v>
       </c>
       <c r="AN99" t="n">
-        <v>2845055120.481928</v>
+        <v>2820924268.502582</v>
       </c>
       <c r="AO99" t="n">
         <v>0</v>
@@ -23828,7 +23828,7 @@
         <v>122.5</v>
       </c>
       <c r="H100" t="n">
-        <v>16529770250</v>
+        <v>16389570000</v>
       </c>
       <c r="I100" t="n">
         <v>500</v>
@@ -23846,7 +23846,7 @@
         <v>10.81</v>
       </c>
       <c r="N100" t="n">
-        <v>5.91927040723591</v>
+        <v>5.869065039686286</v>
       </c>
       <c r="O100" t="n">
         <v>1.18</v>
@@ -23924,7 +23924,7 @@
         <v>349625391.8</v>
       </c>
       <c r="AN100" t="n">
-        <v>2801655974.576271</v>
+        <v>2777893220.338983</v>
       </c>
       <c r="AO100" t="n">
         <v>0</v>
@@ -24063,7 +24063,7 @@
         <v>24.7</v>
       </c>
       <c r="H101" t="n">
-        <v>641135683</v>
+        <v>634684900</v>
       </c>
       <c r="I101" t="n">
         <v>200</v>
@@ -24081,7 +24081,7 @@
         <v>6.28</v>
       </c>
       <c r="N101" t="n">
-        <v>2.067749482178101</v>
+        <v>2.046944832613941</v>
       </c>
       <c r="O101" t="n">
         <v>0.49</v>
@@ -24159,7 +24159,7 @@
         <v>42633867</v>
       </c>
       <c r="AN101" t="n">
-        <v>66301518.40744571</v>
+        <v>65634426.05997932</v>
       </c>
       <c r="AO101" t="n">
         <v>0</v>
@@ -24298,7 +24298,7 @@
         <v>24.88</v>
       </c>
       <c r="H102" t="n">
-        <v>641135683</v>
+        <v>634684900</v>
       </c>
       <c r="I102" t="n">
         <v>3600</v>
@@ -24316,7 +24316,7 @@
         <v>6.32</v>
       </c>
       <c r="N102" t="n">
-        <v>1.48350319144646</v>
+        <v>1.46857693258804</v>
       </c>
       <c r="O102" t="n">
         <v>0.49</v>
@@ -24394,7 +24394,7 @@
         <v>59424311.94</v>
       </c>
       <c r="AN102" t="n">
-        <v>65892670.4008222</v>
+        <v>65229691.67523124</v>
       </c>
       <c r="AO102" t="n">
         <v>0</v>
@@ -32993,7 +32993,7 @@
         <v>2.45</v>
       </c>
       <c r="H139" t="n">
-        <v>26701190</v>
+        <v>26167170</v>
       </c>
       <c r="I139" t="n">
         <v>4000</v>
@@ -33011,7 +33011,7 @@
         <v>186.65</v>
       </c>
       <c r="N139" t="n">
-        <v>4.949999999999999</v>
+        <v>4.851000704462984</v>
       </c>
       <c r="O139" t="n">
         <v>4.19</v>
@@ -33089,7 +33089,7 @@
         <v>106804.76</v>
       </c>
       <c r="AN139" t="n">
-        <v>108163.2909341327</v>
+        <v>106000.0405087904</v>
       </c>
       <c r="AO139" t="n">
         <v>0</v>
@@ -33463,7 +33463,7 @@
         <v>13.48</v>
       </c>
       <c r="H141" t="n">
-        <v>296327459</v>
+        <v>290670700</v>
       </c>
       <c r="I141" t="n">
         <v>200</v>
@@ -33481,7 +33481,7 @@
         <v>2.98</v>
       </c>
       <c r="N141" t="n">
-        <v>1.179566868206217</v>
+        <v>1.15704946289945</v>
       </c>
       <c r="O141" t="n">
         <v>0.5</v>
@@ -33559,7 +33559,7 @@
         <v>45922500</v>
       </c>
       <c r="AN141" t="n">
-        <v>76968171.16883117</v>
+        <v>75498883.11688311</v>
       </c>
       <c r="AO141" t="n">
         <v>0</v>
@@ -33698,7 +33698,7 @@
         <v>12.05</v>
       </c>
       <c r="H142" t="n">
-        <v>296327459</v>
+        <v>290670700</v>
       </c>
       <c r="I142" t="n">
         <v>3600</v>
@@ -33716,7 +33716,7 @@
         <v>3.05</v>
       </c>
       <c r="N142" t="n">
-        <v>0.9020217227459307</v>
+        <v>0.8848025304525208</v>
       </c>
       <c r="O142" t="n">
         <v>0.51</v>
@@ -33794,7 +33794,7 @@
         <v>60052500</v>
       </c>
       <c r="AN142" t="n">
-        <v>75019609.87341772</v>
+        <v>73587518.98734176</v>
       </c>
       <c r="AO142" t="n">
         <v>0</v>
@@ -34403,7 +34403,7 @@
         <v>51.52</v>
       </c>
       <c r="H145" t="n">
-        <v>8542938000</v>
+        <v>8589801000</v>
       </c>
       <c r="I145" t="n">
         <v>0</v>
@@ -34421,7 +34421,7 @@
         <v>10.18</v>
       </c>
       <c r="N145" t="n">
-        <v>1.846006971661118</v>
+        <v>1.856133397103157</v>
       </c>
       <c r="O145" t="n">
         <v>0.73</v>
@@ -34499,7 +34499,7 @@
         <v>441028665.6</v>
       </c>
       <c r="AN145" t="n">
-        <v>1963893793.103448</v>
+        <v>1974666896.551724</v>
       </c>
       <c r="AO145" t="n">
         <v>0</v>
@@ -34638,7 +34638,7 @@
         <v>37.85</v>
       </c>
       <c r="H146" t="n">
-        <v>8542938000</v>
+        <v>8589801000</v>
       </c>
       <c r="I146" t="n">
         <v>400</v>
@@ -34656,7 +34656,7 @@
         <v>8.16</v>
       </c>
       <c r="N146" t="n">
-        <v>1.6648582330978</v>
+        <v>1.673990952002896</v>
       </c>
       <c r="O146" t="n">
         <v>0.58</v>
@@ -34734,7 +34734,7 @@
         <v>489015806.4</v>
       </c>
       <c r="AN146" t="n">
-        <v>2447833237.82235</v>
+        <v>2461261031.518624</v>
       </c>
       <c r="AO146" t="n">
         <v>0</v>
@@ -38633,7 +38633,7 @@
         <v>3.01</v>
       </c>
       <c r="H163" t="n">
-        <v>30016120</v>
+        <v>29666440</v>
       </c>
       <c r="I163" t="n">
         <v>0</v>
@@ -38651,7 +38651,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="N163" t="n">
-        <v>0.5594179147669563</v>
+        <v>0.5529008413931922</v>
       </c>
       <c r="O163" t="n">
         <v>0.07000000000000001</v>
@@ -38729,7 +38729,7 @@
         <v>8649345</v>
       </c>
       <c r="AN163" t="n">
-        <v>7504030</v>
+        <v>7416610</v>
       </c>
       <c r="AO163" t="n">
         <v>0</v>
@@ -38868,7 +38868,7 @@
         <v>4</v>
       </c>
       <c r="H164" t="n">
-        <v>30016120</v>
+        <v>29666440</v>
       </c>
       <c r="I164" t="n">
         <v>2200</v>
@@ -38886,7 +38886,7 @@
         <v>1.51</v>
       </c>
       <c r="N164" t="n">
-        <v>0.02797089573834782</v>
+        <v>0.02764504206965961</v>
       </c>
       <c r="O164" t="n">
         <v>0.11</v>
@@ -38964,7 +38964,7 @@
         <v>172986900</v>
       </c>
       <c r="AN164" t="n">
-        <v>4675408.099688473</v>
+        <v>4620940.809968848</v>
       </c>
       <c r="AO164" t="n">
         <v>0</v>
@@ -40748,7 +40748,7 @@
         <v>3.95</v>
       </c>
       <c r="H172" t="n">
-        <v>215243758</v>
+        <v>212736300</v>
       </c>
       <c r="I172" t="n">
         <v>2500</v>
@@ -40766,7 +40766,7 @@
         <v>0.38</v>
       </c>
       <c r="N172" t="n">
-        <v>0.04765643503893229</v>
+        <v>0.04710126674787388</v>
       </c>
       <c r="O172" t="n">
         <v>0.08</v>
@@ -40844,7 +40844,7 @@
         <v>640901679.6</v>
       </c>
       <c r="AN172" t="n">
-        <v>215243758</v>
+        <v>212736300</v>
       </c>
       <c r="AO172" t="n">
         <v>0</v>
@@ -42628,7 +42628,7 @@
         <v>36</v>
       </c>
       <c r="H180" t="n">
-        <v>3544396000</v>
+        <v>3519843000</v>
       </c>
       <c r="I180" t="n">
         <v>0</v>
@@ -42646,7 +42646,7 @@
         <v>12.71</v>
       </c>
       <c r="N180" t="n">
-        <v>8.659276391563147</v>
+        <v>8.599291216869899</v>
       </c>
       <c r="O180" t="n">
         <v>0.8</v>
@@ -42724,7 +42724,7 @@
         <v>84360399.48</v>
       </c>
       <c r="AN180" t="n">
-        <v>459714137.4837873</v>
+        <v>456529571.9844358</v>
       </c>
       <c r="AO180" t="n">
         <v>4.0605</v>
@@ -42863,7 +42863,7 @@
         <v>37.91</v>
       </c>
       <c r="H181" t="n">
-        <v>3544396000</v>
+        <v>3519843000</v>
       </c>
       <c r="I181" t="n">
         <v>300</v>
@@ -42881,7 +42881,7 @@
         <v>13.08</v>
       </c>
       <c r="N181" t="n">
-        <v>4.329638195781573</v>
+        <v>4.299645608434949</v>
       </c>
       <c r="O181" t="n">
         <v>0.83</v>
@@ -42959,7 +42959,7 @@
         <v>168720798.96</v>
       </c>
       <c r="AN181" t="n">
-        <v>446397481.1083123</v>
+        <v>443305163.7279597</v>
       </c>
       <c r="AO181" t="n">
         <v>4.0605</v>
@@ -45448,7 +45448,7 @@
         <v>2.39</v>
       </c>
       <c r="H192" t="n">
-        <v>21607225</v>
+        <v>21539000</v>
       </c>
       <c r="I192" t="n">
         <v>7400</v>
@@ -45466,7 +45466,7 @@
         <v>21.95</v>
       </c>
       <c r="N192" t="n">
-        <v>2.209141866178554</v>
+        <v>2.20216648161066</v>
       </c>
       <c r="O192" t="n">
         <v>0.32</v>
@@ -45544,7 +45544,7 @@
         <v>357000.03</v>
       </c>
       <c r="AN192" t="n">
-        <v>1817260.302775441</v>
+        <v>1811522.287636669</v>
       </c>
       <c r="AO192" t="n">
         <v>0</v>
@@ -45683,7 +45683,7 @@
         <v>1.52</v>
       </c>
       <c r="H193" t="n">
-        <v>21607225</v>
+        <v>21539000</v>
       </c>
       <c r="I193" t="n">
         <v>21900</v>
@@ -45701,7 +45701,7 @@
         <v>14.71</v>
       </c>
       <c r="N193" t="n">
-        <v>1.104571072320913</v>
+        <v>1.101083379597341</v>
       </c>
       <c r="O193" t="n">
         <v>0.22</v>
@@ -45779,7 +45779,7 @@
         <v>713999.97</v>
       </c>
       <c r="AN193" t="n">
-        <v>2711069.636135508</v>
+        <v>2702509.410288582</v>
       </c>
       <c r="AO193" t="n">
         <v>0</v>
@@ -46858,7 +46858,7 @@
         <v>32.4</v>
       </c>
       <c r="H198" t="n">
-        <v>299419624</v>
+        <v>295931500</v>
       </c>
       <c r="I198" t="n">
         <v>500</v>
@@ -46876,7 +46876,7 @@
         <v>8.289999999999999</v>
       </c>
       <c r="N198" t="n">
-        <v>6.614917971983695</v>
+        <v>6.537856709839743</v>
       </c>
       <c r="O198" t="n">
         <v>0.2</v>
@@ -46954,7 +46954,7 @@
         <v>26538458.42</v>
       </c>
       <c r="AN198" t="n">
-        <v>14713495.03685504</v>
+        <v>14542088.45208845</v>
       </c>
       <c r="AO198" t="n">
         <v>0</v>
@@ -48006,7 +48006,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>IBOVESPA</t>
+          <t>Brazil Stock Exchange Index</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
@@ -56242,7 +56242,7 @@
         <v>3.17</v>
       </c>
       <c r="H238" t="n">
-        <v>133323736</v>
+        <v>131770600</v>
       </c>
       <c r="I238" t="n">
         <v>48500</v>
@@ -56260,7 +56260,7 @@
         <v>4.2</v>
       </c>
       <c r="N238" t="n">
-        <v>1.556708735990338</v>
+        <v>1.538574077812284</v>
       </c>
       <c r="O238" t="n">
         <v>0.75</v>
@@ -56338,7 +56338,7 @@
         <v>23184000</v>
       </c>
       <c r="AN238" t="n">
-        <v>19266435.83815029</v>
+        <v>19041994.21965318</v>
       </c>
       <c r="AO238" t="n">
         <v>0</v>
@@ -58357,7 +58357,7 @@
         <v>5.14</v>
       </c>
       <c r="H247" t="n">
-        <v>19325207</v>
+        <v>19100080</v>
       </c>
       <c r="I247" t="n">
         <v>5900</v>
@@ -58375,7 +58375,7 @@
         <v>4.4</v>
       </c>
       <c r="N247" t="n">
-        <v>0.02908221025964313</v>
+        <v>0.02874342005940762</v>
       </c>
       <c r="O247" t="n">
         <v>0.05</v>
@@ -58453,7 +58453,7 @@
         <v>5648272.88</v>
       </c>
       <c r="AN247" t="n">
-        <v>32754588.13559322</v>
+        <v>32373016.94915254</v>
       </c>
       <c r="AO247" t="n">
         <v>0</v>
@@ -60707,7 +60707,7 @@
         <v>42.5</v>
       </c>
       <c r="H257" t="n">
-        <v>13500050000</v>
+        <v>13408320000</v>
       </c>
       <c r="I257" t="n">
         <v>200</v>
@@ -60725,7 +60725,7 @@
         <v>9.57</v>
       </c>
       <c r="N257" t="n">
-        <v>3.363600463160372</v>
+        <v>3.340745505550164</v>
       </c>
       <c r="O257" t="n">
         <v>0.64</v>
@@ -60803,7 +60803,7 @@
         <v>836829598.4699999</v>
       </c>
       <c r="AN257" t="n">
-        <v>2454554545.454545</v>
+        <v>2437876363.636364</v>
       </c>
       <c r="AO257" t="n">
         <v>0</v>
@@ -60942,7 +60942,7 @@
         <v>38</v>
       </c>
       <c r="H258" t="n">
-        <v>13500050000</v>
+        <v>13408320000</v>
       </c>
       <c r="I258" t="n">
         <v>0</v>
@@ -60960,7 +60960,7 @@
         <v>8.94</v>
       </c>
       <c r="N258" t="n">
-        <v>7.718044435468618</v>
+        <v>7.665601947028536</v>
       </c>
       <c r="O258" t="n">
         <v>0.59</v>
@@ -61038,7 +61038,7 @@
         <v>364698655.02</v>
       </c>
       <c r="AN258" t="n">
-        <v>2626468871.595331</v>
+        <v>2608622568.093385</v>
       </c>
       <c r="AO258" t="n">
         <v>0</v>
@@ -61177,7 +61177,7 @@
         <v>36.5</v>
       </c>
       <c r="H259" t="n">
-        <v>13500050000</v>
+        <v>13408320000</v>
       </c>
       <c r="I259" t="n">
         <v>0</v>
@@ -61195,7 +61195,7 @@
         <v>9.949999999999999</v>
       </c>
       <c r="N259" t="n">
-        <v>9.102510533753867</v>
+        <v>9.040660889399865</v>
       </c>
       <c r="O259" t="n">
         <v>0.66</v>
@@ -61273,7 +61273,7 @@
         <v>309229021.44</v>
       </c>
       <c r="AN259" t="n">
-        <v>2360148601.398602</v>
+        <v>2344111888.111888</v>
       </c>
       <c r="AO259" t="n">
         <v>0</v>
@@ -61647,7 +61647,7 @@
         <v>44.65</v>
       </c>
       <c r="H261" t="n">
-        <v>296391600</v>
+        <v>283157700</v>
       </c>
       <c r="I261" t="n">
         <v>700</v>
@@ -61665,7 +61665,7 @@
         <v>22.68</v>
       </c>
       <c r="N261" t="n">
-        <v>1.891684190871237</v>
+        <v>1.807220395630174</v>
       </c>
       <c r="O261" t="n">
         <v>0.21</v>
@@ -61743,7 +61743,7 @@
         <v>11657091.15</v>
       </c>
       <c r="AN261" t="n">
-        <v>19183922.33009709</v>
+        <v>18327359.22330097</v>
       </c>
       <c r="AO261" t="n">
         <v>0</v>
@@ -61882,7 +61882,7 @@
         <v>41</v>
       </c>
       <c r="H262" t="n">
-        <v>296391600</v>
+        <v>283157700</v>
       </c>
       <c r="I262" t="n">
         <v>0</v>
@@ -61900,7 +61900,7 @@
         <v>19.78</v>
       </c>
       <c r="N262" t="n">
-        <v>13.77228233889013</v>
+        <v>13.15734923267309</v>
       </c>
       <c r="O262" t="n">
         <v>0.18</v>
@@ -61978,7 +61978,7 @@
         <v>1601153.28</v>
       </c>
       <c r="AN262" t="n">
-        <v>21987507.41839762</v>
+        <v>21005764.09495549</v>
       </c>
       <c r="AO262" t="n">
         <v>0</v>
@@ -64232,7 +64232,7 @@
         <v>1.84</v>
       </c>
       <c r="H272" t="n">
-        <v>12327139</v>
+        <v>12183530</v>
       </c>
       <c r="I272" t="n">
         <v>2300</v>
@@ -64250,7 +64250,7 @@
         <v>0.96</v>
       </c>
       <c r="N272" t="n">
-        <v>4.727971957812885</v>
+        <v>4.672891916540571</v>
       </c>
       <c r="O272" t="n">
         <v>1.87</v>
@@ -64328,7 +64328,7 @@
         <v>37941114.78</v>
       </c>
       <c r="AN272" t="n">
-        <v>10908972.56637168</v>
+        <v>10781884.95575221</v>
       </c>
       <c r="AO272" t="n">
         <v>0</v>
@@ -66582,7 +66582,7 @@
         <v>31.8</v>
       </c>
       <c r="H282" t="n">
-        <v>771259055</v>
+        <v>759306300</v>
       </c>
       <c r="I282" t="n">
         <v>200</v>
@@ -66600,7 +66600,7 @@
         <v>17.82</v>
       </c>
       <c r="N282" t="n">
-        <v>0.3931085676909674</v>
+        <v>0.3870162821384677</v>
       </c>
       <c r="O282" t="n">
         <v>0.52</v>
@@ -66678,7 +66678,7 @@
         <v>42378103.55</v>
       </c>
       <c r="AN282" t="n">
-        <v>86078019.53124999</v>
+        <v>84744006.69642857</v>
       </c>
       <c r="AO282" t="n">
         <v>0</v>
@@ -66817,7 +66817,7 @@
         <v>30.1</v>
       </c>
       <c r="H283" t="n">
-        <v>771259055</v>
+        <v>759306300</v>
       </c>
       <c r="I283" t="n">
         <v>0</v>
@@ -66835,7 +66835,7 @@
         <v>18.34</v>
       </c>
       <c r="N283" t="n">
-        <v>8.782886519574156</v>
+        <v>8.646771824932065</v>
       </c>
       <c r="O283" t="n">
         <v>0.54</v>
@@ -66913,7 +66913,7 @@
         <v>1896779.1</v>
       </c>
       <c r="AN283" t="n">
-        <v>83560027.62730227</v>
+        <v>82265037.91982664</v>
       </c>
       <c r="AO283" t="n">
         <v>0</v>
@@ -71282,7 +71282,7 @@
         <v>75</v>
       </c>
       <c r="H302" t="n">
-        <v>474638</v>
+        <v>70366650</v>
       </c>
       <c r="I302" t="n">
         <v>2</v>
@@ -71375,10 +71375,10 @@
         <v>0</v>
       </c>
       <c r="AM302" t="n">
-        <v>3122.823869991447</v>
+        <v>462968.9453253503</v>
       </c>
       <c r="AN302" t="n">
-        <v>1898552</v>
+        <v>281466600</v>
       </c>
       <c r="AO302" t="n">
         <v>0</v>
@@ -75512,7 +75512,7 @@
         <v>5.97</v>
       </c>
       <c r="H320" t="n">
-        <v>15512895204</v>
+        <v>15332180000</v>
       </c>
       <c r="I320" t="n">
         <v>300</v>
@@ -75530,7 +75530,7 @@
         <v>11.35</v>
       </c>
       <c r="N320" t="n">
-        <v>0.7995248931327127</v>
+        <v>0.7902109448164564</v>
       </c>
       <c r="O320" t="n">
         <v>0.49</v>
@@ -75608,7 +75608,7 @@
         <v>1412512331.45</v>
       </c>
       <c r="AN320" t="n">
-        <v>3432056461.061947</v>
+        <v>3392075221.238938</v>
       </c>
       <c r="AO320" t="n">
         <v>0</v>
@@ -75982,7 +75982,7 @@
         <v>0.92</v>
       </c>
       <c r="H322" t="n">
-        <v>344910030</v>
+        <v>342684300</v>
       </c>
       <c r="I322" t="n">
         <v>14800</v>
@@ -76000,7 +76000,7 @@
         <v>2.24</v>
       </c>
       <c r="N322" t="n">
-        <v>0.8742066690382857</v>
+        <v>0.8685653485771828</v>
       </c>
       <c r="O322" t="n">
         <v>0.13</v>
@@ -76078,7 +76078,7 @@
         <v>142942061.98</v>
       </c>
       <c r="AN322" t="n">
-        <v>27748192.2767498</v>
+        <v>27569131.13435237</v>
       </c>
       <c r="AO322" t="n">
         <v>0</v>
@@ -76217,7 +76217,7 @@
         <v>0.91</v>
       </c>
       <c r="H323" t="n">
-        <v>344910030</v>
+        <v>342684300</v>
       </c>
       <c r="I323" t="n">
         <v>14600</v>
@@ -76235,7 +76235,7 @@
         <v>2</v>
       </c>
       <c r="N323" t="n">
-        <v>4.355456790280586</v>
+        <v>4.327350704638973</v>
       </c>
       <c r="O323" t="n">
         <v>0.11</v>
@@ -76313,7 +76313,7 @@
         <v>28690654.02</v>
       </c>
       <c r="AN323" t="n">
-        <v>31100994.58972047</v>
+        <v>30900297.56537421</v>
       </c>
       <c r="AO323" t="n">
         <v>0</v>
@@ -76687,7 +76687,7 @@
         <v>7.5</v>
       </c>
       <c r="H325" t="n">
-        <v>602458200</v>
+        <v>601599400</v>
       </c>
       <c r="I325" t="n">
         <v>0</v>
@@ -76783,7 +76783,7 @@
         <v>8742210.08</v>
       </c>
       <c r="AN325" t="n">
-        <v>6917650.706166035</v>
+        <v>6907789.642898151</v>
       </c>
       <c r="AO325" t="n">
         <v>0</v>
@@ -76922,7 +76922,7 @@
         <v>6.86</v>
       </c>
       <c r="H326" t="n">
-        <v>602458200</v>
+        <v>601599400</v>
       </c>
       <c r="I326" t="n">
         <v>200</v>
@@ -77018,7 +77018,7 @@
         <v>2719637.39</v>
       </c>
       <c r="AN326" t="n">
-        <v>5945506.760090793</v>
+        <v>5937031.481298727</v>
       </c>
       <c r="AO326" t="n">
         <v>0.4906</v>
@@ -77157,7 +77157,7 @@
         <v>6.5</v>
       </c>
       <c r="H327" t="n">
-        <v>602458200</v>
+        <v>601599400</v>
       </c>
       <c r="I327" t="n">
         <v>0</v>
@@ -77253,7 +77253,7 @@
         <v>4627783.64</v>
       </c>
       <c r="AN327" t="n">
-        <v>8741413.232733604</v>
+        <v>8728952.408589669</v>
       </c>
       <c r="AO327" t="n">
         <v>0</v>
@@ -77392,7 +77392,7 @@
         <v>1.41</v>
       </c>
       <c r="H328" t="n">
-        <v>96570220</v>
+        <v>95445200</v>
       </c>
       <c r="I328" t="n">
         <v>15000</v>
@@ -77410,7 +77410,7 @@
         <v>0.11</v>
       </c>
       <c r="N328" t="n">
-        <v>0.01116965910445202</v>
+        <v>0.01103953524343472</v>
       </c>
       <c r="O328" t="n">
         <v>0.02</v>
@@ -77488,7 +77488,7 @@
         <v>1659121826.79</v>
       </c>
       <c r="AN328" t="n">
-        <v>965702200</v>
+        <v>954452000</v>
       </c>
       <c r="AO328" t="n">
         <v>0</v>
@@ -83267,7 +83267,7 @@
         <v>38.66</v>
       </c>
       <c r="H353" t="n">
-        <v>157484087</v>
+        <v>153845000</v>
       </c>
       <c r="I353" t="n">
         <v>0</v>
@@ -83285,7 +83285,7 @@
         <v>3.42</v>
       </c>
       <c r="N353" t="n">
-        <v>2.049793912135059</v>
+        <v>2.002427993962452</v>
       </c>
       <c r="O353" t="n">
         <v>0.78</v>
@@ -83363,7 +83363,7 @@
         <v>9672800</v>
       </c>
       <c r="AN353" t="n">
-        <v>63501647.98387097</v>
+        <v>62034274.19354839</v>
       </c>
       <c r="AO353" t="n">
         <v>0</v>
@@ -83502,7 +83502,7 @@
         <v>77.56999999999999</v>
       </c>
       <c r="H354" t="n">
-        <v>157484087</v>
+        <v>153845000</v>
       </c>
       <c r="I354" t="n">
         <v>200</v>
@@ -83520,7 +83520,7 @@
         <v>6.19</v>
       </c>
       <c r="N354" t="n">
-        <v>2.236328815686478</v>
+        <v>2.184652514442848</v>
       </c>
       <c r="O354" t="n">
         <v>1.42</v>
@@ -83598,7 +83598,7 @@
         <v>8865980</v>
       </c>
       <c r="AN354" t="n">
-        <v>34996463.77777778</v>
+        <v>34187777.77777778</v>
       </c>
       <c r="AO354" t="n">
         <v>0</v>
@@ -83737,7 +83737,7 @@
         <v>79.98</v>
       </c>
       <c r="H355" t="n">
-        <v>157484087</v>
+        <v>153845000</v>
       </c>
       <c r="I355" t="n">
         <v>300</v>
@@ -83755,7 +83755,7 @@
         <v>6.02</v>
       </c>
       <c r="N355" t="n">
-        <v>2.146853773140353</v>
+        <v>2.097245029771025</v>
       </c>
       <c r="O355" t="n">
         <v>1.38</v>
@@ -83833,7 +83833,7 @@
         <v>9235490</v>
       </c>
       <c r="AN355" t="n">
-        <v>36037548.51258581</v>
+        <v>35204805.49199085</v>
       </c>
       <c r="AO355" t="n">
         <v>0</v>
@@ -86087,7 +86087,7 @@
         <v>11.99</v>
       </c>
       <c r="H365" t="n">
-        <v>1183612524</v>
+        <v>1150808000</v>
       </c>
       <c r="I365" t="n">
         <v>700</v>
@@ -86105,7 +86105,7 @@
         <v>20.34</v>
       </c>
       <c r="N365" t="n">
-        <v>3.131117120714704</v>
+        <v>3.044336350276272</v>
       </c>
       <c r="O365" t="n">
         <v>0.27</v>
@@ -86183,7 +86183,7 @@
         <v>45966751.6</v>
       </c>
       <c r="AN365" t="n">
-        <v>125916225.9574468</v>
+        <v>122426382.9787234</v>
       </c>
       <c r="AO365" t="n">
         <v>0</v>
@@ -86322,7 +86322,7 @@
         <v>8.08</v>
       </c>
       <c r="H366" t="n">
-        <v>1183612524</v>
+        <v>1150808000</v>
       </c>
       <c r="I366" t="n">
         <v>2700</v>
@@ -86340,7 +86340,7 @@
         <v>14.31</v>
       </c>
       <c r="N366" t="n">
-        <v>14.21627580546124</v>
+        <v>13.82226327906888</v>
       </c>
       <c r="O366" t="n">
         <v>0.19</v>
@@ -86418,7 +86418,7 @@
         <v>10124120.05</v>
       </c>
       <c r="AN366" t="n">
-        <v>179063921.9364599</v>
+        <v>174101059.0015129</v>
       </c>
       <c r="AO366" t="n">
         <v>0</v>
@@ -89612,7 +89612,7 @@
         <v>1.31</v>
       </c>
       <c r="H380" t="n">
-        <v>87593565</v>
+        <v>86573140</v>
       </c>
       <c r="I380" t="n">
         <v>27000</v>
@@ -89630,7 +89630,7 @@
         <v>39.8</v>
       </c>
       <c r="N380" t="n">
-        <v>0.3247330027870802</v>
+        <v>0.3209500117149734</v>
       </c>
       <c r="O380" t="n">
         <v>0.24</v>
@@ -89708,7 +89708,7 @@
         <v>2643454.56</v>
       </c>
       <c r="AN380" t="n">
-        <v>8271347.025495751</v>
+        <v>8174989.612842305</v>
       </c>
       <c r="AO380" t="n">
         <v>0</v>
@@ -92667,7 +92667,7 @@
         <v>0.32</v>
       </c>
       <c r="H393" t="n">
-        <v>15800194</v>
+        <v>15616130</v>
       </c>
       <c r="I393" t="n">
         <v>89000</v>
@@ -92685,7 +92685,7 @@
         <v>1.29</v>
       </c>
       <c r="N393" t="n">
-        <v>0.2818880884832905</v>
+        <v>0.2786042396192456</v>
       </c>
       <c r="O393" t="n">
         <v>0.13</v>
@@ -92763,7 +92763,7 @@
         <v>22936192.23</v>
       </c>
       <c r="AN393" t="n">
-        <v>10394864.47368421</v>
+        <v>10273769.73684211</v>
       </c>
       <c r="AO393" t="n">
         <v>0</v>
@@ -94547,7 +94547,7 @@
         <v>8.25</v>
       </c>
       <c r="H401" t="n">
-        <v>92732392</v>
+        <v>91652130</v>
       </c>
       <c r="I401" t="n">
         <v>3700</v>
@@ -94565,7 +94565,7 @@
         <v>5.91</v>
       </c>
       <c r="N401" t="n">
-        <v>0.6337418970147038</v>
+        <v>0.6263592848078183</v>
       </c>
       <c r="O401" t="n">
         <v>0.23</v>
@@ -94643,7 +94643,7 @@
         <v>11442628.44</v>
       </c>
       <c r="AN401" t="n">
-        <v>39799309.87124463</v>
+        <v>39335678.11158798</v>
       </c>
       <c r="AO401" t="n">
         <v>0</v>
@@ -94782,7 +94782,7 @@
         <v>3.86</v>
       </c>
       <c r="H402" t="n">
-        <v>6030555728</v>
+        <v>5857644000</v>
       </c>
       <c r="I402" t="n">
         <v>3500</v>
@@ -94800,7 +94800,7 @@
         <v>9.42</v>
       </c>
       <c r="N402" t="n">
-        <v>0.679777620971791</v>
+        <v>0.6602866273719451</v>
       </c>
       <c r="O402" t="n">
         <v>0.66</v>
@@ -94878,7 +94878,7 @@
         <v>483489419.2399999</v>
       </c>
       <c r="AN402" t="n">
-        <v>1157496300.959693</v>
+        <v>1124307869.481766</v>
       </c>
       <c r="AO402" t="n">
         <v>0</v>
@@ -95017,7 +95017,7 @@
         <v>3.98</v>
       </c>
       <c r="H403" t="n">
-        <v>6030555728</v>
+        <v>5857644000</v>
       </c>
       <c r="I403" t="n">
         <v>9500</v>
@@ -95035,7 +95035,7 @@
         <v>9.92</v>
       </c>
       <c r="N403" t="n">
-        <v>1.475025948727256</v>
+        <v>1.432733115837068</v>
       </c>
       <c r="O403" t="n">
         <v>0.6899999999999999</v>
@@ -95113,7 +95113,7 @@
         <v>222820003.58</v>
       </c>
       <c r="AN403" t="n">
-        <v>1100466373.722628</v>
+        <v>1068913138.686131</v>
       </c>
       <c r="AO403" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-06-15 06:26
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1770,7 +1770,7 @@
         <v>7.69</v>
       </c>
       <c r="H6" t="n">
-        <v>485121269</v>
+        <v>485121300</v>
       </c>
       <c r="I6" t="n">
         <v>100</v>
@@ -1788,7 +1788,7 @@
         <v>13.39</v>
       </c>
       <c r="N6" t="n">
-        <v>5.984217268990593</v>
+        <v>5.984217651391339</v>
       </c>
       <c r="O6" t="n">
         <v>1.24</v>
@@ -1866,7 +1866,7 @@
         <v>34696585</v>
       </c>
       <c r="AN6" t="n">
-        <v>52051638.30472103</v>
+        <v>52051641.63090128</v>
       </c>
       <c r="AO6" t="n">
         <v>0</v>
@@ -7394,7 +7394,7 @@
         <v>0.54</v>
       </c>
       <c r="H30" t="n">
-        <v>105478204</v>
+        <v>2636955000</v>
       </c>
       <c r="I30" t="n">
         <v>4800</v>
@@ -7412,7 +7412,7 @@
         <v>1.36</v>
       </c>
       <c r="N30" t="n">
-        <v>0.1615573327227789</v>
+        <v>4.038933164902917</v>
       </c>
       <c r="O30" t="n">
         <v>0.12</v>
@@ -7490,7 +7490,7 @@
         <v>119151337.21</v>
       </c>
       <c r="AN30" t="n">
-        <v>81766049.61240309</v>
+        <v>2044151162.790698</v>
       </c>
       <c r="AO30" t="n">
         <v>0</v>
@@ -8804,7 +8804,7 @@
         <v>26</v>
       </c>
       <c r="H36" t="n">
-        <v>214269120</v>
+        <v>215600000</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
@@ -8822,7 +8822,7 @@
         <v>10.3</v>
       </c>
       <c r="N36" t="n">
-        <v>1.957366110787172</v>
+        <v>1.969523809523809</v>
       </c>
       <c r="O36" t="n">
         <v>0.85</v>
@@ -8900,7 +8900,7 @@
         <v>12348000</v>
       </c>
       <c r="AN36" t="n">
-        <v>38330790.69767442</v>
+        <v>38568872.98747764</v>
       </c>
       <c r="AO36" t="n">
         <v>0</v>
@@ -9039,7 +9039,7 @@
         <v>18</v>
       </c>
       <c r="H37" t="n">
-        <v>214269120</v>
+        <v>215600000</v>
       </c>
       <c r="I37" t="n">
         <v>1800</v>
@@ -9057,7 +9057,7 @@
         <v>7.41</v>
       </c>
       <c r="N37" t="n">
-        <v>1.957366110787172</v>
+        <v>1.969523809523809</v>
       </c>
       <c r="O37" t="n">
         <v>0.61</v>
@@ -9135,7 +9135,7 @@
         <v>12348000</v>
       </c>
       <c r="AN37" t="n">
-        <v>53300776.11940299</v>
+        <v>53631840.7960199</v>
       </c>
       <c r="AO37" t="n">
         <v>0</v>
@@ -11389,7 +11389,7 @@
         <v>8.76</v>
       </c>
       <c r="H47" t="n">
-        <v>3035672083</v>
+        <v>3037598000</v>
       </c>
       <c r="I47" t="n">
         <v>4600</v>
@@ -11407,7 +11407,7 @@
         <v>8.390000000000001</v>
       </c>
       <c r="N47" t="n">
-        <v>0.8143091189914718</v>
+        <v>0.8148257399349207</v>
       </c>
       <c r="O47" t="n">
         <v>0.07000000000000001</v>
@@ -11485,7 +11485,7 @@
         <v>249024468</v>
       </c>
       <c r="AN47" t="n">
-        <v>462050545.3576865</v>
+        <v>462343683.4094368</v>
       </c>
       <c r="AO47" t="n">
         <v>0.3403</v>
@@ -11624,7 +11624,7 @@
         <v>8.69</v>
       </c>
       <c r="H48" t="n">
-        <v>3035672083</v>
+        <v>3037598000</v>
       </c>
       <c r="I48" t="n">
         <v>2700</v>
@@ -11642,7 +11642,7 @@
         <v>8.449999999999999</v>
       </c>
       <c r="N48" t="n">
-        <v>2.215489918502981</v>
+        <v>2.216895488531861</v>
       </c>
       <c r="O48" t="n">
         <v>0.07000000000000001</v>
@@ -11720,7 +11720,7 @@
         <v>91529595.08</v>
       </c>
       <c r="AN48" t="n">
-        <v>458560737.6132931</v>
+        <v>458851661.63142</v>
       </c>
       <c r="AO48" t="n">
         <v>0.3691</v>
@@ -13896,7 +13896,7 @@
         <v>0.66</v>
       </c>
       <c r="BM57" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="BN57" t="n">
         <v>5.19</v>
@@ -13911,7 +13911,7 @@
         <v>5.07</v>
       </c>
       <c r="BR57" t="n">
-        <v>5.29</v>
+        <v>5.19</v>
       </c>
       <c r="BS57" t="n">
         <v>5.1</v>
@@ -14428,7 +14428,7 @@
         <v>390.95</v>
       </c>
       <c r="H60" t="n">
-        <v>178240404</v>
+        <v>177784500</v>
       </c>
       <c r="I60" t="n">
         <v>16</v>
@@ -14446,7 +14446,7 @@
         <v>2.87</v>
       </c>
       <c r="N60" t="n">
-        <v>12.59559608244657</v>
+        <v>12.5633790176986</v>
       </c>
       <c r="O60" t="n">
         <v>0.64</v>
@@ -14524,7 +14524,7 @@
         <v>59731412.5</v>
       </c>
       <c r="AN60" t="n">
-        <v>22448413.60201511</v>
+        <v>22390994.96221662</v>
       </c>
       <c r="AO60" t="n">
         <v>0</v>
@@ -14898,7 +14898,7 @@
         <v>105.25</v>
       </c>
       <c r="H62" t="n">
-        <v>10388145530</v>
+        <v>10388150000</v>
       </c>
       <c r="I62" t="n">
         <v>900</v>
@@ -14916,7 +14916,7 @@
         <v>4.26</v>
       </c>
       <c r="N62" t="n">
-        <v>1.061699862876002</v>
+        <v>1.061700319723509</v>
       </c>
       <c r="O62" t="n">
         <v>0.17</v>
@@ -14994,7 +14994,7 @@
         <v>2822812821.4</v>
       </c>
       <c r="AN62" t="n">
-        <v>4257436692.622951</v>
+        <v>4257438524.590164</v>
       </c>
       <c r="AO62" t="n">
         <v>0</v>
@@ -18658,7 +18658,7 @@
         <v>2.7</v>
       </c>
       <c r="H78" t="n">
-        <v>1182619730</v>
+        <v>0</v>
       </c>
       <c r="I78" t="n">
         <v>375700</v>
@@ -18676,7 +18676,7 @@
         <v>11.86</v>
       </c>
       <c r="N78" t="n">
-        <v>0.8785380010305798</v>
+        <v>0</v>
       </c>
       <c r="O78" t="n">
         <v>0.34</v>
@@ -18754,7 +18754,7 @@
         <v>113881959.62</v>
       </c>
       <c r="AN78" t="n">
-        <v>176247351.7138599</v>
+        <v>0</v>
       </c>
       <c r="AO78" t="n">
         <v>0</v>
@@ -20491,7 +20491,7 @@
         <v>0</v>
       </c>
       <c r="BR85" t="n">
-        <v>26.5</v>
+        <v>29</v>
       </c>
       <c r="BS85" t="n">
         <v>0</v>
@@ -20773,7 +20773,7 @@
         <v>19.9</v>
       </c>
       <c r="H87" t="n">
-        <v>9019155437</v>
+        <v>9019156000</v>
       </c>
       <c r="I87" t="n">
         <v>100</v>
@@ -20791,7 +20791,7 @@
         <v>7.13</v>
       </c>
       <c r="N87" t="n">
-        <v>0.962351452736847</v>
+        <v>0.9623515128094193</v>
       </c>
       <c r="O87" t="n">
         <v>0.21</v>
@@ -20869,7 +20869,7 @@
         <v>580126647.04</v>
       </c>
       <c r="AN87" t="n">
-        <v>1642833412.932605</v>
+        <v>1642833515.482696</v>
       </c>
       <c r="AO87" t="n">
         <v>0</v>
@@ -22418,7 +22418,7 @@
         <v>48</v>
       </c>
       <c r="H94" t="n">
-        <v>8130706000</v>
+        <v>8466620000</v>
       </c>
       <c r="I94" t="n">
         <v>100</v>
@@ -22436,7 +22436,7 @@
         <v>5.78</v>
       </c>
       <c r="N94" t="n">
-        <v>0.7634081022363698</v>
+        <v>0.794947733512501</v>
       </c>
       <c r="O94" t="n">
         <v>0.36</v>
@@ -22514,7 +22514,7 @@
         <v>1209900967.64</v>
       </c>
       <c r="AN94" t="n">
-        <v>2924714388.489209</v>
+        <v>3045546762.589928</v>
       </c>
       <c r="AO94" t="n">
         <v>0</v>
@@ -22653,7 +22653,7 @@
         <v>43.01</v>
       </c>
       <c r="H95" t="n">
-        <v>8130706000</v>
+        <v>8466620000</v>
       </c>
       <c r="I95" t="n">
         <v>0</v>
@@ -22671,7 +22671,7 @@
         <v>4.65</v>
       </c>
       <c r="N95" t="n">
-        <v>4.262891700647628</v>
+        <v>4.439009863416192</v>
       </c>
       <c r="O95" t="n">
         <v>0.29</v>
@@ -22749,7 +22749,7 @@
         <v>216671749.24</v>
       </c>
       <c r="AN95" t="n">
-        <v>3629779464.285714</v>
+        <v>3779741071.428571</v>
       </c>
       <c r="AO95" t="n">
         <v>0</v>
@@ -23593,7 +23593,7 @@
         <v>124.99</v>
       </c>
       <c r="H99" t="n">
-        <v>16722962679</v>
+        <v>16644280000</v>
       </c>
       <c r="I99" t="n">
         <v>0</v>
@@ -23611,7 +23611,7 @@
         <v>10.65</v>
       </c>
       <c r="N99" t="n">
-        <v>1.652333949511368</v>
+        <v>1.64455960567973</v>
       </c>
       <c r="O99" t="n">
         <v>1.16</v>
@@ -23689,7 +23689,7 @@
         <v>1267125769.6</v>
       </c>
       <c r="AN99" t="n">
-        <v>2878306829.432014</v>
+        <v>2864764199.655766</v>
       </c>
       <c r="AO99" t="n">
         <v>0</v>
@@ -23828,7 +23828,7 @@
         <v>127.8</v>
       </c>
       <c r="H100" t="n">
-        <v>16722962679</v>
+        <v>16644280000</v>
       </c>
       <c r="I100" t="n">
         <v>1600</v>
@@ -23846,7 +23846,7 @@
         <v>10.81</v>
       </c>
       <c r="N100" t="n">
-        <v>5.988452144827315</v>
+        <v>5.960276069399604</v>
       </c>
       <c r="O100" t="n">
         <v>1.18</v>
@@ -23924,7 +23924,7 @@
         <v>349625391.8</v>
       </c>
       <c r="AN100" t="n">
-        <v>2834400454.067796</v>
+        <v>2821064406.779661</v>
       </c>
       <c r="AO100" t="n">
         <v>0</v>
@@ -24063,7 +24063,7 @@
         <v>24.4</v>
       </c>
       <c r="H101" t="n">
-        <v>624175052</v>
+        <v>622711400</v>
       </c>
       <c r="I101" t="n">
         <v>1000</v>
@@ -24081,7 +24081,7 @@
         <v>6.28</v>
       </c>
       <c r="N101" t="n">
-        <v>2.013049148227628</v>
+        <v>2.008328672132885</v>
       </c>
       <c r="O101" t="n">
         <v>0.49</v>
@@ -24159,7 +24159,7 @@
         <v>42633867</v>
       </c>
       <c r="AN101" t="n">
-        <v>64547575.18097208</v>
+        <v>64396215.09824198</v>
       </c>
       <c r="AO101" t="n">
         <v>0</v>
@@ -24298,7 +24298,7 @@
         <v>24.29</v>
       </c>
       <c r="H102" t="n">
-        <v>624175052</v>
+        <v>622711400</v>
       </c>
       <c r="I102" t="n">
         <v>5300</v>
@@ -24316,7 +24316,7 @@
         <v>6.32</v>
       </c>
       <c r="N102" t="n">
-        <v>1.472776471640407</v>
+        <v>1.469322901650126</v>
       </c>
       <c r="O102" t="n">
         <v>0.49</v>
@@ -24394,7 +24394,7 @@
         <v>58273656.12</v>
       </c>
       <c r="AN102" t="n">
-        <v>64149542.85714285</v>
+        <v>63999116.1356629</v>
       </c>
       <c r="AO102" t="n">
         <v>0</v>
@@ -28763,7 +28763,7 @@
         <v>0.58</v>
       </c>
       <c r="H121" t="n">
-        <v>15220214</v>
+        <v>15492010</v>
       </c>
       <c r="I121" t="n">
         <v>19200</v>
@@ -28781,7 +28781,7 @@
         <v>0.19</v>
       </c>
       <c r="N121" t="n">
-        <v>0.03514507341214292</v>
+        <v>0.03577267893550328</v>
       </c>
       <c r="O121" t="n">
         <v>0.02</v>
@@ -28859,7 +28859,7 @@
         <v>129011019.48</v>
       </c>
       <c r="AN121" t="n">
-        <v>5090372.575250836</v>
+        <v>5181274.247491638</v>
       </c>
       <c r="AO121" t="n">
         <v>0</v>
@@ -32288,7 +32288,7 @@
         <v>6.51</v>
       </c>
       <c r="H136" t="n">
-        <v>432203600</v>
+        <v>432627200</v>
       </c>
       <c r="I136" t="n">
         <v>0</v>
@@ -32306,7 +32306,7 @@
         <v>89.8</v>
       </c>
       <c r="N136" t="n">
-        <v>1.008881952158698</v>
+        <v>1.009870750944581</v>
       </c>
       <c r="O136" t="n">
         <v>0.49</v>
@@ -32384,7 +32384,7 @@
         <v>3812747.4</v>
       </c>
       <c r="AN136" t="n">
-        <v>7306907.8613694</v>
+        <v>7314069.315300085</v>
       </c>
       <c r="AO136" t="n">
         <v>0</v>
@@ -32523,7 +32523,7 @@
         <v>3.77</v>
       </c>
       <c r="H137" t="n">
-        <v>432203600</v>
+        <v>432627200</v>
       </c>
       <c r="I137" t="n">
         <v>100</v>
@@ -32541,7 +32541,7 @@
         <v>51.86</v>
       </c>
       <c r="N137" t="n">
-        <v>2.594814845470342</v>
+        <v>2.597358007000096</v>
       </c>
       <c r="O137" t="n">
         <v>0.29</v>
@@ -32619,7 +32619,7 @@
         <v>1482422.55</v>
       </c>
       <c r="AN137" t="n">
-        <v>12648627.45098039</v>
+        <v>12661024.29031314</v>
       </c>
       <c r="AO137" t="n">
         <v>0</v>
@@ -34403,7 +34403,7 @@
         <v>51.52</v>
       </c>
       <c r="H145" t="n">
-        <v>8462453000</v>
+        <v>8563313000</v>
       </c>
       <c r="I145" t="n">
         <v>0</v>
@@ -34421,7 +34421,7 @@
         <v>10.18</v>
       </c>
       <c r="N145" t="n">
-        <v>1.828615311893232</v>
+        <v>1.850409718356412</v>
       </c>
       <c r="O145" t="n">
         <v>0.73</v>
@@ -34499,7 +34499,7 @@
         <v>441028665.6</v>
       </c>
       <c r="AN145" t="n">
-        <v>1945391494.252874</v>
+        <v>1968577701.149426</v>
       </c>
       <c r="AO145" t="n">
         <v>0</v>
@@ -34638,7 +34638,7 @@
         <v>37.59</v>
       </c>
       <c r="H146" t="n">
-        <v>8462453000</v>
+        <v>8563313000</v>
       </c>
       <c r="I146" t="n">
         <v>300</v>
@@ -34656,7 +34656,7 @@
         <v>8.16</v>
       </c>
       <c r="N146" t="n">
-        <v>1.649173217604199</v>
+        <v>1.668828938082358</v>
       </c>
       <c r="O146" t="n">
         <v>0.58</v>
@@ -34734,7 +34734,7 @@
         <v>489015806.4</v>
       </c>
       <c r="AN146" t="n">
-        <v>2424771633.237822</v>
+        <v>2453671346.704871</v>
       </c>
       <c r="AO146" t="n">
         <v>0</v>
@@ -38398,7 +38398,7 @@
         <v>0.73</v>
       </c>
       <c r="H162" t="n">
-        <v>263838796</v>
+        <v>2638387968</v>
       </c>
       <c r="I162" t="n">
         <v>474000</v>
@@ -38416,7 +38416,7 @@
         <v>28.13</v>
       </c>
       <c r="N162" t="n">
-        <v>0.2554999591531327</v>
+        <v>2.554999599278481</v>
       </c>
       <c r="O162" t="n">
         <v>0.14</v>
@@ -38494,7 +38494,7 @@
         <v>10842691.98</v>
       </c>
       <c r="AN162" t="n">
-        <v>129332743.1372549</v>
+        <v>1293327435.294118</v>
       </c>
       <c r="AO162" t="n">
         <v>0.0376</v>
@@ -38586,7 +38586,7 @@
         <v>0.71</v>
       </c>
       <c r="BR162" t="n">
-        <v>16.93</v>
+        <v>169.26</v>
       </c>
       <c r="BS162" t="n">
         <v>0.73</v>
@@ -40748,7 +40748,7 @@
         <v>3.9</v>
       </c>
       <c r="H172" t="n">
-        <v>210043358</v>
+        <v>210043400</v>
       </c>
       <c r="I172" t="n">
         <v>400</v>
@@ -40766,7 +40766,7 @@
         <v>0.38</v>
       </c>
       <c r="N172" t="n">
-        <v>0.04650503103502867</v>
+        <v>0.04650504033411492</v>
       </c>
       <c r="O172" t="n">
         <v>0.08</v>
@@ -40844,7 +40844,7 @@
         <v>640901679.6</v>
       </c>
       <c r="AN172" t="n">
-        <v>210043358</v>
+        <v>210043400</v>
       </c>
       <c r="AO172" t="n">
         <v>0</v>
@@ -45448,7 +45448,7 @@
         <v>2.42</v>
       </c>
       <c r="H192" t="n">
-        <v>21721559</v>
+        <v>21658000</v>
       </c>
       <c r="I192" t="n">
         <v>0</v>
@@ -45466,7 +45466,7 @@
         <v>21.95</v>
       </c>
       <c r="N192" t="n">
-        <v>2.220831475840492</v>
+        <v>2.214333147254917</v>
       </c>
       <c r="O192" t="n">
         <v>0.32</v>
@@ -45544,7 +45544,7 @@
         <v>357000.03</v>
       </c>
       <c r="AN192" t="n">
-        <v>1826876.282590412</v>
+        <v>1821530.698065601</v>
       </c>
       <c r="AO192" t="n">
         <v>0</v>
@@ -45683,7 +45683,7 @@
         <v>1.52</v>
       </c>
       <c r="H193" t="n">
-        <v>21721559</v>
+        <v>21658000</v>
       </c>
       <c r="I193" t="n">
         <v>1400</v>
@@ -45701,7 +45701,7 @@
         <v>14.71</v>
       </c>
       <c r="N193" t="n">
-        <v>1.110415877888622</v>
+        <v>1.107166713186277</v>
       </c>
       <c r="O193" t="n">
         <v>0.22</v>
@@ -45779,7 +45779,7 @@
         <v>713999.97</v>
       </c>
       <c r="AN193" t="n">
-        <v>2725415.181932246</v>
+        <v>2717440.401505646</v>
       </c>
       <c r="AO193" t="n">
         <v>0</v>
@@ -47563,7 +47563,7 @@
         <v>7.25</v>
       </c>
       <c r="H201" t="n">
-        <v>133199900</v>
+        <v>133200000</v>
       </c>
       <c r="I201" t="n">
         <v>800</v>
@@ -47581,7 +47581,7 @@
         <v>1.99</v>
       </c>
       <c r="N201" t="n">
-        <v>1.572001272974093</v>
+        <v>1.572002453156115</v>
       </c>
       <c r="O201" t="n">
         <v>0.25</v>
@@ -47659,7 +47659,7 @@
         <v>28893848.04</v>
       </c>
       <c r="AN201" t="n">
-        <v>105714206.3492063</v>
+        <v>105714285.7142857</v>
       </c>
       <c r="AO201" t="n">
         <v>0</v>
@@ -48006,7 +48006,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>IBOVESPA</t>
+          <t>Brazil Stock Exchange Index</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
@@ -56242,7 +56242,7 @@
         <v>3.17</v>
       </c>
       <c r="H238" t="n">
-        <v>131770594</v>
+        <v>131770600</v>
       </c>
       <c r="I238" t="n">
         <v>1000</v>
@@ -56260,7 +56260,7 @@
         <v>4.2</v>
       </c>
       <c r="N238" t="n">
-        <v>1.538574007755348</v>
+        <v>1.538574077812284</v>
       </c>
       <c r="O238" t="n">
         <v>0.75</v>
@@ -56338,7 +56338,7 @@
         <v>23184000</v>
       </c>
       <c r="AN238" t="n">
-        <v>19041993.35260116</v>
+        <v>19041994.21965318</v>
       </c>
       <c r="AO238" t="n">
         <v>0</v>
@@ -58357,7 +58357,7 @@
         <v>5.38</v>
       </c>
       <c r="H247" t="n">
-        <v>19991908</v>
+        <v>19991910</v>
       </c>
       <c r="I247" t="n">
         <v>17100</v>
@@ -58375,7 +58375,7 @@
         <v>4.4</v>
       </c>
       <c r="N247" t="n">
-        <v>0.03008551846029082</v>
+        <v>0.03008552147006043</v>
       </c>
       <c r="O247" t="n">
         <v>0.05</v>
@@ -58453,7 +58453,7 @@
         <v>5648272.88</v>
       </c>
       <c r="AN247" t="n">
-        <v>33884589.83050848</v>
+        <v>33884593.22033899</v>
       </c>
       <c r="AO247" t="n">
         <v>0</v>
@@ -59767,7 +59767,7 @@
         <v>18.49</v>
       </c>
       <c r="H253" t="n">
-        <v>183439990</v>
+        <v>183440000</v>
       </c>
       <c r="I253" t="n">
         <v>800</v>
@@ -59785,7 +59785,7 @@
         <v>7.29</v>
       </c>
       <c r="N253" t="n">
-        <v>0.1833967083768231</v>
+        <v>0.1833967183744636</v>
       </c>
       <c r="O253" t="n">
         <v>0.12</v>
@@ -59863,7 +59863,7 @@
         <v>24405758.4</v>
       </c>
       <c r="AN253" t="n">
-        <v>126510337.9310345</v>
+        <v>126510344.8275862</v>
       </c>
       <c r="AO253" t="n">
         <v>0</v>
@@ -60002,7 +60002,7 @@
         <v>3.97</v>
       </c>
       <c r="H254" t="n">
-        <v>281873972</v>
+        <v>281874000</v>
       </c>
       <c r="I254" t="n">
         <v>1100</v>
@@ -60020,7 +60020,7 @@
         <v>0.59</v>
       </c>
       <c r="N254" t="n">
-        <v>0.6591391588378182</v>
+        <v>0.6591392243135211</v>
       </c>
       <c r="O254" t="n">
         <v>0.6899999999999999</v>
@@ -60098,7 +60098,7 @@
         <v>520437330</v>
       </c>
       <c r="AN254" t="n">
-        <v>179537561.7834395</v>
+        <v>179537579.6178344</v>
       </c>
       <c r="AO254" t="n">
         <v>0</v>
@@ -66118,7 +66118,7 @@
         <v>1947900</v>
       </c>
       <c r="J280" t="n">
-        <v>96126871</v>
+        <v>137324101</v>
       </c>
       <c r="K280" t="n">
         <v>0</v>
@@ -66130,7 +66130,7 @@
         <v>227.17</v>
       </c>
       <c r="N280" t="n">
-        <v>10.20250171746332</v>
+        <v>7.141751224512841</v>
       </c>
       <c r="O280" t="n">
         <v>1.63</v>
@@ -66202,10 +66202,10 @@
         <v>59.79</v>
       </c>
       <c r="AL280" t="n">
-        <v>1032234856.375839</v>
+        <v>1474621218.791946</v>
       </c>
       <c r="AM280" t="n">
-        <v>30760598.72</v>
+        <v>43943712.32</v>
       </c>
       <c r="AN280" t="n">
         <v>417084273.0693069</v>
@@ -71282,7 +71282,7 @@
         <v>75.48</v>
       </c>
       <c r="H302" t="n">
-        <v>472053</v>
+        <v>472050</v>
       </c>
       <c r="I302" t="n">
         <v>25</v>
@@ -71375,10 +71375,10 @@
         <v>0</v>
       </c>
       <c r="AM302" t="n">
-        <v>3105.816172116587</v>
+        <v>3105.796433975919</v>
       </c>
       <c r="AN302" t="n">
-        <v>1888212</v>
+        <v>1888200</v>
       </c>
       <c r="AO302" t="n">
         <v>0</v>
@@ -75048,7 +75048,7 @@
         <v>5526000</v>
       </c>
       <c r="J318" t="n">
-        <v>2289292590</v>
+        <v>2240292590</v>
       </c>
       <c r="K318" t="n">
         <v>10.34</v>
@@ -75060,7 +75060,7 @@
         <v>21.41</v>
       </c>
       <c r="N318" t="n">
-        <v>1.407943109626357</v>
+        <v>1.438737842724899</v>
       </c>
       <c r="O318" t="n">
         <v>0.86</v>
@@ -75132,10 +75132,10 @@
         <v>30.64</v>
       </c>
       <c r="AL318" t="n">
-        <v>54227443523.80952</v>
+        <v>53066759763.12576</v>
       </c>
       <c r="AM318" t="n">
-        <v>4441227624.599999</v>
+        <v>4346167624.599999</v>
       </c>
       <c r="AN318" t="n">
         <v>7216366300.756144</v>
@@ -75512,7 +75512,7 @@
         <v>5.89</v>
       </c>
       <c r="H320" t="n">
-        <v>15126727107</v>
+        <v>15126720000</v>
       </c>
       <c r="I320" t="n">
         <v>700</v>
@@ -75530,7 +75530,7 @@
         <v>11.35</v>
       </c>
       <c r="N320" t="n">
-        <v>0.7796220315182297</v>
+        <v>0.7796216652279054</v>
       </c>
       <c r="O320" t="n">
         <v>0.49</v>
@@ -75608,7 +75608,7 @@
         <v>1412512331.45</v>
       </c>
       <c r="AN320" t="n">
-        <v>3346621041.371682</v>
+        <v>3346619469.026549</v>
       </c>
       <c r="AO320" t="n">
         <v>0</v>
@@ -75982,7 +75982,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="H322" t="n">
-        <v>350126875</v>
+        <v>347652700</v>
       </c>
       <c r="I322" t="n">
         <v>86900</v>
@@ -76000,7 +76000,7 @@
         <v>2.24</v>
       </c>
       <c r="N322" t="n">
-        <v>0.8874292496931279</v>
+        <v>0.8811582221867147</v>
       </c>
       <c r="O322" t="n">
         <v>0.13</v>
@@ -76078,7 +76078,7 @@
         <v>142942061.98</v>
       </c>
       <c r="AN322" t="n">
-        <v>28167890.1850362</v>
+        <v>27968841.51246983</v>
       </c>
       <c r="AO322" t="n">
         <v>0</v>
@@ -76217,7 +76217,7 @@
         <v>0.89</v>
       </c>
       <c r="H323" t="n">
-        <v>350126875</v>
+        <v>347652700</v>
       </c>
       <c r="I323" t="n">
         <v>48100</v>
@@ -76235,7 +76235,7 @@
         <v>2</v>
       </c>
       <c r="N323" t="n">
-        <v>4.421334094512914</v>
+        <v>4.39009069372201</v>
       </c>
       <c r="O323" t="n">
         <v>0.11</v>
@@ -76313,7 +76313,7 @@
         <v>28690654.02</v>
       </c>
       <c r="AN323" t="n">
-        <v>31571404.41839495</v>
+        <v>31348304.77908025</v>
       </c>
       <c r="AO323" t="n">
         <v>0</v>
@@ -76687,7 +76687,7 @@
         <v>6.91</v>
       </c>
       <c r="H325" t="n">
-        <v>574309400</v>
+        <v>574595600</v>
       </c>
       <c r="I325" t="n">
         <v>0</v>
@@ -76783,7 +76783,7 @@
         <v>8742210.08</v>
       </c>
       <c r="AN325" t="n">
-        <v>6594435.641290619</v>
+        <v>6597721.896888277</v>
       </c>
       <c r="AO325" t="n">
         <v>0</v>
@@ -76922,7 +76922,7 @@
         <v>6.87</v>
       </c>
       <c r="H326" t="n">
-        <v>574309400</v>
+        <v>574595600</v>
       </c>
       <c r="I326" t="n">
         <v>100</v>
@@ -77018,7 +77018,7 @@
         <v>2719637.39</v>
       </c>
       <c r="AN326" t="n">
-        <v>5667713.411625382</v>
+        <v>5670537.846639692</v>
       </c>
       <c r="AO326" t="n">
         <v>0.4906</v>
@@ -77157,7 +77157,7 @@
         <v>6.5</v>
       </c>
       <c r="H327" t="n">
-        <v>574309400</v>
+        <v>574595600</v>
       </c>
       <c r="I327" t="n">
         <v>0</v>
@@ -77253,7 +77253,7 @@
         <v>4627783.64</v>
       </c>
       <c r="AN327" t="n">
-        <v>8332986.070806732</v>
+        <v>8337138.711549623</v>
       </c>
       <c r="AO327" t="n">
         <v>0</v>
@@ -77392,7 +77392,7 @@
         <v>1.38</v>
       </c>
       <c r="H328" t="n">
-        <v>93414449</v>
+        <v>93414450</v>
       </c>
       <c r="I328" t="n">
         <v>1600</v>
@@ -77410,7 +77410,7 @@
         <v>0.11</v>
       </c>
       <c r="N328" t="n">
-        <v>0.01080465127614102</v>
+        <v>0.01080465139180462</v>
       </c>
       <c r="O328" t="n">
         <v>0.02</v>
@@ -77488,7 +77488,7 @@
         <v>1659121826.79</v>
       </c>
       <c r="AN328" t="n">
-        <v>934144490</v>
+        <v>934144500</v>
       </c>
       <c r="AO328" t="n">
         <v>0</v>
@@ -79977,7 +79977,7 @@
         <v>12.27</v>
       </c>
       <c r="H339" t="n">
-        <v>708436820</v>
+        <v>708436900</v>
       </c>
       <c r="I339" t="n">
         <v>3900</v>
@@ -79995,7 +79995,7 @@
         <v>14.33</v>
       </c>
       <c r="N339" t="n">
-        <v>1.783779976847498</v>
+        <v>1.783780178280278</v>
       </c>
       <c r="O339" t="n">
         <v>0.31</v>
@@ -80073,7 +80073,7 @@
         <v>61201558.14</v>
       </c>
       <c r="AN339" t="n">
-        <v>57973553.19148936</v>
+        <v>57973559.73813421</v>
       </c>
       <c r="AO339" t="n">
         <v>0</v>
@@ -86087,7 +86087,7 @@
         <v>11.1</v>
       </c>
       <c r="H365" t="n">
-        <v>1040445785</v>
+        <v>1074768000</v>
       </c>
       <c r="I365" t="n">
         <v>1300</v>
@@ -86105,7 +86105,7 @@
         <v>20.34</v>
       </c>
       <c r="N365" t="n">
-        <v>2.752385214360024</v>
+        <v>2.843180869887704</v>
       </c>
       <c r="O365" t="n">
         <v>0.27</v>
@@ -86183,7 +86183,7 @@
         <v>45966751.6</v>
       </c>
       <c r="AN365" t="n">
-        <v>110685721.8085106</v>
+        <v>114337021.2765957</v>
       </c>
       <c r="AO365" t="n">
         <v>0</v>
@@ -86322,7 +86322,7 @@
         <v>7.99</v>
       </c>
       <c r="H366" t="n">
-        <v>1040445785</v>
+        <v>1074768000</v>
       </c>
       <c r="I366" t="n">
         <v>300</v>
@@ -86340,7 +86340,7 @@
         <v>14.31</v>
       </c>
       <c r="N366" t="n">
-        <v>12.49671149997871</v>
+        <v>12.90895289215777</v>
       </c>
       <c r="O366" t="n">
         <v>0.19</v>
@@ -86418,7 +86418,7 @@
         <v>10124120.05</v>
       </c>
       <c r="AN366" t="n">
-        <v>157404808.623298</v>
+        <v>162597276.8532526</v>
       </c>
       <c r="AO366" t="n">
         <v>0</v>
@@ -94547,7 +94547,7 @@
         <v>8.33</v>
       </c>
       <c r="H401" t="n">
-        <v>92540801</v>
+        <v>92540880</v>
       </c>
       <c r="I401" t="n">
         <v>10700</v>
@@ -94565,7 +94565,7 @@
         <v>5.91</v>
       </c>
       <c r="N401" t="n">
-        <v>0.6324325460837913</v>
+        <v>0.6324330859772286</v>
       </c>
       <c r="O401" t="n">
         <v>0.23</v>
@@ -94643,7 +94643,7 @@
         <v>11442628.44</v>
       </c>
       <c r="AN401" t="n">
-        <v>39717081.97424892</v>
+        <v>39717115.87982833</v>
       </c>
       <c r="AO401" t="n">
         <v>0</v>
@@ -94782,7 +94782,7 @@
         <v>3.93</v>
       </c>
       <c r="H402" t="n">
-        <v>6028218895</v>
+        <v>5967580000</v>
       </c>
       <c r="I402" t="n">
         <v>1400</v>
@@ -94800,7 +94800,7 @@
         <v>9.42</v>
       </c>
       <c r="N402" t="n">
-        <v>0.679514207971564</v>
+        <v>0.672678857194509</v>
       </c>
       <c r="O402" t="n">
         <v>0.66</v>
@@ -94878,7 +94878,7 @@
         <v>483489419.2399999</v>
       </c>
       <c r="AN402" t="n">
-        <v>1157047772.552783</v>
+        <v>1145408829.174664</v>
       </c>
       <c r="AO402" t="n">
         <v>0</v>
@@ -95017,7 +95017,7 @@
         <v>4.06</v>
       </c>
       <c r="H403" t="n">
-        <v>6028218895</v>
+        <v>5967580000</v>
       </c>
       <c r="I403" t="n">
         <v>5000</v>
@@ -95035,7 +95035,7 @@
         <v>9.92</v>
       </c>
       <c r="N403" t="n">
-        <v>1.474454377968555</v>
+        <v>1.459622586727184</v>
       </c>
       <c r="O403" t="n">
         <v>0.6899999999999999</v>
@@ -95113,7 +95113,7 @@
         <v>222820003.58</v>
       </c>
       <c r="AN403" t="n">
-        <v>1100039944.343066</v>
+        <v>1088974452.554744</v>
       </c>
       <c r="AO403" t="n">
         <v>0</v>
@@ -95487,7 +95487,7 @@
         <v>20.69</v>
       </c>
       <c r="H405" t="n">
-        <v>695984818</v>
+        <v>704257800</v>
       </c>
       <c r="I405" t="n">
         <v>0</v>
@@ -95505,7 +95505,7 @@
         <v>6.94</v>
       </c>
       <c r="N405" t="n">
-        <v>0.5006145757692335</v>
+        <v>0.506565244903336</v>
       </c>
       <c r="O405" t="n">
         <v>0.53</v>
@@ -95583,7 +95583,7 @@
         <v>53525040.6</v>
       </c>
       <c r="AN405" t="n">
-        <v>171424832.0197045</v>
+        <v>173462512.315271</v>
       </c>
       <c r="AO405" t="n">
         <v>0.9505</v>
@@ -95722,7 +95722,7 @@
         <v>18.43</v>
       </c>
       <c r="H406" t="n">
-        <v>695984818</v>
+        <v>704257800</v>
       </c>
       <c r="I406" t="n">
         <v>700</v>
@@ -95740,7 +95740,7 @@
         <v>7.58</v>
       </c>
       <c r="N406" t="n">
-        <v>0.4180620945590932</v>
+        <v>0.4230314848298586</v>
       </c>
       <c r="O406" t="n">
         <v>0.58</v>
@@ -95818,7 +95818,7 @@
         <v>64094343.5</v>
       </c>
       <c r="AN406" t="n">
-        <v>157107182.3927765</v>
+        <v>158974672.6862303</v>
       </c>
       <c r="AO406" t="n">
         <v>0.7018</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-06-21 06:05
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -49532,7 +49532,7 @@
         <v>0</v>
       </c>
       <c r="AQ209" t="n">
-        <v>0.0598</v>
+        <v>0</v>
       </c>
       <c r="AR209" t="n">
         <v>0</v>
@@ -49547,7 +49547,7 @@
         <v>0</v>
       </c>
       <c r="AV209" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW209" t="n">
         <v>0</v>
@@ -49570,7 +49570,7 @@
         <v>8.720000000000001</v>
       </c>
       <c r="BC209" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="BD209" t="n">
         <v>4336.06</v>
@@ -49585,7 +49585,7 @@
         <v>356.54</v>
       </c>
       <c r="BH209" t="n">
-        <v>-91.3</v>
+        <v>-100</v>
       </c>
       <c r="BI209" t="n">
         <v>36.59</v>
@@ -49764,28 +49764,28 @@
         <v>0</v>
       </c>
       <c r="AP210" t="n">
-        <v>1.4028</v>
+        <v>0</v>
       </c>
       <c r="AQ210" t="n">
-        <v>0.4878</v>
+        <v>0</v>
       </c>
       <c r="AR210" t="n">
-        <v>0.4059</v>
+        <v>0</v>
       </c>
       <c r="AS210" t="n">
-        <v>0.3649</v>
+        <v>0</v>
       </c>
       <c r="AT210" t="n">
-        <v>0.1646</v>
+        <v>0</v>
       </c>
       <c r="AU210" t="n">
         <v>0</v>
       </c>
       <c r="AV210" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AW210" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX210" t="inlineStr">
         <is>
@@ -49805,7 +49805,7 @@
         <v>1.73</v>
       </c>
       <c r="BC210" t="n">
-        <v>7.85</v>
+        <v>0</v>
       </c>
       <c r="BD210" t="n">
         <v>37.57</v>
@@ -49820,7 +49820,7 @@
         <v>-86.53</v>
       </c>
       <c r="BH210" t="n">
-        <v>-38.86</v>
+        <v>-100</v>
       </c>
       <c r="BI210" t="n">
         <v>9.630000000000001</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-06-22 06:33
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1770,7 +1770,7 @@
         <v>7.6</v>
       </c>
       <c r="H6" t="n">
-        <v>479443637</v>
+        <v>479443700</v>
       </c>
       <c r="I6" t="n">
         <v>200</v>
@@ -1788,7 +1788,7 @@
         <v>13.39</v>
       </c>
       <c r="N6" t="n">
-        <v>5.914180794334658</v>
+        <v>5.914181571471659</v>
       </c>
       <c r="O6" t="n">
         <v>1.24</v>
@@ -1866,7 +1866,7 @@
         <v>34696585</v>
       </c>
       <c r="AN6" t="n">
-        <v>51442450.32188841</v>
+        <v>51442457.08154506</v>
       </c>
       <c r="AO6" t="n">
         <v>0</v>
@@ -2475,7 +2475,7 @@
         <v>23.38</v>
       </c>
       <c r="H9" t="n">
-        <v>204185622</v>
+        <v>204192200</v>
       </c>
       <c r="I9" t="n">
         <v>200</v>
@@ -2493,7 +2493,7 @@
         <v>2.59</v>
       </c>
       <c r="N9" t="n">
-        <v>0.3079624528181185</v>
+        <v>0.3079723740701381</v>
       </c>
       <c r="O9" t="n">
         <v>0.36</v>
@@ -2571,7 +2571,7 @@
         <v>81220091.82000001</v>
       </c>
       <c r="AN9" t="n">
-        <v>71144816.02787456</v>
+        <v>71147108.01393728</v>
       </c>
       <c r="AO9" t="n">
         <v>0</v>
@@ -2710,7 +2710,7 @@
         <v>58</v>
       </c>
       <c r="H10" t="n">
-        <v>204185622</v>
+        <v>204192200</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -2728,7 +2728,7 @@
         <v>6.01</v>
       </c>
       <c r="N10" t="n">
-        <v>57.51211460870338</v>
+        <v>57.51396740659477</v>
       </c>
       <c r="O10" t="n">
         <v>0.84</v>
@@ -2806,7 +2806,7 @@
         <v>434912.52</v>
       </c>
       <c r="AN10" t="n">
-        <v>30612537.03148426</v>
+        <v>30613523.23838081</v>
       </c>
       <c r="AO10" t="n">
         <v>0</v>
@@ -2945,7 +2945,7 @@
         <v>55</v>
       </c>
       <c r="H11" t="n">
-        <v>204185622</v>
+        <v>204192200</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -2963,7 +2963,7 @@
         <v>5.7</v>
       </c>
       <c r="N11" t="n">
-        <v>28.45552419268139</v>
+        <v>28.45644090971713</v>
       </c>
       <c r="O11" t="n">
         <v>0.79</v>
@@ -3041,7 +3041,7 @@
         <v>879011.7000000001</v>
       </c>
       <c r="AN11" t="n">
-        <v>32307851.58227848</v>
+        <v>32308892.40506329</v>
       </c>
       <c r="AO11" t="n">
         <v>0</v>
@@ -9274,7 +9274,7 @@
         <v>93.90000000000001</v>
       </c>
       <c r="H38" t="n">
-        <v>490366559</v>
+        <v>490366600</v>
       </c>
       <c r="I38" t="n">
         <v>800</v>
@@ -9292,7 +9292,7 @@
         <v>17.37</v>
       </c>
       <c r="N38" t="n">
-        <v>3.955248184807312</v>
+        <v>3.955248515509258</v>
       </c>
       <c r="O38" t="n">
         <v>2.37</v>
@@ -9370,7 +9370,7 @@
         <v>12707817.55</v>
       </c>
       <c r="AN38" t="n">
-        <v>21959989.20734438</v>
+        <v>21959991.04343932</v>
       </c>
       <c r="AO38" t="n">
         <v>0</v>
@@ -10684,7 +10684,7 @@
         <v>6.6</v>
       </c>
       <c r="H44" t="n">
-        <v>7531939</v>
+        <v>7531940</v>
       </c>
       <c r="I44" t="n">
         <v>0</v>
@@ -10702,7 +10702,7 @@
         <v>0.75</v>
       </c>
       <c r="N44" t="n">
-        <v>0.3365818551774681</v>
+        <v>0.3365818998647465</v>
       </c>
       <c r="O44" t="n">
         <v>0.03</v>
@@ -10780,7 +10780,7 @@
         <v>5719748.64</v>
       </c>
       <c r="AN44" t="n">
-        <v>7531939</v>
+        <v>7531940</v>
       </c>
       <c r="AO44" t="n">
         <v>0</v>
@@ -10919,7 +10919,7 @@
         <v>3.55</v>
       </c>
       <c r="H45" t="n">
-        <v>7531939</v>
+        <v>7531940</v>
       </c>
       <c r="I45" t="n">
         <v>400</v>
@@ -10937,7 +10937,7 @@
         <v>0.63</v>
       </c>
       <c r="N45" t="n">
-        <v>0.205850285059062</v>
+        <v>0.2058503123893796</v>
       </c>
       <c r="O45" t="n">
         <v>0.02</v>
@@ -11015,7 +11015,7 @@
         <v>9352251.359999999</v>
       </c>
       <c r="AN45" t="n">
-        <v>8966594.047619049</v>
+        <v>8966595.238095239</v>
       </c>
       <c r="AO45" t="n">
         <v>0</v>
@@ -13958,7 +13958,7 @@
         <v>21.49</v>
       </c>
       <c r="H58" t="n">
-        <v>101087300</v>
+        <v>101229300</v>
       </c>
       <c r="I58" t="n">
         <v>0</v>
@@ -13976,7 +13976,7 @@
         <v>13.78</v>
       </c>
       <c r="N58" t="n">
-        <v>1.876959686295569</v>
+        <v>1.879596301136938</v>
       </c>
       <c r="O58" t="n">
         <v>0.17</v>
@@ -14054,7 +14054,7 @@
         <v>6872145.189999999</v>
       </c>
       <c r="AN58" t="n">
-        <v>14358991.47727273</v>
+        <v>14379161.93181818</v>
       </c>
       <c r="AO58" t="n">
         <v>0</v>
@@ -14193,7 +14193,7 @@
         <v>18.02</v>
       </c>
       <c r="H59" t="n">
-        <v>101087300</v>
+        <v>101229300</v>
       </c>
       <c r="I59" t="n">
         <v>400</v>
@@ -14211,7 +14211,7 @@
         <v>12.47</v>
       </c>
       <c r="N59" t="n">
-        <v>10.87639545247701</v>
+        <v>10.89167381241196</v>
       </c>
       <c r="O59" t="n">
         <v>0.15</v>
@@ -14289,7 +14289,7 @@
         <v>1185938.81</v>
       </c>
       <c r="AN59" t="n">
-        <v>15869277.86499215</v>
+        <v>15891569.85871272</v>
       </c>
       <c r="AO59" t="n">
         <v>0</v>
@@ -14428,7 +14428,7 @@
         <v>381</v>
       </c>
       <c r="H60" t="n">
-        <v>173259750</v>
+        <v>173259800</v>
       </c>
       <c r="I60" t="n">
         <v>13</v>
@@ -14446,7 +14446,7 @@
         <v>2.87</v>
       </c>
       <c r="N60" t="n">
-        <v>12.24363151884279</v>
+        <v>12.24363505215953</v>
       </c>
       <c r="O60" t="n">
         <v>0.64</v>
@@ -14524,7 +14524,7 @@
         <v>59731412.5</v>
       </c>
       <c r="AN60" t="n">
-        <v>21821127.20403023</v>
+        <v>21821133.50125945</v>
       </c>
       <c r="AO60" t="n">
         <v>0</v>
@@ -14898,7 +14898,7 @@
         <v>105.4</v>
       </c>
       <c r="H62" t="n">
-        <v>10402949584</v>
+        <v>10402950000</v>
       </c>
       <c r="I62" t="n">
         <v>900</v>
@@ -14916,7 +14916,7 @@
         <v>4.26</v>
       </c>
       <c r="N62" t="n">
-        <v>1.063212881927999</v>
+        <v>1.063212924444456</v>
       </c>
       <c r="O62" t="n">
         <v>0.17</v>
@@ -14994,7 +14994,7 @@
         <v>2822812821.4</v>
       </c>
       <c r="AN62" t="n">
-        <v>4263503927.868853</v>
+        <v>4263504098.360656</v>
       </c>
       <c r="AO62" t="n">
         <v>0</v>
@@ -18893,7 +18893,7 @@
         <v>3.1</v>
       </c>
       <c r="H79" t="n">
-        <v>6699493493</v>
+        <v>6737688000</v>
       </c>
       <c r="I79" t="n">
         <v>41000</v>
@@ -18911,7 +18911,7 @@
         <v>2.47</v>
       </c>
       <c r="N79" t="n">
-        <v>0.9367168672570458</v>
+        <v>0.9420571872350934</v>
       </c>
       <c r="O79" t="n">
         <v>0.03</v>
@@ -18989,7 +18989,7 @@
         <v>531401092.4</v>
       </c>
       <c r="AN79" t="n">
-        <v>4060299086.666667</v>
+        <v>4083447272.727273</v>
       </c>
       <c r="AO79" t="n">
         <v>0</v>
@@ -19128,7 +19128,7 @@
         <v>3.28</v>
       </c>
       <c r="H80" t="n">
-        <v>6699493493</v>
+        <v>6737688000</v>
       </c>
       <c r="I80" t="n">
         <v>24500</v>
@@ -19146,7 +19146,7 @@
         <v>3.36</v>
       </c>
       <c r="N80" t="n">
-        <v>1.805750735326648</v>
+        <v>1.816045507487074</v>
       </c>
       <c r="O80" t="n">
         <v>0.04</v>
@@ -19224,7 +19224,7 @@
         <v>275659512.02</v>
       </c>
       <c r="AN80" t="n">
-        <v>2977552663.555555</v>
+        <v>2994528000</v>
       </c>
       <c r="AO80" t="n">
         <v>0</v>
@@ -19598,7 +19598,7 @@
         <v>9.359999999999999</v>
       </c>
       <c r="H82" t="n">
-        <v>395272000</v>
+        <v>395694800</v>
       </c>
       <c r="I82" t="n">
         <v>14200</v>
@@ -19616,7 +19616,7 @@
         <v>6.04</v>
       </c>
       <c r="N82" t="n">
-        <v>1.005125005085738</v>
+        <v>1.006200130194904</v>
       </c>
       <c r="O82" t="n">
         <v>1.01</v>
@@ -19694,7 +19694,7 @@
         <v>65949124.8</v>
       </c>
       <c r="AN82" t="n">
-        <v>70333096.08540925</v>
+        <v>70408327.40213522</v>
       </c>
       <c r="AO82" t="n">
         <v>0</v>
@@ -20491,7 +20491,7 @@
         <v>0</v>
       </c>
       <c r="BR85" t="n">
-        <v>29</v>
+        <v>26.5</v>
       </c>
       <c r="BS85" t="n">
         <v>0</v>
@@ -20773,7 +20773,7 @@
         <v>10.99</v>
       </c>
       <c r="H87" t="n">
-        <v>4980929458</v>
+        <v>4980931000</v>
       </c>
       <c r="I87" t="n">
         <v>3800</v>
@@ -20791,7 +20791,7 @@
         <v>7.13</v>
       </c>
       <c r="N87" t="n">
-        <v>0.5314693524652752</v>
+        <v>0.531469516997969</v>
       </c>
       <c r="O87" t="n">
         <v>0.21</v>
@@ -20869,7 +20869,7 @@
         <v>580126647.04</v>
       </c>
       <c r="AN87" t="n">
-        <v>907273125.3187613</v>
+        <v>907273406.1930783</v>
       </c>
       <c r="AO87" t="n">
         <v>0</v>
@@ -21243,7 +21243,7 @@
         <v>26.44</v>
       </c>
       <c r="H89" t="n">
-        <v>1943841606</v>
+        <v>1943826000</v>
       </c>
       <c r="I89" t="n">
         <v>4300</v>
@@ -21261,7 +21261,7 @@
         <v>11.38</v>
       </c>
       <c r="N89" t="n">
-        <v>8.137445131900822</v>
+        <v>8.137379800976566</v>
       </c>
       <c r="O89" t="n">
         <v>1.53</v>
@@ -21339,7 +21339,7 @@
         <v>95908776.3</v>
       </c>
       <c r="AN89" t="n">
-        <v>211978364.8854962</v>
+        <v>211976663.0316249</v>
       </c>
       <c r="AO89" t="n">
         <v>0</v>
@@ -21478,7 +21478,7 @@
         <v>23.75</v>
       </c>
       <c r="H90" t="n">
-        <v>1943841606</v>
+        <v>1943826000</v>
       </c>
       <c r="I90" t="n">
         <v>1800</v>
@@ -21496,7 +21496,7 @@
         <v>10.59</v>
       </c>
       <c r="N90" t="n">
-        <v>44.52457368138738</v>
+        <v>44.52421621887874</v>
       </c>
       <c r="O90" t="n">
         <v>1.42</v>
@@ -21574,7 +21574,7 @@
         <v>17528576.7</v>
       </c>
       <c r="AN90" t="n">
-        <v>227882954.982415</v>
+        <v>227881125.4396249</v>
       </c>
       <c r="AO90" t="n">
         <v>0</v>
@@ -21713,7 +21713,7 @@
         <v>28.32</v>
       </c>
       <c r="H91" t="n">
-        <v>1943841606</v>
+        <v>1943826000</v>
       </c>
       <c r="I91" t="n">
         <v>1400</v>
@@ -21731,7 +21731,7 @@
         <v>11.3</v>
       </c>
       <c r="N91" t="n">
-        <v>9.876473959891051</v>
+        <v>9.876394667292239</v>
       </c>
       <c r="O91" t="n">
         <v>1.52</v>
@@ -21809,7 +21809,7 @@
         <v>79021360.05</v>
       </c>
       <c r="AN91" t="n">
-        <v>213608967.6923077</v>
+        <v>213607252.7472528</v>
       </c>
       <c r="AO91" t="n">
         <v>0</v>
@@ -21948,7 +21948,7 @@
         <v>9</v>
       </c>
       <c r="H92" t="n">
-        <v>73314660</v>
+        <v>73874190</v>
       </c>
       <c r="I92" t="n">
         <v>200</v>
@@ -21966,7 +21966,7 @@
         <v>3.42</v>
       </c>
       <c r="N92" t="n">
-        <v>0.1353720483164855</v>
+        <v>0.1364051939683173</v>
       </c>
       <c r="O92" t="n">
         <v>0.15</v>
@@ -22044,7 +22044,7 @@
         <v>23342055.36</v>
       </c>
       <c r="AN92" t="n">
-        <v>51996212.76595745</v>
+        <v>52393042.55319149</v>
       </c>
       <c r="AO92" t="n">
         <v>0</v>
@@ -22183,7 +22183,7 @@
         <v>5.23</v>
       </c>
       <c r="H93" t="n">
-        <v>73314660</v>
+        <v>73874190</v>
       </c>
       <c r="I93" t="n">
         <v>3200</v>
@@ -22201,7 +22201,7 @@
         <v>2.3</v>
       </c>
       <c r="N93" t="n">
-        <v>0.1799676391962926</v>
+        <v>0.1813411338446959</v>
       </c>
       <c r="O93" t="n">
         <v>0.1</v>
@@ -22279,7 +22279,7 @@
         <v>17557944.64</v>
       </c>
       <c r="AN93" t="n">
-        <v>77173326.31578948</v>
+        <v>77762305.2631579</v>
       </c>
       <c r="AO93" t="n">
         <v>0</v>
@@ -22418,7 +22418,7 @@
         <v>45.8</v>
       </c>
       <c r="H94" t="n">
-        <v>8145905000</v>
+        <v>8132226000</v>
       </c>
       <c r="I94" t="n">
         <v>400</v>
@@ -22436,7 +22436,7 @@
         <v>5.78</v>
       </c>
       <c r="N94" t="n">
-        <v>0.7648351664723526</v>
+        <v>0.7635508180491664</v>
       </c>
       <c r="O94" t="n">
         <v>0.36</v>
@@ -22514,7 +22514,7 @@
         <v>1209900967.64</v>
       </c>
       <c r="AN94" t="n">
-        <v>2930181654.676259</v>
+        <v>2925261151.079137</v>
       </c>
       <c r="AO94" t="n">
         <v>0</v>
@@ -22653,7 +22653,7 @@
         <v>43.01</v>
       </c>
       <c r="H95" t="n">
-        <v>8145905000</v>
+        <v>8132226000</v>
       </c>
       <c r="I95" t="n">
         <v>0</v>
@@ -22671,7 +22671,7 @@
         <v>4.65</v>
       </c>
       <c r="N95" t="n">
-        <v>4.270860466331461</v>
+        <v>4.26368862964555</v>
       </c>
       <c r="O95" t="n">
         <v>0.29</v>
@@ -22749,7 +22749,7 @@
         <v>216671749.24</v>
       </c>
       <c r="AN95" t="n">
-        <v>3636564732.142857</v>
+        <v>3630458035.714285</v>
       </c>
       <c r="AO95" t="n">
         <v>0</v>
@@ -23593,7 +23593,7 @@
         <v>131.9</v>
       </c>
       <c r="H99" t="n">
-        <v>16933140628</v>
+        <v>16835940000</v>
       </c>
       <c r="I99" t="n">
         <v>0</v>
@@ -23611,7 +23611,7 @@
         <v>10.65</v>
       </c>
       <c r="N99" t="n">
-        <v>1.673100853512624</v>
+        <v>1.663496819787194</v>
       </c>
       <c r="O99" t="n">
         <v>1.16</v>
@@ -23689,7 +23689,7 @@
         <v>1267125769.6</v>
       </c>
       <c r="AN99" t="n">
-        <v>2914482035.800344</v>
+        <v>2897752151.462995</v>
       </c>
       <c r="AO99" t="n">
         <v>0</v>
@@ -23828,7 +23828,7 @@
         <v>123.9</v>
       </c>
       <c r="H100" t="n">
-        <v>16933140628</v>
+        <v>16835940000</v>
       </c>
       <c r="I100" t="n">
         <v>1400</v>
@@ -23846,7 +23846,7 @@
         <v>10.81</v>
       </c>
       <c r="N100" t="n">
-        <v>6.06371635569977</v>
+        <v>6.028909047903999</v>
       </c>
       <c r="O100" t="n">
         <v>1.18</v>
@@ -23924,7 +23924,7 @@
         <v>349625391.8</v>
       </c>
       <c r="AN100" t="n">
-        <v>2870023835.254237</v>
+        <v>2853549152.542373</v>
       </c>
       <c r="AO100" t="n">
         <v>0</v>
@@ -24063,7 +24063,7 @@
         <v>24.61</v>
       </c>
       <c r="H101" t="n">
-        <v>630227710</v>
+        <v>628084800</v>
       </c>
       <c r="I101" t="n">
         <v>500</v>
@@ -24081,7 +24081,7 @@
         <v>6.28</v>
       </c>
       <c r="N101" t="n">
-        <v>2.032569790701838</v>
+        <v>2.025658615485197</v>
       </c>
       <c r="O101" t="n">
         <v>0.49</v>
@@ -24159,7 +24159,7 @@
         <v>42633867</v>
       </c>
       <c r="AN101" t="n">
-        <v>65173496.38055843</v>
+        <v>64951892.45087901</v>
       </c>
       <c r="AO101" t="n">
         <v>0</v>
@@ -24298,7 +24298,7 @@
         <v>24.5</v>
       </c>
       <c r="H102" t="n">
-        <v>630227710</v>
+        <v>628084800</v>
       </c>
       <c r="I102" t="n">
         <v>4000</v>
@@ -24316,7 +24316,7 @@
         <v>6.32</v>
       </c>
       <c r="N102" t="n">
-        <v>1.487058061820474</v>
+        <v>1.482001744015509</v>
       </c>
       <c r="O102" t="n">
         <v>0.49</v>
@@ -24394,7 +24394,7 @@
         <v>58273656.12</v>
       </c>
       <c r="AN102" t="n">
-        <v>64771604.31654676</v>
+        <v>64551366.90647481</v>
       </c>
       <c r="AO102" t="n">
         <v>0</v>
@@ -26883,7 +26883,7 @@
         <v>18</v>
       </c>
       <c r="H113" t="n">
-        <v>465821550</v>
+        <v>465821600</v>
       </c>
       <c r="I113" t="n">
         <v>0</v>
@@ -26901,7 +26901,7 @@
         <v>20.65</v>
       </c>
       <c r="N113" t="n">
-        <v>1.745835588149623</v>
+        <v>1.745835775542798</v>
       </c>
       <c r="O113" t="n">
         <v>0.54</v>
@@ -26979,7 +26979,7 @@
         <v>8431470.34</v>
       </c>
       <c r="AN113" t="n">
-        <v>34530878.42846553</v>
+        <v>34530882.13491475</v>
       </c>
       <c r="AO113" t="n">
         <v>0</v>
@@ -27118,7 +27118,7 @@
         <v>15</v>
       </c>
       <c r="H114" t="n">
-        <v>465821550</v>
+        <v>465821600</v>
       </c>
       <c r="I114" t="n">
         <v>600</v>
@@ -27136,7 +27136,7 @@
         <v>23.27</v>
       </c>
       <c r="N114" t="n">
-        <v>1.436926815621928</v>
+        <v>1.436926969857688</v>
       </c>
       <c r="O114" t="n">
         <v>0.61</v>
@@ -27214,7 +27214,7 @@
         <v>10244057.54</v>
       </c>
       <c r="AN114" t="n">
-        <v>30666329.82225148</v>
+        <v>30666333.11389072</v>
       </c>
       <c r="AO114" t="n">
         <v>0</v>
@@ -27353,7 +27353,7 @@
         <v>15.01</v>
       </c>
       <c r="H115" t="n">
-        <v>465821550</v>
+        <v>465821600</v>
       </c>
       <c r="I115" t="n">
         <v>0</v>
@@ -27371,7 +27371,7 @@
         <v>22.56</v>
       </c>
       <c r="N115" t="n">
-        <v>2.720863874056142</v>
+        <v>2.720864166106163</v>
       </c>
       <c r="O115" t="n">
         <v>0.59</v>
@@ -27449,7 +27449,7 @@
         <v>5410032.13</v>
       </c>
       <c r="AN115" t="n">
-        <v>31624002.03665988</v>
+        <v>31624005.43109301</v>
       </c>
       <c r="AO115" t="n">
         <v>0</v>
@@ -28763,7 +28763,7 @@
         <v>0.47</v>
       </c>
       <c r="H121" t="n">
-        <v>12553869</v>
+        <v>12553870</v>
       </c>
       <c r="I121" t="n">
         <v>1800</v>
@@ -28781,7 +28781,7 @@
         <v>0.19</v>
       </c>
       <c r="N121" t="n">
-        <v>0.0289882026370605</v>
+        <v>0.02898820494616558</v>
       </c>
       <c r="O121" t="n">
         <v>0.02</v>
@@ -28859,7 +28859,7 @@
         <v>129011019.48</v>
       </c>
       <c r="AN121" t="n">
-        <v>4198618.394648829</v>
+        <v>4198618.72909699</v>
       </c>
       <c r="AO121" t="n">
         <v>0</v>
@@ -42628,7 +42628,7 @@
         <v>36</v>
       </c>
       <c r="H180" t="n">
-        <v>3461924000</v>
+        <v>3398969000</v>
       </c>
       <c r="I180" t="n">
         <v>0</v>
@@ -42646,7 +42646,7 @@
         <v>12.71</v>
       </c>
       <c r="N180" t="n">
-        <v>8.457789920366082</v>
+        <v>8.303985225509509</v>
       </c>
       <c r="O180" t="n">
         <v>0.8</v>
@@ -42724,7 +42724,7 @@
         <v>84360399.48</v>
       </c>
       <c r="AN180" t="n">
-        <v>449017380.0259404</v>
+        <v>440852010.3761349</v>
       </c>
       <c r="AO180" t="n">
         <v>4.0605</v>
@@ -42863,7 +42863,7 @@
         <v>35.99</v>
       </c>
       <c r="H181" t="n">
-        <v>3461924000</v>
+        <v>3398969000</v>
       </c>
       <c r="I181" t="n">
         <v>400</v>
@@ -42881,7 +42881,7 @@
         <v>13.08</v>
       </c>
       <c r="N181" t="n">
-        <v>4.228894960183041</v>
+        <v>4.151992612754754</v>
       </c>
       <c r="O181" t="n">
         <v>0.83</v>
@@ -42959,7 +42959,7 @@
         <v>168720798.96</v>
       </c>
       <c r="AN181" t="n">
-        <v>436010579.3450881</v>
+        <v>428081738.0352645</v>
       </c>
       <c r="AO181" t="n">
         <v>4.0605</v>
@@ -45213,7 +45213,7 @@
         <v>2.81</v>
       </c>
       <c r="H191" t="n">
-        <v>5419837</v>
+        <v>5419840</v>
       </c>
       <c r="I191" t="n">
         <v>300</v>
@@ -45231,7 +45231,7 @@
         <v>0.02</v>
       </c>
       <c r="N191" t="n">
-        <v>0.02860624776650598</v>
+        <v>0.02860626360069865</v>
       </c>
       <c r="O191" t="n">
         <v>0.01</v>
@@ -45309,7 +45309,7 @@
         <v>256931318.49</v>
       </c>
       <c r="AN191" t="n">
-        <v>90330616.66666667</v>
+        <v>90330666.66666667</v>
       </c>
       <c r="AO191" t="n">
         <v>0</v>
@@ -45448,7 +45448,7 @@
         <v>2.9</v>
       </c>
       <c r="H192" t="n">
-        <v>23613331</v>
+        <v>24593330</v>
       </c>
       <c r="I192" t="n">
         <v>18200</v>
@@ -45466,7 +45466,7 @@
         <v>21.95</v>
       </c>
       <c r="N192" t="n">
-        <v>2.414247924573004</v>
+        <v>2.514443892343651</v>
       </c>
       <c r="O192" t="n">
         <v>0.32</v>
@@ -45544,7 +45544,7 @@
         <v>357000.03</v>
       </c>
       <c r="AN192" t="n">
-        <v>1985982.422203532</v>
+        <v>2068404.541631623</v>
       </c>
       <c r="AO192" t="n">
         <v>0</v>
@@ -45683,7 +45683,7 @@
         <v>1.65</v>
       </c>
       <c r="H193" t="n">
-        <v>23613331</v>
+        <v>24593330</v>
       </c>
       <c r="I193" t="n">
         <v>25100</v>
@@ -45701,7 +45701,7 @@
         <v>14.71</v>
       </c>
       <c r="N193" t="n">
-        <v>1.207124114444991</v>
+        <v>1.257222104645187</v>
       </c>
       <c r="O193" t="n">
         <v>0.22</v>
@@ -45779,7 +45779,7 @@
         <v>713999.97</v>
       </c>
       <c r="AN193" t="n">
-        <v>2962776.787954831</v>
+        <v>3085737.766624843</v>
       </c>
       <c r="AO193" t="n">
         <v>0</v>
@@ -47563,7 +47563,7 @@
         <v>7.24</v>
       </c>
       <c r="H201" t="n">
-        <v>133016244</v>
+        <v>133016300</v>
       </c>
       <c r="I201" t="n">
         <v>200</v>
@@ -47581,7 +47581,7 @@
         <v>1.99</v>
       </c>
       <c r="N201" t="n">
-        <v>1.569833797879972</v>
+        <v>1.569834458781905</v>
       </c>
       <c r="O201" t="n">
         <v>0.25</v>
@@ -47659,7 +47659,7 @@
         <v>28893848.04</v>
       </c>
       <c r="AN201" t="n">
-        <v>105568447.6190476</v>
+        <v>105568492.0634921</v>
       </c>
       <c r="AO201" t="n">
         <v>0</v>
@@ -48006,7 +48006,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>IBOVESPA</t>
+          <t>Brazil Stock Exchange Index</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
@@ -49532,7 +49532,7 @@
         <v>0</v>
       </c>
       <c r="AQ209" t="n">
-        <v>0</v>
+        <v>0.0598</v>
       </c>
       <c r="AR209" t="n">
         <v>0</v>
@@ -49547,7 +49547,7 @@
         <v>0</v>
       </c>
       <c r="AV209" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW209" t="n">
         <v>0</v>
@@ -49570,7 +49570,7 @@
         <v>8.720000000000001</v>
       </c>
       <c r="BC209" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="BD209" t="n">
         <v>4336.06</v>
@@ -49585,7 +49585,7 @@
         <v>356.54</v>
       </c>
       <c r="BH209" t="n">
-        <v>-100</v>
+        <v>-91.3</v>
       </c>
       <c r="BI209" t="n">
         <v>36.59</v>
@@ -49764,28 +49764,28 @@
         <v>0</v>
       </c>
       <c r="AP210" t="n">
-        <v>0</v>
+        <v>1.4028</v>
       </c>
       <c r="AQ210" t="n">
-        <v>0</v>
+        <v>0.4878</v>
       </c>
       <c r="AR210" t="n">
-        <v>0</v>
+        <v>0.4059</v>
       </c>
       <c r="AS210" t="n">
-        <v>0</v>
+        <v>0.3649</v>
       </c>
       <c r="AT210" t="n">
-        <v>0</v>
+        <v>0.1646</v>
       </c>
       <c r="AU210" t="n">
         <v>0</v>
       </c>
       <c r="AV210" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AW210" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX210" t="inlineStr">
         <is>
@@ -49805,7 +49805,7 @@
         <v>1.73</v>
       </c>
       <c r="BC210" t="n">
-        <v>0</v>
+        <v>7.85</v>
       </c>
       <c r="BD210" t="n">
         <v>37.57</v>
@@ -49820,7 +49820,7 @@
         <v>-86.53</v>
       </c>
       <c r="BH210" t="n">
-        <v>-100</v>
+        <v>-38.86</v>
       </c>
       <c r="BI210" t="n">
         <v>9.630000000000001</v>
@@ -57887,7 +57887,7 @@
         <v>0.96</v>
       </c>
       <c r="H245" t="n">
-        <v>275209433</v>
+        <v>275209500</v>
       </c>
       <c r="I245" t="n">
         <v>50800</v>
@@ -57905,7 +57905,7 @@
         <v>2.22</v>
       </c>
       <c r="N245" t="n">
-        <v>0.1375999773007818</v>
+        <v>0.137600010799628</v>
       </c>
       <c r="O245" t="n">
         <v>0.14</v>
@@ -57983,7 +57983,7 @@
         <v>146205035.4</v>
       </c>
       <c r="AN245" t="n">
-        <v>23244039.94932432</v>
+        <v>23244045.60810811</v>
       </c>
       <c r="AO245" t="n">
         <v>0</v>
@@ -60707,7 +60707,7 @@
         <v>39.86</v>
       </c>
       <c r="H257" t="n">
-        <v>12955270000</v>
+        <v>12723890000</v>
       </c>
       <c r="I257" t="n">
         <v>400</v>
@@ -60725,7 +60725,7 @@
         <v>9.57</v>
       </c>
       <c r="N257" t="n">
-        <v>3.227865983634703</v>
+        <v>3.170216576768355</v>
       </c>
       <c r="O257" t="n">
         <v>0.64</v>
@@ -60803,7 +60803,7 @@
         <v>836829598.4699999</v>
       </c>
       <c r="AN257" t="n">
-        <v>2355503636.363636</v>
+        <v>2313434545.454545</v>
       </c>
       <c r="AO257" t="n">
         <v>0</v>
@@ -60942,7 +60942,7 @@
         <v>38</v>
       </c>
       <c r="H258" t="n">
-        <v>12955270000</v>
+        <v>12723890000</v>
       </c>
       <c r="I258" t="n">
         <v>0</v>
@@ -60960,7 +60960,7 @@
         <v>8.94</v>
       </c>
       <c r="N258" t="n">
-        <v>7.406591052143772</v>
+        <v>7.274309977519698</v>
       </c>
       <c r="O258" t="n">
         <v>0.59</v>
@@ -61038,7 +61038,7 @@
         <v>364698655.02</v>
       </c>
       <c r="AN258" t="n">
-        <v>2520480544.747082</v>
+        <v>2475464980.544747</v>
       </c>
       <c r="AO258" t="n">
         <v>0</v>
@@ -61177,7 +61177,7 @@
         <v>32.6</v>
       </c>
       <c r="H259" t="n">
-        <v>12955270000</v>
+        <v>12723890000</v>
       </c>
       <c r="I259" t="n">
         <v>200</v>
@@ -61195,7 +61195,7 @@
         <v>9.949999999999999</v>
       </c>
       <c r="N259" t="n">
-        <v>8.735188509866665</v>
+        <v>8.57917879973226</v>
       </c>
       <c r="O259" t="n">
         <v>0.66</v>
@@ -61273,7 +61273,7 @@
         <v>309229021.44</v>
       </c>
       <c r="AN259" t="n">
-        <v>2264907342.657343</v>
+        <v>2224456293.706294</v>
       </c>
       <c r="AO259" t="n">
         <v>0</v>
@@ -64232,7 +64232,7 @@
         <v>2.24</v>
       </c>
       <c r="H272" t="n">
-        <v>14832126</v>
+        <v>14832130</v>
       </c>
       <c r="I272" t="n">
         <v>6100</v>
@@ -64250,7 +64250,7 @@
         <v>0.96</v>
       </c>
       <c r="N272" t="n">
-        <v>5.688738952545874</v>
+        <v>5.688740486712709</v>
       </c>
       <c r="O272" t="n">
         <v>1.87</v>
@@ -64328,7 +64328,7 @@
         <v>37941114.78</v>
       </c>
       <c r="AN272" t="n">
-        <v>13125775.22123894</v>
+        <v>13125778.76106195</v>
       </c>
       <c r="AO272" t="n">
         <v>0</v>
@@ -66582,7 +66582,7 @@
         <v>35</v>
       </c>
       <c r="H282" t="n">
-        <v>836651200</v>
+        <v>834557100</v>
       </c>
       <c r="I282" t="n">
         <v>400</v>
@@ -66600,7 +66600,7 @@
         <v>17.82</v>
       </c>
       <c r="N282" t="n">
-        <v>0.4264387597873053</v>
+        <v>0.4253714029164007</v>
       </c>
       <c r="O282" t="n">
         <v>0.52</v>
@@ -66678,7 +66678,7 @@
         <v>42378103.55</v>
       </c>
       <c r="AN282" t="n">
-        <v>93376249.99999999</v>
+        <v>93142533.48214285</v>
       </c>
       <c r="AO282" t="n">
         <v>0</v>
@@ -66817,7 +66817,7 @@
         <v>32</v>
       </c>
       <c r="H283" t="n">
-        <v>836651200</v>
+        <v>834557100</v>
       </c>
       <c r="I283" t="n">
         <v>200</v>
@@ -66835,7 +66835,7 @@
         <v>18.34</v>
       </c>
       <c r="N283" t="n">
-        <v>9.527554326173249</v>
+        <v>9.503707289900021</v>
       </c>
       <c r="O283" t="n">
         <v>0.54</v>
@@ -66913,7 +66913,7 @@
         <v>1896779.1</v>
       </c>
       <c r="AN283" t="n">
-        <v>90644767.06392199</v>
+        <v>90417887.32394366</v>
       </c>
       <c r="AO283" t="n">
         <v>0</v>
@@ -67287,7 +67287,7 @@
         <v>1.45</v>
       </c>
       <c r="H285" t="n">
-        <v>4766853</v>
+        <v>4766850</v>
       </c>
       <c r="I285" t="n">
         <v>11600</v>
@@ -67305,7 +67305,7 @@
         <v>0.05</v>
       </c>
       <c r="N285" t="n">
-        <v>0.04832086593203123</v>
+        <v>0.04832083552148621</v>
       </c>
       <c r="O285" t="n">
         <v>0.02</v>
@@ -67383,7 +67383,7 @@
         <v>178674864.1</v>
       </c>
       <c r="AN285" t="n">
-        <v>23834265</v>
+        <v>23834250</v>
       </c>
       <c r="AO285" t="n">
         <v>0</v>
@@ -67757,7 +67757,7 @@
         <v>39.79</v>
       </c>
       <c r="H287" t="n">
-        <v>710981755</v>
+        <v>720955800</v>
       </c>
       <c r="I287" t="n">
         <v>300</v>
@@ -67775,7 +67775,7 @@
         <v>21.05</v>
       </c>
       <c r="N287" t="n">
-        <v>11.99427063903727</v>
+        <v>12.16253289647865</v>
       </c>
       <c r="O287" t="n">
         <v>0.54</v>
@@ -67853,7 +67853,7 @@
         <v>16864244.22</v>
       </c>
       <c r="AN287" t="n">
-        <v>29898307.61143818</v>
+        <v>30317737.59461733</v>
       </c>
       <c r="AO287" t="n">
         <v>0.3943</v>
@@ -67992,7 +67992,7 @@
         <v>39.7</v>
       </c>
       <c r="H288" t="n">
-        <v>710981755</v>
+        <v>720955800</v>
       </c>
       <c r="I288" t="n">
         <v>400</v>
@@ -68010,7 +68010,7 @@
         <v>21.15</v>
       </c>
       <c r="N288" t="n">
-        <v>12.66803564238072</v>
+        <v>12.84574984766114</v>
       </c>
       <c r="O288" t="n">
         <v>0.54</v>
@@ -68088,7 +68088,7 @@
         <v>15967298.72</v>
       </c>
       <c r="AN288" t="n">
-        <v>29748190.58577406</v>
+        <v>30165514.64435147</v>
       </c>
       <c r="AO288" t="n">
         <v>0.4337</v>
@@ -72457,7 +72457,7 @@
         <v>8.42</v>
       </c>
       <c r="H307" t="n">
-        <v>407113800</v>
+        <v>405892400</v>
       </c>
       <c r="I307" t="n">
         <v>0</v>
@@ -72475,7 +72475,7 @@
         <v>9.75</v>
       </c>
       <c r="N307" t="n">
-        <v>1.465952621173094</v>
+        <v>1.461554552300211</v>
       </c>
       <c r="O307" t="n">
         <v>0.39</v>
@@ -72553,7 +72553,7 @@
         <v>13774554.64</v>
       </c>
       <c r="AN307" t="n">
-        <v>40549183.26693227</v>
+        <v>40427529.88047809</v>
       </c>
       <c r="AO307" t="n">
         <v>0</v>
@@ -72692,7 +72692,7 @@
         <v>8.5</v>
       </c>
       <c r="H308" t="n">
-        <v>407113800</v>
+        <v>405892400</v>
       </c>
       <c r="I308" t="n">
         <v>0</v>
@@ -72710,7 +72710,7 @@
         <v>9.6</v>
       </c>
       <c r="N308" t="n">
-        <v>0.7330743472165352</v>
+        <v>0.7308750186560926</v>
       </c>
       <c r="O308" t="n">
         <v>0.39</v>
@@ -72788,7 +72788,7 @@
         <v>27545425.04</v>
       </c>
       <c r="AN308" t="n">
-        <v>41205850.20242915</v>
+        <v>41082226.72064777</v>
       </c>
       <c r="AO308" t="n">
         <v>0</v>
@@ -75982,7 +75982,7 @@
         <v>0.96</v>
       </c>
       <c r="H322" t="n">
-        <v>354641848</v>
+        <v>354492200</v>
       </c>
       <c r="I322" t="n">
         <v>38500</v>
@@ -76000,7 +76000,7 @@
         <v>2.24</v>
       </c>
       <c r="N322" t="n">
-        <v>0.8988728702428921</v>
+        <v>0.8984935734169684</v>
       </c>
       <c r="O322" t="n">
         <v>0.13</v>
@@ -76078,7 +76078,7 @@
         <v>142942061.98</v>
       </c>
       <c r="AN322" t="n">
-        <v>28531122.1238938</v>
+        <v>28519082.86403862</v>
       </c>
       <c r="AO322" t="n">
         <v>0</v>
@@ -76217,7 +76217,7 @@
         <v>0.9</v>
       </c>
       <c r="H323" t="n">
-        <v>354641848</v>
+        <v>354492200</v>
       </c>
       <c r="I323" t="n">
         <v>32300</v>
@@ -76235,7 +76235,7 @@
         <v>2</v>
       </c>
       <c r="N323" t="n">
-        <v>4.478348295609888</v>
+        <v>4.476458569765291</v>
       </c>
       <c r="O323" t="n">
         <v>0.11</v>
@@ -76313,7 +76313,7 @@
         <v>28690654.02</v>
       </c>
       <c r="AN323" t="n">
-        <v>31978525.51848512</v>
+        <v>31965031.55996393</v>
       </c>
       <c r="AO323" t="n">
         <v>0</v>
@@ -80682,7 +80682,7 @@
         <v>5.89</v>
       </c>
       <c r="H342" t="n">
-        <v>397060440</v>
+        <v>397060400</v>
       </c>
       <c r="I342" t="n">
         <v>12600</v>
@@ -80700,7 +80700,7 @@
         <v>0.62</v>
       </c>
       <c r="N342" t="n">
-        <v>2.685606692099692</v>
+        <v>2.685606421550786</v>
       </c>
       <c r="O342" t="n">
         <v>0.1</v>
@@ -80778,7 +80778,7 @@
         <v>61075833.72000001</v>
       </c>
       <c r="AN342" t="n">
-        <v>431587434.7826087</v>
+        <v>431587391.3043478</v>
       </c>
       <c r="AO342" t="n">
         <v>0</v>
@@ -82327,7 +82327,7 @@
         <v>9.75</v>
       </c>
       <c r="H349" t="n">
-        <v>35873930</v>
+        <v>33947850</v>
       </c>
       <c r="I349" t="n">
         <v>0</v>
@@ -82345,7 +82345,7 @@
         <v>0.41</v>
       </c>
       <c r="N349" t="n">
-        <v>0.1055246698373322</v>
+        <v>0.09985902472735156</v>
       </c>
       <c r="O349" t="n">
         <v>0.15</v>
@@ -82423,7 +82423,7 @@
         <v>72003052.8</v>
       </c>
       <c r="AN349" t="n">
-        <v>39859922.22222222</v>
+        <v>37719833.33333334</v>
       </c>
       <c r="AO349" t="n">
         <v>0</v>
@@ -82562,7 +82562,7 @@
         <v>1.59</v>
       </c>
       <c r="H350" t="n">
-        <v>35873930</v>
+        <v>33947850</v>
       </c>
       <c r="I350" t="n">
         <v>4500</v>
@@ -82580,7 +82580,7 @@
         <v>0.1</v>
       </c>
       <c r="N350" t="n">
-        <v>0.05551476372133811</v>
+        <v>0.05253416259655488</v>
       </c>
       <c r="O350" t="n">
         <v>0.04</v>
@@ -82658,7 +82658,7 @@
         <v>136866265.2</v>
       </c>
       <c r="AN350" t="n">
-        <v>155973608.6956522</v>
+        <v>147599347.8260869</v>
       </c>
       <c r="AO350" t="n">
         <v>0</v>
@@ -82797,7 +82797,7 @@
         <v>11.51</v>
       </c>
       <c r="H351" t="n">
-        <v>35873930</v>
+        <v>33947850</v>
       </c>
       <c r="I351" t="n">
         <v>0</v>
@@ -82815,7 +82815,7 @@
         <v>0.42</v>
       </c>
       <c r="N351" t="n">
-        <v>45.23808555710356</v>
+        <v>42.80924177472939</v>
       </c>
       <c r="O351" t="n">
         <v>0.15</v>
@@ -82893,7 +82893,7 @@
         <v>167958</v>
       </c>
       <c r="AN351" t="n">
-        <v>37762031.57894737</v>
+        <v>35734578.94736842</v>
       </c>
       <c r="AO351" t="n">
         <v>0</v>
@@ -83267,7 +83267,7 @@
         <v>38.66</v>
       </c>
       <c r="H353" t="n">
-        <v>157157083</v>
+        <v>155155300</v>
       </c>
       <c r="I353" t="n">
         <v>0</v>
@@ -83285,7 +83285,7 @@
         <v>3.42</v>
       </c>
       <c r="N353" t="n">
-        <v>2.045537667448929</v>
+        <v>2.019482700975933</v>
       </c>
       <c r="O353" t="n">
         <v>0.78</v>
@@ -83363,7 +83363,7 @@
         <v>9672800</v>
       </c>
       <c r="AN353" t="n">
-        <v>63369791.53225806</v>
+        <v>62562620.96774194</v>
       </c>
       <c r="AO353" t="n">
         <v>0</v>
@@ -83502,7 +83502,7 @@
         <v>79.23999999999999</v>
       </c>
       <c r="H354" t="n">
-        <v>157157083</v>
+        <v>155155300</v>
       </c>
       <c r="I354" t="n">
         <v>200</v>
@@ -83520,7 +83520,7 @@
         <v>6.19</v>
       </c>
       <c r="N354" t="n">
-        <v>2.231685245139285</v>
+        <v>2.2032592302261</v>
       </c>
       <c r="O354" t="n">
         <v>1.42</v>
@@ -83598,7 +83598,7 @@
         <v>8865980</v>
       </c>
       <c r="AN354" t="n">
-        <v>34923796.22222222</v>
+        <v>34478955.55555555</v>
       </c>
       <c r="AO354" t="n">
         <v>0</v>
@@ -83737,7 +83737,7 @@
         <v>79.98</v>
       </c>
       <c r="H355" t="n">
-        <v>157157083</v>
+        <v>155155300</v>
       </c>
       <c r="I355" t="n">
         <v>0</v>
@@ -83755,7 +83755,7 @@
         <v>6.02</v>
       </c>
       <c r="N355" t="n">
-        <v>2.142395990867837</v>
+        <v>2.115107294794321</v>
       </c>
       <c r="O355" t="n">
         <v>1.38</v>
@@ -83833,7 +83833,7 @@
         <v>9235490</v>
       </c>
       <c r="AN355" t="n">
-        <v>35962719.22196797</v>
+        <v>35504645.30892448</v>
       </c>
       <c r="AO355" t="n">
         <v>0</v>
@@ -86087,7 +86087,7 @@
         <v>10.1</v>
       </c>
       <c r="H365" t="n">
-        <v>979412132</v>
+        <v>986958900</v>
       </c>
       <c r="I365" t="n">
         <v>0</v>
@@ -86105,7 +86105,7 @@
         <v>20.34</v>
       </c>
       <c r="N365" t="n">
-        <v>2.590927379153762</v>
+        <v>2.610891526213482</v>
       </c>
       <c r="O365" t="n">
         <v>0.27</v>
@@ -86183,7 +86183,7 @@
         <v>45966751.6</v>
       </c>
       <c r="AN365" t="n">
-        <v>104192780</v>
+        <v>104995627.6595745</v>
       </c>
       <c r="AO365" t="n">
         <v>0</v>
@@ -86322,7 +86322,7 @@
         <v>7.76</v>
       </c>
       <c r="H366" t="n">
-        <v>979412132</v>
+        <v>986958900</v>
       </c>
       <c r="I366" t="n">
         <v>7900</v>
@@ -86340,7 +86340,7 @@
         <v>14.31</v>
       </c>
       <c r="N366" t="n">
-        <v>11.76364115231921</v>
+        <v>11.85428478201421</v>
       </c>
       <c r="O366" t="n">
         <v>0.19</v>
@@ -86418,7 +86418,7 @@
         <v>10124120.05</v>
       </c>
       <c r="AN366" t="n">
-        <v>148171275.6429652</v>
+        <v>149312995.4614221</v>
       </c>
       <c r="AO366" t="n">
         <v>0</v>
@@ -89612,7 +89612,7 @@
         <v>1.22</v>
       </c>
       <c r="H380" t="n">
-        <v>80625361</v>
+        <v>80625360</v>
       </c>
       <c r="I380" t="n">
         <v>13100</v>
@@ -89630,7 +89630,7 @@
         <v>39.8</v>
       </c>
       <c r="N380" t="n">
-        <v>0.2988999885816082</v>
+        <v>0.2988999848743381</v>
       </c>
       <c r="O380" t="n">
         <v>0.24</v>
@@ -89708,7 +89708,7 @@
         <v>2643454.56</v>
       </c>
       <c r="AN380" t="n">
-        <v>7613348.536355052</v>
+        <v>7613348.441926346</v>
       </c>
       <c r="AO380" t="n">
         <v>0</v>
@@ -94782,7 +94782,7 @@
         <v>3.96</v>
       </c>
       <c r="H402" t="n">
-        <v>5873764125</v>
+        <v>5974737000</v>
       </c>
       <c r="I402" t="n">
         <v>1100</v>
@@ -94800,7 +94800,7 @@
         <v>9.42</v>
       </c>
       <c r="N402" t="n">
-        <v>0.6621037236258425</v>
+        <v>0.6734856101129351</v>
       </c>
       <c r="O402" t="n">
         <v>0.66</v>
@@ -94878,7 +94878,7 @@
         <v>483489419.2399999</v>
       </c>
       <c r="AN402" t="n">
-        <v>1127401943.378119</v>
+        <v>1146782533.589252</v>
       </c>
       <c r="AO402" t="n">
         <v>0</v>
@@ -95017,7 +95017,7 @@
         <v>4.01</v>
       </c>
       <c r="H403" t="n">
-        <v>5873764125</v>
+        <v>5974737000</v>
       </c>
       <c r="I403" t="n">
         <v>2900</v>
@@ -95035,7 +95035,7 @@
         <v>9.92</v>
       </c>
       <c r="N403" t="n">
-        <v>1.436675970151692</v>
+        <v>1.461373131982247</v>
       </c>
       <c r="O403" t="n">
         <v>0.6899999999999999</v>
@@ -95113,7 +95113,7 @@
         <v>222820003.58</v>
       </c>
       <c r="AN403" t="n">
-        <v>1071854767.335766</v>
+        <v>1090280474.452555</v>
       </c>
       <c r="AO403" t="n">
         <v>0</v>
@@ -95487,7 +95487,7 @@
         <v>20.69</v>
       </c>
       <c r="H405" t="n">
-        <v>741949831</v>
+        <v>735213600</v>
       </c>
       <c r="I405" t="n">
         <v>0</v>
@@ -95505,7 +95505,7 @@
         <v>6.94</v>
       </c>
       <c r="N405" t="n">
-        <v>0.5336767272531503</v>
+        <v>0.528831426986344</v>
       </c>
       <c r="O405" t="n">
         <v>0.53</v>
@@ -95583,7 +95583,7 @@
         <v>53525040.6</v>
       </c>
       <c r="AN405" t="n">
-        <v>182746263.7931035</v>
+        <v>181087093.5960591</v>
       </c>
       <c r="AO405" t="n">
         <v>0.9505</v>
@@ -95722,7 +95722,7 @@
         <v>19.99</v>
       </c>
       <c r="H406" t="n">
-        <v>741949831</v>
+        <v>735213600</v>
       </c>
       <c r="I406" t="n">
         <v>200</v>
@@ -95740,7 +95740,7 @@
         <v>7.58</v>
       </c>
       <c r="N406" t="n">
-        <v>0.4456722221283068</v>
+        <v>0.4416259228866273</v>
       </c>
       <c r="O406" t="n">
         <v>0.58</v>
@@ -95818,7 +95818,7 @@
         <v>64094343.5</v>
       </c>
       <c r="AN406" t="n">
-        <v>167483031.8284425</v>
+        <v>165962437.9232506</v>
       </c>
       <c r="AO406" t="n">
         <v>0.7018</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-06-29 05:34
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -8804,7 +8804,7 @@
         <v>26</v>
       </c>
       <c r="H36" t="n">
-        <v>210699870</v>
+        <v>210700000</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
@@ -8822,7 +8822,7 @@
         <v>10.3</v>
       </c>
       <c r="N36" t="n">
-        <v>1.924760717201166</v>
+        <v>1.924761904761905</v>
       </c>
       <c r="O36" t="n">
         <v>0.85</v>
@@ -8900,7 +8900,7 @@
         <v>12348000</v>
       </c>
       <c r="AN36" t="n">
-        <v>37692284.43649374</v>
+        <v>37692307.6923077</v>
       </c>
       <c r="AO36" t="n">
         <v>0</v>
@@ -9039,7 +9039,7 @@
         <v>17</v>
       </c>
       <c r="H37" t="n">
-        <v>210699870</v>
+        <v>210700000</v>
       </c>
       <c r="I37" t="n">
         <v>1800</v>
@@ -9057,7 +9057,7 @@
         <v>7.41</v>
       </c>
       <c r="N37" t="n">
-        <v>1.924760717201166</v>
+        <v>1.924761904761905</v>
       </c>
       <c r="O37" t="n">
         <v>0.61</v>
@@ -9135,7 +9135,7 @@
         <v>12348000</v>
       </c>
       <c r="AN37" t="n">
-        <v>52412902.98507463</v>
+        <v>52412935.32338309</v>
       </c>
       <c r="AO37" t="n">
         <v>0</v>
@@ -11389,7 +11389,7 @@
         <v>8.5</v>
       </c>
       <c r="H47" t="n">
-        <v>2964926650</v>
+        <v>2979937000</v>
       </c>
       <c r="I47" t="n">
         <v>8000</v>
@@ -11407,7 +11407,7 @@
         <v>8.390000000000001</v>
       </c>
       <c r="N47" t="n">
-        <v>0.7953318877083194</v>
+        <v>0.7993583650583282</v>
       </c>
       <c r="O47" t="n">
         <v>0.07000000000000001</v>
@@ -11485,7 +11485,7 @@
         <v>249024468</v>
       </c>
       <c r="AN47" t="n">
-        <v>451282595.1293759</v>
+        <v>453567275.4946727</v>
       </c>
       <c r="AO47" t="n">
         <v>0.3403</v>
@@ -11624,7 +11624,7 @@
         <v>8.779999999999999</v>
       </c>
       <c r="H48" t="n">
-        <v>2964926650</v>
+        <v>2979937000</v>
       </c>
       <c r="I48" t="n">
         <v>3300</v>
@@ -11642,7 +11642,7 @@
         <v>8.449999999999999</v>
       </c>
       <c r="N48" t="n">
-        <v>2.163858586360961</v>
+        <v>2.174813418829341</v>
       </c>
       <c r="O48" t="n">
         <v>0.07000000000000001</v>
@@ -11720,7 +11720,7 @@
         <v>91529595.08</v>
       </c>
       <c r="AN48" t="n">
-        <v>447874116.3141994</v>
+        <v>450141540.7854985</v>
       </c>
       <c r="AO48" t="n">
         <v>0.3691</v>
@@ -11859,7 +11859,7 @@
         <v>52.43</v>
       </c>
       <c r="H49" t="n">
-        <v>980973900</v>
+        <v>980858500</v>
       </c>
       <c r="I49" t="n">
         <v>0</v>
@@ -11877,7 +11877,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="N49" t="n">
-        <v>1.071138156786464</v>
+        <v>1.071012150025944</v>
       </c>
       <c r="O49" t="n">
         <v>0.08</v>
@@ -11955,7 +11955,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN49" t="n">
-        <v>179337093.2358318</v>
+        <v>179315996.3436929</v>
       </c>
       <c r="AO49" t="n">
         <v>2.4346</v>
@@ -12094,7 +12094,7 @@
         <v>32.56</v>
       </c>
       <c r="H50" t="n">
-        <v>980973900</v>
+        <v>980858500</v>
       </c>
       <c r="I50" t="n">
         <v>200</v>
@@ -12112,7 +12112,7 @@
         <v>5.78</v>
       </c>
       <c r="N50" t="n">
-        <v>1.071138156786464</v>
+        <v>1.071012150025944</v>
       </c>
       <c r="O50" t="n">
         <v>0.06</v>
@@ -12190,7 +12190,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN50" t="n">
-        <v>257473464.5669291</v>
+        <v>257443175.8530184</v>
       </c>
       <c r="AO50" t="n">
         <v>3.526</v>
@@ -14428,7 +14428,7 @@
         <v>389.99</v>
       </c>
       <c r="H60" t="n">
-        <v>177347987</v>
+        <v>177347900</v>
       </c>
       <c r="I60" t="n">
         <v>87</v>
@@ -14446,7 +14446,7 @@
         <v>2.87</v>
       </c>
       <c r="N60" t="n">
-        <v>12.53253224385075</v>
+        <v>12.53252609587962</v>
       </c>
       <c r="O60" t="n">
         <v>0.64</v>
@@ -14524,7 +14524,7 @@
         <v>59731412.5</v>
       </c>
       <c r="AN60" t="n">
-        <v>22336018.5138539</v>
+        <v>22336007.55667506</v>
       </c>
       <c r="AO60" t="n">
         <v>0</v>
@@ -19598,7 +19598,7 @@
         <v>9.51</v>
       </c>
       <c r="H82" t="n">
-        <v>396963000</v>
+        <v>402036000</v>
       </c>
       <c r="I82" t="n">
         <v>19100</v>
@@ -19616,7 +19616,7 @@
         <v>6.04</v>
       </c>
       <c r="N82" t="n">
-        <v>1.009424996948557</v>
+        <v>1.022324972537012</v>
       </c>
       <c r="O82" t="n">
         <v>1.01</v>
@@ -19694,7 +19694,7 @@
         <v>65949124.8</v>
       </c>
       <c r="AN82" t="n">
-        <v>70633985.76512456</v>
+        <v>71536654.80427046</v>
       </c>
       <c r="AO82" t="n">
         <v>0</v>
@@ -21243,7 +21243,7 @@
         <v>26.94</v>
       </c>
       <c r="H89" t="n">
-        <v>2027170922</v>
+        <v>1998929000</v>
       </c>
       <c r="I89" t="n">
         <v>11200</v>
@@ -21261,7 +21261,7 @@
         <v>11.38</v>
       </c>
       <c r="N89" t="n">
-        <v>8.486284118953982</v>
+        <v>8.36805581784907</v>
       </c>
       <c r="O89" t="n">
         <v>1.53</v>
@@ -21339,7 +21339,7 @@
         <v>95908776.3</v>
       </c>
       <c r="AN89" t="n">
-        <v>221065531.2977099</v>
+        <v>217985714.2857143</v>
       </c>
       <c r="AO89" t="n">
         <v>0</v>
@@ -21478,7 +21478,7 @@
         <v>25.17</v>
       </c>
       <c r="H90" t="n">
-        <v>2027170922</v>
+        <v>1998929000</v>
       </c>
       <c r="I90" t="n">
         <v>24300</v>
@@ -21496,7 +21496,7 @@
         <v>10.59</v>
       </c>
       <c r="N90" t="n">
-        <v>46.43326946123355</v>
+        <v>45.78637542773225</v>
       </c>
       <c r="O90" t="n">
         <v>1.42</v>
@@ -21574,7 +21574,7 @@
         <v>17528576.7</v>
       </c>
       <c r="AN90" t="n">
-        <v>237651925.2051583</v>
+        <v>234341031.6529895</v>
       </c>
       <c r="AO90" t="n">
         <v>0</v>
@@ -21713,7 +21713,7 @@
         <v>29.26</v>
       </c>
       <c r="H91" t="n">
-        <v>2027170922</v>
+        <v>1998929000</v>
       </c>
       <c r="I91" t="n">
         <v>12200</v>
@@ -21731,7 +21731,7 @@
         <v>11.3</v>
       </c>
       <c r="N91" t="n">
-        <v>10.29986227354233</v>
+        <v>10.15636775920057</v>
       </c>
       <c r="O91" t="n">
         <v>1.52</v>
@@ -21809,7 +21809,7 @@
         <v>79021360.05</v>
       </c>
       <c r="AN91" t="n">
-        <v>222766035.3846154</v>
+        <v>219662527.4725275</v>
       </c>
       <c r="AO91" t="n">
         <v>0</v>
@@ -21948,7 +21948,7 @@
         <v>9</v>
       </c>
       <c r="H92" t="n">
-        <v>72970330</v>
+        <v>72798170</v>
       </c>
       <c r="I92" t="n">
         <v>0</v>
@@ -21966,7 +21966,7 @@
         <v>3.42</v>
       </c>
       <c r="N92" t="n">
-        <v>0.1347362592751558</v>
+        <v>0.1344183739867542</v>
       </c>
       <c r="O92" t="n">
         <v>0.15</v>
@@ -22044,7 +22044,7 @@
         <v>23342055.36</v>
       </c>
       <c r="AN92" t="n">
-        <v>51752007.09219859</v>
+        <v>51629907.80141845</v>
       </c>
       <c r="AO92" t="n">
         <v>0</v>
@@ -22183,7 +22183,7 @@
         <v>4.98</v>
       </c>
       <c r="H93" t="n">
-        <v>72970330</v>
+        <v>72798170</v>
       </c>
       <c r="I93" t="n">
         <v>400</v>
@@ -22201,7 +22201,7 @@
         <v>2.3</v>
       </c>
       <c r="N93" t="n">
-        <v>0.1791224022790859</v>
+        <v>0.1786997960941287</v>
       </c>
       <c r="O93" t="n">
         <v>0.1</v>
@@ -22279,7 +22279,7 @@
         <v>17557944.64</v>
       </c>
       <c r="AN93" t="n">
-        <v>76810873.68421052</v>
+        <v>76629652.63157895</v>
       </c>
       <c r="AO93" t="n">
         <v>0</v>
@@ -22418,7 +22418,7 @@
         <v>45.69</v>
       </c>
       <c r="H94" t="n">
-        <v>8073298000</v>
+        <v>8101992000</v>
       </c>
       <c r="I94" t="n">
         <v>0</v>
@@ -22436,7 +22436,7 @@
         <v>5.78</v>
       </c>
       <c r="N94" t="n">
-        <v>0.7580179513278035</v>
+        <v>0.7607120878622656</v>
       </c>
       <c r="O94" t="n">
         <v>0.36</v>
@@ -22514,7 +22514,7 @@
         <v>1209900967.64</v>
       </c>
       <c r="AN94" t="n">
-        <v>2904064028.776978</v>
+        <v>2914385611.510792</v>
       </c>
       <c r="AO94" t="n">
         <v>0</v>
@@ -22653,7 +22653,7 @@
         <v>43.01</v>
       </c>
       <c r="H95" t="n">
-        <v>8073298000</v>
+        <v>8101992000</v>
       </c>
       <c r="I95" t="n">
         <v>0</v>
@@ -22671,7 +22671,7 @@
         <v>4.65</v>
       </c>
       <c r="N95" t="n">
-        <v>4.23279295070503</v>
+        <v>4.247837082722395</v>
       </c>
       <c r="O95" t="n">
         <v>0.29</v>
@@ -22749,7 +22749,7 @@
         <v>216671749.24</v>
       </c>
       <c r="AN95" t="n">
-        <v>3604150892.857142</v>
+        <v>3616960714.285714</v>
       </c>
       <c r="AO95" t="n">
         <v>0</v>
@@ -23593,7 +23593,7 @@
         <v>126</v>
       </c>
       <c r="H99" t="n">
-        <v>16803020846</v>
+        <v>16637410000</v>
       </c>
       <c r="I99" t="n">
         <v>0</v>
@@ -23611,7 +23611,7 @@
         <v>10.65</v>
       </c>
       <c r="N99" t="n">
-        <v>1.660244200213289</v>
+        <v>1.64388080644714</v>
       </c>
       <c r="O99" t="n">
         <v>1.16</v>
@@ -23689,7 +23689,7 @@
         <v>1267125769.6</v>
       </c>
       <c r="AN99" t="n">
-        <v>2892086204.130809</v>
+        <v>2863581755.593804</v>
       </c>
       <c r="AO99" t="n">
         <v>0</v>
@@ -23828,7 +23828,7 @@
         <v>123.9</v>
       </c>
       <c r="H100" t="n">
-        <v>16803020846</v>
+        <v>16637410000</v>
       </c>
       <c r="I100" t="n">
         <v>300</v>
@@ -23846,7 +23846,7 @@
         <v>10.81</v>
       </c>
       <c r="N100" t="n">
-        <v>6.017120779152747</v>
+        <v>5.957815939156855</v>
       </c>
       <c r="O100" t="n">
         <v>1.18</v>
@@ -23924,7 +23924,7 @@
         <v>349625391.8</v>
       </c>
       <c r="AN100" t="n">
-        <v>2847969634.915254</v>
+        <v>2819900000</v>
       </c>
       <c r="AO100" t="n">
         <v>0</v>
@@ -24063,7 +24063,7 @@
         <v>24.69</v>
       </c>
       <c r="H101" t="n">
-        <v>637965451</v>
+        <v>631910000</v>
       </c>
       <c r="I101" t="n">
         <v>0</v>
@@ -24081,7 +24081,7 @@
         <v>6.28</v>
       </c>
       <c r="N101" t="n">
-        <v>2.057525054260267</v>
+        <v>2.037995403982472</v>
       </c>
       <c r="O101" t="n">
         <v>0.49</v>
@@ -24159,7 +24159,7 @@
         <v>42633867</v>
       </c>
       <c r="AN101" t="n">
-        <v>65973676.42192347</v>
+        <v>65347466.39089969</v>
       </c>
       <c r="AO101" t="n">
         <v>0</v>
@@ -24298,7 +24298,7 @@
         <v>24.7</v>
       </c>
       <c r="H102" t="n">
-        <v>637965451</v>
+        <v>631910000</v>
       </c>
       <c r="I102" t="n">
         <v>1300</v>
@@ -24316,7 +24316,7 @@
         <v>6.32</v>
       </c>
       <c r="N102" t="n">
-        <v>1.50531570100668</v>
+        <v>1.491027520584545</v>
       </c>
       <c r="O102" t="n">
         <v>0.49</v>
@@ -24394,7 +24394,7 @@
         <v>58273656.12</v>
       </c>
       <c r="AN102" t="n">
-        <v>65566850.05138746</v>
+        <v>64944501.54162384</v>
       </c>
       <c r="AO102" t="n">
         <v>0</v>
@@ -26883,7 +26883,7 @@
         <v>18</v>
       </c>
       <c r="H113" t="n">
-        <v>459493785</v>
+        <v>458736400</v>
       </c>
       <c r="I113" t="n">
         <v>0</v>
@@ -26901,7 +26901,7 @@
         <v>20.65</v>
       </c>
       <c r="N113" t="n">
-        <v>1.722119988623479</v>
+        <v>1.719281413021018</v>
       </c>
       <c r="O113" t="n">
         <v>0.54</v>
@@ -26979,7 +26979,7 @@
         <v>8431470.34</v>
       </c>
       <c r="AN113" t="n">
-        <v>34061807.63528539</v>
+        <v>34005663.45441067</v>
       </c>
       <c r="AO113" t="n">
         <v>0</v>
@@ -27118,7 +27118,7 @@
         <v>14.69</v>
       </c>
       <c r="H114" t="n">
-        <v>459493785</v>
+        <v>458736400</v>
       </c>
       <c r="I114" t="n">
         <v>2300</v>
@@ -27136,7 +27136,7 @@
         <v>23.27</v>
       </c>
       <c r="N114" t="n">
-        <v>1.417407462746446</v>
+        <v>1.415071145724939</v>
       </c>
       <c r="O114" t="n">
         <v>0.61</v>
@@ -27214,7 +27214,7 @@
         <v>10244057.54</v>
       </c>
       <c r="AN114" t="n">
-        <v>30249755.43120474</v>
+        <v>30199894.66754444</v>
       </c>
       <c r="AO114" t="n">
         <v>0</v>
@@ -27353,7 +27353,7 @@
         <v>14.51</v>
       </c>
       <c r="H115" t="n">
-        <v>459493785</v>
+        <v>458736400</v>
       </c>
       <c r="I115" t="n">
         <v>0</v>
@@ -27371,7 +27371,7 @@
         <v>22.56</v>
       </c>
       <c r="N115" t="n">
-        <v>2.683903395967447</v>
+        <v>2.679479509856442</v>
       </c>
       <c r="O115" t="n">
         <v>0.59</v>
@@ -27449,7 +27449,7 @@
         <v>5410032.13</v>
       </c>
       <c r="AN115" t="n">
-        <v>31194418.53360489</v>
+        <v>31143000.67888663</v>
       </c>
       <c r="AO115" t="n">
         <v>0</v>
@@ -28763,7 +28763,7 @@
         <v>0.46</v>
       </c>
       <c r="H121" t="n">
-        <v>12286756</v>
+        <v>12286760</v>
       </c>
       <c r="I121" t="n">
         <v>100</v>
@@ -28781,7 +28781,7 @@
         <v>0.19</v>
       </c>
       <c r="N121" t="n">
-        <v>0.02837141065277318</v>
+        <v>0.02837141988919348</v>
       </c>
       <c r="O121" t="n">
         <v>0.02</v>
@@ -28859,7 +28859,7 @@
         <v>129011019.48</v>
       </c>
       <c r="AN121" t="n">
-        <v>4109282.943143812</v>
+        <v>4109284.280936454</v>
       </c>
       <c r="AO121" t="n">
         <v>0</v>
@@ -32758,7 +32758,7 @@
         <v>4.74</v>
       </c>
       <c r="H138" t="n">
-        <v>63146134</v>
+        <v>63146180</v>
       </c>
       <c r="I138" t="n">
         <v>82800</v>
@@ -32776,7 +32776,7 @@
         <v>15.76</v>
       </c>
       <c r="N138" t="n">
-        <v>0.3363140635150498</v>
+        <v>0.3363143085094135</v>
       </c>
       <c r="O138" t="n">
         <v>0.2</v>
@@ -32854,7 +32854,7 @@
         <v>2797615.38</v>
       </c>
       <c r="AN138" t="n">
-        <v>32888611.45833334</v>
+        <v>32888635.41666667</v>
       </c>
       <c r="AO138" t="n">
         <v>0</v>
@@ -34403,7 +34403,7 @@
         <v>51.52</v>
       </c>
       <c r="H145" t="n">
-        <v>8650398000</v>
+        <v>8681144000</v>
       </c>
       <c r="I145" t="n">
         <v>0</v>
@@ -34421,7 +34421,7 @@
         <v>10.18</v>
       </c>
       <c r="N145" t="n">
-        <v>1.869227543924982</v>
+        <v>1.875871315698895</v>
       </c>
       <c r="O145" t="n">
         <v>0.73</v>
@@ -34499,7 +34499,7 @@
         <v>441028665.6</v>
       </c>
       <c r="AN145" t="n">
-        <v>1988597241.379311</v>
+        <v>1995665287.356322</v>
       </c>
       <c r="AO145" t="n">
         <v>0</v>
@@ -34638,7 +34638,7 @@
         <v>38.86</v>
       </c>
       <c r="H146" t="n">
-        <v>8650398000</v>
+        <v>8681144000</v>
       </c>
       <c r="I146" t="n">
         <v>0</v>
@@ -34656,7 +34656,7 @@
         <v>8.16</v>
       </c>
       <c r="N146" t="n">
-        <v>1.685800169669117</v>
+        <v>1.691791987850968</v>
       </c>
       <c r="O146" t="n">
         <v>0.58</v>
@@ -34734,7 +34734,7 @@
         <v>489015806.4</v>
       </c>
       <c r="AN146" t="n">
-        <v>2478624068.767908</v>
+        <v>2487433810.888252</v>
       </c>
       <c r="AO146" t="n">
         <v>0</v>
@@ -37223,7 +37223,7 @@
         <v>5.85</v>
       </c>
       <c r="H157" t="n">
-        <v>41818670</v>
+        <v>40407480</v>
       </c>
       <c r="I157" t="n">
         <v>59700</v>
@@ -37241,7 +37241,7 @@
         <v>8.27</v>
       </c>
       <c r="N157" t="n">
-        <v>0.003502876867757888</v>
+        <v>0.003384670697953558</v>
       </c>
       <c r="O157" t="n">
         <v>0.62</v>
@@ -37319,7 +37319,7 @@
         <v>1653465426.75</v>
       </c>
       <c r="AN157" t="n">
-        <v>6993088.628762541</v>
+        <v>6757103.678929766</v>
       </c>
       <c r="AO157" t="n">
         <v>0</v>
@@ -37458,7 +37458,7 @@
         <v>10.5</v>
       </c>
       <c r="H158" t="n">
-        <v>41818670</v>
+        <v>40407480</v>
       </c>
       <c r="I158" t="n">
         <v>100</v>
@@ -37476,7 +37476,7 @@
         <v>14.74</v>
       </c>
       <c r="N158" t="n">
-        <v>3.563991771028704</v>
+        <v>3.443723251074387</v>
       </c>
       <c r="O158" t="n">
         <v>1.1</v>
@@ -37554,7 +37554,7 @@
         <v>1625112</v>
       </c>
       <c r="AN158" t="n">
-        <v>3926635.680751174</v>
+        <v>3794129.577464789</v>
       </c>
       <c r="AO158" t="n">
         <v>0</v>
@@ -37693,7 +37693,7 @@
         <v>6.59</v>
       </c>
       <c r="H159" t="n">
-        <v>41818670</v>
+        <v>40407480</v>
       </c>
       <c r="I159" t="n">
         <v>0</v>
@@ -37711,7 +37711,7 @@
         <v>8.83</v>
       </c>
       <c r="N159" t="n">
-        <v>7.115078773226653</v>
+        <v>6.874977210599488</v>
       </c>
       <c r="O159" t="n">
         <v>0.66</v>
@@ -37789,7 +37789,7 @@
         <v>814029.75</v>
       </c>
       <c r="AN159" t="n">
-        <v>6554650.470219436</v>
+        <v>6333460.815047022</v>
       </c>
       <c r="AO159" t="n">
         <v>0</v>
@@ -37928,7 +37928,7 @@
         <v>10.04</v>
       </c>
       <c r="H160" t="n">
-        <v>41818670</v>
+        <v>40407480</v>
       </c>
       <c r="I160" t="n">
         <v>0</v>
@@ -37946,7 +37946,7 @@
         <v>13.4</v>
       </c>
       <c r="N160" t="n">
-        <v>6.428737416916336</v>
+        <v>6.21179675487763</v>
       </c>
       <c r="O160" t="n">
         <v>1</v>
@@ -38024,7 +38024,7 @@
         <v>900936.75</v>
       </c>
       <c r="AN160" t="n">
-        <v>4320110.537190082</v>
+        <v>4174326.446280992</v>
       </c>
       <c r="AO160" t="n">
         <v>0</v>
@@ -39103,7 +39103,7 @@
         <v>3.61</v>
       </c>
       <c r="H165" t="n">
-        <v>223013375</v>
+        <v>223013400</v>
       </c>
       <c r="I165" t="n">
         <v>49300</v>
@@ -39121,7 +39121,7 @@
         <v>5.28</v>
       </c>
       <c r="N165" t="n">
-        <v>0.1909499479842438</v>
+        <v>0.1909499693899048</v>
       </c>
       <c r="O165" t="n">
         <v>0.18</v>
@@ -39199,7 +39199,7 @@
         <v>46950197</v>
       </c>
       <c r="AN165" t="n">
-        <v>24806827.03003337</v>
+        <v>24806829.810901</v>
       </c>
       <c r="AO165" t="n">
         <v>0</v>
@@ -40748,7 +40748,7 @@
         <v>3.95</v>
       </c>
       <c r="H172" t="n">
-        <v>212736258</v>
+        <v>212736300</v>
       </c>
       <c r="I172" t="n">
         <v>1100</v>
@@ -40766,7 +40766,7 @@
         <v>0.38</v>
       </c>
       <c r="N172" t="n">
-        <v>0.04710125744878763</v>
+        <v>0.04710126674787388</v>
       </c>
       <c r="O172" t="n">
         <v>0.08</v>
@@ -40844,7 +40844,7 @@
         <v>640901679.6</v>
       </c>
       <c r="AN172" t="n">
-        <v>212736258</v>
+        <v>212736300</v>
       </c>
       <c r="AO172" t="n">
         <v>0</v>
@@ -45448,7 +45448,7 @@
         <v>2.5</v>
       </c>
       <c r="H192" t="n">
-        <v>22908640</v>
+        <v>22530670</v>
       </c>
       <c r="I192" t="n">
         <v>7800</v>
@@ -45466,7 +45466,7 @@
         <v>21.95</v>
       </c>
       <c r="N192" t="n">
-        <v>2.342199691131678</v>
+        <v>2.303555702782434</v>
       </c>
       <c r="O192" t="n">
         <v>0.32</v>
@@ -45544,7 +45544,7 @@
         <v>357000.03</v>
       </c>
       <c r="AN192" t="n">
-        <v>1926714.886459209</v>
+        <v>1894925.9882254</v>
       </c>
       <c r="AO192" t="n">
         <v>0</v>
@@ -45683,7 +45683,7 @@
         <v>1.59</v>
       </c>
       <c r="H193" t="n">
-        <v>22908640</v>
+        <v>22530670</v>
       </c>
       <c r="I193" t="n">
         <v>14300</v>
@@ -45701,7 +45701,7 @@
         <v>14.71</v>
       </c>
       <c r="N193" t="n">
-        <v>1.171099993183473</v>
+        <v>1.151777996573305</v>
       </c>
       <c r="O193" t="n">
         <v>0.22</v>
@@ -45779,7 +45779,7 @@
         <v>713999.97</v>
       </c>
       <c r="AN193" t="n">
-        <v>2874358.845671267</v>
+        <v>2826934.755332497</v>
       </c>
       <c r="AO193" t="n">
         <v>0</v>
@@ -47563,7 +47563,7 @@
         <v>7.1</v>
       </c>
       <c r="H201" t="n">
-        <v>132856334</v>
+        <v>130444100</v>
       </c>
       <c r="I201" t="n">
         <v>100</v>
@@ -47581,7 +47581,7 @@
         <v>1.99</v>
       </c>
       <c r="N201" t="n">
-        <v>1.56794656880877</v>
+        <v>1.539477816814876</v>
       </c>
       <c r="O201" t="n">
         <v>0.25</v>
@@ -47659,7 +47659,7 @@
         <v>28893848.04</v>
       </c>
       <c r="AN201" t="n">
-        <v>105441534.9206349</v>
+        <v>103527063.4920635</v>
       </c>
       <c r="AO201" t="n">
         <v>0</v>
@@ -48006,7 +48006,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>IBOVESPA</t>
+          <t>Brazil Stock Exchange Index</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
@@ -58357,7 +58357,7 @@
         <v>5.37</v>
       </c>
       <c r="H247" t="n">
-        <v>19954753</v>
+        <v>19954750</v>
       </c>
       <c r="I247" t="n">
         <v>200</v>
@@ -58375,7 +58375,7 @@
         <v>4.4</v>
       </c>
       <c r="N247" t="n">
-        <v>0.03002960446556896</v>
+        <v>0.03002959995091456</v>
       </c>
       <c r="O247" t="n">
         <v>0.05</v>
@@ -58453,7 +58453,7 @@
         <v>5648272.88</v>
       </c>
       <c r="AN247" t="n">
-        <v>33821615.25423729</v>
+        <v>33821610.16949153</v>
       </c>
       <c r="AO247" t="n">
         <v>0</v>
@@ -59767,7 +59767,7 @@
         <v>18.68</v>
       </c>
       <c r="H253" t="n">
-        <v>185324992</v>
+        <v>185325000</v>
       </c>
       <c r="I253" t="n">
         <v>500</v>
@@ -59785,7 +59785,7 @@
         <v>7.29</v>
       </c>
       <c r="N253" t="n">
-        <v>0.1852812656213134</v>
+        <v>0.1852812736194258</v>
       </c>
       <c r="O253" t="n">
         <v>0.12</v>
@@ -59863,7 +59863,7 @@
         <v>24405758.4</v>
       </c>
       <c r="AN253" t="n">
-        <v>127810339.3103448</v>
+        <v>127810344.8275862</v>
       </c>
       <c r="AO253" t="n">
         <v>0</v>
@@ -60707,7 +60707,7 @@
         <v>41.6</v>
       </c>
       <c r="H257" t="n">
-        <v>12605950000</v>
+        <v>13049630000</v>
       </c>
       <c r="I257" t="n">
         <v>500</v>
@@ -60725,7 +60725,7 @@
         <v>9.57</v>
       </c>
       <c r="N257" t="n">
-        <v>3.140831275334276</v>
+        <v>3.251376218019303</v>
       </c>
       <c r="O257" t="n">
         <v>0.64</v>
@@ -60803,7 +60803,7 @@
         <v>836829598.4699999</v>
       </c>
       <c r="AN257" t="n">
-        <v>2291990909.090909</v>
+        <v>2372660000</v>
       </c>
       <c r="AO257" t="n">
         <v>0</v>
@@ -60942,7 +60942,7 @@
         <v>38</v>
       </c>
       <c r="H258" t="n">
-        <v>12605950000</v>
+        <v>13049630000</v>
       </c>
       <c r="I258" t="n">
         <v>0</v>
@@ -60960,7 +60960,7 @@
         <v>8.94</v>
       </c>
       <c r="N258" t="n">
-        <v>7.206883104232624</v>
+        <v>7.460537124412454</v>
       </c>
       <c r="O258" t="n">
         <v>0.59</v>
@@ -61038,7 +61038,7 @@
         <v>364698655.02</v>
       </c>
       <c r="AN258" t="n">
-        <v>2452519455.252918</v>
+        <v>2538838521.400778</v>
       </c>
       <c r="AO258" t="n">
         <v>0</v>
@@ -61177,7 +61177,7 @@
         <v>32.6</v>
       </c>
       <c r="H259" t="n">
-        <v>12605950000</v>
+        <v>13049630000</v>
       </c>
       <c r="I259" t="n">
         <v>0</v>
@@ -61195,7 +61195,7 @@
         <v>9.949999999999999</v>
       </c>
       <c r="N259" t="n">
-        <v>8.499656865194911</v>
+        <v>8.798811451556881</v>
       </c>
       <c r="O259" t="n">
         <v>0.66</v>
@@ -61273,7 +61273,7 @@
         <v>309229021.44</v>
       </c>
       <c r="AN259" t="n">
-        <v>2203837412.587413</v>
+        <v>2281403846.153846</v>
       </c>
       <c r="AO259" t="n">
         <v>0</v>
@@ -67287,7 +67287,7 @@
         <v>1.38</v>
       </c>
       <c r="H285" t="n">
-        <v>4536729</v>
+        <v>4536730</v>
       </c>
       <c r="I285" t="n">
         <v>1700</v>
@@ -67305,7 +67305,7 @@
         <v>0.05</v>
       </c>
       <c r="N285" t="n">
-        <v>0.04598813384405983</v>
+        <v>0.04598814398090818</v>
       </c>
       <c r="O285" t="n">
         <v>0.02</v>
@@ -67383,7 +67383,7 @@
         <v>178674864.1</v>
       </c>
       <c r="AN285" t="n">
-        <v>22683645</v>
+        <v>22683650</v>
       </c>
       <c r="AO285" t="n">
         <v>0</v>
@@ -67757,7 +67757,7 @@
         <v>39.8</v>
       </c>
       <c r="H287" t="n">
-        <v>724318126</v>
+        <v>722636900</v>
       </c>
       <c r="I287" t="n">
         <v>1900</v>
@@ -67775,7 +67775,7 @@
         <v>21.05</v>
       </c>
       <c r="N287" t="n">
-        <v>12.21925537597557</v>
+        <v>12.19089307341637</v>
       </c>
       <c r="O287" t="n">
         <v>0.54</v>
@@ -67853,7 +67853,7 @@
         <v>16864244.22</v>
       </c>
       <c r="AN287" t="n">
-        <v>30459130.61396131</v>
+        <v>30388431.4550042</v>
       </c>
       <c r="AO287" t="n">
         <v>0.3943</v>
@@ -67992,7 +67992,7 @@
         <v>39.88</v>
       </c>
       <c r="H288" t="n">
-        <v>724318126</v>
+        <v>722636900</v>
       </c>
       <c r="I288" t="n">
         <v>1900</v>
@@ -68010,7 +68010,7 @@
         <v>21.15</v>
       </c>
       <c r="N288" t="n">
-        <v>12.90565865025665</v>
+        <v>12.87570312644592</v>
       </c>
       <c r="O288" t="n">
         <v>0.54</v>
@@ -68088,7 +68088,7 @@
         <v>15967298.72</v>
       </c>
       <c r="AN288" t="n">
-        <v>30306197.74058577</v>
+        <v>30235853.55648536</v>
       </c>
       <c r="AO288" t="n">
         <v>0.4337</v>
@@ -72654,7 +72654,7 @@
         <v>0.48</v>
       </c>
       <c r="BU307" t="n">
-        <v>357</v>
+        <v>217</v>
       </c>
     </row>
     <row r="308">
@@ -72889,7 +72889,7 @@
         <v>0.48</v>
       </c>
       <c r="BU308" t="n">
-        <v>2777</v>
+        <v>967</v>
       </c>
     </row>
     <row r="309">
@@ -75512,7 +75512,7 @@
         <v>5.97</v>
       </c>
       <c r="H320" t="n">
-        <v>15306577982</v>
+        <v>15332180000</v>
       </c>
       <c r="I320" t="n">
         <v>2300</v>
@@ -75530,7 +75530,7 @@
         <v>11.35</v>
       </c>
       <c r="N320" t="n">
-        <v>0.78889143285971</v>
+        <v>0.7902109448164564</v>
       </c>
       <c r="O320" t="n">
         <v>0.49</v>
@@ -75608,7 +75608,7 @@
         <v>1412512331.45</v>
       </c>
       <c r="AN320" t="n">
-        <v>3386411057.964602</v>
+        <v>3392075221.238938</v>
       </c>
       <c r="AO320" t="n">
         <v>0</v>
@@ -75982,7 +75982,7 @@
         <v>0.9</v>
       </c>
       <c r="H322" t="n">
-        <v>334611081</v>
+        <v>335221100</v>
       </c>
       <c r="I322" t="n">
         <v>15200</v>
@@ -76000,7 +76000,7 @@
         <v>2.24</v>
       </c>
       <c r="N322" t="n">
-        <v>0.8481030213714283</v>
+        <v>0.8496491714733552</v>
       </c>
       <c r="O322" t="n">
         <v>0.13</v>
@@ -76078,7 +76078,7 @@
         <v>142942061.98</v>
       </c>
       <c r="AN322" t="n">
-        <v>26919636.44408689</v>
+        <v>26968712.79163315</v>
       </c>
       <c r="AO322" t="n">
         <v>0</v>
@@ -76217,7 +76217,7 @@
         <v>0.89</v>
       </c>
       <c r="H323" t="n">
-        <v>334611081</v>
+        <v>335221100</v>
       </c>
       <c r="I323" t="n">
         <v>8200</v>
@@ -76235,7 +76235,7 @@
         <v>2</v>
       </c>
       <c r="N323" t="n">
-        <v>4.225403664963229</v>
+        <v>4.233106866275612</v>
       </c>
       <c r="O323" t="n">
         <v>0.11</v>
@@ -76313,7 +76313,7 @@
         <v>28690654.02</v>
       </c>
       <c r="AN323" t="n">
-        <v>30172324.70694319</v>
+        <v>30227330.92876465</v>
       </c>
       <c r="AO323" t="n">
         <v>0</v>
@@ -77392,7 +77392,7 @@
         <v>1.26</v>
       </c>
       <c r="H328" t="n">
-        <v>85291440</v>
+        <v>85291450</v>
       </c>
       <c r="I328" t="n">
         <v>10200</v>
@@ -77410,7 +77410,7 @@
         <v>0.11</v>
       </c>
       <c r="N328" t="n">
-        <v>0.009865114828648247</v>
+        <v>0.009865115985284228</v>
       </c>
       <c r="O328" t="n">
         <v>0.02</v>
@@ -77488,7 +77488,7 @@
         <v>1659121826.79</v>
       </c>
       <c r="AN328" t="n">
-        <v>852914400</v>
+        <v>852914500</v>
       </c>
       <c r="AO328" t="n">
         <v>0</v>
@@ -80682,7 +80682,7 @@
         <v>5.9</v>
       </c>
       <c r="H342" t="n">
-        <v>400458730</v>
+        <v>397734600</v>
       </c>
       <c r="I342" t="n">
         <v>13500</v>
@@ -80700,7 +80700,7 @@
         <v>0.62</v>
       </c>
       <c r="N342" t="n">
-        <v>2.708591783149547</v>
+        <v>2.690166523362524</v>
       </c>
       <c r="O342" t="n">
         <v>0.1</v>
@@ -80778,7 +80778,7 @@
         <v>61075833.72000001</v>
       </c>
       <c r="AN342" t="n">
-        <v>435281228.2608696</v>
+        <v>432320217.3913043</v>
       </c>
       <c r="AO342" t="n">
         <v>0</v>
@@ -85617,7 +85617,7 @@
         <v>0.86</v>
       </c>
       <c r="H363" t="n">
-        <v>77839555</v>
+        <v>77839560</v>
       </c>
       <c r="I363" t="n">
         <v>89500</v>
@@ -85635,7 +85635,7 @@
         <v>0.74</v>
       </c>
       <c r="N363" t="n">
-        <v>0.2753335083286167</v>
+        <v>0.2753335260145804</v>
       </c>
       <c r="O363" t="n">
         <v>0.11</v>
@@ -85713,7 +85713,7 @@
         <v>163434690.6</v>
       </c>
       <c r="AN363" t="n">
-        <v>73433542.45283018</v>
+        <v>73433547.16981132</v>
       </c>
       <c r="AO363" t="n">
         <v>0</v>
@@ -86087,7 +86087,7 @@
         <v>10.4</v>
       </c>
       <c r="H365" t="n">
-        <v>1009206838</v>
+        <v>1006878000</v>
       </c>
       <c r="I365" t="n">
         <v>0</v>
@@ -86105,7 +86105,7 @@
         <v>20.34</v>
       </c>
       <c r="N365" t="n">
-        <v>2.669746006171991</v>
+        <v>2.663585320655985</v>
       </c>
       <c r="O365" t="n">
         <v>0.27</v>
@@ -86183,7 +86183,7 @@
         <v>45966751.6</v>
       </c>
       <c r="AN365" t="n">
-        <v>107362429.5744681</v>
+        <v>107114680.8510638</v>
       </c>
       <c r="AO365" t="n">
         <v>0</v>
@@ -86322,7 +86322,7 @@
         <v>7.48</v>
       </c>
       <c r="H366" t="n">
-        <v>1009206838</v>
+        <v>1006878000</v>
       </c>
       <c r="I366" t="n">
         <v>600</v>
@@ -86340,7 +86340,7 @@
         <v>14.31</v>
       </c>
       <c r="N366" t="n">
-        <v>12.12150299430714</v>
+        <v>12.09353150647399</v>
       </c>
       <c r="O366" t="n">
         <v>0.19</v>
@@ -86418,7 +86418,7 @@
         <v>10124120.05</v>
       </c>
       <c r="AN366" t="n">
-        <v>152678795.4614221</v>
+        <v>152326475.0378215</v>
       </c>
       <c r="AO366" t="n">
         <v>0</v>
@@ -89612,7 +89612,7 @@
         <v>1.2</v>
       </c>
       <c r="H380" t="n">
-        <v>79303635</v>
+        <v>79303640</v>
       </c>
       <c r="I380" t="n">
         <v>9400</v>
@@ -89630,7 +89630,7 @@
         <v>39.8</v>
       </c>
       <c r="N380" t="n">
-        <v>0.2939999933269138</v>
+        <v>0.2940000118632642</v>
       </c>
       <c r="O380" t="n">
         <v>0.24</v>
@@ -89708,7 +89708,7 @@
         <v>2643454.56</v>
       </c>
       <c r="AN380" t="n">
-        <v>7488539.660056657</v>
+        <v>7488540.132200189</v>
       </c>
       <c r="AO380" t="n">
         <v>0</v>
@@ -92667,7 +92667,7 @@
         <v>1.67</v>
       </c>
       <c r="H393" t="n">
-        <v>8149668</v>
+        <v>8149670</v>
       </c>
       <c r="I393" t="n">
         <v>8900</v>
@@ -92685,7 +92685,7 @@
         <v>1.29</v>
       </c>
       <c r="N393" t="n">
-        <v>1.453966171536439</v>
+        <v>1.453966528352489</v>
       </c>
       <c r="O393" t="n">
         <v>0.13</v>
@@ -92763,7 +92763,7 @@
         <v>2293618.8</v>
       </c>
       <c r="AN393" t="n">
-        <v>5361623.684210526</v>
+        <v>5361625</v>
       </c>
       <c r="AO393" t="n">
         <v>0</v>
@@ -95487,7 +95487,7 @@
         <v>20.69</v>
       </c>
       <c r="H405" t="n">
-        <v>737215364</v>
+        <v>724299600</v>
       </c>
       <c r="I405" t="n">
         <v>0</v>
@@ -95505,7 +95505,7 @@
         <v>6.94</v>
       </c>
       <c r="N405" t="n">
-        <v>0.5302712748245911</v>
+        <v>0.5209811013202669</v>
       </c>
       <c r="O405" t="n">
         <v>0.53</v>
@@ -95583,7 +95583,7 @@
         <v>53525040.6</v>
       </c>
       <c r="AN405" t="n">
-        <v>181580138.9162562</v>
+        <v>178398916.2561577</v>
       </c>
       <c r="AO405" t="n">
         <v>0.9505</v>
@@ -95722,7 +95722,7 @@
         <v>19.44</v>
       </c>
       <c r="H406" t="n">
-        <v>737215364</v>
+        <v>724299600</v>
       </c>
       <c r="I406" t="n">
         <v>100</v>
@@ -95740,7 +95740,7 @@
         <v>7.58</v>
       </c>
       <c r="N406" t="n">
-        <v>0.4428283365442381</v>
+        <v>0.4350701337630519</v>
       </c>
       <c r="O406" t="n">
         <v>0.58</v>
@@ -95818,7 +95818,7 @@
         <v>64094343.5</v>
       </c>
       <c r="AN406" t="n">
-        <v>166414303.3860045</v>
+        <v>163498781.0383747</v>
       </c>
       <c r="AO406" t="n">
         <v>0.7018</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-07-13 04:35
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -8804,7 +8804,7 @@
         <v>26</v>
       </c>
       <c r="H36" t="n">
-        <v>210650851</v>
+        <v>210651000</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
@@ -8822,7 +8822,7 @@
         <v>10.3</v>
       </c>
       <c r="N36" t="n">
-        <v>1.924312924586978</v>
+        <v>1.924314285714286</v>
       </c>
       <c r="O36" t="n">
         <v>0.85</v>
@@ -8900,7 +8900,7 @@
         <v>12348000</v>
       </c>
       <c r="AN36" t="n">
-        <v>37683515.38461538</v>
+        <v>37683542.03935599</v>
       </c>
       <c r="AO36" t="n">
         <v>0</v>
@@ -9039,7 +9039,7 @@
         <v>16.99</v>
       </c>
       <c r="H37" t="n">
-        <v>210650851</v>
+        <v>210651000</v>
       </c>
       <c r="I37" t="n">
         <v>600</v>
@@ -9057,7 +9057,7 @@
         <v>7.41</v>
       </c>
       <c r="N37" t="n">
-        <v>1.924312924586978</v>
+        <v>1.924314285714286</v>
       </c>
       <c r="O37" t="n">
         <v>0.61</v>
@@ -9135,7 +9135,7 @@
         <v>12348000</v>
       </c>
       <c r="AN37" t="n">
-        <v>52400709.2039801</v>
+        <v>52400746.26865672</v>
       </c>
       <c r="AO37" t="n">
         <v>0</v>
@@ -10684,7 +10684,7 @@
         <v>6.01</v>
       </c>
       <c r="H44" t="n">
-        <v>7530027</v>
+        <v>7610530</v>
       </c>
       <c r="I44" t="n">
         <v>0</v>
@@ -10702,7 +10702,7 @@
         <v>0.75</v>
       </c>
       <c r="N44" t="n">
-        <v>0.3364964131011184</v>
+        <v>0.3400938730762127</v>
       </c>
       <c r="O44" t="n">
         <v>0.03</v>
@@ -10780,7 +10780,7 @@
         <v>5719748.64</v>
       </c>
       <c r="AN44" t="n">
-        <v>7530027</v>
+        <v>7610530</v>
       </c>
       <c r="AO44" t="n">
         <v>0</v>
@@ -10919,7 +10919,7 @@
         <v>3.99</v>
       </c>
       <c r="H45" t="n">
-        <v>7530027</v>
+        <v>7610530</v>
       </c>
       <c r="I45" t="n">
         <v>600</v>
@@ -10937,7 +10937,7 @@
         <v>0.63</v>
       </c>
       <c r="N45" t="n">
-        <v>0.2057980294917993</v>
+        <v>0.2079982020500356</v>
       </c>
       <c r="O45" t="n">
         <v>0.02</v>
@@ -11015,7 +11015,7 @@
         <v>9352251.359999999</v>
       </c>
       <c r="AN45" t="n">
-        <v>8964317.857142858</v>
+        <v>9060154.761904763</v>
       </c>
       <c r="AO45" t="n">
         <v>0</v>
@@ -11389,7 +11389,7 @@
         <v>8.68</v>
       </c>
       <c r="H47" t="n">
-        <v>3026716974</v>
+        <v>3027544000</v>
       </c>
       <c r="I47" t="n">
         <v>18900</v>
@@ -11407,7 +11407,7 @@
         <v>8.390000000000001</v>
       </c>
       <c r="N47" t="n">
-        <v>0.8119069402577741</v>
+        <v>0.812128787280453</v>
       </c>
       <c r="O47" t="n">
         <v>0.07000000000000001</v>
@@ -11485,7 +11485,7 @@
         <v>249024468</v>
       </c>
       <c r="AN47" t="n">
-        <v>460687515.0684931</v>
+        <v>460813394.2161339</v>
       </c>
       <c r="AO47" t="n">
         <v>0.3403</v>
@@ -11624,7 +11624,7 @@
         <v>8.800000000000001</v>
       </c>
       <c r="H48" t="n">
-        <v>3026716974</v>
+        <v>3027544000</v>
       </c>
       <c r="I48" t="n">
         <v>4700</v>
@@ -11642,7 +11642,7 @@
         <v>8.449999999999999</v>
       </c>
       <c r="N48" t="n">
-        <v>2.208954313481707</v>
+        <v>2.209557892430698</v>
       </c>
       <c r="O48" t="n">
         <v>0.07000000000000001</v>
@@ -11720,7 +11720,7 @@
         <v>91529595.08</v>
       </c>
       <c r="AN48" t="n">
-        <v>457208002.1148036</v>
+        <v>457332930.5135952</v>
       </c>
       <c r="AO48" t="n">
         <v>0.3691</v>
@@ -11859,7 +11859,7 @@
         <v>48.01</v>
       </c>
       <c r="H49" t="n">
-        <v>921887027</v>
+        <v>943466100</v>
       </c>
       <c r="I49" t="n">
         <v>1300</v>
@@ -11877,7 +11877,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="N49" t="n">
-        <v>1.006620431864836</v>
+        <v>1.030182902261226</v>
       </c>
       <c r="O49" t="n">
         <v>0.08</v>
@@ -11955,7 +11955,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN49" t="n">
-        <v>168535105.4844607</v>
+        <v>172480091.4076782</v>
       </c>
       <c r="AO49" t="n">
         <v>2.4346</v>
@@ -12094,7 +12094,7 @@
         <v>33.74</v>
       </c>
       <c r="H50" t="n">
-        <v>921887027</v>
+        <v>943466100</v>
       </c>
       <c r="I50" t="n">
         <v>900</v>
@@ -12112,7 +12112,7 @@
         <v>5.78</v>
       </c>
       <c r="N50" t="n">
-        <v>1.006620431864836</v>
+        <v>1.030182902261226</v>
       </c>
       <c r="O50" t="n">
         <v>0.06</v>
@@ -12190,7 +12190,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN50" t="n">
-        <v>241965098.9501312</v>
+        <v>247628897.6377953</v>
       </c>
       <c r="AO50" t="n">
         <v>3.526</v>
@@ -14428,7 +14428,7 @@
         <v>387</v>
       </c>
       <c r="H60" t="n">
-        <v>175988172</v>
+        <v>175988300</v>
       </c>
       <c r="I60" t="n">
         <v>8</v>
@@ -14446,7 +14446,7 @@
         <v>2.87</v>
       </c>
       <c r="N60" t="n">
-        <v>12.43643910165359</v>
+        <v>12.43644814694446</v>
       </c>
       <c r="O60" t="n">
         <v>0.64</v>
@@ -14524,7 +14524,7 @@
         <v>59731412.5</v>
       </c>
       <c r="AN60" t="n">
-        <v>22164757.17884131</v>
+        <v>22164773.29974811</v>
       </c>
       <c r="AO60" t="n">
         <v>0</v>
@@ -14898,7 +14898,7 @@
         <v>112</v>
       </c>
       <c r="H62" t="n">
-        <v>11054373120</v>
+        <v>11054370000</v>
       </c>
       <c r="I62" t="n">
         <v>300</v>
@@ -14916,7 +14916,7 @@
         <v>4.26</v>
       </c>
       <c r="N62" t="n">
-        <v>1.129790335704332</v>
+        <v>1.129790016830905</v>
       </c>
       <c r="O62" t="n">
         <v>0.17</v>
@@ -14994,7 +14994,7 @@
         <v>2822812821.4</v>
       </c>
       <c r="AN62" t="n">
-        <v>4530480786.885246</v>
+        <v>4530479508.196721</v>
       </c>
       <c r="AO62" t="n">
         <v>0</v>
@@ -18893,7 +18893,7 @@
         <v>3</v>
       </c>
       <c r="H79" t="n">
-        <v>6357741000</v>
+        <v>6386264000</v>
       </c>
       <c r="I79" t="n">
         <v>22900</v>
@@ -18911,7 +18911,7 @@
         <v>2.47</v>
       </c>
       <c r="N79" t="n">
-        <v>0.8889333557192363</v>
+        <v>0.892921414702007</v>
       </c>
       <c r="O79" t="n">
         <v>0.03</v>
@@ -18989,7 +18989,7 @@
         <v>531401092.4</v>
       </c>
       <c r="AN79" t="n">
-        <v>3853176363.636364</v>
+        <v>3870463030.30303</v>
       </c>
       <c r="AO79" t="n">
         <v>0</v>
@@ -19128,7 +19128,7 @@
         <v>2.99</v>
       </c>
       <c r="H80" t="n">
-        <v>6357741000</v>
+        <v>6386264000</v>
       </c>
       <c r="I80" t="n">
         <v>6000</v>
@@ -19146,7 +19146,7 @@
         <v>3.36</v>
       </c>
       <c r="N80" t="n">
-        <v>1.713636336502429</v>
+        <v>1.721324295044002</v>
       </c>
       <c r="O80" t="n">
         <v>0.04</v>
@@ -19224,7 +19224,7 @@
         <v>275659512.02</v>
       </c>
       <c r="AN80" t="n">
-        <v>2825662666.666667</v>
+        <v>2838339555.555555</v>
       </c>
       <c r="AO80" t="n">
         <v>0</v>
@@ -19598,7 +19598,7 @@
         <v>9.48</v>
       </c>
       <c r="H82" t="n">
-        <v>393158200</v>
+        <v>400767800</v>
       </c>
       <c r="I82" t="n">
         <v>10100</v>
@@ -19616,7 +19616,7 @@
         <v>6.04</v>
       </c>
       <c r="N82" t="n">
-        <v>0.9997498881137539</v>
+        <v>1.01910010578336</v>
       </c>
       <c r="O82" t="n">
         <v>1.01</v>
@@ -19694,7 +19694,7 @@
         <v>65949124.8</v>
       </c>
       <c r="AN82" t="n">
-        <v>69956975.08896796</v>
+        <v>71310996.44128114</v>
       </c>
       <c r="AO82" t="n">
         <v>0</v>
@@ -21243,7 +21243,7 @@
         <v>24.88</v>
       </c>
       <c r="H89" t="n">
-        <v>1914419898</v>
+        <v>1910202000</v>
       </c>
       <c r="I89" t="n">
         <v>10300</v>
@@ -21261,7 +21261,7 @@
         <v>11.38</v>
       </c>
       <c r="N89" t="n">
-        <v>8.014277928463153</v>
+        <v>7.996620670052278</v>
       </c>
       <c r="O89" t="n">
         <v>1.53</v>
@@ -21339,7 +21339,7 @@
         <v>95908776.3</v>
       </c>
       <c r="AN89" t="n">
-        <v>208769890.7306434</v>
+        <v>208309923.6641221</v>
       </c>
       <c r="AO89" t="n">
         <v>0</v>
@@ -21478,7 +21478,7 @@
         <v>25</v>
       </c>
       <c r="H90" t="n">
-        <v>1914419898</v>
+        <v>1910202000</v>
       </c>
       <c r="I90" t="n">
         <v>13800</v>
@@ -21496,7 +21496,7 @@
         <v>10.59</v>
       </c>
       <c r="N90" t="n">
-        <v>43.85065611442371</v>
+        <v>43.75404324756157</v>
       </c>
       <c r="O90" t="n">
         <v>1.42</v>
@@ -21574,7 +21574,7 @@
         <v>17528576.7</v>
       </c>
       <c r="AN90" t="n">
-        <v>224433751.2309496</v>
+        <v>223939273.1535756</v>
       </c>
       <c r="AO90" t="n">
         <v>0</v>
@@ -21713,7 +21713,7 @@
         <v>28.8</v>
       </c>
       <c r="H91" t="n">
-        <v>1914419898</v>
+        <v>1910202000</v>
       </c>
       <c r="I91" t="n">
         <v>2000</v>
@@ -21731,7 +21731,7 @@
         <v>11.3</v>
       </c>
       <c r="N91" t="n">
-        <v>9.726985065312096</v>
+        <v>9.705554327522613</v>
       </c>
       <c r="O91" t="n">
         <v>1.52</v>
@@ -21809,7 +21809,7 @@
         <v>79021360.05</v>
       </c>
       <c r="AN91" t="n">
-        <v>210375812.967033</v>
+        <v>209912307.6923077</v>
       </c>
       <c r="AO91" t="n">
         <v>0</v>
@@ -22418,7 +22418,7 @@
         <v>47.13</v>
       </c>
       <c r="H94" t="n">
-        <v>8326262000</v>
+        <v>8323223000</v>
       </c>
       <c r="I94" t="n">
         <v>200</v>
@@ -22436,7 +22436,7 @@
         <v>5.78</v>
       </c>
       <c r="N94" t="n">
-        <v>0.7817692426884948</v>
+        <v>0.781483904954884</v>
       </c>
       <c r="O94" t="n">
         <v>0.36</v>
@@ -22514,7 +22514,7 @@
         <v>1209900967.64</v>
       </c>
       <c r="AN94" t="n">
-        <v>2995058273.381295</v>
+        <v>2993965107.913669</v>
       </c>
       <c r="AO94" t="n">
         <v>0</v>
@@ -22653,7 +22653,7 @@
         <v>42.6</v>
       </c>
       <c r="H95" t="n">
-        <v>8326262000</v>
+        <v>8323223000</v>
       </c>
       <c r="I95" t="n">
         <v>0</v>
@@ -22671,7 +22671,7 @@
         <v>4.65</v>
       </c>
       <c r="N95" t="n">
-        <v>4.365420810593535</v>
+        <v>4.363827476893083</v>
       </c>
       <c r="O95" t="n">
         <v>0.29</v>
@@ -22749,7 +22749,7 @@
         <v>216671749.24</v>
       </c>
       <c r="AN95" t="n">
-        <v>3717081250</v>
+        <v>3715724553.571428</v>
       </c>
       <c r="AO95" t="n">
         <v>0</v>
@@ -23593,7 +23593,7 @@
         <v>125.1</v>
       </c>
       <c r="H99" t="n">
-        <v>16677569109</v>
+        <v>16574890000</v>
       </c>
       <c r="I99" t="n">
         <v>0</v>
@@ -23611,7 +23611,7 @@
         <v>10.65</v>
       </c>
       <c r="N99" t="n">
-        <v>1.647848779135744</v>
+        <v>1.637703437011688</v>
       </c>
       <c r="O99" t="n">
         <v>1.16</v>
@@ -23689,7 +23689,7 @@
         <v>1267125769.6</v>
       </c>
       <c r="AN99" t="n">
-        <v>2870493822.547332</v>
+        <v>2852820998.27883</v>
       </c>
       <c r="AO99" t="n">
         <v>0</v>
@@ -23828,7 +23828,7 @@
         <v>124.98</v>
       </c>
       <c r="H100" t="n">
-        <v>16677569109</v>
+        <v>16574890000</v>
       </c>
       <c r="I100" t="n">
         <v>1100</v>
@@ -23846,7 +23846,7 @@
         <v>10.81</v>
       </c>
       <c r="N100" t="n">
-        <v>5.972196818133964</v>
+        <v>5.93542767965516</v>
       </c>
       <c r="O100" t="n">
         <v>1.18</v>
@@ -23924,7 +23924,7 @@
         <v>349625391.8</v>
       </c>
       <c r="AN100" t="n">
-        <v>2826706628.644068</v>
+        <v>2809303389.830508</v>
       </c>
       <c r="AO100" t="n">
         <v>0</v>
@@ -24063,7 +24063,7 @@
         <v>25</v>
       </c>
       <c r="H101" t="n">
-        <v>626229171</v>
+        <v>633766700</v>
       </c>
       <c r="I101" t="n">
         <v>300</v>
@@ -24081,7 +24081,7 @@
         <v>6.28</v>
       </c>
       <c r="N101" t="n">
-        <v>2.019673960433849</v>
+        <v>2.043983513153991</v>
       </c>
       <c r="O101" t="n">
         <v>0.49</v>
@@ -24159,7 +24159,7 @@
         <v>42633867</v>
       </c>
       <c r="AN101" t="n">
-        <v>64759997.00103413</v>
+        <v>65539472.59565667</v>
       </c>
       <c r="AO101" t="n">
         <v>0</v>
@@ -24298,7 +24298,7 @@
         <v>24.6</v>
       </c>
       <c r="H102" t="n">
-        <v>626229171</v>
+        <v>633766700</v>
       </c>
       <c r="I102" t="n">
         <v>1500</v>
@@ -24316,7 +24316,7 @@
         <v>6.32</v>
       </c>
       <c r="N102" t="n">
-        <v>1.477623282039919</v>
+        <v>1.495408509645439</v>
       </c>
       <c r="O102" t="n">
         <v>0.49</v>
@@ -24394,7 +24394,7 @@
         <v>58273656.12</v>
       </c>
       <c r="AN102" t="n">
-        <v>64360654.77903391</v>
+        <v>65135323.74100719</v>
       </c>
       <c r="AO102" t="n">
         <v>0</v>
@@ -26883,7 +26883,7 @@
         <v>18</v>
       </c>
       <c r="H113" t="n">
-        <v>422295558</v>
+        <v>426219100</v>
       </c>
       <c r="I113" t="n">
         <v>0</v>
@@ -26901,7 +26901,7 @@
         <v>20.65</v>
       </c>
       <c r="N113" t="n">
-        <v>1.58270611111466</v>
+        <v>1.597411010995741</v>
       </c>
       <c r="O113" t="n">
         <v>0.54</v>
@@ -26979,7 +26979,7 @@
         <v>8431470.34</v>
       </c>
       <c r="AN113" t="n">
-        <v>31304340.84507042</v>
+        <v>31595189.0289103</v>
       </c>
       <c r="AO113" t="n">
         <v>0</v>
@@ -27118,7 +27118,7 @@
         <v>12.8</v>
       </c>
       <c r="H114" t="n">
-        <v>422295558</v>
+        <v>426219100</v>
       </c>
       <c r="I114" t="n">
         <v>7700</v>
@@ -27136,7 +27136,7 @@
         <v>23.27</v>
       </c>
       <c r="N114" t="n">
-        <v>1.302661526518525</v>
+        <v>1.314764536162494</v>
       </c>
       <c r="O114" t="n">
         <v>0.61</v>
@@ -27214,7 +27214,7 @@
         <v>10244057.54</v>
       </c>
       <c r="AN114" t="n">
-        <v>27800892.56089533</v>
+        <v>28059190.25674786</v>
       </c>
       <c r="AO114" t="n">
         <v>0</v>
@@ -27353,7 +27353,7 @@
         <v>13.1</v>
       </c>
       <c r="H115" t="n">
-        <v>422295558</v>
+        <v>426219100</v>
       </c>
       <c r="I115" t="n">
         <v>100</v>
@@ -27371,7 +27371,7 @@
         <v>22.56</v>
       </c>
       <c r="N115" t="n">
-        <v>2.466628536049009</v>
+        <v>2.48954594655984</v>
       </c>
       <c r="O115" t="n">
         <v>0.59</v>
@@ -27449,7 +27449,7 @@
         <v>5410032.13</v>
       </c>
       <c r="AN115" t="n">
-        <v>28669080.65173116</v>
+        <v>28935444.67073999</v>
       </c>
       <c r="AO115" t="n">
         <v>0</v>
@@ -32288,7 +32288,7 @@
         <v>6.51</v>
       </c>
       <c r="H136" t="n">
-        <v>431144700</v>
+        <v>435168500</v>
       </c>
       <c r="I136" t="n">
         <v>0</v>
@@ -32306,7 +32306,7 @@
         <v>89.8</v>
       </c>
       <c r="N136" t="n">
-        <v>1.006410188621465</v>
+        <v>1.015802843377455</v>
       </c>
       <c r="O136" t="n">
         <v>0.49</v>
@@ -32384,7 +32384,7 @@
         <v>3812747.4</v>
       </c>
       <c r="AN136" t="n">
-        <v>7289005.917159763</v>
+        <v>7357032.967032967</v>
       </c>
       <c r="AO136" t="n">
         <v>0</v>
@@ -32523,7 +32523,7 @@
         <v>3.89</v>
       </c>
       <c r="H137" t="n">
-        <v>431144700</v>
+        <v>435168500</v>
       </c>
       <c r="I137" t="n">
         <v>3700</v>
@@ -32541,7 +32541,7 @@
         <v>51.86</v>
       </c>
       <c r="N137" t="n">
-        <v>2.588457542014589</v>
+        <v>2.612615175072721</v>
       </c>
       <c r="O137" t="n">
         <v>0.29</v>
@@ -32619,7 +32619,7 @@
         <v>1482422.55</v>
       </c>
       <c r="AN137" t="n">
-        <v>12617638.27919227</v>
+        <v>12735396.54667837</v>
       </c>
       <c r="AO137" t="n">
         <v>0</v>
@@ -33463,7 +33463,7 @@
         <v>12.74</v>
       </c>
       <c r="H141" t="n">
-        <v>283363938</v>
+        <v>283059300</v>
       </c>
       <c r="I141" t="n">
         <v>100</v>
@@ -33481,7 +33481,7 @@
         <v>2.98</v>
       </c>
       <c r="N141" t="n">
-        <v>1.127964023439491</v>
+        <v>1.126751375469541</v>
       </c>
       <c r="O141" t="n">
         <v>0.5</v>
@@ -33559,7 +33559,7 @@
         <v>45922500</v>
       </c>
       <c r="AN141" t="n">
-        <v>73601022.85714285</v>
+        <v>73521896.1038961</v>
       </c>
       <c r="AO141" t="n">
         <v>0</v>
@@ -33698,7 +33698,7 @@
         <v>12.02</v>
       </c>
       <c r="H142" t="n">
-        <v>283363938</v>
+        <v>283059300</v>
       </c>
       <c r="I142" t="n">
         <v>2500</v>
@@ -33716,7 +33716,7 @@
         <v>3.05</v>
       </c>
       <c r="N142" t="n">
-        <v>0.8625607238066693</v>
+        <v>0.8616334047708256</v>
       </c>
       <c r="O142" t="n">
         <v>0.51</v>
@@ -33794,7 +33794,7 @@
         <v>60052500</v>
       </c>
       <c r="AN142" t="n">
-        <v>71737705.82278481</v>
+        <v>71660582.27848101</v>
       </c>
       <c r="AO142" t="n">
         <v>0</v>
@@ -34403,7 +34403,7 @@
         <v>51.52</v>
       </c>
       <c r="H145" t="n">
-        <v>8792190000</v>
+        <v>8715782000</v>
       </c>
       <c r="I145" t="n">
         <v>0</v>
@@ -34421,7 +34421,7 @@
         <v>10.18</v>
       </c>
       <c r="N145" t="n">
-        <v>1.89986677138113</v>
+        <v>1.883356093123757</v>
       </c>
       <c r="O145" t="n">
         <v>0.73</v>
@@ -34499,7 +34499,7 @@
         <v>441028665.6</v>
       </c>
       <c r="AN145" t="n">
-        <v>2021193103.448276</v>
+        <v>2003628045.977012</v>
       </c>
       <c r="AO145" t="n">
         <v>0</v>
@@ -34638,7 +34638,7 @@
         <v>39.2</v>
       </c>
       <c r="H146" t="n">
-        <v>8792190000</v>
+        <v>8715782000</v>
       </c>
       <c r="I146" t="n">
         <v>1200</v>
@@ -34656,7 +34656,7 @@
         <v>8.16</v>
       </c>
       <c r="N146" t="n">
-        <v>1.713432768499566</v>
+        <v>1.698542283765329</v>
       </c>
       <c r="O146" t="n">
         <v>0.58</v>
@@ -34734,7 +34734,7 @@
         <v>489015806.4</v>
       </c>
       <c r="AN146" t="n">
-        <v>2519252148.997135</v>
+        <v>2497358739.255014</v>
       </c>
       <c r="AO146" t="n">
         <v>0</v>
@@ -36518,7 +36518,7 @@
         <v>36.02</v>
       </c>
       <c r="H154" t="n">
-        <v>8300838947</v>
+        <v>8127221000</v>
       </c>
       <c r="I154" t="n">
         <v>1500</v>
@@ -36536,7 +36536,7 @@
         <v>10.95</v>
       </c>
       <c r="N154" t="n">
-        <v>2.652547165480244</v>
+        <v>2.597067256023889</v>
       </c>
       <c r="O154" t="n">
         <v>0.71</v>
@@ -36614,7 +36614,7 @@
         <v>345171067.18</v>
       </c>
       <c r="AN154" t="n">
-        <v>1309280591.009464</v>
+        <v>1281896056.782334</v>
       </c>
       <c r="AO154" t="n">
         <v>0</v>
@@ -36753,7 +36753,7 @@
         <v>37.7</v>
       </c>
       <c r="H155" t="n">
-        <v>8300838947</v>
+        <v>8127221000</v>
       </c>
       <c r="I155" t="n">
         <v>300</v>
@@ -36771,7 +36771,7 @@
         <v>11.38</v>
       </c>
       <c r="N155" t="n">
-        <v>1.3969964677199</v>
+        <v>1.367777293580949</v>
       </c>
       <c r="O155" t="n">
         <v>0.73</v>
@@ -36849,7 +36849,7 @@
         <v>655393594.0500001</v>
       </c>
       <c r="AN155" t="n">
-        <v>1259611372.837633</v>
+        <v>1233265705.614568</v>
       </c>
       <c r="AO155" t="n">
         <v>0</v>
@@ -38633,7 +38633,7 @@
         <v>3.01</v>
       </c>
       <c r="H163" t="n">
-        <v>18212519</v>
+        <v>19804570</v>
       </c>
       <c r="I163" t="n">
         <v>0</v>
@@ -38651,7 +38651,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="N163" t="n">
-        <v>0.3394312589912878</v>
+        <v>0.3691027105520707</v>
       </c>
       <c r="O163" t="n">
         <v>0.07000000000000001</v>
@@ -38729,7 +38729,7 @@
         <v>8649345</v>
       </c>
       <c r="AN163" t="n">
-        <v>4553129.75</v>
+        <v>4951142.5</v>
       </c>
       <c r="AO163" t="n">
         <v>0</v>
@@ -38868,7 +38868,7 @@
         <v>2.17</v>
       </c>
       <c r="H164" t="n">
-        <v>18212519</v>
+        <v>19804570</v>
       </c>
       <c r="I164" t="n">
         <v>1700</v>
@@ -38886,7 +38886,7 @@
         <v>1.51</v>
       </c>
       <c r="N164" t="n">
-        <v>0.01697156294956439</v>
+        <v>0.01845513552760354</v>
       </c>
       <c r="O164" t="n">
         <v>0.11</v>
@@ -38964,7 +38964,7 @@
         <v>172986900</v>
       </c>
       <c r="AN164" t="n">
-        <v>2836840.965732087</v>
+        <v>3084823.987538941</v>
       </c>
       <c r="AO164" t="n">
         <v>0</v>
@@ -40748,7 +40748,7 @@
         <v>3.87</v>
       </c>
       <c r="H172" t="n">
-        <v>208427628</v>
+        <v>208427700</v>
       </c>
       <c r="I172" t="n">
         <v>400</v>
@@ -40766,7 +40766,7 @@
         <v>0.38</v>
       </c>
       <c r="N172" t="n">
-        <v>0.04614729740084145</v>
+        <v>0.04614731334213217</v>
       </c>
       <c r="O172" t="n">
         <v>0.08</v>
@@ -40844,7 +40844,7 @@
         <v>640901679.6</v>
       </c>
       <c r="AN172" t="n">
-        <v>208427628</v>
+        <v>208427700</v>
       </c>
       <c r="AO172" t="n">
         <v>0</v>
@@ -42628,7 +42628,7 @@
         <v>32.9</v>
       </c>
       <c r="H180" t="n">
-        <v>3564603305</v>
+        <v>3487736000</v>
       </c>
       <c r="I180" t="n">
         <v>500</v>
@@ -42646,7 +42646,7 @@
         <v>12.71</v>
       </c>
       <c r="N180" t="n">
-        <v>8.708644644750324</v>
+        <v>8.520850944647519</v>
       </c>
       <c r="O180" t="n">
         <v>0.8</v>
@@ -42724,7 +42724,7 @@
         <v>84360399.48</v>
       </c>
       <c r="AN180" t="n">
-        <v>462335059.0142672</v>
+        <v>452365239.9481193</v>
       </c>
       <c r="AO180" t="n">
         <v>4.0605</v>
@@ -42863,7 +42863,7 @@
         <v>38.95</v>
       </c>
       <c r="H181" t="n">
-        <v>3564603305</v>
+        <v>3487736000</v>
       </c>
       <c r="I181" t="n">
         <v>0</v>
@@ -42881,7 +42881,7 @@
         <v>13.08</v>
       </c>
       <c r="N181" t="n">
-        <v>4.354322322375162</v>
+        <v>4.260425472323759</v>
       </c>
       <c r="O181" t="n">
         <v>0.83</v>
@@ -42959,7 +42959,7 @@
         <v>168720798.96</v>
       </c>
       <c r="AN181" t="n">
-        <v>448942481.7380353</v>
+        <v>439261460.9571788</v>
       </c>
       <c r="AO181" t="n">
         <v>4.0605</v>
@@ -43104,7 +43104,7 @@
         <v>2475700</v>
       </c>
       <c r="J182" t="n">
-        <v>160239730</v>
+        <v>157368947</v>
       </c>
       <c r="K182" t="n">
         <v>0</v>
@@ -43116,7 +43116,7 @@
         <v>0.46</v>
       </c>
       <c r="N182" t="n">
-        <v>0.01775953597782825</v>
+        <v>0.01808351205408068</v>
       </c>
       <c r="O182" t="n">
         <v>0.02</v>
@@ -43188,10 +43188,10 @@
         <v>0</v>
       </c>
       <c r="AL182" t="n">
-        <v>5684323460.141719</v>
+        <v>5582485675.243579</v>
       </c>
       <c r="AM182" t="n">
-        <v>1283520237.3</v>
+        <v>1260525265.47</v>
       </c>
       <c r="AN182" t="n">
         <v>61182392.12121212</v>
@@ -45448,7 +45448,7 @@
         <v>2.52</v>
       </c>
       <c r="H192" t="n">
-        <v>23318111</v>
+        <v>22927330</v>
       </c>
       <c r="I192" t="n">
         <v>1800</v>
@@ -45466,7 +45466,7 @@
         <v>21.95</v>
       </c>
       <c r="N192" t="n">
-        <v>2.384064369686468</v>
+        <v>2.344110573324041</v>
       </c>
       <c r="O192" t="n">
         <v>0.32</v>
@@ -45544,7 +45544,7 @@
         <v>357000.03</v>
       </c>
       <c r="AN192" t="n">
-        <v>1961153.153910849</v>
+        <v>1928286.795626577</v>
       </c>
       <c r="AO192" t="n">
         <v>0</v>
@@ -45683,7 +45683,7 @@
         <v>1.63</v>
       </c>
       <c r="H193" t="n">
-        <v>23318111</v>
+        <v>22927330</v>
       </c>
       <c r="I193" t="n">
         <v>15600</v>
@@ -45701,7 +45701,7 @@
         <v>14.71</v>
       </c>
       <c r="N193" t="n">
-        <v>1.192032335099398</v>
+        <v>1.172055434400088</v>
       </c>
       <c r="O193" t="n">
         <v>0.22</v>
@@ -45779,7 +45779,7 @@
         <v>713999.97</v>
       </c>
       <c r="AN193" t="n">
-        <v>2925735.382685069</v>
+        <v>2876703.889585948</v>
       </c>
       <c r="AO193" t="n">
         <v>0</v>
@@ -47563,7 +47563,7 @@
         <v>6.98</v>
       </c>
       <c r="H201" t="n">
-        <v>128239422</v>
+        <v>128239400</v>
       </c>
       <c r="I201" t="n">
         <v>1000</v>
@@ -47581,7 +47581,7 @@
         <v>1.99</v>
       </c>
       <c r="N201" t="n">
-        <v>1.513458603418335</v>
+        <v>1.51345834377829</v>
       </c>
       <c r="O201" t="n">
         <v>0.25</v>
@@ -47659,7 +47659,7 @@
         <v>28893848.04</v>
       </c>
       <c r="AN201" t="n">
-        <v>101777319.047619</v>
+        <v>101777301.5873016</v>
       </c>
       <c r="AO201" t="n">
         <v>0</v>
@@ -48006,7 +48006,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>IBOVESPA</t>
+          <t>Brazil Stock Exchange Index</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
@@ -56007,7 +56007,7 @@
         <v>0.7</v>
       </c>
       <c r="H237" t="n">
-        <v>29497796</v>
+        <v>29497800</v>
       </c>
       <c r="I237" t="n">
         <v>34400</v>
@@ -56025,7 +56025,7 @@
         <v>5.38</v>
       </c>
       <c r="N237" t="n">
-        <v>0.4250364529579349</v>
+        <v>0.4250365105943024</v>
       </c>
       <c r="O237" t="n">
         <v>0.11</v>
@@ -56103,7 +56103,7 @@
         <v>10271292.68</v>
       </c>
       <c r="AN237" t="n">
-        <v>2929274.677259186</v>
+        <v>2929275.07447865</v>
       </c>
       <c r="AO237" t="n">
         <v>0</v>
@@ -56180,7 +56180,7 @@
         <v>0.22</v>
       </c>
       <c r="BM237" t="n">
-        <v>-2.29</v>
+        <v>-22.92</v>
       </c>
       <c r="BN237" t="n">
         <v>0.71</v>
@@ -58357,7 +58357,7 @@
         <v>5.15</v>
       </c>
       <c r="H247" t="n">
-        <v>19137235</v>
+        <v>19137240</v>
       </c>
       <c r="I247" t="n">
         <v>7000</v>
@@ -58375,7 +58375,7 @@
         <v>4.4</v>
       </c>
       <c r="N247" t="n">
-        <v>0.02879933405412948</v>
+        <v>0.02879934157855348</v>
       </c>
       <c r="O247" t="n">
         <v>0.05</v>
@@ -58453,7 +58453,7 @@
         <v>5648272.88</v>
       </c>
       <c r="AN247" t="n">
-        <v>32435991.52542373</v>
+        <v>32436000</v>
       </c>
       <c r="AO247" t="n">
         <v>0</v>
@@ -59767,7 +59767,7 @@
         <v>18.5</v>
       </c>
       <c r="H253" t="n">
-        <v>183539203</v>
+        <v>183539200</v>
       </c>
       <c r="I253" t="n">
         <v>200</v>
@@ -59785,7 +59785,7 @@
         <v>7.29</v>
       </c>
       <c r="N253" t="n">
-        <v>0.1834958979680795</v>
+        <v>0.1834958949687874</v>
       </c>
       <c r="O253" t="n">
         <v>0.12</v>
@@ -59863,7 +59863,7 @@
         <v>24405758.4</v>
       </c>
       <c r="AN253" t="n">
-        <v>126578760.6896552</v>
+        <v>126578758.6206897</v>
       </c>
       <c r="AO253" t="n">
         <v>0</v>
@@ -60002,7 +60002,7 @@
         <v>3.99</v>
       </c>
       <c r="H254" t="n">
-        <v>283293910</v>
+        <v>283294000</v>
       </c>
       <c r="I254" t="n">
         <v>16800</v>
@@ -60020,7 +60020,7 @@
         <v>0.59</v>
       </c>
       <c r="N254" t="n">
-        <v>0.6624595673603967</v>
+        <v>0.6624597778180131</v>
       </c>
       <c r="O254" t="n">
         <v>0.6899999999999999</v>
@@ -60098,7 +60098,7 @@
         <v>520437330</v>
       </c>
       <c r="AN254" t="n">
-        <v>180441980.8917197</v>
+        <v>180442038.2165605</v>
       </c>
       <c r="AO254" t="n">
         <v>0</v>
@@ -60707,7 +60707,7 @@
         <v>39.8</v>
       </c>
       <c r="H257" t="n">
-        <v>12644180000</v>
+        <v>12761780000</v>
       </c>
       <c r="I257" t="n">
         <v>0</v>
@@ -60725,7 +60725,7 @@
         <v>9.57</v>
       </c>
       <c r="N257" t="n">
-        <v>3.150356458256311</v>
+        <v>3.179657047103587</v>
       </c>
       <c r="O257" t="n">
         <v>0.64</v>
@@ -60803,7 +60803,7 @@
         <v>836829598.4699999</v>
       </c>
       <c r="AN257" t="n">
-        <v>2298941818.181818</v>
+        <v>2320323636.363636</v>
       </c>
       <c r="AO257" t="n">
         <v>0</v>
@@ -60942,7 +60942,7 @@
         <v>36.01</v>
       </c>
       <c r="H258" t="n">
-        <v>12644180000</v>
+        <v>12761780000</v>
       </c>
       <c r="I258" t="n">
         <v>0</v>
@@ -60960,7 +60960,7 @@
         <v>8.94</v>
       </c>
       <c r="N258" t="n">
-        <v>7.228739381710705</v>
+        <v>7.295971875339329</v>
       </c>
       <c r="O258" t="n">
         <v>0.59</v>
@@ -61038,7 +61038,7 @@
         <v>364698655.02</v>
       </c>
       <c r="AN258" t="n">
-        <v>2459957198.44358</v>
+        <v>2482836575.875486</v>
       </c>
       <c r="AO258" t="n">
         <v>0</v>
@@ -61177,7 +61177,7 @@
         <v>34.3</v>
       </c>
       <c r="H259" t="n">
-        <v>12644180000</v>
+        <v>12761780000</v>
       </c>
       <c r="I259" t="n">
         <v>200</v>
@@ -61195,7 +61195,7 @@
         <v>9.949999999999999</v>
       </c>
       <c r="N259" t="n">
-        <v>8.52543373103655</v>
+        <v>8.604726418009522</v>
       </c>
       <c r="O259" t="n">
         <v>0.66</v>
@@ -61273,7 +61273,7 @@
         <v>309229021.44</v>
       </c>
       <c r="AN259" t="n">
-        <v>2210520979.020979</v>
+        <v>2231080419.58042</v>
       </c>
       <c r="AO259" t="n">
         <v>0</v>
@@ -64232,7 +64232,7 @@
         <v>1.93</v>
       </c>
       <c r="H272" t="n">
-        <v>12779461</v>
+        <v>12779470</v>
       </c>
       <c r="I272" t="n">
         <v>1900</v>
@@ -64250,7 +64250,7 @@
         <v>0.96</v>
       </c>
       <c r="N272" t="n">
-        <v>4.901456310662467</v>
+        <v>4.901459762537847</v>
       </c>
       <c r="O272" t="n">
         <v>1.87</v>
@@ -64328,7 +64328,7 @@
         <v>37941114.78</v>
       </c>
       <c r="AN272" t="n">
-        <v>11309257.5221239</v>
+        <v>11309265.48672567</v>
       </c>
       <c r="AO272" t="n">
         <v>0</v>
@@ -67757,7 +67757,7 @@
         <v>38.7</v>
       </c>
       <c r="H287" t="n">
-        <v>707325840</v>
+        <v>704624800</v>
       </c>
       <c r="I287" t="n">
         <v>0</v>
@@ -67775,7 +67775,7 @@
         <v>21.05</v>
       </c>
       <c r="N287" t="n">
-        <v>11.93259530962841</v>
+        <v>11.88702873279429</v>
       </c>
       <c r="O287" t="n">
         <v>0.54</v>
@@ -67853,7 +67853,7 @@
         <v>16864244.22</v>
       </c>
       <c r="AN287" t="n">
-        <v>29744568.54499579</v>
+        <v>29630984.02018503</v>
       </c>
       <c r="AO287" t="n">
         <v>0.3943</v>
@@ -67992,7 +67992,7 @@
         <v>39</v>
       </c>
       <c r="H288" t="n">
-        <v>707325840</v>
+        <v>704624800</v>
       </c>
       <c r="I288" t="n">
         <v>600</v>
@@ -68010,7 +68010,7 @@
         <v>21.15</v>
       </c>
       <c r="N288" t="n">
-        <v>12.60289576895947</v>
+        <v>12.55476953962818</v>
       </c>
       <c r="O288" t="n">
         <v>0.54</v>
@@ -68088,7 +68088,7 @@
         <v>15967298.72</v>
       </c>
       <c r="AN288" t="n">
-        <v>29595223.43096235</v>
+        <v>29482209.20502092</v>
       </c>
       <c r="AO288" t="n">
         <v>0.4337</v>
@@ -76922,7 +76922,7 @@
         <v>1.15</v>
       </c>
       <c r="H326" t="n">
-        <v>77845372</v>
+        <v>77845370</v>
       </c>
       <c r="I326" t="n">
         <v>8800</v>
@@ -76940,7 +76940,7 @@
         <v>0.11</v>
       </c>
       <c r="N326" t="n">
-        <v>0.009003875812846389</v>
+        <v>0.009003875581519194</v>
       </c>
       <c r="O326" t="n">
         <v>0.02</v>
@@ -77018,7 +77018,7 @@
         <v>1659121826.79</v>
       </c>
       <c r="AN326" t="n">
-        <v>778453720</v>
+        <v>778453700</v>
       </c>
       <c r="AO326" t="n">
         <v>0</v>
@@ -85617,7 +85617,7 @@
         <v>10.1</v>
       </c>
       <c r="H363" t="n">
-        <v>973263750</v>
+        <v>982172900</v>
       </c>
       <c r="I363" t="n">
         <v>100</v>
@@ -85635,7 +85635,7 @@
         <v>20.34</v>
       </c>
       <c r="N363" t="n">
-        <v>2.574662508890448</v>
+        <v>2.598230688113275</v>
       </c>
       <c r="O363" t="n">
         <v>0.27</v>
@@ -85713,7 +85713,7 @@
         <v>45966751.6</v>
       </c>
       <c r="AN363" t="n">
-        <v>103538696.8085106</v>
+        <v>104486478.7234043</v>
       </c>
       <c r="AO363" t="n">
         <v>0</v>
@@ -85852,7 +85852,7 @@
         <v>7.5</v>
       </c>
       <c r="H364" t="n">
-        <v>973263750</v>
+        <v>982172900</v>
       </c>
       <c r="I364" t="n">
         <v>300</v>
@@ -85870,7 +85870,7 @@
         <v>14.31</v>
       </c>
       <c r="N364" t="n">
-        <v>11.68979342555307</v>
+        <v>11.796800516999</v>
       </c>
       <c r="O364" t="n">
         <v>0.19</v>
@@ -85948,7 +85948,7 @@
         <v>10124120.05</v>
       </c>
       <c r="AN364" t="n">
-        <v>147241111.9515885</v>
+        <v>148588940.9984871</v>
       </c>
       <c r="AO364" t="n">
         <v>0</v>
@@ -94077,7 +94077,7 @@
         <v>3.88</v>
       </c>
       <c r="H399" t="n">
-        <v>5950539730</v>
+        <v>5911404000</v>
       </c>
       <c r="I399" t="n">
         <v>1700</v>
@@ -94095,7 +94095,7 @@
         <v>9.42</v>
       </c>
       <c r="N399" t="n">
-        <v>0.67075804015479</v>
+        <v>0.6663465738431742</v>
       </c>
       <c r="O399" t="n">
         <v>0.66</v>
@@ -94173,7 +94173,7 @@
         <v>483489419.2399999</v>
       </c>
       <c r="AN399" t="n">
-        <v>1142138143.953935</v>
+        <v>1134626487.523992</v>
       </c>
       <c r="AO399" t="n">
         <v>0</v>
@@ -94312,7 +94312,7 @@
         <v>4.05</v>
       </c>
       <c r="H400" t="n">
-        <v>5950539730</v>
+        <v>5911404000</v>
       </c>
       <c r="I400" t="n">
         <v>6400</v>
@@ -94330,7 +94330,7 @@
         <v>9.92</v>
       </c>
       <c r="N400" t="n">
-        <v>1.455454672266728</v>
+        <v>1.445882384093623</v>
       </c>
       <c r="O400" t="n">
         <v>0.6899999999999999</v>
@@ -94408,7 +94408,7 @@
         <v>222820003.58</v>
       </c>
       <c r="AN400" t="n">
-        <v>1085864914.233577</v>
+        <v>1078723357.664233</v>
       </c>
       <c r="AO400" t="n">
         <v>0</v>
@@ -94782,7 +94782,7 @@
         <v>20.69</v>
       </c>
       <c r="H402" t="n">
-        <v>737733530</v>
+        <v>737396300</v>
       </c>
       <c r="I402" t="n">
         <v>0</v>
@@ -94800,7 +94800,7 @@
         <v>6.94</v>
       </c>
       <c r="N402" t="n">
-        <v>0.5306439861906429</v>
+        <v>0.5304014201906089</v>
       </c>
       <c r="O402" t="n">
         <v>0.53</v>
@@ -94878,7 +94878,7 @@
         <v>53525040.6</v>
       </c>
       <c r="AN402" t="n">
-        <v>181707766.0098522</v>
+        <v>181624704.4334975</v>
       </c>
       <c r="AO402" t="n">
         <v>0.9505</v>
@@ -95017,7 +95017,7 @@
         <v>20.1</v>
       </c>
       <c r="H403" t="n">
-        <v>737733530</v>
+        <v>737396300</v>
       </c>
       <c r="I403" t="n">
         <v>2000</v>
@@ -95035,7 +95035,7 @@
         <v>7.58</v>
       </c>
       <c r="N403" t="n">
-        <v>0.4431395869590271</v>
+        <v>0.4429370206436392</v>
       </c>
       <c r="O403" t="n">
         <v>0.58</v>
@@ -95113,7 +95113,7 @@
         <v>64094343.5</v>
       </c>
       <c r="AN403" t="n">
-        <v>166531270.8803612</v>
+        <v>166455146.7268623</v>
       </c>
       <c r="AO403" t="n">
         <v>0.7018</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-07-20 04:41
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1770,7 +1770,7 @@
         <v>7.32</v>
       </c>
       <c r="H6" t="n">
-        <v>461780014</v>
+        <v>461780000</v>
       </c>
       <c r="I6" t="n">
         <v>300</v>
@@ -1788,7 +1788,7 @@
         <v>13.39</v>
       </c>
       <c r="N6" t="n">
-        <v>5.696291032445988</v>
+        <v>5.696290859748877</v>
       </c>
       <c r="O6" t="n">
         <v>1.24</v>
@@ -1866,7 +1866,7 @@
         <v>34696585</v>
       </c>
       <c r="AN6" t="n">
-        <v>49547211.8025751</v>
+        <v>49547210.30042918</v>
       </c>
       <c r="AO6" t="n">
         <v>0</v>
@@ -10684,7 +10684,7 @@
         <v>5.5</v>
       </c>
       <c r="H44" t="n">
-        <v>6513569</v>
+        <v>6913660</v>
       </c>
       <c r="I44" t="n">
         <v>0</v>
@@ -10702,7 +10702,7 @@
         <v>0.75</v>
       </c>
       <c r="N44" t="n">
-        <v>0.2910736714472124</v>
+        <v>0.3089526493597803</v>
       </c>
       <c r="O44" t="n">
         <v>0.03</v>
@@ -10780,7 +10780,7 @@
         <v>5719748.64</v>
       </c>
       <c r="AN44" t="n">
-        <v>6513569</v>
+        <v>6913660</v>
       </c>
       <c r="AO44" t="n">
         <v>0</v>
@@ -10919,7 +10919,7 @@
         <v>3.6</v>
       </c>
       <c r="H45" t="n">
-        <v>6513569</v>
+        <v>6913660</v>
       </c>
       <c r="I45" t="n">
         <v>100</v>
@@ -10937,7 +10937,7 @@
         <v>0.63</v>
       </c>
       <c r="N45" t="n">
-        <v>0.1780179095186338</v>
+        <v>0.1889525236199383</v>
       </c>
       <c r="O45" t="n">
         <v>0.02</v>
@@ -11015,7 +11015,7 @@
         <v>9352251.359999999</v>
       </c>
       <c r="AN45" t="n">
-        <v>7754248.80952381</v>
+        <v>8230547.619047619</v>
       </c>
       <c r="AO45" t="n">
         <v>0</v>
@@ -11859,7 +11859,7 @@
         <v>47.47</v>
       </c>
       <c r="H49" t="n">
-        <v>927813041</v>
+        <v>928693800</v>
       </c>
       <c r="I49" t="n">
         <v>1100</v>
@@ -11877,7 +11877,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="N49" t="n">
-        <v>1.013091123606024</v>
+        <v>1.01405283581043</v>
       </c>
       <c r="O49" t="n">
         <v>0.08</v>
@@ -11955,7 +11955,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN49" t="n">
-        <v>169618471.8464351</v>
+        <v>169779488.1170018</v>
       </c>
       <c r="AO49" t="n">
         <v>2.4346</v>
@@ -12094,7 +12094,7 @@
         <v>33</v>
       </c>
       <c r="H50" t="n">
-        <v>927813041</v>
+        <v>928693800</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>
@@ -12112,7 +12112,7 @@
         <v>5.78</v>
       </c>
       <c r="N50" t="n">
-        <v>1.013091123606024</v>
+        <v>1.01405283581043</v>
       </c>
       <c r="O50" t="n">
         <v>0.06</v>
@@ -12190,7 +12190,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN50" t="n">
-        <v>243520483.2020997</v>
+        <v>243751653.5433071</v>
       </c>
       <c r="AO50" t="n">
         <v>3.526</v>
@@ -14428,7 +14428,7 @@
         <v>380.52</v>
       </c>
       <c r="H60" t="n">
-        <v>173041465</v>
+        <v>173041500</v>
       </c>
       <c r="I60" t="n">
         <v>29</v>
@@ -14446,7 +14446,7 @@
         <v>2.87</v>
       </c>
       <c r="N60" t="n">
-        <v>12.22820611792832</v>
+        <v>12.22820859125004</v>
       </c>
       <c r="O60" t="n">
         <v>0.64</v>
@@ -14524,7 +14524,7 @@
         <v>59731412.5</v>
       </c>
       <c r="AN60" t="n">
-        <v>21793635.39042821</v>
+        <v>21793639.79848867</v>
       </c>
       <c r="AO60" t="n">
         <v>0</v>
@@ -18893,7 +18893,7 @@
         <v>2.95</v>
       </c>
       <c r="H79" t="n">
-        <v>6308527901</v>
+        <v>6323380000</v>
       </c>
       <c r="I79" t="n">
         <v>28700</v>
@@ -18911,7 +18911,7 @@
         <v>2.47</v>
       </c>
       <c r="N79" t="n">
-        <v>0.8820524265905705</v>
+        <v>0.8841290330776143</v>
       </c>
       <c r="O79" t="n">
         <v>0.03</v>
@@ -18989,7 +18989,7 @@
         <v>531401092.4</v>
       </c>
       <c r="AN79" t="n">
-        <v>3823350243.030303</v>
+        <v>3832351515.151515</v>
       </c>
       <c r="AO79" t="n">
         <v>0</v>
@@ -19128,7 +19128,7 @@
         <v>3</v>
       </c>
       <c r="H80" t="n">
-        <v>6308527901</v>
+        <v>6323380000</v>
       </c>
       <c r="I80" t="n">
         <v>5600</v>
@@ -19146,7 +19146,7 @@
         <v>3.36</v>
       </c>
       <c r="N80" t="n">
-        <v>1.70037166361338</v>
+        <v>1.70437483022865</v>
       </c>
       <c r="O80" t="n">
         <v>0.04</v>
@@ -19224,7 +19224,7 @@
         <v>275659512.02</v>
       </c>
       <c r="AN80" t="n">
-        <v>2803790178.222222</v>
+        <v>2810391111.111111</v>
       </c>
       <c r="AO80" t="n">
         <v>0</v>
@@ -19598,7 +19598,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="H82" t="n">
-        <v>381744000</v>
+        <v>382589500</v>
       </c>
       <c r="I82" t="n">
         <v>11200</v>
@@ -19616,7 +19616,7 @@
         <v>6.04</v>
       </c>
       <c r="N82" t="n">
-        <v>0.9707250701831905</v>
+        <v>0.9728750661145997</v>
       </c>
       <c r="O82" t="n">
         <v>1.01</v>
@@ -19694,7 +19694,7 @@
         <v>65949124.8</v>
       </c>
       <c r="AN82" t="n">
-        <v>67925978.64768682</v>
+        <v>68076423.48754448</v>
       </c>
       <c r="AO82" t="n">
         <v>0</v>
@@ -20491,7 +20491,7 @@
         <v>0</v>
       </c>
       <c r="BR85" t="n">
-        <v>26.5</v>
+        <v>29</v>
       </c>
       <c r="BS85" t="n">
         <v>0</v>
@@ -21243,7 +21243,7 @@
         <v>24.36</v>
       </c>
       <c r="H89" t="n">
-        <v>1878904873</v>
+        <v>1922574000</v>
       </c>
       <c r="I89" t="n">
         <v>11000</v>
@@ -21261,7 +21261,7 @@
         <v>11.38</v>
       </c>
       <c r="N89" t="n">
-        <v>7.865602456962012</v>
+        <v>8.048413198240336</v>
       </c>
       <c r="O89" t="n">
         <v>1.53</v>
@@ -21339,7 +21339,7 @@
         <v>95908776.3</v>
       </c>
       <c r="AN89" t="n">
-        <v>204896932.7153762</v>
+        <v>209659105.7797165</v>
       </c>
       <c r="AO89" t="n">
         <v>0</v>
@@ -21478,7 +21478,7 @@
         <v>24.32</v>
       </c>
       <c r="H90" t="n">
-        <v>1878904873</v>
+        <v>1922574000</v>
       </c>
       <c r="I90" t="n">
         <v>13900</v>
@@ -21496,7 +21496,7 @@
         <v>10.59</v>
       </c>
       <c r="N90" t="n">
-        <v>43.03716835774236</v>
+        <v>44.03742951930604</v>
       </c>
       <c r="O90" t="n">
         <v>1.42</v>
@@ -21574,7 +21574,7 @@
         <v>17528576.7</v>
       </c>
       <c r="AN90" t="n">
-        <v>220270207.8546307</v>
+        <v>225389683.4701055</v>
       </c>
       <c r="AO90" t="n">
         <v>0</v>
@@ -21713,7 +21713,7 @@
         <v>30</v>
       </c>
       <c r="H91" t="n">
-        <v>1878904873</v>
+        <v>1922574000</v>
       </c>
       <c r="I91" t="n">
         <v>6100</v>
@@ -21731,7 +21731,7 @@
         <v>11.3</v>
       </c>
       <c r="N91" t="n">
-        <v>9.546536607724457</v>
+        <v>9.768415280521358</v>
       </c>
       <c r="O91" t="n">
         <v>1.52</v>
@@ -21809,7 +21809,7 @@
         <v>79021360.05</v>
       </c>
       <c r="AN91" t="n">
-        <v>206473062.967033</v>
+        <v>211271868.1318682</v>
       </c>
       <c r="AO91" t="n">
         <v>0</v>
@@ -22418,7 +22418,7 @@
         <v>46.5</v>
       </c>
       <c r="H94" t="n">
-        <v>8318662000</v>
+        <v>8227464000</v>
       </c>
       <c r="I94" t="n">
         <v>400</v>
@@ -22436,7 +22436,7 @@
         <v>5.78</v>
       </c>
       <c r="N94" t="n">
-        <v>0.7810556636245124</v>
+        <v>0.7724929026406873</v>
       </c>
       <c r="O94" t="n">
         <v>0.36</v>
@@ -22514,7 +22514,7 @@
         <v>1209900967.64</v>
       </c>
       <c r="AN94" t="n">
-        <v>2992324460.431655</v>
+        <v>2959519424.460432</v>
       </c>
       <c r="AO94" t="n">
         <v>0</v>
@@ -22653,7 +22653,7 @@
         <v>42.6</v>
       </c>
       <c r="H95" t="n">
-        <v>8318662000</v>
+        <v>8227464000</v>
       </c>
       <c r="I95" t="n">
         <v>0</v>
@@ -22671,7 +22671,7 @@
         <v>4.65</v>
       </c>
       <c r="N95" t="n">
-        <v>4.361436165603921</v>
+        <v>4.313621474319343</v>
       </c>
       <c r="O95" t="n">
         <v>0.29</v>
@@ -22749,7 +22749,7 @@
         <v>216671749.24</v>
       </c>
       <c r="AN95" t="n">
-        <v>3713688392.857142</v>
+        <v>3672975000</v>
       </c>
       <c r="AO95" t="n">
         <v>0</v>
@@ -23593,7 +23593,7 @@
         <v>125.1</v>
       </c>
       <c r="H99" t="n">
-        <v>16547088620</v>
+        <v>16547090000</v>
       </c>
       <c r="I99" t="n">
         <v>0</v>
@@ -23611,7 +23611,7 @@
         <v>10.65</v>
       </c>
       <c r="N99" t="n">
-        <v>1.634956485714897</v>
+        <v>1.634956622067581</v>
       </c>
       <c r="O99" t="n">
         <v>1.16</v>
@@ -23689,7 +23689,7 @@
         <v>1267125769.6</v>
       </c>
       <c r="AN99" t="n">
-        <v>2848035907.056799</v>
+        <v>2848036144.578313</v>
       </c>
       <c r="AO99" t="n">
         <v>0</v>
@@ -23828,7 +23828,7 @@
         <v>124.01</v>
       </c>
       <c r="H100" t="n">
-        <v>16547088620</v>
+        <v>16547090000</v>
       </c>
       <c r="I100" t="n">
         <v>100</v>
@@ -23846,7 +23846,7 @@
         <v>10.81</v>
       </c>
       <c r="N100" t="n">
-        <v>5.925472073290074</v>
+        <v>5.925472567464708</v>
       </c>
       <c r="O100" t="n">
         <v>1.18</v>
@@ -23924,7 +23924,7 @@
         <v>349625391.8</v>
       </c>
       <c r="AN100" t="n">
-        <v>2804591291.525424</v>
+        <v>2804591525.423728</v>
       </c>
       <c r="AO100" t="n">
         <v>0</v>
@@ -24063,7 +24063,7 @@
         <v>24.65</v>
       </c>
       <c r="H101" t="n">
-        <v>624557030</v>
+        <v>627033800</v>
       </c>
       <c r="I101" t="n">
         <v>300</v>
@@ -24081,7 +24081,7 @@
         <v>6.28</v>
       </c>
       <c r="N101" t="n">
-        <v>2.014281079053889</v>
+        <v>2.022268998024505</v>
       </c>
       <c r="O101" t="n">
         <v>0.49</v>
@@ -24159,7 +24159,7 @@
         <v>42633867</v>
       </c>
       <c r="AN101" t="n">
-        <v>64587076.52533609</v>
+        <v>64843205.79110651</v>
       </c>
       <c r="AO101" t="n">
         <v>0</v>
@@ -24298,7 +24298,7 @@
         <v>24.4</v>
       </c>
       <c r="H102" t="n">
-        <v>624557030</v>
+        <v>627033800</v>
       </c>
       <c r="I102" t="n">
         <v>7700</v>
@@ -24316,7 +24316,7 @@
         <v>6.32</v>
       </c>
       <c r="N102" t="n">
-        <v>1.47367777041754</v>
+        <v>1.479521849846823</v>
       </c>
       <c r="O102" t="n">
         <v>0.49</v>
@@ -24394,7 +24394,7 @@
         <v>58273656.12</v>
       </c>
       <c r="AN102" t="n">
-        <v>64188800.61664954</v>
+        <v>64443350.46248715</v>
       </c>
       <c r="AO102" t="n">
         <v>0</v>
@@ -26883,7 +26883,7 @@
         <v>18</v>
       </c>
       <c r="H113" t="n">
-        <v>415210250</v>
+        <v>422516400</v>
       </c>
       <c r="I113" t="n">
         <v>0</v>
@@ -26901,7 +26901,7 @@
         <v>20.65</v>
       </c>
       <c r="N113" t="n">
-        <v>1.556151343823621</v>
+        <v>1.583533796787335</v>
       </c>
       <c r="O113" t="n">
         <v>0.54</v>
@@ -26979,7 +26979,7 @@
         <v>8431470.34</v>
       </c>
       <c r="AN113" t="n">
-        <v>30779114.15863603</v>
+        <v>31320711.63825056</v>
       </c>
       <c r="AO113" t="n">
         <v>0</v>
@@ -27118,7 +27118,7 @@
         <v>12.5</v>
       </c>
       <c r="H114" t="n">
-        <v>415210250</v>
+        <v>422516400</v>
       </c>
       <c r="I114" t="n">
         <v>5700</v>
@@ -27136,7 +27136,7 @@
         <v>23.27</v>
       </c>
       <c r="N114" t="n">
-        <v>1.280805369236534</v>
+        <v>1.303342761192652</v>
       </c>
       <c r="O114" t="n">
         <v>0.61</v>
@@ -27214,7 +27214,7 @@
         <v>10244057.54</v>
       </c>
       <c r="AN114" t="n">
-        <v>27334447.0046083</v>
+        <v>27815431.20473996</v>
       </c>
       <c r="AO114" t="n">
         <v>0</v>
@@ -27353,7 +27353,7 @@
         <v>13.1</v>
       </c>
       <c r="H115" t="n">
-        <v>415210250</v>
+        <v>422516400</v>
       </c>
       <c r="I115" t="n">
         <v>0</v>
@@ -27371,7 +27371,7 @@
         <v>22.56</v>
       </c>
       <c r="N115" t="n">
-        <v>2.425243248971241</v>
+        <v>2.467918474266067</v>
       </c>
       <c r="O115" t="n">
         <v>0.59</v>
@@ -27449,7 +27449,7 @@
         <v>5410032.13</v>
       </c>
       <c r="AN115" t="n">
-        <v>28188068.56754922</v>
+        <v>28684073.3197556</v>
       </c>
       <c r="AO115" t="n">
         <v>0</v>
@@ -28763,7 +28763,7 @@
         <v>0.42</v>
       </c>
       <c r="H121" t="n">
-        <v>11218346</v>
+        <v>11218350</v>
       </c>
       <c r="I121" t="n">
         <v>3700</v>
@@ -28781,7 +28781,7 @@
         <v>0.19</v>
       </c>
       <c r="N121" t="n">
-        <v>0.02590433969803708</v>
+        <v>0.02590434893445739</v>
       </c>
       <c r="O121" t="n">
         <v>0.02</v>
@@ -28859,7 +28859,7 @@
         <v>129011019.48</v>
       </c>
       <c r="AN121" t="n">
-        <v>3751955.183946488</v>
+        <v>3751956.52173913</v>
       </c>
       <c r="AO121" t="n">
         <v>0</v>
@@ -38633,7 +38633,7 @@
         <v>3.01</v>
       </c>
       <c r="H163" t="n">
-        <v>19804568</v>
+        <v>19804570</v>
       </c>
       <c r="I163" t="n">
         <v>0</v>
@@ -38651,7 +38651,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="N163" t="n">
-        <v>0.3691026732775719</v>
+        <v>0.3691027105520707</v>
       </c>
       <c r="O163" t="n">
         <v>0.07000000000000001</v>
@@ -38729,7 +38729,7 @@
         <v>8649345</v>
       </c>
       <c r="AN163" t="n">
-        <v>4951142</v>
+        <v>4951142.5</v>
       </c>
       <c r="AO163" t="n">
         <v>0</v>
@@ -38868,7 +38868,7 @@
         <v>2.17</v>
       </c>
       <c r="H164" t="n">
-        <v>19804568</v>
+        <v>19804570</v>
       </c>
       <c r="I164" t="n">
         <v>100</v>
@@ -38886,7 +38886,7 @@
         <v>1.51</v>
       </c>
       <c r="N164" t="n">
-        <v>0.0184551336638786</v>
+        <v>0.01845513552760354</v>
       </c>
       <c r="O164" t="n">
         <v>0.11</v>
@@ -38964,7 +38964,7 @@
         <v>172986900</v>
       </c>
       <c r="AN164" t="n">
-        <v>3084823.676012461</v>
+        <v>3084823.987538941</v>
       </c>
       <c r="AO164" t="n">
         <v>0</v>
@@ -40748,7 +40748,7 @@
         <v>3.79</v>
       </c>
       <c r="H172" t="n">
-        <v>204119089</v>
+        <v>204119100</v>
       </c>
       <c r="I172" t="n">
         <v>1400</v>
@@ -40766,7 +40766,7 @@
         <v>0.38</v>
       </c>
       <c r="N172" t="n">
-        <v>0.04519335750091549</v>
+        <v>0.04519335993639047</v>
       </c>
       <c r="O172" t="n">
         <v>0.08</v>
@@ -40844,7 +40844,7 @@
         <v>640901679.6</v>
       </c>
       <c r="AN172" t="n">
-        <v>204119089</v>
+        <v>204119100</v>
       </c>
       <c r="AO172" t="n">
         <v>0</v>
@@ -45213,7 +45213,7 @@
         <v>3.7</v>
       </c>
       <c r="H191" t="n">
-        <v>7136445</v>
+        <v>7136450</v>
       </c>
       <c r="I191" t="n">
         <v>400</v>
@@ -45231,7 +45231,7 @@
         <v>0.02</v>
       </c>
       <c r="N191" t="n">
-        <v>0.03766661503695458</v>
+        <v>0.03766664142727569</v>
       </c>
       <c r="O191" t="n">
         <v>0.01</v>
@@ -45309,7 +45309,7 @@
         <v>256931318.49</v>
       </c>
       <c r="AN191" t="n">
-        <v>118940750</v>
+        <v>118940833.3333333</v>
       </c>
       <c r="AO191" t="n">
         <v>0</v>
@@ -45448,7 +45448,7 @@
         <v>2.64</v>
       </c>
       <c r="H192" t="n">
-        <v>22907494</v>
+        <v>23562000</v>
       </c>
       <c r="I192" t="n">
         <v>2000</v>
@@ -45466,7 +45466,7 @@
         <v>21.95</v>
       </c>
       <c r="N192" t="n">
-        <v>2.342082523074298</v>
+        <v>2.408999797563042</v>
       </c>
       <c r="O192" t="n">
         <v>0.32</v>
@@ -45544,7 +45544,7 @@
         <v>357000.03</v>
       </c>
       <c r="AN192" t="n">
-        <v>1926618.50294365</v>
+        <v>1981665.264928511</v>
       </c>
       <c r="AO192" t="n">
         <v>0</v>
@@ -45683,7 +45683,7 @@
         <v>1.65</v>
       </c>
       <c r="H193" t="n">
-        <v>22907494</v>
+        <v>23562000</v>
       </c>
       <c r="I193" t="n">
         <v>15200</v>
@@ -45701,7 +45701,7 @@
         <v>14.71</v>
       </c>
       <c r="N193" t="n">
-        <v>1.171041409147398</v>
+        <v>1.204500050609246</v>
       </c>
       <c r="O193" t="n">
         <v>0.22</v>
@@ -45779,7 +45779,7 @@
         <v>713999.97</v>
       </c>
       <c r="AN193" t="n">
-        <v>2874215.056461731</v>
+        <v>2956336.26097867</v>
       </c>
       <c r="AO193" t="n">
         <v>0</v>
@@ -47563,7 +47563,7 @@
         <v>6.95</v>
       </c>
       <c r="H201" t="n">
-        <v>127688245</v>
+        <v>127688300</v>
       </c>
       <c r="I201" t="n">
         <v>1100</v>
@@ -47581,7 +47581,7 @@
         <v>1.99</v>
       </c>
       <c r="N201" t="n">
-        <v>1.506953711555548</v>
+        <v>1.50695436065566</v>
       </c>
       <c r="O201" t="n">
         <v>0.25</v>
@@ -47659,7 +47659,7 @@
         <v>28893848.04</v>
       </c>
       <c r="AN201" t="n">
-        <v>101339876.984127</v>
+        <v>101339920.6349206</v>
       </c>
       <c r="AO201" t="n">
         <v>0</v>
@@ -48006,7 +48006,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>IBOVESPA</t>
+          <t>Brazil Stock Exchange Index</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
@@ -51777,7 +51777,7 @@
         <v>0.63</v>
       </c>
       <c r="H219" t="n">
-        <v>8065726</v>
+        <v>8065730</v>
       </c>
       <c r="I219" t="n">
         <v>19200</v>
@@ -51795,7 +51795,7 @@
         <v>0.05</v>
       </c>
       <c r="N219" t="n">
-        <v>0.03655130783434104</v>
+        <v>0.03655132596107028</v>
       </c>
       <c r="O219" t="n">
         <v>0.02</v>
@@ -51873,7 +51873,7 @@
         <v>256438982.35</v>
       </c>
       <c r="AN219" t="n">
-        <v>134428766.6666667</v>
+        <v>134428833.3333333</v>
       </c>
       <c r="AO219" t="n">
         <v>0</v>
@@ -56007,7 +56007,7 @@
         <v>0.68</v>
       </c>
       <c r="H237" t="n">
-        <v>28655009</v>
+        <v>28655010</v>
       </c>
       <c r="I237" t="n">
         <v>66400</v>
@@ -56025,7 +56025,7 @@
         <v>5.38</v>
       </c>
       <c r="N237" t="n">
-        <v>0.4128926576357671</v>
+        <v>0.412892672044859</v>
       </c>
       <c r="O237" t="n">
         <v>0.11</v>
@@ -56103,7 +56103,7 @@
         <v>10271292.68</v>
       </c>
       <c r="AN237" t="n">
-        <v>2845581.827209533</v>
+        <v>2845581.926514399</v>
       </c>
       <c r="AO237" t="n">
         <v>0</v>
@@ -56242,7 +56242,7 @@
         <v>2.74</v>
       </c>
       <c r="H238" t="n">
-        <v>113896347</v>
+        <v>113896300</v>
       </c>
       <c r="I238" t="n">
         <v>11800</v>
@@ -56260,7 +56260,7 @@
         <v>4.2</v>
       </c>
       <c r="N238" t="n">
-        <v>1.329871511943582</v>
+        <v>1.329870963164251</v>
       </c>
       <c r="O238" t="n">
         <v>0.75</v>
@@ -56338,7 +56338,7 @@
         <v>23184000</v>
       </c>
       <c r="AN238" t="n">
-        <v>16459009.68208092</v>
+        <v>16459002.89017341</v>
       </c>
       <c r="AO238" t="n">
         <v>0</v>
@@ -75512,7 +75512,7 @@
         <v>0.79</v>
       </c>
       <c r="H320" t="n">
-        <v>292363839</v>
+        <v>294173400</v>
       </c>
       <c r="I320" t="n">
         <v>14700</v>
@@ -75530,7 +75530,7 @@
         <v>2.24</v>
       </c>
       <c r="N320" t="n">
-        <v>0.7410234426625275</v>
+        <v>0.7456099439429674</v>
       </c>
       <c r="O320" t="n">
         <v>0.13</v>
@@ -75608,7 +75608,7 @@
         <v>142942061.98</v>
       </c>
       <c r="AN320" t="n">
-        <v>23520823.73290426</v>
+        <v>23666403.8616251</v>
       </c>
       <c r="AO320" t="n">
         <v>0</v>
@@ -75747,7 +75747,7 @@
         <v>0.78</v>
       </c>
       <c r="H321" t="n">
-        <v>292363839</v>
+        <v>294173400</v>
       </c>
       <c r="I321" t="n">
         <v>49900</v>
@@ -75765,7 +75765,7 @@
         <v>2</v>
       </c>
       <c r="N321" t="n">
-        <v>3.691913708061926</v>
+        <v>3.714764492496571</v>
       </c>
       <c r="O321" t="n">
         <v>0.11</v>
@@ -75843,7 +75843,7 @@
         <v>28690654.02</v>
       </c>
       <c r="AN321" t="n">
-        <v>26362834.89630298</v>
+        <v>26526005.41027953</v>
       </c>
       <c r="AO321" t="n">
         <v>0</v>
@@ -76922,7 +76922,7 @@
         <v>1.15</v>
       </c>
       <c r="H326" t="n">
-        <v>77845372</v>
+        <v>77845370</v>
       </c>
       <c r="I326" t="n">
         <v>6800</v>
@@ -76940,7 +76940,7 @@
         <v>0.11</v>
       </c>
       <c r="N326" t="n">
-        <v>0.009003875812846389</v>
+        <v>0.009003875581519194</v>
       </c>
       <c r="O326" t="n">
         <v>0.02</v>
@@ -77018,7 +77018,7 @@
         <v>1659121826.79</v>
       </c>
       <c r="AN326" t="n">
-        <v>778453720</v>
+        <v>778453700</v>
       </c>
       <c r="AO326" t="n">
         <v>0</v>
@@ -80212,7 +80212,7 @@
         <v>5.85</v>
       </c>
       <c r="H340" t="n">
-        <v>394363937</v>
+        <v>394364000</v>
       </c>
       <c r="I340" t="n">
         <v>50900</v>
@@ -80230,7 +80230,7 @@
         <v>0.62</v>
       </c>
       <c r="N340" t="n">
-        <v>2.667368293678366</v>
+        <v>2.667368719792893</v>
       </c>
       <c r="O340" t="n">
         <v>0.1</v>
@@ -80308,7 +80308,7 @@
         <v>61075833.72000001</v>
       </c>
       <c r="AN340" t="n">
-        <v>428656453.2608696</v>
+        <v>428656521.7391304</v>
       </c>
       <c r="AO340" t="n">
         <v>0</v>
@@ -85617,7 +85617,7 @@
         <v>10.19</v>
       </c>
       <c r="H363" t="n">
-        <v>984492753</v>
+        <v>987117700</v>
       </c>
       <c r="I363" t="n">
         <v>100</v>
@@ -85635,7 +85635,7 @@
         <v>20.34</v>
       </c>
       <c r="N363" t="n">
-        <v>2.604367604797203</v>
+        <v>2.611311614197249</v>
       </c>
       <c r="O363" t="n">
         <v>0.27</v>
@@ -85713,7 +85713,7 @@
         <v>45966751.6</v>
       </c>
       <c r="AN363" t="n">
-        <v>104733271.5957447</v>
+        <v>105012521.2765957</v>
       </c>
       <c r="AO363" t="n">
         <v>0</v>
@@ -85852,7 +85852,7 @@
         <v>7.36</v>
       </c>
       <c r="H364" t="n">
-        <v>984492753</v>
+        <v>987117700</v>
       </c>
       <c r="I364" t="n">
         <v>1500</v>
@@ -85870,7 +85870,7 @@
         <v>14.31</v>
       </c>
       <c r="N364" t="n">
-        <v>11.8246640867124</v>
+        <v>11.8561921161731</v>
       </c>
       <c r="O364" t="n">
         <v>0.19</v>
@@ -85948,7 +85948,7 @@
         <v>10124120.05</v>
       </c>
       <c r="AN364" t="n">
-        <v>148939902.118003</v>
+        <v>149337019.6671709</v>
       </c>
       <c r="AO364" t="n">
         <v>0</v>
@@ -91962,7 +91962,7 @@
         <v>1.74</v>
       </c>
       <c r="H390" t="n">
-        <v>8491269</v>
+        <v>8491270</v>
       </c>
       <c r="I390" t="n">
         <v>1700</v>
@@ -91980,7 +91980,7 @@
         <v>1.29</v>
       </c>
       <c r="N390" t="n">
-        <v>1.514910531253058</v>
+        <v>1.514910709661083</v>
       </c>
       <c r="O390" t="n">
         <v>0.13</v>
@@ -92058,7 +92058,7 @@
         <v>2293618.8</v>
       </c>
       <c r="AN390" t="n">
-        <v>5586361.184210526</v>
+        <v>5586361.842105263</v>
       </c>
       <c r="AO390" t="n">
         <v>0</v>
@@ -94077,7 +94077,7 @@
         <v>3.87</v>
       </c>
       <c r="H399" t="n">
-        <v>5873894474</v>
+        <v>5872672000</v>
       </c>
       <c r="I399" t="n">
         <v>1500</v>
@@ -94095,7 +94095,7 @@
         <v>9.42</v>
       </c>
       <c r="N399" t="n">
-        <v>0.6621184168543131</v>
+        <v>0.6619806168728684</v>
       </c>
       <c r="O399" t="n">
         <v>0.66</v>
@@ -94173,7 +94173,7 @@
         <v>483489419.2399999</v>
       </c>
       <c r="AN399" t="n">
-        <v>1127426962.380038</v>
+        <v>1127192322.456814</v>
       </c>
       <c r="AO399" t="n">
         <v>0</v>
@@ -94312,7 +94312,7 @@
         <v>3.99</v>
       </c>
       <c r="H400" t="n">
-        <v>5873894474</v>
+        <v>5872672000</v>
       </c>
       <c r="I400" t="n">
         <v>7000</v>
@@ -94330,7 +94330,7 @@
         <v>9.92</v>
       </c>
       <c r="N400" t="n">
-        <v>1.436707852479965</v>
+        <v>1.436408845066226</v>
       </c>
       <c r="O400" t="n">
         <v>0.6899999999999999</v>
@@ -94408,7 +94408,7 @@
         <v>222820003.58</v>
       </c>
       <c r="AN400" t="n">
-        <v>1071878553.649635</v>
+        <v>1071655474.452555</v>
       </c>
       <c r="AO400" t="n">
         <v>0</v>
@@ -94782,7 +94782,7 @@
         <v>20.69</v>
       </c>
       <c r="H402" t="n">
-        <v>670363976</v>
+        <v>675087900</v>
       </c>
       <c r="I402" t="n">
         <v>0</v>
@@ -94800,7 +94800,7 @@
         <v>6.94</v>
       </c>
       <c r="N402" t="n">
-        <v>0.4821857729893996</v>
+        <v>0.4855836419486994</v>
       </c>
       <c r="O402" t="n">
         <v>0.53</v>
@@ -94878,7 +94878,7 @@
         <v>53525040.6</v>
       </c>
       <c r="AN402" t="n">
-        <v>165114279.8029557</v>
+        <v>166277807.8817734</v>
       </c>
       <c r="AO402" t="n">
         <v>0.9505</v>
@@ -95017,7 +95017,7 @@
         <v>16.96</v>
       </c>
       <c r="H403" t="n">
-        <v>670363976</v>
+        <v>675087900</v>
       </c>
       <c r="I403" t="n">
         <v>5000</v>
@@ -95035,7 +95035,7 @@
         <v>7.58</v>
       </c>
       <c r="N403" t="n">
-        <v>0.4026722432378139</v>
+        <v>0.4055097958839379</v>
       </c>
       <c r="O403" t="n">
         <v>0.58</v>
@@ -95113,7 +95113,7 @@
         <v>64094343.5</v>
       </c>
       <c r="AN403" t="n">
-        <v>151323696.6139955</v>
+        <v>152390045.1467269</v>
       </c>
       <c r="AO403" t="n">
         <v>0.7018</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-07-26 04:31
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -11488,31 +11488,31 @@
         <v>461566919.6347032</v>
       </c>
       <c r="AO47" t="n">
-        <v>0</v>
+        <v>0.3403</v>
       </c>
       <c r="AP47" t="n">
-        <v>0</v>
+        <v>0.6589</v>
       </c>
       <c r="AQ47" t="n">
-        <v>0</v>
+        <v>0.6853</v>
       </c>
       <c r="AR47" t="n">
-        <v>0</v>
+        <v>0.6309</v>
       </c>
       <c r="AS47" t="n">
-        <v>0</v>
+        <v>0.5834</v>
       </c>
       <c r="AT47" t="n">
-        <v>0</v>
+        <v>0.3231</v>
       </c>
       <c r="AU47" t="n">
-        <v>0</v>
+        <v>0.2345</v>
       </c>
       <c r="AV47" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AW47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX47" t="inlineStr">
         <is>
@@ -11532,7 +11532,7 @@
         <v>1.07</v>
       </c>
       <c r="BC47" t="n">
-        <v>0</v>
+        <v>8.66</v>
       </c>
       <c r="BD47" t="n">
         <v>43.87</v>
@@ -11547,7 +11547,7 @@
         <v>-87.59</v>
       </c>
       <c r="BH47" t="n">
-        <v>-100</v>
+        <v>-0.05</v>
       </c>
       <c r="BI47" t="n">
         <v>7.04</v>
@@ -11723,31 +11723,31 @@
         <v>458080764.652568</v>
       </c>
       <c r="AO48" t="n">
-        <v>0</v>
+        <v>0.3691</v>
       </c>
       <c r="AP48" t="n">
-        <v>0</v>
+        <v>0.7044</v>
       </c>
       <c r="AQ48" t="n">
-        <v>0</v>
+        <v>0.5017</v>
       </c>
       <c r="AR48" t="n">
-        <v>0</v>
+        <v>0.6309</v>
       </c>
       <c r="AS48" t="n">
-        <v>0</v>
+        <v>0.5834</v>
       </c>
       <c r="AT48" t="n">
-        <v>0</v>
+        <v>0.3231</v>
       </c>
       <c r="AU48" t="n">
-        <v>0</v>
+        <v>0.2345</v>
       </c>
       <c r="AV48" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AW48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX48" t="inlineStr">
         <is>
@@ -11767,7 +11767,7 @@
         <v>1.07</v>
       </c>
       <c r="BC48" t="n">
-        <v>0</v>
+        <v>8.27</v>
       </c>
       <c r="BD48" t="n">
         <v>39.99</v>
@@ -11782,7 +11782,7 @@
         <v>-87.92</v>
       </c>
       <c r="BH48" t="n">
-        <v>-100</v>
+        <v>-7.05</v>
       </c>
       <c r="BI48" t="n">
         <v>7.04</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-07-27 04:42
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1770,7 +1770,7 @@
         <v>7.76</v>
       </c>
       <c r="H6" t="n">
-        <v>489537208</v>
+        <v>489537300</v>
       </c>
       <c r="I6" t="n">
         <v>3100</v>
@@ -1788,7 +1788,7 @@
         <v>13.39</v>
       </c>
       <c r="N6" t="n">
-        <v>6.0386901196184</v>
+        <v>6.038691254485131</v>
       </c>
       <c r="O6" t="n">
         <v>1.24</v>
@@ -1866,7 +1866,7 @@
         <v>34696585</v>
       </c>
       <c r="AN6" t="n">
-        <v>52525451.50214592</v>
+        <v>52525461.37339056</v>
       </c>
       <c r="AO6" t="n">
         <v>0</v>
@@ -1943,7 +1943,7 @@
         <v>0.55</v>
       </c>
       <c r="BM6" t="n">
-        <v>0.52</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="BN6" t="n">
         <v>7.76</v>
@@ -1958,7 +1958,7 @@
         <v>7.69</v>
       </c>
       <c r="BR6" t="n">
-        <v>14.9</v>
+        <v>13.8</v>
       </c>
       <c r="BS6" t="n">
         <v>7.69</v>
@@ -8804,7 +8804,7 @@
         <v>26</v>
       </c>
       <c r="H36" t="n">
-        <v>208052325</v>
+        <v>207025000</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
@@ -8822,7 +8822,7 @@
         <v>10.3</v>
       </c>
       <c r="N36" t="n">
-        <v>1.900575174927114</v>
+        <v>1.891190476190476</v>
       </c>
       <c r="O36" t="n">
         <v>0.85</v>
@@ -8900,7 +8900,7 @@
         <v>12348000</v>
       </c>
       <c r="AN36" t="n">
-        <v>37218662.79069768</v>
+        <v>37034883.72093023</v>
       </c>
       <c r="AO36" t="n">
         <v>0</v>
@@ -9039,7 +9039,7 @@
         <v>16.25</v>
       </c>
       <c r="H37" t="n">
-        <v>208052325</v>
+        <v>207025000</v>
       </c>
       <c r="I37" t="n">
         <v>100</v>
@@ -9057,7 +9057,7 @@
         <v>7.41</v>
       </c>
       <c r="N37" t="n">
-        <v>1.900575174927114</v>
+        <v>1.891190476190476</v>
       </c>
       <c r="O37" t="n">
         <v>0.61</v>
@@ -9135,7 +9135,7 @@
         <v>12348000</v>
       </c>
       <c r="AN37" t="n">
-        <v>51754309.70149254</v>
+        <v>51498756.21890548</v>
       </c>
       <c r="AO37" t="n">
         <v>0</v>
@@ -10684,7 +10684,7 @@
         <v>4.5</v>
       </c>
       <c r="H44" t="n">
-        <v>6725750</v>
+        <v>6604320</v>
       </c>
       <c r="I44" t="n">
         <v>1000</v>
@@ -10702,7 +10702,7 @@
         <v>0.75</v>
       </c>
       <c r="N44" t="n">
-        <v>0.30055546287083</v>
+        <v>0.295129086651612</v>
       </c>
       <c r="O44" t="n">
         <v>0.03</v>
@@ -10780,7 +10780,7 @@
         <v>5719748.64</v>
       </c>
       <c r="AN44" t="n">
-        <v>6725750</v>
+        <v>6604320</v>
       </c>
       <c r="AO44" t="n">
         <v>0</v>
@@ -10919,7 +10919,7 @@
         <v>3.9</v>
       </c>
       <c r="H45" t="n">
-        <v>6725750</v>
+        <v>6604320</v>
       </c>
       <c r="I45" t="n">
         <v>0</v>
@@ -10937,7 +10937,7 @@
         <v>0.63</v>
       </c>
       <c r="N45" t="n">
-        <v>0.1838168836385937</v>
+        <v>0.1804981631716965</v>
       </c>
       <c r="O45" t="n">
         <v>0.02</v>
@@ -11015,7 +11015,7 @@
         <v>9352251.359999999</v>
       </c>
       <c r="AN45" t="n">
-        <v>8006845.238095239</v>
+        <v>7862285.714285715</v>
       </c>
       <c r="AO45" t="n">
         <v>0</v>
@@ -11389,7 +11389,7 @@
         <v>8.66</v>
       </c>
       <c r="H47" t="n">
-        <v>3032494662</v>
+        <v>3031801000</v>
       </c>
       <c r="I47" t="n">
         <v>10900</v>
@@ -11407,7 +11407,7 @@
         <v>8.390000000000001</v>
       </c>
       <c r="N47" t="n">
-        <v>0.8134567861885764</v>
+        <v>0.813270713623209</v>
       </c>
       <c r="O47" t="n">
         <v>0.07000000000000001</v>
@@ -11485,7 +11485,7 @@
         <v>249024468</v>
       </c>
       <c r="AN47" t="n">
-        <v>461566919.6347032</v>
+        <v>461461339.4216134</v>
       </c>
       <c r="AO47" t="n">
         <v>0.3403</v>
@@ -11624,7 +11624,7 @@
         <v>8.9</v>
       </c>
       <c r="H48" t="n">
-        <v>3032494662</v>
+        <v>3031801000</v>
       </c>
       <c r="I48" t="n">
         <v>2400</v>
@@ -11642,7 +11642,7 @@
         <v>8.449999999999999</v>
       </c>
       <c r="N48" t="n">
-        <v>2.213170977589777</v>
+        <v>2.212664730167186</v>
       </c>
       <c r="O48" t="n">
         <v>0.07000000000000001</v>
@@ -11720,7 +11720,7 @@
         <v>91529595.08</v>
       </c>
       <c r="AN48" t="n">
-        <v>458080764.652568</v>
+        <v>457975981.8731118</v>
       </c>
       <c r="AO48" t="n">
         <v>0.3691</v>
@@ -11859,7 +11859,7 @@
         <v>47.3</v>
       </c>
       <c r="H49" t="n">
-        <v>937234100</v>
+        <v>926847300</v>
       </c>
       <c r="I49" t="n">
         <v>0</v>
@@ -11877,7 +11877,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="N49" t="n">
-        <v>1.023378100427973</v>
+        <v>1.012036618450818</v>
       </c>
       <c r="O49" t="n">
         <v>0.08</v>
@@ -11955,7 +11955,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN49" t="n">
-        <v>171340786.1060329</v>
+        <v>169441919.5612431</v>
       </c>
       <c r="AO49" t="n">
         <v>2.4346</v>
@@ -12094,7 +12094,7 @@
         <v>33.01</v>
       </c>
       <c r="H50" t="n">
-        <v>937234100</v>
+        <v>926847300</v>
       </c>
       <c r="I50" t="n">
         <v>1900</v>
@@ -12112,7 +12112,7 @@
         <v>5.78</v>
       </c>
       <c r="N50" t="n">
-        <v>1.023378100427973</v>
+        <v>1.012036618450818</v>
       </c>
       <c r="O50" t="n">
         <v>0.06</v>
@@ -12190,7 +12190,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN50" t="n">
-        <v>245993202.0997375</v>
+        <v>243267007.8740157</v>
       </c>
       <c r="AO50" t="n">
         <v>3.526</v>
@@ -14428,7 +14428,7 @@
         <v>379.52</v>
       </c>
       <c r="H60" t="n">
-        <v>172586677</v>
+        <v>172586700</v>
       </c>
       <c r="I60" t="n">
         <v>12</v>
@@ -14446,7 +14446,7 @@
         <v>2.87</v>
       </c>
       <c r="N60" t="n">
-        <v>12.1960679168101</v>
+        <v>12.19606954213581</v>
       </c>
       <c r="O60" t="n">
         <v>0.64</v>
@@ -14524,7 +14524,7 @@
         <v>59731412.5</v>
       </c>
       <c r="AN60" t="n">
-        <v>21736357.30478589</v>
+        <v>21736360.20151133</v>
       </c>
       <c r="AO60" t="n">
         <v>0</v>
@@ -18893,7 +18893,7 @@
         <v>3</v>
       </c>
       <c r="H79" t="n">
-        <v>6400845000</v>
+        <v>6393543000</v>
       </c>
       <c r="I79" t="n">
         <v>3300</v>
@@ -18911,7 +18911,7 @@
         <v>2.47</v>
       </c>
       <c r="N79" t="n">
-        <v>0.8949601163823274</v>
+        <v>0.8939391576230037</v>
       </c>
       <c r="O79" t="n">
         <v>0.03</v>
@@ -18989,7 +18989,7 @@
         <v>531401092.4</v>
       </c>
       <c r="AN79" t="n">
-        <v>3879300000</v>
+        <v>3874874545.454545</v>
       </c>
       <c r="AO79" t="n">
         <v>0</v>
@@ -19128,7 +19128,7 @@
         <v>3</v>
       </c>
       <c r="H80" t="n">
-        <v>6400845000</v>
+        <v>6393543000</v>
       </c>
       <c r="I80" t="n">
         <v>3900</v>
@@ -19146,7 +19146,7 @@
         <v>3.36</v>
       </c>
       <c r="N80" t="n">
-        <v>1.725254390878755</v>
+        <v>1.723286243304146</v>
       </c>
       <c r="O80" t="n">
         <v>0.04</v>
@@ -19224,7 +19224,7 @@
         <v>275659512.02</v>
       </c>
       <c r="AN80" t="n">
-        <v>2844820000</v>
+        <v>2841574666.666667</v>
       </c>
       <c r="AO80" t="n">
         <v>0</v>
@@ -19598,7 +19598,7 @@
         <v>9.19</v>
       </c>
       <c r="H82" t="n">
-        <v>383857700</v>
+        <v>388508000</v>
       </c>
       <c r="I82" t="n">
         <v>1300</v>
@@ -19616,7 +19616,7 @@
         <v>6.04</v>
       </c>
       <c r="N82" t="n">
-        <v>0.9760999328682523</v>
+        <v>0.9879250376344644</v>
       </c>
       <c r="O82" t="n">
         <v>1.01</v>
@@ -19694,7 +19694,7 @@
         <v>65949124.8</v>
       </c>
       <c r="AN82" t="n">
-        <v>68302081.85053381</v>
+        <v>69129537.36654805</v>
       </c>
       <c r="AO82" t="n">
         <v>0</v>
@@ -20491,7 +20491,7 @@
         <v>0</v>
       </c>
       <c r="BR85" t="n">
-        <v>29</v>
+        <v>26.5</v>
       </c>
       <c r="BS85" t="n">
         <v>0</v>
@@ -21948,7 +21948,7 @@
         <v>9</v>
       </c>
       <c r="H92" t="n">
-        <v>73314660</v>
+        <v>77661760</v>
       </c>
       <c r="I92" t="n">
         <v>0</v>
@@ -21966,7 +21966,7 @@
         <v>3.42</v>
       </c>
       <c r="N92" t="n">
-        <v>0.1353720483164855</v>
+        <v>0.1433987626357853</v>
       </c>
       <c r="O92" t="n">
         <v>0.15</v>
@@ -22044,7 +22044,7 @@
         <v>23342055.36</v>
       </c>
       <c r="AN92" t="n">
-        <v>51996212.76595745</v>
+        <v>55079262.41134752</v>
       </c>
       <c r="AO92" t="n">
         <v>0</v>
@@ -22183,7 +22183,7 @@
         <v>6.11</v>
       </c>
       <c r="H93" t="n">
-        <v>73314660</v>
+        <v>77661760</v>
       </c>
       <c r="I93" t="n">
         <v>100</v>
@@ -22201,7 +22201,7 @@
         <v>2.3</v>
       </c>
       <c r="N93" t="n">
-        <v>0.1799676391962926</v>
+        <v>0.1906385926502158</v>
       </c>
       <c r="O93" t="n">
         <v>0.1</v>
@@ -22279,7 +22279,7 @@
         <v>17557944.64</v>
       </c>
       <c r="AN93" t="n">
-        <v>77173326.31578948</v>
+        <v>81749221.05263159</v>
       </c>
       <c r="AO93" t="n">
         <v>0</v>
@@ -22418,7 +22418,7 @@
         <v>46.8</v>
       </c>
       <c r="H94" t="n">
-        <v>8227464000</v>
+        <v>8273063000</v>
       </c>
       <c r="I94" t="n">
         <v>200</v>
@@ -22436,7 +22436,7 @@
         <v>5.78</v>
       </c>
       <c r="N94" t="n">
-        <v>0.7724929026406873</v>
+        <v>0.7767742831325999</v>
       </c>
       <c r="O94" t="n">
         <v>0.36</v>
@@ -22514,7 +22514,7 @@
         <v>1209900967.64</v>
       </c>
       <c r="AN94" t="n">
-        <v>2959519424.460432</v>
+        <v>2975921942.446043</v>
       </c>
       <c r="AO94" t="n">
         <v>0</v>
@@ -22653,7 +22653,7 @@
         <v>42.6</v>
       </c>
       <c r="H95" t="n">
-        <v>8227464000</v>
+        <v>8273063000</v>
       </c>
       <c r="I95" t="n">
         <v>0</v>
@@ -22671,7 +22671,7 @@
         <v>4.65</v>
       </c>
       <c r="N95" t="n">
-        <v>4.313621474319343</v>
+        <v>4.337528819961633</v>
       </c>
       <c r="O95" t="n">
         <v>0.29</v>
@@ -22749,7 +22749,7 @@
         <v>216671749.24</v>
       </c>
       <c r="AN95" t="n">
-        <v>3672975000</v>
+        <v>3693331696.428571</v>
       </c>
       <c r="AO95" t="n">
         <v>0</v>
@@ -23593,7 +23593,7 @@
         <v>126.1</v>
       </c>
       <c r="H99" t="n">
-        <v>16529806245</v>
+        <v>16624870000</v>
       </c>
       <c r="I99" t="n">
         <v>0</v>
@@ -23611,7 +23611,7 @@
         <v>10.65</v>
       </c>
       <c r="N99" t="n">
-        <v>1.633248878307715</v>
+        <v>1.642641775533503</v>
       </c>
       <c r="O99" t="n">
         <v>1.16</v>
@@ -23689,7 +23689,7 @@
         <v>1267125769.6</v>
       </c>
       <c r="AN99" t="n">
-        <v>2845061315.834768</v>
+        <v>2861423407.917384</v>
       </c>
       <c r="AO99" t="n">
         <v>0</v>
@@ -23828,7 +23828,7 @@
         <v>123.1</v>
       </c>
       <c r="H100" t="n">
-        <v>16529806245</v>
+        <v>16624870000</v>
       </c>
       <c r="I100" t="n">
         <v>800</v>
@@ -23846,7 +23846,7 @@
         <v>10.81</v>
       </c>
       <c r="N100" t="n">
-        <v>5.919283296957611</v>
+        <v>5.953325395744328</v>
       </c>
       <c r="O100" t="n">
         <v>1.18</v>
@@ -23924,7 +23924,7 @@
         <v>349625391.8</v>
       </c>
       <c r="AN100" t="n">
-        <v>2801662075.423728</v>
+        <v>2817774576.271186</v>
       </c>
       <c r="AO100" t="n">
         <v>0</v>
@@ -24063,7 +24063,7 @@
         <v>24.34</v>
       </c>
       <c r="H101" t="n">
-        <v>623796614</v>
+        <v>622065200</v>
       </c>
       <c r="I101" t="n">
         <v>200</v>
@@ -24081,7 +24081,7 @@
         <v>6.28</v>
       </c>
       <c r="N101" t="n">
-        <v>2.011828634381207</v>
+        <v>2.006244589541925</v>
       </c>
       <c r="O101" t="n">
         <v>0.49</v>
@@ -24159,7 +24159,7 @@
         <v>42633867</v>
       </c>
       <c r="AN101" t="n">
-        <v>64508439.91726991</v>
+        <v>64329389.8655636</v>
       </c>
       <c r="AO101" t="n">
         <v>0</v>
@@ -24298,7 +24298,7 @@
         <v>24.29</v>
       </c>
       <c r="H102" t="n">
-        <v>623796614</v>
+        <v>622065200</v>
       </c>
       <c r="I102" t="n">
         <v>1600</v>
@@ -24316,7 +24316,7 @@
         <v>6.32</v>
       </c>
       <c r="N102" t="n">
-        <v>1.471883525694252</v>
+        <v>1.467798156063252</v>
       </c>
       <c r="O102" t="n">
         <v>0.49</v>
@@ -24394,7 +24394,7 @@
         <v>58273656.12</v>
       </c>
       <c r="AN102" t="n">
-        <v>64110648.92086331</v>
+        <v>63932702.98047276</v>
       </c>
       <c r="AO102" t="n">
         <v>0</v>
@@ -28763,7 +28763,7 @@
         <v>0.42</v>
       </c>
       <c r="H121" t="n">
-        <v>11218346</v>
+        <v>11218350</v>
       </c>
       <c r="I121" t="n">
         <v>3100</v>
@@ -28781,7 +28781,7 @@
         <v>0.19</v>
       </c>
       <c r="N121" t="n">
-        <v>0.02590433969803708</v>
+        <v>0.02590434893445739</v>
       </c>
       <c r="O121" t="n">
         <v>0.02</v>
@@ -28859,7 +28859,7 @@
         <v>129011019.48</v>
       </c>
       <c r="AN121" t="n">
-        <v>3751955.183946488</v>
+        <v>3751956.52173913</v>
       </c>
       <c r="AO121" t="n">
         <v>0</v>
@@ -32288,7 +32288,7 @@
         <v>6.51</v>
       </c>
       <c r="H136" t="n">
-        <v>431356500</v>
+        <v>434109600</v>
       </c>
       <c r="I136" t="n">
         <v>0</v>
@@ -32306,7 +32306,7 @@
         <v>89.8</v>
       </c>
       <c r="N136" t="n">
-        <v>1.006904588014407</v>
+        <v>1.013331079840222</v>
       </c>
       <c r="O136" t="n">
         <v>0.49</v>
@@ -32384,7 +32384,7 @@
         <v>3812747.4</v>
       </c>
       <c r="AN136" t="n">
-        <v>7292586.644125106</v>
+        <v>7339131.022823331</v>
       </c>
       <c r="AO136" t="n">
         <v>0</v>
@@ -32523,7 +32523,7 @@
         <v>3.84</v>
       </c>
       <c r="H137" t="n">
-        <v>431356500</v>
+        <v>434109600</v>
       </c>
       <c r="I137" t="n">
         <v>3300</v>
@@ -32541,7 +32541,7 @@
         <v>51.86</v>
       </c>
       <c r="N137" t="n">
-        <v>2.589729122779466</v>
+        <v>2.606257871616969</v>
       </c>
       <c r="O137" t="n">
         <v>0.29</v>
@@ -32619,7 +32619,7 @@
         <v>1482422.55</v>
       </c>
       <c r="AN137" t="n">
-        <v>12623836.69885865</v>
+        <v>12704407.37489025</v>
       </c>
       <c r="AO137" t="n">
         <v>0</v>
@@ -32758,7 +32758,7 @@
         <v>4.77</v>
       </c>
       <c r="H138" t="n">
-        <v>63545796</v>
+        <v>63545840</v>
       </c>
       <c r="I138" t="n">
         <v>127600</v>
@@ -32776,7 +32776,7 @@
         <v>15.76</v>
       </c>
       <c r="N138" t="n">
-        <v>0.3384426491106866</v>
+        <v>0.3384428834531215</v>
       </c>
       <c r="O138" t="n">
         <v>0.2</v>
@@ -32854,7 +32854,7 @@
         <v>2797615.38</v>
       </c>
       <c r="AN138" t="n">
-        <v>33096768.75</v>
+        <v>33096791.66666667</v>
       </c>
       <c r="AO138" t="n">
         <v>0</v>
@@ -40748,7 +40748,7 @@
         <v>3.6</v>
       </c>
       <c r="H172" t="n">
-        <v>193886238</v>
+        <v>193886200</v>
       </c>
       <c r="I172" t="n">
         <v>2200</v>
@@ -40766,7 +40766,7 @@
         <v>0.38</v>
       </c>
       <c r="N172" t="n">
-        <v>0.04292773454638329</v>
+        <v>0.0429277261329243</v>
       </c>
       <c r="O172" t="n">
         <v>0.08</v>
@@ -40844,7 +40844,7 @@
         <v>640901679.6</v>
       </c>
       <c r="AN172" t="n">
-        <v>193886238</v>
+        <v>193886200</v>
       </c>
       <c r="AO172" t="n">
         <v>0</v>
@@ -45448,7 +45448,7 @@
         <v>2.87</v>
       </c>
       <c r="H192" t="n">
-        <v>22905568</v>
+        <v>23522330</v>
       </c>
       <c r="I192" t="n">
         <v>5500</v>
@@ -45466,7 +45466,7 @@
         <v>21.95</v>
       </c>
       <c r="N192" t="n">
-        <v>2.341885607124459</v>
+        <v>2.40494390154533</v>
       </c>
       <c r="O192" t="n">
         <v>0.32</v>
@@ -45544,7 +45544,7 @@
         <v>357000.03</v>
       </c>
       <c r="AN192" t="n">
-        <v>1926456.518082422</v>
+        <v>1978328.847771236</v>
       </c>
       <c r="AO192" t="n">
         <v>0</v>
@@ -45683,7 +45683,7 @@
         <v>1.53</v>
       </c>
       <c r="H193" t="n">
-        <v>22905568</v>
+        <v>23522330</v>
       </c>
       <c r="I193" t="n">
         <v>5200</v>
@@ -45701,7 +45701,7 @@
         <v>14.71</v>
       </c>
       <c r="N193" t="n">
-        <v>1.170942951160068</v>
+        <v>1.202472102344766</v>
       </c>
       <c r="O193" t="n">
         <v>0.22</v>
@@ -45779,7 +45779,7 @@
         <v>713999.97</v>
       </c>
       <c r="AN193" t="n">
-        <v>2873973.400250941</v>
+        <v>2951358.845671267</v>
       </c>
       <c r="AO193" t="n">
         <v>0</v>
@@ -47563,7 +47563,7 @@
         <v>7</v>
       </c>
       <c r="H201" t="n">
-        <v>128606800</v>
+        <v>128606900</v>
       </c>
       <c r="I201" t="n">
         <v>1100</v>
@@ -47581,7 +47581,7 @@
         <v>1.99</v>
       </c>
       <c r="N201" t="n">
-        <v>1.51779433252671</v>
+        <v>1.517795512708732</v>
       </c>
       <c r="O201" t="n">
         <v>0.25</v>
@@ -47659,7 +47659,7 @@
         <v>28893848.04</v>
       </c>
       <c r="AN201" t="n">
-        <v>102068888.8888889</v>
+        <v>102068968.2539683</v>
       </c>
       <c r="AO201" t="n">
         <v>0</v>
@@ -48006,7 +48006,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>IBOVESPA</t>
+          <t>Brazil Stock Exchange Index</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
@@ -51777,7 +51777,7 @@
         <v>0.54</v>
       </c>
       <c r="H219" t="n">
-        <v>6913485</v>
+        <v>6913480</v>
       </c>
       <c r="I219" t="n">
         <v>2100</v>
@@ -51795,7 +51795,7 @@
         <v>0.05</v>
       </c>
       <c r="N219" t="n">
-        <v>0.03132971767737948</v>
+        <v>0.03132969501896792</v>
       </c>
       <c r="O219" t="n">
         <v>0.02</v>
@@ -51873,7 +51873,7 @@
         <v>256438982.35</v>
       </c>
       <c r="AN219" t="n">
-        <v>115224750</v>
+        <v>115224666.6666667</v>
       </c>
       <c r="AO219" t="n">
         <v>0</v>
@@ -56007,7 +56007,7 @@
         <v>0.66</v>
       </c>
       <c r="H237" t="n">
-        <v>27812209</v>
+        <v>27812210</v>
       </c>
       <c r="I237" t="n">
         <v>60800</v>
@@ -56025,7 +56025,7 @@
         <v>5.38</v>
       </c>
       <c r="N237" t="n">
-        <v>0.4007486749954048</v>
+        <v>0.4007486894044967</v>
       </c>
       <c r="O237" t="n">
         <v>0.11</v>
@@ -56103,7 +56103,7 @@
         <v>10271292.68</v>
       </c>
       <c r="AN237" t="n">
-        <v>2761887.686196623</v>
+        <v>2761887.785501489</v>
       </c>
       <c r="AO237" t="n">
         <v>0</v>
@@ -56242,7 +56242,7 @@
         <v>2.71</v>
       </c>
       <c r="H238" t="n">
-        <v>112649281</v>
+        <v>112649300</v>
       </c>
       <c r="I238" t="n">
         <v>4100</v>
@@ -56260,7 +56260,7 @@
         <v>4.2</v>
       </c>
       <c r="N238" t="n">
-        <v>1.315310574823154</v>
+        <v>1.315310796670117</v>
       </c>
       <c r="O238" t="n">
         <v>0.75</v>
@@ -56338,7 +56338,7 @@
         <v>23184000</v>
       </c>
       <c r="AN238" t="n">
-        <v>16278797.83236994</v>
+        <v>16278800.57803468</v>
       </c>
       <c r="AO238" t="n">
         <v>0</v>
@@ -59767,7 +59767,7 @@
         <v>17.11</v>
       </c>
       <c r="H253" t="n">
-        <v>169748949</v>
+        <v>169749000</v>
       </c>
       <c r="I253" t="n">
         <v>1300</v>
@@ -59785,7 +59785,7 @@
         <v>7.29</v>
       </c>
       <c r="N253" t="n">
-        <v>0.1697088977001428</v>
+        <v>0.1697089486881096</v>
       </c>
       <c r="O253" t="n">
         <v>0.12</v>
@@ -59863,7 +59863,7 @@
         <v>24405758.4</v>
       </c>
       <c r="AN253" t="n">
-        <v>117068240.6896552</v>
+        <v>117068275.862069</v>
       </c>
       <c r="AO253" t="n">
         <v>0</v>
@@ -60002,7 +60002,7 @@
         <v>3.98</v>
       </c>
       <c r="H254" t="n">
-        <v>282583901</v>
+        <v>282584000</v>
       </c>
       <c r="I254" t="n">
         <v>9700</v>
@@ -60020,7 +60020,7 @@
         <v>0.59</v>
       </c>
       <c r="N254" t="n">
-        <v>0.660799269562389</v>
+        <v>0.6607995010657671</v>
       </c>
       <c r="O254" t="n">
         <v>0.6899999999999999</v>
@@ -60098,7 +60098,7 @@
         <v>520437330</v>
       </c>
       <c r="AN254" t="n">
-        <v>179989745.8598726</v>
+        <v>179989808.9171974</v>
       </c>
       <c r="AO254" t="n">
         <v>0</v>
@@ -63970,7 +63970,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Neogrid Participacoes SA</t>
+          <t>NEOGRID ON</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -64170,7 +64170,7 @@
         <v>2.16</v>
       </c>
       <c r="BM271" t="n">
-        <v>-1.1</v>
+        <v>0</v>
       </c>
       <c r="BN271" t="n">
         <v>0</v>
@@ -64194,7 +64194,7 @@
         <v>0.89</v>
       </c>
       <c r="BU271" t="n">
-        <v>40853</v>
+        <v>25403</v>
       </c>
     </row>
     <row r="272">
@@ -67287,7 +67287,7 @@
         <v>1.24</v>
       </c>
       <c r="H285" t="n">
-        <v>4076478</v>
+        <v>4076480</v>
       </c>
       <c r="I285" t="n">
         <v>1100</v>
@@ -67305,7 +67305,7 @@
         <v>0.05</v>
       </c>
       <c r="N285" t="n">
-        <v>0.04132263925757199</v>
+        <v>0.04132265953126868</v>
       </c>
       <c r="O285" t="n">
         <v>0.02</v>
@@ -67383,7 +67383,7 @@
         <v>178674864.1</v>
       </c>
       <c r="AN285" t="n">
-        <v>20382390</v>
+        <v>20382400</v>
       </c>
       <c r="AO285" t="n">
         <v>0</v>
@@ -75042,7 +75042,7 @@
         <v>5.8</v>
       </c>
       <c r="H318" t="n">
-        <v>14895583689</v>
+        <v>14895580000</v>
       </c>
       <c r="I318" t="n">
         <v>400</v>
@@ -75060,7 +75060,7 @@
         <v>11.35</v>
       </c>
       <c r="N318" t="n">
-        <v>0.7677090446679654</v>
+        <v>0.7677088545392182</v>
       </c>
       <c r="O318" t="n">
         <v>0.49</v>
@@ -75138,7 +75138,7 @@
         <v>1412512331.45</v>
       </c>
       <c r="AN318" t="n">
-        <v>3295483117.035398</v>
+        <v>3295482300.884956</v>
       </c>
       <c r="AO318" t="n">
         <v>0</v>
@@ -76922,7 +76922,7 @@
         <v>1.14</v>
       </c>
       <c r="H326" t="n">
-        <v>77168457</v>
+        <v>77168460</v>
       </c>
       <c r="I326" t="n">
         <v>1300</v>
@@ -76940,7 +76940,7 @@
         <v>0.11</v>
       </c>
       <c r="N326" t="n">
-        <v>0.00892558138840902</v>
+        <v>0.008925581735399814</v>
       </c>
       <c r="O326" t="n">
         <v>0.02</v>
@@ -77018,7 +77018,7 @@
         <v>1659121826.79</v>
       </c>
       <c r="AN326" t="n">
-        <v>771684570</v>
+        <v>771684600</v>
       </c>
       <c r="AO326" t="n">
         <v>0</v>
@@ -82797,7 +82797,7 @@
         <v>38.66</v>
       </c>
       <c r="H351" t="n">
-        <v>153468374</v>
+        <v>153468400</v>
       </c>
       <c r="I351" t="n">
         <v>0</v>
@@ -82815,7 +82815,7 @@
         <v>3.42</v>
       </c>
       <c r="N351" t="n">
-        <v>1.99752587529981</v>
+        <v>1.997526213712679</v>
       </c>
       <c r="O351" t="n">
         <v>0.78</v>
@@ -82893,7 +82893,7 @@
         <v>9672800</v>
       </c>
       <c r="AN351" t="n">
-        <v>61882408.87096775</v>
+        <v>61882419.35483871</v>
       </c>
       <c r="AO351" t="n">
         <v>0</v>
@@ -83032,7 +83032,7 @@
         <v>77.09</v>
       </c>
       <c r="H352" t="n">
-        <v>153468374</v>
+        <v>153468400</v>
       </c>
       <c r="I352" t="n">
         <v>100</v>
@@ -83050,7 +83050,7 @@
         <v>6.19</v>
       </c>
       <c r="N352" t="n">
-        <v>2.179304294234817</v>
+        <v>2.179304663443861</v>
       </c>
       <c r="O352" t="n">
         <v>1.42</v>
@@ -83128,7 +83128,7 @@
         <v>8865980</v>
       </c>
       <c r="AN352" t="n">
-        <v>34104083.11111111</v>
+        <v>34104088.88888889</v>
       </c>
       <c r="AO352" t="n">
         <v>0</v>
@@ -83267,7 +83267,7 @@
         <v>79.98</v>
       </c>
       <c r="H353" t="n">
-        <v>153468374</v>
+        <v>153468400</v>
       </c>
       <c r="I353" t="n">
         <v>0</v>
@@ -83285,7 +83285,7 @@
         <v>6.02</v>
       </c>
       <c r="N353" t="n">
-        <v>2.092110790721446</v>
+        <v>2.092111145158514</v>
       </c>
       <c r="O353" t="n">
         <v>1.38</v>
@@ -83363,7 +83363,7 @@
         <v>9235490</v>
       </c>
       <c r="AN353" t="n">
-        <v>35118621.05263158</v>
+        <v>35118627.00228833</v>
       </c>
       <c r="AO353" t="n">
         <v>0</v>
@@ -85617,7 +85617,7 @@
         <v>10.45</v>
       </c>
       <c r="H363" t="n">
-        <v>989112625</v>
+        <v>1008847000</v>
       </c>
       <c r="I363" t="n">
         <v>600</v>
@@ -85635,7 +85635,7 @@
         <v>20.34</v>
       </c>
       <c r="N363" t="n">
-        <v>2.616588969493332</v>
+        <v>2.668794094207867</v>
       </c>
       <c r="O363" t="n">
         <v>0.27</v>
@@ -85713,7 +85713,7 @@
         <v>45966751.6</v>
       </c>
       <c r="AN363" t="n">
-        <v>105224747.3404255</v>
+        <v>107324148.9361702</v>
       </c>
       <c r="AO363" t="n">
         <v>0</v>
@@ -85852,7 +85852,7 @@
         <v>7.36</v>
       </c>
       <c r="H364" t="n">
-        <v>989112625</v>
+        <v>1008847000</v>
       </c>
       <c r="I364" t="n">
         <v>1300</v>
@@ -85870,7 +85870,7 @@
         <v>14.31</v>
       </c>
       <c r="N364" t="n">
-        <v>11.88015300154407</v>
+        <v>12.11718100873369</v>
       </c>
       <c r="O364" t="n">
         <v>0.19</v>
@@ -85948,7 +85948,7 @@
         <v>10124120.05</v>
       </c>
       <c r="AN364" t="n">
-        <v>149638823.7518911</v>
+        <v>152624357.0347958</v>
       </c>
       <c r="AO364" t="n">
         <v>0</v>
@@ -88907,7 +88907,7 @@
         <v>1.13</v>
       </c>
       <c r="H377" t="n">
-        <v>74677586</v>
+        <v>74677590</v>
       </c>
       <c r="I377" t="n">
         <v>8700</v>
@@ -88925,7 +88925,7 @@
         <v>39.8</v>
       </c>
       <c r="N377" t="n">
-        <v>0.2768499802773232</v>
+        <v>0.2768499951064035</v>
       </c>
       <c r="O377" t="n">
         <v>0.24</v>
@@ -89003,7 +89003,7 @@
         <v>2643454.56</v>
       </c>
       <c r="AN377" t="n">
-        <v>7051707.837582625</v>
+        <v>7051708.21529745</v>
       </c>
       <c r="AO377" t="n">
         <v>0</v>
@@ -93842,7 +93842,7 @@
         <v>3.45</v>
       </c>
       <c r="H398" t="n">
-        <v>38365656</v>
+        <v>38365690</v>
       </c>
       <c r="I398" t="n">
         <v>400</v>
@@ -93860,7 +93860,7 @@
         <v>5.91</v>
       </c>
       <c r="N398" t="n">
-        <v>0.2619317797409575</v>
+        <v>0.2619320118673289</v>
       </c>
       <c r="O398" t="n">
         <v>0.23</v>
@@ -93938,7 +93938,7 @@
         <v>11454105.73</v>
       </c>
       <c r="AN398" t="n">
-        <v>16465946.78111588</v>
+        <v>16465961.37339056</v>
       </c>
       <c r="AO398" t="n">
         <v>0</v>
@@ -94077,7 +94077,7 @@
         <v>3.88</v>
       </c>
       <c r="H399" t="n">
-        <v>5899980296</v>
+        <v>5868736000</v>
       </c>
       <c r="I399" t="n">
         <v>1800</v>
@@ -94095,7 +94095,7 @@
         <v>9.42</v>
       </c>
       <c r="N399" t="n">
-        <v>0.6650588685838147</v>
+        <v>0.6615369422205105</v>
       </c>
       <c r="O399" t="n">
         <v>0.66</v>
@@ -94173,7 +94173,7 @@
         <v>483489419.2399999</v>
       </c>
       <c r="AN399" t="n">
-        <v>1132433838.003839</v>
+        <v>1126436852.207294</v>
       </c>
       <c r="AO399" t="n">
         <v>0</v>
@@ -94312,7 +94312,7 @@
         <v>3.96</v>
       </c>
       <c r="H400" t="n">
-        <v>5899980296</v>
+        <v>5868736000</v>
       </c>
       <c r="I400" t="n">
         <v>4400</v>
@@ -94330,7 +94330,7 @@
         <v>9.92</v>
       </c>
       <c r="N400" t="n">
-        <v>1.44308823698835</v>
+        <v>1.435446130783156</v>
       </c>
       <c r="O400" t="n">
         <v>0.6899999999999999</v>
@@ -94408,7 +94408,7 @@
         <v>222820003.58</v>
       </c>
       <c r="AN400" t="n">
-        <v>1076638740.145985</v>
+        <v>1070937226.277372</v>
       </c>
       <c r="AO400" t="n">
         <v>0</v>
@@ -94782,7 +94782,7 @@
         <v>20.15</v>
       </c>
       <c r="H402" t="n">
-        <v>670324100</v>
+        <v>669661300</v>
       </c>
       <c r="I402" t="n">
         <v>200</v>
@@ -94800,7 +94800,7 @@
         <v>6.94</v>
       </c>
       <c r="N402" t="n">
-        <v>0.4821570906010672</v>
+        <v>0.4816803455166365</v>
       </c>
       <c r="O402" t="n">
         <v>0.53</v>
@@ -94878,7 +94878,7 @@
         <v>53525040.6</v>
       </c>
       <c r="AN402" t="n">
-        <v>165104458.1280788</v>
+        <v>164941206.8965517</v>
       </c>
       <c r="AO402" t="n">
         <v>0.9505</v>
@@ -95017,7 +95017,7 @@
         <v>16.92</v>
       </c>
       <c r="H403" t="n">
-        <v>670324100</v>
+        <v>669661300</v>
       </c>
       <c r="I403" t="n">
         <v>0</v>
@@ -95035,7 +95035,7 @@
         <v>7.58</v>
       </c>
       <c r="N403" t="n">
-        <v>0.4026482906404993</v>
+        <v>0.4022501619039128</v>
       </c>
       <c r="O403" t="n">
         <v>0.58</v>
@@ -95113,7 +95113,7 @@
         <v>64094343.5</v>
       </c>
       <c r="AN403" t="n">
-        <v>151314695.2595937</v>
+        <v>151165079.006772</v>
       </c>
       <c r="AO403" t="n">
         <v>0.7018</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-08-02 04:31
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -94179,28 +94179,28 @@
         <v>0</v>
       </c>
       <c r="AP399" t="n">
-        <v>0.6951000000000001</v>
+        <v>0</v>
       </c>
       <c r="AQ399" t="n">
-        <v>0.3795</v>
+        <v>0</v>
       </c>
       <c r="AR399" t="n">
-        <v>0.3404</v>
+        <v>0</v>
       </c>
       <c r="AS399" t="n">
-        <v>0.1871</v>
+        <v>0</v>
       </c>
       <c r="AT399" t="n">
-        <v>0.587</v>
+        <v>0</v>
       </c>
       <c r="AU399" t="n">
-        <v>1.2127</v>
+        <v>0</v>
       </c>
       <c r="AV399" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AW399" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX399" t="inlineStr">
         <is>
@@ -94220,7 +94220,7 @@
         <v>0.55</v>
       </c>
       <c r="BC399" t="n">
-        <v>9.449999999999999</v>
+        <v>0</v>
       </c>
       <c r="BD399" t="n">
         <v>3.7</v>
@@ -94235,7 +94235,7 @@
         <v>-85.34</v>
       </c>
       <c r="BH399" t="n">
-        <v>151.99</v>
+        <v>-100</v>
       </c>
       <c r="BI399" t="n">
         <v>1.43</v>
@@ -94414,28 +94414,28 @@
         <v>0</v>
       </c>
       <c r="AP400" t="n">
-        <v>0.7439</v>
+        <v>0</v>
       </c>
       <c r="AQ400" t="n">
-        <v>0.4159</v>
+        <v>0</v>
       </c>
       <c r="AR400" t="n">
-        <v>0.3745</v>
+        <v>0</v>
       </c>
       <c r="AS400" t="n">
-        <v>0.2058</v>
+        <v>0</v>
       </c>
       <c r="AT400" t="n">
-        <v>0.6457000000000001</v>
+        <v>0</v>
       </c>
       <c r="AU400" t="n">
-        <v>1.334</v>
+        <v>0</v>
       </c>
       <c r="AV400" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AW400" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX400" t="inlineStr">
         <is>
@@ -94455,7 +94455,7 @@
         <v>0.55</v>
       </c>
       <c r="BC400" t="n">
-        <v>10.33</v>
+        <v>0</v>
       </c>
       <c r="BD400" t="n">
         <v>-2.78</v>
@@ -94470,7 +94470,7 @@
         <v>-86.26000000000001</v>
       </c>
       <c r="BH400" t="n">
-        <v>158.32</v>
+        <v>-100</v>
       </c>
       <c r="BI400" t="n">
         <v>1.43</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-08-03 04:35
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1473,7 +1473,7 @@
         <v>1.02</v>
       </c>
       <c r="BM4" t="n">
-        <v>0.99</v>
+        <v>0.76</v>
       </c>
       <c r="BN4" t="n">
         <v>16.1</v>
@@ -1488,7 +1488,7 @@
         <v>15.85</v>
       </c>
       <c r="BR4" t="n">
-        <v>16.08</v>
+        <v>21.06</v>
       </c>
       <c r="BS4" t="n">
         <v>16.1</v>
@@ -1770,7 +1770,7 @@
         <v>7.17</v>
       </c>
       <c r="H6" t="n">
-        <v>451687275</v>
+        <v>452317300</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -1788,7 +1788,7 @@
         <v>13.39</v>
       </c>
       <c r="N6" t="n">
-        <v>5.571791970304858</v>
+        <v>5.579563648699144</v>
       </c>
       <c r="O6" t="n">
         <v>1.24</v>
@@ -1866,7 +1866,7 @@
         <v>34696585</v>
       </c>
       <c r="AN6" t="n">
-        <v>48464299.89270386</v>
+        <v>48531899.1416309</v>
       </c>
       <c r="AO6" t="n">
         <v>0</v>
@@ -8804,7 +8804,7 @@
         <v>26</v>
       </c>
       <c r="H36" t="n">
-        <v>203582362</v>
+        <v>205849000</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
@@ -8822,7 +8822,7 @@
         <v>10.3</v>
       </c>
       <c r="N36" t="n">
-        <v>1.859741693683187</v>
+        <v>1.880447619047619</v>
       </c>
       <c r="O36" t="n">
         <v>0.85</v>
@@ -8900,7 +8900,7 @@
         <v>12348000</v>
       </c>
       <c r="AN36" t="n">
-        <v>36419027.19141324</v>
+        <v>36824508.05008945</v>
       </c>
       <c r="AO36" t="n">
         <v>0</v>
@@ -9039,7 +9039,7 @@
         <v>16.01</v>
       </c>
       <c r="H37" t="n">
-        <v>203582362</v>
+        <v>205849000</v>
       </c>
       <c r="I37" t="n">
         <v>300</v>
@@ -9057,7 +9057,7 @@
         <v>7.41</v>
       </c>
       <c r="N37" t="n">
-        <v>1.859741693683187</v>
+        <v>1.880447619047619</v>
       </c>
       <c r="O37" t="n">
         <v>0.61</v>
@@ -9135,7 +9135,7 @@
         <v>12348000</v>
       </c>
       <c r="AN37" t="n">
-        <v>50642378.60696518</v>
+        <v>51206218.90547264</v>
       </c>
       <c r="AO37" t="n">
         <v>0</v>
@@ -10684,7 +10684,7 @@
         <v>4.1</v>
       </c>
       <c r="H44" t="n">
-        <v>6089835</v>
+        <v>6063600</v>
       </c>
       <c r="I44" t="n">
         <v>100</v>
@@ -10702,7 +10702,7 @@
         <v>0.75</v>
       </c>
       <c r="N44" t="n">
-        <v>0.2721381522108287</v>
+        <v>0.2709657814613336</v>
       </c>
       <c r="O44" t="n">
         <v>0.03</v>
@@ -10780,7 +10780,7 @@
         <v>5719748.64</v>
       </c>
       <c r="AN44" t="n">
-        <v>6089835</v>
+        <v>6063600</v>
       </c>
       <c r="AO44" t="n">
         <v>0</v>
@@ -10919,7 +10919,7 @@
         <v>3.6</v>
       </c>
       <c r="H45" t="n">
-        <v>6089835</v>
+        <v>6063600</v>
       </c>
       <c r="I45" t="n">
         <v>100</v>
@@ -10937,7 +10937,7 @@
         <v>0.63</v>
       </c>
       <c r="N45" t="n">
-        <v>0.1664371247181705</v>
+        <v>0.165720113835777</v>
       </c>
       <c r="O45" t="n">
         <v>0.02</v>
@@ -11015,7 +11015,7 @@
         <v>9352251.359999999</v>
       </c>
       <c r="AN45" t="n">
-        <v>7249803.571428572</v>
+        <v>7218571.428571429</v>
       </c>
       <c r="AO45" t="n">
         <v>0</v>
@@ -11389,7 +11389,7 @@
         <v>8.74</v>
       </c>
       <c r="H47" t="n">
-        <v>3073862289</v>
+        <v>3074545000</v>
       </c>
       <c r="I47" t="n">
         <v>9800</v>
@@ -11407,7 +11407,7 @@
         <v>8.390000000000001</v>
       </c>
       <c r="N47" t="n">
-        <v>0.8245535169869331</v>
+        <v>0.8247366519823265</v>
       </c>
       <c r="O47" t="n">
         <v>0.07000000000000001</v>
@@ -11485,7 +11485,7 @@
         <v>249024468</v>
       </c>
       <c r="AN47" t="n">
-        <v>467863362.1004566</v>
+        <v>467967275.4946727</v>
       </c>
       <c r="AO47" t="n">
         <v>0.3403</v>
@@ -11624,7 +11624,7 @@
         <v>9.140000000000001</v>
       </c>
       <c r="H48" t="n">
-        <v>3073862289</v>
+        <v>3074545000</v>
       </c>
       <c r="I48" t="n">
         <v>2400</v>
@@ -11642,7 +11642,7 @@
         <v>8.449999999999999</v>
       </c>
       <c r="N48" t="n">
-        <v>2.243361840787464</v>
+        <v>2.243860095966678</v>
       </c>
       <c r="O48" t="n">
         <v>0.07000000000000001</v>
@@ -11720,7 +11720,7 @@
         <v>91529595.08</v>
       </c>
       <c r="AN48" t="n">
-        <v>464329650.9063444</v>
+        <v>464432779.4561933</v>
       </c>
       <c r="AO48" t="n">
         <v>0.3691</v>
@@ -11859,7 +11859,7 @@
         <v>47.3</v>
       </c>
       <c r="H49" t="n">
-        <v>922115500</v>
+        <v>923385000</v>
       </c>
       <c r="I49" t="n">
         <v>0</v>
@@ -11877,7 +11877,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="N49" t="n">
-        <v>1.006869904504318</v>
+        <v>1.008256088061332</v>
       </c>
       <c r="O49" t="n">
         <v>0.08</v>
@@ -11955,7 +11955,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN49" t="n">
-        <v>168576873.857404</v>
+        <v>168808957.952468</v>
       </c>
       <c r="AO49" t="n">
         <v>2.4346</v>
@@ -12094,7 +12094,7 @@
         <v>32.71</v>
       </c>
       <c r="H50" t="n">
-        <v>922115500</v>
+        <v>923385000</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>
@@ -12112,7 +12112,7 @@
         <v>5.78</v>
       </c>
       <c r="N50" t="n">
-        <v>1.006869904504318</v>
+        <v>1.008256088061332</v>
       </c>
       <c r="O50" t="n">
         <v>0.06</v>
@@ -12190,7 +12190,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN50" t="n">
-        <v>242025065.6167979</v>
+        <v>242358267.7165354</v>
       </c>
       <c r="AO50" t="n">
         <v>3.526</v>
@@ -12548,7 +12548,7 @@
         <v>7.19</v>
       </c>
       <c r="H52" t="n">
-        <v>200661972</v>
+        <v>191492700</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
@@ -13958,7 +13958,7 @@
         <v>21.49</v>
       </c>
       <c r="H58" t="n">
-        <v>91148030</v>
+        <v>84923520</v>
       </c>
       <c r="I58" t="n">
         <v>0</v>
@@ -13976,7 +13976,7 @@
         <v>13.78</v>
       </c>
       <c r="N58" t="n">
-        <v>1.692410201828114</v>
+        <v>1.576835304319291</v>
       </c>
       <c r="O58" t="n">
         <v>0.17</v>
@@ -14054,7 +14054,7 @@
         <v>6872145.189999999</v>
       </c>
       <c r="AN58" t="n">
-        <v>12947163.35227273</v>
+        <v>12063000</v>
       </c>
       <c r="AO58" t="n">
         <v>0</v>
@@ -14193,7 +14193,7 @@
         <v>17.6</v>
       </c>
       <c r="H59" t="n">
-        <v>91148030</v>
+        <v>84923520</v>
       </c>
       <c r="I59" t="n">
         <v>0</v>
@@ -14211,7 +14211,7 @@
         <v>12.47</v>
       </c>
       <c r="N59" t="n">
-        <v>9.806988800712238</v>
+        <v>9.137268348608981</v>
       </c>
       <c r="O59" t="n">
         <v>0.15</v>
@@ -14289,7 +14289,7 @@
         <v>1185938.81</v>
       </c>
       <c r="AN59" t="n">
-        <v>14308952.90423862</v>
+        <v>13331792.77864992</v>
       </c>
       <c r="AO59" t="n">
         <v>0</v>
@@ -14428,7 +14428,7 @@
         <v>377.21</v>
       </c>
       <c r="H60" t="n">
-        <v>171536281</v>
+        <v>171536300</v>
       </c>
       <c r="I60" t="n">
         <v>50</v>
@@ -14446,7 +14446,7 @@
         <v>2.87</v>
       </c>
       <c r="N60" t="n">
-        <v>12.12184028129253</v>
+        <v>12.12184162395289</v>
       </c>
       <c r="O60" t="n">
         <v>0.64</v>
@@ -14524,7 +14524,7 @@
         <v>59731412.5</v>
       </c>
       <c r="AN60" t="n">
-        <v>21604065.61712846</v>
+        <v>21604068.01007557</v>
       </c>
       <c r="AO60" t="n">
         <v>0</v>
@@ -14898,7 +14898,7 @@
         <v>116</v>
       </c>
       <c r="H62" t="n">
-        <v>11449169840</v>
+        <v>11449170000</v>
       </c>
       <c r="I62" t="n">
         <v>100</v>
@@ -14916,7 +14916,7 @@
         <v>4.26</v>
       </c>
       <c r="N62" t="n">
-        <v>1.170139753439905</v>
+        <v>1.170139769792389</v>
       </c>
       <c r="O62" t="n">
         <v>0.17</v>
@@ -14994,7 +14994,7 @@
         <v>2822812821.4</v>
       </c>
       <c r="AN62" t="n">
-        <v>4692282721.311476</v>
+        <v>4692282786.885246</v>
       </c>
       <c r="AO62" t="n">
         <v>0</v>
@@ -18893,7 +18893,7 @@
         <v>2.95</v>
       </c>
       <c r="H79" t="n">
-        <v>6308746201</v>
+        <v>6352498000</v>
       </c>
       <c r="I79" t="n">
         <v>2900</v>
@@ -18911,7 +18911,7 @@
         <v>2.47</v>
       </c>
       <c r="N79" t="n">
-        <v>0.8820829490908664</v>
+        <v>0.8882002843997163</v>
       </c>
       <c r="O79" t="n">
         <v>0.03</v>
@@ -18989,7 +18989,7 @@
         <v>531401092.4</v>
       </c>
       <c r="AN79" t="n">
-        <v>3823482546.060606</v>
+        <v>3849998787.878788</v>
       </c>
       <c r="AO79" t="n">
         <v>0</v>
@@ -19128,7 +19128,7 @@
         <v>3.04</v>
       </c>
       <c r="H80" t="n">
-        <v>6308746201</v>
+        <v>6352498000</v>
       </c>
       <c r="I80" t="n">
         <v>600</v>
@@ -19146,7 +19146,7 @@
         <v>3.36</v>
       </c>
       <c r="N80" t="n">
-        <v>1.700430503193706</v>
+        <v>1.712223162340052</v>
       </c>
       <c r="O80" t="n">
         <v>0.04</v>
@@ -19224,7 +19224,7 @@
         <v>275659512.02</v>
       </c>
       <c r="AN80" t="n">
-        <v>2803887200.444445</v>
+        <v>2823332444.444445</v>
       </c>
       <c r="AO80" t="n">
         <v>0</v>
@@ -19598,7 +19598,7 @@
         <v>9.33</v>
       </c>
       <c r="H82" t="n">
-        <v>384703200</v>
+        <v>394426500</v>
       </c>
       <c r="I82" t="n">
         <v>10500</v>
@@ -19616,7 +19616,7 @@
         <v>6.04</v>
       </c>
       <c r="N82" t="n">
-        <v>0.9782499287996614</v>
+        <v>1.002975009154329</v>
       </c>
       <c r="O82" t="n">
         <v>1.01</v>
@@ -19694,7 +19694,7 @@
         <v>65949124.8</v>
       </c>
       <c r="AN82" t="n">
-        <v>68452526.69039145</v>
+        <v>70182651.2455516</v>
       </c>
       <c r="AO82" t="n">
         <v>0</v>
@@ -21948,7 +21948,7 @@
         <v>9</v>
       </c>
       <c r="H92" t="n">
-        <v>82310150</v>
+        <v>78221290</v>
       </c>
       <c r="I92" t="n">
         <v>0</v>
@@ -21966,7 +21966,7 @@
         <v>3.42</v>
       </c>
       <c r="N92" t="n">
-        <v>0.1519817946743144</v>
+        <v>0.144431908287617</v>
       </c>
       <c r="O92" t="n">
         <v>0.15</v>
@@ -22044,7 +22044,7 @@
         <v>23342055.36</v>
       </c>
       <c r="AN92" t="n">
-        <v>58375992.90780142</v>
+        <v>55476092.19858156</v>
       </c>
       <c r="AO92" t="n">
         <v>0</v>
@@ -22183,7 +22183,7 @@
         <v>6.24</v>
       </c>
       <c r="H93" t="n">
-        <v>82310150</v>
+        <v>78221290</v>
       </c>
       <c r="I93" t="n">
         <v>300</v>
@@ -22201,7 +22201,7 @@
         <v>2.3</v>
       </c>
       <c r="N93" t="n">
-        <v>0.2020491314751064</v>
+        <v>0.192012087298619</v>
       </c>
       <c r="O93" t="n">
         <v>0.1</v>
@@ -22279,7 +22279,7 @@
         <v>17557944.64</v>
       </c>
       <c r="AN93" t="n">
-        <v>86642263.15789475</v>
+        <v>82338200</v>
       </c>
       <c r="AO93" t="n">
         <v>0</v>
@@ -22418,7 +22418,7 @@
         <v>46.51</v>
       </c>
       <c r="H94" t="n">
-        <v>8083066000</v>
+        <v>8158211000</v>
       </c>
       <c r="I94" t="n">
         <v>0</v>
@@ -22436,7 +22436,7 @@
         <v>5.78</v>
       </c>
       <c r="N94" t="n">
-        <v>0.7589350882089851</v>
+        <v>0.7659906012041116</v>
       </c>
       <c r="O94" t="n">
         <v>0.36</v>
@@ -22514,7 +22514,7 @@
         <v>1209900967.64</v>
       </c>
       <c r="AN94" t="n">
-        <v>2907577697.841727</v>
+        <v>2934608273.381295</v>
       </c>
       <c r="AO94" t="n">
         <v>0</v>
@@ -22653,7 +22653,7 @@
         <v>40</v>
       </c>
       <c r="H95" t="n">
-        <v>8083066000</v>
+        <v>8158211000</v>
       </c>
       <c r="I95" t="n">
         <v>0</v>
@@ -22671,7 +22671,7 @@
         <v>4.65</v>
       </c>
       <c r="N95" t="n">
-        <v>4.23791426810747</v>
+        <v>4.277312445442275</v>
       </c>
       <c r="O95" t="n">
         <v>0.29</v>
@@ -22749,7 +22749,7 @@
         <v>216671749.24</v>
       </c>
       <c r="AN95" t="n">
-        <v>3608511607.142857</v>
+        <v>3642058482.142857</v>
       </c>
       <c r="AO95" t="n">
         <v>0</v>
@@ -23593,7 +23593,7 @@
         <v>124.54</v>
       </c>
       <c r="H99" t="n">
-        <v>16504020750</v>
+        <v>16445650000</v>
       </c>
       <c r="I99" t="n">
         <v>200</v>
@@ -23611,7 +23611,7 @@
         <v>10.65</v>
       </c>
       <c r="N99" t="n">
-        <v>1.630701109134795</v>
+        <v>1.62493371171038</v>
       </c>
       <c r="O99" t="n">
         <v>1.16</v>
@@ -23689,7 +23689,7 @@
         <v>1267125769.6</v>
       </c>
       <c r="AN99" t="n">
-        <v>2840623192.771084</v>
+        <v>2830576592.082616</v>
       </c>
       <c r="AO99" t="n">
         <v>0</v>
@@ -23828,7 +23828,7 @@
         <v>122.5</v>
       </c>
       <c r="H100" t="n">
-        <v>16504020750</v>
+        <v>16445650000</v>
       </c>
       <c r="I100" t="n">
         <v>0</v>
@@ -23846,7 +23846,7 @@
         <v>10.81</v>
       </c>
       <c r="N100" t="n">
-        <v>5.910049574093893</v>
+        <v>5.889147150896379</v>
       </c>
       <c r="O100" t="n">
         <v>1.18</v>
@@ -23924,7 +23924,7 @@
         <v>349625391.8</v>
       </c>
       <c r="AN100" t="n">
-        <v>2797291652.542373</v>
+        <v>2787398305.084745</v>
       </c>
       <c r="AO100" t="n">
         <v>0</v>
@@ -24063,7 +24063,7 @@
         <v>24.06</v>
       </c>
       <c r="H101" t="n">
-        <v>626531054</v>
+        <v>621124300</v>
       </c>
       <c r="I101" t="n">
         <v>1100</v>
@@ -24081,7 +24081,7 @@
         <v>6.28</v>
       </c>
       <c r="N101" t="n">
-        <v>1.879534366064228</v>
+        <v>1.863314611453541</v>
       </c>
       <c r="O101" t="n">
         <v>0.49</v>
@@ -24159,7 +24159,7 @@
         <v>45834767.09999999</v>
       </c>
       <c r="AN101" t="n">
-        <v>64791215.51189245</v>
+        <v>64232088.93485005</v>
       </c>
       <c r="AO101" t="n">
         <v>0</v>
@@ -24298,7 +24298,7 @@
         <v>24.43</v>
       </c>
       <c r="H102" t="n">
-        <v>626531054</v>
+        <v>621124300</v>
       </c>
       <c r="I102" t="n">
         <v>600</v>
@@ -24316,7 +24316,7 @@
         <v>6.32</v>
       </c>
       <c r="N102" t="n">
-        <v>1.376550118543903</v>
+        <v>1.364670950205604</v>
       </c>
       <c r="O102" t="n">
         <v>0.49</v>
@@ -24394,7 +24394,7 @@
         <v>62582552.4</v>
       </c>
       <c r="AN102" t="n">
-        <v>64391680.78108941</v>
+        <v>63836002.05549846</v>
       </c>
       <c r="AO102" t="n">
         <v>0</v>
@@ -28769,7 +28769,7 @@
         <v>26200</v>
       </c>
       <c r="J121" t="n">
-        <v>26710356</v>
+        <v>8013000</v>
       </c>
       <c r="K121" t="n">
         <v>0</v>
@@ -28781,7 +28781,7 @@
         <v>0.19</v>
       </c>
       <c r="N121" t="n">
-        <v>1.3568301429254e-05</v>
+        <v>4.522827424069428e-05</v>
       </c>
       <c r="O121" t="n">
         <v>0.02</v>
@@ -28853,10 +28853,10 @@
         <v>0</v>
       </c>
       <c r="AL121" t="n">
-        <v>433068209.0634441</v>
+        <v>129918731.1178248</v>
       </c>
       <c r="AM121" t="n">
-        <v>129011019.48</v>
+        <v>38702790</v>
       </c>
       <c r="AN121" t="n">
         <v>1965.217391304348</v>
@@ -28936,7 +28936,7 @@
         <v>4.83</v>
       </c>
       <c r="BM121" t="n">
-        <v>-0.63</v>
+        <v>-2.13</v>
       </c>
       <c r="BN121" t="n">
         <v>1.24</v>
@@ -28998,7 +28998,7 @@
         <v>44</v>
       </c>
       <c r="H122" t="n">
-        <v>245203295</v>
+        <v>241942298</v>
       </c>
       <c r="I122" t="n">
         <v>0</v>
@@ -29016,7 +29016,7 @@
         <v>2.81</v>
       </c>
       <c r="N122" t="n">
-        <v>0.7021609750919887</v>
+        <v>0.6928228263803572</v>
       </c>
       <c r="O122" t="n">
         <v>0.43</v>
@@ -29094,7 +29094,7 @@
         <v>51264375.23999999</v>
       </c>
       <c r="AN122" t="n">
-        <v>71487841.10787171</v>
+        <v>70537113.11953352</v>
       </c>
       <c r="AO122" t="n">
         <v>0</v>
@@ -29233,7 +29233,7 @@
         <v>32.64</v>
       </c>
       <c r="H123" t="n">
-        <v>245203295</v>
+        <v>241942298</v>
       </c>
       <c r="I123" t="n">
         <v>1500</v>
@@ -29251,7 +29251,7 @@
         <v>2.69</v>
       </c>
       <c r="N123" t="n">
-        <v>0.6074904047401316</v>
+        <v>0.5994112947616692</v>
       </c>
       <c r="O123" t="n">
         <v>0.41</v>
@@ -29329,7 +29329,7 @@
         <v>59253353.51</v>
       </c>
       <c r="AN123" t="n">
-        <v>74304028.7878788</v>
+        <v>73315847.87878789</v>
       </c>
       <c r="AO123" t="n">
         <v>0</v>
@@ -32288,7 +32288,7 @@
         <v>6.51</v>
       </c>
       <c r="H136" t="n">
-        <v>430297600</v>
+        <v>431991800</v>
       </c>
       <c r="I136" t="n">
         <v>0</v>
@@ -32306,7 +32306,7 @@
         <v>89.8</v>
       </c>
       <c r="N136" t="n">
-        <v>1.004432824477173</v>
+        <v>1.008387552765756</v>
       </c>
       <c r="O136" t="n">
         <v>0.49</v>
@@ -32384,7 +32384,7 @@
         <v>3812747.4</v>
       </c>
       <c r="AN136" t="n">
-        <v>7274684.69991547</v>
+        <v>7303327.134404058</v>
       </c>
       <c r="AO136" t="n">
         <v>0</v>
@@ -32523,7 +32523,7 @@
         <v>3.74</v>
       </c>
       <c r="H137" t="n">
-        <v>430297600</v>
+        <v>431991800</v>
       </c>
       <c r="I137" t="n">
         <v>10200</v>
@@ -32541,7 +32541,7 @@
         <v>51.86</v>
       </c>
       <c r="N137" t="n">
-        <v>2.583371819323714</v>
+        <v>2.593543264705465</v>
       </c>
       <c r="O137" t="n">
         <v>0.29</v>
@@ -32619,7 +32619,7 @@
         <v>1482422.55</v>
       </c>
       <c r="AN137" t="n">
-        <v>12592847.52707053</v>
+        <v>12642429.03131402</v>
       </c>
       <c r="AO137" t="n">
         <v>0</v>
@@ -34106,7 +34106,7 @@
         <v>1.33</v>
       </c>
       <c r="BM143" t="n">
-        <v>1.05</v>
+        <v>0.79</v>
       </c>
       <c r="BN143" t="n">
         <v>7.12</v>
@@ -34121,7 +34121,7 @@
         <v>6.84</v>
       </c>
       <c r="BR143" t="n">
-        <v>6.61</v>
+        <v>8.83</v>
       </c>
       <c r="BS143" t="n">
         <v>6.85</v>
@@ -34873,7 +34873,7 @@
         <v>150</v>
       </c>
       <c r="H147" t="n">
-        <v>1347458593</v>
+        <v>1347459000</v>
       </c>
       <c r="I147" t="n">
         <v>0</v>
@@ -34891,7 +34891,7 @@
         <v>17.51</v>
       </c>
       <c r="N147" t="n">
-        <v>5.453992851539172</v>
+        <v>5.453994498918247</v>
       </c>
       <c r="O147" t="n">
         <v>2.27</v>
@@ -34969,7 +34969,7 @@
         <v>126024849.5</v>
       </c>
       <c r="AN147" t="n">
-        <v>67541784.11027569</v>
+        <v>67541804.5112782</v>
       </c>
       <c r="AO147" t="n">
         <v>0</v>
@@ -35108,7 +35108,7 @@
         <v>36.47</v>
       </c>
       <c r="H148" t="n">
-        <v>1347458593</v>
+        <v>1347459000</v>
       </c>
       <c r="I148" t="n">
         <v>100</v>
@@ -35126,7 +35126,7 @@
         <v>5.57</v>
       </c>
       <c r="N148" t="n">
-        <v>3.605968688516685</v>
+        <v>3.605969777699881</v>
       </c>
       <c r="O148" t="n">
         <v>0.72</v>
@@ -35204,7 +35204,7 @@
         <v>190611369</v>
       </c>
       <c r="AN148" t="n">
-        <v>212198203.6220472</v>
+        <v>212198267.7165354</v>
       </c>
       <c r="AO148" t="n">
         <v>0</v>
@@ -38633,7 +38633,7 @@
         <v>3.01</v>
       </c>
       <c r="H163" t="n">
-        <v>17271728</v>
+        <v>17271740</v>
       </c>
       <c r="I163" t="n">
         <v>0</v>
@@ -38651,7 +38651,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="N163" t="n">
-        <v>0.3218975024814018</v>
+        <v>0.3218977261283947</v>
       </c>
       <c r="O163" t="n">
         <v>0.07000000000000001</v>
@@ -38729,7 +38729,7 @@
         <v>8649345</v>
       </c>
       <c r="AN163" t="n">
-        <v>4317932</v>
+        <v>4317935</v>
       </c>
       <c r="AO163" t="n">
         <v>0</v>
@@ -38868,7 +38868,7 @@
         <v>1.7</v>
       </c>
       <c r="H164" t="n">
-        <v>17271728</v>
+        <v>17271740</v>
       </c>
       <c r="I164" t="n">
         <v>100</v>
@@ -38886,7 +38886,7 @@
         <v>1.51</v>
       </c>
       <c r="N164" t="n">
-        <v>0.01609487512407009</v>
+        <v>0.01609488630641974</v>
       </c>
       <c r="O164" t="n">
         <v>0.11</v>
@@ -38964,7 +38964,7 @@
         <v>172986900</v>
       </c>
       <c r="AN164" t="n">
-        <v>2690300.31152648</v>
+        <v>2690302.180685358</v>
       </c>
       <c r="AO164" t="n">
         <v>0</v>
@@ -40748,7 +40748,7 @@
         <v>3.45</v>
       </c>
       <c r="H172" t="n">
-        <v>185807653</v>
+        <v>185807600</v>
       </c>
       <c r="I172" t="n">
         <v>400</v>
@@ -40766,7 +40766,7 @@
         <v>0.38</v>
       </c>
       <c r="N172" t="n">
-        <v>0.04113908076689022</v>
+        <v>0.04113906903232899</v>
       </c>
       <c r="O172" t="n">
         <v>0.08</v>
@@ -40844,7 +40844,7 @@
         <v>640901679.6</v>
       </c>
       <c r="AN172" t="n">
-        <v>185807653</v>
+        <v>185807600</v>
       </c>
       <c r="AO172" t="n">
         <v>0</v>
@@ -42628,7 +42628,7 @@
         <v>34.99</v>
       </c>
       <c r="H180" t="n">
-        <v>3717936107</v>
+        <v>3493717000</v>
       </c>
       <c r="I180" t="n">
         <v>200</v>
@@ -42646,7 +42646,7 @@
         <v>12.71</v>
       </c>
       <c r="N180" t="n">
-        <v>9.083250392079581</v>
+        <v>8.535463062508486</v>
       </c>
       <c r="O180" t="n">
         <v>0.8</v>
@@ -42724,7 +42724,7 @@
         <v>84360399.48</v>
       </c>
       <c r="AN180" t="n">
-        <v>482222581.9714656</v>
+        <v>453140985.7328146</v>
       </c>
       <c r="AO180" t="n">
         <v>4.0605</v>
@@ -42863,7 +42863,7 @@
         <v>38</v>
       </c>
       <c r="H181" t="n">
-        <v>3717936107</v>
+        <v>3493717000</v>
       </c>
       <c r="I181" t="n">
         <v>400</v>
@@ -42881,7 +42881,7 @@
         <v>13.08</v>
       </c>
       <c r="N181" t="n">
-        <v>4.54162519603979</v>
+        <v>4.267731531254243</v>
       </c>
       <c r="O181" t="n">
         <v>0.83</v>
@@ -42959,7 +42959,7 @@
         <v>168720798.96</v>
       </c>
       <c r="AN181" t="n">
-        <v>468253917.7581864</v>
+        <v>440014735.5163728</v>
       </c>
       <c r="AO181" t="n">
         <v>4.0605</v>
@@ -45448,7 +45448,7 @@
         <v>2.5</v>
       </c>
       <c r="H192" t="n">
-        <v>21953007</v>
+        <v>22134000</v>
       </c>
       <c r="I192" t="n">
         <v>1400</v>
@@ -45466,7 +45466,7 @@
         <v>21.95</v>
       </c>
       <c r="N192" t="n">
-        <v>2.244494924832359</v>
+        <v>2.262999809831949</v>
       </c>
       <c r="O192" t="n">
         <v>0.32</v>
@@ -45544,7 +45544,7 @@
         <v>357000.03</v>
       </c>
       <c r="AN192" t="n">
-        <v>1846342.052144659</v>
+        <v>1861564.339781329</v>
       </c>
       <c r="AO192" t="n">
         <v>0</v>
@@ -45683,7 +45683,7 @@
         <v>1.54</v>
       </c>
       <c r="H193" t="n">
-        <v>21953007</v>
+        <v>22134000</v>
       </c>
       <c r="I193" t="n">
         <v>2200</v>
@@ -45701,7 +45701,7 @@
         <v>14.71</v>
       </c>
       <c r="N193" t="n">
-        <v>1.12224760387595</v>
+        <v>1.131500047542019</v>
       </c>
       <c r="O193" t="n">
         <v>0.22</v>
@@ -45779,7 +45779,7 @@
         <v>713999.97</v>
       </c>
       <c r="AN193" t="n">
-        <v>2754455.081555835</v>
+        <v>2777164.366373902</v>
       </c>
       <c r="AO193" t="n">
         <v>0</v>
@@ -47563,7 +47563,7 @@
         <v>6.66</v>
       </c>
       <c r="H201" t="n">
-        <v>122360247</v>
+        <v>122360300</v>
       </c>
       <c r="I201" t="n">
         <v>0</v>
@@ -47581,7 +47581,7 @@
         <v>1.99</v>
       </c>
       <c r="N201" t="n">
-        <v>1.444073637032944</v>
+        <v>1.444074262529416</v>
       </c>
       <c r="O201" t="n">
         <v>0.25</v>
@@ -47659,7 +47659,7 @@
         <v>28893848.04</v>
       </c>
       <c r="AN201" t="n">
-        <v>97111307.14285715</v>
+        <v>97111349.20634921</v>
       </c>
       <c r="AO201" t="n">
         <v>0</v>
@@ -48006,7 +48006,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>IBOVESPA</t>
+          <t>Brazil Stock Exchange Index</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
@@ -49192,7 +49192,7 @@
         <v>1.56</v>
       </c>
       <c r="H208" t="n">
-        <v>82225048</v>
+        <v>84610610</v>
       </c>
       <c r="I208" t="n">
         <v>106000</v>
@@ -49210,7 +49210,7 @@
         <v>0.16</v>
       </c>
       <c r="N208" t="n">
-        <v>23.8791919688837</v>
+        <v>24.5719892896183</v>
       </c>
       <c r="O208" t="n">
         <v>0.16</v>
@@ -49288,7 +49288,7 @@
         <v>364253793.28</v>
       </c>
       <c r="AN208" t="n">
-        <v>316250184.6153846</v>
+        <v>325425423.0769231</v>
       </c>
       <c r="AO208" t="n">
         <v>0</v>
@@ -49427,7 +49427,7 @@
         <v>1.54</v>
       </c>
       <c r="H209" t="n">
-        <v>82225048</v>
+        <v>84610610</v>
       </c>
       <c r="I209" t="n">
         <v>26500</v>
@@ -49445,7 +49445,7 @@
         <v>0.14</v>
       </c>
       <c r="N209" t="n">
-        <v>78.99490211815312</v>
+        <v>81.28674920453956</v>
       </c>
       <c r="O209" t="n">
         <v>0.13</v>
@@ -49523,7 +49523,7 @@
         <v>110109463.04</v>
       </c>
       <c r="AN209" t="n">
-        <v>373750218.1818182</v>
+        <v>384593681.8181818</v>
       </c>
       <c r="AO209" t="n">
         <v>0</v>
@@ -49835,7 +49835,7 @@
         <v>1.44</v>
       </c>
       <c r="BM210" t="n">
-        <v>1.76</v>
+        <v>1.82</v>
       </c>
       <c r="BN210" t="n">
         <v>14.68</v>
@@ -49850,7 +49850,7 @@
         <v>14.24</v>
       </c>
       <c r="BR210" t="n">
-        <v>8.34</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="BS210" t="n">
         <v>14.52</v>
@@ -51777,7 +51777,7 @@
         <v>0.54</v>
       </c>
       <c r="H219" t="n">
-        <v>6913479</v>
+        <v>6913480</v>
       </c>
       <c r="I219" t="n">
         <v>1900</v>
@@ -51795,7 +51795,7 @@
         <v>0.05</v>
       </c>
       <c r="N219" t="n">
-        <v>0.03132969048728561</v>
+        <v>0.03132969501896792</v>
       </c>
       <c r="O219" t="n">
         <v>0.02</v>
@@ -51873,7 +51873,7 @@
         <v>256438982.35</v>
       </c>
       <c r="AN219" t="n">
-        <v>115224650</v>
+        <v>115224666.6666667</v>
       </c>
       <c r="AO219" t="n">
         <v>0</v>
@@ -54603,7 +54603,7 @@
         <v>1267100</v>
       </c>
       <c r="J231" t="n">
-        <v>372555324</v>
+        <v>1609809601</v>
       </c>
       <c r="K231" t="n">
         <v>0</v>
@@ -54615,7 +54615,7 @@
         <v>0.8100000000000001</v>
       </c>
       <c r="N231" t="n">
-        <v>0.1333211806496342</v>
+        <v>0.03085427967514464</v>
       </c>
       <c r="O231" t="n">
         <v>0.07000000000000001</v>
@@ -54687,10 +54687,10 @@
         <v>11.57</v>
       </c>
       <c r="AL231" t="n">
-        <v>14941020806.25</v>
+        <v>64560072540.10417</v>
       </c>
       <c r="AM231" t="n">
-        <v>2294940795.84</v>
+        <v>9916427142.16</v>
       </c>
       <c r="AN231" t="n">
         <v>1443445314.492754</v>
@@ -56007,7 +56007,7 @@
         <v>0.64</v>
       </c>
       <c r="H237" t="n">
-        <v>26969413</v>
+        <v>26969420</v>
       </c>
       <c r="I237" t="n">
         <v>12600</v>
@@ -56025,7 +56025,7 @@
         <v>5.38</v>
       </c>
       <c r="N237" t="n">
-        <v>0.3886047499914101</v>
+        <v>0.3886048508550533</v>
       </c>
       <c r="O237" t="n">
         <v>0.11</v>
@@ -56103,7 +56103,7 @@
         <v>10271292.68</v>
       </c>
       <c r="AN237" t="n">
-        <v>2678193.942403178</v>
+        <v>2678194.637537239</v>
       </c>
       <c r="AO237" t="n">
         <v>0</v>
@@ -56242,7 +56242,7 @@
         <v>2.76</v>
       </c>
       <c r="H238" t="n">
-        <v>114727679</v>
+        <v>114727700</v>
       </c>
       <c r="I238" t="n">
         <v>200</v>
@@ -56260,7 +56260,7 @@
         <v>4.2</v>
       </c>
       <c r="N238" t="n">
-        <v>1.33957827403813</v>
+        <v>1.339578519237405</v>
       </c>
       <c r="O238" t="n">
         <v>0.75</v>
@@ -56338,7 +56338,7 @@
         <v>23184000</v>
       </c>
       <c r="AN238" t="n">
-        <v>16579144.36416185</v>
+        <v>16579147.39884393</v>
       </c>
       <c r="AO238" t="n">
         <v>0</v>
@@ -58357,7 +58357,7 @@
         <v>5.2</v>
       </c>
       <c r="H247" t="n">
-        <v>19323038</v>
+        <v>19323040</v>
       </c>
       <c r="I247" t="n">
         <v>0</v>
@@ -58375,7 +58375,7 @@
         <v>4.4</v>
       </c>
       <c r="N247" t="n">
-        <v>0.02907894616451322</v>
+        <v>0.02907894917428282</v>
       </c>
       <c r="O247" t="n">
         <v>0.05</v>
@@ -58453,7 +58453,7 @@
         <v>5648272.88</v>
       </c>
       <c r="AN247" t="n">
-        <v>32750911.86440678</v>
+        <v>32750915.25423729</v>
       </c>
       <c r="AO247" t="n">
         <v>0</v>
@@ -59767,7 +59767,7 @@
         <v>18.5</v>
       </c>
       <c r="H253" t="n">
-        <v>183539221</v>
+        <v>183539200</v>
       </c>
       <c r="I253" t="n">
         <v>0</v>
@@ -59785,7 +59785,7 @@
         <v>7.29</v>
       </c>
       <c r="N253" t="n">
-        <v>0.1834959159638325</v>
+        <v>0.1834958949687874</v>
       </c>
       <c r="O253" t="n">
         <v>0.12</v>
@@ -59863,7 +59863,7 @@
         <v>24405758.4</v>
       </c>
       <c r="AN253" t="n">
-        <v>126578773.1034483</v>
+        <v>126578758.6206897</v>
       </c>
       <c r="AO253" t="n">
         <v>0</v>
@@ -60410,7 +60410,7 @@
         <v>1.43</v>
       </c>
       <c r="BM255" t="n">
-        <v>1.67</v>
+        <v>1.93</v>
       </c>
       <c r="BN255" t="n">
         <v>15.13</v>
@@ -60425,7 +60425,7 @@
         <v>14.53</v>
       </c>
       <c r="BR255" t="n">
-        <v>8.83</v>
+        <v>7.66</v>
       </c>
       <c r="BS255" t="n">
         <v>15.13</v>
@@ -62995,7 +62995,7 @@
         <v>2.4</v>
       </c>
       <c r="BM266" t="n">
-        <v>2.5</v>
+        <v>2.83</v>
       </c>
       <c r="BN266" t="n">
         <v>29.12</v>
@@ -63010,7 +63010,7 @@
         <v>27.88</v>
       </c>
       <c r="BR266" t="n">
-        <v>11.27</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="BS266" t="n">
         <v>28.95</v>
@@ -64232,7 +64232,7 @@
         <v>1.44</v>
       </c>
       <c r="H272" t="n">
-        <v>9534943</v>
+        <v>9534940</v>
       </c>
       <c r="I272" t="n">
         <v>5700</v>
@@ -64250,7 +64250,7 @@
         <v>0.96</v>
       </c>
       <c r="N272" t="n">
-        <v>3.657048332410648</v>
+        <v>3.657047181785521</v>
       </c>
       <c r="O272" t="n">
         <v>1.87</v>
@@ -64328,7 +64328,7 @@
         <v>37941114.78</v>
       </c>
       <c r="AN272" t="n">
-        <v>8438002.654867258</v>
+        <v>8438000</v>
       </c>
       <c r="AO272" t="n">
         <v>0</v>
@@ -67287,7 +67287,7 @@
         <v>1.23</v>
       </c>
       <c r="H285" t="n">
-        <v>4043609</v>
+        <v>4043610</v>
       </c>
       <c r="I285" t="n">
         <v>7200</v>
@@ -67305,7 +67305,7 @@
         <v>0.05</v>
       </c>
       <c r="N285" t="n">
-        <v>0.04098945118940209</v>
+        <v>0.04098946132625043</v>
       </c>
       <c r="O285" t="n">
         <v>0.02</v>
@@ -67383,7 +67383,7 @@
         <v>178674864.1</v>
       </c>
       <c r="AN285" t="n">
-        <v>20218045</v>
+        <v>20218050</v>
       </c>
       <c r="AO285" t="n">
         <v>0</v>
@@ -71282,7 +71282,7 @@
         <v>41.65</v>
       </c>
       <c r="H302" t="n">
-        <v>260482</v>
+        <v>260480</v>
       </c>
       <c r="I302" t="n">
         <v>1</v>
@@ -71375,10 +71375,10 @@
         <v>0</v>
       </c>
       <c r="AM302" t="n">
-        <v>1713.810119086782</v>
+        <v>1713.796960326337</v>
       </c>
       <c r="AN302" t="n">
-        <v>1041928</v>
+        <v>1041920</v>
       </c>
       <c r="AO302" t="n">
         <v>0</v>
@@ -75042,7 +75042,7 @@
         <v>5.82</v>
       </c>
       <c r="H318" t="n">
-        <v>14946947720</v>
+        <v>14946950000</v>
       </c>
       <c r="I318" t="n">
         <v>100</v>
@@ -75060,7 +75060,7 @@
         <v>11.35</v>
       </c>
       <c r="N318" t="n">
-        <v>0.7703563146234507</v>
+        <v>0.7703564321332212</v>
       </c>
       <c r="O318" t="n">
         <v>0.49</v>
@@ -75138,7 +75138,7 @@
         <v>1412512331.45</v>
       </c>
       <c r="AN318" t="n">
-        <v>3306846840.707965</v>
+        <v>3306847345.132744</v>
       </c>
       <c r="AO318" t="n">
         <v>0</v>
@@ -76217,7 +76217,7 @@
         <v>6.51</v>
       </c>
       <c r="H323" t="n">
-        <v>558051800</v>
+        <v>553041900</v>
       </c>
       <c r="I323" t="n">
         <v>0</v>
@@ -76313,7 +76313,7 @@
         <v>8742210.08</v>
       </c>
       <c r="AN323" t="n">
-        <v>6407759.788724308</v>
+        <v>6350234.240440923</v>
       </c>
       <c r="AO323" t="n">
         <v>0</v>
@@ -76452,7 +76452,7 @@
         <v>6.65</v>
       </c>
       <c r="H324" t="n">
-        <v>558051800</v>
+        <v>553041900</v>
       </c>
       <c r="I324" t="n">
         <v>0</v>
@@ -76548,7 +76548,7 @@
         <v>2719637.39</v>
       </c>
       <c r="AN324" t="n">
-        <v>5507271.29181881</v>
+        <v>5457829.862824435</v>
       </c>
       <c r="AO324" t="n">
         <v>0.4906</v>
@@ -76687,7 +76687,7 @@
         <v>6.5</v>
       </c>
       <c r="H325" t="n">
-        <v>558051800</v>
+        <v>553041900</v>
       </c>
       <c r="I325" t="n">
         <v>0</v>
@@ -76783,7 +76783,7 @@
         <v>4627783.64</v>
       </c>
       <c r="AN325" t="n">
-        <v>8097095.182820661</v>
+        <v>8024403.656413233</v>
       </c>
       <c r="AO325" t="n">
         <v>0</v>
@@ -77800,7 +77800,7 @@
         <v>3.1</v>
       </c>
       <c r="BM329" t="n">
-        <v>3.38</v>
+        <v>3.63</v>
       </c>
       <c r="BN329" t="n">
         <v>28.75</v>
@@ -77815,7 +77815,7 @@
         <v>28.4</v>
       </c>
       <c r="BR329" t="n">
-        <v>8.470000000000001</v>
+        <v>7.87</v>
       </c>
       <c r="BS329" t="n">
         <v>28.75</v>
@@ -78035,7 +78035,7 @@
         <v>1.55</v>
       </c>
       <c r="BM330" t="n">
-        <v>3.38</v>
+        <v>3.63</v>
       </c>
       <c r="BN330" t="n">
         <v>14.7</v>
@@ -78050,7 +78050,7 @@
         <v>13.84</v>
       </c>
       <c r="BR330" t="n">
-        <v>4.28</v>
+        <v>3.98</v>
       </c>
       <c r="BS330" t="n">
         <v>14</v>
@@ -81857,7 +81857,7 @@
         <v>9.130000000000001</v>
       </c>
       <c r="H347" t="n">
-        <v>38292664</v>
+        <v>36846990</v>
       </c>
       <c r="I347" t="n">
         <v>0</v>
@@ -81875,7 +81875,7 @@
         <v>0.41</v>
       </c>
       <c r="N347" t="n">
-        <v>0.1126394773528269</v>
+        <v>0.1083869666426144</v>
       </c>
       <c r="O347" t="n">
         <v>0.15</v>
@@ -81953,7 +81953,7 @@
         <v>72003052.8</v>
       </c>
       <c r="AN347" t="n">
-        <v>42547404.44444444</v>
+        <v>40941100</v>
       </c>
       <c r="AO347" t="n">
         <v>0</v>
@@ -82092,7 +82092,7 @@
         <v>2.49</v>
       </c>
       <c r="H348" t="n">
-        <v>38292664</v>
+        <v>36846990</v>
       </c>
       <c r="I348" t="n">
         <v>700</v>
@@ -82110,7 +82110,7 @@
         <v>0.1</v>
       </c>
       <c r="N348" t="n">
-        <v>0.05925774494794938</v>
+        <v>0.05702057019380113</v>
       </c>
       <c r="O348" t="n">
         <v>0.04</v>
@@ -82188,7 +82188,7 @@
         <v>136866265.2</v>
       </c>
       <c r="AN348" t="n">
-        <v>166489843.4782609</v>
+        <v>160204304.3478261</v>
       </c>
       <c r="AO348" t="n">
         <v>0</v>
@@ -82327,7 +82327,7 @@
         <v>11.51</v>
       </c>
       <c r="H349" t="n">
-        <v>38292664</v>
+        <v>36846990</v>
       </c>
       <c r="I349" t="n">
         <v>0</v>
@@ -82345,7 +82345,7 @@
         <v>0.42</v>
       </c>
       <c r="N349" t="n">
-        <v>48.28818058800414</v>
+        <v>46.46514296431251</v>
       </c>
       <c r="O349" t="n">
         <v>0.15</v>
@@ -82423,7 +82423,7 @@
         <v>167958</v>
       </c>
       <c r="AN349" t="n">
-        <v>40308067.36842106</v>
+        <v>38786305.2631579</v>
       </c>
       <c r="AO349" t="n">
         <v>0</v>
@@ -85617,7 +85617,7 @@
         <v>10.59</v>
       </c>
       <c r="H363" t="n">
-        <v>1015916413</v>
+        <v>1021284000</v>
       </c>
       <c r="I363" t="n">
         <v>2100</v>
@@ -85635,7 +85635,7 @@
         <v>20.34</v>
       </c>
       <c r="N363" t="n">
-        <v>2.687495450968521</v>
+        <v>2.701694813692251</v>
       </c>
       <c r="O363" t="n">
         <v>0.27</v>
@@ -85713,7 +85713,7 @@
         <v>45966751.6</v>
       </c>
       <c r="AN363" t="n">
-        <v>108076214.1489362</v>
+        <v>108647234.0425532</v>
       </c>
       <c r="AO363" t="n">
         <v>0</v>
@@ -85852,7 +85852,7 @@
         <v>7.4</v>
       </c>
       <c r="H364" t="n">
-        <v>1015916413</v>
+        <v>1021284000</v>
       </c>
       <c r="I364" t="n">
         <v>100</v>
@@ -85870,7 +85870,7 @@
         <v>14.31</v>
       </c>
       <c r="N364" t="n">
-        <v>12.20209116552307</v>
+        <v>12.26656082569862</v>
       </c>
       <c r="O364" t="n">
         <v>0.19</v>
@@ -85948,7 +85948,7 @@
         <v>10124120.05</v>
       </c>
       <c r="AN364" t="n">
-        <v>153693859.7579425</v>
+        <v>154505900.1512859</v>
       </c>
       <c r="AO364" t="n">
         <v>0</v>
@@ -88907,7 +88907,7 @@
         <v>1.13</v>
       </c>
       <c r="H377" t="n">
-        <v>74677586</v>
+        <v>74677590</v>
       </c>
       <c r="I377" t="n">
         <v>3000</v>
@@ -88925,7 +88925,7 @@
         <v>39.8</v>
       </c>
       <c r="N377" t="n">
-        <v>0.2768499802773232</v>
+        <v>0.2768499951064035</v>
       </c>
       <c r="O377" t="n">
         <v>0.24</v>
@@ -89003,7 +89003,7 @@
         <v>2643454.56</v>
       </c>
       <c r="AN377" t="n">
-        <v>7051707.837582625</v>
+        <v>7051708.21529745</v>
       </c>
       <c r="AO377" t="n">
         <v>0</v>
@@ -90255,7 +90255,7 @@
         <v>2.66</v>
       </c>
       <c r="BM382" t="n">
-        <v>-2.12</v>
+        <v>-1.89</v>
       </c>
       <c r="BN382" t="n">
         <v>6.71</v>
@@ -90490,7 +90490,7 @@
         <v>2.66</v>
       </c>
       <c r="BM383" t="n">
-        <v>-2.12</v>
+        <v>-1.89</v>
       </c>
       <c r="BN383" t="n">
         <v>7.65</v>
@@ -90725,7 +90725,7 @@
         <v>2.66</v>
       </c>
       <c r="BM384" t="n">
-        <v>-2.12</v>
+        <v>-1.89</v>
       </c>
       <c r="BN384" t="n">
         <v>0</v>
@@ -90960,7 +90960,7 @@
         <v>6.65</v>
       </c>
       <c r="BM385" t="n">
-        <v>3.66</v>
+        <v>2.43</v>
       </c>
       <c r="BN385" t="n">
         <v>76.93000000000001</v>
@@ -90975,7 +90975,7 @@
         <v>75.23999999999999</v>
       </c>
       <c r="BR385" t="n">
-        <v>20.87</v>
+        <v>31.36</v>
       </c>
       <c r="BS385" t="n">
         <v>75.7</v>
@@ -92875,7 +92875,7 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>Vitru Brsl Emprndmnts Prtcpcs e Cmrc SA</t>
+          <t>Vitru Educacao SA</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
@@ -94077,7 +94077,7 @@
         <v>3.75</v>
       </c>
       <c r="H399" t="n">
-        <v>5887388000</v>
+        <v>5753969000</v>
       </c>
       <c r="I399" t="n">
         <v>5100</v>
@@ -94095,7 +94095,7 @@
         <v>9.42</v>
       </c>
       <c r="N399" t="n">
-        <v>0.6636394370415923</v>
+        <v>0.6486001513599535</v>
       </c>
       <c r="O399" t="n">
         <v>0.66</v>
@@ -94173,34 +94173,34 @@
         <v>483489419.2399999</v>
       </c>
       <c r="AN399" t="n">
-        <v>1130016890.59501</v>
+        <v>1104408637.236084</v>
       </c>
       <c r="AO399" t="n">
         <v>0</v>
       </c>
       <c r="AP399" t="n">
-        <v>0</v>
+        <v>0.6951000000000001</v>
       </c>
       <c r="AQ399" t="n">
-        <v>0</v>
+        <v>0.3795</v>
       </c>
       <c r="AR399" t="n">
-        <v>0</v>
+        <v>0.3404</v>
       </c>
       <c r="AS399" t="n">
-        <v>0</v>
+        <v>0.1871</v>
       </c>
       <c r="AT399" t="n">
-        <v>0</v>
+        <v>0.587</v>
       </c>
       <c r="AU399" t="n">
-        <v>0</v>
+        <v>1.2127</v>
       </c>
       <c r="AV399" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AW399" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX399" t="inlineStr">
         <is>
@@ -94220,7 +94220,7 @@
         <v>0.55</v>
       </c>
       <c r="BC399" t="n">
-        <v>0</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="BD399" t="n">
         <v>3.7</v>
@@ -94235,7 +94235,7 @@
         <v>-85.34</v>
       </c>
       <c r="BH399" t="n">
-        <v>-100</v>
+        <v>151.99</v>
       </c>
       <c r="BI399" t="n">
         <v>1.43</v>
@@ -94312,7 +94312,7 @@
         <v>4</v>
       </c>
       <c r="H400" t="n">
-        <v>5887388000</v>
+        <v>5753969000</v>
       </c>
       <c r="I400" t="n">
         <v>8300</v>
@@ -94330,7 +94330,7 @@
         <v>9.92</v>
       </c>
       <c r="N400" t="n">
-        <v>1.440008261577823</v>
+        <v>1.407375035731072</v>
       </c>
       <c r="O400" t="n">
         <v>0.6899999999999999</v>
@@ -94408,34 +94408,34 @@
         <v>222820003.58</v>
       </c>
       <c r="AN400" t="n">
-        <v>1074340875.912409</v>
+        <v>1049994343.065693</v>
       </c>
       <c r="AO400" t="n">
         <v>0</v>
       </c>
       <c r="AP400" t="n">
-        <v>0</v>
+        <v>0.7439</v>
       </c>
       <c r="AQ400" t="n">
-        <v>0</v>
+        <v>0.4159</v>
       </c>
       <c r="AR400" t="n">
-        <v>0</v>
+        <v>0.3745</v>
       </c>
       <c r="AS400" t="n">
-        <v>0</v>
+        <v>0.2058</v>
       </c>
       <c r="AT400" t="n">
-        <v>0</v>
+        <v>0.6457000000000001</v>
       </c>
       <c r="AU400" t="n">
-        <v>0</v>
+        <v>1.334</v>
       </c>
       <c r="AV400" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AW400" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX400" t="inlineStr">
         <is>
@@ -94455,7 +94455,7 @@
         <v>0.55</v>
       </c>
       <c r="BC400" t="n">
-        <v>0</v>
+        <v>10.33</v>
       </c>
       <c r="BD400" t="n">
         <v>-2.78</v>
@@ -94470,7 +94470,7 @@
         <v>-86.26000000000001</v>
       </c>
       <c r="BH400" t="n">
-        <v>-100</v>
+        <v>158.32</v>
       </c>
       <c r="BI400" t="n">
         <v>1.43</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-08-10 03:17
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1770,7 +1770,7 @@
         <v>7.1</v>
       </c>
       <c r="H6" t="n">
-        <v>447017900</v>
+        <v>445377100</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -1788,7 +1788,7 @@
         <v>13.39</v>
       </c>
       <c r="N6" t="n">
-        <v>5.514192857885004</v>
+        <v>5.493952756445626</v>
       </c>
       <c r="O6" t="n">
         <v>1.24</v>
@@ -1866,7 +1866,7 @@
         <v>34696585</v>
       </c>
       <c r="AN6" t="n">
-        <v>47963293.99141631</v>
+        <v>47787242.48927038</v>
       </c>
       <c r="AO6" t="n">
         <v>0</v>
@@ -2475,7 +2475,7 @@
         <v>23.89</v>
       </c>
       <c r="H9" t="n">
-        <v>208068994</v>
+        <v>207305200</v>
       </c>
       <c r="I9" t="n">
         <v>100</v>
@@ -2493,7 +2493,7 @@
         <v>2.59</v>
       </c>
       <c r="N9" t="n">
-        <v>0.3138195389077806</v>
+        <v>0.3126675485208778</v>
       </c>
       <c r="O9" t="n">
         <v>0.36</v>
@@ -2571,7 +2571,7 @@
         <v>81220091.82000001</v>
       </c>
       <c r="AN9" t="n">
-        <v>72497907.31707317</v>
+        <v>72231777.00348432</v>
       </c>
       <c r="AO9" t="n">
         <v>0</v>
@@ -2710,7 +2710,7 @@
         <v>58</v>
       </c>
       <c r="H10" t="n">
-        <v>208068994</v>
+        <v>207305200</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -2728,7 +2728,7 @@
         <v>6.01</v>
       </c>
       <c r="N10" t="n">
-        <v>58.60592784268432</v>
+        <v>58.3907931645656</v>
       </c>
       <c r="O10" t="n">
         <v>0.84</v>
@@ -2806,7 +2806,7 @@
         <v>434912.52</v>
       </c>
       <c r="AN10" t="n">
-        <v>31194751.72413793</v>
+        <v>31080239.88005997</v>
       </c>
       <c r="AO10" t="n">
         <v>0</v>
@@ -2945,7 +2945,7 @@
         <v>55</v>
       </c>
       <c r="H11" t="n">
-        <v>208068994</v>
+        <v>207305200</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -2963,7 +2963,7 @@
         <v>5.7</v>
       </c>
       <c r="N11" t="n">
-        <v>28.99671502097185</v>
+        <v>28.8902718814778</v>
       </c>
       <c r="O11" t="n">
         <v>0.79</v>
@@ -3041,7 +3041,7 @@
         <v>879011.7000000001</v>
       </c>
       <c r="AN11" t="n">
-        <v>32922309.17721519</v>
+        <v>32801455.69620253</v>
       </c>
       <c r="AO11" t="n">
         <v>0</v>
@@ -7394,7 +7394,7 @@
         <v>10.5</v>
       </c>
       <c r="H30" t="n">
-        <v>81876800</v>
+        <v>81576270</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
@@ -7412,7 +7412,7 @@
         <v>1.36</v>
       </c>
       <c r="N30" t="n">
-        <v>3.135197050946905</v>
+        <v>3.123689264007002</v>
       </c>
       <c r="O30" t="n">
         <v>0.12</v>
@@ -7490,7 +7490,7 @@
         <v>4766053.22</v>
       </c>
       <c r="AN30" t="n">
-        <v>63470387.59689923</v>
+        <v>63237418.60465116</v>
       </c>
       <c r="AO30" t="n">
         <v>0</v>
@@ -8804,7 +8804,7 @@
         <v>26</v>
       </c>
       <c r="H36" t="n">
-        <v>205394000</v>
+        <v>204640200</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
@@ -8822,7 +8822,7 @@
         <v>10.3</v>
       </c>
       <c r="N36" t="n">
-        <v>1.876291156462585</v>
+        <v>1.869405131195335</v>
       </c>
       <c r="O36" t="n">
         <v>0.85</v>
@@ -8900,7 +8900,7 @@
         <v>12348000</v>
       </c>
       <c r="AN36" t="n">
-        <v>36743112.70125224</v>
+        <v>36608264.75849732</v>
       </c>
       <c r="AO36" t="n">
         <v>0</v>
@@ -9039,7 +9039,7 @@
         <v>16</v>
       </c>
       <c r="H37" t="n">
-        <v>205394000</v>
+        <v>204640200</v>
       </c>
       <c r="I37" t="n">
         <v>0</v>
@@ -9057,7 +9057,7 @@
         <v>7.41</v>
       </c>
       <c r="N37" t="n">
-        <v>1.876291156462585</v>
+        <v>1.869405131195335</v>
       </c>
       <c r="O37" t="n">
         <v>0.61</v>
@@ -9135,7 +9135,7 @@
         <v>12348000</v>
       </c>
       <c r="AN37" t="n">
-        <v>51093034.82587066</v>
+        <v>50905522.38805971</v>
       </c>
       <c r="AO37" t="n">
         <v>0</v>
@@ -9274,7 +9274,7 @@
         <v>93.90000000000001</v>
       </c>
       <c r="H38" t="n">
-        <v>489399400</v>
+        <v>487603000</v>
       </c>
       <c r="I38" t="n">
         <v>0</v>
@@ -9292,7 +9292,7 @@
         <v>17.37</v>
       </c>
       <c r="N38" t="n">
-        <v>3.94744717593148</v>
+        <v>3.932957591132554</v>
       </c>
       <c r="O38" t="n">
         <v>2.37</v>
@@ -9370,7 +9370,7 @@
         <v>12707817.55</v>
       </c>
       <c r="AN38" t="n">
-        <v>21916677.11598746</v>
+        <v>21836229.28795343</v>
       </c>
       <c r="AO38" t="n">
         <v>0</v>
@@ -10684,7 +10684,7 @@
         <v>4.4</v>
       </c>
       <c r="H44" t="n">
-        <v>6194950</v>
+        <v>6111830</v>
       </c>
       <c r="I44" t="n">
         <v>300</v>
@@ -10702,7 +10702,7 @@
         <v>0.75</v>
       </c>
       <c r="N44" t="n">
-        <v>0.2768354554825332</v>
+        <v>0.2731210488997992</v>
       </c>
       <c r="O44" t="n">
         <v>0.03</v>
@@ -10780,7 +10780,7 @@
         <v>5719748.64</v>
       </c>
       <c r="AN44" t="n">
-        <v>6194950</v>
+        <v>6111830</v>
       </c>
       <c r="AO44" t="n">
         <v>0</v>
@@ -10919,7 +10919,7 @@
         <v>3.5</v>
       </c>
       <c r="H45" t="n">
-        <v>6194950</v>
+        <v>6111830</v>
       </c>
       <c r="I45" t="n">
         <v>0</v>
@@ -10937,7 +10937,7 @@
         <v>0.63</v>
       </c>
       <c r="N45" t="n">
-        <v>0.1693099510533258</v>
+        <v>0.1670382550539146</v>
       </c>
       <c r="O45" t="n">
         <v>0.02</v>
@@ -11015,7 +11015,7 @@
         <v>9352251.359999999</v>
       </c>
       <c r="AN45" t="n">
-        <v>7374940.476190477</v>
+        <v>7275988.095238095</v>
       </c>
       <c r="AO45" t="n">
         <v>0</v>
@@ -11859,7 +11859,7 @@
         <v>45.71</v>
       </c>
       <c r="H49" t="n">
-        <v>894368698</v>
+        <v>900623000</v>
       </c>
       <c r="I49" t="n">
         <v>1300</v>
@@ -11877,7 +11877,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="N49" t="n">
-        <v>0.9765728106152768</v>
+        <v>0.9834019642923174</v>
       </c>
       <c r="O49" t="n">
         <v>0.08</v>
@@ -11955,7 +11955,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN49" t="n">
-        <v>163504332.3583181</v>
+        <v>164647714.8080439</v>
       </c>
       <c r="AO49" t="n">
         <v>2.4346</v>
@@ -12094,7 +12094,7 @@
         <v>32.77</v>
       </c>
       <c r="H50" t="n">
-        <v>894368698</v>
+        <v>900623000</v>
       </c>
       <c r="I50" t="n">
         <v>700</v>
@@ -12112,7 +12112,7 @@
         <v>5.78</v>
       </c>
       <c r="N50" t="n">
-        <v>0.9765728106152768</v>
+        <v>0.9834019642923174</v>
       </c>
       <c r="O50" t="n">
         <v>0.06</v>
@@ -12190,7 +12190,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN50" t="n">
-        <v>234742440.4199475</v>
+        <v>236383989.5013123</v>
       </c>
       <c r="AO50" t="n">
         <v>3.526</v>
@@ -13958,7 +13958,7 @@
         <v>21.49</v>
       </c>
       <c r="H58" t="n">
-        <v>85719140</v>
+        <v>85404510</v>
       </c>
       <c r="I58" t="n">
         <v>0</v>
@@ -13976,7 +13976,7 @@
         <v>13.78</v>
       </c>
       <c r="N58" t="n">
-        <v>1.591608145869223</v>
+        <v>1.585766187224575</v>
       </c>
       <c r="O58" t="n">
         <v>0.17</v>
@@ -14054,7 +14054,7 @@
         <v>6872145.189999999</v>
       </c>
       <c r="AN58" t="n">
-        <v>12176014.20454546</v>
+        <v>12131322.44318182</v>
       </c>
       <c r="AO58" t="n">
         <v>0</v>
@@ -14193,7 +14193,7 @@
         <v>17.8</v>
       </c>
       <c r="H59" t="n">
-        <v>85719140</v>
+        <v>85404510</v>
       </c>
       <c r="I59" t="n">
         <v>0</v>
@@ -14211,7 +14211,7 @@
         <v>12.47</v>
       </c>
       <c r="N59" t="n">
-        <v>9.222872353759971</v>
+        <v>9.189020027095664</v>
       </c>
       <c r="O59" t="n">
         <v>0.15</v>
@@ -14289,7 +14289,7 @@
         <v>1185938.81</v>
       </c>
       <c r="AN59" t="n">
-        <v>13456693.87755102</v>
+        <v>13407301.41287284</v>
       </c>
       <c r="AO59" t="n">
         <v>0</v>
@@ -14428,7 +14428,7 @@
         <v>378.01</v>
       </c>
       <c r="H60" t="n">
-        <v>171560976</v>
+        <v>170931300</v>
       </c>
       <c r="I60" t="n">
         <v>29</v>
@@ -14446,7 +14446,7 @@
         <v>2.87</v>
       </c>
       <c r="N60" t="n">
-        <v>12.12358538643297</v>
+        <v>12.07908849133611</v>
       </c>
       <c r="O60" t="n">
         <v>0.64</v>
@@ -14524,7 +14524,7 @@
         <v>59731412.5</v>
       </c>
       <c r="AN60" t="n">
-        <v>21607175.8186398</v>
+        <v>21527871.53652393</v>
       </c>
       <c r="AO60" t="n">
         <v>0</v>
@@ -14898,7 +14898,7 @@
         <v>112.5</v>
       </c>
       <c r="H62" t="n">
-        <v>11081822625</v>
+        <v>11041140000</v>
       </c>
       <c r="I62" t="n">
         <v>100</v>
@@ -14916,7 +14916,7 @@
         <v>4.26</v>
       </c>
       <c r="N62" t="n">
-        <v>1.132595758059107</v>
+        <v>1.128437870854004</v>
       </c>
       <c r="O62" t="n">
         <v>0.17</v>
@@ -14994,7 +14994,7 @@
         <v>2822812821.4</v>
       </c>
       <c r="AN62" t="n">
-        <v>4541730584.016394</v>
+        <v>4525057377.04918</v>
       </c>
       <c r="AO62" t="n">
         <v>0</v>
@@ -16073,7 +16073,7 @@
         <v>180</v>
       </c>
       <c r="H67" t="n">
-        <v>1639077000</v>
+        <v>1633061000</v>
       </c>
       <c r="I67" t="n">
         <v>0</v>
@@ -16091,7 +16091,7 @@
         <v>4.43</v>
       </c>
       <c r="N67" t="n">
-        <v>0.4496880268878719</v>
+        <v>0.448037510670661</v>
       </c>
       <c r="O67" t="n">
         <v>0.06</v>
@@ -16169,7 +16169,7 @@
         <v>252228482.01</v>
       </c>
       <c r="AN67" t="n">
-        <v>593868478.2608696</v>
+        <v>591688768.1159421</v>
       </c>
       <c r="AO67" t="n">
         <v>0</v>
@@ -18893,7 +18893,7 @@
         <v>2.97</v>
       </c>
       <c r="H79" t="n">
-        <v>6361306441</v>
+        <v>6293936000</v>
       </c>
       <c r="I79" t="n">
         <v>46800</v>
@@ -18911,7 +18911,7 @@
         <v>2.47</v>
       </c>
       <c r="N79" t="n">
-        <v>0.8894318723201404</v>
+        <v>0.880012200742702</v>
       </c>
       <c r="O79" t="n">
         <v>0.03</v>
@@ -18989,7 +18989,7 @@
         <v>531401092.4</v>
       </c>
       <c r="AN79" t="n">
-        <v>3855337236.969697</v>
+        <v>3814506666.666667</v>
       </c>
       <c r="AO79" t="n">
         <v>0</v>
@@ -19128,7 +19128,7 @@
         <v>2.97</v>
       </c>
       <c r="H80" t="n">
-        <v>6361306441</v>
+        <v>6293936000</v>
       </c>
       <c r="I80" t="n">
         <v>24400</v>
@@ -19146,7 +19146,7 @@
         <v>3.36</v>
       </c>
       <c r="N80" t="n">
-        <v>1.714597349109462</v>
+        <v>1.696438629573106</v>
       </c>
       <c r="O80" t="n">
         <v>0.04</v>
@@ -19224,7 +19224,7 @@
         <v>275659512.02</v>
       </c>
       <c r="AN80" t="n">
-        <v>2827247307.111111</v>
+        <v>2797304888.888889</v>
       </c>
       <c r="AO80" t="n">
         <v>0</v>
@@ -19598,7 +19598,7 @@
         <v>8.6</v>
       </c>
       <c r="H82" t="n">
-        <v>365679400</v>
+        <v>361516700</v>
       </c>
       <c r="I82" t="n">
         <v>22300</v>
@@ -19616,7 +19616,7 @@
         <v>6.04</v>
       </c>
       <c r="N82" t="n">
-        <v>0.9298748931994923</v>
+        <v>0.9192896914683543</v>
       </c>
       <c r="O82" t="n">
         <v>1.01</v>
@@ -19694,7 +19694,7 @@
         <v>65949124.8</v>
       </c>
       <c r="AN82" t="n">
-        <v>65067508.89679715</v>
+        <v>64326814.94661921</v>
       </c>
       <c r="AO82" t="n">
         <v>0</v>
@@ -20773,7 +20773,7 @@
         <v>10.01</v>
       </c>
       <c r="H87" t="n">
-        <v>4527823000</v>
+        <v>4511204000</v>
       </c>
       <c r="I87" t="n">
         <v>0</v>
@@ -20791,7 +20791,7 @@
         <v>7.13</v>
       </c>
       <c r="N87" t="n">
-        <v>0.483122513213352</v>
+        <v>0.4813492519690206</v>
       </c>
       <c r="O87" t="n">
         <v>0.21</v>
@@ -20869,7 +20869,7 @@
         <v>580126647.04</v>
       </c>
       <c r="AN87" t="n">
-        <v>824740072.8597449</v>
+        <v>821712932.6047359</v>
       </c>
       <c r="AO87" t="n">
         <v>0</v>
@@ -21243,7 +21243,7 @@
         <v>24</v>
       </c>
       <c r="H89" t="n">
-        <v>1842702000</v>
+        <v>1810076000</v>
       </c>
       <c r="I89" t="n">
         <v>4800</v>
@@ -21261,7 +21261,7 @@
         <v>11.38</v>
       </c>
       <c r="N89" t="n">
-        <v>7.714047468250307</v>
+        <v>7.577466234443031</v>
       </c>
       <c r="O89" t="n">
         <v>1.53</v>
@@ -21339,7 +21339,7 @@
         <v>95908776.3</v>
       </c>
       <c r="AN89" t="n">
-        <v>200948964.0130861</v>
+        <v>197391057.7971647</v>
       </c>
       <c r="AO89" t="n">
         <v>0</v>
@@ -21478,7 +21478,7 @@
         <v>23.79</v>
       </c>
       <c r="H90" t="n">
-        <v>1842702000</v>
+        <v>1810076000</v>
       </c>
       <c r="I90" t="n">
         <v>5600</v>
@@ -21496,7 +21496,7 @@
         <v>10.59</v>
       </c>
       <c r="N90" t="n">
-        <v>42.20792513062398</v>
+        <v>41.4606118019839</v>
       </c>
       <c r="O90" t="n">
         <v>1.42</v>
@@ -21574,7 +21574,7 @@
         <v>17528576.7</v>
       </c>
       <c r="AN90" t="n">
-        <v>216026025.7913248</v>
+        <v>212201172.3329426</v>
       </c>
       <c r="AO90" t="n">
         <v>0</v>
@@ -21713,7 +21713,7 @@
         <v>27.1</v>
       </c>
       <c r="H91" t="n">
-        <v>1842702000</v>
+        <v>1810076000</v>
       </c>
       <c r="I91" t="n">
         <v>1300</v>
@@ -21731,7 +21731,7 @@
         <v>11.3</v>
       </c>
       <c r="N91" t="n">
-        <v>9.362593259997933</v>
+        <v>9.196823663122968</v>
       </c>
       <c r="O91" t="n">
         <v>1.52</v>
@@ -21809,7 +21809,7 @@
         <v>79021360.05</v>
       </c>
       <c r="AN91" t="n">
-        <v>202494725.2747253</v>
+        <v>198909450.5494505</v>
       </c>
       <c r="AO91" t="n">
         <v>0</v>
@@ -21948,7 +21948,7 @@
         <v>9</v>
       </c>
       <c r="H92" t="n">
-        <v>78066990</v>
+        <v>72773080</v>
       </c>
       <c r="I92" t="n">
         <v>0</v>
@@ -21966,7 +21966,7 @@
         <v>3.42</v>
       </c>
       <c r="N92" t="n">
-        <v>0.1441470006435629</v>
+        <v>0.1343720464897398</v>
       </c>
       <c r="O92" t="n">
         <v>0.15</v>
@@ -22044,7 +22044,7 @@
         <v>23342055.36</v>
       </c>
       <c r="AN92" t="n">
-        <v>55366659.57446809</v>
+        <v>51612113.47517731</v>
       </c>
       <c r="AO92" t="n">
         <v>0</v>
@@ -22183,7 +22183,7 @@
         <v>5.07</v>
       </c>
       <c r="H93" t="n">
-        <v>78066990</v>
+        <v>72773080</v>
       </c>
       <c r="I93" t="n">
         <v>2500</v>
@@ -22201,7 +22201,7 @@
         <v>2.3</v>
       </c>
       <c r="N93" t="n">
-        <v>0.1916333225777844</v>
+        <v>0.178638206937643</v>
       </c>
       <c r="O93" t="n">
         <v>0.1</v>
@@ -22279,7 +22279,7 @@
         <v>17557944.64</v>
       </c>
       <c r="AN93" t="n">
-        <v>82175778.94736843</v>
+        <v>76603242.10526316</v>
       </c>
       <c r="AO93" t="n">
         <v>0</v>
@@ -22418,7 +22418,7 @@
         <v>46</v>
       </c>
       <c r="H94" t="n">
-        <v>8064753000</v>
+        <v>8035152000</v>
       </c>
       <c r="I94" t="n">
         <v>0</v>
@@ -22436,7 +22436,7 @@
         <v>5.78</v>
       </c>
       <c r="N94" t="n">
-        <v>0.7572156443407337</v>
+        <v>0.7544363477785043</v>
       </c>
       <c r="O94" t="n">
         <v>0.36</v>
@@ -22514,7 +22514,7 @@
         <v>1209900967.64</v>
       </c>
       <c r="AN94" t="n">
-        <v>2900990287.769784</v>
+        <v>2890342446.043166</v>
       </c>
       <c r="AO94" t="n">
         <v>0</v>
@@ -22653,7 +22653,7 @@
         <v>40</v>
       </c>
       <c r="H95" t="n">
-        <v>8064753000</v>
+        <v>8035152000</v>
       </c>
       <c r="I95" t="n">
         <v>0</v>
@@ -22671,7 +22671,7 @@
         <v>4.65</v>
       </c>
       <c r="N95" t="n">
-        <v>4.228312846568682</v>
+        <v>4.212793178629529</v>
       </c>
       <c r="O95" t="n">
         <v>0.29</v>
@@ -22749,7 +22749,7 @@
         <v>216671749.24</v>
       </c>
       <c r="AN95" t="n">
-        <v>3600336160.714285</v>
+        <v>3587121428.571428</v>
       </c>
       <c r="AO95" t="n">
         <v>0</v>
@@ -23358,7 +23358,7 @@
         <v>29.99</v>
       </c>
       <c r="H98" t="n">
-        <v>7771176000</v>
+        <v>7742652000</v>
       </c>
       <c r="I98" t="n">
         <v>0</v>
@@ -23376,7 +23376,7 @@
         <v>24.76</v>
       </c>
       <c r="N98" t="n">
-        <v>1.577436281019349</v>
+        <v>1.571646321754522</v>
       </c>
       <c r="O98" t="n">
         <v>3.06</v>
@@ -23454,7 +23454,7 @@
         <v>576395765.0400001</v>
       </c>
       <c r="AN98" t="n">
-        <v>540040027.7970812</v>
+        <v>538057817.9291174</v>
       </c>
       <c r="AO98" t="n">
         <v>0</v>
@@ -23593,7 +23593,7 @@
         <v>124.6</v>
       </c>
       <c r="H99" t="n">
-        <v>16288275050</v>
+        <v>16337790000</v>
       </c>
       <c r="I99" t="n">
         <v>100</v>
@@ -23611,7 +23611,7 @@
         <v>10.65</v>
       </c>
       <c r="N99" t="n">
-        <v>1.609384076297141</v>
+        <v>1.614276464952418</v>
       </c>
       <c r="O99" t="n">
         <v>1.16</v>
@@ -23689,7 +23689,7 @@
         <v>1267125769.6</v>
       </c>
       <c r="AN99" t="n">
-        <v>2803489681.583477</v>
+        <v>2812012048.192771</v>
       </c>
       <c r="AO99" t="n">
         <v>0</v>
@@ -23828,7 +23828,7 @@
         <v>121.75</v>
       </c>
       <c r="H100" t="n">
-        <v>16288275050</v>
+        <v>16337790000</v>
       </c>
       <c r="I100" t="n">
         <v>300</v>
@@ -23846,7 +23846,7 @@
         <v>10.81</v>
       </c>
       <c r="N100" t="n">
-        <v>5.832791565169154</v>
+        <v>5.850522747987666</v>
       </c>
       <c r="O100" t="n">
         <v>1.18</v>
@@ -23924,7 +23924,7 @@
         <v>349625391.8</v>
       </c>
       <c r="AN100" t="n">
-        <v>2760724584.745762</v>
+        <v>2769116949.152542</v>
       </c>
       <c r="AO100" t="n">
         <v>0</v>
@@ -24063,7 +24063,7 @@
         <v>24.18</v>
       </c>
       <c r="H101" t="n">
-        <v>623502041</v>
+        <v>618319400</v>
       </c>
       <c r="I101" t="n">
         <v>4000</v>
@@ -24081,7 +24081,7 @@
         <v>6.28</v>
       </c>
       <c r="N101" t="n">
-        <v>1.870447611317742</v>
+        <v>1.854900174675482</v>
       </c>
       <c r="O101" t="n">
         <v>0.49</v>
@@ -24159,7 +24159,7 @@
         <v>45834767.09999999</v>
       </c>
       <c r="AN101" t="n">
-        <v>64477977.35263702</v>
+        <v>63942026.88728025</v>
       </c>
       <c r="AO101" t="n">
         <v>0</v>
@@ -24298,7 +24298,7 @@
         <v>24.39</v>
       </c>
       <c r="H102" t="n">
-        <v>623502041</v>
+        <v>618319400</v>
       </c>
       <c r="I102" t="n">
         <v>1800</v>
@@ -24316,7 +24316,7 @@
         <v>6.32</v>
       </c>
       <c r="N102" t="n">
-        <v>1.369895080174135</v>
+        <v>1.358508310057357</v>
       </c>
       <c r="O102" t="n">
         <v>0.49</v>
@@ -24394,7 +24394,7 @@
         <v>62582552.4</v>
       </c>
       <c r="AN102" t="n">
-        <v>64080374.20349435</v>
+        <v>63547728.67420349</v>
       </c>
       <c r="AO102" t="n">
         <v>0</v>
@@ -26883,7 +26883,7 @@
         <v>17</v>
       </c>
       <c r="H113" t="n">
-        <v>368796570</v>
+        <v>376142900</v>
       </c>
       <c r="I113" t="n">
         <v>0</v>
@@ -26901,7 +26901,7 @@
         <v>20.65</v>
       </c>
       <c r="N113" t="n">
-        <v>1.382199206313047</v>
+        <v>1.409732248432484</v>
       </c>
       <c r="O113" t="n">
         <v>0.54</v>
@@ -26979,7 +26979,7 @@
         <v>8431470.34</v>
       </c>
       <c r="AN113" t="n">
-        <v>27338515.19644181</v>
+        <v>27883091.17865085</v>
       </c>
       <c r="AO113" t="n">
         <v>0</v>
@@ -27118,7 +27118,7 @@
         <v>10.8</v>
       </c>
       <c r="H114" t="n">
-        <v>368796570</v>
+        <v>376142900</v>
       </c>
       <c r="I114" t="n">
         <v>5500</v>
@@ -27136,7 +27136,7 @@
         <v>23.27</v>
       </c>
       <c r="N114" t="n">
-        <v>1.137632385067607</v>
+        <v>1.160293720880447</v>
       </c>
       <c r="O114" t="n">
         <v>0.61</v>
@@ -27214,7 +27214,7 @@
         <v>10244057.54</v>
       </c>
       <c r="AN114" t="n">
-        <v>24278905.20079</v>
+        <v>24762534.56221198</v>
       </c>
       <c r="AO114" t="n">
         <v>0</v>
@@ -27353,7 +27353,7 @@
         <v>11.09</v>
       </c>
       <c r="H115" t="n">
-        <v>368796570</v>
+        <v>376142900</v>
       </c>
       <c r="I115" t="n">
         <v>0</v>
@@ -27371,7 +27371,7 @@
         <v>22.56</v>
       </c>
       <c r="N115" t="n">
-        <v>2.154140924113144</v>
+        <v>2.197050840805265</v>
       </c>
       <c r="O115" t="n">
         <v>0.59</v>
@@ -27449,7 +27449,7 @@
         <v>5410032.13</v>
       </c>
       <c r="AN115" t="n">
-        <v>25037105.90631365</v>
+        <v>25535838.42498303</v>
       </c>
       <c r="AO115" t="n">
         <v>0</v>
@@ -28763,7 +28763,7 @@
         <v>1.81</v>
       </c>
       <c r="H121" t="n">
-        <v>14503530</v>
+        <v>14421790</v>
       </c>
       <c r="I121" t="n">
         <v>0</v>
@@ -28781,7 +28781,7 @@
         <v>0.19</v>
       </c>
       <c r="N121" t="n">
-        <v>0.1116354037267081</v>
+        <v>0.1110062411779616</v>
       </c>
       <c r="O121" t="n">
         <v>0.02</v>
@@ -28859,7 +28859,7 @@
         <v>38702790</v>
       </c>
       <c r="AN121" t="n">
-        <v>4850678.929765886</v>
+        <v>4823341.137123746</v>
       </c>
       <c r="AO121" t="n">
         <v>0</v>
@@ -32288,7 +32288,7 @@
         <v>6.51</v>
       </c>
       <c r="H136" t="n">
-        <v>431351100</v>
+        <v>429767800</v>
       </c>
       <c r="I136" t="n">
         <v>0</v>
@@ -32306,7 +32306,7 @@
         <v>89.8</v>
       </c>
       <c r="N136" t="n">
-        <v>1.006891982930734</v>
+        <v>1.003196125712393</v>
       </c>
       <c r="O136" t="n">
         <v>0.49</v>
@@ -32384,7 +32384,7 @@
         <v>3812747.4</v>
       </c>
       <c r="AN136" t="n">
-        <v>7292495.350803044</v>
+        <v>7265727.810650888</v>
       </c>
       <c r="AO136" t="n">
         <v>0</v>
@@ -32523,7 +32523,7 @@
         <v>3.75</v>
       </c>
       <c r="H137" t="n">
-        <v>431351100</v>
+        <v>429767800</v>
       </c>
       <c r="I137" t="n">
         <v>0</v>
@@ -32541,7 +32541,7 @@
         <v>51.86</v>
       </c>
       <c r="N137" t="n">
-        <v>2.58969670287328</v>
+        <v>2.580191066305622</v>
       </c>
       <c r="O137" t="n">
         <v>0.29</v>
@@ -32619,7 +32619,7 @@
         <v>1482422.55</v>
       </c>
       <c r="AN137" t="n">
-        <v>12623678.66549605</v>
+        <v>12577342.69827334</v>
       </c>
       <c r="AO137" t="n">
         <v>0</v>
@@ -32993,7 +32993,7 @@
         <v>2.3</v>
       </c>
       <c r="H139" t="n">
-        <v>24516640</v>
+        <v>24426650</v>
       </c>
       <c r="I139" t="n">
         <v>0</v>
@@ -33011,7 +33011,7 @@
         <v>186.65</v>
       </c>
       <c r="N139" t="n">
-        <v>4.545017207098259</v>
+        <v>4.528334411312754</v>
       </c>
       <c r="O139" t="n">
         <v>4.19</v>
@@ -33089,7 +33089,7 @@
         <v>106804.76</v>
       </c>
       <c r="AN139" t="n">
-        <v>99313.94312565826</v>
+        <v>98949.404520781</v>
       </c>
       <c r="AO139" t="n">
         <v>0</v>
@@ -34403,7 +34403,7 @@
         <v>51.52</v>
       </c>
       <c r="H145" t="n">
-        <v>8608097000</v>
+        <v>8565357000</v>
       </c>
       <c r="I145" t="n">
         <v>0</v>
@@ -34421,7 +34421,7 @@
         <v>10.18</v>
       </c>
       <c r="N145" t="n">
-        <v>1.860086901571234</v>
+        <v>1.850851397583169</v>
       </c>
       <c r="O145" t="n">
         <v>0.73</v>
@@ -34499,7 +34499,7 @@
         <v>441028665.6</v>
       </c>
       <c r="AN145" t="n">
-        <v>1978872873.563219</v>
+        <v>1969047586.206897</v>
       </c>
       <c r="AO145" t="n">
         <v>0</v>
@@ -34638,7 +34638,7 @@
         <v>38.2</v>
       </c>
       <c r="H146" t="n">
-        <v>8608097000</v>
+        <v>8565357000</v>
       </c>
       <c r="I146" t="n">
         <v>400</v>
@@ -34656,7 +34656,7 @@
         <v>8.16</v>
       </c>
       <c r="N146" t="n">
-        <v>1.67755649891811</v>
+        <v>1.669227275308784</v>
       </c>
       <c r="O146" t="n">
         <v>0.58</v>
@@ -34734,7 +34734,7 @@
         <v>489015806.4</v>
       </c>
       <c r="AN146" t="n">
-        <v>2466503438.395415</v>
+        <v>2454257020.057306</v>
       </c>
       <c r="AO146" t="n">
         <v>0</v>
@@ -37223,7 +37223,7 @@
         <v>5.32</v>
       </c>
       <c r="H157" t="n">
-        <v>40659710</v>
+        <v>40510470</v>
       </c>
       <c r="I157" t="n">
         <v>8300</v>
@@ -37241,7 +37241,7 @@
         <v>8.27</v>
       </c>
       <c r="N157" t="n">
-        <v>0.003405798357736964</v>
+        <v>0.003393297497624862</v>
       </c>
       <c r="O157" t="n">
         <v>0.62</v>
@@ -37319,7 +37319,7 @@
         <v>1653465426.75</v>
       </c>
       <c r="AN157" t="n">
-        <v>6799282.608695651</v>
+        <v>6774326.086956521</v>
       </c>
       <c r="AO157" t="n">
         <v>0</v>
@@ -37458,7 +37458,7 @@
         <v>10.5</v>
       </c>
       <c r="H158" t="n">
-        <v>40659710</v>
+        <v>40510470</v>
       </c>
       <c r="I158" t="n">
         <v>0</v>
@@ -37476,7 +37476,7 @@
         <v>14.74</v>
       </c>
       <c r="N158" t="n">
-        <v>3.465219526408026</v>
+        <v>3.452500563038117</v>
       </c>
       <c r="O158" t="n">
         <v>1.1</v>
@@ -37554,7 +37554,7 @@
         <v>1625112</v>
       </c>
       <c r="AN158" t="n">
-        <v>3817813.145539906</v>
+        <v>3803800</v>
       </c>
       <c r="AO158" t="n">
         <v>0</v>
@@ -37693,7 +37693,7 @@
         <v>6.59</v>
       </c>
       <c r="H159" t="n">
-        <v>40659710</v>
+        <v>40510470</v>
       </c>
       <c r="I159" t="n">
         <v>0</v>
@@ -37711,7 +37711,7 @@
         <v>8.83</v>
       </c>
       <c r="N159" t="n">
-        <v>6.917891925940052</v>
+        <v>6.892500052977178</v>
       </c>
       <c r="O159" t="n">
         <v>0.66</v>
@@ -37789,7 +37789,7 @@
         <v>814029.75</v>
       </c>
       <c r="AN159" t="n">
-        <v>6372995.297805643</v>
+        <v>6349603.448275862</v>
       </c>
       <c r="AO159" t="n">
         <v>0</v>
@@ -37928,7 +37928,7 @@
         <v>10</v>
       </c>
       <c r="H160" t="n">
-        <v>40659710</v>
+        <v>40510470</v>
       </c>
       <c r="I160" t="n">
         <v>0</v>
@@ -37946,7 +37946,7 @@
         <v>13.4</v>
       </c>
       <c r="N160" t="n">
-        <v>6.250571790972007</v>
+        <v>6.227629292511376</v>
       </c>
       <c r="O160" t="n">
         <v>1</v>
@@ -38024,7 +38024,7 @@
         <v>900936.75</v>
       </c>
       <c r="AN160" t="n">
-        <v>4200383.26446281</v>
+        <v>4184965.909090909</v>
       </c>
       <c r="AO160" t="n">
         <v>0</v>
@@ -38633,7 +38633,7 @@
         <v>3.01</v>
       </c>
       <c r="H163" t="n">
-        <v>17775510</v>
+        <v>17710270</v>
       </c>
       <c r="I163" t="n">
         <v>0</v>
@@ -38651,7 +38651,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="N163" t="n">
-        <v>0.331286613263779</v>
+        <v>0.3300707191122565</v>
       </c>
       <c r="O163" t="n">
         <v>0.07000000000000001</v>
@@ -38729,7 +38729,7 @@
         <v>8649345</v>
       </c>
       <c r="AN163" t="n">
-        <v>4443877.5</v>
+        <v>4427567.5</v>
       </c>
       <c r="AO163" t="n">
         <v>0</v>
@@ -38868,7 +38868,7 @@
         <v>1.8</v>
       </c>
       <c r="H164" t="n">
-        <v>17775510</v>
+        <v>17710270</v>
       </c>
       <c r="I164" t="n">
         <v>0</v>
@@ -38886,7 +38886,7 @@
         <v>1.51</v>
       </c>
       <c r="N164" t="n">
-        <v>0.01656433066318895</v>
+        <v>0.01650353595561282</v>
       </c>
       <c r="O164" t="n">
         <v>0.11</v>
@@ -38964,7 +38964,7 @@
         <v>172986900</v>
       </c>
       <c r="AN164" t="n">
-        <v>2768771.028037383</v>
+        <v>2758609.034267913</v>
       </c>
       <c r="AO164" t="n">
         <v>0</v>
@@ -39103,7 +39103,7 @@
         <v>3.54</v>
       </c>
       <c r="H165" t="n">
-        <v>218257671</v>
+        <v>217456600</v>
       </c>
       <c r="I165" t="n">
         <v>83900</v>
@@ -39121,7 +39121,7 @@
         <v>5.28</v>
       </c>
       <c r="N165" t="n">
-        <v>0.1868779884821356</v>
+        <v>0.1861920903122089</v>
       </c>
       <c r="O165" t="n">
         <v>0.18</v>
@@ -39199,7 +39199,7 @@
         <v>46950197</v>
       </c>
       <c r="AN165" t="n">
-        <v>24277827.6974416</v>
+        <v>24188720.80088988</v>
       </c>
       <c r="AO165" t="n">
         <v>0</v>
@@ -40748,7 +40748,7 @@
         <v>3.27</v>
       </c>
       <c r="H172" t="n">
-        <v>175765932</v>
+        <v>175120800</v>
       </c>
       <c r="I172" t="n">
         <v>3600</v>
@@ -40766,7 +40766,7 @@
         <v>0.38</v>
       </c>
       <c r="N172" t="n">
-        <v>0.03891577529702576</v>
+        <v>0.03877293867525698</v>
       </c>
       <c r="O172" t="n">
         <v>0.08</v>
@@ -40844,7 +40844,7 @@
         <v>640901679.6</v>
       </c>
       <c r="AN172" t="n">
-        <v>175765932</v>
+        <v>175120800</v>
       </c>
       <c r="AO172" t="n">
         <v>0</v>
@@ -42158,7 +42158,7 @@
         <v>205</v>
       </c>
       <c r="H178" t="n">
-        <v>1305806000</v>
+        <v>1308387000</v>
       </c>
       <c r="I178" t="n">
         <v>0</v>
@@ -42176,7 +42176,7 @@
         <v>52.85</v>
       </c>
       <c r="N178" t="n">
-        <v>0.530432934776959</v>
+        <v>0.5314813657113086</v>
       </c>
       <c r="O178" t="n">
         <v>0.67</v>
@@ -42254,7 +42254,7 @@
         <v>24125385.06</v>
       </c>
       <c r="AN178" t="n">
-        <v>196066966.966967</v>
+        <v>196454504.5045045</v>
       </c>
       <c r="AO178" t="n">
         <v>0</v>
@@ -42628,7 +42628,7 @@
         <v>34.99</v>
       </c>
       <c r="H180" t="n">
-        <v>3611860000</v>
+        <v>3475279000</v>
       </c>
       <c r="I180" t="n">
         <v>0</v>
@@ -42646,7 +42646,7 @@
         <v>12.71</v>
       </c>
       <c r="N180" t="n">
-        <v>8.824096976644615</v>
+        <v>8.490417379659378</v>
       </c>
       <c r="O180" t="n">
         <v>0.8</v>
@@ -42724,7 +42724,7 @@
         <v>84360399.48</v>
       </c>
       <c r="AN180" t="n">
-        <v>468464332.0363165</v>
+        <v>450749546.0440986</v>
       </c>
       <c r="AO180" t="n">
         <v>4.0605</v>
@@ -42863,7 +42863,7 @@
         <v>38.02</v>
       </c>
       <c r="H181" t="n">
-        <v>3611860000</v>
+        <v>3475279000</v>
       </c>
       <c r="I181" t="n">
         <v>300</v>
@@ -42881,7 +42881,7 @@
         <v>13.08</v>
       </c>
       <c r="N181" t="n">
-        <v>4.412048488322307</v>
+        <v>4.245208689829689</v>
       </c>
       <c r="O181" t="n">
         <v>0.83</v>
@@ -42959,7 +42959,7 @@
         <v>168720798.96</v>
       </c>
       <c r="AN181" t="n">
-        <v>454894206.5491183</v>
+        <v>437692569.2695214</v>
       </c>
       <c r="AO181" t="n">
         <v>4.0605</v>
@@ -45213,7 +45213,7 @@
         <v>3.59</v>
       </c>
       <c r="H191" t="n">
-        <v>6910620</v>
+        <v>6885260</v>
       </c>
       <c r="I191" t="n">
         <v>0</v>
@@ -45231,7 +45231,7 @@
         <v>0.02</v>
       </c>
       <c r="N191" t="n">
-        <v>0.03647469618369917</v>
+        <v>0.03634084447499307</v>
       </c>
       <c r="O191" t="n">
         <v>0.01</v>
@@ -45309,7 +45309,7 @@
         <v>256931318.49</v>
       </c>
       <c r="AN191" t="n">
-        <v>115177000</v>
+        <v>114754333.3333333</v>
       </c>
       <c r="AO191" t="n">
         <v>0</v>
@@ -45448,7 +45448,7 @@
         <v>2.53</v>
       </c>
       <c r="H192" t="n">
-        <v>21971556</v>
+        <v>21890930</v>
       </c>
       <c r="I192" t="n">
         <v>0</v>
@@ -45466,7 +45466,7 @@
         <v>21.95</v>
       </c>
       <c r="N192" t="n">
-        <v>2.246391391059547</v>
+        <v>2.238148117242455</v>
       </c>
       <c r="O192" t="n">
         <v>0.32</v>
@@ -45544,7 +45544,7 @@
         <v>357000.03</v>
       </c>
       <c r="AN192" t="n">
-        <v>1847902.102607233</v>
+        <v>1841121.110176619</v>
       </c>
       <c r="AO192" t="n">
         <v>0</v>
@@ -45683,7 +45683,7 @@
         <v>1.51</v>
       </c>
       <c r="H193" t="n">
-        <v>21971556</v>
+        <v>21890930</v>
       </c>
       <c r="I193" t="n">
         <v>1000</v>
@@ -45701,7 +45701,7 @@
         <v>14.71</v>
       </c>
       <c r="N193" t="n">
-        <v>1.123195837109069</v>
+        <v>1.119074199680989</v>
       </c>
       <c r="O193" t="n">
         <v>0.22</v>
@@ -45779,7 +45779,7 @@
         <v>713999.97</v>
       </c>
       <c r="AN193" t="n">
-        <v>2756782.43412798</v>
+        <v>2746666.248431619</v>
       </c>
       <c r="AO193" t="n">
         <v>0</v>
@@ -46858,7 +46858,7 @@
         <v>34</v>
       </c>
       <c r="H198" t="n">
-        <v>295165400</v>
+        <v>308795200</v>
       </c>
       <c r="I198" t="n">
         <v>500</v>
@@ -46876,7 +46876,7 @@
         <v>8.289999999999999</v>
       </c>
       <c r="N198" t="n">
-        <v>6.520931671358175</v>
+        <v>6.822047569408141</v>
       </c>
       <c r="O198" t="n">
         <v>0.2</v>
@@ -46954,7 +46954,7 @@
         <v>26538458.42</v>
       </c>
       <c r="AN198" t="n">
-        <v>14504442.26044226</v>
+        <v>15174211.3022113</v>
       </c>
       <c r="AO198" t="n">
         <v>0</v>
@@ -47563,7 +47563,7 @@
         <v>6.51</v>
       </c>
       <c r="H201" t="n">
-        <v>119368405</v>
+        <v>118930300</v>
       </c>
       <c r="I201" t="n">
         <v>200</v>
@@ -47581,7 +47581,7 @@
         <v>1.99</v>
       </c>
       <c r="N201" t="n">
-        <v>1.40876445562562</v>
+        <v>1.403594019178624</v>
       </c>
       <c r="O201" t="n">
         <v>0.25</v>
@@ -47659,7 +47659,7 @@
         <v>28893848.04</v>
       </c>
       <c r="AN201" t="n">
-        <v>94736829.36507936</v>
+        <v>94389126.98412699</v>
       </c>
       <c r="AO201" t="n">
         <v>0</v>
@@ -56712,7 +56712,7 @@
         <v>2.5</v>
       </c>
       <c r="H240" t="n">
-        <v>2524470</v>
+        <v>2515200</v>
       </c>
       <c r="I240" t="n">
         <v>0</v>
@@ -56808,7 +56808,7 @@
         <v>54534.6</v>
       </c>
       <c r="AN240" t="n">
-        <v>97057.67012687428</v>
+        <v>96701.26874279123</v>
       </c>
       <c r="AO240" t="n">
         <v>0</v>
@@ -56947,7 +56947,7 @@
         <v>3</v>
       </c>
       <c r="H241" t="n">
-        <v>2524470</v>
+        <v>2515200</v>
       </c>
       <c r="I241" t="n">
         <v>0</v>
@@ -57043,7 +57043,7 @@
         <v>55732.8</v>
       </c>
       <c r="AN241" t="n">
-        <v>75245.00745156483</v>
+        <v>74968.70342771983</v>
       </c>
       <c r="AO241" t="n">
         <v>0</v>
@@ -58357,7 +58357,7 @@
         <v>5.25</v>
       </c>
       <c r="H247" t="n">
-        <v>19470349</v>
+        <v>19398890</v>
       </c>
       <c r="I247" t="n">
         <v>900</v>
@@ -58375,7 +58375,7 @@
         <v>4.4</v>
       </c>
       <c r="N247" t="n">
-        <v>0.02930063224919828</v>
+        <v>0.02919309468631764</v>
       </c>
       <c r="O247" t="n">
         <v>0.05</v>
@@ -58453,7 +58453,7 @@
         <v>5648272.88</v>
       </c>
       <c r="AN247" t="n">
-        <v>33000591.52542373</v>
+        <v>32879474.57627119</v>
       </c>
       <c r="AO247" t="n">
         <v>0</v>
@@ -59767,7 +59767,7 @@
         <v>17.11</v>
       </c>
       <c r="H253" t="n">
-        <v>169414200</v>
+        <v>168792300</v>
       </c>
       <c r="I253" t="n">
         <v>0</v>
@@ -59785,7 +59785,7 @@
         <v>7.29</v>
       </c>
       <c r="N253" t="n">
-        <v>0.169374227682267</v>
+        <v>0.1687524744160378</v>
       </c>
       <c r="O253" t="n">
         <v>0.12</v>
@@ -59863,7 +59863,7 @@
         <v>24405758.4</v>
       </c>
       <c r="AN253" t="n">
-        <v>116837379.3103448</v>
+        <v>116408482.7586207</v>
       </c>
       <c r="AO253" t="n">
         <v>0</v>
@@ -60002,7 +60002,7 @@
         <v>3.98</v>
       </c>
       <c r="H254" t="n">
-        <v>282026502</v>
+        <v>280991400</v>
       </c>
       <c r="I254" t="n">
         <v>1000</v>
@@ -60020,7 +60020,7 @@
         <v>0.59</v>
       </c>
       <c r="N254" t="n">
-        <v>0.6594958377293958</v>
+        <v>0.657075336621222</v>
       </c>
       <c r="O254" t="n">
         <v>0.6899999999999999</v>
@@ -60098,7 +60098,7 @@
         <v>520437330</v>
       </c>
       <c r="AN254" t="n">
-        <v>179634714.6496815</v>
+        <v>178975414.0127389</v>
       </c>
       <c r="AO254" t="n">
         <v>0</v>
@@ -60707,7 +60707,7 @@
         <v>37.66</v>
       </c>
       <c r="H257" t="n">
-        <v>12521660000</v>
+        <v>12364400000</v>
       </c>
       <c r="I257" t="n">
         <v>100</v>
@@ -60725,7 +60725,7 @@
         <v>9.57</v>
       </c>
       <c r="N257" t="n">
-        <v>3.119830028447058</v>
+        <v>3.080647965503839</v>
       </c>
       <c r="O257" t="n">
         <v>0.64</v>
@@ -60803,7 +60803,7 @@
         <v>836829598.4699999</v>
       </c>
       <c r="AN257" t="n">
-        <v>2276665454.545455</v>
+        <v>2248072727.272727</v>
       </c>
       <c r="AO257" t="n">
         <v>0</v>
@@ -60942,7 +60942,7 @@
         <v>38</v>
       </c>
       <c r="H258" t="n">
-        <v>12521660000</v>
+        <v>12364400000</v>
       </c>
       <c r="I258" t="n">
         <v>0</v>
@@ -60960,7 +60960,7 @@
         <v>8.94</v>
       </c>
       <c r="N258" t="n">
-        <v>7.158694100083332</v>
+        <v>7.06878779100138</v>
       </c>
       <c r="O258" t="n">
         <v>0.59</v>
@@ -61038,7 +61038,7 @@
         <v>364698655.02</v>
       </c>
       <c r="AN258" t="n">
-        <v>2436120622.568093</v>
+        <v>2405525291.828794</v>
       </c>
       <c r="AO258" t="n">
         <v>0</v>
@@ -61177,7 +61177,7 @@
         <v>32</v>
       </c>
       <c r="H259" t="n">
-        <v>12521660000</v>
+        <v>12364400000</v>
       </c>
       <c r="I259" t="n">
         <v>0</v>
@@ -61195,7 +61195,7 @@
         <v>9.949999999999999</v>
       </c>
       <c r="N259" t="n">
-        <v>8.442823696955527</v>
+        <v>8.336789955855446</v>
       </c>
       <c r="O259" t="n">
         <v>0.66</v>
@@ -61273,7 +61273,7 @@
         <v>309229021.44</v>
       </c>
       <c r="AN259" t="n">
-        <v>2189101398.601398</v>
+        <v>2161608391.608392</v>
       </c>
       <c r="AO259" t="n">
         <v>0</v>
@@ -61647,7 +61647,7 @@
         <v>38.29</v>
       </c>
       <c r="H261" t="n">
-        <v>242299100</v>
+        <v>241409800</v>
       </c>
       <c r="I261" t="n">
         <v>0</v>
@@ -61665,7 +61665,7 @@
         <v>22.68</v>
       </c>
       <c r="N261" t="n">
-        <v>1.546445233037403</v>
+        <v>1.540769381390657</v>
       </c>
       <c r="O261" t="n">
         <v>0.21</v>
@@ -61743,7 +61743,7 @@
         <v>11657091.15</v>
       </c>
       <c r="AN261" t="n">
-        <v>15682789.64401295</v>
+        <v>15625229.77346278</v>
       </c>
       <c r="AO261" t="n">
         <v>0</v>
@@ -61882,7 +61882,7 @@
         <v>35.1</v>
       </c>
       <c r="H262" t="n">
-        <v>242299100</v>
+        <v>241409800</v>
       </c>
       <c r="I262" t="n">
         <v>0</v>
@@ -61900,7 +61900,7 @@
         <v>19.78</v>
       </c>
       <c r="N262" t="n">
-        <v>11.25879281214101</v>
+        <v>11.21747014751767</v>
       </c>
       <c r="O262" t="n">
         <v>0.18</v>
@@ -61978,7 +61978,7 @@
         <v>1601153.28</v>
       </c>
       <c r="AN262" t="n">
-        <v>17974710.68249258</v>
+        <v>17908738.87240356</v>
       </c>
       <c r="AO262" t="n">
         <v>0</v>
@@ -63057,7 +63057,7 @@
         <v>16</v>
       </c>
       <c r="H267" t="n">
-        <v>26757732</v>
+        <v>27285390</v>
       </c>
       <c r="I267" t="n">
         <v>0</v>
@@ -63075,7 +63075,7 @@
         <v>4.28</v>
       </c>
       <c r="N267" t="n">
-        <v>0.3577231683772277</v>
+        <v>0.3647774094309759</v>
       </c>
       <c r="O267" t="n">
         <v>0.1</v>
@@ -63153,7 +63153,7 @@
         <v>2565643.74</v>
       </c>
       <c r="AN267" t="n">
-        <v>41808956.25</v>
+        <v>42633421.875</v>
       </c>
       <c r="AO267" t="n">
         <v>0</v>
@@ -63292,7 +63292,7 @@
         <v>12</v>
       </c>
       <c r="H268" t="n">
-        <v>26757732</v>
+        <v>27285390</v>
       </c>
       <c r="I268" t="n">
         <v>600</v>
@@ -63310,7 +63310,7 @@
         <v>2.74</v>
       </c>
       <c r="N268" t="n">
-        <v>0.1788615841886138</v>
+        <v>0.1823887047154879</v>
       </c>
       <c r="O268" t="n">
         <v>0.07000000000000001</v>
@@ -63388,7 +63388,7 @@
         <v>5131287.48</v>
       </c>
       <c r="AN268" t="n">
-        <v>65262760.97560976</v>
+        <v>66549731.70731708</v>
       </c>
       <c r="AO268" t="n">
         <v>0</v>
@@ -64232,7 +64232,7 @@
         <v>1.42</v>
       </c>
       <c r="H272" t="n">
-        <v>9383964</v>
+        <v>9349520</v>
       </c>
       <c r="I272" t="n">
         <v>2500</v>
@@ -64250,7 +64250,7 @@
         <v>0.96</v>
       </c>
       <c r="N272" t="n">
-        <v>3.599141588743798</v>
+        <v>3.585930878122712</v>
       </c>
       <c r="O272" t="n">
         <v>1.87</v>
@@ -64328,7 +64328,7 @@
         <v>37941114.78</v>
       </c>
       <c r="AN272" t="n">
-        <v>8304392.920353984</v>
+        <v>8273911.50442478</v>
       </c>
       <c r="AO272" t="n">
         <v>0</v>
@@ -66582,7 +66582,7 @@
         <v>30.22</v>
       </c>
       <c r="H282" t="n">
-        <v>721072800</v>
+        <v>718426100</v>
       </c>
       <c r="I282" t="n">
         <v>0</v>
@@ -66600,7 +66600,7 @@
         <v>17.82</v>
       </c>
       <c r="N282" t="n">
-        <v>0.3675287748925234</v>
+        <v>0.3661797593582972</v>
       </c>
       <c r="O282" t="n">
         <v>0.52</v>
@@ -66678,7 +66678,7 @@
         <v>42378103.55</v>
       </c>
       <c r="AN282" t="n">
-        <v>80476874.99999999</v>
+        <v>80181484.37499999</v>
       </c>
       <c r="AO282" t="n">
         <v>0</v>
@@ -66817,7 +66817,7 @@
         <v>29.5</v>
       </c>
       <c r="H283" t="n">
-        <v>721072800</v>
+        <v>718426100</v>
       </c>
       <c r="I283" t="n">
         <v>0</v>
@@ -66835,7 +66835,7 @@
         <v>18.34</v>
       </c>
       <c r="N283" t="n">
-        <v>8.211379216483353</v>
+        <v>8.181239323018691</v>
       </c>
       <c r="O283" t="n">
         <v>0.54</v>
@@ -66913,7 +66913,7 @@
         <v>1896779.1</v>
       </c>
       <c r="AN283" t="n">
-        <v>78122730.22751896</v>
+        <v>77835980.49837486</v>
       </c>
       <c r="AO283" t="n">
         <v>0</v>
@@ -71282,7 +71282,7 @@
         <v>41.65</v>
       </c>
       <c r="H302" t="n">
-        <v>259969</v>
+        <v>259010</v>
       </c>
       <c r="I302" t="n">
         <v>10</v>
@@ -71375,10 +71375,10 @@
         <v>0</v>
       </c>
       <c r="AM302" t="n">
-        <v>1710.434897032699</v>
+        <v>1704.125271399434</v>
       </c>
       <c r="AN302" t="n">
-        <v>1039876</v>
+        <v>1036040</v>
       </c>
       <c r="AO302" t="n">
         <v>0</v>
@@ -75042,7 +75042,7 @@
         <v>5.82</v>
       </c>
       <c r="H318" t="n">
-        <v>14917463599</v>
+        <v>14862710000</v>
       </c>
       <c r="I318" t="n">
         <v>300</v>
@@ -75060,7 +75060,7 @@
         <v>11.35</v>
       </c>
       <c r="N318" t="n">
-        <v>0.7688367215119367</v>
+        <v>0.7660147553467931</v>
       </c>
       <c r="O318" t="n">
         <v>0.49</v>
@@ -75138,7 +75138,7 @@
         <v>1412512331.45</v>
       </c>
       <c r="AN318" t="n">
-        <v>3300323805.088496</v>
+        <v>3288210176.991151</v>
       </c>
       <c r="AO318" t="n">
         <v>0</v>
@@ -75512,7 +75512,7 @@
         <v>0.85</v>
       </c>
       <c r="H320" t="n">
-        <v>311639163</v>
+        <v>313538600</v>
       </c>
       <c r="I320" t="n">
         <v>35600</v>
@@ -75530,7 +75530,7 @@
         <v>2.24</v>
       </c>
       <c r="N320" t="n">
-        <v>0.7898764460425702</v>
+        <v>0.7946907336070692</v>
       </c>
       <c r="O320" t="n">
         <v>0.13</v>
@@ -75608,7 +75608,7 @@
         <v>142942442.86</v>
       </c>
       <c r="AN320" t="n">
-        <v>25071533.62831859</v>
+        <v>25224344.32823813</v>
       </c>
       <c r="AO320" t="n">
         <v>0</v>
@@ -75747,7 +75747,7 @@
         <v>0.82</v>
       </c>
       <c r="H321" t="n">
-        <v>311639163</v>
+        <v>313538600</v>
       </c>
       <c r="I321" t="n">
         <v>43000</v>
@@ -75765,7 +75765,7 @@
         <v>2</v>
       </c>
       <c r="N321" t="n">
-        <v>3.935318751402238</v>
+        <v>3.959304472488285</v>
       </c>
       <c r="O321" t="n">
         <v>0.11</v>
@@ -75843,7 +75843,7 @@
         <v>28690654.02</v>
       </c>
       <c r="AN321" t="n">
-        <v>28100916.41118124</v>
+        <v>28272191.1632101</v>
       </c>
       <c r="AO321" t="n">
         <v>0</v>
@@ -76217,7 +76217,7 @@
         <v>6.01</v>
       </c>
       <c r="H323" t="n">
-        <v>530847800</v>
+        <v>528899300</v>
       </c>
       <c r="I323" t="n">
         <v>0</v>
@@ -76313,7 +76313,7 @@
         <v>8742210.08</v>
       </c>
       <c r="AN323" t="n">
-        <v>6095393.271328511</v>
+        <v>6073019.86450798</v>
       </c>
       <c r="AO323" t="n">
         <v>0</v>
@@ -76452,7 +76452,7 @@
         <v>6.78</v>
       </c>
       <c r="H324" t="n">
-        <v>530847800</v>
+        <v>528899300</v>
       </c>
       <c r="I324" t="n">
         <v>0</v>
@@ -76548,7 +76548,7 @@
         <v>2719637.39</v>
       </c>
       <c r="AN324" t="n">
-        <v>5238801.934274154</v>
+        <v>5219572.683311951</v>
       </c>
       <c r="AO324" t="n">
         <v>0.4906</v>
@@ -76687,7 +76687,7 @@
         <v>6.5</v>
       </c>
       <c r="H325" t="n">
-        <v>530847800</v>
+        <v>528899300</v>
       </c>
       <c r="I325" t="n">
         <v>0</v>
@@ -76783,7 +76783,7 @@
         <v>4627783.64</v>
       </c>
       <c r="AN325" t="n">
-        <v>7702376.668601276</v>
+        <v>7674104.759141033</v>
       </c>
       <c r="AO325" t="n">
         <v>0</v>
@@ -81857,7 +81857,7 @@
         <v>9.130000000000001</v>
       </c>
       <c r="H347" t="n">
-        <v>35193648</v>
+        <v>35383370</v>
       </c>
       <c r="I347" t="n">
         <v>0</v>
@@ -81875,7 +81875,7 @@
         <v>0.41</v>
       </c>
       <c r="N347" t="n">
-        <v>0.1035235917997077</v>
+        <v>0.1040816670206517</v>
       </c>
       <c r="O347" t="n">
         <v>0.15</v>
@@ -81953,7 +81953,7 @@
         <v>72003052.8</v>
       </c>
       <c r="AN347" t="n">
-        <v>39104053.33333334</v>
+        <v>39314855.55555555</v>
       </c>
       <c r="AO347" t="n">
         <v>0</v>
@@ -82092,7 +82092,7 @@
         <v>2.24</v>
       </c>
       <c r="H348" t="n">
-        <v>35193648</v>
+        <v>35383370</v>
       </c>
       <c r="I348" t="n">
         <v>1600</v>
@@ -82110,7 +82110,7 @@
         <v>0.1</v>
       </c>
       <c r="N348" t="n">
-        <v>0.05446203003718698</v>
+        <v>0.0547556240761657</v>
       </c>
       <c r="O348" t="n">
         <v>0.04</v>
@@ -82188,7 +82188,7 @@
         <v>136866265.2</v>
       </c>
       <c r="AN348" t="n">
-        <v>153015860.8695652</v>
+        <v>153840739.1304348</v>
       </c>
       <c r="AO348" t="n">
         <v>0</v>
@@ -82327,7 +82327,7 @@
         <v>11.51</v>
       </c>
       <c r="H349" t="n">
-        <v>35193648</v>
+        <v>35383370</v>
       </c>
       <c r="I349" t="n">
         <v>0</v>
@@ -82345,7 +82345,7 @@
         <v>0.42</v>
       </c>
       <c r="N349" t="n">
-        <v>44.38022985746436</v>
+        <v>44.61947490444039</v>
       </c>
       <c r="O349" t="n">
         <v>0.15</v>
@@ -82423,7 +82423,7 @@
         <v>167958</v>
       </c>
       <c r="AN349" t="n">
-        <v>37045945.2631579</v>
+        <v>37245652.63157895</v>
       </c>
       <c r="AO349" t="n">
         <v>0</v>
@@ -82797,7 +82797,7 @@
         <v>38.66</v>
       </c>
       <c r="H351" t="n">
-        <v>151516725</v>
+        <v>150973000</v>
       </c>
       <c r="I351" t="n">
         <v>0</v>
@@ -82815,7 +82815,7 @@
         <v>3.42</v>
       </c>
       <c r="N351" t="n">
-        <v>1.97212344693367</v>
+        <v>1.965046387809114</v>
       </c>
       <c r="O351" t="n">
         <v>0.78</v>
@@ -82893,7 +82893,7 @@
         <v>9672800</v>
       </c>
       <c r="AN351" t="n">
-        <v>61095453.62903226</v>
+        <v>60876209.67741936</v>
       </c>
       <c r="AO351" t="n">
         <v>0</v>
@@ -83032,7 +83032,7 @@
         <v>75</v>
       </c>
       <c r="H352" t="n">
-        <v>151516725</v>
+        <v>150973000</v>
       </c>
       <c r="I352" t="n">
         <v>300</v>
@@ -83050,7 +83050,7 @@
         <v>6.19</v>
       </c>
       <c r="N352" t="n">
-        <v>2.151590199560568</v>
+        <v>2.143869115427736</v>
       </c>
       <c r="O352" t="n">
         <v>1.42</v>
@@ -83128,7 +83128,7 @@
         <v>8865980</v>
       </c>
       <c r="AN352" t="n">
-        <v>33670383.33333334</v>
+        <v>33549555.55555556</v>
       </c>
       <c r="AO352" t="n">
         <v>0</v>
@@ -83267,7 +83267,7 @@
         <v>79.98</v>
       </c>
       <c r="H353" t="n">
-        <v>151516725</v>
+        <v>150973000</v>
       </c>
       <c r="I353" t="n">
         <v>0</v>
@@ -83285,7 +83285,7 @@
         <v>6.02</v>
       </c>
       <c r="N353" t="n">
-        <v>2.065505531108799</v>
+        <v>2.05809336591778</v>
       </c>
       <c r="O353" t="n">
         <v>1.38</v>
@@ -83363,7 +83363,7 @@
         <v>9235490</v>
       </c>
       <c r="AN353" t="n">
-        <v>34672019.45080092</v>
+        <v>34547597.25400458</v>
       </c>
       <c r="AO353" t="n">
         <v>0</v>
@@ -85147,7 +85147,7 @@
         <v>0.71</v>
       </c>
       <c r="H361" t="n">
-        <v>64136129</v>
+        <v>63900720</v>
       </c>
       <c r="I361" t="n">
         <v>45200</v>
@@ -85165,7 +85165,7 @@
         <v>0.74</v>
       </c>
       <c r="N361" t="n">
-        <v>0.2268618494567028</v>
+        <v>0.226029162452491</v>
       </c>
       <c r="O361" t="n">
         <v>0.11</v>
@@ -85243,7 +85243,7 @@
         <v>163434690.6</v>
       </c>
       <c r="AN361" t="n">
-        <v>60505782.07547169</v>
+        <v>60283698.11320754</v>
       </c>
       <c r="AO361" t="n">
         <v>0</v>
@@ -85617,7 +85617,7 @@
         <v>10.42</v>
       </c>
       <c r="H363" t="n">
-        <v>999695606</v>
+        <v>999570400</v>
       </c>
       <c r="I363" t="n">
         <v>0</v>
@@ -85635,7 +85635,7 @@
         <v>20.34</v>
       </c>
       <c r="N363" t="n">
-        <v>2.644585085050909</v>
+        <v>2.644253866309752</v>
       </c>
       <c r="O363" t="n">
         <v>0.27</v>
@@ -85713,7 +85713,7 @@
         <v>45966751.6</v>
       </c>
       <c r="AN363" t="n">
-        <v>106350596.3829787</v>
+        <v>106337276.5957447</v>
       </c>
       <c r="AO363" t="n">
         <v>0</v>
@@ -85852,7 +85852,7 @@
         <v>7.3</v>
       </c>
       <c r="H364" t="n">
-        <v>999695606</v>
+        <v>999570400</v>
       </c>
       <c r="I364" t="n">
         <v>1500</v>
@@ -85870,7 +85870,7 @@
         <v>14.31</v>
       </c>
       <c r="N364" t="n">
-        <v>12.00726434388735</v>
+        <v>12.00576050458825</v>
       </c>
       <c r="O364" t="n">
         <v>0.19</v>
@@ -85948,7 +85948,7 @@
         <v>10124120.05</v>
       </c>
       <c r="AN364" t="n">
-        <v>151239879.8789712</v>
+        <v>151220937.9727685</v>
       </c>
       <c r="AO364" t="n">
         <v>0</v>
@@ -88437,7 +88437,7 @@
         <v>9</v>
       </c>
       <c r="H375" t="n">
-        <v>17698860</v>
+        <v>17633900</v>
       </c>
       <c r="I375" t="n">
         <v>0</v>
@@ -88455,7 +88455,7 @@
         <v>0.73</v>
       </c>
       <c r="N375" t="n">
-        <v>0.4584441302935677</v>
+        <v>0.4567615060621839</v>
       </c>
       <c r="O375" t="n">
         <v>0.24</v>
@@ -88533,7 +88533,7 @@
         <v>19824366.83</v>
       </c>
       <c r="AN375" t="n">
-        <v>4154661.971830986</v>
+        <v>4139413.145539906</v>
       </c>
       <c r="AO375" t="n">
         <v>0</v>
@@ -88672,7 +88672,7 @@
         <v>1.65</v>
       </c>
       <c r="H376" t="n">
-        <v>17698860</v>
+        <v>17633900</v>
       </c>
       <c r="I376" t="n">
         <v>0</v>
@@ -88690,7 +88690,7 @@
         <v>0.12</v>
       </c>
       <c r="N376" t="n">
-        <v>0.2382617965809849</v>
+        <v>0.2373873060032923</v>
       </c>
       <c r="O376" t="n">
         <v>0.04</v>
@@ -88768,7 +88768,7 @@
         <v>38144447.58</v>
       </c>
       <c r="AN376" t="n">
-        <v>26416208.95522388</v>
+        <v>26319253.73134328</v>
       </c>
       <c r="AO376" t="n">
         <v>0</v>
@@ -88907,7 +88907,7 @@
         <v>1.15</v>
       </c>
       <c r="H377" t="n">
-        <v>75849398</v>
+        <v>75571000</v>
       </c>
       <c r="I377" t="n">
         <v>6900</v>
@@ -88925,7 +88925,7 @@
         <v>39.8</v>
       </c>
       <c r="N377" t="n">
-        <v>0.2811942038451382</v>
+        <v>0.2801621072692091</v>
       </c>
       <c r="O377" t="n">
         <v>0.24</v>
@@ -89003,7 +89003,7 @@
         <v>2643454.56</v>
       </c>
       <c r="AN377" t="n">
-        <v>7162360.528800756</v>
+        <v>7136071.765816809</v>
       </c>
       <c r="AO377" t="n">
         <v>0</v>
@@ -91962,7 +91962,7 @@
         <v>1.63</v>
       </c>
       <c r="H390" t="n">
-        <v>7938769</v>
+        <v>7909640</v>
       </c>
       <c r="I390" t="n">
         <v>6800</v>
@@ -91980,7 +91980,7 @@
         <v>1.29</v>
       </c>
       <c r="N390" t="n">
-        <v>1.416340097491353</v>
+        <v>1.411143250133806</v>
       </c>
       <c r="O390" t="n">
         <v>0.13</v>
@@ -92058,7 +92058,7 @@
         <v>2293618.8</v>
       </c>
       <c r="AN390" t="n">
-        <v>5222874.342105263</v>
+        <v>5203710.52631579</v>
       </c>
       <c r="AO390" t="n">
         <v>0</v>
@@ -94077,7 +94077,7 @@
         <v>3.86</v>
       </c>
       <c r="H399" t="n">
-        <v>5837610464</v>
+        <v>5805775000</v>
       </c>
       <c r="I399" t="n">
         <v>3600</v>
@@ -94095,7 +94095,7 @@
         <v>9.42</v>
       </c>
       <c r="N399" t="n">
-        <v>0.6580284027478857</v>
+        <v>0.6544398386160639</v>
       </c>
       <c r="O399" t="n">
         <v>0.66</v>
@@ -94173,7 +94173,7 @@
         <v>483489419.2399999</v>
       </c>
       <c r="AN399" t="n">
-        <v>1120462661.036468</v>
+        <v>1114352207.293666</v>
       </c>
       <c r="AO399" t="n">
         <v>0</v>
@@ -94312,7 +94312,7 @@
         <v>3.94</v>
       </c>
       <c r="H400" t="n">
-        <v>5837610464</v>
+        <v>5805775000</v>
       </c>
       <c r="I400" t="n">
         <v>5400</v>
@@ -94330,7 +94330,7 @@
         <v>9.92</v>
       </c>
       <c r="N400" t="n">
-        <v>1.427833072329044</v>
+        <v>1.420046371134701</v>
       </c>
       <c r="O400" t="n">
         <v>0.6899999999999999</v>
@@ -94408,7 +94408,7 @@
         <v>222820003.58</v>
       </c>
       <c r="AN400" t="n">
-        <v>1065257383.941606</v>
+        <v>1059447992.70073</v>
       </c>
       <c r="AO400" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-08-16 02:26
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -833,7 +833,7 @@
         <v>968664351</v>
       </c>
       <c r="I2" t="n">
-        <v>33600</v>
+        <v>43600</v>
       </c>
       <c r="J2" t="n">
         <v>152359482</v>
@@ -1068,7 +1068,7 @@
         <v>3033282090</v>
       </c>
       <c r="I3" t="n">
-        <v>516800</v>
+        <v>516900</v>
       </c>
       <c r="J3" t="n">
         <v>129510368</v>
@@ -1303,7 +1303,7 @@
         <v>232985542500</v>
       </c>
       <c r="I4" t="n">
-        <v>33534900</v>
+        <v>33535500</v>
       </c>
       <c r="J4" t="n">
         <v>15763664889</v>
@@ -1538,7 +1538,7 @@
         <v>138528002</v>
       </c>
       <c r="I5" t="n">
-        <v>16100</v>
+        <v>16200</v>
       </c>
       <c r="J5" t="n">
         <v>62120196</v>
@@ -1773,7 +1773,7 @@
         <v>465244891</v>
       </c>
       <c r="I6" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="J6" t="n">
         <v>63084700</v>
@@ -2008,7 +2008,7 @@
         <v>1872627198</v>
       </c>
       <c r="I7" t="n">
-        <v>239400</v>
+        <v>239500</v>
       </c>
       <c r="J7" t="n">
         <v>102683444</v>
@@ -2243,7 +2243,7 @@
         <v>27561658</v>
       </c>
       <c r="I8" t="n">
-        <v>28100</v>
+        <v>28300</v>
       </c>
       <c r="J8" t="n">
         <v>18969571</v>
@@ -3183,7 +3183,7 @@
         <v>509627507</v>
       </c>
       <c r="I12" t="n">
-        <v>672500</v>
+        <v>672700</v>
       </c>
       <c r="J12" t="n">
         <v>95961536</v>
@@ -3418,7 +3418,7 @@
         <v>12978927377</v>
       </c>
       <c r="I13" t="n">
-        <v>5725300</v>
+        <v>5725400</v>
       </c>
       <c r="J13" t="n">
         <v>504190947</v>
@@ -3888,7 +3888,7 @@
         <v>7628282156</v>
       </c>
       <c r="I15" t="n">
-        <v>2375200</v>
+        <v>2375300</v>
       </c>
       <c r="J15" t="n">
         <v>343551533</v>
@@ -4358,7 +4358,7 @@
         <v>10308516010</v>
       </c>
       <c r="I17" t="n">
-        <v>1706000</v>
+        <v>1706100</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -4593,7 +4593,7 @@
         <v>10308516010</v>
       </c>
       <c r="I18" t="n">
-        <v>21400</v>
+        <v>21600</v>
       </c>
       <c r="J18" t="n">
         <v>671494278</v>
@@ -4828,7 +4828,7 @@
         <v>10308516010</v>
       </c>
       <c r="I19" t="n">
-        <v>45900</v>
+        <v>46000</v>
       </c>
       <c r="J19" t="n">
         <v>317386323</v>
@@ -5063,7 +5063,7 @@
         <v>241842071</v>
       </c>
       <c r="I20" t="n">
-        <v>129800</v>
+        <v>129900</v>
       </c>
       <c r="J20" t="n">
         <v>513516302</v>
@@ -5298,7 +5298,7 @@
         <v>251070909</v>
       </c>
       <c r="I21" t="n">
-        <v>1524600</v>
+        <v>1525500</v>
       </c>
       <c r="J21" t="n">
         <v>1670418690</v>
@@ -5533,7 +5533,7 @@
         <v>750435863</v>
       </c>
       <c r="I22" t="n">
-        <v>983000</v>
+        <v>984600</v>
       </c>
       <c r="J22" t="n">
         <v>200245046</v>
@@ -6003,7 +6003,7 @@
         <v>874125466</v>
       </c>
       <c r="I24" t="n">
-        <v>14874700</v>
+        <v>14877600</v>
       </c>
       <c r="J24" t="n">
         <v>403868805</v>
@@ -6473,7 +6473,7 @@
         <v>10992826417</v>
       </c>
       <c r="I26" t="n">
-        <v>11232200</v>
+        <v>11232400</v>
       </c>
       <c r="J26" t="n">
         <v>1354393401</v>
@@ -6692,7 +6692,7 @@
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>3500</v>
+        <v>3600</v>
       </c>
       <c r="J27" t="n">
         <v>23804898</v>
@@ -6927,7 +6927,7 @@
         <v>6373276295</v>
       </c>
       <c r="I28" t="n">
-        <v>713033</v>
+        <v>713073</v>
       </c>
       <c r="J28" t="n">
         <v>83789224</v>
@@ -7867,7 +7867,7 @@
         <v>266537648</v>
       </c>
       <c r="I32" t="n">
-        <v>2019400</v>
+        <v>2021200</v>
       </c>
       <c r="J32" t="n">
         <v>73325687</v>
@@ -8102,7 +8102,7 @@
         <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>724100</v>
+        <v>724600</v>
       </c>
       <c r="J33" t="n">
         <v>40011514</v>
@@ -8337,7 +8337,7 @@
         <v>3070503302</v>
       </c>
       <c r="I34" t="n">
-        <v>3501800</v>
+        <v>3503700</v>
       </c>
       <c r="J34" t="n">
         <v>206489813</v>
@@ -8572,7 +8572,7 @@
         <v>74182273495</v>
       </c>
       <c r="I35" t="n">
-        <v>47158500</v>
+        <v>47158800</v>
       </c>
       <c r="J35" t="n">
         <v>5046500000</v>
@@ -9512,7 +9512,7 @@
         <v>3425367924</v>
       </c>
       <c r="I39" t="n">
-        <v>1200</v>
+        <v>1300</v>
       </c>
       <c r="J39" t="n">
         <v>168174945</v>
@@ -9747,7 +9747,7 @@
         <v>105332724110</v>
       </c>
       <c r="I40" t="n">
-        <v>43600800</v>
+        <v>43600900</v>
       </c>
       <c r="J40" t="n">
         <v>5730834040</v>
@@ -9982,7 +9982,7 @@
         <v>164625126652</v>
       </c>
       <c r="I41" t="n">
-        <v>7146600</v>
+        <v>7146700</v>
       </c>
       <c r="J41" t="n">
         <v>5303870781</v>
@@ -10217,7 +10217,7 @@
         <v>164625126652</v>
       </c>
       <c r="I42" t="n">
-        <v>41889200</v>
+        <v>41889400</v>
       </c>
       <c r="J42" t="n">
         <v>5288141247</v>
@@ -10687,7 +10687,7 @@
         <v>6228000</v>
       </c>
       <c r="I44" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="J44" t="n">
         <v>607192</v>
@@ -11157,7 +11157,7 @@
         <v>3201731247</v>
       </c>
       <c r="I46" t="n">
-        <v>33554500</v>
+        <v>33555600</v>
       </c>
       <c r="J46" t="n">
         <v>1000540922</v>
@@ -11392,7 +11392,7 @@
         <v>3034039714</v>
       </c>
       <c r="I47" t="n">
-        <v>13100</v>
+        <v>13300</v>
       </c>
       <c r="J47" t="n">
         <v>254106600</v>
@@ -11627,7 +11627,7 @@
         <v>3034039714</v>
       </c>
       <c r="I48" t="n">
-        <v>1700</v>
+        <v>1800</v>
       </c>
       <c r="J48" t="n">
         <v>93397546</v>
@@ -12097,7 +12097,7 @@
         <v>912189900</v>
       </c>
       <c r="I50" t="n">
-        <v>1700</v>
+        <v>1800</v>
       </c>
       <c r="J50" t="n">
         <v>11540870</v>
@@ -12332,7 +12332,7 @@
         <v>670438586</v>
       </c>
       <c r="I51" t="n">
-        <v>2463100</v>
+        <v>2468100</v>
       </c>
       <c r="J51" t="n">
         <v>975864785</v>
@@ -12551,7 +12551,7 @@
         <v>181196815</v>
       </c>
       <c r="I52" t="n">
-        <v>2200</v>
+        <v>2400</v>
       </c>
       <c r="J52" t="n">
         <v>26633197</v>
@@ -12786,7 +12786,7 @@
         <v>781640973</v>
       </c>
       <c r="I53" t="n">
-        <v>40600</v>
+        <v>41500</v>
       </c>
       <c r="J53" t="n">
         <v>136852484</v>
@@ -13021,7 +13021,7 @@
         <v>2103573248</v>
       </c>
       <c r="I54" t="n">
-        <v>282000</v>
+        <v>282900</v>
       </c>
       <c r="J54" t="n">
         <v>233212121</v>
@@ -13256,7 +13256,7 @@
         <v>6146458073</v>
       </c>
       <c r="I55" t="n">
-        <v>14300</v>
+        <v>16100</v>
       </c>
       <c r="J55" t="n">
         <v>84052790</v>
@@ -13491,7 +13491,7 @@
         <v>6146458073</v>
       </c>
       <c r="I56" t="n">
-        <v>30300</v>
+        <v>30400</v>
       </c>
       <c r="J56" t="n">
         <v>39675836</v>
@@ -13726,7 +13726,7 @@
         <v>1181034783</v>
       </c>
       <c r="I57" t="n">
-        <v>1280400</v>
+        <v>1280500</v>
       </c>
       <c r="J57" t="n">
         <v>233858065</v>
@@ -14431,7 +14431,7 @@
         <v>164041992</v>
       </c>
       <c r="I60" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="J60" t="n">
         <v>454750</v>
@@ -14666,7 +14666,7 @@
         <v>1956687146</v>
       </c>
       <c r="I61" t="n">
-        <v>822400</v>
+        <v>824400</v>
       </c>
       <c r="J61" t="n">
         <v>85608392</v>
@@ -15136,7 +15136,7 @@
         <v>323687122</v>
       </c>
       <c r="I63" t="n">
-        <v>1400</v>
+        <v>1600</v>
       </c>
       <c r="J63" t="n">
         <v>122894462</v>
@@ -15371,7 +15371,7 @@
         <v>205766487000</v>
       </c>
       <c r="I64" t="n">
-        <v>16694800</v>
+        <v>16694900</v>
       </c>
       <c r="J64" t="n">
         <v>0</v>
@@ -15606,7 +15606,7 @@
         <v>205766487000</v>
       </c>
       <c r="I65" t="n">
-        <v>16100</v>
+        <v>16700</v>
       </c>
       <c r="J65" t="n">
         <v>7298813414</v>
@@ -15841,7 +15841,7 @@
         <v>205766487000</v>
       </c>
       <c r="I66" t="n">
-        <v>1700</v>
+        <v>1800</v>
       </c>
       <c r="J66" t="n">
         <v>2972355254</v>
@@ -16311,7 +16311,7 @@
         <v>7628710616</v>
       </c>
       <c r="I68" t="n">
-        <v>52600</v>
+        <v>53100</v>
       </c>
       <c r="J68" t="n">
         <v>137989898</v>
@@ -16546,7 +16546,7 @@
         <v>7628710616</v>
       </c>
       <c r="I69" t="n">
-        <v>1949200</v>
+        <v>1949700</v>
       </c>
       <c r="J69" t="n">
         <v>255106712</v>
@@ -16781,7 +16781,7 @@
         <v>8555874905</v>
       </c>
       <c r="I70" t="n">
-        <v>6927200</v>
+        <v>6927300</v>
       </c>
       <c r="J70" t="n">
         <v>464557268</v>
@@ -17251,7 +17251,7 @@
         <v>3496033456</v>
       </c>
       <c r="I72" t="n">
-        <v>140000</v>
+        <v>143700</v>
       </c>
       <c r="J72" t="n">
         <v>451668652</v>
@@ -17486,7 +17486,7 @@
         <v>3496033456</v>
       </c>
       <c r="I73" t="n">
-        <v>15822700</v>
+        <v>15823100</v>
       </c>
       <c r="J73" t="n">
         <v>345060392</v>
@@ -17721,7 +17721,7 @@
         <v>3496033456</v>
       </c>
       <c r="I74" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="J74" t="n">
         <v>478790</v>
@@ -17956,7 +17956,7 @@
         <v>6192831654</v>
       </c>
       <c r="I75" t="n">
-        <v>6600</v>
+        <v>6700</v>
       </c>
       <c r="J75" t="n">
         <v>205064841</v>
@@ -18426,7 +18426,7 @@
         <v>6192831654</v>
       </c>
       <c r="I77" t="n">
-        <v>1151300</v>
+        <v>1151400</v>
       </c>
       <c r="J77" t="n">
         <v>202536545</v>
@@ -18896,7 +18896,7 @@
         <v>6057803047</v>
       </c>
       <c r="I79" t="n">
-        <v>23300</v>
+        <v>23400</v>
       </c>
       <c r="J79" t="n">
         <v>320121140</v>
@@ -19601,7 +19601,7 @@
         <v>347782200</v>
       </c>
       <c r="I82" t="n">
-        <v>26200</v>
+        <v>26300</v>
       </c>
       <c r="J82" t="n">
         <v>42275080</v>
@@ -19836,7 +19836,7 @@
         <v>1630800138</v>
       </c>
       <c r="I83" t="n">
-        <v>564700</v>
+        <v>564900</v>
       </c>
       <c r="J83" t="n">
         <v>350000000</v>
@@ -20071,7 +20071,7 @@
         <v>569931729</v>
       </c>
       <c r="I84" t="n">
-        <v>1032400</v>
+        <v>1037000</v>
       </c>
       <c r="J84" t="n">
         <v>104171852</v>
@@ -20541,7 +20541,7 @@
         <v>7221989203</v>
       </c>
       <c r="I86" t="n">
-        <v>2186100</v>
+        <v>2187600</v>
       </c>
       <c r="J86" t="n">
         <v>651072697</v>
@@ -20776,7 +20776,7 @@
         <v>4087287000</v>
       </c>
       <c r="I87" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="J87" t="n">
         <v>453223943</v>
@@ -21246,7 +21246,7 @@
         <v>1813813665</v>
       </c>
       <c r="I89" t="n">
-        <v>2800</v>
+        <v>3000</v>
       </c>
       <c r="J89" t="n">
         <v>35920890</v>
@@ -21481,7 +21481,7 @@
         <v>1813813665</v>
       </c>
       <c r="I90" t="n">
-        <v>1900</v>
+        <v>2900</v>
       </c>
       <c r="J90" t="n">
         <v>6565010</v>
@@ -21716,7 +21716,7 @@
         <v>1813813665</v>
       </c>
       <c r="I91" t="n">
-        <v>1500</v>
+        <v>1700</v>
       </c>
       <c r="J91" t="n">
         <v>29596015</v>
@@ -22186,7 +22186,7 @@
         <v>72471390</v>
       </c>
       <c r="I93" t="n">
-        <v>3600</v>
+        <v>3700</v>
       </c>
       <c r="J93" t="n">
         <v>4292896</v>
@@ -23596,7 +23596,7 @@
         <v>16338294044</v>
       </c>
       <c r="I99" t="n">
-        <v>1700</v>
+        <v>2300</v>
       </c>
       <c r="J99" t="n">
         <v>103862768</v>
@@ -24066,7 +24066,7 @@
         <v>610170652</v>
       </c>
       <c r="I101" t="n">
-        <v>800</v>
+        <v>900</v>
       </c>
       <c r="J101" t="n">
         <v>10759335</v>
@@ -24301,7 +24301,7 @@
         <v>610170652</v>
       </c>
       <c r="I102" t="n">
-        <v>5600</v>
+        <v>5700</v>
       </c>
       <c r="J102" t="n">
         <v>14690740</v>
@@ -24771,7 +24771,7 @@
         <v>5383120130</v>
       </c>
       <c r="I104" t="n">
-        <v>2600</v>
+        <v>2800</v>
       </c>
       <c r="J104" t="n">
         <v>23044454</v>
@@ -25006,7 +25006,7 @@
         <v>33467187752</v>
       </c>
       <c r="I105" t="n">
-        <v>138800</v>
+        <v>138900</v>
       </c>
       <c r="J105" t="n">
         <v>956601911</v>
@@ -25241,7 +25241,7 @@
         <v>33467187752</v>
       </c>
       <c r="I106" t="n">
-        <v>25688400</v>
+        <v>25688600</v>
       </c>
       <c r="J106" t="n">
         <v>1905179984</v>
@@ -26181,7 +26181,7 @@
         <v>4355601043</v>
       </c>
       <c r="I110" t="n">
-        <v>34294600</v>
+        <v>34296600</v>
       </c>
       <c r="J110" t="n">
         <v>2064266831</v>
@@ -26416,7 +26416,7 @@
         <v>47673063447</v>
       </c>
       <c r="I111" t="n">
-        <v>5172500</v>
+        <v>5173100</v>
       </c>
       <c r="J111" t="n">
         <v>1152254440</v>
@@ -26651,7 +26651,7 @@
         <v>40917478455</v>
       </c>
       <c r="I112" t="n">
-        <v>25292400</v>
+        <v>25292500</v>
       </c>
       <c r="J112" t="n">
         <v>2982810590</v>
@@ -27121,7 +27121,7 @@
         <v>365306038</v>
       </c>
       <c r="I114" t="n">
-        <v>1500</v>
+        <v>1700</v>
       </c>
       <c r="J114" t="n">
         <v>12342238</v>
@@ -27356,7 +27356,7 @@
         <v>365306038</v>
       </c>
       <c r="I115" t="n">
-        <v>3000</v>
+        <v>4100</v>
       </c>
       <c r="J115" t="n">
         <v>6518111</v>
@@ -27591,7 +27591,7 @@
         <v>13155972112</v>
       </c>
       <c r="I116" t="n">
-        <v>26020500</v>
+        <v>26021500</v>
       </c>
       <c r="J116" t="n">
         <v>3966570932</v>
@@ -28061,7 +28061,7 @@
         <v>21264955544</v>
       </c>
       <c r="I118" t="n">
-        <v>7255200</v>
+        <v>7255300</v>
       </c>
       <c r="J118" t="n">
         <v>380253069</v>
@@ -28296,7 +28296,7 @@
         <v>5954157266</v>
       </c>
       <c r="I119" t="n">
-        <v>15097400</v>
+        <v>15097700</v>
       </c>
       <c r="J119" t="n">
         <v>1326093947</v>
@@ -28531,7 +28531,7 @@
         <v>554554212</v>
       </c>
       <c r="I120" t="n">
-        <v>101500</v>
+        <v>101700</v>
       </c>
       <c r="J120" t="n">
         <v>41800000</v>
@@ -28766,7 +28766,7 @@
         <v>11321242</v>
       </c>
       <c r="I121" t="n">
-        <v>2300</v>
+        <v>2900</v>
       </c>
       <c r="J121" t="n">
         <v>8013000</v>
@@ -29236,7 +29236,7 @@
         <v>220702930</v>
       </c>
       <c r="I123" t="n">
-        <v>2600</v>
+        <v>3200</v>
       </c>
       <c r="J123" t="n">
         <v>3326971</v>
@@ -29941,7 +29941,7 @@
         <v>9800342350</v>
       </c>
       <c r="I126" t="n">
-        <v>4485100</v>
+        <v>4485300</v>
       </c>
       <c r="J126" t="n">
         <v>308047594</v>
@@ -30176,7 +30176,7 @@
         <v>704291957</v>
       </c>
       <c r="I127" t="n">
-        <v>17520900</v>
+        <v>17550300</v>
       </c>
       <c r="J127" t="n">
         <v>525591097</v>
@@ -30411,7 +30411,7 @@
         <v>53838946071</v>
       </c>
       <c r="I128" t="n">
-        <v>6096500</v>
+        <v>6096600</v>
       </c>
       <c r="J128" t="n">
         <v>3000000000</v>
@@ -30646,7 +30646,7 @@
         <v>9649924462</v>
       </c>
       <c r="I129" t="n">
-        <v>11468600</v>
+        <v>11468700</v>
       </c>
       <c r="J129" t="n">
         <v>384000000</v>
@@ -30881,7 +30881,7 @@
         <v>2653434588</v>
       </c>
       <c r="I130" t="n">
-        <v>4578500</v>
+        <v>4580300</v>
       </c>
       <c r="J130" t="n">
         <v>1255007048</v>
@@ -31116,7 +31116,7 @@
         <v>2200544387</v>
       </c>
       <c r="I131" t="n">
-        <v>347400</v>
+        <v>347500</v>
       </c>
       <c r="J131" t="n">
         <v>116217243</v>
@@ -31351,7 +31351,7 @@
         <v>828692818</v>
       </c>
       <c r="I132" t="n">
-        <v>58400</v>
+        <v>58500</v>
       </c>
       <c r="J132" t="n">
         <v>116481187</v>
@@ -31586,7 +31586,7 @@
         <v>828692818</v>
       </c>
       <c r="I133" t="n">
-        <v>5200</v>
+        <v>5300</v>
       </c>
       <c r="J133" t="n">
         <v>6493280</v>
@@ -31821,7 +31821,7 @@
         <v>5450253830</v>
       </c>
       <c r="I134" t="n">
-        <v>8469400</v>
+        <v>8469900</v>
       </c>
       <c r="J134" t="n">
         <v>520500000</v>
@@ -32056,7 +32056,7 @@
         <v>326543100</v>
       </c>
       <c r="I135" t="n">
-        <v>34200</v>
+        <v>34300</v>
       </c>
       <c r="J135" t="n">
         <v>50602842</v>
@@ -32526,7 +32526,7 @@
         <v>431806800</v>
       </c>
       <c r="I137" t="n">
-        <v>5500</v>
+        <v>5600</v>
       </c>
       <c r="J137" t="n">
         <v>21177465</v>
@@ -32761,7 +32761,7 @@
         <v>97447629</v>
       </c>
       <c r="I138" t="n">
-        <v>432800</v>
+        <v>433400</v>
       </c>
       <c r="J138" t="n">
         <v>13321978</v>
@@ -33231,7 +33231,7 @@
         <v>4576789337</v>
       </c>
       <c r="I140" t="n">
-        <v>2831200</v>
+        <v>2831300</v>
       </c>
       <c r="J140" t="n">
         <v>919034196</v>
@@ -33466,7 +33466,7 @@
         <v>254343590</v>
       </c>
       <c r="I141" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="J141" t="n">
         <v>9750000</v>
@@ -33701,7 +33701,7 @@
         <v>254343590</v>
       </c>
       <c r="I142" t="n">
-        <v>10900</v>
+        <v>11000</v>
       </c>
       <c r="J142" t="n">
         <v>12750000</v>
@@ -33936,7 +33936,7 @@
         <v>4123679935</v>
       </c>
       <c r="I143" t="n">
-        <v>5033400</v>
+        <v>5033500</v>
       </c>
       <c r="J143" t="n">
         <v>696334224</v>
@@ -34171,7 +34171,7 @@
         <v>37103171758</v>
       </c>
       <c r="I144" t="n">
-        <v>4181500</v>
+        <v>4181700</v>
       </c>
       <c r="J144" t="n">
         <v>1416381520</v>
@@ -34641,7 +34641,7 @@
         <v>8544599000</v>
       </c>
       <c r="I146" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="J146" t="n">
         <v>101878293</v>
@@ -35111,7 +35111,7 @@
         <v>1270963954</v>
       </c>
       <c r="I148" t="n">
-        <v>5200</v>
+        <v>5300</v>
       </c>
       <c r="J148" t="n">
         <v>22241700</v>
@@ -35346,7 +35346,7 @@
         <v>47539872433</v>
       </c>
       <c r="I149" t="n">
-        <v>13652000</v>
+        <v>13652200</v>
       </c>
       <c r="J149" t="n">
         <v>1937029517</v>
@@ -35581,7 +35581,7 @@
         <v>23391535139</v>
       </c>
       <c r="I150" t="n">
-        <v>6336400</v>
+        <v>6336500</v>
       </c>
       <c r="J150" t="n">
         <v>0</v>
@@ -35816,7 +35816,7 @@
         <v>23391535139</v>
       </c>
       <c r="I151" t="n">
-        <v>3500</v>
+        <v>3600</v>
       </c>
       <c r="J151" t="n">
         <v>975954372</v>
@@ -36051,7 +36051,7 @@
         <v>23391535139</v>
       </c>
       <c r="I152" t="n">
-        <v>6500</v>
+        <v>6600</v>
       </c>
       <c r="J152" t="n">
         <v>1542412758</v>
@@ -36286,7 +36286,7 @@
         <v>156129534</v>
       </c>
       <c r="I153" t="n">
-        <v>796900</v>
+        <v>797900</v>
       </c>
       <c r="J153" t="n">
         <v>205017990</v>
@@ -36521,7 +36521,7 @@
         <v>7745858676</v>
       </c>
       <c r="I154" t="n">
-        <v>2000</v>
+        <v>2200</v>
       </c>
       <c r="J154" t="n">
         <v>75529774</v>
@@ -36756,7 +36756,7 @@
         <v>7745858676</v>
       </c>
       <c r="I155" t="n">
-        <v>1500</v>
+        <v>1600</v>
       </c>
       <c r="J155" t="n">
         <v>143412165</v>
@@ -36991,7 +36991,7 @@
         <v>19953538</v>
       </c>
       <c r="I156" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="J156" t="n">
         <v>14860568</v>
@@ -37226,7 +37226,7 @@
         <v>40822690</v>
       </c>
       <c r="I157" t="n">
-        <v>7200</v>
+        <v>8900</v>
       </c>
       <c r="J157" t="n">
         <v>2204620569</v>
@@ -38166,7 +38166,7 @@
         <v>43952608221</v>
       </c>
       <c r="I161" t="n">
-        <v>22107700</v>
+        <v>22115900</v>
       </c>
       <c r="J161" t="n">
         <v>1259387047</v>
@@ -38401,7 +38401,7 @@
         <v>246266018</v>
       </c>
       <c r="I162" t="n">
-        <v>147100</v>
+        <v>150200</v>
       </c>
       <c r="J162" t="n">
         <v>36142306</v>
@@ -39341,7 +39341,7 @@
         <v>1935229930</v>
       </c>
       <c r="I166" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="J166" t="n">
         <v>31257700</v>
@@ -39576,7 +39576,7 @@
         <v>1935229930</v>
       </c>
       <c r="I167" t="n">
-        <v>164800</v>
+        <v>169200</v>
       </c>
       <c r="J167" t="n">
         <v>61361556</v>
@@ -39811,7 +39811,7 @@
         <v>857735582</v>
       </c>
       <c r="I168" t="n">
-        <v>2662900</v>
+        <v>2663200</v>
       </c>
       <c r="J168" t="n">
         <v>200000000</v>
@@ -40046,7 +40046,7 @@
         <v>2965421359</v>
       </c>
       <c r="I169" t="n">
-        <v>3233500</v>
+        <v>3233700</v>
       </c>
       <c r="J169" t="n">
         <v>277359027</v>
@@ -40281,7 +40281,7 @@
         <v>2330982332</v>
       </c>
       <c r="I170" t="n">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="J170" t="n">
         <v>117725000</v>
@@ -40516,7 +40516,7 @@
         <v>2330982332</v>
       </c>
       <c r="I171" t="n">
-        <v>1653400</v>
+        <v>1653500</v>
       </c>
       <c r="J171" t="n">
         <v>235450000</v>
@@ -40751,7 +40751,7 @@
         <v>178089414</v>
       </c>
       <c r="I172" t="n">
-        <v>3600</v>
+        <v>3700</v>
       </c>
       <c r="J172" t="n">
         <v>53857284</v>
@@ -40986,7 +40986,7 @@
         <v>8350718</v>
       </c>
       <c r="I173" t="n">
-        <v>30400</v>
+        <v>30500</v>
       </c>
       <c r="J173" t="n">
         <v>43862205</v>
@@ -41456,7 +41456,7 @@
         <v>1887679152</v>
       </c>
       <c r="I175" t="n">
-        <v>1942000</v>
+        <v>1943000</v>
       </c>
       <c r="J175" t="n">
         <v>399086646</v>
@@ -41691,7 +41691,7 @@
         <v>9995521510</v>
       </c>
       <c r="I176" t="n">
-        <v>4323200</v>
+        <v>4323700</v>
       </c>
       <c r="J176" t="n">
         <v>547191026</v>
@@ -41926,7 +41926,7 @@
         <v>6055238266</v>
       </c>
       <c r="I177" t="n">
-        <v>270100</v>
+        <v>270300</v>
       </c>
       <c r="J177" t="n">
         <v>280335091</v>
@@ -42396,7 +42396,7 @@
         <v>0</v>
       </c>
       <c r="I179" t="n">
-        <v>56351</v>
+        <v>56367</v>
       </c>
       <c r="J179" t="n">
         <v>49031062</v>
@@ -42866,7 +42866,7 @@
         <v>3462123155</v>
       </c>
       <c r="I181" t="n">
-        <v>1300</v>
+        <v>1600</v>
       </c>
       <c r="J181" t="n">
         <v>62955522</v>
@@ -43101,7 +43101,7 @@
         <v>33114478</v>
       </c>
       <c r="I182" t="n">
-        <v>1888600</v>
+        <v>1892100</v>
       </c>
       <c r="J182" t="n">
         <v>157368961</v>
@@ -43336,7 +43336,7 @@
         <v>46235264784</v>
       </c>
       <c r="I183" t="n">
-        <v>19300</v>
+        <v>19400</v>
       </c>
       <c r="J183" t="n">
         <v>716975719</v>
@@ -43571,7 +43571,7 @@
         <v>46235264784</v>
       </c>
       <c r="I184" t="n">
-        <v>10371500</v>
+        <v>10371800</v>
       </c>
       <c r="J184" t="n">
         <v>1261042330</v>
@@ -43806,7 +43806,7 @@
         <v>8441371688</v>
       </c>
       <c r="I185" t="n">
-        <v>6175400</v>
+        <v>6180800</v>
       </c>
       <c r="J185" t="n">
         <v>752350487</v>
@@ -44276,7 +44276,7 @@
         <v>14038515807</v>
       </c>
       <c r="I187" t="n">
-        <v>32300</v>
+        <v>32400</v>
       </c>
       <c r="J187" t="n">
         <v>486802764</v>
@@ -44511,7 +44511,7 @@
         <v>14038515807</v>
       </c>
       <c r="I188" t="n">
-        <v>10613600</v>
+        <v>10613700</v>
       </c>
       <c r="J188" t="n">
         <v>835885284</v>
@@ -44981,7 +44981,7 @@
         <v>3191082556</v>
       </c>
       <c r="I190" t="n">
-        <v>3241200</v>
+        <v>3241300</v>
       </c>
       <c r="J190" t="n">
         <v>902160000</v>
@@ -45216,7 +45216,7 @@
         <v>5314867</v>
       </c>
       <c r="I191" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="J191" t="n">
         <v>1928769</v>
@@ -45686,7 +45686,7 @@
         <v>23608750</v>
       </c>
       <c r="I193" t="n">
-        <v>31400</v>
+        <v>31600</v>
       </c>
       <c r="J193" t="n">
         <v>7933333</v>
@@ -45921,7 +45921,7 @@
         <v>3382705293</v>
       </c>
       <c r="I194" t="n">
-        <v>23963300</v>
+        <v>23965700</v>
       </c>
       <c r="J194" t="n">
         <v>502630884</v>
@@ -46391,7 +46391,7 @@
         <v>229544006</v>
       </c>
       <c r="I196" t="n">
-        <v>782600</v>
+        <v>783000</v>
       </c>
       <c r="J196" t="n">
         <v>103188981</v>
@@ -46626,7 +46626,7 @@
         <v>4375682661</v>
       </c>
       <c r="I197" t="n">
-        <v>2624400</v>
+        <v>2624600</v>
       </c>
       <c r="J197" t="n">
         <v>1360382643</v>
@@ -47566,7 +47566,7 @@
         <v>125001658</v>
       </c>
       <c r="I201" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="J201" t="n">
         <v>7894494</v>
@@ -47801,7 +47801,7 @@
         <v>15173945729</v>
       </c>
       <c r="I202" t="n">
-        <v>4178900</v>
+        <v>4179000</v>
       </c>
       <c r="J202" t="n">
         <v>704009059</v>
@@ -48255,7 +48255,7 @@
         <v>53572383</v>
       </c>
       <c r="I204" t="n">
-        <v>124200</v>
+        <v>125100</v>
       </c>
       <c r="J204" t="n">
         <v>27558749</v>
@@ -48490,7 +48490,7 @@
         <v>7401451274</v>
       </c>
       <c r="I205" t="n">
-        <v>2804900</v>
+        <v>2805000</v>
       </c>
       <c r="J205" t="n">
         <v>0</v>
@@ -48725,7 +48725,7 @@
         <v>7401451274</v>
       </c>
       <c r="I206" t="n">
-        <v>29400</v>
+        <v>29500</v>
       </c>
       <c r="J206" t="n">
         <v>770992429</v>
@@ -48960,7 +48960,7 @@
         <v>7401451274</v>
       </c>
       <c r="I207" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="J207" t="n">
         <v>435368756</v>
@@ -49195,7 +49195,7 @@
         <v>80793308</v>
       </c>
       <c r="I208" t="n">
-        <v>33900</v>
+        <v>34100</v>
       </c>
       <c r="J208" t="n">
         <v>41772224</v>
@@ -49430,7 +49430,7 @@
         <v>80793308</v>
       </c>
       <c r="I209" t="n">
-        <v>15000</v>
+        <v>15500</v>
       </c>
       <c r="J209" t="n">
         <v>12627232</v>
@@ -49665,7 +49665,7 @@
         <v>4631965781</v>
       </c>
       <c r="I210" t="n">
-        <v>1041900</v>
+        <v>1042000</v>
       </c>
       <c r="J210" t="n">
         <v>327611110</v>
@@ -49900,7 +49900,7 @@
         <v>4291523270</v>
       </c>
       <c r="I211" t="n">
-        <v>1717000</v>
+        <v>1717200</v>
       </c>
       <c r="J211" t="n">
         <v>81422761</v>
@@ -50135,7 +50135,7 @@
         <v>19297745793</v>
       </c>
       <c r="I212" t="n">
-        <v>3900</v>
+        <v>4000</v>
       </c>
       <c r="J212" t="n">
         <v>238170004</v>
@@ -50370,7 +50370,7 @@
         <v>19297745793</v>
       </c>
       <c r="I213" t="n">
-        <v>4301800</v>
+        <v>4301900</v>
       </c>
       <c r="J213" t="n">
         <v>465157744</v>
@@ -50605,7 +50605,7 @@
         <v>141273388211</v>
       </c>
       <c r="I214" t="n">
-        <v>141500</v>
+        <v>141600</v>
       </c>
       <c r="J214" t="n">
         <v>3853634012</v>
@@ -50840,7 +50840,7 @@
         <v>141273388211</v>
       </c>
       <c r="I215" t="n">
-        <v>24814300</v>
+        <v>24817000</v>
       </c>
       <c r="J215" t="n">
         <v>7360052833</v>
@@ -51545,7 +51545,7 @@
         <v>593106944</v>
       </c>
       <c r="I218" t="n">
-        <v>1044700</v>
+        <v>1046200</v>
       </c>
       <c r="J218" t="n">
         <v>303541864</v>
@@ -51780,7 +51780,7 @@
         <v>5644632</v>
       </c>
       <c r="I219" t="n">
-        <v>60500</v>
+        <v>60600</v>
       </c>
       <c r="J219" t="n">
         <v>12802745</v>
@@ -52720,7 +52720,7 @@
         <v>1444034929</v>
       </c>
       <c r="I223" t="n">
-        <v>869900</v>
+        <v>871700</v>
       </c>
       <c r="J223" t="n">
         <v>286431078</v>
@@ -52955,7 +52955,7 @@
         <v>1040888447</v>
       </c>
       <c r="I224" t="n">
-        <v>1823200</v>
+        <v>1823300</v>
       </c>
       <c r="J224" t="n">
         <v>179720130</v>
@@ -53425,7 +53425,7 @@
         <v>22059344270</v>
       </c>
       <c r="I226" t="n">
-        <v>369000</v>
+        <v>370500</v>
       </c>
       <c r="J226" t="n">
         <v>2312800469</v>
@@ -53660,7 +53660,7 @@
         <v>22059344270</v>
       </c>
       <c r="I227" t="n">
-        <v>2662300</v>
+        <v>2667900</v>
       </c>
       <c r="J227" t="n">
         <v>3928678381</v>
@@ -54130,7 +54130,7 @@
         <v>1850599132</v>
       </c>
       <c r="I229" t="n">
-        <v>429700</v>
+        <v>429800</v>
       </c>
       <c r="J229" t="n">
         <v>195434352</v>
@@ -54365,7 +54365,7 @@
         <v>4464199460</v>
       </c>
       <c r="I230" t="n">
-        <v>393400</v>
+        <v>394000</v>
       </c>
       <c r="J230" t="n">
         <v>135539000</v>
@@ -54600,7 +54600,7 @@
         <v>1989871650</v>
       </c>
       <c r="I231" t="n">
-        <v>7620000</v>
+        <v>7622800</v>
       </c>
       <c r="J231" t="n">
         <v>1609809601</v>
@@ -54835,7 +54835,7 @@
         <v>207336800</v>
       </c>
       <c r="I232" t="n">
-        <v>3829800</v>
+        <v>3834200</v>
       </c>
       <c r="J232" t="n">
         <v>206917263</v>
@@ -55070,7 +55070,7 @@
         <v>2067996626</v>
       </c>
       <c r="I233" t="n">
-        <v>458600</v>
+        <v>458700</v>
       </c>
       <c r="J233" t="n">
         <v>87859154</v>
@@ -55305,7 +55305,7 @@
         <v>2940781441</v>
       </c>
       <c r="I234" t="n">
-        <v>6400</v>
+        <v>7300</v>
       </c>
       <c r="J234" t="n">
         <v>107306486</v>
@@ -55775,7 +55775,7 @@
         <v>11309623308</v>
       </c>
       <c r="I236" t="n">
-        <v>25930800</v>
+        <v>25933500</v>
       </c>
       <c r="J236" t="n">
         <v>1006845095</v>
@@ -56010,7 +56010,7 @@
         <v>248706186</v>
       </c>
       <c r="I237" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="J237" t="n">
         <v>46687694</v>
@@ -56245,7 +56245,7 @@
         <v>110378545</v>
       </c>
       <c r="I238" t="n">
-        <v>31000</v>
+        <v>31100</v>
       </c>
       <c r="J238" t="n">
         <v>23184000</v>
@@ -56480,7 +56480,7 @@
         <v>2295947942</v>
       </c>
       <c r="I239" t="n">
-        <v>19504700</v>
+        <v>19508700</v>
       </c>
       <c r="J239" t="n">
         <v>568561350</v>
@@ -57185,7 +57185,7 @@
         <v>1614376242</v>
       </c>
       <c r="I242" t="n">
-        <v>406100</v>
+        <v>406700</v>
       </c>
       <c r="J242" t="n">
         <v>333548825</v>
@@ -57655,7 +57655,7 @@
         <v>2421632038</v>
       </c>
       <c r="I244" t="n">
-        <v>1701500</v>
+        <v>1701600</v>
       </c>
       <c r="J244" t="n">
         <v>104214394</v>
@@ -57890,7 +57890,7 @@
         <v>183844987</v>
       </c>
       <c r="I245" t="n">
-        <v>622600</v>
+        <v>622700</v>
       </c>
       <c r="J245" t="n">
         <v>286676540</v>
@@ -58360,7 +58360,7 @@
         <v>20144156</v>
       </c>
       <c r="I247" t="n">
-        <v>18100</v>
+        <v>18200</v>
       </c>
       <c r="J247" t="n">
         <v>3715969</v>
@@ -58595,7 +58595,7 @@
         <v>3040097401</v>
       </c>
       <c r="I248" t="n">
-        <v>26562700</v>
+        <v>26565500</v>
       </c>
       <c r="J248" t="n">
         <v>775945010</v>
@@ -58830,7 +58830,7 @@
         <v>3661532249</v>
       </c>
       <c r="I249" t="n">
-        <v>1339100</v>
+        <v>1339500</v>
       </c>
       <c r="J249" t="n">
         <v>234238661</v>
@@ -60005,7 +60005,7 @@
         <v>267505086</v>
       </c>
       <c r="I254" t="n">
-        <v>2000</v>
+        <v>2100</v>
       </c>
       <c r="J254" t="n">
         <v>71001000</v>
@@ -60240,7 +60240,7 @@
         <v>27932525186</v>
       </c>
       <c r="I255" t="n">
-        <v>14531600</v>
+        <v>14532000</v>
       </c>
       <c r="J255" t="n">
         <v>2020000000</v>
@@ -60475,7 +60475,7 @@
         <v>2892202520</v>
       </c>
       <c r="I256" t="n">
-        <v>4781200</v>
+        <v>4781500</v>
       </c>
       <c r="J256" t="n">
         <v>402158941</v>
@@ -62120,7 +62120,7 @@
         <v>306746930</v>
       </c>
       <c r="I263" t="n">
-        <v>863600</v>
+        <v>863700</v>
       </c>
       <c r="J263" t="n">
         <v>105774820</v>
@@ -62590,7 +62590,7 @@
         <v>443048720</v>
       </c>
       <c r="I265" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="J265" t="n">
         <v>4577200</v>
@@ -62825,7 +62825,7 @@
         <v>13744678030</v>
       </c>
       <c r="I266" t="n">
-        <v>5127200</v>
+        <v>5127300</v>
       </c>
       <c r="J266" t="n">
         <v>513163701</v>
@@ -63530,7 +63530,7 @@
         <v>1378579210</v>
       </c>
       <c r="I269" t="n">
-        <v>755800</v>
+        <v>756000</v>
       </c>
       <c r="J269" t="n">
         <v>153719601</v>
@@ -63765,7 +63765,7 @@
         <v>6146798</v>
       </c>
       <c r="I270" t="n">
-        <v>1100</v>
+        <v>1500</v>
       </c>
       <c r="J270" t="n">
         <v>2655569</v>
@@ -64235,7 +64235,7 @@
         <v>8957131</v>
       </c>
       <c r="I272" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="J272" t="n">
         <v>6621486</v>
@@ -64470,7 +64470,7 @@
         <v>26488780</v>
       </c>
       <c r="I273" t="n">
-        <v>1500</v>
+        <v>1700</v>
       </c>
       <c r="J273" t="n">
         <v>13244400</v>
@@ -64940,7 +64940,7 @@
         <v>1360109084</v>
       </c>
       <c r="I275" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="J275" t="n">
         <v>53949006</v>
@@ -65175,7 +65175,7 @@
         <v>37003410</v>
       </c>
       <c r="I276" t="n">
-        <v>479000</v>
+        <v>479100</v>
       </c>
       <c r="J276" t="n">
         <v>328544466</v>
@@ -65410,7 +65410,7 @@
         <v>37003410</v>
       </c>
       <c r="I277" t="n">
-        <v>11500</v>
+        <v>11600</v>
       </c>
       <c r="J277" t="n">
         <v>1577272</v>
@@ -65645,7 +65645,7 @@
         <v>875797208</v>
       </c>
       <c r="I278" t="n">
-        <v>28967000</v>
+        <v>28967100</v>
       </c>
       <c r="J278" t="n">
         <v>1135097787</v>
@@ -65880,7 +65880,7 @@
         <v>1939533261</v>
       </c>
       <c r="I279" t="n">
-        <v>731300</v>
+        <v>731800</v>
       </c>
       <c r="J279" t="n">
         <v>199959554</v>
@@ -66115,7 +66115,7 @@
         <v>8558036312</v>
       </c>
       <c r="I280" t="n">
-        <v>5275500</v>
+        <v>5279500</v>
       </c>
       <c r="J280" t="n">
         <v>549296404</v>
@@ -66350,7 +66350,7 @@
         <v>2838979</v>
       </c>
       <c r="I281" t="n">
-        <v>500</v>
+        <v>700</v>
       </c>
       <c r="J281" t="n">
         <v>3148038</v>
@@ -66585,7 +66585,7 @@
         <v>864920520</v>
       </c>
       <c r="I282" t="n">
-        <v>8200</v>
+        <v>8300</v>
       </c>
       <c r="J282" t="n">
         <v>22907083</v>
@@ -66820,7 +66820,7 @@
         <v>864920520</v>
       </c>
       <c r="I283" t="n">
-        <v>800</v>
+        <v>1200</v>
       </c>
       <c r="J283" t="n">
         <v>1025286</v>
@@ -67290,7 +67290,7 @@
         <v>4183570</v>
       </c>
       <c r="I285" t="n">
-        <v>38700</v>
+        <v>38800</v>
       </c>
       <c r="J285" t="n">
         <v>3287486</v>
@@ -67525,7 +67525,7 @@
         <v>127409201</v>
       </c>
       <c r="I286" t="n">
-        <v>15500</v>
+        <v>15900</v>
       </c>
       <c r="J286" t="n">
         <v>79469626</v>
@@ -68230,7 +68230,7 @@
         <v>579768707101</v>
       </c>
       <c r="I289" t="n">
-        <v>9581700</v>
+        <v>9582600</v>
       </c>
       <c r="J289" t="n">
         <v>7442231382</v>
@@ -68465,7 +68465,7 @@
         <v>579768707101</v>
       </c>
       <c r="I290" t="n">
-        <v>34128400</v>
+        <v>34128900</v>
       </c>
       <c r="J290" t="n">
         <v>5446501379</v>
@@ -68700,7 +68700,7 @@
         <v>890778062</v>
       </c>
       <c r="I291" t="n">
-        <v>198000</v>
+        <v>198500</v>
       </c>
       <c r="J291" t="n">
         <v>123812773</v>
@@ -68935,7 +68935,7 @@
         <v>2350186170</v>
       </c>
       <c r="I292" t="n">
-        <v>2603400</v>
+        <v>2605700</v>
       </c>
       <c r="J292" t="n">
         <v>723898206</v>
@@ -69170,7 +69170,7 @@
         <v>2649535285</v>
       </c>
       <c r="I293" t="n">
-        <v>31600</v>
+        <v>31800</v>
       </c>
       <c r="J293" t="n">
         <v>129950956</v>
@@ -69405,7 +69405,7 @@
         <v>2649535285</v>
       </c>
       <c r="I294" t="n">
-        <v>1041100</v>
+        <v>1041600</v>
       </c>
       <c r="J294" t="n">
         <v>129937768</v>
@@ -70110,7 +70110,7 @@
         <v>232856274</v>
       </c>
       <c r="I297" t="n">
-        <v>12356700</v>
+        <v>12368700</v>
       </c>
       <c r="J297" t="n">
         <v>297198233</v>
@@ -70345,7 +70345,7 @@
         <v>1695177000</v>
       </c>
       <c r="I298" t="n">
-        <v>799400</v>
+        <v>799500</v>
       </c>
       <c r="J298" t="n">
         <v>150377481</v>
@@ -70580,7 +70580,7 @@
         <v>5030344243</v>
       </c>
       <c r="I299" t="n">
-        <v>2691600</v>
+        <v>2691700</v>
       </c>
       <c r="J299" t="n">
         <v>450945982</v>
@@ -70815,7 +70815,7 @@
         <v>5030344243</v>
       </c>
       <c r="I300" t="n">
-        <v>18629900</v>
+        <v>18630100</v>
       </c>
       <c r="J300" t="n">
         <v>798952621</v>
@@ -71050,7 +71050,7 @@
         <v>471730490</v>
       </c>
       <c r="I301" t="n">
-        <v>1069200</v>
+        <v>1069300</v>
       </c>
       <c r="J301" t="n">
         <v>141800000</v>
@@ -71285,7 +71285,7 @@
         <v>278870</v>
       </c>
       <c r="I302" t="n">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="J302" t="n">
         <v>0</v>
@@ -71520,7 +71520,7 @@
         <v>51258134431</v>
       </c>
       <c r="I303" t="n">
-        <v>4986300</v>
+        <v>4986500</v>
       </c>
       <c r="J303" t="n">
         <v>872495263</v>
@@ -71755,7 +71755,7 @@
         <v>940811653</v>
       </c>
       <c r="I304" t="n">
-        <v>979600</v>
+        <v>979800</v>
       </c>
       <c r="J304" t="n">
         <v>57007156</v>
@@ -71990,7 +71990,7 @@
         <v>30179057420</v>
       </c>
       <c r="I305" t="n">
-        <v>2050500</v>
+        <v>2050600</v>
       </c>
       <c r="J305" t="n">
         <v>646586060</v>
@@ -72225,7 +72225,7 @@
         <v>203432840</v>
       </c>
       <c r="I306" t="n">
-        <v>1327000</v>
+        <v>1327200</v>
       </c>
       <c r="J306" t="n">
         <v>140986886</v>
@@ -72460,7 +72460,7 @@
         <v>474303868</v>
       </c>
       <c r="I307" t="n">
-        <v>3107800</v>
+        <v>3108000</v>
       </c>
       <c r="J307" t="n">
         <v>284014325</v>
@@ -72695,7 +72695,7 @@
         <v>30781278805</v>
       </c>
       <c r="I308" t="n">
-        <v>10017300</v>
+        <v>10018100</v>
       </c>
       <c r="J308" t="n">
         <v>1752367344</v>
@@ -72930,7 +72930,7 @@
         <v>25356045701</v>
       </c>
       <c r="I309" t="n">
-        <v>14802300</v>
+        <v>14814600</v>
       </c>
       <c r="J309" t="n">
         <v>1858828617</v>
@@ -73165,7 +73165,7 @@
         <v>326806072</v>
       </c>
       <c r="I310" t="n">
-        <v>16414000</v>
+        <v>16418000</v>
       </c>
       <c r="J310" t="n">
         <v>1358936900</v>
@@ -73400,7 +73400,7 @@
         <v>1785387282</v>
       </c>
       <c r="I311" t="n">
-        <v>742700</v>
+        <v>742900</v>
       </c>
       <c r="J311" t="n">
         <v>230501219</v>
@@ -73870,7 +73870,7 @@
         <v>1879101165</v>
       </c>
       <c r="I313" t="n">
-        <v>5628400</v>
+        <v>5628500</v>
       </c>
       <c r="J313" t="n">
         <v>223882733</v>
@@ -74105,7 +74105,7 @@
         <v>65333800</v>
       </c>
       <c r="I314" t="n">
-        <v>47300</v>
+        <v>47400</v>
       </c>
       <c r="J314" t="n">
         <v>42655504</v>
@@ -74340,7 +74340,7 @@
         <v>65333800</v>
       </c>
       <c r="I315" t="n">
-        <v>5302700</v>
+        <v>5314200</v>
       </c>
       <c r="J315" t="n">
         <v>84633668</v>
@@ -74575,7 +74575,7 @@
         <v>75408228378</v>
       </c>
       <c r="I316" t="n">
-        <v>10175800</v>
+        <v>10176900</v>
       </c>
       <c r="J316" t="n">
         <v>2240292590</v>
@@ -74810,7 +74810,7 @@
         <v>3090751439</v>
       </c>
       <c r="I317" t="n">
-        <v>2641800</v>
+        <v>2641900</v>
       </c>
       <c r="J317" t="n">
         <v>293482126</v>
@@ -75045,7 +75045,7 @@
         <v>14256696841</v>
       </c>
       <c r="I318" t="n">
-        <v>2300</v>
+        <v>2400</v>
       </c>
       <c r="J318" t="n">
         <v>2568204239</v>
@@ -75280,7 +75280,7 @@
         <v>37713760590</v>
       </c>
       <c r="I319" t="n">
-        <v>12264300</v>
+        <v>12264400</v>
       </c>
       <c r="J319" t="n">
         <v>1082620720</v>
@@ -75515,7 +75515,7 @@
         <v>279308700</v>
       </c>
       <c r="I320" t="n">
-        <v>342500</v>
+        <v>342600</v>
       </c>
       <c r="J320" t="n">
         <v>310744441</v>
@@ -75750,7 +75750,7 @@
         <v>279308700</v>
       </c>
       <c r="I321" t="n">
-        <v>157900</v>
+        <v>158800</v>
       </c>
       <c r="J321" t="n">
         <v>62370987</v>
@@ -75985,7 +75985,7 @@
         <v>519079759</v>
       </c>
       <c r="I322" t="n">
-        <v>127400</v>
+        <v>127700</v>
       </c>
       <c r="J322" t="n">
         <v>93170747</v>
@@ -76220,7 +76220,7 @@
         <v>601149360</v>
       </c>
       <c r="I323" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="J323" t="n">
         <v>46011632</v>
@@ -76455,7 +76455,7 @@
         <v>601149360</v>
       </c>
       <c r="I324" t="n">
-        <v>2200</v>
+        <v>3200</v>
       </c>
       <c r="J324" t="n">
         <v>14313881</v>
@@ -76690,7 +76690,7 @@
         <v>601149360</v>
       </c>
       <c r="I325" t="n">
-        <v>3700</v>
+        <v>4000</v>
       </c>
       <c r="J325" t="n">
         <v>24356756</v>
@@ -77395,7 +77395,7 @@
         <v>250557323</v>
       </c>
       <c r="I328" t="n">
-        <v>2000</v>
+        <v>2200</v>
       </c>
       <c r="J328" t="n">
         <v>2495225</v>
@@ -77630,7 +77630,7 @@
         <v>112981740531</v>
       </c>
       <c r="I329" t="n">
-        <v>4989900</v>
+        <v>4990100</v>
       </c>
       <c r="J329" t="n">
         <v>0</v>
@@ -78100,7 +78100,7 @@
         <v>112981740531</v>
       </c>
       <c r="I331" t="n">
-        <v>762200</v>
+        <v>762300</v>
       </c>
       <c r="J331" t="n">
         <v>3679836020</v>
@@ -78570,7 +78570,7 @@
         <v>9960016111</v>
       </c>
       <c r="I333" t="n">
-        <v>187800</v>
+        <v>187900</v>
       </c>
       <c r="J333" t="n">
         <v>503735259</v>
@@ -78805,7 +78805,7 @@
         <v>9960016111</v>
       </c>
       <c r="I334" t="n">
-        <v>3188700</v>
+        <v>3188900</v>
       </c>
       <c r="J334" t="n">
         <v>1007470260</v>
@@ -79040,7 +79040,7 @@
         <v>1990043857</v>
       </c>
       <c r="I335" t="n">
-        <v>2862200</v>
+        <v>2865400</v>
       </c>
       <c r="J335" t="n">
         <v>230663994</v>
@@ -79510,7 +79510,7 @@
         <v>708137842</v>
       </c>
       <c r="I337" t="n">
-        <v>74500</v>
+        <v>74600</v>
       </c>
       <c r="J337" t="n">
         <v>57737319</v>
@@ -79745,7 +79745,7 @@
         <v>1450691363</v>
       </c>
       <c r="I338" t="n">
-        <v>1248200</v>
+        <v>1248300</v>
       </c>
       <c r="J338" t="n">
         <v>128721560</v>
@@ -79980,7 +79980,7 @@
         <v>446838491</v>
       </c>
       <c r="I339" t="n">
-        <v>279800</v>
+        <v>280500</v>
       </c>
       <c r="J339" t="n">
         <v>6313033484</v>
@@ -80215,7 +80215,7 @@
         <v>410699982</v>
       </c>
       <c r="I340" t="n">
-        <v>17800</v>
+        <v>17900</v>
       </c>
       <c r="J340" t="n">
         <v>6741262</v>
@@ -80685,7 +80685,7 @@
         <v>881917139</v>
       </c>
       <c r="I342" t="n">
-        <v>467800</v>
+        <v>468400</v>
       </c>
       <c r="J342" t="n">
         <v>204682016</v>
@@ -80920,7 +80920,7 @@
         <v>3595956582</v>
       </c>
       <c r="I343" t="n">
-        <v>3073600</v>
+        <v>3073700</v>
       </c>
       <c r="J343" t="n">
         <v>583759291</v>
@@ -81155,7 +81155,7 @@
         <v>6663245052</v>
       </c>
       <c r="I344" t="n">
-        <v>3744100</v>
+        <v>3744500</v>
       </c>
       <c r="J344" t="n">
         <v>498745930</v>
@@ -81390,7 +81390,7 @@
         <v>10569528998</v>
       </c>
       <c r="I345" t="n">
-        <v>8919200</v>
+        <v>8924600</v>
       </c>
       <c r="J345" t="n">
         <v>616129844</v>
@@ -81625,7 +81625,7 @@
         <v>4866729680</v>
       </c>
       <c r="I346" t="n">
-        <v>1658600</v>
+        <v>1658700</v>
       </c>
       <c r="J346" t="n">
         <v>332435391</v>
@@ -82095,7 +82095,7 @@
         <v>39740085</v>
       </c>
       <c r="I348" t="n">
-        <v>5200</v>
+        <v>5800</v>
       </c>
       <c r="J348" t="n">
         <v>5052280</v>
@@ -82565,7 +82565,7 @@
         <v>715217741</v>
       </c>
       <c r="I350" t="n">
-        <v>509200</v>
+        <v>510200</v>
       </c>
       <c r="J350" t="n">
         <v>141902688</v>
@@ -83740,7 +83740,7 @@
         <v>561340824</v>
       </c>
       <c r="I355" t="n">
-        <v>1577400</v>
+        <v>1577500</v>
       </c>
       <c r="J355" t="n">
         <v>152644445</v>
@@ -83975,7 +83975,7 @@
         <v>13096792675</v>
       </c>
       <c r="I356" t="n">
-        <v>3665700</v>
+        <v>3666200</v>
       </c>
       <c r="J356" t="n">
         <v>0</v>
@@ -84210,7 +84210,7 @@
         <v>13096792675</v>
       </c>
       <c r="I357" t="n">
-        <v>285000</v>
+        <v>285100</v>
       </c>
       <c r="J357" t="n">
         <v>590714069</v>
@@ -84445,7 +84445,7 @@
         <v>13096792675</v>
       </c>
       <c r="I358" t="n">
-        <v>470600</v>
+        <v>470800</v>
       </c>
       <c r="J358" t="n">
         <v>442782652</v>
@@ -84680,7 +84680,7 @@
         <v>699011637</v>
       </c>
       <c r="I359" t="n">
-        <v>13400</v>
+        <v>13500</v>
       </c>
       <c r="J359" t="n">
         <v>51089845</v>
@@ -84915,7 +84915,7 @@
         <v>699011637</v>
       </c>
       <c r="I360" t="n">
-        <v>343500</v>
+        <v>344000</v>
       </c>
       <c r="J360" t="n">
         <v>88208032</v>
@@ -85150,7 +85150,7 @@
         <v>62579315</v>
       </c>
       <c r="I361" t="n">
-        <v>112400</v>
+        <v>112500</v>
       </c>
       <c r="J361" t="n">
         <v>73619230</v>
@@ -85385,7 +85385,7 @@
         <v>584892916</v>
       </c>
       <c r="I362" t="n">
-        <v>44800</v>
+        <v>45000</v>
       </c>
       <c r="J362" t="n">
         <v>60906215</v>
@@ -85620,7 +85620,7 @@
         <v>1085649640</v>
       </c>
       <c r="I363" t="n">
-        <v>800</v>
+        <v>1000</v>
       </c>
       <c r="J363" t="n">
         <v>83575912</v>
@@ -85855,7 +85855,7 @@
         <v>1085649640</v>
       </c>
       <c r="I364" t="n">
-        <v>12200</v>
+        <v>12400</v>
       </c>
       <c r="J364" t="n">
         <v>18407491</v>
@@ -86090,7 +86090,7 @@
         <v>4135574764</v>
       </c>
       <c r="I365" t="n">
-        <v>1947900</v>
+        <v>1948100</v>
       </c>
       <c r="J365" t="n">
         <v>122578152</v>
@@ -86560,7 +86560,7 @@
         <v>2198386013</v>
       </c>
       <c r="I367" t="n">
-        <v>167100</v>
+        <v>167200</v>
       </c>
       <c r="J367" t="n">
         <v>66002915</v>
@@ -87030,7 +87030,7 @@
         <v>14662793</v>
       </c>
       <c r="I369" t="n">
-        <v>66600</v>
+        <v>67700</v>
       </c>
       <c r="J369" t="n">
         <v>54196747</v>
@@ -87265,7 +87265,7 @@
         <v>17533404702</v>
       </c>
       <c r="I370" t="n">
-        <v>4748600</v>
+        <v>4749600</v>
       </c>
       <c r="J370" t="n">
         <v>599401581</v>
@@ -87500,7 +87500,7 @@
         <v>362854260</v>
       </c>
       <c r="I371" t="n">
-        <v>18700</v>
+        <v>18900</v>
       </c>
       <c r="J371" t="n">
         <v>44000000</v>
@@ -87735,7 +87735,7 @@
         <v>994459625</v>
       </c>
       <c r="I372" t="n">
-        <v>543900</v>
+        <v>544500</v>
       </c>
       <c r="J372" t="n">
         <v>242617538</v>
@@ -87970,7 +87970,7 @@
         <v>4982408436</v>
       </c>
       <c r="I373" t="n">
-        <v>10743500</v>
+        <v>10744500</v>
       </c>
       <c r="J373" t="n">
         <v>500737647</v>
@@ -88205,7 +88205,7 @@
         <v>2175716754</v>
       </c>
       <c r="I374" t="n">
-        <v>389700</v>
+        <v>389900</v>
       </c>
       <c r="J374" t="n">
         <v>132450415</v>
@@ -88910,7 +88910,7 @@
         <v>76153423</v>
       </c>
       <c r="I377" t="n">
-        <v>4800</v>
+        <v>4900</v>
       </c>
       <c r="J377" t="n">
         <v>66086364</v>
@@ -89380,7 +89380,7 @@
         <v>6461338459</v>
       </c>
       <c r="I379" t="n">
-        <v>6400</v>
+        <v>6600</v>
       </c>
       <c r="J379" t="n">
         <v>39059883</v>
@@ -89615,7 +89615,7 @@
         <v>6461338459</v>
       </c>
       <c r="I380" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="J380" t="n">
         <v>2337871</v>
@@ -89850,7 +89850,7 @@
         <v>6461338459</v>
       </c>
       <c r="I381" t="n">
-        <v>164900</v>
+        <v>165000</v>
       </c>
       <c r="J381" t="n">
         <v>71775511</v>
@@ -90085,7 +90085,7 @@
         <v>7438539082</v>
       </c>
       <c r="I382" t="n">
-        <v>492500</v>
+        <v>493500</v>
       </c>
       <c r="J382" t="n">
         <v>705260684</v>
@@ -90320,7 +90320,7 @@
         <v>7438539082</v>
       </c>
       <c r="I383" t="n">
-        <v>7588700</v>
+        <v>7588900</v>
       </c>
       <c r="J383" t="n">
         <v>547752163</v>
@@ -90790,7 +90790,7 @@
         <v>317153892874</v>
       </c>
       <c r="I385" t="n">
-        <v>22933900</v>
+        <v>22934000</v>
       </c>
       <c r="J385" t="n">
         <v>4255762795</v>
@@ -91025,7 +91025,7 @@
         <v>3428051141</v>
       </c>
       <c r="I386" t="n">
-        <v>16086600</v>
+        <v>16087600</v>
       </c>
       <c r="J386" t="n">
         <v>1221826865</v>
@@ -91260,7 +91260,7 @@
         <v>40353396567</v>
       </c>
       <c r="I387" t="n">
-        <v>6127800</v>
+        <v>6128200</v>
       </c>
       <c r="J387" t="n">
         <v>1198563531</v>
@@ -91495,7 +91495,7 @@
         <v>478465780</v>
       </c>
       <c r="I388" t="n">
-        <v>267000</v>
+        <v>271000</v>
       </c>
       <c r="J388" t="n">
         <v>157589984</v>
@@ -91730,7 +91730,7 @@
         <v>4939442927</v>
       </c>
       <c r="I389" t="n">
-        <v>5820000</v>
+        <v>5820100</v>
       </c>
       <c r="J389" t="n">
         <v>236197769</v>
@@ -91965,7 +91965,7 @@
         <v>7383800</v>
       </c>
       <c r="I390" t="n">
-        <v>2300</v>
+        <v>2600</v>
       </c>
       <c r="J390" t="n">
         <v>4880040</v>
@@ -92200,7 +92200,7 @@
         <v>96152066120</v>
       </c>
       <c r="I391" t="n">
-        <v>6414400</v>
+        <v>6414500</v>
       </c>
       <c r="J391" t="n">
         <v>3226546622</v>
@@ -92435,7 +92435,7 @@
         <v>1324484892</v>
       </c>
       <c r="I392" t="n">
-        <v>225400</v>
+        <v>225500</v>
       </c>
       <c r="J392" t="n">
         <v>81836375</v>
@@ -92670,7 +92670,7 @@
         <v>287979075</v>
       </c>
       <c r="I393" t="n">
-        <v>157800</v>
+        <v>157900</v>
       </c>
       <c r="J393" t="n">
         <v>114500510</v>
@@ -92905,7 +92905,7 @@
         <v>1906690341</v>
       </c>
       <c r="I394" t="n">
-        <v>1123600</v>
+        <v>1123700</v>
       </c>
       <c r="J394" t="n">
         <v>149829337</v>
@@ -93140,7 +93140,7 @@
         <v>4342884683</v>
       </c>
       <c r="I395" t="n">
-        <v>2016900</v>
+        <v>2017000</v>
       </c>
       <c r="J395" t="n">
         <v>317982170</v>
@@ -93375,7 +93375,7 @@
         <v>775101630</v>
       </c>
       <c r="I396" t="n">
-        <v>373100</v>
+        <v>373700</v>
       </c>
       <c r="J396" t="n">
         <v>322820608</v>
@@ -93610,7 +93610,7 @@
         <v>199776877500</v>
       </c>
       <c r="I397" t="n">
-        <v>7327800</v>
+        <v>7327900</v>
       </c>
       <c r="J397" t="n">
         <v>4197317998</v>
@@ -94080,7 +94080,7 @@
         <v>5534326335</v>
       </c>
       <c r="I399" t="n">
-        <v>6200</v>
+        <v>8000</v>
       </c>
       <c r="J399" t="n">
         <v>1028700892</v>
@@ -94315,7 +94315,7 @@
         <v>5534326335</v>
       </c>
       <c r="I400" t="n">
-        <v>6900</v>
+        <v>13900</v>
       </c>
       <c r="J400" t="n">
         <v>474085114</v>
@@ -94785,7 +94785,7 @@
         <v>670559797</v>
       </c>
       <c r="I402" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="J402" t="n">
         <v>16571220</v>
@@ -95020,7 +95020,7 @@
         <v>670559797</v>
       </c>
       <c r="I403" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="J403" t="n">
         <v>19843450</v>
@@ -95255,7 +95255,7 @@
         <v>2010398519</v>
       </c>
       <c r="I404" t="n">
-        <v>9219500</v>
+        <v>9219800</v>
       </c>
       <c r="J404" t="n">
         <v>274088851</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-08-17 02:25
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -44375,28 +44375,28 @@
         <v>0</v>
       </c>
       <c r="AP187" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="AQ187" t="n">
-        <v>0.45</v>
+        <v>0</v>
       </c>
       <c r="AR187" t="n">
-        <v>1.59</v>
+        <v>0</v>
       </c>
       <c r="AS187" t="n">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="AT187" t="n">
-        <v>2.41</v>
+        <v>0</v>
       </c>
       <c r="AU187" t="n">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="AV187" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AW187" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX187" t="inlineStr">
         <is>
@@ -44416,7 +44416,7 @@
         <v>0.95</v>
       </c>
       <c r="BC187" t="n">
-        <v>17.19</v>
+        <v>0</v>
       </c>
       <c r="BD187" t="n">
         <v>63.99</v>
@@ -44431,7 +44431,7 @@
         <v>-90.37</v>
       </c>
       <c r="BH187" t="n">
-        <v>74.92</v>
+        <v>-100</v>
       </c>
       <c r="BI187" t="n">
         <v>14.62</v>
@@ -44610,28 +44610,28 @@
         <v>0</v>
       </c>
       <c r="AP188" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="AQ188" t="n">
-        <v>0.45</v>
+        <v>0</v>
       </c>
       <c r="AR188" t="n">
-        <v>1.59</v>
+        <v>0</v>
       </c>
       <c r="AS188" t="n">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="AT188" t="n">
-        <v>2.41</v>
+        <v>0</v>
       </c>
       <c r="AU188" t="n">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="AV188" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AW188" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX188" t="inlineStr">
         <is>
@@ -44651,7 +44651,7 @@
         <v>0.95</v>
       </c>
       <c r="BC188" t="n">
-        <v>17.19</v>
+        <v>0</v>
       </c>
       <c r="BD188" t="n">
         <v>46.68</v>
@@ -44666,7 +44666,7 @@
         <v>-91.39</v>
       </c>
       <c r="BH188" t="n">
-        <v>56.46</v>
+        <v>-100</v>
       </c>
       <c r="BI188" t="n">
         <v>14.62</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-08-23 02:29
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -833,7 +833,7 @@
         <v>887127966</v>
       </c>
       <c r="I2" t="n">
-        <v>20800</v>
+        <v>21000</v>
       </c>
       <c r="J2" t="n">
         <v>152359482</v>
@@ -1015,7 +1015,7 @@
         <v>2.36</v>
       </c>
       <c r="BQ2" t="n">
-        <v>3.01</v>
+        <v>2.98</v>
       </c>
       <c r="BR2" t="n">
         <v>0</v>
@@ -1068,7 +1068,7 @@
         <v>3041859275</v>
       </c>
       <c r="I3" t="n">
-        <v>506700</v>
+        <v>507000</v>
       </c>
       <c r="J3" t="n">
         <v>129510368</v>
@@ -1229,7 +1229,7 @@
         <v>27.39</v>
       </c>
       <c r="BJ3" t="n">
-        <v>1.97</v>
+        <v>0</v>
       </c>
       <c r="BK3" t="n">
         <v>22.74</v>
@@ -1303,7 +1303,7 @@
         <v>232269900000</v>
       </c>
       <c r="I4" t="n">
-        <v>19912500</v>
+        <v>19913900</v>
       </c>
       <c r="J4" t="n">
         <v>15484664889</v>
@@ -1485,7 +1485,7 @@
         <v>11.09</v>
       </c>
       <c r="BQ4" t="n">
-        <v>14.88</v>
+        <v>14.87</v>
       </c>
       <c r="BR4" t="n">
         <v>19.76</v>
@@ -1538,7 +1538,7 @@
         <v>132315990</v>
       </c>
       <c r="I5" t="n">
-        <v>130100</v>
+        <v>130200</v>
       </c>
       <c r="J5" t="n">
         <v>62120196</v>
@@ -1773,7 +1773,7 @@
         <v>472504313</v>
       </c>
       <c r="I6" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="J6" t="n">
         <v>63084700</v>
@@ -2008,7 +2008,7 @@
         <v>1960226121</v>
       </c>
       <c r="I7" t="n">
-        <v>144000</v>
+        <v>144600</v>
       </c>
       <c r="J7" t="n">
         <v>102683444</v>
@@ -2243,7 +2243,7 @@
         <v>26367702</v>
       </c>
       <c r="I8" t="n">
-        <v>17000</v>
+        <v>17300</v>
       </c>
       <c r="J8" t="n">
         <v>18969571</v>
@@ -3183,7 +3183,7 @@
         <v>483646157</v>
       </c>
       <c r="I12" t="n">
-        <v>308500</v>
+        <v>309500</v>
       </c>
       <c r="J12" t="n">
         <v>95961536</v>
@@ -3653,7 +3653,7 @@
         <v>7501479905</v>
       </c>
       <c r="I14" t="n">
-        <v>8200</v>
+        <v>8300</v>
       </c>
       <c r="J14" t="n">
         <v>339510689</v>
@@ -3888,7 +3888,7 @@
         <v>7501479905</v>
       </c>
       <c r="I15" t="n">
-        <v>952400</v>
+        <v>952900</v>
       </c>
       <c r="J15" t="n">
         <v>343551533</v>
@@ -4123,7 +4123,7 @@
         <v>916697788</v>
       </c>
       <c r="I16" t="n">
-        <v>518300</v>
+        <v>518500</v>
       </c>
       <c r="J16" t="n">
         <v>219305733</v>
@@ -4358,7 +4358,7 @@
         <v>10590909436</v>
       </c>
       <c r="I17" t="n">
-        <v>1246700</v>
+        <v>1249700</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -4828,7 +4828,7 @@
         <v>10590909436</v>
       </c>
       <c r="I19" t="n">
-        <v>12200</v>
+        <v>12800</v>
       </c>
       <c r="J19" t="n">
         <v>317386323</v>
@@ -5063,7 +5063,7 @@
         <v>323515266</v>
       </c>
       <c r="I20" t="n">
-        <v>878300</v>
+        <v>879300</v>
       </c>
       <c r="J20" t="n">
         <v>513516302</v>
@@ -5533,7 +5533,7 @@
         <v>933142601</v>
       </c>
       <c r="I22" t="n">
-        <v>1919500</v>
+        <v>1919600</v>
       </c>
       <c r="J22" t="n">
         <v>200245046</v>
@@ -5706,7 +5706,7 @@
         <v>0.67</v>
       </c>
       <c r="BN22" t="n">
-        <v>4.67</v>
+        <v>4.69</v>
       </c>
       <c r="BO22" t="n">
         <v>8.82</v>
@@ -5768,7 +5768,7 @@
         <v>418640859</v>
       </c>
       <c r="I23" t="n">
-        <v>25700</v>
+        <v>26000</v>
       </c>
       <c r="J23" t="n">
         <v>37886057</v>
@@ -6003,7 +6003,7 @@
         <v>957168772</v>
       </c>
       <c r="I24" t="n">
-        <v>15724700</v>
+        <v>15724900</v>
       </c>
       <c r="J24" t="n">
         <v>403868805</v>
@@ -6238,7 +6238,7 @@
         <v>1143429853</v>
       </c>
       <c r="I25" t="n">
-        <v>1459600</v>
+        <v>1459900</v>
       </c>
       <c r="J25" t="n">
         <v>346494097</v>
@@ -6473,7 +6473,7 @@
         <v>11376900683</v>
       </c>
       <c r="I26" t="n">
-        <v>8741800</v>
+        <v>8742700</v>
       </c>
       <c r="J26" t="n">
         <v>1354393401</v>
@@ -6692,7 +6692,7 @@
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>8900</v>
+        <v>9300</v>
       </c>
       <c r="J27" t="n">
         <v>23804898</v>
@@ -6927,7 +6927,7 @@
         <v>7315602837</v>
       </c>
       <c r="I28" t="n">
-        <v>980493</v>
+        <v>980494</v>
       </c>
       <c r="J28" t="n">
         <v>83836843</v>
@@ -7109,7 +7109,7 @@
         <v>46.47</v>
       </c>
       <c r="BQ28" t="n">
-        <v>149</v>
+        <v>148.8</v>
       </c>
       <c r="BR28" t="n">
         <v>0</v>
@@ -7162,7 +7162,7 @@
         <v>10745366459</v>
       </c>
       <c r="I29" t="n">
-        <v>2033300</v>
+        <v>2033400</v>
       </c>
       <c r="J29" t="n">
         <v>1050377974</v>
@@ -7397,7 +7397,7 @@
         <v>66412217</v>
       </c>
       <c r="I30" t="n">
-        <v>1800</v>
+        <v>2100</v>
       </c>
       <c r="J30" t="n">
         <v>7813202</v>
@@ -7632,7 +7632,7 @@
         <v>417217357</v>
       </c>
       <c r="I31" t="n">
-        <v>1640400</v>
+        <v>1640700</v>
       </c>
       <c r="J31" t="n">
         <v>37899458</v>
@@ -7867,7 +7867,7 @@
         <v>417217357</v>
       </c>
       <c r="I32" t="n">
-        <v>13386700</v>
+        <v>13391700</v>
       </c>
       <c r="J32" t="n">
         <v>73325687</v>
@@ -8102,7 +8102,7 @@
         <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>1928200</v>
+        <v>1928300</v>
       </c>
       <c r="J33" t="n">
         <v>40011514</v>
@@ -8337,7 +8337,7 @@
         <v>3126255642</v>
       </c>
       <c r="I34" t="n">
-        <v>4123900</v>
+        <v>4124000</v>
       </c>
       <c r="J34" t="n">
         <v>206489813</v>
@@ -8572,7 +8572,7 @@
         <v>76151685770</v>
       </c>
       <c r="I35" t="n">
-        <v>43621500</v>
+        <v>43621600</v>
       </c>
       <c r="J35" t="n">
         <v>5046500000</v>
@@ -9042,7 +9042,7 @@
         <v>206223442</v>
       </c>
       <c r="I37" t="n">
-        <v>1200</v>
+        <v>1300</v>
       </c>
       <c r="J37" t="n">
         <v>4900000</v>
@@ -9512,7 +9512,7 @@
         <v>3612958552</v>
       </c>
       <c r="I39" t="n">
-        <v>3100</v>
+        <v>3200</v>
       </c>
       <c r="J39" t="n">
         <v>168174945</v>
@@ -9673,10 +9673,10 @@
         <v>129.92</v>
       </c>
       <c r="BJ39" t="n">
-        <v>0.72</v>
+        <v>0</v>
       </c>
       <c r="BK39" t="n">
-        <v>63.99</v>
+        <v>64.45</v>
       </c>
       <c r="BL39" t="n">
         <v>19.15</v>
@@ -9747,7 +9747,7 @@
         <v>105619217078</v>
       </c>
       <c r="I40" t="n">
-        <v>46529700</v>
+        <v>46529800</v>
       </c>
       <c r="J40" t="n">
         <v>5730834040</v>
@@ -9982,7 +9982,7 @@
         <v>171315270385</v>
       </c>
       <c r="I41" t="n">
-        <v>5401700</v>
+        <v>5402200</v>
       </c>
       <c r="J41" t="n">
         <v>5303870781</v>
@@ -10143,10 +10143,10 @@
         <v>16.58</v>
       </c>
       <c r="BJ41" t="n">
-        <v>2.87</v>
+        <v>0</v>
       </c>
       <c r="BK41" t="n">
-        <v>13.93</v>
+        <v>14.33</v>
       </c>
       <c r="BL41" t="n">
         <v>2.04</v>
@@ -10217,7 +10217,7 @@
         <v>171315270385</v>
       </c>
       <c r="I42" t="n">
-        <v>41406100</v>
+        <v>41406200</v>
       </c>
       <c r="J42" t="n">
         <v>5288141247</v>
@@ -10378,10 +10378,10 @@
         <v>16.58</v>
       </c>
       <c r="BJ42" t="n">
-        <v>3.11</v>
+        <v>0</v>
       </c>
       <c r="BK42" t="n">
-        <v>15.75</v>
+        <v>16.24</v>
       </c>
       <c r="BL42" t="n">
         <v>2.04</v>
@@ -10390,7 +10390,7 @@
         <v>2.34</v>
       </c>
       <c r="BN42" t="n">
-        <v>16.28</v>
+        <v>16.29</v>
       </c>
       <c r="BO42" t="n">
         <v>21.35</v>
@@ -10452,7 +10452,7 @@
         <v>72200626143</v>
       </c>
       <c r="I43" t="n">
-        <v>15767000</v>
+        <v>15770200</v>
       </c>
       <c r="J43" t="n">
         <v>1941400000</v>
@@ -10687,7 +10687,7 @@
         <v>6848922</v>
       </c>
       <c r="I44" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="J44" t="n">
         <v>607192</v>
@@ -10922,7 +10922,7 @@
         <v>6848922</v>
       </c>
       <c r="I45" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="J45" t="n">
         <v>992808</v>
@@ -11157,7 +11157,7 @@
         <v>3992158599</v>
       </c>
       <c r="I46" t="n">
-        <v>22044600</v>
+        <v>22044700</v>
       </c>
       <c r="J46" t="n">
         <v>1000540922</v>
@@ -11392,7 +11392,7 @@
         <v>3015971483</v>
       </c>
       <c r="I47" t="n">
-        <v>8500</v>
+        <v>8600</v>
       </c>
       <c r="J47" t="n">
         <v>254106600</v>
@@ -11553,10 +11553,10 @@
         <v>7.04</v>
       </c>
       <c r="BJ47" t="n">
-        <v>0.59</v>
+        <v>0</v>
       </c>
       <c r="BK47" t="n">
-        <v>8.51</v>
+        <v>8.56</v>
       </c>
       <c r="BL47" t="n">
         <v>0.98</v>
@@ -11627,7 +11627,7 @@
         <v>3015971483</v>
       </c>
       <c r="I48" t="n">
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="J48" t="n">
         <v>93397546</v>
@@ -12097,7 +12097,7 @@
         <v>915768000</v>
       </c>
       <c r="I50" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="J50" t="n">
         <v>11540870</v>
@@ -12258,10 +12258,10 @@
         <v>40.31</v>
       </c>
       <c r="BJ50" t="n">
-        <v>-1.27</v>
+        <v>0</v>
       </c>
       <c r="BK50" t="n">
-        <v>32.97</v>
+        <v>32.55</v>
       </c>
       <c r="BL50" t="n">
         <v>6.15</v>
@@ -12551,7 +12551,7 @@
         <v>153843825</v>
       </c>
       <c r="I52" t="n">
-        <v>2100</v>
+        <v>2200</v>
       </c>
       <c r="J52" t="n">
         <v>26633197</v>
@@ -12786,7 +12786,7 @@
         <v>903225826</v>
       </c>
       <c r="I53" t="n">
-        <v>26200</v>
+        <v>26300</v>
       </c>
       <c r="J53" t="n">
         <v>136852484</v>
@@ -13256,7 +13256,7 @@
         <v>6558961758</v>
       </c>
       <c r="I55" t="n">
-        <v>6000</v>
+        <v>6100</v>
       </c>
       <c r="J55" t="n">
         <v>84052790</v>
@@ -13417,10 +13417,10 @@
         <v>21.53</v>
       </c>
       <c r="BJ55" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="BK55" t="n">
-        <v>51.9</v>
+        <v>51.91</v>
       </c>
       <c r="BL55" t="n">
         <v>5.93</v>
@@ -13491,7 +13491,7 @@
         <v>6558961758</v>
       </c>
       <c r="I56" t="n">
-        <v>76600</v>
+        <v>76700</v>
       </c>
       <c r="J56" t="n">
         <v>39675836</v>
@@ -13652,10 +13652,10 @@
         <v>21.53</v>
       </c>
       <c r="BJ56" t="n">
-        <v>-5.51</v>
+        <v>0</v>
       </c>
       <c r="BK56" t="n">
-        <v>65</v>
+        <v>61.42</v>
       </c>
       <c r="BL56" t="n">
         <v>5.93</v>
@@ -13726,7 +13726,7 @@
         <v>1187999130</v>
       </c>
       <c r="I57" t="n">
-        <v>861900</v>
+        <v>864400</v>
       </c>
       <c r="J57" t="n">
         <v>233858065</v>
@@ -14196,7 +14196,7 @@
         <v>92323140</v>
       </c>
       <c r="I59" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="J59" t="n">
         <v>710143</v>
@@ -14357,10 +14357,10 @@
         <v>29.92</v>
       </c>
       <c r="BJ59" t="n">
-        <v>11.05</v>
+        <v>0</v>
       </c>
       <c r="BK59" t="n">
-        <v>17.01</v>
+        <v>18.89</v>
       </c>
       <c r="BL59" t="n">
         <v>1.67</v>
@@ -14431,7 +14431,7 @@
         <v>167147908</v>
       </c>
       <c r="I60" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J60" t="n">
         <v>454750</v>
@@ -14666,7 +14666,7 @@
         <v>1951870998</v>
       </c>
       <c r="I61" t="n">
-        <v>283700</v>
+        <v>284100</v>
       </c>
       <c r="J61" t="n">
         <v>85608392</v>
@@ -14901,7 +14901,7 @@
         <v>10303408831</v>
       </c>
       <c r="I62" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="J62" t="n">
         <v>98699749</v>
@@ -15062,10 +15062,10 @@
         <v>157.26</v>
       </c>
       <c r="BJ62" t="n">
-        <v>-0.71</v>
+        <v>0</v>
       </c>
       <c r="BK62" t="n">
-        <v>107.78</v>
+        <v>107.01</v>
       </c>
       <c r="BL62" t="n">
         <v>28.6</v>
@@ -15136,7 +15136,7 @@
         <v>307401432</v>
       </c>
       <c r="I63" t="n">
-        <v>22800</v>
+        <v>23800</v>
       </c>
       <c r="J63" t="n">
         <v>122894462</v>
@@ -15371,7 +15371,7 @@
         <v>213421593469</v>
       </c>
       <c r="I64" t="n">
-        <v>13336400</v>
+        <v>13336500</v>
       </c>
       <c r="J64" t="n">
         <v>0</v>
@@ -15606,7 +15606,7 @@
         <v>213421593469</v>
       </c>
       <c r="I65" t="n">
-        <v>19900</v>
+        <v>20000</v>
       </c>
       <c r="J65" t="n">
         <v>7298813414</v>
@@ -15841,7 +15841,7 @@
         <v>213421593469</v>
       </c>
       <c r="I66" t="n">
-        <v>5300</v>
+        <v>5400</v>
       </c>
       <c r="J66" t="n">
         <v>2972355254</v>
@@ -16311,7 +16311,7 @@
         <v>7932856945</v>
       </c>
       <c r="I68" t="n">
-        <v>18800</v>
+        <v>18900</v>
       </c>
       <c r="J68" t="n">
         <v>137989898</v>
@@ -16472,10 +16472,10 @@
         <v>23.21</v>
       </c>
       <c r="BJ68" t="n">
-        <v>-0.33</v>
+        <v>0</v>
       </c>
       <c r="BK68" t="n">
-        <v>18.07</v>
+        <v>18.01</v>
       </c>
       <c r="BL68" t="n">
         <v>2.87</v>
@@ -16546,7 +16546,7 @@
         <v>7932856945</v>
       </c>
       <c r="I69" t="n">
-        <v>1424300</v>
+        <v>1426200</v>
       </c>
       <c r="J69" t="n">
         <v>255106712</v>
@@ -16710,7 +16710,7 @@
         <v>0</v>
       </c>
       <c r="BK69" t="n">
-        <v>20.42</v>
+        <v>21.03</v>
       </c>
       <c r="BL69" t="n">
         <v>2.87</v>
@@ -16781,7 +16781,7 @@
         <v>8733675005</v>
       </c>
       <c r="I70" t="n">
-        <v>4306800</v>
+        <v>4307300</v>
       </c>
       <c r="J70" t="n">
         <v>464557268</v>
@@ -17016,7 +17016,7 @@
         <v>1275696499</v>
       </c>
       <c r="I71" t="n">
-        <v>348200</v>
+        <v>348500</v>
       </c>
       <c r="J71" t="n">
         <v>0</v>
@@ -17251,7 +17251,7 @@
         <v>3625167239</v>
       </c>
       <c r="I72" t="n">
-        <v>93300</v>
+        <v>93400</v>
       </c>
       <c r="J72" t="n">
         <v>451668652</v>
@@ -17486,7 +17486,7 @@
         <v>3625167239</v>
       </c>
       <c r="I73" t="n">
-        <v>11288700</v>
+        <v>11289300</v>
       </c>
       <c r="J73" t="n">
         <v>345060392</v>
@@ -18117,10 +18117,10 @@
         <v>27.14</v>
       </c>
       <c r="BJ75" t="n">
-        <v>0.54</v>
+        <v>0</v>
       </c>
       <c r="BK75" t="n">
-        <v>16.7</v>
+        <v>16.79</v>
       </c>
       <c r="BL75" t="n">
         <v>3.11</v>
@@ -18426,7 +18426,7 @@
         <v>6215608912</v>
       </c>
       <c r="I77" t="n">
-        <v>1186800</v>
+        <v>1186900</v>
       </c>
       <c r="J77" t="n">
         <v>202536545</v>
@@ -18587,10 +18587,10 @@
         <v>27.14</v>
       </c>
       <c r="BJ77" t="n">
-        <v>1.75</v>
+        <v>0</v>
       </c>
       <c r="BK77" t="n">
-        <v>13.13</v>
+        <v>13.36</v>
       </c>
       <c r="BL77" t="n">
         <v>3.11</v>
@@ -18661,7 +18661,7 @@
         <v>1208900971</v>
       </c>
       <c r="I78" t="n">
-        <v>197000</v>
+        <v>198000</v>
       </c>
       <c r="J78" t="n">
         <v>438007537</v>
@@ -19057,10 +19057,10 @@
         <v>8.199999999999999</v>
       </c>
       <c r="BJ79" t="n">
-        <v>0.74</v>
+        <v>0</v>
       </c>
       <c r="BK79" t="n">
-        <v>2.71</v>
+        <v>2.73</v>
       </c>
       <c r="BL79" t="n">
         <v>1.66</v>
@@ -19131,7 +19131,7 @@
         <v>5766791980</v>
       </c>
       <c r="I80" t="n">
-        <v>3700</v>
+        <v>3800</v>
       </c>
       <c r="J80" t="n">
         <v>166059947</v>
@@ -19295,7 +19295,7 @@
         <v>0</v>
       </c>
       <c r="BK80" t="n">
-        <v>2.64</v>
+        <v>2.68</v>
       </c>
       <c r="BL80" t="n">
         <v>1.66</v>
@@ -19601,7 +19601,7 @@
         <v>342428200</v>
       </c>
       <c r="I82" t="n">
-        <v>20900</v>
+        <v>21000</v>
       </c>
       <c r="J82" t="n">
         <v>42275080</v>
@@ -19836,7 +19836,7 @@
         <v>1718499946</v>
       </c>
       <c r="I83" t="n">
-        <v>856000</v>
+        <v>856200</v>
       </c>
       <c r="J83" t="n">
         <v>350000000</v>
@@ -20071,7 +20071,7 @@
         <v>583362070</v>
       </c>
       <c r="I84" t="n">
-        <v>3761200</v>
+        <v>3761400</v>
       </c>
       <c r="J84" t="n">
         <v>104171852</v>
@@ -20541,7 +20541,7 @@
         <v>7278991866</v>
       </c>
       <c r="I86" t="n">
-        <v>1957800</v>
+        <v>1957900</v>
       </c>
       <c r="J86" t="n">
         <v>651072697</v>
@@ -21246,7 +21246,7 @@
         <v>1799106457</v>
       </c>
       <c r="I89" t="n">
-        <v>16200</v>
+        <v>16500</v>
       </c>
       <c r="J89" t="n">
         <v>35920890</v>
@@ -21481,7 +21481,7 @@
         <v>1799106457</v>
       </c>
       <c r="I90" t="n">
-        <v>3900</v>
+        <v>4200</v>
       </c>
       <c r="J90" t="n">
         <v>6565010</v>
@@ -21716,7 +21716,7 @@
         <v>1799106457</v>
       </c>
       <c r="I91" t="n">
-        <v>1400</v>
+        <v>1600</v>
       </c>
       <c r="J91" t="n">
         <v>29596015</v>
@@ -22186,7 +22186,7 @@
         <v>73314660</v>
       </c>
       <c r="I93" t="n">
-        <v>8000</v>
+        <v>12000</v>
       </c>
       <c r="J93" t="n">
         <v>4292896</v>
@@ -22421,7 +22421,7 @@
         <v>8126292000</v>
       </c>
       <c r="I94" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="J94" t="n">
         <v>151997609</v>
@@ -23831,7 +23831,7 @@
         <v>16283712699</v>
       </c>
       <c r="I100" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="J100" t="n">
         <v>28657819</v>
@@ -24066,7 +24066,7 @@
         <v>600585281</v>
       </c>
       <c r="I101" t="n">
-        <v>6000</v>
+        <v>6100</v>
       </c>
       <c r="J101" t="n">
         <v>10759335</v>
@@ -24301,7 +24301,7 @@
         <v>600585281</v>
       </c>
       <c r="I102" t="n">
-        <v>4200</v>
+        <v>4300</v>
       </c>
       <c r="J102" t="n">
         <v>14690740</v>
@@ -24536,7 +24536,7 @@
         <v>5506742344</v>
       </c>
       <c r="I103" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="J103" t="n">
         <v>15527137</v>
@@ -24771,7 +24771,7 @@
         <v>5506742344</v>
       </c>
       <c r="I104" t="n">
-        <v>3900</v>
+        <v>4000</v>
       </c>
       <c r="J104" t="n">
         <v>23044454</v>
@@ -25241,7 +25241,7 @@
         <v>33597163112</v>
       </c>
       <c r="I106" t="n">
-        <v>14179700</v>
+        <v>14179800</v>
       </c>
       <c r="J106" t="n">
         <v>1905179984</v>
@@ -25476,7 +25476,7 @@
         <v>32049060118</v>
       </c>
       <c r="I107" t="n">
-        <v>8746100</v>
+        <v>8746200</v>
       </c>
       <c r="J107" t="n">
         <v>5432044538</v>
@@ -25946,7 +25946,7 @@
         <v>2568763842</v>
       </c>
       <c r="I109" t="n">
-        <v>7300</v>
+        <v>7500</v>
       </c>
       <c r="J109" t="n">
         <v>31210514</v>
@@ -26416,7 +26416,7 @@
         <v>48763388928</v>
       </c>
       <c r="I111" t="n">
-        <v>1010800</v>
+        <v>1010900</v>
       </c>
       <c r="J111" t="n">
         <v>1152254440</v>
@@ -26651,7 +26651,7 @@
         <v>42206760362</v>
       </c>
       <c r="I112" t="n">
-        <v>13743100</v>
+        <v>13743200</v>
       </c>
       <c r="J112" t="n">
         <v>2982810590</v>
@@ -27121,7 +27121,7 @@
         <v>360424285</v>
       </c>
       <c r="I114" t="n">
-        <v>18200</v>
+        <v>18300</v>
       </c>
       <c r="J114" t="n">
         <v>12342238</v>
@@ -27591,7 +27591,7 @@
         <v>14438311576</v>
       </c>
       <c r="I116" t="n">
-        <v>37679000</v>
+        <v>37679100</v>
       </c>
       <c r="J116" t="n">
         <v>3966570932</v>
@@ -27826,7 +27826,7 @@
         <v>1571178585</v>
       </c>
       <c r="I117" t="n">
-        <v>167200</v>
+        <v>167300</v>
       </c>
       <c r="J117" t="n">
         <v>364542552</v>
@@ -28061,7 +28061,7 @@
         <v>20723793950</v>
       </c>
       <c r="I118" t="n">
-        <v>3877000</v>
+        <v>3877100</v>
       </c>
       <c r="J118" t="n">
         <v>380253069</v>
@@ -28296,7 +28296,7 @@
         <v>6351985419</v>
       </c>
       <c r="I119" t="n">
-        <v>17103400</v>
+        <v>17104400</v>
       </c>
       <c r="J119" t="n">
         <v>1326093947</v>
@@ -28531,7 +28531,7 @@
         <v>552178001</v>
       </c>
       <c r="I120" t="n">
-        <v>54700</v>
+        <v>54800</v>
       </c>
       <c r="J120" t="n">
         <v>41800000</v>
@@ -29941,7 +29941,7 @@
         <v>9210620132</v>
       </c>
       <c r="I126" t="n">
-        <v>3707600</v>
+        <v>3707900</v>
       </c>
       <c r="J126" t="n">
         <v>308047594</v>
@@ -30176,7 +30176,7 @@
         <v>819922085</v>
       </c>
       <c r="I127" t="n">
-        <v>12421100</v>
+        <v>12451100</v>
       </c>
       <c r="J127" t="n">
         <v>525591097</v>
@@ -30881,7 +30881,7 @@
         <v>3237915384</v>
       </c>
       <c r="I130" t="n">
-        <v>1770200</v>
+        <v>1770400</v>
       </c>
       <c r="J130" t="n">
         <v>1255007048</v>
@@ -31351,7 +31351,7 @@
         <v>830510256</v>
       </c>
       <c r="I132" t="n">
-        <v>54200</v>
+        <v>55000</v>
       </c>
       <c r="J132" t="n">
         <v>116481187</v>
@@ -32056,7 +32056,7 @@
         <v>317785908</v>
       </c>
       <c r="I135" t="n">
-        <v>53500</v>
+        <v>53700</v>
       </c>
       <c r="J135" t="n">
         <v>50602842</v>
@@ -32291,7 +32291,7 @@
         <v>429027000</v>
       </c>
       <c r="I136" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="J136" t="n">
         <v>54467820</v>
@@ -32761,7 +32761,7 @@
         <v>118965196</v>
       </c>
       <c r="I138" t="n">
-        <v>195800</v>
+        <v>203600</v>
       </c>
       <c r="J138" t="n">
         <v>13321978</v>
@@ -33231,7 +33231,7 @@
         <v>4585979948</v>
       </c>
       <c r="I140" t="n">
-        <v>1360200</v>
+        <v>1360300</v>
       </c>
       <c r="J140" t="n">
         <v>919034196</v>
@@ -33466,7 +33466,7 @@
         <v>246611740</v>
       </c>
       <c r="I141" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="J141" t="n">
         <v>9750000</v>
@@ -33701,7 +33701,7 @@
         <v>246611740</v>
       </c>
       <c r="I142" t="n">
-        <v>1600</v>
+        <v>1700</v>
       </c>
       <c r="J142" t="n">
         <v>12750000</v>
@@ -33936,7 +33936,7 @@
         <v>4658475168</v>
       </c>
       <c r="I143" t="n">
-        <v>9382500</v>
+        <v>9382600</v>
       </c>
       <c r="J143" t="n">
         <v>696334224</v>
@@ -34641,7 +34641,7 @@
         <v>8605753000</v>
       </c>
       <c r="I146" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="J146" t="n">
         <v>101878293</v>
@@ -35111,7 +35111,7 @@
         <v>1175285322</v>
       </c>
       <c r="I148" t="n">
-        <v>600</v>
+        <v>800</v>
       </c>
       <c r="J148" t="n">
         <v>22241700</v>
@@ -35346,7 +35346,7 @@
         <v>49309249746</v>
       </c>
       <c r="I149" t="n">
-        <v>27481200</v>
+        <v>27481600</v>
       </c>
       <c r="J149" t="n">
         <v>1937029517</v>
@@ -35581,7 +35581,7 @@
         <v>24543083964</v>
       </c>
       <c r="I150" t="n">
-        <v>2492300</v>
+        <v>2492400</v>
       </c>
       <c r="J150" t="n">
         <v>0</v>
@@ -35816,7 +35816,7 @@
         <v>24543083964</v>
       </c>
       <c r="I151" t="n">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="J151" t="n">
         <v>975954372</v>
@@ -36051,7 +36051,7 @@
         <v>24543083964</v>
       </c>
       <c r="I152" t="n">
-        <v>6600</v>
+        <v>6800</v>
       </c>
       <c r="J152" t="n">
         <v>1542412758</v>
@@ -36286,7 +36286,7 @@
         <v>157863779</v>
       </c>
       <c r="I153" t="n">
-        <v>922100</v>
+        <v>923000</v>
       </c>
       <c r="J153" t="n">
         <v>205017990</v>
@@ -36521,7 +36521,7 @@
         <v>6918130932</v>
       </c>
       <c r="I154" t="n">
-        <v>5100</v>
+        <v>5300</v>
       </c>
       <c r="J154" t="n">
         <v>75529774</v>
@@ -36756,7 +36756,7 @@
         <v>6918130932</v>
       </c>
       <c r="I155" t="n">
-        <v>2300</v>
+        <v>2400</v>
       </c>
       <c r="J155" t="n">
         <v>143412165</v>
@@ -37226,7 +37226,7 @@
         <v>39678410</v>
       </c>
       <c r="I157" t="n">
-        <v>2600</v>
+        <v>2700</v>
       </c>
       <c r="J157" t="n">
         <v>2204620569</v>
@@ -38166,7 +38166,7 @@
         <v>45048273566</v>
       </c>
       <c r="I161" t="n">
-        <v>15802500</v>
+        <v>15802600</v>
       </c>
       <c r="J161" t="n">
         <v>1259387047</v>
@@ -38401,7 +38401,7 @@
         <v>253357531</v>
       </c>
       <c r="I162" t="n">
-        <v>48000</v>
+        <v>48100</v>
       </c>
       <c r="J162" t="n">
         <v>36142306</v>
@@ -39106,7 +39106,7 @@
         <v>230426569</v>
       </c>
       <c r="I165" t="n">
-        <v>22000</v>
+        <v>22300</v>
       </c>
       <c r="J165" t="n">
         <v>61776575</v>
@@ -39341,7 +39341,7 @@
         <v>1957625510</v>
       </c>
       <c r="I166" t="n">
-        <v>1600</v>
+        <v>1900</v>
       </c>
       <c r="J166" t="n">
         <v>31257700</v>
@@ -39576,7 +39576,7 @@
         <v>1957625510</v>
       </c>
       <c r="I167" t="n">
-        <v>118000</v>
+        <v>118100</v>
       </c>
       <c r="J167" t="n">
         <v>61361556</v>
@@ -39811,7 +39811,7 @@
         <v>856000041</v>
       </c>
       <c r="I168" t="n">
-        <v>1417500</v>
+        <v>1417700</v>
       </c>
       <c r="J168" t="n">
         <v>200000000</v>
@@ -40046,7 +40046,7 @@
         <v>3125834929</v>
       </c>
       <c r="I169" t="n">
-        <v>6322500</v>
+        <v>6322700</v>
       </c>
       <c r="J169" t="n">
         <v>277359027</v>
@@ -40281,7 +40281,7 @@
         <v>2401866849</v>
       </c>
       <c r="I170" t="n">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="J170" t="n">
         <v>117725000</v>
@@ -40516,7 +40516,7 @@
         <v>2401866849</v>
       </c>
       <c r="I171" t="n">
-        <v>1848100</v>
+        <v>1848700</v>
       </c>
       <c r="J171" t="n">
         <v>235450000</v>
@@ -40751,7 +40751,7 @@
         <v>184730508</v>
       </c>
       <c r="I172" t="n">
-        <v>1400</v>
+        <v>1500</v>
       </c>
       <c r="J172" t="n">
         <v>53857284</v>
@@ -40986,7 +40986,7 @@
         <v>9234146</v>
       </c>
       <c r="I173" t="n">
-        <v>5000</v>
+        <v>5200</v>
       </c>
       <c r="J173" t="n">
         <v>43862205</v>
@@ -41691,7 +41691,7 @@
         <v>10221528046</v>
       </c>
       <c r="I176" t="n">
-        <v>8766200</v>
+        <v>8766300</v>
       </c>
       <c r="J176" t="n">
         <v>547191026</v>
@@ -41926,7 +41926,7 @@
         <v>6531807616</v>
       </c>
       <c r="I177" t="n">
-        <v>189400</v>
+        <v>190200</v>
       </c>
       <c r="J177" t="n">
         <v>280335091</v>
@@ -42396,7 +42396,7 @@
         <v>0</v>
       </c>
       <c r="I179" t="n">
-        <v>13904</v>
+        <v>13906</v>
       </c>
       <c r="J179" t="n">
         <v>49031062</v>
@@ -43101,7 +43101,7 @@
         <v>34621157</v>
       </c>
       <c r="I182" t="n">
-        <v>3756100</v>
+        <v>3758600</v>
       </c>
       <c r="J182" t="n">
         <v>157368961</v>
@@ -43336,7 +43336,7 @@
         <v>41640648132</v>
       </c>
       <c r="I183" t="n">
-        <v>27700</v>
+        <v>27800</v>
       </c>
       <c r="J183" t="n">
         <v>716975719</v>
@@ -43571,7 +43571,7 @@
         <v>41640648132</v>
       </c>
       <c r="I184" t="n">
-        <v>14608300</v>
+        <v>14608700</v>
       </c>
       <c r="J184" t="n">
         <v>1261042330</v>
@@ -43806,7 +43806,7 @@
         <v>9103441336</v>
       </c>
       <c r="I185" t="n">
-        <v>4686700</v>
+        <v>4688900</v>
       </c>
       <c r="J185" t="n">
         <v>752350487</v>
@@ -44041,7 +44041,7 @@
         <v>9560322019</v>
       </c>
       <c r="I186" t="n">
-        <v>7821600</v>
+        <v>7821700</v>
       </c>
       <c r="J186" t="n">
         <v>2303692568</v>
@@ -44276,7 +44276,7 @@
         <v>12613191438</v>
       </c>
       <c r="I187" t="n">
-        <v>52300</v>
+        <v>52400</v>
       </c>
       <c r="J187" t="n">
         <v>486802764</v>
@@ -44511,7 +44511,7 @@
         <v>12613191438</v>
       </c>
       <c r="I188" t="n">
-        <v>12182900</v>
+        <v>12183000</v>
       </c>
       <c r="J188" t="n">
         <v>835885284</v>
@@ -44981,7 +44981,7 @@
         <v>3238754322</v>
       </c>
       <c r="I190" t="n">
-        <v>1713800</v>
+        <v>1713900</v>
       </c>
       <c r="J190" t="n">
         <v>902160000</v>
@@ -45451,7 +45451,7 @@
         <v>22932784</v>
       </c>
       <c r="I192" t="n">
-        <v>11600</v>
+        <v>12600</v>
       </c>
       <c r="J192" t="n">
         <v>3966667</v>
@@ -45686,7 +45686,7 @@
         <v>22932784</v>
       </c>
       <c r="I193" t="n">
-        <v>87100</v>
+        <v>87400</v>
       </c>
       <c r="J193" t="n">
         <v>7933333</v>
@@ -45921,7 +45921,7 @@
         <v>3287205412</v>
       </c>
       <c r="I194" t="n">
-        <v>18069200</v>
+        <v>18070200</v>
       </c>
       <c r="J194" t="n">
         <v>502630884</v>
@@ -46156,7 +46156,7 @@
         <v>244947335</v>
       </c>
       <c r="I195" t="n">
-        <v>288400</v>
+        <v>288600</v>
       </c>
       <c r="J195" t="n">
         <v>133851072</v>
@@ -46391,7 +46391,7 @@
         <v>232175025</v>
       </c>
       <c r="I196" t="n">
-        <v>536900</v>
+        <v>538300</v>
       </c>
       <c r="J196" t="n">
         <v>103188981</v>
@@ -46626,7 +46626,7 @@
         <v>4734129385</v>
       </c>
       <c r="I197" t="n">
-        <v>2236000</v>
+        <v>2238500</v>
       </c>
       <c r="J197" t="n">
         <v>1360382643</v>
@@ -47566,7 +47566,7 @@
         <v>135588387</v>
       </c>
       <c r="I201" t="n">
-        <v>2700</v>
+        <v>2800</v>
       </c>
       <c r="J201" t="n">
         <v>7894494</v>
@@ -48014,7 +48014,7 @@
       <c r="E203" t="inlineStr"/>
       <c r="F203" t="inlineStr"/>
       <c r="G203" t="n">
-        <v>171031.73</v>
+        <v>170448.88</v>
       </c>
       <c r="H203" t="n">
         <v>0</v>
@@ -48181,7 +48181,7 @@
         <v>0</v>
       </c>
       <c r="BJ203" t="n">
-        <v>0</v>
+        <v>-0.34</v>
       </c>
       <c r="BK203" t="n">
         <v>171031.73</v>
@@ -48193,7 +48193,7 @@
         <v>0</v>
       </c>
       <c r="BN203" t="n">
-        <v>171979.78</v>
+        <v>170448.88</v>
       </c>
       <c r="BO203" t="n">
         <v>199354.81</v>
@@ -48202,7 +48202,7 @@
         <v>133874.44</v>
       </c>
       <c r="BQ203" t="n">
-        <v>167928.33</v>
+        <v>170448.88</v>
       </c>
       <c r="BR203" t="n">
         <v>0</v>
@@ -48725,7 +48725,7 @@
         <v>6828200865</v>
       </c>
       <c r="I206" t="n">
-        <v>24800</v>
+        <v>25600</v>
       </c>
       <c r="J206" t="n">
         <v>770992429</v>
@@ -49195,7 +49195,7 @@
         <v>75668118</v>
       </c>
       <c r="I208" t="n">
-        <v>2900</v>
+        <v>4500</v>
       </c>
       <c r="J208" t="n">
         <v>41772224</v>
@@ -49430,7 +49430,7 @@
         <v>75668118</v>
       </c>
       <c r="I209" t="n">
-        <v>5600</v>
+        <v>5700</v>
       </c>
       <c r="J209" t="n">
         <v>12627232</v>
@@ -49665,7 +49665,7 @@
         <v>4606212203</v>
       </c>
       <c r="I210" t="n">
-        <v>2234000</v>
+        <v>2234800</v>
       </c>
       <c r="J210" t="n">
         <v>327611110</v>
@@ -49900,7 +49900,7 @@
         <v>4092144000</v>
       </c>
       <c r="I211" t="n">
-        <v>883400</v>
+        <v>883500</v>
       </c>
       <c r="J211" t="n">
         <v>81422761</v>
@@ -50061,10 +50061,10 @@
         <v>65.09</v>
       </c>
       <c r="BJ211" t="n">
-        <v>1.01</v>
+        <v>0</v>
       </c>
       <c r="BK211" t="n">
-        <v>49.5</v>
+        <v>50</v>
       </c>
       <c r="BL211" t="n">
         <v>6.54</v>
@@ -50135,7 +50135,7 @@
         <v>19418510375</v>
       </c>
       <c r="I212" t="n">
-        <v>24900</v>
+        <v>25000</v>
       </c>
       <c r="J212" t="n">
         <v>238170004</v>
@@ -50370,7 +50370,7 @@
         <v>19418510375</v>
       </c>
       <c r="I213" t="n">
-        <v>1855900</v>
+        <v>1857400</v>
       </c>
       <c r="J213" t="n">
         <v>465157744</v>
@@ -50766,10 +50766,10 @@
         <v>8.24</v>
       </c>
       <c r="BJ214" t="n">
-        <v>2.78</v>
+        <v>0</v>
       </c>
       <c r="BK214" t="n">
-        <v>12.6</v>
+        <v>12.95</v>
       </c>
       <c r="BL214" t="n">
         <v>1.42</v>
@@ -50840,7 +50840,7 @@
         <v>141791125000</v>
       </c>
       <c r="I215" t="n">
-        <v>30759300</v>
+        <v>30761200</v>
       </c>
       <c r="J215" t="n">
         <v>7360052833</v>
@@ -51001,10 +51001,10 @@
         <v>8.24</v>
       </c>
       <c r="BJ215" t="n">
-        <v>2.54</v>
+        <v>0</v>
       </c>
       <c r="BK215" t="n">
-        <v>12.19</v>
+        <v>12.5</v>
       </c>
       <c r="BL215" t="n">
         <v>1.42</v>
@@ -51075,7 +51075,7 @@
         <v>441939488529</v>
       </c>
       <c r="I216" t="n">
-        <v>1649900</v>
+        <v>1650000</v>
       </c>
       <c r="J216" t="n">
         <v>5617742977</v>
@@ -51236,10 +51236,10 @@
         <v>19.49</v>
       </c>
       <c r="BJ216" t="n">
-        <v>2.63</v>
+        <v>0</v>
       </c>
       <c r="BK216" t="n">
-        <v>40.33</v>
+        <v>41.39</v>
       </c>
       <c r="BL216" t="n">
         <v>3.97</v>
@@ -51310,7 +51310,7 @@
         <v>441939488529</v>
       </c>
       <c r="I217" t="n">
-        <v>29492600</v>
+        <v>29493100</v>
       </c>
       <c r="J217" t="n">
         <v>5409126215</v>
@@ -51471,10 +51471,10 @@
         <v>19.49</v>
       </c>
       <c r="BJ217" t="n">
-        <v>2.91</v>
+        <v>0</v>
       </c>
       <c r="BK217" t="n">
-        <v>37.51</v>
+        <v>38.6</v>
       </c>
       <c r="BL217" t="n">
         <v>3.97</v>
@@ -51545,7 +51545,7 @@
         <v>743677424</v>
       </c>
       <c r="I218" t="n">
-        <v>1427400</v>
+        <v>1427700</v>
       </c>
       <c r="J218" t="n">
         <v>303541864</v>
@@ -52015,7 +52015,7 @@
         <v>6946961871</v>
       </c>
       <c r="I220" t="n">
-        <v>3922900</v>
+        <v>3924900</v>
       </c>
       <c r="J220" t="n">
         <v>683756108</v>
@@ -52720,7 +52720,7 @@
         <v>1495332446</v>
       </c>
       <c r="I223" t="n">
-        <v>969200</v>
+        <v>969300</v>
       </c>
       <c r="J223" t="n">
         <v>286431078</v>
@@ -52955,7 +52955,7 @@
         <v>1101684233</v>
       </c>
       <c r="I224" t="n">
-        <v>2113400</v>
+        <v>2113700</v>
       </c>
       <c r="J224" t="n">
         <v>179720130</v>
@@ -53190,7 +53190,7 @@
         <v>23297804422</v>
       </c>
       <c r="I225" t="n">
-        <v>6382400</v>
+        <v>6385000</v>
       </c>
       <c r="J225" t="n">
         <v>0</v>
@@ -53660,7 +53660,7 @@
         <v>23297804422</v>
       </c>
       <c r="I227" t="n">
-        <v>4556300</v>
+        <v>4556800</v>
       </c>
       <c r="J227" t="n">
         <v>3928678381</v>
@@ -53895,7 +53895,7 @@
         <v>867967133</v>
       </c>
       <c r="I228" t="n">
-        <v>25000</v>
+        <v>25100</v>
       </c>
       <c r="J228" t="n">
         <v>96226962</v>
@@ -54130,7 +54130,7 @@
         <v>1903530037</v>
       </c>
       <c r="I229" t="n">
-        <v>325900</v>
+        <v>326200</v>
       </c>
       <c r="J229" t="n">
         <v>195434352</v>
@@ -54365,7 +54365,7 @@
         <v>4367063523</v>
       </c>
       <c r="I230" t="n">
-        <v>181000</v>
+        <v>181500</v>
       </c>
       <c r="J230" t="n">
         <v>135539000</v>
@@ -54600,7 +54600,7 @@
         <v>1967513719</v>
       </c>
       <c r="I231" t="n">
-        <v>2767700</v>
+        <v>2768200</v>
       </c>
       <c r="J231" t="n">
         <v>1609809601</v>
@@ -54835,7 +54835,7 @@
         <v>215193880</v>
       </c>
       <c r="I232" t="n">
-        <v>2885100</v>
+        <v>2892000</v>
       </c>
       <c r="J232" t="n">
         <v>206917263</v>
@@ -55070,7 +55070,7 @@
         <v>2050632807</v>
       </c>
       <c r="I233" t="n">
-        <v>380500</v>
+        <v>380600</v>
       </c>
       <c r="J233" t="n">
         <v>87859154</v>
@@ -55305,7 +55305,7 @@
         <v>3004579200</v>
       </c>
       <c r="I234" t="n">
-        <v>20300</v>
+        <v>20500</v>
       </c>
       <c r="J234" t="n">
         <v>107306486</v>
@@ -55540,7 +55540,7 @@
         <v>187394339</v>
       </c>
       <c r="I235" t="n">
-        <v>208100</v>
+        <v>209100</v>
       </c>
       <c r="J235" t="n">
         <v>147554631</v>
@@ -55775,7 +55775,7 @@
         <v>11065215329</v>
       </c>
       <c r="I236" t="n">
-        <v>19170900</v>
+        <v>19171800</v>
       </c>
       <c r="J236" t="n">
         <v>1006845095</v>
@@ -55936,10 +55936,10 @@
         <v>10.07</v>
       </c>
       <c r="BJ236" t="n">
-        <v>4.67</v>
+        <v>0</v>
       </c>
       <c r="BK236" t="n">
-        <v>10.5</v>
+        <v>10.99</v>
       </c>
       <c r="BL236" t="n">
         <v>1.38</v>
@@ -56010,7 +56010,7 @@
         <v>18643331</v>
       </c>
       <c r="I237" t="n">
-        <v>16200</v>
+        <v>16300</v>
       </c>
       <c r="J237" t="n">
         <v>46687694</v>
@@ -56245,7 +56245,7 @@
         <v>106829782</v>
       </c>
       <c r="I238" t="n">
-        <v>8200</v>
+        <v>12700</v>
       </c>
       <c r="J238" t="n">
         <v>23184000</v>
@@ -56480,7 +56480,7 @@
         <v>2308358845</v>
       </c>
       <c r="I239" t="n">
-        <v>2315500</v>
+        <v>2317300</v>
       </c>
       <c r="J239" t="n">
         <v>568561350</v>
@@ -57185,7 +57185,7 @@
         <v>1647730597</v>
       </c>
       <c r="I242" t="n">
-        <v>126100</v>
+        <v>126900</v>
       </c>
       <c r="J242" t="n">
         <v>333548825</v>
@@ -57420,7 +57420,7 @@
         <v>5864699741</v>
       </c>
       <c r="I243" t="n">
-        <v>1078400</v>
+        <v>1078500</v>
       </c>
       <c r="J243" t="n">
         <v>339000000</v>
@@ -57655,7 +57655,7 @@
         <v>2450078216</v>
       </c>
       <c r="I244" t="n">
-        <v>690800</v>
+        <v>691200</v>
       </c>
       <c r="J244" t="n">
         <v>104214394</v>
@@ -57890,7 +57890,7 @@
         <v>197806715</v>
       </c>
       <c r="I245" t="n">
-        <v>326900</v>
+        <v>327000</v>
       </c>
       <c r="J245" t="n">
         <v>286676540</v>
@@ -58125,7 +58125,7 @@
         <v>573428648</v>
       </c>
       <c r="I246" t="n">
-        <v>752000</v>
+        <v>752200</v>
       </c>
       <c r="J246" t="n">
         <v>206269341</v>
@@ -58360,7 +58360,7 @@
         <v>19100075</v>
       </c>
       <c r="I247" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="J247" t="n">
         <v>3715969</v>
@@ -58595,7 +58595,7 @@
         <v>3227931497</v>
       </c>
       <c r="I248" t="n">
-        <v>34903700</v>
+        <v>34903900</v>
       </c>
       <c r="J248" t="n">
         <v>775945010</v>
@@ -58756,10 +58756,10 @@
         <v>14.38</v>
       </c>
       <c r="BJ248" t="n">
-        <v>7.22</v>
+        <v>0</v>
       </c>
       <c r="BK248" t="n">
-        <v>3.88</v>
+        <v>4.16</v>
       </c>
       <c r="BL248" t="n">
         <v>0.47</v>
@@ -58830,7 +58830,7 @@
         <v>3665834000</v>
       </c>
       <c r="I249" t="n">
-        <v>369100</v>
+        <v>369600</v>
       </c>
       <c r="J249" t="n">
         <v>234238661</v>
@@ -59065,7 +59065,7 @@
         <v>1485175543</v>
       </c>
       <c r="I250" t="n">
-        <v>1533100</v>
+        <v>1534500</v>
       </c>
       <c r="J250" t="n">
         <v>820539225</v>
@@ -59770,7 +59770,7 @@
         <v>175503202</v>
       </c>
       <c r="I253" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="J253" t="n">
         <v>9921040</v>
@@ -60005,7 +60005,7 @@
         <v>293944089</v>
       </c>
       <c r="I254" t="n">
-        <v>3300</v>
+        <v>3500</v>
       </c>
       <c r="J254" t="n">
         <v>71001000</v>
@@ -60240,7 +60240,7 @@
         <v>29289985500</v>
       </c>
       <c r="I255" t="n">
-        <v>24240500</v>
+        <v>24240600</v>
       </c>
       <c r="J255" t="n">
         <v>2020000000</v>
@@ -60475,7 +60475,7 @@
         <v>3026628647</v>
       </c>
       <c r="I256" t="n">
-        <v>6554000</v>
+        <v>6554300</v>
       </c>
       <c r="J256" t="n">
         <v>402158941</v>
@@ -61415,7 +61415,7 @@
         <v>2864834307</v>
       </c>
       <c r="I260" t="n">
-        <v>12338400</v>
+        <v>12338500</v>
       </c>
       <c r="J260" t="n">
         <v>562835771</v>
@@ -62120,7 +62120,7 @@
         <v>315208906</v>
       </c>
       <c r="I263" t="n">
-        <v>829800</v>
+        <v>832700</v>
       </c>
       <c r="J263" t="n">
         <v>105774820</v>
@@ -62590,7 +62590,7 @@
         <v>447634480</v>
       </c>
       <c r="I265" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="J265" t="n">
         <v>4577200</v>
@@ -62825,7 +62825,7 @@
         <v>13783571923</v>
       </c>
       <c r="I266" t="n">
-        <v>4737600</v>
+        <v>4739300</v>
       </c>
       <c r="J266" t="n">
         <v>513163701</v>
@@ -63530,7 +63530,7 @@
         <v>1397311187</v>
       </c>
       <c r="I269" t="n">
-        <v>1026600</v>
+        <v>1028600</v>
       </c>
       <c r="J269" t="n">
         <v>153719601</v>
@@ -63765,7 +63765,7 @@
         <v>6134359</v>
       </c>
       <c r="I270" t="n">
-        <v>1100</v>
+        <v>1800</v>
       </c>
       <c r="J270" t="n">
         <v>2655569</v>
@@ -64470,7 +64470,7 @@
         <v>29137680</v>
       </c>
       <c r="I273" t="n">
-        <v>3300</v>
+        <v>4300</v>
       </c>
       <c r="J273" t="n">
         <v>13244400</v>
@@ -64940,7 +64940,7 @@
         <v>1367607677</v>
       </c>
       <c r="I275" t="n">
-        <v>2700</v>
+        <v>2800</v>
       </c>
       <c r="J275" t="n">
         <v>53949006</v>
@@ -65175,7 +65175,7 @@
         <v>27669545</v>
       </c>
       <c r="I276" t="n">
-        <v>261800</v>
+        <v>263800</v>
       </c>
       <c r="J276" t="n">
         <v>328544466</v>
@@ -65410,7 +65410,7 @@
         <v>27669545</v>
       </c>
       <c r="I277" t="n">
-        <v>9000</v>
+        <v>17700</v>
       </c>
       <c r="J277" t="n">
         <v>1577272</v>
@@ -65645,7 +65645,7 @@
         <v>1305361522</v>
       </c>
       <c r="I278" t="n">
-        <v>52640800</v>
+        <v>52642900</v>
       </c>
       <c r="J278" t="n">
         <v>1135097787</v>
@@ -65827,7 +65827,7 @@
         <v>0.53</v>
       </c>
       <c r="BQ278" t="n">
-        <v>1.15</v>
+        <v>1.14</v>
       </c>
       <c r="BR278" t="n">
         <v>0</v>
@@ -66115,7 +66115,7 @@
         <v>8761275880</v>
       </c>
       <c r="I280" t="n">
-        <v>3397900</v>
+        <v>3400700</v>
       </c>
       <c r="J280" t="n">
         <v>549296404</v>
@@ -66350,7 +66350,7 @@
         <v>2990631</v>
       </c>
       <c r="I281" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="J281" t="n">
         <v>3148038</v>
@@ -67055,7 +67055,7 @@
         <v>1408769882</v>
       </c>
       <c r="I284" t="n">
-        <v>4900400</v>
+        <v>4903700</v>
       </c>
       <c r="J284" t="n">
         <v>491810224</v>
@@ -67290,7 +67290,7 @@
         <v>37528975</v>
       </c>
       <c r="I285" t="n">
-        <v>74600</v>
+        <v>75100</v>
       </c>
       <c r="J285" t="n">
         <v>3287486</v>
@@ -67525,7 +67525,7 @@
         <v>144634712</v>
       </c>
       <c r="I286" t="n">
-        <v>50200</v>
+        <v>50300</v>
       </c>
       <c r="J286" t="n">
         <v>79469626</v>
@@ -67760,7 +67760,7 @@
         <v>703115134</v>
       </c>
       <c r="I287" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="J287" t="n">
         <v>9317262</v>
@@ -68230,7 +68230,7 @@
         <v>608834381514</v>
       </c>
       <c r="I289" t="n">
-        <v>5982100</v>
+        <v>5987600</v>
       </c>
       <c r="J289" t="n">
         <v>7442231382</v>
@@ -68700,7 +68700,7 @@
         <v>876593906</v>
       </c>
       <c r="I291" t="n">
-        <v>62400</v>
+        <v>62700</v>
       </c>
       <c r="J291" t="n">
         <v>123812773</v>
@@ -68935,7 +68935,7 @@
         <v>2439536514</v>
       </c>
       <c r="I292" t="n">
-        <v>3810100</v>
+        <v>3810500</v>
       </c>
       <c r="J292" t="n">
         <v>723898206</v>
@@ -69170,7 +69170,7 @@
         <v>2635969152</v>
       </c>
       <c r="I293" t="n">
-        <v>1600</v>
+        <v>1700</v>
       </c>
       <c r="J293" t="n">
         <v>129950956</v>
@@ -69331,10 +69331,10 @@
         <v>5.25</v>
       </c>
       <c r="BJ293" t="n">
-        <v>3.32</v>
+        <v>0</v>
       </c>
       <c r="BK293" t="n">
-        <v>9.65</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="BL293" t="n">
         <v>1.24</v>
@@ -69405,7 +69405,7 @@
         <v>2635969152</v>
       </c>
       <c r="I294" t="n">
-        <v>1085200</v>
+        <v>1085300</v>
       </c>
       <c r="J294" t="n">
         <v>129937768</v>
@@ -69569,7 +69569,7 @@
         <v>0</v>
       </c>
       <c r="BK294" t="n">
-        <v>10.01</v>
+        <v>10.41</v>
       </c>
       <c r="BL294" t="n">
         <v>1.24</v>
@@ -69640,7 +69640,7 @@
         <v>29820985</v>
       </c>
       <c r="I295" t="n">
-        <v>800</v>
+        <v>900</v>
       </c>
       <c r="J295" t="n">
         <v>12425418</v>
@@ -69875,7 +69875,7 @@
         <v>1406916919</v>
       </c>
       <c r="I296" t="n">
-        <v>871400</v>
+        <v>871600</v>
       </c>
       <c r="J296" t="n">
         <v>203901000</v>
@@ -70110,7 +70110,7 @@
         <v>251750450</v>
       </c>
       <c r="I297" t="n">
-        <v>6581800</v>
+        <v>6582800</v>
       </c>
       <c r="J297" t="n">
         <v>306800000</v>
@@ -70345,7 +70345,7 @@
         <v>1730843908</v>
       </c>
       <c r="I298" t="n">
-        <v>430800</v>
+        <v>430900</v>
       </c>
       <c r="J298" t="n">
         <v>150377481</v>
@@ -70580,7 +70580,7 @@
         <v>5433034424</v>
       </c>
       <c r="I299" t="n">
-        <v>1310700</v>
+        <v>1310800</v>
       </c>
       <c r="J299" t="n">
         <v>450945982</v>
@@ -70815,7 +70815,7 @@
         <v>5433034424</v>
       </c>
       <c r="I300" t="n">
-        <v>15407400</v>
+        <v>15412900</v>
       </c>
       <c r="J300" t="n">
         <v>798952621</v>
@@ -71050,7 +71050,7 @@
         <v>482120013</v>
       </c>
       <c r="I301" t="n">
-        <v>1000700</v>
+        <v>1001300</v>
       </c>
       <c r="J301" t="n">
         <v>141800000</v>
@@ -71520,7 +71520,7 @@
         <v>54836328273</v>
       </c>
       <c r="I303" t="n">
-        <v>5593900</v>
+        <v>5594100</v>
       </c>
       <c r="J303" t="n">
         <v>872495263</v>
@@ -71755,7 +71755,7 @@
         <v>955439847</v>
       </c>
       <c r="I304" t="n">
-        <v>779100</v>
+        <v>780400</v>
       </c>
       <c r="J304" t="n">
         <v>57007156</v>
@@ -71990,7 +71990,7 @@
         <v>30111509822</v>
       </c>
       <c r="I305" t="n">
-        <v>1426900</v>
+        <v>1427100</v>
       </c>
       <c r="J305" t="n">
         <v>646586060</v>
@@ -72172,7 +72172,7 @@
         <v>43.13</v>
       </c>
       <c r="BQ305" t="n">
-        <v>46.57</v>
+        <v>46.56</v>
       </c>
       <c r="BR305" t="n">
         <v>8.199999999999999</v>
@@ -72225,7 +72225,7 @@
         <v>219939555</v>
       </c>
       <c r="I306" t="n">
-        <v>724100</v>
+        <v>724300</v>
       </c>
       <c r="J306" t="n">
         <v>140986886</v>
@@ -72460,7 +72460,7 @@
         <v>457263027</v>
       </c>
       <c r="I307" t="n">
-        <v>1344700</v>
+        <v>1344800</v>
       </c>
       <c r="J307" t="n">
         <v>284014325</v>
@@ -72695,7 +72695,7 @@
         <v>32296124344</v>
       </c>
       <c r="I308" t="n">
-        <v>10709300</v>
+        <v>10709500</v>
       </c>
       <c r="J308" t="n">
         <v>1752367344</v>
@@ -72930,7 +72930,7 @@
         <v>26431869000</v>
       </c>
       <c r="I309" t="n">
-        <v>12338500</v>
+        <v>12339000</v>
       </c>
       <c r="J309" t="n">
         <v>1858828617</v>
@@ -73165,7 +73165,7 @@
         <v>326144632</v>
       </c>
       <c r="I310" t="n">
-        <v>8305500</v>
+        <v>8306200</v>
       </c>
       <c r="J310" t="n">
         <v>1358936900</v>
@@ -73400,7 +73400,7 @@
         <v>1784078461</v>
       </c>
       <c r="I311" t="n">
-        <v>609700</v>
+        <v>609800</v>
       </c>
       <c r="J311" t="n">
         <v>230501219</v>
@@ -73635,7 +73635,7 @@
         <v>2022976573</v>
       </c>
       <c r="I312" t="n">
-        <v>34700</v>
+        <v>34800</v>
       </c>
       <c r="J312" t="n">
         <v>125841938</v>
@@ -73870,7 +73870,7 @@
         <v>2022976573</v>
       </c>
       <c r="I313" t="n">
-        <v>2293400</v>
+        <v>2295100</v>
       </c>
       <c r="J313" t="n">
         <v>223882733</v>
@@ -74105,7 +74105,7 @@
         <v>77792188</v>
       </c>
       <c r="I314" t="n">
-        <v>364600</v>
+        <v>366600</v>
       </c>
       <c r="J314" t="n">
         <v>42655504</v>
@@ -74575,7 +74575,7 @@
         <v>76730001000</v>
       </c>
       <c r="I316" t="n">
-        <v>16834300</v>
+        <v>16834400</v>
       </c>
       <c r="J316" t="n">
         <v>2240292590</v>
@@ -74810,7 +74810,7 @@
         <v>3084496938</v>
       </c>
       <c r="I317" t="n">
-        <v>1680000</v>
+        <v>1680100</v>
       </c>
       <c r="J317" t="n">
         <v>293482126</v>
@@ -75045,7 +75045,7 @@
         <v>13945347279</v>
       </c>
       <c r="I318" t="n">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="J318" t="n">
         <v>2568204239</v>
@@ -75280,7 +75280,7 @@
         <v>38099145463</v>
       </c>
       <c r="I319" t="n">
-        <v>15550300</v>
+        <v>15550700</v>
       </c>
       <c r="J319" t="n">
         <v>1082620720</v>
@@ -75515,7 +75515,7 @@
         <v>275515397</v>
       </c>
       <c r="I320" t="n">
-        <v>9700</v>
+        <v>10600</v>
       </c>
       <c r="J320" t="n">
         <v>310744441</v>
@@ -75750,7 +75750,7 @@
         <v>275515397</v>
       </c>
       <c r="I321" t="n">
-        <v>57400</v>
+        <v>58200</v>
       </c>
       <c r="J321" t="n">
         <v>62370987</v>
@@ -75985,7 +75985,7 @@
         <v>526414633</v>
       </c>
       <c r="I322" t="n">
-        <v>167800</v>
+        <v>168000</v>
       </c>
       <c r="J322" t="n">
         <v>93170747</v>
@@ -77395,7 +77395,7 @@
         <v>250110861</v>
       </c>
       <c r="I328" t="n">
-        <v>2500</v>
+        <v>2600</v>
       </c>
       <c r="J328" t="n">
         <v>2495225</v>
@@ -77630,7 +77630,7 @@
         <v>111547287420</v>
       </c>
       <c r="I329" t="n">
-        <v>4993200</v>
+        <v>4993300</v>
       </c>
       <c r="J329" t="n">
         <v>0</v>
@@ -77791,10 +77791,10 @@
         <v>33.03</v>
       </c>
       <c r="BJ329" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BK329" t="n">
-        <v>28.97</v>
+        <v>29.55</v>
       </c>
       <c r="BL329" t="n">
         <v>3.1</v>
@@ -77865,7 +77865,7 @@
         <v>111547287420</v>
       </c>
       <c r="I330" t="n">
-        <v>129100</v>
+        <v>129600</v>
       </c>
       <c r="J330" t="n">
         <v>3818695031</v>
@@ -78029,7 +78029,7 @@
         <v>0</v>
       </c>
       <c r="BK330" t="n">
-        <v>14.39</v>
+        <v>14.57</v>
       </c>
       <c r="BL330" t="n">
         <v>1.55</v>
@@ -78100,7 +78100,7 @@
         <v>111547287420</v>
       </c>
       <c r="I331" t="n">
-        <v>170300</v>
+        <v>170400</v>
       </c>
       <c r="J331" t="n">
         <v>3679836020</v>
@@ -78261,7 +78261,7 @@
         <v>16.52</v>
       </c>
       <c r="BJ331" t="n">
-        <v>2.07</v>
+        <v>0</v>
       </c>
       <c r="BK331" t="n">
         <v>14.78</v>
@@ -78335,7 +78335,7 @@
         <v>10229682490</v>
       </c>
       <c r="I332" t="n">
-        <v>1838200</v>
+        <v>1839000</v>
       </c>
       <c r="J332" t="n">
         <v>0</v>
@@ -78570,7 +78570,7 @@
         <v>10229682490</v>
       </c>
       <c r="I333" t="n">
-        <v>75600</v>
+        <v>75700</v>
       </c>
       <c r="J333" t="n">
         <v>503735259</v>
@@ -78805,7 +78805,7 @@
         <v>10229682490</v>
       </c>
       <c r="I334" t="n">
-        <v>1219500</v>
+        <v>1220500</v>
       </c>
       <c r="J334" t="n">
         <v>1007470260</v>
@@ -79040,7 +79040,7 @@
         <v>1891443936</v>
       </c>
       <c r="I335" t="n">
-        <v>2605600</v>
+        <v>2607300</v>
       </c>
       <c r="J335" t="n">
         <v>230663994</v>
@@ -79275,7 +79275,7 @@
         <v>83707682500</v>
       </c>
       <c r="I336" t="n">
-        <v>28308400</v>
+        <v>28308500</v>
       </c>
       <c r="J336" t="n">
         <v>3524534025</v>
@@ -79510,7 +79510,7 @@
         <v>717097394</v>
       </c>
       <c r="I337" t="n">
-        <v>3900</v>
+        <v>4000</v>
       </c>
       <c r="J337" t="n">
         <v>57737319</v>
@@ -79745,7 +79745,7 @@
         <v>1428808699</v>
       </c>
       <c r="I338" t="n">
-        <v>1494800</v>
+        <v>1496300</v>
       </c>
       <c r="J338" t="n">
         <v>128721560</v>
@@ -79980,7 +79980,7 @@
         <v>382229271</v>
       </c>
       <c r="I339" t="n">
-        <v>356100</v>
+        <v>360800</v>
       </c>
       <c r="J339" t="n">
         <v>6313033484</v>
@@ -80215,7 +80215,7 @@
         <v>410542987</v>
       </c>
       <c r="I340" t="n">
-        <v>10600</v>
+        <v>11000</v>
       </c>
       <c r="J340" t="n">
         <v>6741262</v>
@@ -80685,7 +80685,7 @@
         <v>912881727</v>
       </c>
       <c r="I342" t="n">
-        <v>220000</v>
+        <v>221000</v>
       </c>
       <c r="J342" t="n">
         <v>204682016</v>
@@ -80920,7 +80920,7 @@
         <v>3566769400</v>
       </c>
       <c r="I343" t="n">
-        <v>4122600</v>
+        <v>4123000</v>
       </c>
       <c r="J343" t="n">
         <v>583759291</v>
@@ -81155,7 +81155,7 @@
         <v>7925072522</v>
       </c>
       <c r="I344" t="n">
-        <v>5486000</v>
+        <v>5486100</v>
       </c>
       <c r="J344" t="n">
         <v>498745930</v>
@@ -81328,7 +81328,7 @@
         <v>0.79</v>
       </c>
       <c r="BN344" t="n">
-        <v>15.89</v>
+        <v>15.9</v>
       </c>
       <c r="BO344" t="n">
         <v>19.48</v>
@@ -81390,7 +81390,7 @@
         <v>10665208239</v>
       </c>
       <c r="I345" t="n">
-        <v>11020400</v>
+        <v>11024500</v>
       </c>
       <c r="J345" t="n">
         <v>616129844</v>
@@ -81625,7 +81625,7 @@
         <v>6120133822</v>
       </c>
       <c r="I346" t="n">
-        <v>3706200</v>
+        <v>3706400</v>
       </c>
       <c r="J346" t="n">
         <v>332435391</v>
@@ -82095,7 +82095,7 @@
         <v>32912570</v>
       </c>
       <c r="I348" t="n">
-        <v>12300</v>
+        <v>12400</v>
       </c>
       <c r="J348" t="n">
         <v>5052280</v>
@@ -82565,7 +82565,7 @@
         <v>905338604</v>
       </c>
       <c r="I350" t="n">
-        <v>703900</v>
+        <v>704500</v>
       </c>
       <c r="J350" t="n">
         <v>141902688</v>
@@ -82738,7 +82738,7 @@
         <v>0.18</v>
       </c>
       <c r="BN350" t="n">
-        <v>6.38</v>
+        <v>6.41</v>
       </c>
       <c r="BO350" t="n">
         <v>10.47</v>
@@ -83505,7 +83505,7 @@
         <v>56847343033</v>
       </c>
       <c r="I354" t="n">
-        <v>13545800</v>
+        <v>13547500</v>
       </c>
       <c r="J354" t="n">
         <v>1264117615</v>
@@ -83740,7 +83740,7 @@
         <v>552572710</v>
       </c>
       <c r="I355" t="n">
-        <v>242800</v>
+        <v>244200</v>
       </c>
       <c r="J355" t="n">
         <v>152644445</v>
@@ -83975,7 +83975,7 @@
         <v>12942816053</v>
       </c>
       <c r="I356" t="n">
-        <v>1875800</v>
+        <v>1875900</v>
       </c>
       <c r="J356" t="n">
         <v>0</v>
@@ -84157,7 +84157,7 @@
         <v>30.76</v>
       </c>
       <c r="BQ356" t="n">
-        <v>37.4</v>
+        <v>37.38</v>
       </c>
       <c r="BR356" t="n">
         <v>2.65</v>
@@ -84210,7 +84210,7 @@
         <v>12942816053</v>
       </c>
       <c r="I357" t="n">
-        <v>116600</v>
+        <v>116700</v>
       </c>
       <c r="J357" t="n">
         <v>590714069</v>
@@ -84445,7 +84445,7 @@
         <v>12942816053</v>
       </c>
       <c r="I358" t="n">
-        <v>179100</v>
+        <v>179200</v>
       </c>
       <c r="J358" t="n">
         <v>442782652</v>
@@ -84680,7 +84680,7 @@
         <v>736796649</v>
       </c>
       <c r="I359" t="n">
-        <v>6000</v>
+        <v>6200</v>
       </c>
       <c r="J359" t="n">
         <v>51089845</v>
@@ -84915,7 +84915,7 @@
         <v>736796649</v>
       </c>
       <c r="I360" t="n">
-        <v>323200</v>
+        <v>326700</v>
       </c>
       <c r="J360" t="n">
         <v>88208032</v>
@@ -85150,7 +85150,7 @@
         <v>58832225</v>
       </c>
       <c r="I361" t="n">
-        <v>133000</v>
+        <v>133100</v>
       </c>
       <c r="J361" t="n">
         <v>73619230</v>
@@ -85385,7 +85385,7 @@
         <v>571072124</v>
       </c>
       <c r="I362" t="n">
-        <v>46500</v>
+        <v>47100</v>
       </c>
       <c r="J362" t="n">
         <v>60176215</v>
@@ -86090,7 +86090,7 @@
         <v>3817081959</v>
       </c>
       <c r="I365" t="n">
-        <v>3280000</v>
+        <v>3280300</v>
       </c>
       <c r="J365" t="n">
         <v>122578152</v>
@@ -86325,7 +86325,7 @@
         <v>844857869</v>
       </c>
       <c r="I366" t="n">
-        <v>501900</v>
+        <v>502400</v>
       </c>
       <c r="J366" t="n">
         <v>65492864</v>
@@ -86560,7 +86560,7 @@
         <v>2269179428</v>
       </c>
       <c r="I367" t="n">
-        <v>244500</v>
+        <v>244600</v>
       </c>
       <c r="J367" t="n">
         <v>66002915</v>
@@ -87030,7 +87030,7 @@
         <v>18968855</v>
       </c>
       <c r="I369" t="n">
-        <v>163200</v>
+        <v>165200</v>
       </c>
       <c r="J369" t="n">
         <v>54196747</v>
@@ -87447,7 +87447,7 @@
         <v>26.76</v>
       </c>
       <c r="BQ370" t="n">
-        <v>31.32</v>
+        <v>31.29</v>
       </c>
       <c r="BR370" t="n">
         <v>13.43</v>
@@ -87500,7 +87500,7 @@
         <v>367400016</v>
       </c>
       <c r="I371" t="n">
-        <v>11000</v>
+        <v>11100</v>
       </c>
       <c r="J371" t="n">
         <v>44000000</v>
@@ -87735,7 +87735,7 @@
         <v>1062501939</v>
       </c>
       <c r="I372" t="n">
-        <v>440200</v>
+        <v>440400</v>
       </c>
       <c r="J372" t="n">
         <v>242617538</v>
@@ -87970,7 +87970,7 @@
         <v>5653327484</v>
       </c>
       <c r="I373" t="n">
-        <v>1923900</v>
+        <v>1924000</v>
       </c>
       <c r="J373" t="n">
         <v>500737647</v>
@@ -88205,7 +88205,7 @@
         <v>2130943411</v>
       </c>
       <c r="I374" t="n">
-        <v>590500</v>
+        <v>590700</v>
       </c>
       <c r="J374" t="n">
         <v>132450415</v>
@@ -89145,7 +89145,7 @@
         <v>38586060463</v>
       </c>
       <c r="I378" t="n">
-        <v>12008000</v>
+        <v>12008200</v>
       </c>
       <c r="J378" t="n">
         <v>1115849873</v>
@@ -89306,7 +89306,7 @@
         <v>14.69</v>
       </c>
       <c r="BJ378" t="n">
-        <v>0.76</v>
+        <v>0</v>
       </c>
       <c r="BK378" t="n">
         <v>34.58</v>
@@ -89380,7 +89380,7 @@
         <v>6585009740</v>
       </c>
       <c r="I379" t="n">
-        <v>4600</v>
+        <v>4700</v>
       </c>
       <c r="J379" t="n">
         <v>39059883</v>
@@ -89615,7 +89615,7 @@
         <v>6585009740</v>
       </c>
       <c r="I380" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="J380" t="n">
         <v>2337871</v>
@@ -89850,7 +89850,7 @@
         <v>6585009740</v>
       </c>
       <c r="I381" t="n">
-        <v>151000</v>
+        <v>151100</v>
       </c>
       <c r="J381" t="n">
         <v>71775511</v>
@@ -90023,7 +90023,7 @@
         <v>2.39</v>
       </c>
       <c r="BN381" t="n">
-        <v>59.28</v>
+        <v>59.3</v>
       </c>
       <c r="BO381" t="n">
         <v>72.75</v>
@@ -90085,7 +90085,7 @@
         <v>7682626223</v>
       </c>
       <c r="I382" t="n">
-        <v>711200</v>
+        <v>711300</v>
       </c>
       <c r="J382" t="n">
         <v>705260684</v>
@@ -90320,7 +90320,7 @@
         <v>7682626223</v>
       </c>
       <c r="I383" t="n">
-        <v>10455700</v>
+        <v>10457400</v>
       </c>
       <c r="J383" t="n">
         <v>547752163</v>
@@ -90555,7 +90555,7 @@
         <v>7682626223</v>
       </c>
       <c r="I384" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="J384" t="n">
         <v>66261</v>
@@ -90790,7 +90790,7 @@
         <v>333070094351</v>
       </c>
       <c r="I385" t="n">
-        <v>28372500</v>
+        <v>28372600</v>
       </c>
       <c r="J385" t="n">
         <v>4255762795</v>
@@ -91025,7 +91025,7 @@
         <v>3347805991</v>
       </c>
       <c r="I386" t="n">
-        <v>43951600</v>
+        <v>43952200</v>
       </c>
       <c r="J386" t="n">
         <v>1221826865</v>
@@ -91442,7 +91442,7 @@
         <v>18.55</v>
       </c>
       <c r="BQ387" t="n">
-        <v>34.41</v>
+        <v>34.33</v>
       </c>
       <c r="BR387" t="n">
         <v>7.92</v>
@@ -91965,7 +91965,7 @@
         <v>7271259</v>
       </c>
       <c r="I390" t="n">
-        <v>2300</v>
+        <v>2700</v>
       </c>
       <c r="J390" t="n">
         <v>4880040</v>
@@ -92435,7 +92435,7 @@
         <v>1383564805</v>
       </c>
       <c r="I392" t="n">
-        <v>162000</v>
+        <v>162100</v>
       </c>
       <c r="J392" t="n">
         <v>81836375</v>
@@ -92670,7 +92670,7 @@
         <v>286251250</v>
       </c>
       <c r="I393" t="n">
-        <v>32000</v>
+        <v>33900</v>
       </c>
       <c r="J393" t="n">
         <v>114500510</v>
@@ -92905,7 +92905,7 @@
         <v>2025692204</v>
       </c>
       <c r="I394" t="n">
-        <v>618700</v>
+        <v>618900</v>
       </c>
       <c r="J394" t="n">
         <v>149829337</v>
@@ -93140,7 +93140,7 @@
         <v>4346815331</v>
       </c>
       <c r="I395" t="n">
-        <v>1114500</v>
+        <v>1114600</v>
       </c>
       <c r="J395" t="n">
         <v>317982170</v>
@@ -93375,7 +93375,7 @@
         <v>825101421</v>
       </c>
       <c r="I396" t="n">
-        <v>762200</v>
+        <v>778300</v>
       </c>
       <c r="J396" t="n">
         <v>322820608</v>
@@ -93610,7 +93610,7 @@
         <v>206801859781</v>
       </c>
       <c r="I397" t="n">
-        <v>7851700</v>
+        <v>7857400</v>
       </c>
       <c r="J397" t="n">
         <v>4197317998</v>
@@ -94080,7 +94080,7 @@
         <v>5374113825</v>
       </c>
       <c r="I399" t="n">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="J399" t="n">
         <v>1028700892</v>
@@ -94315,7 +94315,7 @@
         <v>5374113825</v>
       </c>
       <c r="I400" t="n">
-        <v>3100</v>
+        <v>3900</v>
       </c>
       <c r="J400" t="n">
         <v>474085114</v>
@@ -94550,7 +94550,7 @@
         <v>1239280800</v>
       </c>
       <c r="I401" t="n">
-        <v>354200</v>
+        <v>354700</v>
       </c>
       <c r="J401" t="n">
         <v>159907282</v>
@@ -94785,7 +94785,7 @@
         <v>661716569</v>
       </c>
       <c r="I402" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="J402" t="n">
         <v>16571220</v>
@@ -95020,7 +95020,7 @@
         <v>661716569</v>
       </c>
       <c r="I403" t="n">
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="J403" t="n">
         <v>19843450</v>
@@ -95255,7 +95255,7 @@
         <v>2157078824</v>
       </c>
       <c r="I404" t="n">
-        <v>4995100</v>
+        <v>5001500</v>
       </c>
       <c r="J404" t="n">
         <v>274088851</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-08-31 06:37
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -6173,7 +6173,7 @@
         <v>0.39</v>
       </c>
       <c r="BM24" t="n">
-        <v>0.36</v>
+        <v>0.41</v>
       </c>
       <c r="BN24" t="n">
         <v>2.84</v>
@@ -6188,7 +6188,7 @@
         <v>2.68</v>
       </c>
       <c r="BR24" t="n">
-        <v>7.74</v>
+        <v>6.75</v>
       </c>
       <c r="BS24" t="n">
         <v>2.78</v>
@@ -10684,7 +10684,7 @@
         <v>4.46</v>
       </c>
       <c r="H44" t="n">
-        <v>5772636</v>
+        <v>6133260</v>
       </c>
       <c r="I44" t="n">
         <v>0</v>
@@ -10702,7 +10702,7 @@
         <v>0.75</v>
       </c>
       <c r="N44" t="n">
-        <v>0.2579633921815138</v>
+        <v>0.2740786972764593</v>
       </c>
       <c r="O44" t="n">
         <v>0.03</v>
@@ -10780,7 +10780,7 @@
         <v>5719748.64</v>
       </c>
       <c r="AN44" t="n">
-        <v>5772636</v>
+        <v>6133260</v>
       </c>
       <c r="AO44" t="n">
         <v>0</v>
@@ -10919,7 +10919,7 @@
         <v>3.45</v>
       </c>
       <c r="H45" t="n">
-        <v>5772636</v>
+        <v>6133260</v>
       </c>
       <c r="I45" t="n">
         <v>700</v>
@@ -10937,7 +10937,7 @@
         <v>0.63</v>
       </c>
       <c r="N45" t="n">
-        <v>0.1577679753038631</v>
+        <v>0.1676239437602113</v>
       </c>
       <c r="O45" t="n">
         <v>0.02</v>
@@ -11015,7 +11015,7 @@
         <v>9352251.359999999</v>
       </c>
       <c r="AN45" t="n">
-        <v>6872185.714285715</v>
+        <v>7301500</v>
       </c>
       <c r="AO45" t="n">
         <v>0</v>
@@ -11859,7 +11859,7 @@
         <v>46.38</v>
       </c>
       <c r="H49" t="n">
-        <v>912652000</v>
+        <v>914960100</v>
       </c>
       <c r="I49" t="n">
         <v>0</v>
@@ -11877,7 +11877,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="N49" t="n">
-        <v>0.9965365858026189</v>
+        <v>0.9990568302043087</v>
       </c>
       <c r="O49" t="n">
         <v>0.08</v>
@@ -11955,7 +11955,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN49" t="n">
-        <v>166846800.7312614</v>
+        <v>167268756.8555759</v>
       </c>
       <c r="AO49" t="n">
         <v>2.4346</v>
@@ -12094,7 +12094,7 @@
         <v>32.9</v>
       </c>
       <c r="H50" t="n">
-        <v>912652000</v>
+        <v>914960100</v>
       </c>
       <c r="I50" t="n">
         <v>1500</v>
@@ -12112,7 +12112,7 @@
         <v>5.78</v>
       </c>
       <c r="N50" t="n">
-        <v>0.9965365858026189</v>
+        <v>0.9990568302043087</v>
       </c>
       <c r="O50" t="n">
         <v>0.06</v>
@@ -12190,7 +12190,7 @@
         <v>70976350.5</v>
       </c>
       <c r="AN50" t="n">
-        <v>239541207.3490814</v>
+        <v>240147007.8740157</v>
       </c>
       <c r="AO50" t="n">
         <v>3.526</v>
@@ -14428,7 +14428,7 @@
         <v>373.48</v>
       </c>
       <c r="H60" t="n">
-        <v>169840034</v>
+        <v>169840000</v>
       </c>
       <c r="I60" t="n">
         <v>10</v>
@@ -14446,7 +14446,7 @@
         <v>2.87</v>
       </c>
       <c r="N60" t="n">
-        <v>12.00197272271102</v>
+        <v>12.00197032005563</v>
       </c>
       <c r="O60" t="n">
         <v>0.64</v>
@@ -14524,7 +14524,7 @@
         <v>59731412.5</v>
       </c>
       <c r="AN60" t="n">
-        <v>21390432.49370277</v>
+        <v>21390428.2115869</v>
       </c>
       <c r="AO60" t="n">
         <v>0</v>
@@ -14898,7 +14898,7 @@
         <v>105</v>
       </c>
       <c r="H62" t="n">
-        <v>10363469550</v>
+        <v>10363470000</v>
       </c>
       <c r="I62" t="n">
         <v>800</v>
@@ -14916,7 +14916,7 @@
         <v>4.26</v>
       </c>
       <c r="N62" t="n">
-        <v>1.059177903156948</v>
+        <v>1.059177949148308</v>
       </c>
       <c r="O62" t="n">
         <v>0.17</v>
@@ -14994,7 +14994,7 @@
         <v>2822812821.4</v>
       </c>
       <c r="AN62" t="n">
-        <v>4247323586.065574</v>
+        <v>4247323770.491803</v>
       </c>
       <c r="AO62" t="n">
         <v>0</v>
@@ -18893,7 +18893,7 @@
         <v>2.67</v>
       </c>
       <c r="H79" t="n">
-        <v>5704756873</v>
+        <v>5704812000</v>
       </c>
       <c r="I79" t="n">
         <v>14800</v>
@@ -18911,7 +18911,7 @@
         <v>2.47</v>
       </c>
       <c r="N79" t="n">
-        <v>0.7976337303891849</v>
+        <v>0.7976414381943787</v>
       </c>
       <c r="O79" t="n">
         <v>0.03</v>
@@ -18989,7 +18989,7 @@
         <v>531401092.4</v>
       </c>
       <c r="AN79" t="n">
-        <v>3457428407.878788</v>
+        <v>3457461818.181818</v>
       </c>
       <c r="AO79" t="n">
         <v>0</v>
@@ -19128,7 +19128,7 @@
         <v>2.69</v>
       </c>
       <c r="H80" t="n">
-        <v>5704756873</v>
+        <v>5704812000</v>
       </c>
       <c r="I80" t="n">
         <v>17500</v>
@@ -19146,7 +19146,7 @@
         <v>3.36</v>
       </c>
       <c r="N80" t="n">
-        <v>1.537633991143202</v>
+        <v>1.53764884982183</v>
       </c>
       <c r="O80" t="n">
         <v>0.04</v>
@@ -19224,7 +19224,7 @@
         <v>275659512.02</v>
       </c>
       <c r="AN80" t="n">
-        <v>2535447499.111111</v>
+        <v>2535472000</v>
       </c>
       <c r="AO80" t="n">
         <v>0</v>
@@ -19598,7 +19598,7 @@
         <v>8.34</v>
       </c>
       <c r="H82" t="n">
-        <v>350460400</v>
+        <v>352574200</v>
       </c>
       <c r="I82" t="n">
         <v>17600</v>
@@ -19616,7 +19616,7 @@
         <v>6.04</v>
       </c>
       <c r="N82" t="n">
-        <v>0.8911749664341261</v>
+        <v>0.8965500834061105</v>
       </c>
       <c r="O82" t="n">
         <v>1.01</v>
@@ -19694,7 +19694,7 @@
         <v>65949124.8</v>
       </c>
       <c r="AN82" t="n">
-        <v>62359501.77935943</v>
+        <v>62735622.77580071</v>
       </c>
       <c r="AO82" t="n">
         <v>0</v>
@@ -21948,7 +21948,7 @@
         <v>9</v>
       </c>
       <c r="H92" t="n">
-        <v>73960270</v>
+        <v>73529860</v>
       </c>
       <c r="I92" t="n">
         <v>0</v>
@@ -21966,7 +21966,7 @@
         <v>3.42</v>
       </c>
       <c r="N92" t="n">
-        <v>0.1365641366125181</v>
+        <v>0.1357694049269876</v>
       </c>
       <c r="O92" t="n">
         <v>0.15</v>
@@ -22044,7 +22044,7 @@
         <v>23342055.36</v>
       </c>
       <c r="AN92" t="n">
-        <v>52454092.19858156</v>
+        <v>52148836.87943263</v>
       </c>
       <c r="AO92" t="n">
         <v>0</v>
@@ -22183,7 +22183,7 @@
         <v>5.15</v>
       </c>
       <c r="H93" t="n">
-        <v>73960270</v>
+        <v>73529860</v>
       </c>
       <c r="I93" t="n">
         <v>1300</v>
@@ -22201,7 +22201,7 @@
         <v>2.3</v>
       </c>
       <c r="N93" t="n">
-        <v>0.1815524369371744</v>
+        <v>0.1804958969274891</v>
       </c>
       <c r="O93" t="n">
         <v>0.1</v>
@@ -22279,7 +22279,7 @@
         <v>17557944.64</v>
       </c>
       <c r="AN93" t="n">
-        <v>77852915.78947368</v>
+        <v>77399852.63157895</v>
       </c>
       <c r="AO93" t="n">
         <v>0</v>
@@ -23358,7 +23358,7 @@
         <v>30</v>
       </c>
       <c r="H98" t="n">
-        <v>7786536000</v>
+        <v>7789132000</v>
       </c>
       <c r="I98" t="n">
         <v>5400</v>
@@ -23376,7 +23376,7 @@
         <v>24.76</v>
       </c>
       <c r="N98" t="n">
-        <v>1.580554138763975</v>
+        <v>1.581081089200502</v>
       </c>
       <c r="O98" t="n">
         <v>3.06</v>
@@ -23454,7 +23454,7 @@
         <v>576395765.0400001</v>
       </c>
       <c r="AN98" t="n">
-        <v>541107435.7192495</v>
+        <v>541287838.7769284</v>
       </c>
       <c r="AO98" t="n">
         <v>0</v>
@@ -23593,7 +23593,7 @@
         <v>125.39</v>
       </c>
       <c r="H99" t="n">
-        <v>16502698530</v>
+        <v>16482640000</v>
       </c>
       <c r="I99" t="n">
         <v>200</v>
@@ -23611,7 +23611,7 @@
         <v>10.65</v>
       </c>
       <c r="N99" t="n">
-        <v>1.630570465478126</v>
+        <v>1.62858855648673</v>
       </c>
       <c r="O99" t="n">
         <v>1.16</v>
@@ -23689,7 +23689,7 @@
         <v>1267125769.6</v>
       </c>
       <c r="AN99" t="n">
-        <v>2840395616.179002</v>
+        <v>2836943201.376936</v>
       </c>
       <c r="AO99" t="n">
         <v>0</v>
@@ -23828,7 +23828,7 @@
         <v>120.71</v>
       </c>
       <c r="H100" t="n">
-        <v>16502698530</v>
+        <v>16482640000</v>
       </c>
       <c r="I100" t="n">
         <v>700</v>
@@ -23846,7 +23846,7 @@
         <v>10.81</v>
       </c>
       <c r="N100" t="n">
-        <v>5.909576090337042</v>
+        <v>5.902393179670654</v>
       </c>
       <c r="O100" t="n">
         <v>1.18</v>
@@ -23924,7 +23924,7 @@
         <v>349625391.8</v>
       </c>
       <c r="AN100" t="n">
-        <v>2797067547.457627</v>
+        <v>2793667796.610169</v>
       </c>
       <c r="AO100" t="n">
         <v>0</v>
@@ -24063,7 +24063,7 @@
         <v>23.29</v>
       </c>
       <c r="H101" t="n">
-        <v>587926522</v>
+        <v>585418000</v>
       </c>
       <c r="I101" t="n">
         <v>1100</v>
@@ -24081,7 +24081,7 @@
         <v>6.28</v>
       </c>
       <c r="N101" t="n">
-        <v>1.763724392852866</v>
+        <v>1.756199062261626</v>
       </c>
       <c r="O101" t="n">
         <v>0.49</v>
@@ -24159,7 +24159,7 @@
         <v>45834767.09999999</v>
       </c>
       <c r="AN101" t="n">
-        <v>60799019.85522234</v>
+        <v>60539607.03205791</v>
       </c>
       <c r="AO101" t="n">
         <v>0</v>
@@ -24298,7 +24298,7 @@
         <v>22.58</v>
       </c>
       <c r="H102" t="n">
-        <v>587926522</v>
+        <v>585418000</v>
       </c>
       <c r="I102" t="n">
         <v>4000</v>
@@ -24316,7 +24316,7 @@
         <v>6.32</v>
       </c>
       <c r="N102" t="n">
-        <v>1.291732178935546</v>
+        <v>1.286220710294967</v>
       </c>
       <c r="O102" t="n">
         <v>0.49</v>
@@ -24394,7 +24394,7 @@
         <v>62582552.4</v>
       </c>
       <c r="AN102" t="n">
-        <v>60424102.98047276</v>
+        <v>60166289.82528263</v>
       </c>
       <c r="AO102" t="n">
         <v>0</v>
@@ -30816,7 +30816,7 @@
         <v>3.99</v>
       </c>
       <c r="BM129" t="n">
-        <v>5.05</v>
+        <v>5.02</v>
       </c>
       <c r="BN129" t="n">
         <v>24.49</v>
@@ -30831,7 +30831,7 @@
         <v>22.45</v>
       </c>
       <c r="BR129" t="n">
-        <v>4.56</v>
+        <v>4.58</v>
       </c>
       <c r="BS129" t="n">
         <v>24.06</v>
@@ -32288,7 +32288,7 @@
         <v>6.46</v>
       </c>
       <c r="H136" t="n">
-        <v>430642300</v>
+        <v>429371600</v>
       </c>
       <c r="I136" t="n">
         <v>0</v>
@@ -32306,7 +32306,7 @@
         <v>89.8</v>
       </c>
       <c r="N136" t="n">
-        <v>1.00523744898495</v>
+        <v>1.002271286054775</v>
       </c>
       <c r="O136" t="n">
         <v>0.49</v>
@@ -32384,7 +32384,7 @@
         <v>3812747.4</v>
       </c>
       <c r="AN136" t="n">
-        <v>7280512.256973796</v>
+        <v>7259029.585798817</v>
       </c>
       <c r="AO136" t="n">
         <v>0</v>
@@ -32523,7 +32523,7 @@
         <v>3.66</v>
       </c>
       <c r="H137" t="n">
-        <v>430642300</v>
+        <v>429371600</v>
       </c>
       <c r="I137" t="n">
         <v>9800</v>
@@ -32541,7 +32541,7 @@
         <v>51.86</v>
       </c>
       <c r="N137" t="n">
-        <v>2.585441290001963</v>
+        <v>2.577812405781334</v>
       </c>
       <c r="O137" t="n">
         <v>0.29</v>
@@ -32619,7 +32619,7 @@
         <v>1482422.55</v>
       </c>
       <c r="AN137" t="n">
-        <v>12602935.32338308</v>
+        <v>12565747.73192859</v>
       </c>
       <c r="AO137" t="n">
         <v>0</v>
@@ -33463,7 +33463,7 @@
         <v>11.5</v>
       </c>
       <c r="H141" t="n">
-        <v>254008632</v>
+        <v>256640500</v>
       </c>
       <c r="I141" t="n">
         <v>0</v>
@@ -33481,7 +33481,7 @@
         <v>2.98</v>
       </c>
       <c r="N141" t="n">
-        <v>1.011111719300996</v>
+        <v>1.021588184441178</v>
       </c>
       <c r="O141" t="n">
         <v>0.5</v>
@@ -33559,7 +33559,7 @@
         <v>45922500</v>
       </c>
       <c r="AN141" t="n">
-        <v>65976268.05194805</v>
+        <v>66659870.12987013</v>
       </c>
       <c r="AO141" t="n">
         <v>0</v>
@@ -33698,7 +33698,7 @@
         <v>10.75</v>
       </c>
       <c r="H142" t="n">
-        <v>254008632</v>
+        <v>256640500</v>
       </c>
       <c r="I142" t="n">
         <v>4000</v>
@@ -33716,7 +33716,7 @@
         <v>3.05</v>
       </c>
       <c r="N142" t="n">
-        <v>0.7732030794654678</v>
+        <v>0.7812144939844303</v>
       </c>
       <c r="O142" t="n">
         <v>0.51</v>
@@ -33794,7 +33794,7 @@
         <v>60052500</v>
       </c>
       <c r="AN142" t="n">
-        <v>64305982.78481013</v>
+        <v>64972278.48101266</v>
       </c>
       <c r="AO142" t="n">
         <v>0</v>
@@ -34403,7 +34403,7 @@
         <v>51.52</v>
       </c>
       <c r="H145" t="n">
-        <v>8501837000</v>
+        <v>8505912000</v>
       </c>
       <c r="I145" t="n">
         <v>0</v>
@@ -34421,7 +34421,7 @@
         <v>10.18</v>
       </c>
       <c r="N145" t="n">
-        <v>1.837125632180223</v>
+        <v>1.838006181519281</v>
       </c>
       <c r="O145" t="n">
         <v>0.73</v>
@@ -34499,7 +34499,7 @@
         <v>441028665.6</v>
       </c>
       <c r="AN145" t="n">
-        <v>1954445287.356322</v>
+        <v>1955382068.965517</v>
       </c>
       <c r="AO145" t="n">
         <v>0</v>
@@ -34638,7 +34638,7 @@
         <v>37.14</v>
       </c>
       <c r="H146" t="n">
-        <v>8501837000</v>
+        <v>8505912000</v>
       </c>
       <c r="I146" t="n">
         <v>800</v>
@@ -34656,7 +34656,7 @@
         <v>8.16</v>
       </c>
       <c r="N146" t="n">
-        <v>1.656848419818276</v>
+        <v>1.657642560815188</v>
       </c>
       <c r="O146" t="n">
         <v>0.58</v>
@@ -34734,7 +34734,7 @@
         <v>489015806.4</v>
       </c>
       <c r="AN146" t="n">
-        <v>2436056446.991404</v>
+        <v>2437224068.767908</v>
       </c>
       <c r="AO146" t="n">
         <v>0</v>
@@ -36518,7 +36518,7 @@
         <v>33.39</v>
       </c>
       <c r="H154" t="n">
-        <v>7349712419</v>
+        <v>7324813000</v>
       </c>
       <c r="I154" t="n">
         <v>3100</v>
@@ -36536,7 +36536,7 @@
         <v>10.95</v>
       </c>
       <c r="N154" t="n">
-        <v>2.348613070147474</v>
+        <v>2.34065641857138</v>
       </c>
       <c r="O154" t="n">
         <v>0.71</v>
@@ -36614,7 +36614,7 @@
         <v>345171067.18</v>
       </c>
       <c r="AN154" t="n">
-        <v>1159260633.911672</v>
+        <v>1155333280.757098</v>
       </c>
       <c r="AO154" t="n">
         <v>0</v>
@@ -36753,7 +36753,7 @@
         <v>33.49</v>
       </c>
       <c r="H155" t="n">
-        <v>7349712419</v>
+        <v>7324813000</v>
       </c>
       <c r="I155" t="n">
         <v>1500</v>
@@ -36771,7 +36771,7 @@
         <v>11.38</v>
       </c>
       <c r="N155" t="n">
-        <v>1.236925852152674</v>
+        <v>1.232735384103194</v>
       </c>
       <c r="O155" t="n">
         <v>0.73</v>
@@ -36849,7 +36849,7 @@
         <v>655393594.0500001</v>
       </c>
       <c r="AN155" t="n">
-        <v>1115282612.898331</v>
+        <v>1111504248.861912</v>
       </c>
       <c r="AO155" t="n">
         <v>0</v>
@@ -40748,7 +40748,7 @@
         <v>3.2</v>
       </c>
       <c r="H172" t="n">
-        <v>172343330</v>
+        <v>172343300</v>
       </c>
       <c r="I172" t="n">
         <v>7600</v>
@@ -40766,7 +40766,7 @@
         <v>0.38</v>
       </c>
       <c r="N172" t="n">
-        <v>0.0381579878871018</v>
+        <v>0.03815798124489733</v>
       </c>
       <c r="O172" t="n">
         <v>0.08</v>
@@ -40844,7 +40844,7 @@
         <v>640901679.6</v>
       </c>
       <c r="AN172" t="n">
-        <v>172343330</v>
+        <v>172343300</v>
       </c>
       <c r="AO172" t="n">
         <v>0</v>
@@ -42628,7 +42628,7 @@
         <v>33.59</v>
       </c>
       <c r="H180" t="n">
-        <v>3235599000</v>
+        <v>3214194000</v>
       </c>
       <c r="I180" t="n">
         <v>0</v>
@@ -42646,7 +42646,7 @@
         <v>12.71</v>
       </c>
       <c r="N180" t="n">
-        <v>7.904857705872969</v>
+        <v>7.852563376694906</v>
       </c>
       <c r="O180" t="n">
         <v>0.8</v>
@@ -42724,7 +42724,7 @@
         <v>84360399.48</v>
       </c>
       <c r="AN180" t="n">
-        <v>419662645.9143969</v>
+        <v>416886381.3229572</v>
       </c>
       <c r="AO180" t="n">
         <v>4.0605</v>
@@ -42863,7 +42863,7 @@
         <v>34.26</v>
       </c>
       <c r="H181" t="n">
-        <v>3235599000</v>
+        <v>3214194000</v>
       </c>
       <c r="I181" t="n">
         <v>200</v>
@@ -42881,7 +42881,7 @@
         <v>13.08</v>
       </c>
       <c r="N181" t="n">
-        <v>3.952428852936484</v>
+        <v>3.926281688347453</v>
       </c>
       <c r="O181" t="n">
         <v>0.83</v>
@@ -42959,7 +42959,7 @@
         <v>168720798.96</v>
       </c>
       <c r="AN181" t="n">
-        <v>407506171.2846348</v>
+        <v>404810327.4559194</v>
       </c>
       <c r="AO181" t="n">
         <v>4.0605</v>
@@ -45448,7 +45448,7 @@
         <v>2.78</v>
       </c>
       <c r="H192" t="n">
-        <v>26080295</v>
+        <v>26497330</v>
       </c>
       <c r="I192" t="n">
         <v>12700</v>
@@ -45466,7 +45466,7 @@
         <v>21.95</v>
       </c>
       <c r="N192" t="n">
-        <v>2.666472514021918</v>
+        <v>2.709110542651775</v>
       </c>
       <c r="O192" t="n">
         <v>0.32</v>
@@ -45544,7 +45544,7 @@
         <v>357000.03</v>
       </c>
       <c r="AN192" t="n">
-        <v>2193464.676198486</v>
+        <v>2228539.108494533</v>
       </c>
       <c r="AO192" t="n">
         <v>0</v>
@@ -45683,7 +45683,7 @@
         <v>1.95</v>
       </c>
       <c r="H193" t="n">
-        <v>26080295</v>
+        <v>26497330</v>
       </c>
       <c r="I193" t="n">
         <v>25600</v>
@@ -45701,7 +45701,7 @@
         <v>14.71</v>
       </c>
       <c r="N193" t="n">
-        <v>1.333236425065956</v>
+        <v>1.354555442068156</v>
       </c>
       <c r="O193" t="n">
         <v>0.22</v>
@@ -45779,7 +45779,7 @@
         <v>713999.97</v>
       </c>
       <c r="AN193" t="n">
-        <v>3272308.030112924</v>
+        <v>3324633.626097867</v>
       </c>
       <c r="AO193" t="n">
         <v>0</v>
@@ -47563,7 +47563,7 @@
         <v>7.51</v>
       </c>
       <c r="H201" t="n">
-        <v>137976728</v>
+        <v>137976800</v>
       </c>
       <c r="I201" t="n">
         <v>8000</v>
@@ -47581,7 +47581,7 @@
         <v>1.99</v>
       </c>
       <c r="N201" t="n">
-        <v>1.628376538246652</v>
+        <v>1.628377387977707</v>
       </c>
       <c r="O201" t="n">
         <v>0.25</v>
@@ -47659,7 +47659,7 @@
         <v>28893848.04</v>
       </c>
       <c r="AN201" t="n">
-        <v>109505339.6825397</v>
+        <v>109505396.8253968</v>
       </c>
       <c r="AO201" t="n">
         <v>0</v>
@@ -56007,7 +56007,7 @@
         <v>3.69</v>
       </c>
       <c r="H237" t="n">
-        <v>17460379</v>
+        <v>17460380</v>
       </c>
       <c r="I237" t="n">
         <v>14000</v>
@@ -56025,7 +56025,7 @@
         <v>5.38</v>
       </c>
       <c r="N237" t="n">
-        <v>0.2515882053513833</v>
+        <v>0.2515882197604752</v>
       </c>
       <c r="O237" t="n">
         <v>0.11</v>
@@ -56103,7 +56103,7 @@
         <v>10271292.68</v>
       </c>
       <c r="AN237" t="n">
-        <v>1733900.595829196</v>
+        <v>1733900.695134062</v>
       </c>
       <c r="AO237" t="n">
         <v>0</v>
@@ -56242,7 +56242,7 @@
         <v>2.48</v>
       </c>
       <c r="H238" t="n">
-        <v>103088665</v>
+        <v>103088600</v>
       </c>
       <c r="I238" t="n">
         <v>6500</v>
@@ -56260,7 +56260,7 @@
         <v>4.2</v>
       </c>
       <c r="N238" t="n">
-        <v>1.203679331241373</v>
+        <v>1.203678572291235</v>
       </c>
       <c r="O238" t="n">
         <v>0.75</v>
@@ -56338,7 +56338,7 @@
         <v>23184000</v>
       </c>
       <c r="AN238" t="n">
-        <v>14897205.92485549</v>
+        <v>14897196.53179191</v>
       </c>
       <c r="AO238" t="n">
         <v>0</v>
@@ -58357,7 +58357,7 @@
         <v>5.39</v>
       </c>
       <c r="H247" t="n">
-        <v>20029067</v>
+        <v>20029070</v>
       </c>
       <c r="I247" t="n">
         <v>3100</v>
@@ -58375,7 +58375,7 @@
         <v>4.4</v>
       </c>
       <c r="N247" t="n">
-        <v>0.03014143847455189</v>
+        <v>0.03014144298920629</v>
       </c>
       <c r="O247" t="n">
         <v>0.05</v>
@@ -58453,7 +58453,7 @@
         <v>5648272.88</v>
       </c>
       <c r="AN247" t="n">
-        <v>33947571.18644068</v>
+        <v>33947576.27118644</v>
       </c>
       <c r="AO247" t="n">
         <v>0</v>
@@ -59767,7 +59767,7 @@
         <v>18.49</v>
       </c>
       <c r="H253" t="n">
-        <v>183440045</v>
+        <v>183440000</v>
       </c>
       <c r="I253" t="n">
         <v>400</v>
@@ -59785,7 +59785,7 @@
         <v>7.29</v>
       </c>
       <c r="N253" t="n">
-        <v>0.1833967633638461</v>
+        <v>0.1833967183744636</v>
       </c>
       <c r="O253" t="n">
         <v>0.12</v>
@@ -59863,7 +59863,7 @@
         <v>24405758.4</v>
       </c>
       <c r="AN253" t="n">
-        <v>126510375.862069</v>
+        <v>126510344.8275862</v>
       </c>
       <c r="AO253" t="n">
         <v>0</v>
@@ -63057,7 +63057,7 @@
         <v>16</v>
       </c>
       <c r="H267" t="n">
-        <v>47009650</v>
+        <v>45276070</v>
       </c>
       <c r="I267" t="n">
         <v>0</v>
@@ -63075,7 +63075,7 @@
         <v>4.28</v>
       </c>
       <c r="N267" t="n">
-        <v>0.6284703405469694</v>
+        <v>0.6052941711229167</v>
       </c>
       <c r="O267" t="n">
         <v>0.1</v>
@@ -63153,7 +63153,7 @@
         <v>2565643.74</v>
       </c>
       <c r="AN267" t="n">
-        <v>73452578.125</v>
+        <v>70743859.375</v>
       </c>
       <c r="AO267" t="n">
         <v>0</v>
@@ -63292,7 +63292,7 @@
         <v>25</v>
       </c>
       <c r="H268" t="n">
-        <v>47009650</v>
+        <v>45276070</v>
       </c>
       <c r="I268" t="n">
         <v>300</v>
@@ -63310,7 +63310,7 @@
         <v>2.74</v>
       </c>
       <c r="N268" t="n">
-        <v>0.3142351702734847</v>
+        <v>0.3026470855614584</v>
       </c>
       <c r="O268" t="n">
         <v>0.07000000000000001</v>
@@ -63388,7 +63388,7 @@
         <v>5131287.48</v>
       </c>
       <c r="AN268" t="n">
-        <v>114657682.9268293</v>
+        <v>110429439.0243903</v>
       </c>
       <c r="AO268" t="n">
         <v>0</v>
@@ -66582,7 +66582,7 @@
         <v>28.66</v>
       </c>
       <c r="H282" t="n">
-        <v>684884290</v>
+        <v>687654900</v>
       </c>
       <c r="I282" t="n">
         <v>500</v>
@@ -66600,7 +66600,7 @@
         <v>17.82</v>
       </c>
       <c r="N282" t="n">
-        <v>0.3490835932888271</v>
+        <v>0.350495765400998</v>
       </c>
       <c r="O282" t="n">
         <v>0.52</v>
@@ -66678,7 +66678,7 @@
         <v>42378103.55</v>
       </c>
       <c r="AN282" t="n">
-        <v>76437978.79464285</v>
+        <v>76747198.66071428</v>
       </c>
       <c r="AO282" t="n">
         <v>0</v>
@@ -66817,7 +66817,7 @@
         <v>30.37</v>
       </c>
       <c r="H283" t="n">
-        <v>684884290</v>
+        <v>687654900</v>
       </c>
       <c r="I283" t="n">
         <v>400</v>
@@ -66835,7 +66835,7 @@
         <v>18.34</v>
       </c>
       <c r="N283" t="n">
-        <v>7.799274393101443</v>
+        <v>7.830825339650779</v>
       </c>
       <c r="O283" t="n">
         <v>0.54</v>
@@ -66913,7 +66913,7 @@
         <v>1896779.1</v>
       </c>
       <c r="AN283" t="n">
-        <v>74201981.58179848</v>
+        <v>74502156.01300108</v>
       </c>
       <c r="AO283" t="n">
         <v>0</v>
@@ -75042,7 +75042,7 @@
         <v>5.48</v>
       </c>
       <c r="H318" t="n">
-        <v>14073757968</v>
+        <v>14073760000</v>
       </c>
       <c r="I318" t="n">
         <v>300</v>
@@ -75060,7 +75060,7 @@
         <v>11.35</v>
       </c>
       <c r="N318" t="n">
-        <v>0.7253526622444696</v>
+        <v>0.7253527669724756</v>
       </c>
       <c r="O318" t="n">
         <v>0.49</v>
@@ -75138,7 +75138,7 @@
         <v>1412512331.45</v>
       </c>
       <c r="AN318" t="n">
-        <v>3113663267.256638</v>
+        <v>3113663716.814159</v>
       </c>
       <c r="AO318" t="n">
         <v>0</v>
@@ -80212,7 +80212,7 @@
         <v>6.27</v>
       </c>
       <c r="H340" t="n">
-        <v>422677188</v>
+        <v>422677200</v>
       </c>
       <c r="I340" t="n">
         <v>21800</v>
@@ -80230,7 +80230,7 @@
         <v>0.62</v>
       </c>
       <c r="N340" t="n">
-        <v>2.858871270808745</v>
+        <v>2.858871351973417</v>
       </c>
       <c r="O340" t="n">
         <v>0.1</v>
@@ -80308,7 +80308,7 @@
         <v>61075833.72000001</v>
       </c>
       <c r="AN340" t="n">
-        <v>459431726.0869565</v>
+        <v>459431739.1304348</v>
       </c>
       <c r="AO340" t="n">
         <v>0</v>
@@ -82797,7 +82797,7 @@
         <v>38.66</v>
       </c>
       <c r="H351" t="n">
-        <v>159454288</v>
+        <v>157023300</v>
       </c>
       <c r="I351" t="n">
         <v>0</v>
@@ -82815,7 +82815,7 @@
         <v>3.42</v>
       </c>
       <c r="N351" t="n">
-        <v>2.075437811099165</v>
+        <v>2.043796364031098</v>
       </c>
       <c r="O351" t="n">
         <v>0.78</v>
@@ -82893,7 +82893,7 @@
         <v>9672800</v>
       </c>
       <c r="AN351" t="n">
-        <v>64296083.87096775</v>
+        <v>63315846.77419355</v>
       </c>
       <c r="AO351" t="n">
         <v>0</v>
@@ -83032,7 +83032,7 @@
         <v>82.09999999999999</v>
       </c>
       <c r="H352" t="n">
-        <v>159454288</v>
+        <v>157023300</v>
       </c>
       <c r="I352" t="n">
         <v>300</v>
@@ -83050,7 +83050,7 @@
         <v>6.19</v>
       </c>
       <c r="N352" t="n">
-        <v>2.264306355213975</v>
+        <v>2.229785480003339</v>
       </c>
       <c r="O352" t="n">
         <v>1.42</v>
@@ -83128,7 +83128,7 @@
         <v>8865980</v>
       </c>
       <c r="AN352" t="n">
-        <v>35434286.22222222</v>
+        <v>34894066.66666666</v>
       </c>
       <c r="AO352" t="n">
         <v>0</v>
@@ -83267,7 +83267,7 @@
         <v>79.52</v>
       </c>
       <c r="H353" t="n">
-        <v>159454288</v>
+        <v>157023300</v>
       </c>
       <c r="I353" t="n">
         <v>0</v>
@@ -83285,7 +83285,7 @@
         <v>6.02</v>
       </c>
       <c r="N353" t="n">
-        <v>2.173711937233433</v>
+        <v>2.140572234932852</v>
       </c>
       <c r="O353" t="n">
         <v>1.38</v>
@@ -83363,7 +83363,7 @@
         <v>9235490</v>
       </c>
       <c r="AN353" t="n">
-        <v>36488395.42334096</v>
+        <v>35932105.2631579</v>
       </c>
       <c r="AO353" t="n">
         <v>0</v>
@@ -88907,7 +88907,7 @@
         <v>1.13</v>
       </c>
       <c r="H377" t="n">
-        <v>74677586</v>
+        <v>74677590</v>
       </c>
       <c r="I377" t="n">
         <v>10600</v>
@@ -88925,7 +88925,7 @@
         <v>39.8</v>
       </c>
       <c r="N377" t="n">
-        <v>0.2768499802773232</v>
+        <v>0.2768499951064035</v>
       </c>
       <c r="O377" t="n">
         <v>0.24</v>
@@ -89003,7 +89003,7 @@
         <v>2643454.56</v>
       </c>
       <c r="AN377" t="n">
-        <v>7051707.837582625</v>
+        <v>7051708.21529745</v>
       </c>
       <c r="AO377" t="n">
         <v>0</v>
@@ -94077,7 +94077,7 @@
         <v>3.62</v>
       </c>
       <c r="H399" t="n">
-        <v>5347521987</v>
+        <v>5492235000</v>
       </c>
       <c r="I399" t="n">
         <v>4500</v>
@@ -94095,7 +94095,7 @@
         <v>9.42</v>
       </c>
       <c r="N399" t="n">
-        <v>0.6027845423165956</v>
+        <v>0.6190969142003432</v>
       </c>
       <c r="O399" t="n">
         <v>0.66</v>
@@ -94173,7 +94173,7 @@
         <v>483489419.2399999</v>
       </c>
       <c r="AN399" t="n">
-        <v>1026395774.856046</v>
+        <v>1054171785.028791</v>
       </c>
       <c r="AO399" t="n">
         <v>0</v>
@@ -94312,7 +94312,7 @@
         <v>3.73</v>
       </c>
       <c r="H400" t="n">
-        <v>5347521987</v>
+        <v>5492235000</v>
       </c>
       <c r="I400" t="n">
         <v>2400</v>
@@ -94330,7 +94330,7 @@
         <v>9.92</v>
       </c>
       <c r="N400" t="n">
-        <v>1.307961330262088</v>
+        <v>1.343356981827403</v>
       </c>
       <c r="O400" t="n">
         <v>0.6899999999999999</v>
@@ -94408,7 +94408,7 @@
         <v>222820003.58</v>
       </c>
       <c r="AN400" t="n">
-        <v>975825180.109489</v>
+        <v>1002232664.233577</v>
       </c>
       <c r="AO400" t="n">
         <v>0</v>
@@ -94782,7 +94782,7 @@
         <v>19.69</v>
       </c>
       <c r="H402" t="n">
-        <v>649912459</v>
+        <v>653159100</v>
       </c>
       <c r="I402" t="n">
         <v>0</v>
@@ -94800,7 +94800,7 @@
         <v>6.94</v>
       </c>
       <c r="N402" t="n">
-        <v>0.4674752114340293</v>
+        <v>0.4698104862343626</v>
       </c>
       <c r="O402" t="n">
         <v>0.53</v>
@@ -94878,7 +94878,7 @@
         <v>53525040.6</v>
       </c>
       <c r="AN402" t="n">
-        <v>160076960.3448276</v>
+        <v>160876625.6157636</v>
       </c>
       <c r="AO402" t="n">
         <v>0.9505</v>
@@ -95017,7 +95017,7 @@
         <v>16.69</v>
       </c>
       <c r="H403" t="n">
-        <v>649912459</v>
+        <v>653159100</v>
       </c>
       <c r="I403" t="n">
         <v>1700</v>
@@ -95035,7 +95035,7 @@
         <v>7.58</v>
       </c>
       <c r="N403" t="n">
-        <v>0.3903874867132386</v>
+        <v>0.3923376693919955</v>
       </c>
       <c r="O403" t="n">
         <v>0.58</v>
@@ -95113,7 +95113,7 @@
         <v>64094343.5</v>
       </c>
       <c r="AN403" t="n">
-        <v>146707101.3544018</v>
+        <v>147439977.4266366</v>
       </c>
       <c r="AO403" t="n">
         <v>0.7018</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-09-09 05:37
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>24.58</v>
+        <v>24.59</v>
       </c>
       <c r="G3" t="n">
-        <v>3287990391</v>
+        <v>3289325632</v>
       </c>
       <c r="H3" t="n">
-        <v>910000</v>
+        <v>665200</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8181252375063874</v>
+        <v>0.8184574752049049</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>642185623.2421875</v>
+        <v>642446412.5</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>44.98</v>
+        <v>45</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,28 +1196,28 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>101.38</v>
+        <v>101.3</v>
       </c>
       <c r="BD3" t="n">
-        <v>64.42</v>
+        <v>64.36</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-80.19</v>
+        <v>-80.2</v>
       </c>
       <c r="BG3" t="n">
-        <v>-14.01</v>
+        <v>-14.05</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
       </c>
       <c r="BI3" t="n">
-        <v>-0.77</v>
+        <v>0.04</v>
       </c>
       <c r="BJ3" t="n">
-        <v>24.77</v>
+        <v>24.58</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>24.99</v>
+        <v>24.88</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>24.4</v>
+        <v>24.51</v>
       </c>
       <c r="BQ3" t="n">
         <v>5.6</v>
       </c>
       <c r="BR3" t="n">
-        <v>24.71</v>
+        <v>24.85</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>492123</v>
+        <v>515457</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.74</v>
+        <v>15.82</v>
       </c>
       <c r="G4" t="n">
-        <v>243728544855</v>
+        <v>244967316474</v>
       </c>
       <c r="H4" t="n">
-        <v>27639000</v>
+        <v>25579200</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.75974575518694</v>
+        <v>2.773772404052444</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>24131539094.55445</v>
+        <v>24254189749.90099</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.65</v>
+        <v>19.75</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,28 +1426,28 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-26.27</v>
+        <v>-26.65</v>
       </c>
       <c r="BD4" t="n">
-        <v>-39.8</v>
+        <v>-40.11</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.84</v>
+        <v>-92.87</v>
       </c>
       <c r="BG4" t="n">
-        <v>-27.66</v>
+        <v>-28.02</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
       </c>
       <c r="BI4" t="n">
-        <v>-0.63</v>
+        <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.84</v>
+        <v>15.82</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.88</v>
+        <v>16.03</v>
       </c>
       <c r="BN4" t="n">
         <v>17</v>
@@ -1465,19 +1465,19 @@
         <v>11.09</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.62</v>
+        <v>15.74</v>
       </c>
       <c r="BQ4" t="n">
-        <v>15.18</v>
+        <v>15.26</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.76</v>
+        <v>15.95</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>31333600</v>
+        <v>31747403</v>
       </c>
     </row>
     <row r="5">
@@ -1743,7 +1743,7 @@
         <v>466195850</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I6" t="n">
         <v>63084700</v>
@@ -1916,7 +1916,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>0</v>
+        <v>7.39</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
@@ -1925,19 +1925,19 @@
         <v>5.96</v>
       </c>
       <c r="BP6" t="n">
-        <v>0</v>
+        <v>7.39</v>
       </c>
       <c r="BQ6" t="n">
         <v>13.14</v>
       </c>
       <c r="BR6" t="n">
-        <v>0</v>
+        <v>7.39</v>
       </c>
       <c r="BS6" t="n">
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>482</v>
+        <v>377</v>
       </c>
     </row>
     <row r="7">
@@ -2427,13 +2427,13 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>23.89</v>
+        <v>23.01</v>
       </c>
       <c r="G9" t="n">
         <v>208480200</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="I9" t="n">
         <v>8407877</v>
@@ -2576,16 +2576,16 @@
         <v>0</v>
       </c>
       <c r="BC9" t="n">
-        <v>186.3</v>
+        <v>197.25</v>
       </c>
       <c r="BD9" t="n">
-        <v>133.76</v>
+        <v>142.7</v>
       </c>
       <c r="BE9" t="n">
         <v>-100</v>
       </c>
       <c r="BF9" t="n">
-        <v>-75.39</v>
+        <v>-74.45</v>
       </c>
       <c r="BG9" t="n">
         <v>-100</v>
@@ -2594,7 +2594,7 @@
         <v>35.36</v>
       </c>
       <c r="BI9" t="n">
-        <v>0</v>
+        <v>-3.68</v>
       </c>
       <c r="BJ9" t="n">
         <v>23.89</v>
@@ -2606,7 +2606,7 @@
         <v>5.88</v>
       </c>
       <c r="BM9" t="n">
-        <v>0</v>
+        <v>23.01</v>
       </c>
       <c r="BN9" t="n">
         <v>34.04</v>
@@ -2615,13 +2615,13 @@
         <v>21.5</v>
       </c>
       <c r="BP9" t="n">
-        <v>0</v>
+        <v>23.01</v>
       </c>
       <c r="BQ9" t="n">
-        <v>4.06</v>
+        <v>3.91</v>
       </c>
       <c r="BR9" t="n">
-        <v>0</v>
+        <v>23.01</v>
       </c>
       <c r="BS9" t="n">
         <v>0.4</v>
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5.19</v>
+        <v>5.2</v>
       </c>
       <c r="G12" t="n">
-        <v>498040294</v>
+        <v>498999989</v>
       </c>
       <c r="H12" t="n">
-        <v>401000</v>
+        <v>553300</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.09006982719259604</v>
+        <v>0.09024338656891348</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>535527197.8494623</v>
+        <v>536559127.9569892</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>7.02</v>
+        <v>7.03</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,28 +3266,28 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>619.6</v>
+        <v>618.22</v>
       </c>
       <c r="BD12" t="n">
-        <v>487.55</v>
+        <v>486.42</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-15</v>
+        <v>-15.16</v>
       </c>
       <c r="BG12" t="n">
-        <v>249.11</v>
+        <v>248.44</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
       </c>
       <c r="BI12" t="n">
-        <v>0.58</v>
+        <v>0.19</v>
       </c>
       <c r="BJ12" t="n">
-        <v>5.16</v>
+        <v>5.19</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3305,19 +3305,19 @@
         <v>4.42</v>
       </c>
       <c r="BP12" t="n">
-        <v>5.15</v>
+        <v>5.16</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.51</v>
+        <v>1.52</v>
       </c>
       <c r="BR12" t="n">
-        <v>5.25</v>
+        <v>5.16</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>445753</v>
+        <v>452237</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>28.81</v>
+        <v>29.22</v>
       </c>
       <c r="G13" t="n">
-        <v>14525742440</v>
+        <v>14732457751</v>
       </c>
       <c r="H13" t="n">
-        <v>4062000</v>
+        <v>5794500</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>5.023841515800142</v>
+        <v>5.095335621223186</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1511523667.013528</v>
+        <v>1533034105.202914</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>52.15</v>
+        <v>52.89</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,28 +3496,28 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>13.06</v>
+        <v>11.48</v>
       </c>
       <c r="BD13" t="n">
-        <v>-7.68</v>
+        <v>-8.98</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-90.95999999999999</v>
+        <v>-91.09</v>
       </c>
       <c r="BG13" t="n">
-        <v>-69.81999999999999</v>
+        <v>-70.25</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
       </c>
       <c r="BI13" t="n">
-        <v>0.03</v>
+        <v>1.42</v>
       </c>
       <c r="BJ13" t="n">
-        <v>28.8</v>
+        <v>28.81</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>29.06</v>
+        <v>29.49</v>
       </c>
       <c r="BN13" t="n">
         <v>32.43</v>
@@ -3535,19 +3535,19 @@
         <v>21.06</v>
       </c>
       <c r="BP13" t="n">
-        <v>28.56</v>
+        <v>28.96</v>
       </c>
       <c r="BQ13" t="n">
-        <v>14.72</v>
+        <v>14.93</v>
       </c>
       <c r="BR13" t="n">
-        <v>28.95</v>
+        <v>29.32</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>4345510</v>
+        <v>4385448</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>10.2</v>
+        <v>10</v>
       </c>
       <c r="G14" t="n">
-        <v>8022662525</v>
+        <v>7813653684</v>
       </c>
       <c r="H14" t="n">
-        <v>1300</v>
+        <v>35600</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.331152104735997</v>
+        <v>3.244367918259752</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>890417594.3396226</v>
+        <v>867220164.7058824</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>8.19</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,25 +3726,25 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>8.65</v>
+        <v>10.83</v>
       </c>
       <c r="BD14" t="n">
-        <v>-11.28</v>
+        <v>-9.51</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-86.06999999999999</v>
+        <v>-85.79000000000001</v>
       </c>
       <c r="BG14" t="n">
-        <v>-41.74</v>
+        <v>-40.58</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
       </c>
       <c r="BI14" t="n">
-        <v>0</v>
+        <v>-1.96</v>
       </c>
       <c r="BJ14" t="n">
         <v>10.2</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>10.2</v>
+        <v>10.02</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,19 +3765,19 @@
         <v>7.65</v>
       </c>
       <c r="BP14" t="n">
-        <v>9.93</v>
+        <v>9.57</v>
       </c>
       <c r="BQ14" t="n">
-        <v>10.07</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="BR14" t="n">
-        <v>9.93</v>
+        <v>9.99</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>11450</v>
+        <v>11380</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>13.57</v>
+        <v>13.05</v>
       </c>
       <c r="G15" t="n">
-        <v>8022662525</v>
+        <v>7813653684</v>
       </c>
       <c r="H15" t="n">
-        <v>3030500</v>
+        <v>9515700</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.291971182217715</v>
+        <v>3.206207749036195</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>669112804.4203503</v>
+        <v>651680874.3953295</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>9.02</v>
+        <v>8.68</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,25 +3956,25 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-18.33</v>
+        <v>-15.07</v>
       </c>
       <c r="BD15" t="n">
-        <v>-33.32</v>
+        <v>-30.66</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-89.53</v>
+        <v>-89.11</v>
       </c>
       <c r="BG15" t="n">
-        <v>-54.4</v>
+        <v>-52.58</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
       </c>
       <c r="BI15" t="n">
-        <v>0</v>
+        <v>-3.83</v>
       </c>
       <c r="BJ15" t="n">
         <v>13.57</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>13.75</v>
+        <v>13.74</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>13.38</v>
+        <v>12.51</v>
       </c>
       <c r="BQ15" t="n">
-        <v>13.4</v>
+        <v>12.88</v>
       </c>
       <c r="BR15" t="n">
-        <v>13.75</v>
+        <v>13.69</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>1931513</v>
+        <v>1967073</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.5</v>
+        <v>4.37</v>
       </c>
       <c r="G16" t="n">
-        <v>986875650</v>
+        <v>958365883</v>
       </c>
       <c r="H16" t="n">
-        <v>52300</v>
+        <v>179500</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4668749297470486</v>
+        <v>0.4533874194763983</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>277212261.2359551</v>
+        <v>269203899.7191011</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4177,7 +4177,7 @@
         <v>1.42</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="BA16" t="n">
         <v>0.08</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-61.36</v>
+        <v>-60.21</v>
       </c>
       <c r="BD16" t="n">
-        <v>-68.45</v>
+        <v>-67.51000000000001</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.22</v>
+        <v>-98.17</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4204,7 +4204,7 @@
         <v>1.68</v>
       </c>
       <c r="BI16" t="n">
-        <v>0</v>
+        <v>-2.89</v>
       </c>
       <c r="BJ16" t="n">
         <v>4.5</v>
@@ -4216,7 +4216,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.6</v>
+        <v>4.58</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
@@ -4225,19 +4225,19 @@
         <v>2.96</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.48</v>
+        <v>4.35</v>
       </c>
       <c r="BQ16" t="n">
-        <v>61.41</v>
+        <v>59.63</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.53</v>
+        <v>4.58</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>137287</v>
+        <v>136900</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>33.64</v>
+        <v>33.91</v>
       </c>
       <c r="G17" t="n">
-        <v>11088641986</v>
+        <v>11177648128</v>
       </c>
       <c r="H17" t="n">
-        <v>1272000</v>
+        <v>523500</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>5007515347.723989</v>
+        <v>5047709595.375723</v>
       </c>
       <c r="AL17" t="n">
-        <v>1386080248.25</v>
+        <v>1397206016</v>
       </c>
       <c r="AM17" t="n">
-        <v>3433016094.736842</v>
+        <v>3460572175.851393</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>18</v>
+        <v>18.14</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>56.47</v>
+        <v>55.23</v>
       </c>
       <c r="BD17" t="n">
-        <v>27.76</v>
+        <v>26.74</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-86.48</v>
+        <v>-86.59</v>
       </c>
       <c r="BG17" t="n">
-        <v>-51.45</v>
+        <v>-51.83</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>33.64</v>
+        <v>33.91</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,28 +4446,28 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>33.78</v>
+        <v>34.12</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
       </c>
       <c r="BO17" t="n">
-        <v>29.03</v>
+        <v>29.28</v>
       </c>
       <c r="BP17" t="n">
-        <v>33.05</v>
+        <v>33.41</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.67</v>
+        <v>2.69</v>
       </c>
       <c r="BR17" t="n">
-        <v>33.31</v>
+        <v>33.78</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1046988</v>
+        <v>1079027</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>11.66</v>
+        <v>11.65</v>
       </c>
       <c r="G18" t="n">
-        <v>11088641986</v>
+        <v>11177648128</v>
       </c>
       <c r="H18" t="n">
-        <v>5300</v>
+        <v>3700</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.264931663056448</v>
+        <v>3.291138566624007</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3300191067.261905</v>
+        <v>3326680990.476191</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4646,25 +4646,25 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>50.3</v>
+        <v>50.43</v>
       </c>
       <c r="BD18" t="n">
-        <v>22.72</v>
+        <v>22.82</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-87.03</v>
+        <v>-87.02</v>
       </c>
       <c r="BG18" t="n">
-        <v>-53.31</v>
+        <v>-53.27</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
       </c>
       <c r="BI18" t="n">
-        <v>0</v>
+        <v>-0.09</v>
       </c>
       <c r="BJ18" t="n">
         <v>11.66</v>
@@ -4685,19 +4685,19 @@
         <v>10.11</v>
       </c>
       <c r="BP18" t="n">
-        <v>11.45</v>
+        <v>11.65</v>
       </c>
       <c r="BQ18" t="n">
         <v>0.92</v>
       </c>
       <c r="BR18" t="n">
-        <v>11.56</v>
+        <v>11.99</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>9740</v>
+        <v>9863</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.92</v>
+        <v>11.07</v>
       </c>
       <c r="G19" t="n">
-        <v>11088641986</v>
+        <v>11177648128</v>
       </c>
       <c r="H19" t="n">
-        <v>7000</v>
+        <v>9400</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.907616273696295</v>
+        <v>6.96306222241701</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3520203805.079365</v>
+        <v>3548459723.174603</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>6.01</v>
+        <v>6.09</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,25 +4876,25 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>60.49</v>
+        <v>58.31</v>
       </c>
       <c r="BD19" t="n">
-        <v>31.04</v>
+        <v>29.26</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-86.15000000000001</v>
+        <v>-86.34</v>
       </c>
       <c r="BG19" t="n">
-        <v>-51.92</v>
+        <v>-52.57</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
       </c>
       <c r="BI19" t="n">
-        <v>0</v>
+        <v>1.37</v>
       </c>
       <c r="BJ19" t="n">
         <v>10.92</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>10.99</v>
+        <v>11.1</v>
       </c>
       <c r="BN19" t="n">
         <v>11.41</v>
@@ -4915,19 +4915,19 @@
         <v>8.98</v>
       </c>
       <c r="BP19" t="n">
-        <v>10.82</v>
+        <v>10.83</v>
       </c>
       <c r="BQ19" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="BR19" t="n">
-        <v>10.88</v>
+        <v>10.83</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>13862</v>
+        <v>13971</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5.55</v>
+        <v>5.42</v>
       </c>
       <c r="G22" t="n">
-        <v>1111360898</v>
+        <v>1085328999</v>
       </c>
       <c r="H22" t="n">
-        <v>1569300</v>
+        <v>1444100</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.09426186138245071</v>
+        <v>0.09205392401532198</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>252009273.9229025</v>
+        <v>246106348.9795918</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,28 +5566,28 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>435.23</v>
+        <v>448.06</v>
       </c>
       <c r="BD22" t="n">
-        <v>337.01</v>
+        <v>347.49</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-65.95</v>
+        <v>-65.13</v>
       </c>
       <c r="BG22" t="n">
-        <v>3007.92</v>
+        <v>3082.47</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
       </c>
       <c r="BI22" t="n">
-        <v>0.36</v>
+        <v>-2.34</v>
       </c>
       <c r="BJ22" t="n">
-        <v>5.53</v>
+        <v>5.55</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>5.57</v>
+        <v>5.68</v>
       </c>
       <c r="BN22" t="n">
         <v>8.82</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>5.15</v>
+        <v>5.42</v>
       </c>
       <c r="BQ22" t="n">
-        <v>8.27</v>
+        <v>8.07</v>
       </c>
       <c r="BR22" t="n">
-        <v>5.15</v>
+        <v>5.59</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1574097</v>
+        <v>1598837</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.93</v>
+        <v>3.05</v>
       </c>
       <c r="G24" t="n">
-        <v>1183335024</v>
+        <v>1231800125</v>
       </c>
       <c r="H24" t="n">
-        <v>5843700</v>
+        <v>8673200</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2860603873994232</v>
+        <v>0.2977763809990618</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1066067589.189189</v>
+        <v>1109729842.342342</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>1.35</v>
+        <v>1.41</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,28 +6026,28 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>144.25</v>
+        <v>134.64</v>
       </c>
       <c r="BD24" t="n">
-        <v>99.43000000000001</v>
+        <v>91.58</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-87.03</v>
+        <v>-87.54000000000001</v>
       </c>
       <c r="BG24" t="n">
-        <v>-50.25</v>
+        <v>-52.2</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
       </c>
       <c r="BI24" t="n">
-        <v>-1.35</v>
+        <v>4.1</v>
       </c>
       <c r="BJ24" t="n">
-        <v>2.97</v>
+        <v>2.93</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>2.97</v>
+        <v>3.05</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.8</v>
+        <v>2.93</v>
       </c>
       <c r="BQ24" t="n">
-        <v>7.2</v>
+        <v>7.49</v>
       </c>
       <c r="BR24" t="n">
-        <v>2.84</v>
+        <v>2.99</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>10086517</v>
+        <v>9586443</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>3.84</v>
+        <v>4.13</v>
       </c>
       <c r="G25" t="n">
-        <v>1330536546</v>
+        <v>1431020259</v>
       </c>
       <c r="H25" t="n">
-        <v>511700</v>
+        <v>1595300</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.6634662744918277</v>
+        <v>0.713572041906965</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>489167847.7941176</v>
+        <v>526110389.3382353</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>8.949999999999999</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,28 +6256,28 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>4.42</v>
+        <v>-2.91</v>
       </c>
       <c r="BD25" t="n">
-        <v>-14.74</v>
+        <v>-20.73</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-93.97</v>
+        <v>-94.39</v>
       </c>
       <c r="BG25" t="n">
-        <v>-42.72</v>
+        <v>-46.74</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
       </c>
       <c r="BI25" t="n">
-        <v>-0.26</v>
+        <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>3.85</v>
+        <v>4.13</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>3.88</v>
+        <v>4.16</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>3.7</v>
+        <v>3.86</v>
       </c>
       <c r="BQ25" t="n">
-        <v>16.23</v>
+        <v>17.45</v>
       </c>
       <c r="BR25" t="n">
-        <v>3.78</v>
+        <v>3.86</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1019877</v>
+        <v>1018647</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>9.08</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="G26" t="n">
-        <v>12297888336</v>
+        <v>12365608244</v>
       </c>
       <c r="H26" t="n">
-        <v>8201900</v>
+        <v>13676600</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.15858023339765</v>
+        <v>0.1594534759026149</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>4392102977.142858</v>
+        <v>4416288658.571429</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>1.74</v>
+        <v>1.75</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,28 +6486,28 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-4.67</v>
+        <v>-5.19</v>
       </c>
       <c r="BD26" t="n">
-        <v>-22.16</v>
+        <v>-22.59</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-92.73999999999999</v>
+        <v>-92.78</v>
       </c>
       <c r="BG26" t="n">
-        <v>-86.86</v>
+        <v>-86.93000000000001</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
       </c>
       <c r="BI26" t="n">
-        <v>-0.77</v>
+        <v>0.55</v>
       </c>
       <c r="BJ26" t="n">
-        <v>9.15</v>
+        <v>9.08</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,7 +6516,7 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>9.27</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="BN26" t="n">
         <v>10.6</v>
@@ -6525,19 +6525,19 @@
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>9.01</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="BQ26" t="n">
-        <v>12.66</v>
+        <v>12.73</v>
       </c>
       <c r="BR26" t="n">
-        <v>9.039999999999999</v>
+        <v>9.26</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>11232863</v>
+        <v>11236307</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>17.69</v>
+        <v>17.05</v>
       </c>
       <c r="G34" t="n">
-        <v>3652804672</v>
+        <v>3520650932</v>
       </c>
       <c r="H34" t="n">
-        <v>3075900</v>
+        <v>3813700</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.3211241932748919</v>
+        <v>0.3095063360510825</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>759418850.7276508</v>
+        <v>731944060.7068608</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>41.28</v>
+        <v>39.78</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,28 +8314,28 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>109.66</v>
+        <v>117.53</v>
       </c>
       <c r="BD34" t="n">
-        <v>71.18000000000001</v>
+        <v>77.61</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-87.03</v>
+        <v>-86.54000000000001</v>
       </c>
       <c r="BG34" t="n">
-        <v>42.78</v>
+        <v>48.14</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
       </c>
       <c r="BI34" t="n">
-        <v>-0.39</v>
+        <v>-3.62</v>
       </c>
       <c r="BJ34" t="n">
-        <v>17.76</v>
+        <v>17.69</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,28 +8344,28 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>17.76</v>
+        <v>18.28</v>
       </c>
       <c r="BN34" t="n">
-        <v>31.28</v>
+        <v>31.12</v>
       </c>
       <c r="BO34" t="n">
         <v>14.32</v>
       </c>
       <c r="BP34" t="n">
-        <v>16.67</v>
+        <v>16.75</v>
       </c>
       <c r="BQ34" t="n">
-        <v>11.22</v>
+        <v>10.81</v>
       </c>
       <c r="BR34" t="n">
-        <v>16.99</v>
+        <v>17.87</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>2938220</v>
+        <v>2990130</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>17.37</v>
+        <v>17.64</v>
       </c>
       <c r="G35" t="n">
-        <v>87657709235</v>
+        <v>89020239279</v>
       </c>
       <c r="H35" t="n">
-        <v>29095000</v>
+        <v>35875800</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.277374879893125</v>
+        <v>7.39049261935769</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7244438779.752067</v>
+        <v>7357044568.512397</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.13</v>
+        <v>10.29</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,28 +8544,28 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-45.85</v>
+        <v>-46.67</v>
       </c>
       <c r="BD35" t="n">
-        <v>-55.78</v>
+        <v>-56.46</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-93.59</v>
+        <v>-93.68000000000001</v>
       </c>
       <c r="BG35" t="n">
-        <v>-47.51</v>
+        <v>-48.32</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
       </c>
       <c r="BI35" t="n">
-        <v>0.52</v>
+        <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>17.28</v>
+        <v>17.64</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>17.61</v>
+        <v>17.88</v>
       </c>
       <c r="BN35" t="n">
         <v>20.08</v>
@@ -8583,19 +8583,19 @@
         <v>11.7</v>
       </c>
       <c r="BP35" t="n">
-        <v>17.12</v>
+        <v>17.55</v>
       </c>
       <c r="BQ35" t="n">
-        <v>16.62</v>
+        <v>16.88</v>
       </c>
       <c r="BR35" t="n">
-        <v>17.25</v>
+        <v>17.68</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>34640477</v>
+        <v>34435973</v>
       </c>
     </row>
     <row r="36">
@@ -8625,13 +8625,13 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>26</v>
+        <v>25.9</v>
       </c>
       <c r="G36" t="n">
-        <v>200850857</v>
+        <v>198305054</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I36" t="n">
         <v>4900000</v>
@@ -8646,7 +8646,7 @@
         <v>1.52</v>
       </c>
       <c r="M36" t="n">
-        <v>1.955452287428218</v>
+        <v>1.93066675066702</v>
       </c>
       <c r="N36" t="n">
         <v>0.87</v>
@@ -8724,7 +8724,7 @@
         <v>11319000</v>
       </c>
       <c r="AM36" t="n">
-        <v>27665407.30027548</v>
+        <v>27314745.73002755</v>
       </c>
       <c r="AN36" t="n">
         <v>0</v>
@@ -8765,7 +8765,7 @@
         <v>24.36</v>
       </c>
       <c r="AZ36" t="n">
-        <v>66.65000000000001</v>
+        <v>66.39</v>
       </c>
       <c r="BA36" t="n">
         <v>2.44</v>
@@ -8774,25 +8774,25 @@
         <v>14.49</v>
       </c>
       <c r="BC36" t="n">
-        <v>14.76</v>
+        <v>15.21</v>
       </c>
       <c r="BD36" t="n">
-        <v>-6.3</v>
+        <v>-5.93</v>
       </c>
       <c r="BE36" t="n">
         <v>156.33</v>
       </c>
       <c r="BF36" t="n">
-        <v>-90.59999999999999</v>
+        <v>-90.56</v>
       </c>
       <c r="BG36" t="n">
-        <v>-44.28</v>
+        <v>-44.06</v>
       </c>
       <c r="BH36" t="n">
         <v>17.13</v>
       </c>
       <c r="BI36" t="n">
-        <v>0</v>
+        <v>-0.38</v>
       </c>
       <c r="BJ36" t="n">
         <v>26</v>
@@ -8804,7 +8804,7 @@
         <v>2.31</v>
       </c>
       <c r="BM36" t="n">
-        <v>0</v>
+        <v>25.9</v>
       </c>
       <c r="BN36" t="n">
         <v>29.05</v>
@@ -8813,13 +8813,13 @@
         <v>17.14</v>
       </c>
       <c r="BP36" t="n">
-        <v>0</v>
+        <v>25.9</v>
       </c>
       <c r="BQ36" t="n">
-        <v>11.25</v>
+        <v>11.2</v>
       </c>
       <c r="BR36" t="n">
-        <v>0</v>
+        <v>25.9</v>
       </c>
       <c r="BS36" t="n">
         <v>1.24</v>
@@ -8855,13 +8855,13 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>14.99</v>
+        <v>14.8</v>
       </c>
       <c r="G37" t="n">
-        <v>200851000</v>
+        <v>198305054</v>
       </c>
       <c r="H37" t="n">
-        <v>500</v>
+        <v>2100</v>
       </c>
       <c r="I37" t="n">
         <v>4900000</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.955453679653679</v>
+        <v>1.93066675066702</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>48050478.46889953</v>
+        <v>47441400.4784689</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -8995,7 +8995,7 @@
         <v>24.36</v>
       </c>
       <c r="AZ37" t="n">
-        <v>66.66</v>
+        <v>65.81</v>
       </c>
       <c r="BA37" t="n">
         <v>2.44</v>
@@ -9004,25 +9004,25 @@
         <v>15.53</v>
       </c>
       <c r="BC37" t="n">
-        <v>99.06</v>
+        <v>101.61</v>
       </c>
       <c r="BD37" t="n">
-        <v>62.53</v>
+        <v>64.61</v>
       </c>
       <c r="BE37" t="n">
         <v>344.67</v>
       </c>
       <c r="BF37" t="n">
-        <v>-83.69</v>
+        <v>-83.48</v>
       </c>
       <c r="BG37" t="n">
-        <v>3.62</v>
+        <v>4.95</v>
       </c>
       <c r="BH37" t="n">
         <v>17.13</v>
       </c>
       <c r="BI37" t="n">
-        <v>0</v>
+        <v>-1.27</v>
       </c>
       <c r="BJ37" t="n">
         <v>14.99</v>
@@ -9034,7 +9034,7 @@
         <v>2.31</v>
       </c>
       <c r="BM37" t="n">
-        <v>14.99</v>
+        <v>15</v>
       </c>
       <c r="BN37" t="n">
         <v>20.9</v>
@@ -9043,19 +9043,19 @@
         <v>12.9</v>
       </c>
       <c r="BP37" t="n">
-        <v>14.99</v>
+        <v>14.8</v>
       </c>
       <c r="BQ37" t="n">
-        <v>6.48</v>
+        <v>6.4</v>
       </c>
       <c r="BR37" t="n">
-        <v>14.99</v>
+        <v>15</v>
       </c>
       <c r="BS37" t="n">
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>830</v>
+        <v>837</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>68.15000000000001</v>
+        <v>69.48999999999999</v>
       </c>
       <c r="G39" t="n">
-        <v>3820373912</v>
+        <v>3895491842</v>
       </c>
       <c r="H39" t="n">
-        <v>4100</v>
+        <v>2600</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1917660128285953</v>
+        <v>0.1955366034199482</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>401299780.6722689</v>
+        <v>409190319.5378152</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>199.11</v>
+        <v>203.03</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,25 +9464,25 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>205.95</v>
+        <v>200.05</v>
       </c>
       <c r="BD39" t="n">
-        <v>149.81</v>
+        <v>144.99</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-72.11</v>
+        <v>-72.64</v>
       </c>
       <c r="BG39" t="n">
-        <v>34.59</v>
+        <v>32</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
       </c>
       <c r="BI39" t="n">
-        <v>0</v>
+        <v>1.97</v>
       </c>
       <c r="BJ39" t="n">
         <v>68.15000000000001</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>68.97</v>
+        <v>69.97</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>67.53</v>
+        <v>68.15000000000001</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.52</v>
+        <v>4.61</v>
       </c>
       <c r="BR39" t="n">
-        <v>67.53</v>
+        <v>68.15000000000001</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3993</v>
+        <v>4080</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>22.52</v>
+        <v>22.6</v>
       </c>
       <c r="G40" t="n">
-        <v>129058406823</v>
+        <v>129516850586</v>
       </c>
       <c r="H40" t="n">
-        <v>26788000</v>
+        <v>30149100</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.3915791780314469</v>
+        <v>0.392970153143478</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6693900768.827801</v>
+        <v>6717678972.302904</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>11.37</v>
+        <v>11.41</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,28 +9694,28 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>96.48999999999999</v>
+        <v>95.79000000000001</v>
       </c>
       <c r="BD40" t="n">
-        <v>60.43</v>
+        <v>59.86</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-87.75</v>
+        <v>-87.79000000000001</v>
       </c>
       <c r="BG40" t="n">
-        <v>23.85</v>
+        <v>23.41</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
       </c>
       <c r="BI40" t="n">
-        <v>-0.04</v>
+        <v>0.36</v>
       </c>
       <c r="BJ40" t="n">
-        <v>22.53</v>
+        <v>22.52</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>22.73</v>
+        <v>23.21</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>22.11</v>
+        <v>22.58</v>
       </c>
       <c r="BQ40" t="n">
-        <v>9.01</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="BR40" t="n">
-        <v>22.32</v>
+        <v>22.84</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>28692737</v>
+        <v>29100909</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>15.81</v>
+        <v>16.04</v>
       </c>
       <c r="G41" t="n">
-        <v>188210977989</v>
+        <v>192079241161</v>
       </c>
       <c r="H41" t="n">
-        <v>9542100</v>
+        <v>8647400</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.254232020637266</v>
+        <v>1.28001000440003</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>29000150691.6795</v>
+        <v>29596185078.73652</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>23.66</v>
+        <v>24.01</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,28 +9924,28 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>89.03</v>
+        <v>86.31999999999999</v>
       </c>
       <c r="BD41" t="n">
-        <v>54.34</v>
+        <v>52.13</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-84.02</v>
+        <v>-84.23999999999999</v>
       </c>
       <c r="BG41" t="n">
-        <v>-12.9</v>
+        <v>-14.15</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
       </c>
       <c r="BI41" t="n">
-        <v>0.83</v>
+        <v>1.45</v>
       </c>
       <c r="BJ41" t="n">
-        <v>15.68</v>
+        <v>15.81</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,7 +9954,7 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>15.87</v>
+        <v>16.29</v>
       </c>
       <c r="BN41" t="n">
         <v>18.28</v>
@@ -9963,19 +9963,19 @@
         <v>13.34</v>
       </c>
       <c r="BP41" t="n">
-        <v>15.5</v>
+        <v>15.96</v>
       </c>
       <c r="BQ41" t="n">
-        <v>6.76</v>
+        <v>6.86</v>
       </c>
       <c r="BR41" t="n">
-        <v>15.67</v>
+        <v>15.99</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>6816525</v>
+        <v>7057236</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>17.9</v>
+        <v>18.22</v>
       </c>
       <c r="G42" t="n">
-        <v>188210977989</v>
+        <v>192079241161</v>
       </c>
       <c r="H42" t="n">
-        <v>44559000</v>
+        <v>43084300</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.25796272378815</v>
+        <v>1.283817383958201</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>25606935780.81633</v>
+        <v>26133230089.93197</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>25.93</v>
+        <v>26.39</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,28 +10154,28 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>66.95999999999999</v>
+        <v>64.03</v>
       </c>
       <c r="BD42" t="n">
-        <v>36.32</v>
+        <v>33.93</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-85.88</v>
+        <v>-86.13</v>
       </c>
       <c r="BG42" t="n">
-        <v>-15.56</v>
+        <v>-17.04</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
       </c>
       <c r="BI42" t="n">
-        <v>-0.06</v>
+        <v>1.79</v>
       </c>
       <c r="BJ42" t="n">
-        <v>17.91</v>
+        <v>17.9</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>17.98</v>
+        <v>18.49</v>
       </c>
       <c r="BN42" t="n">
         <v>21.33</v>
@@ -10193,19 +10193,19 @@
         <v>15.64</v>
       </c>
       <c r="BP42" t="n">
-        <v>17.63</v>
+        <v>18.08</v>
       </c>
       <c r="BQ42" t="n">
-        <v>7.66</v>
+        <v>7.79</v>
       </c>
       <c r="BR42" t="n">
-        <v>17.74</v>
+        <v>18.1</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>37610992</v>
+        <v>38628200</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>42.16</v>
+        <v>42.35</v>
       </c>
       <c r="G43" t="n">
-        <v>81849423703</v>
+        <v>82218244687</v>
       </c>
       <c r="H43" t="n">
-        <v>4935200</v>
+        <v>5026300</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9969479135.566381</v>
+        <v>10014402519.73203</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>76.52</v>
+        <v>76.87</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,28 +10384,28 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-42.04</v>
+        <v>-42.3</v>
       </c>
       <c r="BD43" t="n">
-        <v>-52.68</v>
+        <v>-52.89</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-86.65000000000001</v>
+        <v>-86.70999999999999</v>
       </c>
       <c r="BG43" t="n">
-        <v>15.32</v>
+        <v>14.8</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
       </c>
       <c r="BI43" t="n">
-        <v>-0.09</v>
+        <v>0.45</v>
       </c>
       <c r="BJ43" t="n">
-        <v>42.2</v>
+        <v>42.16</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>42.28</v>
+        <v>42.79</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>41.38</v>
+        <v>41.82</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.91</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="BR43" t="n">
-        <v>41.74</v>
+        <v>42.48</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6489121</v>
+        <v>6436722</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>3.95</v>
+        <v>3.96</v>
       </c>
       <c r="G46" t="n">
-        <v>3952136997</v>
+        <v>3962142398</v>
       </c>
       <c r="H46" t="n">
-        <v>47216200</v>
+        <v>31049400</v>
       </c>
       <c r="I46" t="n">
         <v>1000541644</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.06869560877481121</v>
+        <v>0.06886952154991309</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249156.24</v>
       </c>
       <c r="AM46" t="n">
-        <v>3874644114.705882</v>
+        <v>3884453331.372549</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.26</v>
+        <v>3.27</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,25 +11074,25 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>2.38</v>
+        <v>2.12</v>
       </c>
       <c r="BD46" t="n">
-        <v>-16.41</v>
+        <v>-16.62</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.29000000000001</v>
+        <v>-89.31999999999999</v>
       </c>
       <c r="BG46" t="n">
-        <v>86.8</v>
+        <v>86.33</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
       </c>
       <c r="BI46" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="BJ46" t="n">
         <v>3.95</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.08</v>
+        <v>3.99</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>3.79</v>
+        <v>3.8</v>
       </c>
       <c r="BQ46" t="n">
-        <v>8.640000000000001</v>
+        <v>8.66</v>
       </c>
       <c r="BR46" t="n">
-        <v>3.8</v>
+        <v>3.99</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>15490403</v>
+        <v>16708023</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>8.85</v>
+        <v>8.91</v>
       </c>
       <c r="G47" t="n">
-        <v>3086619000</v>
+        <v>3107545101</v>
       </c>
       <c r="H47" t="n">
-        <v>7000</v>
+        <v>7700</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7278602725543464</v>
+        <v>0.7327948879303807</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>547272872.3404256</v>
+        <v>550983173.9361702</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>11.62</v>
+        <v>11.7</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,28 +11304,28 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>62.41</v>
+        <v>61.32</v>
       </c>
       <c r="BD47" t="n">
-        <v>32.61</v>
+        <v>31.72</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-83.52</v>
+        <v>-83.63</v>
       </c>
       <c r="BG47" t="n">
-        <v>-2.6</v>
+        <v>-3.26</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
       </c>
       <c r="BI47" t="n">
-        <v>-0.34</v>
+        <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>8.880000000000001</v>
+        <v>8.91</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11334,7 +11334,7 @@
         <v>1.29</v>
       </c>
       <c r="BM47" t="n">
-        <v>8.93</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="BN47" t="n">
         <v>9.25</v>
@@ -11343,19 +11343,19 @@
         <v>7.2</v>
       </c>
       <c r="BP47" t="n">
-        <v>8.83</v>
+        <v>8.85</v>
       </c>
       <c r="BQ47" t="n">
-        <v>6.84</v>
+        <v>6.89</v>
       </c>
       <c r="BR47" t="n">
-        <v>8.93</v>
+        <v>8.9</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>12773</v>
+        <v>12638</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>8.970000000000001</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="G48" t="n">
-        <v>3086619000</v>
+        <v>3107545101</v>
       </c>
       <c r="H48" t="n">
-        <v>3700</v>
+        <v>2900</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>1.980288637710655</v>
+        <v>1.993714240301026</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>539618706.2937063</v>
+        <v>543277115.5594406</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>11.74</v>
+        <v>11.83</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,19 +11534,19 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>60.24</v>
+        <v>59</v>
       </c>
       <c r="BD48" t="n">
-        <v>30.84</v>
+        <v>29.82</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-83.73999999999999</v>
+        <v>-83.87</v>
       </c>
       <c r="BG48" t="n">
-        <v>-8.18</v>
+        <v>-8.890000000000001</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
@@ -11555,7 +11555,7 @@
         <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>8.970000000000001</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11564,7 +11564,7 @@
         <v>1.29</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.199999999999999</v>
+        <v>9.08</v>
       </c>
       <c r="BN48" t="n">
         <v>9.48</v>
@@ -11573,19 +11573,19 @@
         <v>7.21</v>
       </c>
       <c r="BP48" t="n">
-        <v>8.93</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="BQ48" t="n">
-        <v>6.94</v>
+        <v>6.99</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.199999999999999</v>
+        <v>9.07</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2604</v>
+        <v>2643</v>
       </c>
     </row>
     <row r="49">
@@ -11851,7 +11851,7 @@
         <v>933292214</v>
       </c>
       <c r="H50" t="n">
-        <v>600</v>
+        <v>100</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -12045,7 +12045,7 @@
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>843</v>
+        <v>790</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.63</v>
+        <v>6.79</v>
       </c>
       <c r="G53" t="n">
-        <v>907331427</v>
+        <v>929227790</v>
       </c>
       <c r="H53" t="n">
-        <v>22400</v>
+        <v>9800</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.357077902537692</v>
+        <v>2.413960571689683</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>46221672.28731534</v>
+        <v>47337126.33723892</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-40.56</v>
+        <v>-41.96</v>
       </c>
       <c r="BD53" t="n">
-        <v>-51.47</v>
+        <v>-52.61</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.63</v>
+        <v>-95.73</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12690,10 +12690,10 @@
         <v>2.38</v>
       </c>
       <c r="BI53" t="n">
-        <v>1.38</v>
+        <v>2.41</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6.54</v>
+        <v>6.63</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.09</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.63</v>
+        <v>6.8</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>6.37</v>
+        <v>6.54</v>
       </c>
       <c r="BQ53" t="n">
-        <v>77.70999999999999</v>
+        <v>79.58</v>
       </c>
       <c r="BR53" t="n">
-        <v>6.37</v>
+        <v>6.54</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>43250</v>
+        <v>43533</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>9.68</v>
+        <v>9.59</v>
       </c>
       <c r="G54" t="n">
-        <v>2257493199</v>
+        <v>2236503115</v>
       </c>
       <c r="H54" t="n">
-        <v>844400</v>
+        <v>183600</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.26711192575235</v>
+        <v>1.255330368328068</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>308822599.0424077</v>
+        <v>305951178.5225719</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>15.41</v>
+        <v>15.26</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,25 +12902,25 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>55.04</v>
+        <v>56.49</v>
       </c>
       <c r="BD54" t="n">
-        <v>26.59</v>
+        <v>27.77</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-89.84</v>
+        <v>-89.75</v>
       </c>
       <c r="BG54" t="n">
-        <v>-32.68</v>
+        <v>-32.05</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
       </c>
       <c r="BI54" t="n">
-        <v>0</v>
+        <v>-0.93</v>
       </c>
       <c r="BJ54" t="n">
         <v>9.68</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>9.68</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="BN54" t="n">
         <v>11.75</v>
@@ -12941,19 +12941,19 @@
         <v>8.279999999999999</v>
       </c>
       <c r="BP54" t="n">
-        <v>9.18</v>
+        <v>9.58</v>
       </c>
       <c r="BQ54" t="n">
-        <v>9.65</v>
+        <v>9.56</v>
       </c>
       <c r="BR54" t="n">
-        <v>9.199999999999999</v>
+        <v>9.69</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>260373</v>
+        <v>275693</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>50.64</v>
+        <v>51.97</v>
       </c>
       <c r="G55" t="n">
-        <v>6685785000</v>
+        <v>5338025917</v>
       </c>
       <c r="H55" t="n">
-        <v>5400</v>
+        <v>3900</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1.032092375357227</v>
+        <v>0.8240372444514696</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>336307092.555332</v>
+        <v>268512370.0704225</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>53.26</v>
+        <v>54.66</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,28 +13132,28 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>23.84</v>
+        <v>20.67</v>
       </c>
       <c r="BD55" t="n">
-        <v>1.12</v>
+        <v>-1.47</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-81.48</v>
+        <v>-81.95999999999999</v>
       </c>
       <c r="BG55" t="n">
-        <v>-68.25</v>
+        <v>-69.06999999999999</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
       </c>
       <c r="BI55" t="n">
-        <v>-1.82</v>
+        <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>51.58</v>
+        <v>51.97</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>51.6</v>
+        <v>51.99</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>34.46</v>
       </c>
       <c r="BP55" t="n">
-        <v>50.16</v>
+        <v>51.4</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.2</v>
+        <v>7.39</v>
       </c>
       <c r="BR55" t="n">
-        <v>50.7</v>
+        <v>51.59</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>7185</v>
+        <v>7201</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>61.23</v>
+        <v>61.58</v>
       </c>
       <c r="G56" t="n">
-        <v>6685785000</v>
+        <v>5338025917</v>
       </c>
       <c r="H56" t="n">
-        <v>13800</v>
+        <v>39600</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.186475508329608</v>
+        <v>1.745713170607371</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>278110856.9051581</v>
+        <v>222047667.0965058</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>58.47</v>
+        <v>58.81</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,28 +13362,28 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>2.42</v>
+        <v>1.84</v>
       </c>
       <c r="BD56" t="n">
-        <v>-16.37</v>
+        <v>-16.85</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-84.68000000000001</v>
+        <v>-84.77</v>
       </c>
       <c r="BG56" t="n">
-        <v>-71.13</v>
+        <v>-71.29000000000001</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
       </c>
       <c r="BI56" t="n">
-        <v>-0.37</v>
+        <v>0.57</v>
       </c>
       <c r="BJ56" t="n">
-        <v>61.46</v>
+        <v>61.23</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,28 +13392,28 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>61.46</v>
+        <v>62.66</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
       </c>
       <c r="BO56" t="n">
-        <v>44.76</v>
+        <v>45.75</v>
       </c>
       <c r="BP56" t="n">
-        <v>59.78</v>
+        <v>60.61</v>
       </c>
       <c r="BQ56" t="n">
-        <v>8.710000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="BR56" t="n">
-        <v>61.13</v>
+        <v>60.61</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>34207</v>
+        <v>33134</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>5.98</v>
+        <v>5.82</v>
       </c>
       <c r="G57" t="n">
-        <v>1398470844</v>
+        <v>1361053600</v>
       </c>
       <c r="H57" t="n">
-        <v>3392100</v>
+        <v>2969300</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4185998848489575</v>
+        <v>0.4073998987377238</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>104597669.7083022</v>
+        <v>101799072.5504862</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>9.119999999999999</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,28 +13592,28 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>119.59</v>
+        <v>125.62</v>
       </c>
       <c r="BD57" t="n">
-        <v>79.29000000000001</v>
+        <v>84.22</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-81.15000000000001</v>
+        <v>-80.63</v>
       </c>
       <c r="BG57" t="n">
-        <v>4.75</v>
+        <v>7.63</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
       </c>
       <c r="BI57" t="n">
-        <v>-0.17</v>
+        <v>-2.68</v>
       </c>
       <c r="BJ57" t="n">
-        <v>5.99</v>
+        <v>5.98</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,28 +13622,28 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>5.99</v>
+        <v>6.08</v>
       </c>
       <c r="BN57" t="n">
-        <v>6.02</v>
+        <v>6.08</v>
       </c>
       <c r="BO57" t="n">
         <v>3.37</v>
       </c>
       <c r="BP57" t="n">
-        <v>5.84</v>
+        <v>5.82</v>
       </c>
       <c r="BQ57" t="n">
-        <v>5.77</v>
+        <v>5.62</v>
       </c>
       <c r="BR57" t="n">
-        <v>5.93</v>
+        <v>5.98</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1022957</v>
+        <v>1126425</v>
       </c>
     </row>
     <row r="58">
@@ -13903,13 +13903,13 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>18.86</v>
+        <v>21</v>
       </c>
       <c r="G59" t="n">
-        <v>93644010</v>
+        <v>93636910</v>
       </c>
       <c r="H59" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I59" t="n">
         <v>710143</v>
@@ -13924,7 +13924,7 @@
         <v>0.61</v>
       </c>
       <c r="M59" t="n">
-        <v>9.947206008654277</v>
+        <v>9.946451820931415</v>
       </c>
       <c r="N59" t="n">
         <v>0.15</v>
@@ -14002,7 +14002,7 @@
         <v>1881878.95</v>
       </c>
       <c r="AM59" t="n">
-        <v>15818244.93243243</v>
+        <v>15817045.60810811</v>
       </c>
       <c r="AN59" t="n">
         <v>1.4</v>
@@ -14043,7 +14043,7 @@
         <v>35.09</v>
       </c>
       <c r="AZ59" t="n">
-        <v>23.32</v>
+        <v>25.97</v>
       </c>
       <c r="BA59" t="n">
         <v>3.69</v>
@@ -14052,25 +14052,25 @@
         <v>22.8</v>
       </c>
       <c r="BC59" t="n">
-        <v>127.88</v>
+        <v>104.66</v>
       </c>
       <c r="BD59" t="n">
-        <v>86.06999999999999</v>
+        <v>67.11</v>
       </c>
       <c r="BE59" t="n">
         <v>23.67</v>
       </c>
       <c r="BF59" t="n">
-        <v>-80.45</v>
+        <v>-82.44</v>
       </c>
       <c r="BG59" t="n">
-        <v>20.88</v>
+        <v>8.56</v>
       </c>
       <c r="BH59" t="n">
         <v>30.98</v>
       </c>
       <c r="BI59" t="n">
-        <v>0</v>
+        <v>11.35</v>
       </c>
       <c r="BJ59" t="n">
         <v>18.86</v>
@@ -14082,7 +14082,7 @@
         <v>2.65</v>
       </c>
       <c r="BM59" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="BN59" t="n">
         <v>25.98</v>
@@ -14091,13 +14091,13 @@
         <v>15.66</v>
       </c>
       <c r="BP59" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="BQ59" t="n">
-        <v>7.11</v>
+        <v>7.92</v>
       </c>
       <c r="BR59" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="BS59" t="n">
         <v>1.42</v>
@@ -14136,10 +14136,10 @@
         <v>377</v>
       </c>
       <c r="G60" t="n">
-        <v>171440800</v>
+        <v>171440787</v>
       </c>
       <c r="H60" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.82353050178348</v>
+        <v>12.82352952940177</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-25137947.21407625</v>
+        <v>-25137945.30791789</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14312,7 +14312,7 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="BN60" t="n">
         <v>405</v>
@@ -14321,13 +14321,13 @@
         <v>306.27</v>
       </c>
       <c r="BP60" t="n">
-        <v>377</v>
+        <v>370.01</v>
       </c>
       <c r="BQ60" t="n">
         <v>2.88</v>
       </c>
       <c r="BR60" t="n">
-        <v>378</v>
+        <v>373.01</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>26.05</v>
+        <v>25.74</v>
       </c>
       <c r="G61" t="n">
-        <v>2230098233</v>
+        <v>2203560196</v>
       </c>
       <c r="H61" t="n">
-        <v>1648600</v>
+        <v>543200</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.182697660177988</v>
+        <v>1.168623628011524</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>175046957.0643642</v>
+        <v>172963908.6342229</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>32.82</v>
+        <v>32.43</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-17.45</v>
+        <v>-16.46</v>
       </c>
       <c r="BD61" t="n">
-        <v>-32.6</v>
+        <v>-31.79</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-90.31999999999999</v>
+        <v>-90.2</v>
       </c>
       <c r="BG61" t="n">
-        <v>-54.87</v>
+        <v>-54.33</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>26.05</v>
+        <v>25.74</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>26.15</v>
+        <v>26.17</v>
       </c>
       <c r="BN61" t="n">
         <v>28.25</v>
@@ -14551,19 +14551,19 @@
         <v>18.71</v>
       </c>
       <c r="BP61" t="n">
-        <v>24.8</v>
+        <v>25.32</v>
       </c>
       <c r="BQ61" t="n">
-        <v>13.99</v>
+        <v>13.82</v>
       </c>
       <c r="BR61" t="n">
-        <v>25.28</v>
+        <v>26</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>397775</v>
+        <v>447533</v>
       </c>
     </row>
     <row r="62">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.29</v>
+        <v>1.34</v>
       </c>
       <c r="G63" t="n">
-        <v>336057503</v>
+        <v>349083006</v>
       </c>
       <c r="H63" t="n">
-        <v>1300</v>
+        <v>3100</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.4133333860667188</v>
+        <v>0.429354082561069</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>190941763.0681818</v>
+        <v>198342617.0454545</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-77.58</v>
+        <v>-78.42</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14990,7 +14990,7 @@
         <v>-5.91</v>
       </c>
       <c r="BI63" t="n">
-        <v>0</v>
+        <v>3.88</v>
       </c>
       <c r="BJ63" t="n">
         <v>1.29</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.29</v>
+        <v>1.34</v>
       </c>
       <c r="BN63" t="n">
         <v>1.54</v>
@@ -15011,19 +15011,19 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.29</v>
+        <v>1.34</v>
       </c>
       <c r="BQ63" t="n">
-        <v>4.94</v>
+        <v>5.13</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.29</v>
+        <v>1.34</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>14050</v>
+        <v>14057</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>59.24</v>
+        <v>60.53</v>
       </c>
       <c r="G64" t="n">
-        <v>232142905977</v>
+        <v>234620025618</v>
       </c>
       <c r="H64" t="n">
-        <v>8157200</v>
+        <v>16775900</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>66558777648.46946</v>
+        <v>67269004199.22311</v>
       </c>
       <c r="AL64" t="n">
-        <v>18556587208.39328</v>
+        <v>18754598370.7434</v>
       </c>
       <c r="AM64" t="n">
-        <v>20671674619.50134</v>
+        <v>20892255175.24488</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>23.7</v>
+        <v>24.21</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,28 +15202,28 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-19.41</v>
+        <v>-21.13</v>
       </c>
       <c r="BD64" t="n">
-        <v>-34.2</v>
+        <v>-35.6</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-88.7</v>
+        <v>-88.94</v>
       </c>
       <c r="BG64" t="n">
-        <v>-82.45</v>
+        <v>-82.81999999999999</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
       </c>
       <c r="BI64" t="n">
-        <v>0.39</v>
+        <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>59.01</v>
+        <v>60.53</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>59.82</v>
+        <v>61.3</v>
       </c>
       <c r="BN64" t="n">
         <v>64.72</v>
@@ -15241,19 +15241,19 @@
         <v>44.03</v>
       </c>
       <c r="BP64" t="n">
-        <v>58.13</v>
+        <v>59.95</v>
       </c>
       <c r="BQ64" t="n">
-        <v>37.73</v>
+        <v>38.55</v>
       </c>
       <c r="BR64" t="n">
-        <v>58.66</v>
+        <v>60</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>11307909</v>
+        <v>11445204</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>23.47</v>
+        <v>23.8</v>
       </c>
       <c r="G65" t="n">
-        <v>232142905977</v>
+        <v>234620025618</v>
       </c>
       <c r="H65" t="n">
-        <v>8800</v>
+        <v>6300</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.612273635338936</v>
+        <v>5.672160338291392</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>17388981721.1236</v>
+        <v>17574533754.1573</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>7.9</v>
+        <v>8.01</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,25 +15432,25 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-32.21</v>
+        <v>-33.15</v>
       </c>
       <c r="BD65" t="n">
-        <v>-44.65</v>
+        <v>-45.42</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-90.48999999999999</v>
+        <v>-90.62</v>
       </c>
       <c r="BG65" t="n">
-        <v>-85.23</v>
+        <v>-85.44</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
       </c>
       <c r="BI65" t="n">
-        <v>0</v>
+        <v>1.41</v>
       </c>
       <c r="BJ65" t="n">
         <v>23.47</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>23.6</v>
+        <v>23.86</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>23.23</v>
+        <v>23.52</v>
       </c>
       <c r="BQ65" t="n">
-        <v>14.95</v>
+        <v>15.16</v>
       </c>
       <c r="BR65" t="n">
-        <v>23.57</v>
+        <v>23.53</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>15728</v>
+        <v>15503</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>19.61</v>
+        <v>20.78</v>
       </c>
       <c r="G66" t="n">
-        <v>232142905977</v>
+        <v>234620025618</v>
       </c>
       <c r="H66" t="n">
-        <v>3200</v>
+        <v>2500</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>13.78130626799241</v>
+        <v>13.92836199770083</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>20819991567.44395</v>
+        <v>21042154763.94619</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>7.88</v>
+        <v>8.35</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,25 +15662,25 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-18.87</v>
+        <v>-23.44</v>
       </c>
       <c r="BD66" t="n">
-        <v>-33.76</v>
+        <v>-37.49</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-88.62</v>
+        <v>-89.26000000000001</v>
       </c>
       <c r="BG66" t="n">
-        <v>-82.33</v>
+        <v>-83.31999999999999</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
       </c>
       <c r="BI66" t="n">
-        <v>0</v>
+        <v>5.97</v>
       </c>
       <c r="BJ66" t="n">
         <v>19.61</v>
@@ -15692,28 +15692,28 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>19.7</v>
+        <v>21.16</v>
       </c>
       <c r="BN66" t="n">
-        <v>21.14</v>
+        <v>21.16</v>
       </c>
       <c r="BO66" t="n">
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>19.36</v>
+        <v>19.57</v>
       </c>
       <c r="BQ66" t="n">
-        <v>12.49</v>
+        <v>13.23</v>
       </c>
       <c r="BR66" t="n">
-        <v>19.36</v>
+        <v>21.16</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>7220</v>
+        <v>7182</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>19.3</v>
+        <v>19.34</v>
       </c>
       <c r="G68" t="n">
-        <v>8327906910</v>
+        <v>8554903997</v>
       </c>
       <c r="H68" t="n">
-        <v>40300</v>
+        <v>34900</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>577524751.0402219</v>
+        <v>593266573.9944521</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>35.7</v>
+        <v>35.78</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,25 +16122,25 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>35.77</v>
+        <v>35.49</v>
       </c>
       <c r="BD68" t="n">
-        <v>10.85</v>
+        <v>10.62</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.58</v>
+        <v>-93.59</v>
       </c>
       <c r="BG68" t="n">
-        <v>227.71</v>
+        <v>227.04</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
       </c>
       <c r="BI68" t="n">
-        <v>0</v>
+        <v>0.21</v>
       </c>
       <c r="BJ68" t="n">
         <v>19.3</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>19.46</v>
+        <v>19.64</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,19 +16161,19 @@
         <v>15.07</v>
       </c>
       <c r="BP68" t="n">
-        <v>19.03</v>
+        <v>19.2</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.98</v>
+        <v>13.01</v>
       </c>
       <c r="BR68" t="n">
-        <v>19.29</v>
+        <v>19.3</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>30883</v>
+        <v>31650</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>22.48</v>
+        <v>22.9</v>
       </c>
       <c r="G69" t="n">
-        <v>8327906910</v>
+        <v>8554903997</v>
       </c>
       <c r="H69" t="n">
-        <v>1328200</v>
+        <v>1770900</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>495708744.6428571</v>
+        <v>509220476.0119047</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>39.3</v>
+        <v>40.04</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,28 +16352,28 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>16.56</v>
+        <v>14.42</v>
       </c>
       <c r="BD69" t="n">
-        <v>-4.83</v>
+        <v>-6.57</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-94.48999999999999</v>
+        <v>-94.59</v>
       </c>
       <c r="BG69" t="n">
-        <v>209.55</v>
+        <v>203.87</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
       </c>
       <c r="BI69" t="n">
-        <v>-0.49</v>
+        <v>1.87</v>
       </c>
       <c r="BJ69" t="n">
-        <v>22.59</v>
+        <v>22.48</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,28 +16382,28 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>22.86</v>
+        <v>23.23</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
       </c>
       <c r="BO69" t="n">
-        <v>16.55</v>
+        <v>16.57</v>
       </c>
       <c r="BP69" t="n">
-        <v>22.31</v>
+        <v>22.75</v>
       </c>
       <c r="BQ69" t="n">
-        <v>15.12</v>
+        <v>15.4</v>
       </c>
       <c r="BR69" t="n">
-        <v>22.54</v>
+        <v>22.75</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>1782657</v>
+        <v>1792650</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>17.88</v>
+        <v>18.25</v>
       </c>
       <c r="G70" t="n">
-        <v>8306282346</v>
+        <v>8478168900</v>
       </c>
       <c r="H70" t="n">
-        <v>5236000</v>
+        <v>4666200</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6555998732539473</v>
+        <v>0.6691665687167766</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2741347308.910891</v>
+        <v>2798075544.554456</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.06</v>
+        <v>2.1</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,25 +16582,25 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-52.75</v>
+        <v>-53.7</v>
       </c>
       <c r="BD70" t="n">
-        <v>-61.42</v>
+        <v>-62.2</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
       </c>
       <c r="BF70" t="n">
-        <v>-99.33</v>
+        <v>-99.34</v>
       </c>
       <c r="BG70" t="n">
-        <v>-94.02</v>
+        <v>-94.14</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
       </c>
       <c r="BI70" t="n">
-        <v>0</v>
+        <v>2.07</v>
       </c>
       <c r="BJ70" t="n">
         <v>17.88</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>18.63</v>
+        <v>18.89</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>17.88</v>
+        <v>18.25</v>
       </c>
       <c r="BQ70" t="n">
-        <v>179.32</v>
+        <v>183.03</v>
       </c>
       <c r="BR70" t="n">
-        <v>18.6</v>
+        <v>18.25</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>7057647</v>
+        <v>6948910</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-09-10 05:29
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>24.59</v>
+        <v>24.65</v>
       </c>
       <c r="G3" t="n">
-        <v>3289325632</v>
+        <v>3297351568</v>
       </c>
       <c r="H3" t="n">
-        <v>665200</v>
+        <v>426800</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8184574752049049</v>
+        <v>0.8204545068307224</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>642446412.5</v>
+        <v>644013978.125</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>45</v>
+        <v>45.11</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,28 +1196,28 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>101.3</v>
+        <v>100.81</v>
       </c>
       <c r="BD3" t="n">
-        <v>64.36</v>
+        <v>63.96</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-80.2</v>
+        <v>-80.25</v>
       </c>
       <c r="BG3" t="n">
-        <v>-14.05</v>
+        <v>-14.26</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
       </c>
       <c r="BI3" t="n">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>24.58</v>
+        <v>24.65</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>24.88</v>
+        <v>24.73</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>24.51</v>
+        <v>24.19</v>
       </c>
       <c r="BQ3" t="n">
-        <v>5.6</v>
+        <v>5.61</v>
       </c>
       <c r="BR3" t="n">
-        <v>24.85</v>
+        <v>24.45</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>515457</v>
+        <v>526530</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.82</v>
+        <v>15.58</v>
       </c>
       <c r="G4" t="n">
-        <v>244967316474</v>
+        <v>241251001618</v>
       </c>
       <c r="H4" t="n">
-        <v>25579200</v>
+        <v>22611500</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.773772404052444</v>
+        <v>2.731692457467255</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>24254189749.90099</v>
+        <v>23886237783.9604</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.75</v>
+        <v>19.45</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-26.65</v>
+        <v>-25.52</v>
       </c>
       <c r="BD4" t="n">
-        <v>-40.11</v>
+        <v>-39.19</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.87</v>
+        <v>-92.76000000000001</v>
       </c>
       <c r="BG4" t="n">
-        <v>-28.02</v>
+        <v>-26.91</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.82</v>
+        <v>15.58</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>16.03</v>
+        <v>15.78</v>
       </c>
       <c r="BN4" t="n">
         <v>17</v>
@@ -1465,19 +1465,19 @@
         <v>11.09</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.74</v>
+        <v>15.51</v>
       </c>
       <c r="BQ4" t="n">
-        <v>15.26</v>
+        <v>15.03</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.95</v>
+        <v>15.69</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>31747403</v>
+        <v>31598293</v>
       </c>
     </row>
     <row r="5">
@@ -1737,10 +1737,10 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7.39</v>
+        <v>7.29</v>
       </c>
       <c r="G6" t="n">
-        <v>466195850</v>
+        <v>459887387</v>
       </c>
       <c r="H6" t="n">
         <v>100</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>7.257756602589351</v>
+        <v>7.159546185249855</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>44569392.92543021</v>
+        <v>43966289.38814531</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -1877,7 +1877,7 @@
         <v>5.74</v>
       </c>
       <c r="AZ6" t="n">
-        <v>8.67</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="BA6" t="n">
         <v>0.65</v>
@@ -1886,19 +1886,19 @@
         <v>7.95</v>
       </c>
       <c r="BC6" t="n">
-        <v>-4.79</v>
+        <v>-3.49</v>
       </c>
       <c r="BD6" t="n">
-        <v>-22.26</v>
+        <v>-21.2</v>
       </c>
       <c r="BE6" t="n">
         <v>17.33</v>
       </c>
       <c r="BF6" t="n">
-        <v>-91.22</v>
+        <v>-91.09999999999999</v>
       </c>
       <c r="BG6" t="n">
-        <v>7.63</v>
+        <v>9.1</v>
       </c>
       <c r="BH6" t="n">
         <v>3.86</v>
@@ -1907,7 +1907,7 @@
         <v>0</v>
       </c>
       <c r="BJ6" t="n">
-        <v>7.39</v>
+        <v>7.29</v>
       </c>
       <c r="BK6" t="n">
         <v>0.57</v>
@@ -1916,7 +1916,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>7.39</v>
+        <v>7.29</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
@@ -1925,19 +1925,19 @@
         <v>5.96</v>
       </c>
       <c r="BP6" t="n">
-        <v>7.39</v>
+        <v>7.29</v>
       </c>
       <c r="BQ6" t="n">
-        <v>13.14</v>
+        <v>12.96</v>
       </c>
       <c r="BR6" t="n">
-        <v>7.39</v>
+        <v>7.29</v>
       </c>
       <c r="BS6" t="n">
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>377</v>
+        <v>360</v>
       </c>
     </row>
     <row r="7">
@@ -2597,7 +2597,7 @@
         <v>-3.68</v>
       </c>
       <c r="BJ9" t="n">
-        <v>23.89</v>
+        <v>23.01</v>
       </c>
       <c r="BK9" t="n">
         <v>5.88</v>
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5.2</v>
+        <v>5.1</v>
       </c>
       <c r="G12" t="n">
-        <v>498999989</v>
+        <v>489403793</v>
       </c>
       <c r="H12" t="n">
-        <v>553300</v>
+        <v>381900</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.09024338656891348</v>
+        <v>0.08850792916548846</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>536559127.9569892</v>
+        <v>526240637.6344086</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>7.03</v>
+        <v>6.89</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,28 +3266,28 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>618.22</v>
+        <v>632.3</v>
       </c>
       <c r="BD12" t="n">
-        <v>486.42</v>
+        <v>497.92</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-15.16</v>
+        <v>-13.5</v>
       </c>
       <c r="BG12" t="n">
-        <v>248.44</v>
+        <v>255.27</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
       </c>
       <c r="BI12" t="n">
-        <v>0.19</v>
+        <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>5.19</v>
+        <v>5.1</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.43</v>
       </c>
       <c r="BM12" t="n">
-        <v>5.25</v>
+        <v>5.24</v>
       </c>
       <c r="BN12" t="n">
         <v>8.23</v>
@@ -3305,19 +3305,19 @@
         <v>4.42</v>
       </c>
       <c r="BP12" t="n">
-        <v>5.16</v>
+        <v>5.07</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.52</v>
+        <v>1.49</v>
       </c>
       <c r="BR12" t="n">
-        <v>5.16</v>
+        <v>5.24</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>452237</v>
+        <v>465160</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>29.22</v>
+        <v>28.52</v>
       </c>
       <c r="G13" t="n">
-        <v>14732457751</v>
+        <v>14379524698</v>
       </c>
       <c r="H13" t="n">
-        <v>5794500</v>
+        <v>3908600</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>5.095335621223186</v>
+        <v>4.973270967297001</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1533034105.202914</v>
+        <v>1496308501.352758</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>52.89</v>
+        <v>51.62</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,28 +3496,28 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>11.48</v>
+        <v>14.21</v>
       </c>
       <c r="BD13" t="n">
-        <v>-8.98</v>
+        <v>-6.75</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-91.09</v>
+        <v>-90.87</v>
       </c>
       <c r="BG13" t="n">
-        <v>-70.25</v>
+        <v>-69.52</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
       </c>
       <c r="BI13" t="n">
-        <v>1.42</v>
+        <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>28.81</v>
+        <v>28.52</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>29.49</v>
+        <v>28.96</v>
       </c>
       <c r="BN13" t="n">
         <v>32.43</v>
@@ -3535,19 +3535,19 @@
         <v>21.06</v>
       </c>
       <c r="BP13" t="n">
-        <v>28.96</v>
+        <v>28.3</v>
       </c>
       <c r="BQ13" t="n">
-        <v>14.93</v>
+        <v>14.57</v>
       </c>
       <c r="BR13" t="n">
-        <v>29.32</v>
+        <v>28.92</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>4385448</v>
+        <v>4486072</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>10</v>
+        <v>10.04</v>
       </c>
       <c r="G14" t="n">
-        <v>7813653684</v>
+        <v>7999197250</v>
       </c>
       <c r="H14" t="n">
-        <v>35600</v>
+        <v>7300</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.244367918259752</v>
+        <v>3.321408905397762</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>867220164.7058824</v>
+        <v>887813235.2941177</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>8.029999999999999</v>
+        <v>8.07</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,28 +3726,28 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>10.83</v>
+        <v>10.39</v>
       </c>
       <c r="BD14" t="n">
-        <v>-9.51</v>
+        <v>-9.869999999999999</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-85.79000000000001</v>
+        <v>-85.84</v>
       </c>
       <c r="BG14" t="n">
-        <v>-40.58</v>
+        <v>-40.81</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
       </c>
       <c r="BI14" t="n">
-        <v>-1.96</v>
+        <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>10.2</v>
+        <v>10.04</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>10.02</v>
+        <v>10.04</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,19 +3765,19 @@
         <v>7.65</v>
       </c>
       <c r="BP14" t="n">
-        <v>9.57</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="BQ14" t="n">
-        <v>9.869999999999999</v>
+        <v>9.91</v>
       </c>
       <c r="BR14" t="n">
-        <v>9.99</v>
+        <v>10</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>11380</v>
+        <v>12347</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>13.05</v>
+        <v>13.25</v>
       </c>
       <c r="G15" t="n">
-        <v>7813653684</v>
+        <v>7999197250</v>
       </c>
       <c r="H15" t="n">
-        <v>9515700</v>
+        <v>3557300</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.206207749036195</v>
+        <v>3.282342582131136</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>651680874.3953295</v>
+        <v>667155733.9449542</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>8.68</v>
+        <v>8.81</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,28 +3956,28 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-15.07</v>
+        <v>-16.36</v>
       </c>
       <c r="BD15" t="n">
-        <v>-30.66</v>
+        <v>-31.71</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-89.11</v>
+        <v>-89.27</v>
       </c>
       <c r="BG15" t="n">
-        <v>-52.58</v>
+        <v>-53.3</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
       </c>
       <c r="BI15" t="n">
-        <v>-3.83</v>
+        <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>13.57</v>
+        <v>13.25</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>13.74</v>
+        <v>13.51</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>12.51</v>
+        <v>12.91</v>
       </c>
       <c r="BQ15" t="n">
-        <v>12.88</v>
+        <v>13.08</v>
       </c>
       <c r="BR15" t="n">
-        <v>13.69</v>
+        <v>12.99</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>1967073</v>
+        <v>2240040</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.37</v>
+        <v>4.32</v>
       </c>
       <c r="G16" t="n">
-        <v>958365883</v>
+        <v>947400661</v>
       </c>
       <c r="H16" t="n">
-        <v>179500</v>
+        <v>151000</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4533874194763983</v>
+        <v>0.448199950061269</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>269203899.7191011</v>
+        <v>266123781.1797753</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-60.21</v>
+        <v>-59.75</v>
       </c>
       <c r="BD16" t="n">
-        <v>-67.51000000000001</v>
+        <v>-67.13</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.17</v>
+        <v>-98.15000000000001</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4204,10 +4204,10 @@
         <v>1.68</v>
       </c>
       <c r="BI16" t="n">
-        <v>-2.89</v>
+        <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>4.5</v>
+        <v>4.32</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,28 +4216,28 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.58</v>
+        <v>4.52</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
       </c>
       <c r="BO16" t="n">
-        <v>2.96</v>
+        <v>2.97</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.35</v>
+        <v>4.27</v>
       </c>
       <c r="BQ16" t="n">
-        <v>59.63</v>
+        <v>58.95</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.58</v>
+        <v>4.47</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>136900</v>
+        <v>141217</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>33.91</v>
+        <v>33.39</v>
       </c>
       <c r="G17" t="n">
-        <v>11177648128</v>
+        <v>11006241989</v>
       </c>
       <c r="H17" t="n">
-        <v>523500</v>
+        <v>558600</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>5047709595.375723</v>
+        <v>4970304366.419798</v>
       </c>
       <c r="AL17" t="n">
-        <v>1397206016</v>
+        <v>1375780248.625</v>
       </c>
       <c r="AM17" t="n">
-        <v>3460572175.851393</v>
+        <v>3407505259.752322</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>18.14</v>
+        <v>17.86</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>55.23</v>
+        <v>57.64</v>
       </c>
       <c r="BD17" t="n">
-        <v>26.74</v>
+        <v>28.72</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-86.59</v>
+        <v>-86.38</v>
       </c>
       <c r="BG17" t="n">
-        <v>-51.83</v>
+        <v>-51.08</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>33.91</v>
+        <v>33.39</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,7 +4446,7 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>34.12</v>
+        <v>33.81</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
@@ -4455,19 +4455,19 @@
         <v>29.28</v>
       </c>
       <c r="BP17" t="n">
-        <v>33.41</v>
+        <v>33.26</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.69</v>
+        <v>2.65</v>
       </c>
       <c r="BR17" t="n">
-        <v>33.78</v>
+        <v>33.5</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1079027</v>
+        <v>1069139</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>11.65</v>
+        <v>11.75</v>
       </c>
       <c r="G18" t="n">
-        <v>11177648128</v>
+        <v>11006241989</v>
       </c>
       <c r="H18" t="n">
-        <v>3700</v>
+        <v>2500</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.291138566624007</v>
+        <v>3.240669868006998</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3326680990.476191</v>
+        <v>3275667258.630952</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>6</v>
+        <v>6.05</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,28 +4646,28 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>50.43</v>
+        <v>49.15</v>
       </c>
       <c r="BD18" t="n">
-        <v>22.82</v>
+        <v>21.78</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-87.02</v>
+        <v>-87.13</v>
       </c>
       <c r="BG18" t="n">
-        <v>-53.27</v>
+        <v>-53.66</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
       </c>
       <c r="BI18" t="n">
-        <v>-0.09</v>
+        <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>11.66</v>
+        <v>11.75</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>11.99</v>
+        <v>12</v>
       </c>
       <c r="BN18" t="n">
         <v>13.82</v>
@@ -4685,19 +4685,19 @@
         <v>10.11</v>
       </c>
       <c r="BP18" t="n">
+        <v>11.57</v>
+      </c>
+      <c r="BQ18" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="BR18" t="n">
         <v>11.65</v>
-      </c>
-      <c r="BQ18" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="BR18" t="n">
-        <v>11.99</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>9863</v>
+        <v>9648</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>11.07</v>
+        <v>10.86</v>
       </c>
       <c r="G19" t="n">
-        <v>11177648128</v>
+        <v>11006241989</v>
       </c>
       <c r="H19" t="n">
-        <v>9400</v>
+        <v>7600</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.96306222241701</v>
+        <v>6.856285591278343</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3548459723.174603</v>
+        <v>3494045075.873016</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>6.09</v>
+        <v>5.97</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,28 +4876,28 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>58.31</v>
+        <v>61.37</v>
       </c>
       <c r="BD19" t="n">
-        <v>29.26</v>
+        <v>31.76</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-86.34</v>
+        <v>-86.06999999999999</v>
       </c>
       <c r="BG19" t="n">
-        <v>-52.57</v>
+        <v>-51.66</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
       </c>
       <c r="BI19" t="n">
-        <v>1.37</v>
+        <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>10.92</v>
+        <v>10.86</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,28 +4906,28 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>11.1</v>
+        <v>11.05</v>
       </c>
       <c r="BN19" t="n">
         <v>11.41</v>
       </c>
       <c r="BO19" t="n">
-        <v>8.98</v>
+        <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>10.83</v>
+        <v>10.86</v>
       </c>
       <c r="BQ19" t="n">
-        <v>0.88</v>
+        <v>0.86</v>
       </c>
       <c r="BR19" t="n">
-        <v>10.83</v>
+        <v>11.05</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>13971</v>
+        <v>14046</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5.42</v>
+        <v>5.27</v>
       </c>
       <c r="G22" t="n">
-        <v>1085328999</v>
+        <v>1055292200</v>
       </c>
       <c r="H22" t="n">
-        <v>1444100</v>
+        <v>1469300</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.09205392401532198</v>
+        <v>0.089506304615714</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>246106348.9795918</v>
+        <v>239295283.446712</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,28 +5566,28 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>448.06</v>
+        <v>463.66</v>
       </c>
       <c r="BD22" t="n">
-        <v>347.49</v>
+        <v>360.23</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-65.13</v>
+        <v>-64.14</v>
       </c>
       <c r="BG22" t="n">
-        <v>3082.47</v>
+        <v>3173.05</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
       </c>
       <c r="BI22" t="n">
-        <v>-2.34</v>
+        <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>5.55</v>
+        <v>5.27</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>5.68</v>
+        <v>5.5</v>
       </c>
       <c r="BN22" t="n">
         <v>8.82</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>5.42</v>
+        <v>5.17</v>
       </c>
       <c r="BQ22" t="n">
-        <v>8.07</v>
+        <v>7.85</v>
       </c>
       <c r="BR22" t="n">
-        <v>5.59</v>
+        <v>5.5</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1598837</v>
+        <v>1601227</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>3.05</v>
+        <v>2.91</v>
       </c>
       <c r="G24" t="n">
-        <v>1231800125</v>
+        <v>1175258242</v>
       </c>
       <c r="H24" t="n">
-        <v>8673200</v>
+        <v>6288500</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2977763809990618</v>
+        <v>0.2841078994387012</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1109729842.342342</v>
+        <v>1058791209.009009</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>1.41</v>
+        <v>1.34</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,28 +6026,28 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>134.64</v>
+        <v>145.93</v>
       </c>
       <c r="BD24" t="n">
-        <v>91.58</v>
+        <v>100.8</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-87.54000000000001</v>
+        <v>-86.94</v>
       </c>
       <c r="BG24" t="n">
-        <v>-52.2</v>
+        <v>-49.9</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
       </c>
       <c r="BI24" t="n">
-        <v>4.1</v>
+        <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>2.93</v>
+        <v>2.91</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>3.05</v>
+        <v>3.03</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.93</v>
+        <v>2.9</v>
       </c>
       <c r="BQ24" t="n">
-        <v>7.49</v>
+        <v>7.15</v>
       </c>
       <c r="BR24" t="n">
-        <v>2.99</v>
+        <v>3.01</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>9586443</v>
+        <v>9557933</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>4.13</v>
+        <v>3.91</v>
       </c>
       <c r="G25" t="n">
-        <v>1431020259</v>
+        <v>1354791960</v>
       </c>
       <c r="H25" t="n">
-        <v>1595300</v>
+        <v>2478900</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.713572041906965</v>
+        <v>0.6755611314209489</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>526110389.3382353</v>
+        <v>498085279.4117647</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>9.619999999999999</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,19 +6256,19 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>-2.91</v>
+        <v>2.55</v>
       </c>
       <c r="BD25" t="n">
-        <v>-20.73</v>
+        <v>-16.27</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-94.39</v>
+        <v>-94.06999999999999</v>
       </c>
       <c r="BG25" t="n">
-        <v>-46.74</v>
+        <v>-43.74</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>4.13</v>
+        <v>3.91</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>4.16</v>
+        <v>4.14</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>3.86</v>
+        <v>3.87</v>
       </c>
       <c r="BQ25" t="n">
-        <v>17.45</v>
+        <v>16.52</v>
       </c>
       <c r="BR25" t="n">
-        <v>3.86</v>
+        <v>4.14</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1018647</v>
+        <v>1064750</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>9.130000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G26" t="n">
-        <v>12365608244</v>
+        <v>12460415341</v>
       </c>
       <c r="H26" t="n">
-        <v>13676600</v>
+        <v>5988400</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1594534759026149</v>
+        <v>0.160676005426322</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>4416288658.571429</v>
+        <v>4450148336.071429</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>1.75</v>
+        <v>1.76</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,28 +6486,28 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-5.19</v>
+        <v>-5.92</v>
       </c>
       <c r="BD26" t="n">
-        <v>-22.59</v>
+        <v>-23.18</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-92.78</v>
+        <v>-92.83</v>
       </c>
       <c r="BG26" t="n">
-        <v>-86.93000000000001</v>
+        <v>-87.03</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
       </c>
       <c r="BI26" t="n">
-        <v>0.55</v>
+        <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>9.08</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,7 +6516,7 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>9.470000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="BN26" t="n">
         <v>10.6</v>
@@ -6525,19 +6525,19 @@
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>9.130000000000001</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="BQ26" t="n">
-        <v>12.73</v>
+        <v>12.83</v>
       </c>
       <c r="BR26" t="n">
-        <v>9.26</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>11236307</v>
+        <v>11370577</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>17.05</v>
+        <v>16.64</v>
       </c>
       <c r="G34" t="n">
-        <v>3520650932</v>
+        <v>3435988481</v>
       </c>
       <c r="H34" t="n">
-        <v>3813700</v>
+        <v>4002600</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.3095063360510825</v>
+        <v>0.3020635178006436</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>731944060.7068608</v>
+        <v>714342719.5426196</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>39.78</v>
+        <v>38.83</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,28 +8314,28 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>117.53</v>
+        <v>122.89</v>
       </c>
       <c r="BD34" t="n">
-        <v>77.61</v>
+        <v>81.98999999999999</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-86.54000000000001</v>
+        <v>-86.20999999999999</v>
       </c>
       <c r="BG34" t="n">
-        <v>48.14</v>
+        <v>51.79</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
       </c>
       <c r="BI34" t="n">
-        <v>-3.62</v>
+        <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>17.69</v>
+        <v>16.64</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>18.28</v>
+        <v>17</v>
       </c>
       <c r="BN34" t="n">
         <v>31.12</v>
@@ -8353,19 +8353,19 @@
         <v>14.32</v>
       </c>
       <c r="BP34" t="n">
-        <v>16.75</v>
+        <v>16.1</v>
       </c>
       <c r="BQ34" t="n">
-        <v>10.81</v>
+        <v>10.55</v>
       </c>
       <c r="BR34" t="n">
-        <v>17.87</v>
+        <v>16.99</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>2990130</v>
+        <v>3052970</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>17.64</v>
+        <v>17.29</v>
       </c>
       <c r="G35" t="n">
-        <v>89020239279</v>
+        <v>87253989620</v>
       </c>
       <c r="H35" t="n">
-        <v>35875800</v>
+        <v>57684700</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.39049261935769</v>
+        <v>7.243857930723889</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7357044568.512397</v>
+        <v>7211073522.31405</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.29</v>
+        <v>10.09</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,19 +8544,19 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-46.67</v>
+        <v>-45.6</v>
       </c>
       <c r="BD35" t="n">
-        <v>-56.46</v>
+        <v>-55.58</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-93.68000000000001</v>
+        <v>-93.56</v>
       </c>
       <c r="BG35" t="n">
-        <v>-48.32</v>
+        <v>-47.27</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
@@ -8565,7 +8565,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>17.64</v>
+        <v>17.29</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>17.88</v>
+        <v>17.51</v>
       </c>
       <c r="BN35" t="n">
         <v>20.08</v>
@@ -8583,19 +8583,19 @@
         <v>11.7</v>
       </c>
       <c r="BP35" t="n">
-        <v>17.55</v>
+        <v>17.08</v>
       </c>
       <c r="BQ35" t="n">
-        <v>16.88</v>
+        <v>16.55</v>
       </c>
       <c r="BR35" t="n">
-        <v>17.68</v>
+        <v>17.47</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>34435973</v>
+        <v>34834187</v>
       </c>
     </row>
     <row r="36">
@@ -8825,7 +8825,7 @@
         <v>1.24</v>
       </c>
       <c r="BT36" t="n">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="37">
@@ -8855,13 +8855,13 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>14.8</v>
+        <v>15</v>
       </c>
       <c r="G37" t="n">
-        <v>198305054</v>
+        <v>202125000</v>
       </c>
       <c r="H37" t="n">
-        <v>2100</v>
+        <v>200</v>
       </c>
       <c r="I37" t="n">
         <v>4900000</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.93066675066702</v>
+        <v>1.967857142857143</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>47441400.4784689</v>
+        <v>48355263.15789474</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -8995,7 +8995,7 @@
         <v>24.36</v>
       </c>
       <c r="AZ37" t="n">
-        <v>65.81</v>
+        <v>66.7</v>
       </c>
       <c r="BA37" t="n">
         <v>2.44</v>
@@ -9004,28 +9004,28 @@
         <v>15.53</v>
       </c>
       <c r="BC37" t="n">
-        <v>101.61</v>
+        <v>98.92</v>
       </c>
       <c r="BD37" t="n">
-        <v>64.61</v>
+        <v>62.42</v>
       </c>
       <c r="BE37" t="n">
         <v>344.67</v>
       </c>
       <c r="BF37" t="n">
-        <v>-83.48</v>
+        <v>-83.7</v>
       </c>
       <c r="BG37" t="n">
-        <v>4.95</v>
+        <v>3.56</v>
       </c>
       <c r="BH37" t="n">
         <v>17.13</v>
       </c>
       <c r="BI37" t="n">
-        <v>-1.27</v>
+        <v>0</v>
       </c>
       <c r="BJ37" t="n">
-        <v>14.99</v>
+        <v>15</v>
       </c>
       <c r="BK37" t="n">
         <v>2.31</v>
@@ -9040,13 +9040,13 @@
         <v>20.9</v>
       </c>
       <c r="BO37" t="n">
-        <v>12.9</v>
+        <v>13.05</v>
       </c>
       <c r="BP37" t="n">
-        <v>14.8</v>
+        <v>15</v>
       </c>
       <c r="BQ37" t="n">
-        <v>6.4</v>
+        <v>6.49</v>
       </c>
       <c r="BR37" t="n">
         <v>15</v>
@@ -9055,7 +9055,7 @@
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>837</v>
+        <v>873</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>69.48999999999999</v>
+        <v>68.31</v>
       </c>
       <c r="G39" t="n">
-        <v>3895491842</v>
+        <v>3829343019</v>
       </c>
       <c r="H39" t="n">
-        <v>2600</v>
+        <v>2900</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1955366034199482</v>
+        <v>0.1922162226582197</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>409190319.5378152</v>
+        <v>402241913.7605042</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>203.03</v>
+        <v>199.58</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,28 +9464,28 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>200.05</v>
+        <v>205.23</v>
       </c>
       <c r="BD39" t="n">
-        <v>144.99</v>
+        <v>149.22</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-72.64</v>
+        <v>-72.17</v>
       </c>
       <c r="BG39" t="n">
-        <v>32</v>
+        <v>34.28</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
       </c>
       <c r="BI39" t="n">
-        <v>1.97</v>
+        <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>68.15000000000001</v>
+        <v>68.31</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>69.97</v>
+        <v>69.89</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>68.15000000000001</v>
+        <v>68.31</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.61</v>
+        <v>4.53</v>
       </c>
       <c r="BR39" t="n">
-        <v>68.15000000000001</v>
+        <v>69.89</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>4080</v>
+        <v>4087</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>22.6</v>
+        <v>22.18</v>
       </c>
       <c r="G40" t="n">
-        <v>129516850586</v>
+        <v>127109944228</v>
       </c>
       <c r="H40" t="n">
-        <v>30149100</v>
+        <v>30236100</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.392970153143478</v>
+        <v>0.385667301384608</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6717678972.302904</v>
+        <v>6592839430.912863</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>11.41</v>
+        <v>11.2</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,28 +9694,28 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>95.79000000000001</v>
+        <v>99.5</v>
       </c>
       <c r="BD40" t="n">
-        <v>59.86</v>
+        <v>62.89</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-87.79000000000001</v>
+        <v>-87.56</v>
       </c>
       <c r="BG40" t="n">
-        <v>23.41</v>
+        <v>25.75</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
       </c>
       <c r="BI40" t="n">
-        <v>0.36</v>
+        <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>22.52</v>
+        <v>22.18</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>23.21</v>
+        <v>22.65</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>22.58</v>
+        <v>21.97</v>
       </c>
       <c r="BQ40" t="n">
-        <v>9.039999999999999</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="BR40" t="n">
-        <v>22.84</v>
+        <v>22.44</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>29100909</v>
+        <v>29733273</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>16.04</v>
+        <v>15.83</v>
       </c>
       <c r="G41" t="n">
-        <v>192079241161</v>
+        <v>187257905436</v>
       </c>
       <c r="H41" t="n">
-        <v>8647400</v>
+        <v>8701800</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.28001000440003</v>
+        <v>1.247880775206551</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>29596185078.73652</v>
+        <v>28853298218.18182</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>24.01</v>
+        <v>23.69</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,28 +9924,28 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>86.31999999999999</v>
+        <v>88.79000000000001</v>
       </c>
       <c r="BD41" t="n">
-        <v>52.13</v>
+        <v>54.15</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-84.23999999999999</v>
+        <v>-84.04000000000001</v>
       </c>
       <c r="BG41" t="n">
-        <v>-14.15</v>
+        <v>-13.01</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
       </c>
       <c r="BI41" t="n">
-        <v>1.45</v>
+        <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>15.81</v>
+        <v>15.83</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,7 +9954,7 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>16.29</v>
+        <v>15.97</v>
       </c>
       <c r="BN41" t="n">
         <v>18.28</v>
@@ -9963,19 +9963,19 @@
         <v>13.34</v>
       </c>
       <c r="BP41" t="n">
-        <v>15.96</v>
+        <v>15.73</v>
       </c>
       <c r="BQ41" t="n">
-        <v>6.86</v>
+        <v>6.77</v>
       </c>
       <c r="BR41" t="n">
-        <v>15.99</v>
+        <v>15.93</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>7057236</v>
+        <v>7215953</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>18.22</v>
+        <v>17.79</v>
       </c>
       <c r="G42" t="n">
-        <v>192079241161</v>
+        <v>187257905436</v>
       </c>
       <c r="H42" t="n">
-        <v>43084300</v>
+        <v>30056500</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.283817383958201</v>
+        <v>1.251592586628512</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>26133230089.93197</v>
+        <v>25477266045.71429</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>26.39</v>
+        <v>25.77</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,28 +10154,28 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>64.03</v>
+        <v>67.98999999999999</v>
       </c>
       <c r="BD42" t="n">
-        <v>33.93</v>
+        <v>37.16</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-86.13</v>
+        <v>-85.79000000000001</v>
       </c>
       <c r="BG42" t="n">
-        <v>-17.04</v>
+        <v>-15.04</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
       </c>
       <c r="BI42" t="n">
-        <v>1.79</v>
+        <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>17.9</v>
+        <v>17.79</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>18.49</v>
+        <v>18.15</v>
       </c>
       <c r="BN42" t="n">
         <v>21.33</v>
@@ -10193,19 +10193,19 @@
         <v>15.64</v>
       </c>
       <c r="BP42" t="n">
-        <v>18.08</v>
+        <v>17.74</v>
       </c>
       <c r="BQ42" t="n">
-        <v>7.79</v>
+        <v>7.61</v>
       </c>
       <c r="BR42" t="n">
-        <v>18.1</v>
+        <v>18</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>38628200</v>
+        <v>39559117</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>42.35</v>
+        <v>40.91</v>
       </c>
       <c r="G43" t="n">
-        <v>82218244687</v>
+        <v>79422673703</v>
       </c>
       <c r="H43" t="n">
-        <v>5026300</v>
+        <v>6808900</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>10014402519.73203</v>
+        <v>9673894482.704018</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>76.87</v>
+        <v>74.25</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,28 +10384,28 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-42.3</v>
+        <v>-40.27</v>
       </c>
       <c r="BD43" t="n">
-        <v>-52.89</v>
+        <v>-51.23</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-86.70999999999999</v>
+        <v>-86.23999999999999</v>
       </c>
       <c r="BG43" t="n">
-        <v>14.8</v>
+        <v>18.84</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
       </c>
       <c r="BI43" t="n">
-        <v>0.45</v>
+        <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>42.16</v>
+        <v>40.91</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>42.79</v>
+        <v>42.41</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>41.82</v>
+        <v>40.91</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.949999999999999</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="BR43" t="n">
-        <v>42.48</v>
+        <v>42.26</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6436722</v>
+        <v>6380221</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>3.96</v>
+        <v>3.95</v>
       </c>
       <c r="G46" t="n">
-        <v>3962142398</v>
+        <v>3952136997</v>
       </c>
       <c r="H46" t="n">
-        <v>31049400</v>
+        <v>15318800</v>
       </c>
       <c r="I46" t="n">
         <v>1000541644</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.06886952154991309</v>
+        <v>0.06869560877481121</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249156.24</v>
       </c>
       <c r="AM46" t="n">
-        <v>3884453331.372549</v>
+        <v>3874644114.705882</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.27</v>
+        <v>3.26</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,25 +11074,25 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>2.12</v>
+        <v>2.38</v>
       </c>
       <c r="BD46" t="n">
-        <v>-16.62</v>
+        <v>-16.41</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.31999999999999</v>
+        <v>-89.29000000000001</v>
       </c>
       <c r="BG46" t="n">
-        <v>86.33</v>
+        <v>86.8</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
       </c>
       <c r="BI46" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="BJ46" t="n">
         <v>3.95</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>3.99</v>
+        <v>4</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>3.8</v>
+        <v>3.91</v>
       </c>
       <c r="BQ46" t="n">
-        <v>8.66</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="BR46" t="n">
-        <v>3.99</v>
+        <v>3.91</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>16708023</v>
+        <v>17409503</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>8.91</v>
+        <v>8.92</v>
       </c>
       <c r="G47" t="n">
-        <v>3107545101</v>
+        <v>3111891882</v>
       </c>
       <c r="H47" t="n">
-        <v>7700</v>
+        <v>7200</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7327948879303807</v>
+        <v>0.7338199089010266</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>550983173.9361702</v>
+        <v>551753879.7872341</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>11.7</v>
+        <v>11.71</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,19 +11304,19 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>61.32</v>
+        <v>61.14</v>
       </c>
       <c r="BD47" t="n">
-        <v>31.72</v>
+        <v>31.57</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-83.63</v>
+        <v>-83.65000000000001</v>
       </c>
       <c r="BG47" t="n">
-        <v>-3.26</v>
+        <v>-3.37</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
@@ -11325,7 +11325,7 @@
         <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>8.91</v>
+        <v>8.92</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11343,19 +11343,19 @@
         <v>7.2</v>
       </c>
       <c r="BP47" t="n">
-        <v>8.85</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="BQ47" t="n">
-        <v>6.89</v>
+        <v>6.9</v>
       </c>
       <c r="BR47" t="n">
-        <v>8.9</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>12638</v>
+        <v>12593</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.039999999999999</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="G48" t="n">
-        <v>3107545101</v>
+        <v>3111891882</v>
       </c>
       <c r="H48" t="n">
-        <v>2900</v>
+        <v>3500</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>1.993714240301026</v>
+        <v>1.996503013721042</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>543277115.5594406</v>
+        <v>544037042.3076923</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>11.83</v>
+        <v>11.81</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,19 +11534,19 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>59</v>
+        <v>59.17</v>
       </c>
       <c r="BD48" t="n">
-        <v>29.82</v>
+        <v>29.97</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-83.87</v>
+        <v>-83.84999999999999</v>
       </c>
       <c r="BG48" t="n">
-        <v>-8.890000000000001</v>
+        <v>-8.789999999999999</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
@@ -11555,7 +11555,7 @@
         <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.039999999999999</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11564,7 +11564,7 @@
         <v>1.29</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.08</v>
+        <v>9.06</v>
       </c>
       <c r="BN48" t="n">
         <v>9.48</v>
@@ -11573,13 +11573,13 @@
         <v>7.21</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.029999999999999</v>
+        <v>9</v>
       </c>
       <c r="BQ48" t="n">
-        <v>6.99</v>
+        <v>6.98</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.07</v>
+        <v>9</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>34</v>
+        <v>33.9</v>
       </c>
       <c r="G50" t="n">
         <v>933292214</v>
       </c>
       <c r="H50" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>74.97</v>
+        <v>74.75</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,19 +11994,19 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>146.7</v>
+        <v>147.43</v>
       </c>
       <c r="BD50" t="n">
-        <v>101.43</v>
+        <v>102.02</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-72.90000000000001</v>
+        <v>-72.81999999999999</v>
       </c>
       <c r="BG50" t="n">
-        <v>-10.21</v>
+        <v>-9.94</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
@@ -12015,7 +12015,7 @@
         <v>0</v>
       </c>
       <c r="BJ50" t="n">
-        <v>34</v>
+        <v>33.9</v>
       </c>
       <c r="BK50" t="n">
         <v>7.34</v>
@@ -12024,7 +12024,7 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>34</v>
+        <v>33.9</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
@@ -12033,19 +12033,19 @@
         <v>22.89</v>
       </c>
       <c r="BP50" t="n">
-        <v>34</v>
+        <v>33.9</v>
       </c>
       <c r="BQ50" t="n">
-        <v>4.47</v>
+        <v>4.46</v>
       </c>
       <c r="BR50" t="n">
-        <v>34</v>
+        <v>33.9</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>790</v>
+        <v>753</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.79</v>
+        <v>6.56</v>
       </c>
       <c r="G53" t="n">
-        <v>929227790</v>
+        <v>897751736</v>
       </c>
       <c r="H53" t="n">
-        <v>9800</v>
+        <v>24200</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.413960571689683</v>
+        <v>2.332191651166572</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>47337126.33723892</v>
+        <v>45733659.50076414</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-41.96</v>
+        <v>-39.93</v>
       </c>
       <c r="BD53" t="n">
-        <v>-52.61</v>
+        <v>-50.95</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.73</v>
+        <v>-95.58</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12690,10 +12690,10 @@
         <v>2.38</v>
       </c>
       <c r="BI53" t="n">
-        <v>2.41</v>
+        <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6.63</v>
+        <v>6.56</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.09</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.8</v>
+        <v>6.77</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>6.54</v>
+        <v>6.53</v>
       </c>
       <c r="BQ53" t="n">
-        <v>79.58</v>
+        <v>76.89</v>
       </c>
       <c r="BR53" t="n">
-        <v>6.54</v>
+        <v>6.63</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>43533</v>
+        <v>43210</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>9.59</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="G54" t="n">
-        <v>2236503115</v>
+        <v>2301802413</v>
       </c>
       <c r="H54" t="n">
-        <v>183600</v>
+        <v>268400</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.255330368328068</v>
+        <v>1.291982314511431</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>305951178.5225719</v>
+        <v>314884051.0259918</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>15.26</v>
+        <v>15.71</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,28 +12902,28 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>56.49</v>
+        <v>52.05</v>
       </c>
       <c r="BD54" t="n">
-        <v>27.77</v>
+        <v>24.15</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-89.75</v>
+        <v>-90.04000000000001</v>
       </c>
       <c r="BG54" t="n">
-        <v>-32.05</v>
+        <v>-33.98</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
       </c>
       <c r="BI54" t="n">
-        <v>-0.93</v>
+        <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>9.68</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>9.859999999999999</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="BN54" t="n">
         <v>11.75</v>
@@ -12941,19 +12941,19 @@
         <v>8.279999999999999</v>
       </c>
       <c r="BP54" t="n">
-        <v>9.58</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="BQ54" t="n">
-        <v>9.56</v>
+        <v>9.84</v>
       </c>
       <c r="BR54" t="n">
-        <v>9.69</v>
+        <v>9.65</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>275693</v>
+        <v>277237</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>51.97</v>
+        <v>51.74</v>
       </c>
       <c r="G55" t="n">
-        <v>5338025917</v>
+        <v>6795970408</v>
       </c>
       <c r="H55" t="n">
-        <v>3900</v>
+        <v>300</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>0.8240372444514696</v>
+        <v>1.049101824430511</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>268512370.0704225</v>
+        <v>341849618.1086519</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>54.66</v>
+        <v>54.41</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>20.67</v>
+        <v>21.21</v>
       </c>
       <c r="BD55" t="n">
-        <v>-1.47</v>
+        <v>-1.03</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-81.95999999999999</v>
+        <v>-81.87</v>
       </c>
       <c r="BG55" t="n">
-        <v>-69.06999999999999</v>
+        <v>-68.93000000000001</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>51.97</v>
+        <v>51.74</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>51.99</v>
+        <v>51.74</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>34.46</v>
       </c>
       <c r="BP55" t="n">
-        <v>51.4</v>
+        <v>51.25</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.39</v>
+        <v>7.36</v>
       </c>
       <c r="BR55" t="n">
-        <v>51.59</v>
+        <v>51.25</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>7201</v>
+        <v>7290</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>61.58</v>
+        <v>61.44</v>
       </c>
       <c r="G56" t="n">
-        <v>5338025917</v>
+        <v>6795970408</v>
       </c>
       <c r="H56" t="n">
-        <v>39600</v>
+        <v>7300</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>1.745713170607371</v>
+        <v>2.222509825312177</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>222047667.0965058</v>
+        <v>282694276.5391015</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>58.81</v>
+        <v>58.68</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,28 +13362,28 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>1.84</v>
+        <v>2.07</v>
       </c>
       <c r="BD56" t="n">
-        <v>-16.85</v>
+        <v>-16.66</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-84.77</v>
+        <v>-84.73999999999999</v>
       </c>
       <c r="BG56" t="n">
-        <v>-71.29000000000001</v>
+        <v>-71.23</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
       </c>
       <c r="BI56" t="n">
-        <v>0.57</v>
+        <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>61.23</v>
+        <v>61.44</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>62.66</v>
+        <v>62.2</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>45.75</v>
       </c>
       <c r="BP56" t="n">
-        <v>60.61</v>
+        <v>61.25</v>
       </c>
       <c r="BQ56" t="n">
-        <v>8.76</v>
+        <v>8.74</v>
       </c>
       <c r="BR56" t="n">
-        <v>60.61</v>
+        <v>61.58</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>33134</v>
+        <v>33983</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>5.82</v>
+        <v>5.78</v>
       </c>
       <c r="G57" t="n">
-        <v>1361053600</v>
+        <v>1351699289</v>
       </c>
       <c r="H57" t="n">
-        <v>2969300</v>
+        <v>1265300</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4073998987377238</v>
+        <v>0.4045999022099153</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>101799072.5504862</v>
+        <v>101099423.2610322</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>8.880000000000001</v>
+        <v>8.81</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,28 +13592,28 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>125.62</v>
+        <v>127.19</v>
       </c>
       <c r="BD57" t="n">
-        <v>84.22</v>
+        <v>85.5</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-80.63</v>
+        <v>-80.48999999999999</v>
       </c>
       <c r="BG57" t="n">
-        <v>7.63</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
       </c>
       <c r="BI57" t="n">
-        <v>-2.68</v>
+        <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>5.98</v>
+        <v>5.78</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,28 +13622,28 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>6.08</v>
+        <v>5.86</v>
       </c>
       <c r="BN57" t="n">
         <v>6.08</v>
       </c>
       <c r="BO57" t="n">
-        <v>3.37</v>
+        <v>3.38</v>
       </c>
       <c r="BP57" t="n">
-        <v>5.82</v>
+        <v>5.68</v>
       </c>
       <c r="BQ57" t="n">
-        <v>5.62</v>
+        <v>5.58</v>
       </c>
       <c r="BR57" t="n">
-        <v>5.98</v>
+        <v>5.84</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1126425</v>
+        <v>1207036</v>
       </c>
     </row>
     <row r="58">
@@ -13903,13 +13903,13 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G59" t="n">
-        <v>93636910</v>
+        <v>95156610</v>
       </c>
       <c r="H59" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="I59" t="n">
         <v>710143</v>
@@ -13924,7 +13924,7 @@
         <v>0.61</v>
       </c>
       <c r="M59" t="n">
-        <v>9.946451820931415</v>
+        <v>10.10787986071049</v>
       </c>
       <c r="N59" t="n">
         <v>0.15</v>
@@ -14002,7 +14002,7 @@
         <v>1881878.95</v>
       </c>
       <c r="AM59" t="n">
-        <v>15817045.60810811</v>
+        <v>16073751.68918919</v>
       </c>
       <c r="AN59" t="n">
         <v>1.4</v>
@@ -14043,7 +14043,7 @@
         <v>35.09</v>
       </c>
       <c r="AZ59" t="n">
-        <v>25.97</v>
+        <v>24.73</v>
       </c>
       <c r="BA59" t="n">
         <v>3.69</v>
@@ -14052,28 +14052,28 @@
         <v>22.8</v>
       </c>
       <c r="BC59" t="n">
-        <v>104.66</v>
+        <v>114.89</v>
       </c>
       <c r="BD59" t="n">
-        <v>67.11</v>
+        <v>75.45999999999999</v>
       </c>
       <c r="BE59" t="n">
         <v>23.67</v>
       </c>
       <c r="BF59" t="n">
-        <v>-82.44</v>
+        <v>-81.56</v>
       </c>
       <c r="BG59" t="n">
-        <v>8.56</v>
+        <v>13.99</v>
       </c>
       <c r="BH59" t="n">
         <v>30.98</v>
       </c>
       <c r="BI59" t="n">
-        <v>11.35</v>
+        <v>0</v>
       </c>
       <c r="BJ59" t="n">
-        <v>18.86</v>
+        <v>20</v>
       </c>
       <c r="BK59" t="n">
         <v>2.65</v>
@@ -14091,10 +14091,10 @@
         <v>15.66</v>
       </c>
       <c r="BP59" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="BQ59" t="n">
-        <v>7.92</v>
+        <v>7.54</v>
       </c>
       <c r="BR59" t="n">
         <v>21</v>
@@ -14103,7 +14103,7 @@
         <v>1.42</v>
       </c>
       <c r="BT59" t="n">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
     <row r="60">
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>377</v>
+        <v>372.01</v>
       </c>
       <c r="G60" t="n">
-        <v>171440787</v>
+        <v>169171589</v>
       </c>
       <c r="H60" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.82352952940177</v>
+        <v>12.65379671336507</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-25137945.30791789</v>
+        <v>-24805218.32844575</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2167.75</v>
+        <v>2139.06</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,19 +14282,19 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>206.95</v>
+        <v>211.07</v>
       </c>
       <c r="BD60" t="n">
-        <v>150.63</v>
+        <v>153.99</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-38.7</v>
+        <v>-37.88</v>
       </c>
       <c r="BG60" t="n">
-        <v>93.09999999999999</v>
+        <v>95.69</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>377</v>
+        <v>372.01</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14312,7 +14312,7 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>377</v>
+        <v>372.1</v>
       </c>
       <c r="BN60" t="n">
         <v>405</v>
@@ -14321,19 +14321,19 @@
         <v>306.27</v>
       </c>
       <c r="BP60" t="n">
-        <v>370.01</v>
+        <v>371.5</v>
       </c>
       <c r="BQ60" t="n">
-        <v>2.88</v>
+        <v>2.84</v>
       </c>
       <c r="BR60" t="n">
-        <v>373.01</v>
+        <v>371.5</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
       </c>
       <c r="BT60" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="61">
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>25.74</v>
+        <v>25.54</v>
       </c>
       <c r="G61" t="n">
-        <v>2203560196</v>
+        <v>2186438358</v>
       </c>
       <c r="H61" t="n">
-        <v>543200</v>
+        <v>451700</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.168623628011524</v>
+        <v>1.159543329466421</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>172963908.6342229</v>
+        <v>171619965.3061225</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>32.43</v>
+        <v>32.18</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-16.46</v>
+        <v>-15.8</v>
       </c>
       <c r="BD61" t="n">
-        <v>-31.79</v>
+        <v>-31.25</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-90.2</v>
+        <v>-90.12</v>
       </c>
       <c r="BG61" t="n">
-        <v>-54.33</v>
+        <v>-53.97</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>25.74</v>
+        <v>25.54</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,28 +14542,28 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>26.17</v>
+        <v>25.84</v>
       </c>
       <c r="BN61" t="n">
         <v>28.25</v>
       </c>
       <c r="BO61" t="n">
-        <v>18.71</v>
+        <v>19.2</v>
       </c>
       <c r="BP61" t="n">
-        <v>25.32</v>
+        <v>25.34</v>
       </c>
       <c r="BQ61" t="n">
-        <v>13.82</v>
+        <v>13.72</v>
       </c>
       <c r="BR61" t="n">
-        <v>26</v>
+        <v>25.34</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>447533</v>
+        <v>454761</v>
       </c>
     </row>
     <row r="62">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.34</v>
+        <v>1.33</v>
       </c>
       <c r="G63" t="n">
-        <v>349083006</v>
+        <v>346477912</v>
       </c>
       <c r="H63" t="n">
-        <v>3100</v>
+        <v>10100</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.429354082561069</v>
+        <v>0.4261499513798583</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>198342617.0454545</v>
+        <v>196862450</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-78.42</v>
+        <v>-78.26000000000001</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14990,10 +14990,10 @@
         <v>-5.91</v>
       </c>
       <c r="BI63" t="n">
-        <v>3.88</v>
+        <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.29</v>
+        <v>1.33</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.34</v>
+        <v>1.33</v>
       </c>
       <c r="BN63" t="n">
         <v>1.54</v>
@@ -15011,19 +15011,19 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.34</v>
+        <v>1.33</v>
       </c>
       <c r="BQ63" t="n">
-        <v>5.13</v>
+        <v>5.09</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.34</v>
+        <v>1.33</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>14057</v>
+        <v>14157</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>60.53</v>
+        <v>59.06</v>
       </c>
       <c r="G64" t="n">
-        <v>234620025618</v>
+        <v>229788350003</v>
       </c>
       <c r="H64" t="n">
-        <v>16775900</v>
+        <v>12264400</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>67269004199.22311</v>
+        <v>65883691899.56499</v>
       </c>
       <c r="AL64" t="n">
-        <v>18754598370.7434</v>
+        <v>18368373301.59872</v>
       </c>
       <c r="AM64" t="n">
-        <v>20892255175.24488</v>
+        <v>20462008014.51469</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>24.21</v>
+        <v>23.62</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,19 +15202,19 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-21.13</v>
+        <v>-19.17</v>
       </c>
       <c r="BD64" t="n">
-        <v>-35.6</v>
+        <v>-34</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-88.94</v>
+        <v>-88.67</v>
       </c>
       <c r="BG64" t="n">
-        <v>-82.81999999999999</v>
+        <v>-82.40000000000001</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
@@ -15223,7 +15223,7 @@
         <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>60.53</v>
+        <v>59.06</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,28 +15232,28 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>61.3</v>
+        <v>59.84</v>
       </c>
       <c r="BN64" t="n">
         <v>64.72</v>
       </c>
       <c r="BO64" t="n">
-        <v>44.03</v>
+        <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>59.95</v>
+        <v>58.28</v>
       </c>
       <c r="BQ64" t="n">
-        <v>38.55</v>
+        <v>37.62</v>
       </c>
       <c r="BR64" t="n">
-        <v>60</v>
+        <v>59.84</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>11445204</v>
+        <v>11895563</v>
       </c>
     </row>
     <row r="65">
@@ -15286,10 +15286,10 @@
         <v>23.8</v>
       </c>
       <c r="G65" t="n">
-        <v>234620025618</v>
+        <v>229788350003</v>
       </c>
       <c r="H65" t="n">
-        <v>6300</v>
+        <v>5300</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.672160338291392</v>
+        <v>5.555350024599269</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>17574533754.1573</v>
+        <v>17212610487.1161</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15450,10 +15450,10 @@
         <v>7.12</v>
       </c>
       <c r="BI65" t="n">
-        <v>1.41</v>
+        <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>23.47</v>
+        <v>23.8</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>23.86</v>
+        <v>23.83</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>23.52</v>
+        <v>23.43</v>
       </c>
       <c r="BQ65" t="n">
         <v>15.16</v>
       </c>
       <c r="BR65" t="n">
-        <v>23.53</v>
+        <v>23.6</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>15503</v>
+        <v>13771</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>20.78</v>
+        <v>20.45</v>
       </c>
       <c r="G66" t="n">
-        <v>234620025618</v>
+        <v>229788350003</v>
       </c>
       <c r="H66" t="n">
-        <v>2500</v>
+        <v>1400</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>13.92836199770083</v>
+        <v>13.64152660569233</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>21042154763.94619</v>
+        <v>20608820628.07175</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>8.35</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,28 +15662,28 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-23.44</v>
+        <v>-22.2</v>
       </c>
       <c r="BD66" t="n">
-        <v>-37.49</v>
+        <v>-36.48</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-89.26000000000001</v>
+        <v>-89.09</v>
       </c>
       <c r="BG66" t="n">
-        <v>-83.31999999999999</v>
+        <v>-83.05</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
       </c>
       <c r="BI66" t="n">
-        <v>5.97</v>
+        <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>19.61</v>
+        <v>20.45</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>21.16</v>
+        <v>20.92</v>
       </c>
       <c r="BN66" t="n">
         <v>21.16</v>
@@ -15701,19 +15701,19 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>19.57</v>
+        <v>20.03</v>
       </c>
       <c r="BQ66" t="n">
-        <v>13.23</v>
+        <v>13.02</v>
       </c>
       <c r="BR66" t="n">
-        <v>21.16</v>
+        <v>20.77</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>7182</v>
+        <v>7052</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>19.34</v>
+        <v>19.49</v>
       </c>
       <c r="G68" t="n">
-        <v>8554903997</v>
+        <v>8388023022</v>
       </c>
       <c r="H68" t="n">
-        <v>34900</v>
+        <v>26700</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>593266573.9944521</v>
+        <v>581693690.8460472</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>35.78</v>
+        <v>36.06</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,28 +16122,28 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>35.49</v>
+        <v>34.44</v>
       </c>
       <c r="BD68" t="n">
-        <v>10.62</v>
+        <v>9.77</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.59</v>
+        <v>-93.64</v>
       </c>
       <c r="BG68" t="n">
-        <v>227.04</v>
+        <v>224.52</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
       </c>
       <c r="BI68" t="n">
-        <v>0.21</v>
+        <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>19.3</v>
+        <v>19.49</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>19.64</v>
+        <v>19.49</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,19 +16161,19 @@
         <v>15.07</v>
       </c>
       <c r="BP68" t="n">
-        <v>19.2</v>
+        <v>19.22</v>
       </c>
       <c r="BQ68" t="n">
-        <v>13.01</v>
+        <v>13.11</v>
       </c>
       <c r="BR68" t="n">
-        <v>19.3</v>
+        <v>19.38</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>31650</v>
+        <v>31923</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>22.9</v>
+        <v>22.57</v>
       </c>
       <c r="G69" t="n">
-        <v>8554903997</v>
+        <v>8388023022</v>
       </c>
       <c r="H69" t="n">
-        <v>1770900</v>
+        <v>2330400</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>509220476.0119047</v>
+        <v>499287084.6428571</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>40.04</v>
+        <v>39.46</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,28 +16352,28 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>14.42</v>
+        <v>16.1</v>
       </c>
       <c r="BD69" t="n">
-        <v>-6.57</v>
+        <v>-5.21</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-94.59</v>
+        <v>-94.51000000000001</v>
       </c>
       <c r="BG69" t="n">
-        <v>203.87</v>
+        <v>208.32</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
       </c>
       <c r="BI69" t="n">
-        <v>1.87</v>
+        <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>22.48</v>
+        <v>22.57</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,28 +16382,28 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>23.23</v>
+        <v>23.05</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
       </c>
       <c r="BO69" t="n">
-        <v>16.57</v>
+        <v>16.6</v>
       </c>
       <c r="BP69" t="n">
-        <v>22.75</v>
+        <v>22.54</v>
       </c>
       <c r="BQ69" t="n">
-        <v>15.4</v>
+        <v>15.18</v>
       </c>
       <c r="BR69" t="n">
-        <v>22.75</v>
+        <v>22.68</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>1792650</v>
+        <v>1822340</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>18.25</v>
+        <v>18.42</v>
       </c>
       <c r="G70" t="n">
-        <v>8478168900</v>
+        <v>8557143659</v>
       </c>
       <c r="H70" t="n">
-        <v>4666200</v>
+        <v>2672000</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6691665687167766</v>
+        <v>0.6753999039001869</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2798075544.554456</v>
+        <v>2824139821.452146</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.1</v>
+        <v>2.12</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,28 +16582,28 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-53.7</v>
+        <v>-54.13</v>
       </c>
       <c r="BD70" t="n">
-        <v>-62.2</v>
+        <v>-62.55</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
       </c>
       <c r="BF70" t="n">
-        <v>-99.34</v>
+        <v>-99.34999999999999</v>
       </c>
       <c r="BG70" t="n">
-        <v>-94.14</v>
+        <v>-94.19</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
       </c>
       <c r="BI70" t="n">
-        <v>2.07</v>
+        <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>17.88</v>
+        <v>18.42</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>18.89</v>
+        <v>18.61</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>18.25</v>
+        <v>18.28</v>
       </c>
       <c r="BQ70" t="n">
-        <v>183.03</v>
+        <v>184.74</v>
       </c>
       <c r="BR70" t="n">
-        <v>18.25</v>
+        <v>18.33</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>6948910</v>
+        <v>6559547</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-09-11 05:29
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>24.65</v>
+        <v>25</v>
       </c>
       <c r="G3" t="n">
-        <v>3297351568</v>
+        <v>3352330000</v>
       </c>
       <c r="H3" t="n">
-        <v>426800</v>
+        <v>478900</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8204545068307224</v>
+        <v>0.8341343651602502</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>644013978.125</v>
+        <v>654751953.125</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>45.11</v>
+        <v>45.75</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>100.81</v>
+        <v>97.98999999999999</v>
       </c>
       <c r="BD3" t="n">
-        <v>63.96</v>
+        <v>61.66</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-80.25</v>
+        <v>-80.53</v>
       </c>
       <c r="BG3" t="n">
-        <v>-14.26</v>
+        <v>-15.46</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>24.65</v>
+        <v>25</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>24.73</v>
+        <v>25.18</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>24.19</v>
+        <v>24.49</v>
       </c>
       <c r="BQ3" t="n">
-        <v>5.61</v>
+        <v>5.69</v>
       </c>
       <c r="BR3" t="n">
-        <v>24.45</v>
+        <v>24.63</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>526530</v>
+        <v>523503</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.58</v>
+        <v>15.74</v>
       </c>
       <c r="G4" t="n">
-        <v>241251001618</v>
+        <v>240031061509</v>
       </c>
       <c r="H4" t="n">
-        <v>22611500</v>
+        <v>21311000</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.731692457467255</v>
+        <v>2.717879038364467</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>23886237783.9604</v>
+        <v>23765451634.55445</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.45</v>
+        <v>19.65</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-25.52</v>
+        <v>-26.27</v>
       </c>
       <c r="BD4" t="n">
-        <v>-39.19</v>
+        <v>-39.8</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.76000000000001</v>
+        <v>-92.84</v>
       </c>
       <c r="BG4" t="n">
-        <v>-26.91</v>
+        <v>-27.66</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.58</v>
+        <v>15.74</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.78</v>
+        <v>15.79</v>
       </c>
       <c r="BN4" t="n">
         <v>17</v>
@@ -1465,19 +1465,19 @@
         <v>11.09</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.51</v>
+        <v>15.47</v>
       </c>
       <c r="BQ4" t="n">
-        <v>15.03</v>
+        <v>15.18</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.69</v>
+        <v>15.56</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>31598293</v>
+        <v>31103410</v>
       </c>
     </row>
     <row r="5">
@@ -1740,10 +1740,10 @@
         <v>7.29</v>
       </c>
       <c r="G6" t="n">
-        <v>459887387</v>
+        <v>453664352</v>
       </c>
       <c r="H6" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="I6" t="n">
         <v>63084700</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>7.159546185249855</v>
+        <v>7.062665714607753</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>43966289.38814531</v>
+        <v>43371352.96367113</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -1916,7 +1916,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>7.29</v>
+        <v>7.35</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
@@ -1931,13 +1931,13 @@
         <v>12.96</v>
       </c>
       <c r="BR6" t="n">
-        <v>7.29</v>
+        <v>7.35</v>
       </c>
       <c r="BS6" t="n">
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>360</v>
+        <v>287</v>
       </c>
     </row>
     <row r="7">
@@ -3120,10 +3120,10 @@
         <v>5.1</v>
       </c>
       <c r="G12" t="n">
-        <v>489403793</v>
+        <v>479992152</v>
       </c>
       <c r="H12" t="n">
-        <v>381900</v>
+        <v>634500</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.08850792916548846</v>
+        <v>0.08680584825219441</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>526240637.6344086</v>
+        <v>516120593.5483871</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3296,7 +3296,7 @@
         <v>3.43</v>
       </c>
       <c r="BM12" t="n">
-        <v>5.24</v>
+        <v>5.21</v>
       </c>
       <c r="BN12" t="n">
         <v>8.23</v>
@@ -3305,19 +3305,19 @@
         <v>4.42</v>
       </c>
       <c r="BP12" t="n">
-        <v>5.07</v>
+        <v>5.01</v>
       </c>
       <c r="BQ12" t="n">
         <v>1.49</v>
       </c>
       <c r="BR12" t="n">
-        <v>5.24</v>
+        <v>5.11</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>465160</v>
+        <v>466910</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>28.52</v>
+        <v>29.07</v>
       </c>
       <c r="G13" t="n">
-        <v>14379524698</v>
+        <v>14305710224</v>
       </c>
       <c r="H13" t="n">
-        <v>3908600</v>
+        <v>3944100</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>4.973270967297001</v>
+        <v>4.947741654734844</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1496308501.352758</v>
+        <v>1488627494.693028</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>51.62</v>
+        <v>52.62</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>14.21</v>
+        <v>12.05</v>
       </c>
       <c r="BD13" t="n">
-        <v>-6.75</v>
+        <v>-8.51</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-90.87</v>
+        <v>-91.04000000000001</v>
       </c>
       <c r="BG13" t="n">
-        <v>-69.52</v>
+        <v>-70.09</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>28.52</v>
+        <v>29.07</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>28.96</v>
+        <v>29.22</v>
       </c>
       <c r="BN13" t="n">
         <v>32.43</v>
@@ -3535,19 +3535,19 @@
         <v>21.06</v>
       </c>
       <c r="BP13" t="n">
-        <v>28.3</v>
+        <v>28.2</v>
       </c>
       <c r="BQ13" t="n">
-        <v>14.57</v>
+        <v>14.85</v>
       </c>
       <c r="BR13" t="n">
-        <v>28.92</v>
+        <v>28.46</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>4486072</v>
+        <v>4522623</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>10.04</v>
+        <v>9.94</v>
       </c>
       <c r="G14" t="n">
-        <v>7999197250</v>
+        <v>8082747775</v>
       </c>
       <c r="H14" t="n">
-        <v>7300</v>
+        <v>6000</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.321408905397762</v>
+        <v>3.35610056871256</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>887813235.2941177</v>
+        <v>897086323.5294118</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>8.07</v>
+        <v>7.99</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>10.39</v>
+        <v>11.5</v>
       </c>
       <c r="BD14" t="n">
-        <v>-9.869999999999999</v>
+        <v>-8.960000000000001</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-85.84</v>
+        <v>-85.7</v>
       </c>
       <c r="BG14" t="n">
-        <v>-40.81</v>
+        <v>-40.22</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>10.04</v>
+        <v>9.94</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>10.04</v>
+        <v>9.94</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,19 +3765,19 @@
         <v>7.65</v>
       </c>
       <c r="BP14" t="n">
-        <v>9.800000000000001</v>
+        <v>9.75</v>
       </c>
       <c r="BQ14" t="n">
-        <v>9.91</v>
+        <v>9.81</v>
       </c>
       <c r="BR14" t="n">
-        <v>10</v>
+        <v>9.75</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>12347</v>
+        <v>12320</v>
       </c>
     </row>
     <row r="15">
@@ -3810,10 +3810,10 @@
         <v>13.25</v>
       </c>
       <c r="G15" t="n">
-        <v>7999197250</v>
+        <v>8082747775</v>
       </c>
       <c r="H15" t="n">
-        <v>3557300</v>
+        <v>1838000</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.282342582131136</v>
+        <v>3.316626203024084</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>667155733.9449542</v>
+        <v>674124084.6538782</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>13.51</v>
+        <v>13.33</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>12.91</v>
+        <v>13.05</v>
       </c>
       <c r="BQ15" t="n">
         <v>13.08</v>
       </c>
       <c r="BR15" t="n">
-        <v>12.99</v>
+        <v>13.17</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2240040</v>
+        <v>2318043</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.32</v>
+        <v>4.4</v>
       </c>
       <c r="G16" t="n">
-        <v>947400661</v>
+        <v>953904620</v>
       </c>
       <c r="H16" t="n">
-        <v>151000</v>
+        <v>111500</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.448199950061269</v>
+        <v>0.4512768680105594</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>266123781.1797753</v>
+        <v>267950735.9550562</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-59.75</v>
+        <v>-60.48</v>
       </c>
       <c r="BD16" t="n">
-        <v>-67.13</v>
+        <v>-67.73</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.15000000000001</v>
+        <v>-98.18000000000001</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>4.32</v>
+        <v>4.4</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,7 +4216,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.52</v>
+        <v>4.49</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
@@ -4225,19 +4225,19 @@
         <v>2.97</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.27</v>
+        <v>4.31</v>
       </c>
       <c r="BQ16" t="n">
-        <v>58.95</v>
+        <v>60.04</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.47</v>
+        <v>4.31</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>141217</v>
+        <v>141257</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>33.39</v>
+        <v>33.99</v>
       </c>
       <c r="G17" t="n">
-        <v>11006241989</v>
+        <v>11032206223</v>
       </c>
       <c r="H17" t="n">
-        <v>558600</v>
+        <v>638700</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>4970304366.419798</v>
+        <v>4982029544.346099</v>
       </c>
       <c r="AL17" t="n">
-        <v>1375780248.625</v>
+        <v>1379025777.875</v>
       </c>
       <c r="AM17" t="n">
-        <v>3407505259.752322</v>
+        <v>3415543722.291022</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>17.86</v>
+        <v>18.18</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>57.64</v>
+        <v>54.86</v>
       </c>
       <c r="BD17" t="n">
-        <v>28.72</v>
+        <v>26.44</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-86.38</v>
+        <v>-86.62</v>
       </c>
       <c r="BG17" t="n">
-        <v>-51.08</v>
+        <v>-51.95</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>33.39</v>
+        <v>33.99</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,7 +4446,7 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>33.81</v>
+        <v>33.99</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
@@ -4455,19 +4455,19 @@
         <v>29.28</v>
       </c>
       <c r="BP17" t="n">
-        <v>33.26</v>
+        <v>33.07</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.65</v>
+        <v>2.69</v>
       </c>
       <c r="BR17" t="n">
-        <v>33.5</v>
+        <v>33.39</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1069139</v>
+        <v>1071150</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>11.75</v>
+        <v>11.74</v>
       </c>
       <c r="G18" t="n">
-        <v>11006241989</v>
+        <v>11032206223</v>
       </c>
       <c r="H18" t="n">
-        <v>2500</v>
+        <v>4300</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.240669868006998</v>
+        <v>3.248314758138777</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3275667258.630952</v>
+        <v>3283394709.226191</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>49.15</v>
+        <v>49.28</v>
       </c>
       <c r="BD18" t="n">
-        <v>21.78</v>
+        <v>21.88</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-87.13</v>
+        <v>-87.12</v>
       </c>
       <c r="BG18" t="n">
-        <v>-53.66</v>
+        <v>-53.62</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>11.75</v>
+        <v>11.74</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>12</v>
+        <v>11.95</v>
       </c>
       <c r="BN18" t="n">
         <v>13.82</v>
@@ -4685,19 +4685,19 @@
         <v>10.11</v>
       </c>
       <c r="BP18" t="n">
-        <v>11.57</v>
+        <v>11.58</v>
       </c>
       <c r="BQ18" t="n">
         <v>0.93</v>
       </c>
       <c r="BR18" t="n">
-        <v>11.65</v>
+        <v>11.58</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>9648</v>
+        <v>9678</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.86</v>
+        <v>11.05</v>
       </c>
       <c r="G19" t="n">
-        <v>11006241989</v>
+        <v>11032206223</v>
       </c>
       <c r="H19" t="n">
-        <v>7600</v>
+        <v>9300</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.856285591278343</v>
+        <v>6.872459886159439</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3494045075.873016</v>
+        <v>3502287689.84127</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>5.97</v>
+        <v>6.08</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>61.37</v>
+        <v>58.6</v>
       </c>
       <c r="BD19" t="n">
-        <v>31.76</v>
+        <v>29.49</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-86.06999999999999</v>
+        <v>-86.31</v>
       </c>
       <c r="BG19" t="n">
-        <v>-51.66</v>
+        <v>-52.49</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>10.86</v>
+        <v>11.05</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>11.05</v>
+        <v>11.09</v>
       </c>
       <c r="BN19" t="n">
         <v>11.41</v>
@@ -4915,19 +4915,19 @@
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
+        <v>10.83</v>
+      </c>
+      <c r="BQ19" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="BR19" t="n">
         <v>10.86</v>
-      </c>
-      <c r="BQ19" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="BR19" t="n">
-        <v>11.05</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>14046</v>
+        <v>13927</v>
       </c>
     </row>
     <row r="20">
@@ -5420,10 +5420,10 @@
         <v>5.27</v>
       </c>
       <c r="G22" t="n">
-        <v>1055292200</v>
+        <v>1026087441</v>
       </c>
       <c r="H22" t="n">
-        <v>1469300</v>
+        <v>1203200</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.089506304615714</v>
+        <v>0.08702925602643938</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>239295283.446712</v>
+        <v>232672889.1156462</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>5.5</v>
+        <v>5.29</v>
       </c>
       <c r="BN22" t="n">
         <v>8.82</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>5.17</v>
+        <v>5.04</v>
       </c>
       <c r="BQ22" t="n">
         <v>7.85</v>
       </c>
       <c r="BR22" t="n">
-        <v>5.5</v>
+        <v>5.17</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1601227</v>
+        <v>1567963</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.91</v>
+        <v>2.9</v>
       </c>
       <c r="G24" t="n">
-        <v>1175258242</v>
+        <v>1117458196</v>
       </c>
       <c r="H24" t="n">
-        <v>6288500</v>
+        <v>5255800</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2841078994387012</v>
+        <v>0.2701352685141352</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1058791209.009009</v>
+        <v>1006719095.495495</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6026,19 +6026,19 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>145.93</v>
+        <v>146.77</v>
       </c>
       <c r="BD24" t="n">
-        <v>100.8</v>
+        <v>101.49</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-86.94</v>
+        <v>-86.90000000000001</v>
       </c>
       <c r="BG24" t="n">
-        <v>-49.9</v>
+        <v>-49.73</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
@@ -6047,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>2.91</v>
+        <v>2.9</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>3.03</v>
+        <v>2.97</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.9</v>
+        <v>2.82</v>
       </c>
       <c r="BQ24" t="n">
-        <v>7.15</v>
+        <v>7.12</v>
       </c>
       <c r="BR24" t="n">
-        <v>3.01</v>
+        <v>2.88</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>9557933</v>
+        <v>9434990</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>3.91</v>
+        <v>3.85</v>
       </c>
       <c r="G25" t="n">
-        <v>1354791960</v>
+        <v>1262941648</v>
       </c>
       <c r="H25" t="n">
-        <v>2478900</v>
+        <v>2418000</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.6755611314209489</v>
+        <v>0.6297603719478212</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>498085279.4117647</v>
+        <v>464316782.3529412</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>9.109999999999999</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,19 +6256,19 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>2.55</v>
+        <v>4.15</v>
       </c>
       <c r="BD25" t="n">
-        <v>-16.27</v>
+        <v>-14.96</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-94.06999999999999</v>
+        <v>-93.98</v>
       </c>
       <c r="BG25" t="n">
-        <v>-43.74</v>
+        <v>-42.86</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>3.91</v>
+        <v>3.85</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>4.14</v>
+        <v>4.05</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>3.87</v>
+        <v>3.79</v>
       </c>
       <c r="BQ25" t="n">
-        <v>16.52</v>
+        <v>16.27</v>
       </c>
       <c r="BR25" t="n">
-        <v>4.14</v>
+        <v>3.92</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1064750</v>
+        <v>1130520</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>9.199999999999999</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="G26" t="n">
-        <v>12460415341</v>
+        <v>13456700751</v>
       </c>
       <c r="H26" t="n">
-        <v>5988400</v>
+        <v>15999900</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.160676005426322</v>
+        <v>0.1735230218027824</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>4450148336.071429</v>
+        <v>4805964553.928572</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>1.76</v>
+        <v>1.89</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-5.92</v>
+        <v>-12.21</v>
       </c>
       <c r="BD26" t="n">
-        <v>-23.18</v>
+        <v>-28.32</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-92.83</v>
+        <v>-93.31</v>
       </c>
       <c r="BG26" t="n">
-        <v>-87.03</v>
+        <v>-87.90000000000001</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>9.199999999999999</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,7 +6516,7 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>9.199999999999999</v>
+        <v>9.92</v>
       </c>
       <c r="BN26" t="n">
         <v>10.6</v>
@@ -6525,19 +6525,19 @@
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>8.949999999999999</v>
+        <v>9.09</v>
       </c>
       <c r="BQ26" t="n">
-        <v>12.83</v>
+        <v>13.75</v>
       </c>
       <c r="BR26" t="n">
-        <v>9.050000000000001</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>11370577</v>
+        <v>11381943</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>16.64</v>
+        <v>17</v>
       </c>
       <c r="G34" t="n">
-        <v>3435988481</v>
+        <v>3425913100</v>
       </c>
       <c r="H34" t="n">
-        <v>4002600</v>
+        <v>2287300</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.3020635178006436</v>
+        <v>0.3011777741362306</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>714342719.5426196</v>
+        <v>712248045.7380458</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>38.83</v>
+        <v>39.67</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>122.89</v>
+        <v>118.17</v>
       </c>
       <c r="BD34" t="n">
-        <v>81.98999999999999</v>
+        <v>78.13</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-86.20999999999999</v>
+        <v>-86.5</v>
       </c>
       <c r="BG34" t="n">
-        <v>51.79</v>
+        <v>48.58</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>16.64</v>
+        <v>17</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>17</v>
+        <v>17.05</v>
       </c>
       <c r="BN34" t="n">
         <v>31.12</v>
@@ -8353,19 +8353,19 @@
         <v>14.32</v>
       </c>
       <c r="BP34" t="n">
-        <v>16.1</v>
+        <v>16.4</v>
       </c>
       <c r="BQ34" t="n">
-        <v>10.55</v>
+        <v>10.78</v>
       </c>
       <c r="BR34" t="n">
-        <v>16.99</v>
+        <v>16.5</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>3052970</v>
+        <v>3143817</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>17.29</v>
+        <v>17.66</v>
       </c>
       <c r="G35" t="n">
-        <v>87253989620</v>
+        <v>87352893445</v>
       </c>
       <c r="H35" t="n">
-        <v>57684700</v>
+        <v>83504800</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.243857930723889</v>
+        <v>7.252068962221995</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7211073522.31405</v>
+        <v>7219247392.148761</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.09</v>
+        <v>10.3</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,19 +8544,19 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-45.6</v>
+        <v>-46.74</v>
       </c>
       <c r="BD35" t="n">
-        <v>-55.58</v>
+        <v>-56.51</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-93.56</v>
+        <v>-93.69</v>
       </c>
       <c r="BG35" t="n">
-        <v>-47.27</v>
+        <v>-48.38</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
@@ -8565,7 +8565,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>17.29</v>
+        <v>17.66</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>17.51</v>
+        <v>17.81</v>
       </c>
       <c r="BN35" t="n">
         <v>20.08</v>
@@ -8583,19 +8583,19 @@
         <v>11.7</v>
       </c>
       <c r="BP35" t="n">
-        <v>17.08</v>
+        <v>16.98</v>
       </c>
       <c r="BQ35" t="n">
-        <v>16.55</v>
+        <v>16.9</v>
       </c>
       <c r="BR35" t="n">
-        <v>17.47</v>
+        <v>17.15</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>34834187</v>
+        <v>36094857</v>
       </c>
     </row>
     <row r="36">
@@ -8858,7 +8858,7 @@
         <v>15</v>
       </c>
       <c r="G37" t="n">
-        <v>202125000</v>
+        <v>203118150</v>
       </c>
       <c r="H37" t="n">
         <v>200</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.967857142857143</v>
+        <v>1.977526294725682</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>48355263.15789474</v>
+        <v>48592858.85167465</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -9055,7 +9055,7 @@
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>873</v>
+        <v>843</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>68.31</v>
+        <v>67.42</v>
       </c>
       <c r="G39" t="n">
-        <v>3829343019</v>
+        <v>3715273387</v>
       </c>
       <c r="H39" t="n">
-        <v>2900</v>
+        <v>4300</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1922162226582197</v>
+        <v>0.1864904274828428</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>402241913.7605042</v>
+        <v>390259809.5588235</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>199.58</v>
+        <v>196.98</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>205.23</v>
+        <v>209.26</v>
       </c>
       <c r="BD39" t="n">
-        <v>149.22</v>
+        <v>152.51</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-72.17</v>
+        <v>-71.8</v>
       </c>
       <c r="BG39" t="n">
-        <v>34.28</v>
+        <v>36.05</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>68.31</v>
+        <v>67.42</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>69.89</v>
+        <v>68.22</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>68.31</v>
+        <v>67</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.53</v>
+        <v>4.47</v>
       </c>
       <c r="BR39" t="n">
-        <v>69.89</v>
+        <v>67.56</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>4087</v>
+        <v>4017</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>22.18</v>
+        <v>22.8</v>
       </c>
       <c r="G40" t="n">
-        <v>127109944228</v>
+        <v>128234742508</v>
       </c>
       <c r="H40" t="n">
-        <v>30236100</v>
+        <v>32524900</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.385667301384608</v>
+        <v>0.3890800785664746</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6592839430.912863</v>
+        <v>6651179590.6639</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>11.2</v>
+        <v>11.51</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>99.5</v>
+        <v>94.06999999999999</v>
       </c>
       <c r="BD40" t="n">
-        <v>62.89</v>
+        <v>58.46</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-87.56</v>
+        <v>-87.90000000000001</v>
       </c>
       <c r="BG40" t="n">
-        <v>25.75</v>
+        <v>22.33</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>22.18</v>
+        <v>22.8</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>22.65</v>
+        <v>22.91</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>21.97</v>
+        <v>21.91</v>
       </c>
       <c r="BQ40" t="n">
-        <v>8.880000000000001</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="BR40" t="n">
-        <v>22.44</v>
+        <v>22</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>29733273</v>
+        <v>30359901</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>15.83</v>
+        <v>16.24</v>
       </c>
       <c r="G41" t="n">
-        <v>187257905436</v>
+        <v>190888600871</v>
       </c>
       <c r="H41" t="n">
-        <v>8701800</v>
+        <v>8101200</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.247880775206551</v>
+        <v>1.272075615063473</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>28853298218.18182</v>
+        <v>29412727406.93374</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>23.69</v>
+        <v>24.31</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,19 +9924,19 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>88.79000000000001</v>
+        <v>84.02</v>
       </c>
       <c r="BD41" t="n">
-        <v>54.15</v>
+        <v>50.25</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-84.04000000000001</v>
+        <v>-84.44</v>
       </c>
       <c r="BG41" t="n">
-        <v>-13.01</v>
+        <v>-15.21</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
@@ -9945,7 +9945,7 @@
         <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>15.83</v>
+        <v>16.24</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,7 +9954,7 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>15.97</v>
+        <v>16.33</v>
       </c>
       <c r="BN41" t="n">
         <v>18.28</v>
@@ -9963,19 +9963,19 @@
         <v>13.34</v>
       </c>
       <c r="BP41" t="n">
-        <v>15.73</v>
+        <v>15.64</v>
       </c>
       <c r="BQ41" t="n">
-        <v>6.77</v>
+        <v>6.95</v>
       </c>
       <c r="BR41" t="n">
-        <v>15.93</v>
+        <v>15.77</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>7215953</v>
+        <v>7367271</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>17.79</v>
+        <v>18.48</v>
       </c>
       <c r="G42" t="n">
-        <v>187257905436</v>
+        <v>190888600871</v>
       </c>
       <c r="H42" t="n">
-        <v>30056500</v>
+        <v>51431900</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.251592586628512</v>
+        <v>1.275859393843789</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>25477266045.71429</v>
+        <v>25971238213.7415</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>25.77</v>
+        <v>26.77</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,19 +10154,19 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>67.98999999999999</v>
+        <v>61.72</v>
       </c>
       <c r="BD42" t="n">
-        <v>37.16</v>
+        <v>32.04</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-85.79000000000001</v>
+        <v>-86.31999999999999</v>
       </c>
       <c r="BG42" t="n">
-        <v>-15.04</v>
+        <v>-18.21</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
@@ -10175,7 +10175,7 @@
         <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>17.79</v>
+        <v>18.48</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>18.15</v>
+        <v>18.55</v>
       </c>
       <c r="BN42" t="n">
         <v>21.33</v>
@@ -10193,19 +10193,19 @@
         <v>15.64</v>
       </c>
       <c r="BP42" t="n">
-        <v>17.74</v>
+        <v>17.66</v>
       </c>
       <c r="BQ42" t="n">
-        <v>7.61</v>
+        <v>7.91</v>
       </c>
       <c r="BR42" t="n">
-        <v>18</v>
+        <v>17.75</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>39559117</v>
+        <v>39887876</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>40.91</v>
+        <v>41.2</v>
       </c>
       <c r="G43" t="n">
-        <v>79422673703</v>
+        <v>77265945830</v>
       </c>
       <c r="H43" t="n">
-        <v>6808900</v>
+        <v>5918300</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9673894482.704018</v>
+        <v>9411199248.477465</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>74.25</v>
+        <v>74.78</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-40.27</v>
+        <v>-40.69</v>
       </c>
       <c r="BD43" t="n">
-        <v>-51.23</v>
+        <v>-51.58</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-86.23999999999999</v>
+        <v>-86.34</v>
       </c>
       <c r="BG43" t="n">
-        <v>18.84</v>
+        <v>18</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>40.91</v>
+        <v>41.2</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>42.41</v>
+        <v>41.48</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>40.91</v>
+        <v>40.09</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.640000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="BR43" t="n">
-        <v>42.26</v>
+        <v>40.39</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6380221</v>
+        <v>6458960</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>3.95</v>
+        <v>3.98</v>
       </c>
       <c r="G46" t="n">
-        <v>3952136997</v>
+        <v>3972098127</v>
       </c>
       <c r="H46" t="n">
-        <v>15318800</v>
+        <v>37354700</v>
       </c>
       <c r="I46" t="n">
         <v>1000541644</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.06869560877481121</v>
+        <v>0.06904257093179718</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249156.24</v>
       </c>
       <c r="AM46" t="n">
-        <v>3874644114.705882</v>
+        <v>3894213850</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.26</v>
+        <v>3.28</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>2.38</v>
+        <v>1.61</v>
       </c>
       <c r="BD46" t="n">
-        <v>-16.41</v>
+        <v>-17.04</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.29000000000001</v>
+        <v>-89.37</v>
       </c>
       <c r="BG46" t="n">
-        <v>86.8</v>
+        <v>85.39</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>3.95</v>
+        <v>3.98</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4</v>
+        <v>4.08</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>3.91</v>
+        <v>3.89</v>
       </c>
       <c r="BQ46" t="n">
-        <v>8.640000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="BR46" t="n">
-        <v>3.91</v>
+        <v>3.93</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>17409503</v>
+        <v>17474723</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>8.92</v>
+        <v>8.9</v>
       </c>
       <c r="G47" t="n">
-        <v>3111891882</v>
+        <v>3106519946</v>
       </c>
       <c r="H47" t="n">
-        <v>7200</v>
+        <v>10900</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7338199089010266</v>
+        <v>0.7325531445867058</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>551753879.7872341</v>
+        <v>550801408.8652482</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>11.71</v>
+        <v>11.69</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,19 +11304,19 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>61.14</v>
+        <v>61.5</v>
       </c>
       <c r="BD47" t="n">
-        <v>31.57</v>
+        <v>31.86</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-83.65000000000001</v>
+        <v>-83.61</v>
       </c>
       <c r="BG47" t="n">
-        <v>-3.37</v>
+        <v>-3.15</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
@@ -11325,7 +11325,7 @@
         <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>8.92</v>
+        <v>8.9</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11334,7 +11334,7 @@
         <v>1.29</v>
       </c>
       <c r="BM47" t="n">
-        <v>8.960000000000001</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="BN47" t="n">
         <v>9.25</v>
@@ -11346,16 +11346,16 @@
         <v>8.880000000000001</v>
       </c>
       <c r="BQ47" t="n">
-        <v>6.9</v>
+        <v>6.88</v>
       </c>
       <c r="BR47" t="n">
-        <v>8.890000000000001</v>
+        <v>8.93</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>12593</v>
+        <v>12645</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.029999999999999</v>
+        <v>9.02</v>
       </c>
       <c r="G48" t="n">
-        <v>3111891882</v>
+        <v>3106519946</v>
       </c>
       <c r="H48" t="n">
-        <v>3500</v>
+        <v>1400</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>1.996503013721042</v>
+        <v>1.993056529453528</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>544037042.3076923</v>
+        <v>543097892.6573427</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>11.81</v>
+        <v>11.8</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,19 +11534,19 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>59.17</v>
+        <v>59.35</v>
       </c>
       <c r="BD48" t="n">
-        <v>29.97</v>
+        <v>30.11</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-83.84999999999999</v>
+        <v>-83.83</v>
       </c>
       <c r="BG48" t="n">
-        <v>-8.789999999999999</v>
+        <v>-8.69</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
@@ -11555,7 +11555,7 @@
         <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.029999999999999</v>
+        <v>9.02</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11564,7 +11564,7 @@
         <v>1.29</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.06</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="BN48" t="n">
         <v>9.48</v>
@@ -11573,19 +11573,19 @@
         <v>7.21</v>
       </c>
       <c r="BP48" t="n">
-        <v>9</v>
+        <v>8.92</v>
       </c>
       <c r="BQ48" t="n">
-        <v>6.98</v>
+        <v>6.97</v>
       </c>
       <c r="BR48" t="n">
-        <v>9</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2643</v>
+        <v>2689</v>
       </c>
     </row>
     <row r="49">
@@ -11615,13 +11615,13 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>46.37</v>
+        <v>49.9</v>
       </c>
       <c r="G49" t="n">
-        <v>933292214</v>
+        <v>996908218</v>
       </c>
       <c r="H49" t="n">
-        <v>300</v>
+        <v>6900</v>
       </c>
       <c r="I49" t="n">
         <v>11540870</v>
@@ -11636,7 +11636,7 @@
         <v>1.09</v>
       </c>
       <c r="M49" t="n">
-        <v>0.9441996948109511</v>
+        <v>1.00855918550514</v>
       </c>
       <c r="N49" t="n">
         <v>0.08</v>
@@ -11714,7 +11714,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM49" t="n">
-        <v>233323053.5</v>
+        <v>249227054.5</v>
       </c>
       <c r="AN49" t="n">
         <v>3.3186</v>
@@ -11755,7 +11755,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ49" t="n">
-        <v>55.33</v>
+        <v>59.55</v>
       </c>
       <c r="BA49" t="n">
         <v>9.210000000000001</v>
@@ -11764,19 +11764,19 @@
         <v>27.75</v>
       </c>
       <c r="BC49" t="n">
-        <v>80.89</v>
+        <v>68.09</v>
       </c>
       <c r="BD49" t="n">
-        <v>47.69</v>
+        <v>37.25</v>
       </c>
       <c r="BE49" t="n">
         <v>19.33</v>
       </c>
       <c r="BF49" t="n">
-        <v>-80.13</v>
+        <v>-81.54000000000001</v>
       </c>
       <c r="BG49" t="n">
-        <v>-40.15</v>
+        <v>-44.38</v>
       </c>
       <c r="BH49" t="n">
         <v>42.6</v>
@@ -11785,7 +11785,7 @@
         <v>0</v>
       </c>
       <c r="BJ49" t="n">
-        <v>46.37</v>
+        <v>49.9</v>
       </c>
       <c r="BK49" t="n">
         <v>7.34</v>
@@ -11794,7 +11794,7 @@
         <v>7.6</v>
       </c>
       <c r="BM49" t="n">
-        <v>46.37</v>
+        <v>50.68</v>
       </c>
       <c r="BN49" t="n">
         <v>64.2</v>
@@ -11803,19 +11803,19 @@
         <v>27.62</v>
       </c>
       <c r="BP49" t="n">
-        <v>46.37</v>
+        <v>44.13</v>
       </c>
       <c r="BQ49" t="n">
-        <v>6.1</v>
+        <v>6.57</v>
       </c>
       <c r="BR49" t="n">
-        <v>46.37</v>
+        <v>48.88</v>
       </c>
       <c r="BS49" t="n">
         <v>0.54</v>
       </c>
       <c r="BT49" t="n">
-        <v>137</v>
+        <v>143</v>
       </c>
     </row>
     <row r="50">
@@ -12045,7 +12045,7 @@
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>753</v>
+        <v>727</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.56</v>
+        <v>6.58</v>
       </c>
       <c r="G53" t="n">
-        <v>897751736</v>
+        <v>869986533</v>
       </c>
       <c r="H53" t="n">
-        <v>24200</v>
+        <v>89500</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.332191651166572</v>
+        <v>2.260062829764276</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>45733659.50076414</v>
+        <v>44319232.45033113</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-39.93</v>
+        <v>-40.11</v>
       </c>
       <c r="BD53" t="n">
-        <v>-50.95</v>
+        <v>-51.1</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.58</v>
+        <v>-95.59</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6.56</v>
+        <v>6.58</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.09</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.77</v>
+        <v>6.74</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="BQ53" t="n">
+        <v>77.12</v>
+      </c>
+      <c r="BR53" t="n">
         <v>6.53</v>
-      </c>
-      <c r="BQ53" t="n">
-        <v>76.89</v>
-      </c>
-      <c r="BR53" t="n">
-        <v>6.63</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>43210</v>
+        <v>42567</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>9.869999999999999</v>
+        <v>10.02</v>
       </c>
       <c r="G54" t="n">
-        <v>2301802413</v>
+        <v>2405012533</v>
       </c>
       <c r="H54" t="n">
-        <v>268400</v>
+        <v>344400</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.291982314511431</v>
+        <v>1.349913285895204</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>314884051.0259918</v>
+        <v>329003082.4897401</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>15.71</v>
+        <v>15.95</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,19 +12902,19 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>52.05</v>
+        <v>49.78</v>
       </c>
       <c r="BD54" t="n">
-        <v>24.15</v>
+        <v>22.29</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-90.04000000000001</v>
+        <v>-90.19</v>
       </c>
       <c r="BG54" t="n">
-        <v>-33.98</v>
+        <v>-34.97</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
@@ -12923,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>9.869999999999999</v>
+        <v>10.02</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>9.869999999999999</v>
+        <v>10.05</v>
       </c>
       <c r="BN54" t="n">
         <v>11.75</v>
@@ -12941,19 +12941,19 @@
         <v>8.279999999999999</v>
       </c>
       <c r="BP54" t="n">
-        <v>9.449999999999999</v>
+        <v>9.74</v>
       </c>
       <c r="BQ54" t="n">
-        <v>9.84</v>
+        <v>9.99</v>
       </c>
       <c r="BR54" t="n">
-        <v>9.65</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>277237</v>
+        <v>276570</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>51.74</v>
+        <v>51.95</v>
       </c>
       <c r="G55" t="n">
-        <v>6795970408</v>
+        <v>6648812643</v>
       </c>
       <c r="H55" t="n">
-        <v>300</v>
+        <v>1800</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1.049101824430511</v>
+        <v>1.026384909777839</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>341849618.1086519</v>
+        <v>334447316.0462777</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>54.41</v>
+        <v>54.63</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>21.21</v>
+        <v>20.72</v>
       </c>
       <c r="BD55" t="n">
-        <v>-1.03</v>
+        <v>-1.43</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-81.87</v>
+        <v>-81.95</v>
       </c>
       <c r="BG55" t="n">
-        <v>-68.93000000000001</v>
+        <v>-69.05</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>51.74</v>
+        <v>51.95</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>51.74</v>
+        <v>51.95</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>34.46</v>
       </c>
       <c r="BP55" t="n">
-        <v>51.25</v>
+        <v>51.31</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.36</v>
+        <v>7.39</v>
       </c>
       <c r="BR55" t="n">
-        <v>51.25</v>
+        <v>51.31</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>7290</v>
+        <v>7116</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>61.44</v>
+        <v>60.33</v>
       </c>
       <c r="G56" t="n">
-        <v>6795970408</v>
+        <v>6648812643</v>
       </c>
       <c r="H56" t="n">
-        <v>7300</v>
+        <v>24500</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.222509825312177</v>
+        <v>2.174384309904036</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>282694276.5391015</v>
+        <v>276572905.2828619</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>58.68</v>
+        <v>57.62</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>2.07</v>
+        <v>3.95</v>
       </c>
       <c r="BD56" t="n">
-        <v>-16.66</v>
+        <v>-15.12</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-84.73999999999999</v>
+        <v>-84.45999999999999</v>
       </c>
       <c r="BG56" t="n">
-        <v>-71.23</v>
+        <v>-70.7</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>61.44</v>
+        <v>60.33</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>62.2</v>
+        <v>62.59</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>45.75</v>
       </c>
       <c r="BP56" t="n">
-        <v>61.25</v>
+        <v>60.1</v>
       </c>
       <c r="BQ56" t="n">
-        <v>8.74</v>
+        <v>8.58</v>
       </c>
       <c r="BR56" t="n">
-        <v>61.58</v>
+        <v>61.5</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>33983</v>
+        <v>33210</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>5.78</v>
+        <v>6.06</v>
       </c>
       <c r="G57" t="n">
-        <v>1351699289</v>
+        <v>1407439834</v>
       </c>
       <c r="H57" t="n">
-        <v>1265300</v>
+        <v>1683600</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4045999022099153</v>
+        <v>0.4212845444522087</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>101099423.2610322</v>
+        <v>105268499.1772625</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>8.81</v>
+        <v>9.24</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>127.19</v>
+        <v>116.69</v>
       </c>
       <c r="BD57" t="n">
-        <v>85.5</v>
+        <v>76.93000000000001</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-80.48999999999999</v>
+        <v>-81.39</v>
       </c>
       <c r="BG57" t="n">
-        <v>8.369999999999999</v>
+        <v>3.36</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>5.78</v>
+        <v>6.06</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,28 +13622,28 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>5.86</v>
+        <v>6.06</v>
       </c>
       <c r="BN57" t="n">
         <v>6.08</v>
       </c>
       <c r="BO57" t="n">
-        <v>3.38</v>
+        <v>3.39</v>
       </c>
       <c r="BP57" t="n">
-        <v>5.68</v>
+        <v>5.75</v>
       </c>
       <c r="BQ57" t="n">
-        <v>5.58</v>
+        <v>5.85</v>
       </c>
       <c r="BR57" t="n">
-        <v>5.84</v>
+        <v>5.8</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1207036</v>
+        <v>1235809</v>
       </c>
     </row>
     <row r="58">
@@ -13906,10 +13906,10 @@
         <v>20</v>
       </c>
       <c r="G59" t="n">
-        <v>95156610</v>
+        <v>94446470</v>
       </c>
       <c r="H59" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="I59" t="n">
         <v>710143</v>
@@ -13924,7 +13924,7 @@
         <v>0.61</v>
       </c>
       <c r="M59" t="n">
-        <v>10.10787986071049</v>
+        <v>10.03244621711721</v>
       </c>
       <c r="N59" t="n">
         <v>0.15</v>
@@ -14002,7 +14002,7 @@
         <v>1881878.95</v>
       </c>
       <c r="AM59" t="n">
-        <v>16073751.68918919</v>
+        <v>15953795.60810811</v>
       </c>
       <c r="AN59" t="n">
         <v>1.4</v>
@@ -14082,13 +14082,13 @@
         <v>2.65</v>
       </c>
       <c r="BM59" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="BN59" t="n">
         <v>25.98</v>
       </c>
       <c r="BO59" t="n">
-        <v>15.66</v>
+        <v>15.73</v>
       </c>
       <c r="BP59" t="n">
         <v>20</v>
@@ -14097,13 +14097,13 @@
         <v>7.54</v>
       </c>
       <c r="BR59" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="BS59" t="n">
         <v>1.42</v>
       </c>
       <c r="BT59" t="n">
-        <v>107</v>
+        <v>113</v>
       </c>
     </row>
     <row r="60">
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>372.01</v>
+        <v>374.25</v>
       </c>
       <c r="G60" t="n">
-        <v>169171589</v>
+        <v>167937576</v>
       </c>
       <c r="H60" t="n">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.65379671336507</v>
+        <v>12.56149427809238</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-24805218.32844575</v>
+        <v>-24624278.0058651</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2139.06</v>
+        <v>2151.94</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,19 +14282,19 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>211.07</v>
+        <v>209.21</v>
       </c>
       <c r="BD60" t="n">
-        <v>153.99</v>
+        <v>152.47</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-37.88</v>
+        <v>-38.25</v>
       </c>
       <c r="BG60" t="n">
-        <v>95.69</v>
+        <v>94.52</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>372.01</v>
+        <v>374.25</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14312,7 +14312,7 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>372.1</v>
+        <v>376.99</v>
       </c>
       <c r="BN60" t="n">
         <v>405</v>
@@ -14321,19 +14321,19 @@
         <v>306.27</v>
       </c>
       <c r="BP60" t="n">
-        <v>371.5</v>
+        <v>373</v>
       </c>
       <c r="BQ60" t="n">
-        <v>2.84</v>
+        <v>2.86</v>
       </c>
       <c r="BR60" t="n">
-        <v>371.5</v>
+        <v>376.99</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
       </c>
       <c r="BT60" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="61">
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>25.54</v>
+        <v>26.21</v>
       </c>
       <c r="G61" t="n">
-        <v>2186438358</v>
+        <v>2226361194</v>
       </c>
       <c r="H61" t="n">
-        <v>451700</v>
+        <v>711500</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.159543329466421</v>
+        <v>1.180715780090424</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>171619965.3061225</v>
+        <v>174753625.9026687</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>32.18</v>
+        <v>33.02</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-15.8</v>
+        <v>-17.96</v>
       </c>
       <c r="BD61" t="n">
-        <v>-31.25</v>
+        <v>-33.01</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-90.12</v>
+        <v>-90.37</v>
       </c>
       <c r="BG61" t="n">
-        <v>-53.97</v>
+        <v>-55.15</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>25.54</v>
+        <v>26.21</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,28 +14542,28 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>25.84</v>
+        <v>26.41</v>
       </c>
       <c r="BN61" t="n">
         <v>28.25</v>
       </c>
       <c r="BO61" t="n">
-        <v>19.2</v>
+        <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>25.34</v>
+        <v>25.29</v>
       </c>
       <c r="BQ61" t="n">
-        <v>13.72</v>
+        <v>14.08</v>
       </c>
       <c r="BR61" t="n">
-        <v>25.34</v>
+        <v>25.56</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>454761</v>
+        <v>466568</v>
       </c>
     </row>
     <row r="62">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.33</v>
+        <v>1.35</v>
       </c>
       <c r="G63" t="n">
-        <v>346477912</v>
+        <v>349063566</v>
       </c>
       <c r="H63" t="n">
-        <v>10100</v>
+        <v>19700</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.4261499513798583</v>
+        <v>0.4293301723642919</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>196862450</v>
+        <v>198331571.5909091</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-78.26000000000001</v>
+        <v>-78.58</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.33</v>
+        <v>1.35</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.33</v>
+        <v>1.35</v>
       </c>
       <c r="BN63" t="n">
         <v>1.54</v>
@@ -15011,19 +15011,19 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.33</v>
+        <v>1.35</v>
       </c>
       <c r="BQ63" t="n">
-        <v>5.09</v>
+        <v>5.17</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.33</v>
+        <v>1.35</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>14157</v>
+        <v>14493</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>59.06</v>
+        <v>60.45</v>
       </c>
       <c r="G64" t="n">
-        <v>229788350003</v>
+        <v>234216490006</v>
       </c>
       <c r="H64" t="n">
-        <v>12264400</v>
+        <v>11044700</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>65883691899.56499</v>
+        <v>67153304617.71185</v>
       </c>
       <c r="AL64" t="n">
-        <v>18368373301.59872</v>
+        <v>18722341327.41806</v>
       </c>
       <c r="AM64" t="n">
-        <v>20462008014.51469</v>
+        <v>20856321460.90828</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>23.62</v>
+        <v>24.18</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,19 +15202,19 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-19.17</v>
+        <v>-21.03</v>
       </c>
       <c r="BD64" t="n">
-        <v>-34</v>
+        <v>-35.52</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-88.67</v>
+        <v>-88.93000000000001</v>
       </c>
       <c r="BG64" t="n">
-        <v>-82.40000000000001</v>
+        <v>-82.8</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
@@ -15223,7 +15223,7 @@
         <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>59.06</v>
+        <v>60.45</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>59.84</v>
+        <v>61.1</v>
       </c>
       <c r="BN64" t="n">
         <v>64.72</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>58.28</v>
+        <v>58.39</v>
       </c>
       <c r="BQ64" t="n">
-        <v>37.62</v>
+        <v>38.5</v>
       </c>
       <c r="BR64" t="n">
-        <v>59.84</v>
+        <v>58.71</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>11895563</v>
+        <v>12088805</v>
       </c>
     </row>
     <row r="65">
@@ -15286,10 +15286,10 @@
         <v>23.8</v>
       </c>
       <c r="G65" t="n">
-        <v>229788350003</v>
+        <v>234216490006</v>
       </c>
       <c r="H65" t="n">
-        <v>5300</v>
+        <v>6000</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.555350024599269</v>
+        <v>5.662404484384867</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>17212610487.1161</v>
+        <v>17544306367.49064</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>23.83</v>
+        <v>23.8</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15477,13 +15477,13 @@
         <v>15.16</v>
       </c>
       <c r="BR65" t="n">
-        <v>23.6</v>
+        <v>23.8</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>13771</v>
+        <v>11985</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>20.45</v>
+        <v>20.01</v>
       </c>
       <c r="G66" t="n">
-        <v>229788350003</v>
+        <v>234216490006</v>
       </c>
       <c r="H66" t="n">
-        <v>1400</v>
+        <v>4500</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>13.64152660569233</v>
+        <v>13.90440585811686</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>20608820628.07175</v>
+        <v>21005963229.23767</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>8.210000000000001</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-22.2</v>
+        <v>-20.49</v>
       </c>
       <c r="BD66" t="n">
-        <v>-36.48</v>
+        <v>-35.08</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-89.09</v>
+        <v>-88.84999999999999</v>
       </c>
       <c r="BG66" t="n">
-        <v>-83.05</v>
+        <v>-82.68000000000001</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>20.45</v>
+        <v>20.01</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>20.92</v>
+        <v>20.59</v>
       </c>
       <c r="BN66" t="n">
         <v>21.16</v>
@@ -15701,19 +15701,19 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>20.03</v>
+        <v>19.97</v>
       </c>
       <c r="BQ66" t="n">
-        <v>13.02</v>
+        <v>12.74</v>
       </c>
       <c r="BR66" t="n">
-        <v>20.77</v>
+        <v>20.05</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>7052</v>
+        <v>6961</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>19.49</v>
+        <v>19.21</v>
       </c>
       <c r="G68" t="n">
-        <v>8388023022</v>
+        <v>8255366240</v>
       </c>
       <c r="H68" t="n">
-        <v>26700</v>
+        <v>25700</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>581693690.8460472</v>
+        <v>572494191.4008322</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>36.06</v>
+        <v>35.54</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,19 +16122,19 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>34.44</v>
+        <v>36.4</v>
       </c>
       <c r="BD68" t="n">
-        <v>9.77</v>
+        <v>11.37</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.64</v>
+        <v>-93.55</v>
       </c>
       <c r="BG68" t="n">
-        <v>224.52</v>
+        <v>229.25</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>19.49</v>
+        <v>19.21</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>19.49</v>
+        <v>19.39</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,19 +16161,19 @@
         <v>15.07</v>
       </c>
       <c r="BP68" t="n">
-        <v>19.22</v>
+        <v>19</v>
       </c>
       <c r="BQ68" t="n">
-        <v>13.11</v>
+        <v>12.92</v>
       </c>
       <c r="BR68" t="n">
-        <v>19.38</v>
+        <v>19.39</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>31923</v>
+        <v>32260</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>22.57</v>
+        <v>22.38</v>
       </c>
       <c r="G69" t="n">
-        <v>8388023022</v>
+        <v>8255366240</v>
       </c>
       <c r="H69" t="n">
-        <v>2330400</v>
+        <v>2726600</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>499287084.6428571</v>
+        <v>491390847.6190476</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>39.46</v>
+        <v>39.13</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>16.1</v>
+        <v>17.08</v>
       </c>
       <c r="BD69" t="n">
-        <v>-5.21</v>
+        <v>-4.4</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-94.51000000000001</v>
+        <v>-94.45999999999999</v>
       </c>
       <c r="BG69" t="n">
-        <v>208.32</v>
+        <v>210.93</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>22.57</v>
+        <v>22.38</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,7 +16382,7 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>23.05</v>
+        <v>22.59</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
@@ -16391,19 +16391,19 @@
         <v>16.6</v>
       </c>
       <c r="BP69" t="n">
-        <v>22.54</v>
+        <v>22.14</v>
       </c>
       <c r="BQ69" t="n">
-        <v>15.18</v>
+        <v>15.05</v>
       </c>
       <c r="BR69" t="n">
-        <v>22.68</v>
+        <v>22.24</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>1822340</v>
+        <v>1859817</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>18.42</v>
+        <v>18.81</v>
       </c>
       <c r="G70" t="n">
-        <v>8557143659</v>
+        <v>8819719075</v>
       </c>
       <c r="H70" t="n">
-        <v>2672000</v>
+        <v>3735000</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6753999039001869</v>
+        <v>0.6961245075529993</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2824139821.452146</v>
+        <v>2910798374.587459</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.12</v>
+        <v>2.16</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,19 +16582,19 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-54.13</v>
+        <v>-55.08</v>
       </c>
       <c r="BD70" t="n">
-        <v>-62.55</v>
+        <v>-63.32</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
       </c>
       <c r="BF70" t="n">
-        <v>-99.34999999999999</v>
+        <v>-99.36</v>
       </c>
       <c r="BG70" t="n">
-        <v>-94.19</v>
+        <v>-94.31</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>18.42</v>
+        <v>18.81</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>18.61</v>
+        <v>19.04</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>18.28</v>
+        <v>18.53</v>
       </c>
       <c r="BQ70" t="n">
-        <v>184.74</v>
+        <v>188.65</v>
       </c>
       <c r="BR70" t="n">
-        <v>18.33</v>
+        <v>18.53</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>6559547</v>
+        <v>6219960</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-09-12 05:18
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>25</v>
+        <v>25.1</v>
       </c>
       <c r="G3" t="n">
-        <v>3352330000</v>
+        <v>3357546731</v>
       </c>
       <c r="H3" t="n">
-        <v>478900</v>
+        <v>398500</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8341343651602502</v>
+        <v>0.8354324040170742</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>654751953.125</v>
+        <v>655770845.8984375</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>45.75</v>
+        <v>45.93</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>97.98999999999999</v>
+        <v>97.20999999999999</v>
       </c>
       <c r="BD3" t="n">
-        <v>61.66</v>
+        <v>61.02</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-80.53</v>
+        <v>-80.59999999999999</v>
       </c>
       <c r="BG3" t="n">
-        <v>-15.46</v>
+        <v>-15.79</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>25</v>
+        <v>25.1</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>25.18</v>
+        <v>25.32</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>24.49</v>
+        <v>24.96</v>
       </c>
       <c r="BQ3" t="n">
-        <v>5.69</v>
+        <v>5.71</v>
       </c>
       <c r="BR3" t="n">
-        <v>24.63</v>
+        <v>25</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>523503</v>
+        <v>529000</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.74</v>
+        <v>15.62</v>
       </c>
       <c r="G4" t="n">
-        <v>240031061509</v>
+        <v>241870387427</v>
       </c>
       <c r="H4" t="n">
-        <v>21311000</v>
+        <v>22932100</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.717879038364467</v>
+        <v>2.738705781894346</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>23765451634.55445</v>
+        <v>23947563111.58416</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.65</v>
+        <v>19.5</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-26.27</v>
+        <v>-25.71</v>
       </c>
       <c r="BD4" t="n">
-        <v>-39.8</v>
+        <v>-39.34</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.84</v>
+        <v>-92.78</v>
       </c>
       <c r="BG4" t="n">
-        <v>-27.66</v>
+        <v>-27.1</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.74</v>
+        <v>15.62</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.79</v>
+        <v>15.78</v>
       </c>
       <c r="BN4" t="n">
         <v>17</v>
@@ -1465,19 +1465,19 @@
         <v>11.09</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.47</v>
+        <v>15.59</v>
       </c>
       <c r="BQ4" t="n">
-        <v>15.18</v>
+        <v>15.06</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.56</v>
+        <v>15.78</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>31103410</v>
+        <v>30552467</v>
       </c>
     </row>
     <row r="5">
@@ -1737,13 +1737,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7.29</v>
+        <v>7.37</v>
       </c>
       <c r="G6" t="n">
-        <v>453664352</v>
+        <v>464934231</v>
       </c>
       <c r="H6" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="I6" t="n">
         <v>63084700</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>7.062665714607753</v>
+        <v>7.238115664929348</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>43371352.96367113</v>
+        <v>44448779.2543021</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -1877,7 +1877,7 @@
         <v>5.74</v>
       </c>
       <c r="AZ6" t="n">
-        <v>8.550000000000001</v>
+        <v>8.65</v>
       </c>
       <c r="BA6" t="n">
         <v>0.65</v>
@@ -1886,19 +1886,19 @@
         <v>7.95</v>
       </c>
       <c r="BC6" t="n">
-        <v>-3.49</v>
+        <v>-4.53</v>
       </c>
       <c r="BD6" t="n">
-        <v>-21.2</v>
+        <v>-22.05</v>
       </c>
       <c r="BE6" t="n">
         <v>17.33</v>
       </c>
       <c r="BF6" t="n">
-        <v>-91.09999999999999</v>
+        <v>-91.2</v>
       </c>
       <c r="BG6" t="n">
-        <v>9.1</v>
+        <v>7.92</v>
       </c>
       <c r="BH6" t="n">
         <v>3.86</v>
@@ -1907,7 +1907,7 @@
         <v>0</v>
       </c>
       <c r="BJ6" t="n">
-        <v>7.29</v>
+        <v>7.37</v>
       </c>
       <c r="BK6" t="n">
         <v>0.57</v>
@@ -1916,19 +1916,19 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>7.35</v>
+        <v>7.37</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
       </c>
       <c r="BO6" t="n">
-        <v>5.96</v>
+        <v>6.22</v>
       </c>
       <c r="BP6" t="n">
-        <v>7.29</v>
+        <v>7.35</v>
       </c>
       <c r="BQ6" t="n">
-        <v>12.96</v>
+        <v>13.11</v>
       </c>
       <c r="BR6" t="n">
         <v>7.35</v>
@@ -1937,7 +1937,7 @@
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>287</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5.1</v>
+        <v>5.07</v>
       </c>
       <c r="G12" t="n">
-        <v>479992152</v>
+        <v>486524922</v>
       </c>
       <c r="H12" t="n">
-        <v>634500</v>
+        <v>449000</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.08680584825219441</v>
+        <v>0.08798728973810956</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>516120593.5483871</v>
+        <v>523145077.4193548</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>6.89</v>
+        <v>6.85</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,19 +3266,19 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>632.3</v>
+        <v>636.63</v>
       </c>
       <c r="BD12" t="n">
-        <v>497.92</v>
+        <v>501.46</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-13.5</v>
+        <v>-12.99</v>
       </c>
       <c r="BG12" t="n">
-        <v>255.27</v>
+        <v>257.37</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
@@ -3287,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>5.1</v>
+        <v>5.07</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.43</v>
       </c>
       <c r="BM12" t="n">
-        <v>5.21</v>
+        <v>5.1</v>
       </c>
       <c r="BN12" t="n">
         <v>8.23</v>
@@ -3305,19 +3305,19 @@
         <v>4.42</v>
       </c>
       <c r="BP12" t="n">
-        <v>5.01</v>
+        <v>5.04</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.49</v>
+        <v>1.48</v>
       </c>
       <c r="BR12" t="n">
-        <v>5.11</v>
+        <v>5.1</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>466910</v>
+        <v>482027</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>29.07</v>
+        <v>28.63</v>
       </c>
       <c r="G13" t="n">
-        <v>14305710224</v>
+        <v>14434985043</v>
       </c>
       <c r="H13" t="n">
-        <v>3944100</v>
+        <v>3688300</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>4.947741654734844</v>
+        <v>4.992452360939528</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1488627494.693028</v>
+        <v>1502079609.05307</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>52.62</v>
+        <v>51.82</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>12.05</v>
+        <v>13.77</v>
       </c>
       <c r="BD13" t="n">
-        <v>-8.51</v>
+        <v>-7.1</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-91.04000000000001</v>
+        <v>-90.90000000000001</v>
       </c>
       <c r="BG13" t="n">
-        <v>-70.09</v>
+        <v>-69.63</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>29.07</v>
+        <v>28.63</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>29.22</v>
+        <v>29.21</v>
       </c>
       <c r="BN13" t="n">
         <v>32.43</v>
@@ -3535,19 +3535,19 @@
         <v>21.06</v>
       </c>
       <c r="BP13" t="n">
-        <v>28.2</v>
+        <v>28.47</v>
       </c>
       <c r="BQ13" t="n">
-        <v>14.85</v>
+        <v>14.63</v>
       </c>
       <c r="BR13" t="n">
-        <v>28.46</v>
+        <v>29.08</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>4522623</v>
+        <v>4550534</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>9.94</v>
+        <v>10</v>
       </c>
       <c r="G14" t="n">
-        <v>8082747775</v>
+        <v>7974653792</v>
       </c>
       <c r="H14" t="n">
-        <v>6000</v>
+        <v>2700</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.35610056871256</v>
+        <v>3.311218025310331</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>897086323.5294118</v>
+        <v>885089211.0987792</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>7.99</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>11.5</v>
+        <v>10.83</v>
       </c>
       <c r="BD14" t="n">
-        <v>-8.960000000000001</v>
+        <v>-9.51</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-85.7</v>
+        <v>-85.79000000000001</v>
       </c>
       <c r="BG14" t="n">
-        <v>-40.22</v>
+        <v>-40.58</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>9.94</v>
+        <v>10</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>9.94</v>
+        <v>10</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,19 +3765,19 @@
         <v>7.65</v>
       </c>
       <c r="BP14" t="n">
-        <v>9.75</v>
+        <v>9.77</v>
       </c>
       <c r="BQ14" t="n">
-        <v>9.81</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="BR14" t="n">
-        <v>9.75</v>
+        <v>9.77</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>12320</v>
+        <v>12497</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>13.25</v>
+        <v>13.33</v>
       </c>
       <c r="G15" t="n">
-        <v>8082747775</v>
+        <v>7974653792</v>
       </c>
       <c r="H15" t="n">
-        <v>1838000</v>
+        <v>1699500</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.316626203024084</v>
+        <v>3.272271566904433</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>674124084.6538782</v>
+        <v>665108739.9499583</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>8.81</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-16.36</v>
+        <v>-16.86</v>
       </c>
       <c r="BD15" t="n">
-        <v>-31.71</v>
+        <v>-32.12</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-89.27</v>
+        <v>-89.34</v>
       </c>
       <c r="BG15" t="n">
-        <v>-53.3</v>
+        <v>-53.58</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>13.25</v>
+        <v>13.33</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>13.33</v>
+        <v>13.41</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>13.05</v>
+        <v>13.16</v>
       </c>
       <c r="BQ15" t="n">
-        <v>13.08</v>
+        <v>13.16</v>
       </c>
       <c r="BR15" t="n">
-        <v>13.17</v>
+        <v>13.3</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2318043</v>
+        <v>2338760</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.4</v>
+        <v>4.35</v>
       </c>
       <c r="G16" t="n">
-        <v>953904620</v>
+        <v>953979774</v>
       </c>
       <c r="H16" t="n">
-        <v>111500</v>
+        <v>47600</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4512768680105594</v>
+        <v>0.4513124221540528</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>267950735.9550562</v>
+        <v>267971846.6292135</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-60.48</v>
+        <v>-60.02</v>
       </c>
       <c r="BD16" t="n">
-        <v>-67.73</v>
+        <v>-67.36</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.18000000000001</v>
+        <v>-98.16</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>4.4</v>
+        <v>4.35</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,28 +4216,28 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.49</v>
+        <v>4.44</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
       </c>
       <c r="BO16" t="n">
-        <v>2.97</v>
+        <v>2.98</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.31</v>
+        <v>4.33</v>
       </c>
       <c r="BQ16" t="n">
-        <v>60.04</v>
+        <v>59.36</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.31</v>
+        <v>4.44</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>141257</v>
+        <v>141910</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>33.99</v>
+        <v>33.74</v>
       </c>
       <c r="G17" t="n">
-        <v>11032206223</v>
+        <v>11121612159</v>
       </c>
       <c r="H17" t="n">
-        <v>638700</v>
+        <v>541900</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>4982029544.346099</v>
+        <v>5022404334.808526</v>
       </c>
       <c r="AL17" t="n">
-        <v>1379025777.875</v>
+        <v>1390201519.875</v>
       </c>
       <c r="AM17" t="n">
-        <v>3415543722.291022</v>
+        <v>3443223578.637771</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>18.18</v>
+        <v>18.05</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>54.86</v>
+        <v>56.01</v>
       </c>
       <c r="BD17" t="n">
-        <v>26.44</v>
+        <v>27.38</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-86.62</v>
+        <v>-86.52</v>
       </c>
       <c r="BG17" t="n">
-        <v>-51.95</v>
+        <v>-51.59</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>33.99</v>
+        <v>33.74</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,7 +4446,7 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>33.99</v>
+        <v>34.02</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
@@ -4455,19 +4455,19 @@
         <v>29.28</v>
       </c>
       <c r="BP17" t="n">
-        <v>33.07</v>
+        <v>33.54</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.69</v>
+        <v>2.67</v>
       </c>
       <c r="BR17" t="n">
-        <v>33.39</v>
+        <v>33.92</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1071150</v>
+        <v>1076424</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>11.74</v>
+        <v>11.8</v>
       </c>
       <c r="G18" t="n">
-        <v>11032206223</v>
+        <v>11121612159</v>
       </c>
       <c r="H18" t="n">
-        <v>4300</v>
+        <v>2900</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.248314758138777</v>
+        <v>3.274639376760259</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3283394709.226191</v>
+        <v>3310003618.75</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>6.05</v>
+        <v>6.08</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>49.28</v>
+        <v>48.52</v>
       </c>
       <c r="BD18" t="n">
-        <v>21.88</v>
+        <v>21.26</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-87.12</v>
+        <v>-87.18000000000001</v>
       </c>
       <c r="BG18" t="n">
-        <v>-53.62</v>
+        <v>-53.86</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>11.74</v>
+        <v>11.8</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>11.95</v>
+        <v>11.91</v>
       </c>
       <c r="BN18" t="n">
         <v>13.82</v>
@@ -4685,19 +4685,19 @@
         <v>10.11</v>
       </c>
       <c r="BP18" t="n">
-        <v>11.58</v>
+        <v>11.7</v>
       </c>
       <c r="BQ18" t="n">
         <v>0.93</v>
       </c>
       <c r="BR18" t="n">
-        <v>11.58</v>
+        <v>11.74</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>9678</v>
+        <v>9650</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>11.05</v>
+        <v>10.96</v>
       </c>
       <c r="G19" t="n">
-        <v>11032206223</v>
+        <v>11121612159</v>
       </c>
       <c r="H19" t="n">
-        <v>9300</v>
+        <v>7900</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.872459886159439</v>
+        <v>6.928154884632505</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3502287689.84127</v>
+        <v>3530670526.666667</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>6.08</v>
+        <v>6.03</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>58.6</v>
+        <v>59.9</v>
       </c>
       <c r="BD19" t="n">
-        <v>29.49</v>
+        <v>30.56</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-86.31</v>
+        <v>-86.2</v>
       </c>
       <c r="BG19" t="n">
-        <v>-52.49</v>
+        <v>-52.1</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>11.05</v>
+        <v>10.96</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>11.09</v>
+        <v>11.13</v>
       </c>
       <c r="BN19" t="n">
         <v>11.41</v>
@@ -4915,19 +4915,19 @@
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>10.83</v>
+        <v>10.95</v>
       </c>
       <c r="BQ19" t="n">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="BR19" t="n">
-        <v>10.86</v>
+        <v>11.01</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>13927</v>
+        <v>13908</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5.27</v>
+        <v>4.91</v>
       </c>
       <c r="G22" t="n">
-        <v>1026087441</v>
+        <v>983204392</v>
       </c>
       <c r="H22" t="n">
-        <v>1203200</v>
+        <v>1773300</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.08702925602643938</v>
+        <v>0.0833920612791982</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>232672889.1156462</v>
+        <v>222948841.723356</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,19 +5566,19 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>463.66</v>
+        <v>504.99</v>
       </c>
       <c r="BD22" t="n">
-        <v>360.23</v>
+        <v>393.97</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-64.14</v>
+        <v>-61.51</v>
       </c>
       <c r="BG22" t="n">
-        <v>3173.05</v>
+        <v>3413.03</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
@@ -5587,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>5.27</v>
+        <v>4.91</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>5.29</v>
+        <v>5.36</v>
       </c>
       <c r="BN22" t="n">
         <v>8.82</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>5.04</v>
+        <v>4.89</v>
       </c>
       <c r="BQ22" t="n">
-        <v>7.85</v>
+        <v>7.31</v>
       </c>
       <c r="BR22" t="n">
-        <v>5.17</v>
+        <v>5.34</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1567963</v>
+        <v>1550707</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.9</v>
+        <v>2.93</v>
       </c>
       <c r="G24" t="n">
-        <v>1117458196</v>
+        <v>1183335024</v>
       </c>
       <c r="H24" t="n">
-        <v>5255800</v>
+        <v>4187500</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2701352685141352</v>
+        <v>0.2860603873994232</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1006719095.495495</v>
+        <v>1066067589.189189</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>1.34</v>
+        <v>1.35</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,19 +6026,19 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>146.77</v>
+        <v>144.25</v>
       </c>
       <c r="BD24" t="n">
-        <v>101.49</v>
+        <v>99.43000000000001</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-86.90000000000001</v>
+        <v>-87.03</v>
       </c>
       <c r="BG24" t="n">
-        <v>-49.73</v>
+        <v>-50.25</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
@@ -6047,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>2.9</v>
+        <v>2.93</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>2.97</v>
+        <v>2.95</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.82</v>
+        <v>2.86</v>
       </c>
       <c r="BQ24" t="n">
-        <v>7.12</v>
+        <v>7.2</v>
       </c>
       <c r="BR24" t="n">
-        <v>2.88</v>
+        <v>2.89</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>9434990</v>
+        <v>9270327</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>3.85</v>
+        <v>3.79</v>
       </c>
       <c r="G25" t="n">
-        <v>1262941648</v>
+        <v>1313212246</v>
       </c>
       <c r="H25" t="n">
-        <v>2418000</v>
+        <v>820800</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.6297603719478212</v>
+        <v>0.6548275874796344</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>464316782.3529412</v>
+        <v>482798619.8529412</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>8.970000000000001</v>
+        <v>8.83</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,19 +6256,19 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>4.15</v>
+        <v>5.8</v>
       </c>
       <c r="BD25" t="n">
-        <v>-14.96</v>
+        <v>-13.62</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-93.98</v>
+        <v>-93.89</v>
       </c>
       <c r="BG25" t="n">
-        <v>-42.86</v>
+        <v>-41.96</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>3.85</v>
+        <v>3.79</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>4.05</v>
+        <v>3.96</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>3.79</v>
+        <v>3.74</v>
       </c>
       <c r="BQ25" t="n">
-        <v>16.27</v>
+        <v>16.02</v>
       </c>
       <c r="BR25" t="n">
-        <v>3.92</v>
+        <v>3.86</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1130520</v>
+        <v>1171030</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>9.859999999999999</v>
+        <v>9.82</v>
       </c>
       <c r="G26" t="n">
-        <v>13456700751</v>
+        <v>13300138846</v>
       </c>
       <c r="H26" t="n">
-        <v>15999900</v>
+        <v>6420300</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1735230218027824</v>
+        <v>0.1715041692357606</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>4805964553.928572</v>
+        <v>4750049587.857143</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>1.89</v>
+        <v>1.88</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-12.21</v>
+        <v>-11.86</v>
       </c>
       <c r="BD26" t="n">
-        <v>-28.32</v>
+        <v>-28.03</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-93.31</v>
+        <v>-93.29000000000001</v>
       </c>
       <c r="BG26" t="n">
-        <v>-87.90000000000001</v>
+        <v>-87.84999999999999</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>9.859999999999999</v>
+        <v>9.82</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,7 +6516,7 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>9.92</v>
+        <v>10</v>
       </c>
       <c r="BN26" t="n">
         <v>10.6</v>
@@ -6525,19 +6525,19 @@
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>9.09</v>
+        <v>9.710000000000001</v>
       </c>
       <c r="BQ26" t="n">
-        <v>13.75</v>
+        <v>13.69</v>
       </c>
       <c r="BR26" t="n">
-        <v>9.109999999999999</v>
+        <v>9.85</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>11381943</v>
+        <v>11610410</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>17</v>
+        <v>16.43</v>
       </c>
       <c r="G34" t="n">
-        <v>3425913100</v>
+        <v>3392627477</v>
       </c>
       <c r="H34" t="n">
-        <v>2287300</v>
+        <v>2144200</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.3011777741362306</v>
+        <v>0.2982515791180681</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>712248045.7380458</v>
+        <v>705327957.7962579</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>39.67</v>
+        <v>38.34</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>118.17</v>
+        <v>125.74</v>
       </c>
       <c r="BD34" t="n">
-        <v>78.13</v>
+        <v>84.31</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-86.5</v>
+        <v>-86.03</v>
       </c>
       <c r="BG34" t="n">
-        <v>48.58</v>
+        <v>53.73</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>17</v>
+        <v>16.43</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>17.05</v>
+        <v>17.32</v>
       </c>
       <c r="BN34" t="n">
         <v>31.12</v>
@@ -8353,19 +8353,19 @@
         <v>14.32</v>
       </c>
       <c r="BP34" t="n">
-        <v>16.4</v>
+        <v>16.35</v>
       </c>
       <c r="BQ34" t="n">
-        <v>10.78</v>
+        <v>10.42</v>
       </c>
       <c r="BR34" t="n">
-        <v>16.5</v>
+        <v>17.01</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>3143817</v>
+        <v>3122953</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>17.66</v>
+        <v>17.28</v>
       </c>
       <c r="G35" t="n">
-        <v>87352893445</v>
+        <v>87203523465</v>
       </c>
       <c r="H35" t="n">
-        <v>83504800</v>
+        <v>32548400</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.252068962221995</v>
+        <v>7.23966821219386</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7219247392.148761</v>
+        <v>7206902765.702479</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.3</v>
+        <v>10.08</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,19 +8544,19 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-46.74</v>
+        <v>-45.56</v>
       </c>
       <c r="BD35" t="n">
-        <v>-56.51</v>
+        <v>-55.55</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-93.69</v>
+        <v>-93.55</v>
       </c>
       <c r="BG35" t="n">
-        <v>-48.38</v>
+        <v>-47.24</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
@@ -8565,7 +8565,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>17.66</v>
+        <v>17.28</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>17.81</v>
+        <v>17.83</v>
       </c>
       <c r="BN35" t="n">
         <v>20.08</v>
@@ -8583,19 +8583,19 @@
         <v>11.7</v>
       </c>
       <c r="BP35" t="n">
-        <v>16.98</v>
+        <v>17.2</v>
       </c>
       <c r="BQ35" t="n">
-        <v>16.9</v>
+        <v>16.54</v>
       </c>
       <c r="BR35" t="n">
-        <v>17.15</v>
+        <v>17.8</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>36094857</v>
+        <v>37151143</v>
       </c>
     </row>
     <row r="36">
@@ -9055,7 +9055,7 @@
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>843</v>
+        <v>850</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>67.42</v>
+        <v>69.75</v>
       </c>
       <c r="G39" t="n">
-        <v>3715273387</v>
+        <v>3910067820</v>
       </c>
       <c r="H39" t="n">
-        <v>4300</v>
+        <v>2700</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1864904274828428</v>
+        <v>0.1962682535799908</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>390259809.5588235</v>
+        <v>410721409.6638656</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>196.98</v>
+        <v>203.79</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>209.26</v>
+        <v>198.93</v>
       </c>
       <c r="BD39" t="n">
-        <v>152.51</v>
+        <v>144.08</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-71.8</v>
+        <v>-72.75</v>
       </c>
       <c r="BG39" t="n">
-        <v>36.05</v>
+        <v>31.5</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>67.42</v>
+        <v>69.75</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>68.22</v>
+        <v>69.75</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.47</v>
+        <v>4.62</v>
       </c>
       <c r="BR39" t="n">
-        <v>67.56</v>
+        <v>68</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>4017</v>
+        <v>3933</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>22.8</v>
+        <v>22.49</v>
       </c>
       <c r="G40" t="n">
-        <v>128234742508</v>
+        <v>128886432858</v>
       </c>
       <c r="H40" t="n">
-        <v>32524900</v>
+        <v>22391900</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.3890800785664746</v>
+        <v>0.3910573877388558</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6651179590.6639</v>
+        <v>6684980957.365145</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>11.51</v>
+        <v>11.36</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>94.06999999999999</v>
+        <v>96.75</v>
       </c>
       <c r="BD40" t="n">
-        <v>58.46</v>
+        <v>60.64</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-87.90000000000001</v>
+        <v>-87.73</v>
       </c>
       <c r="BG40" t="n">
-        <v>22.33</v>
+        <v>24.01</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>22.8</v>
+        <v>22.49</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>22.91</v>
+        <v>22.97</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>21.91</v>
+        <v>22.29</v>
       </c>
       <c r="BQ40" t="n">
-        <v>9.119999999999999</v>
+        <v>9</v>
       </c>
       <c r="BR40" t="n">
-        <v>22</v>
+        <v>22.8</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>30359901</v>
+        <v>30950360</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>16.24</v>
+        <v>16.32</v>
       </c>
       <c r="G41" t="n">
-        <v>190888600871</v>
+        <v>195515865004</v>
       </c>
       <c r="H41" t="n">
-        <v>8101200</v>
+        <v>5176200</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.272075615063473</v>
+        <v>1.302911557289405</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>29412727406.93374</v>
+        <v>30125711094.60709</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>24.31</v>
+        <v>24.43</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,19 +9924,19 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>84.02</v>
+        <v>83.12</v>
       </c>
       <c r="BD41" t="n">
-        <v>50.25</v>
+        <v>49.52</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-84.44</v>
+        <v>-84.51000000000001</v>
       </c>
       <c r="BG41" t="n">
-        <v>-15.21</v>
+        <v>-15.62</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
@@ -9945,7 +9945,7 @@
         <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>16.24</v>
+        <v>16.32</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,7 +9954,7 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>16.33</v>
+        <v>16.38</v>
       </c>
       <c r="BN41" t="n">
         <v>18.28</v>
@@ -9963,19 +9963,19 @@
         <v>13.34</v>
       </c>
       <c r="BP41" t="n">
-        <v>15.64</v>
+        <v>16.17</v>
       </c>
       <c r="BQ41" t="n">
-        <v>6.95</v>
+        <v>6.98</v>
       </c>
       <c r="BR41" t="n">
-        <v>15.77</v>
+        <v>16.25</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>7367271</v>
+        <v>7409959</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>18.48</v>
+        <v>18.59</v>
       </c>
       <c r="G42" t="n">
-        <v>190888600871</v>
+        <v>195515865004</v>
       </c>
       <c r="H42" t="n">
-        <v>51431900</v>
+        <v>34171600</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.275859393843789</v>
+        <v>1.306787057334152</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>25971238213.7415</v>
+        <v>26600797959.72789</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>26.77</v>
+        <v>26.92</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,19 +10154,19 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>61.72</v>
+        <v>60.76</v>
       </c>
       <c r="BD42" t="n">
-        <v>32.04</v>
+        <v>31.26</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-86.31999999999999</v>
+        <v>-86.41</v>
       </c>
       <c r="BG42" t="n">
-        <v>-18.21</v>
+        <v>-18.69</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
@@ -10175,7 +10175,7 @@
         <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>18.48</v>
+        <v>18.59</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>18.55</v>
+        <v>18.59</v>
       </c>
       <c r="BN42" t="n">
         <v>21.33</v>
@@ -10193,19 +10193,19 @@
         <v>15.64</v>
       </c>
       <c r="BP42" t="n">
-        <v>17.66</v>
+        <v>18.37</v>
       </c>
       <c r="BQ42" t="n">
-        <v>7.91</v>
+        <v>7.95</v>
       </c>
       <c r="BR42" t="n">
-        <v>17.75</v>
+        <v>18.5</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>39887876</v>
+        <v>40850208</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>41.2</v>
+        <v>39.5</v>
       </c>
       <c r="G43" t="n">
-        <v>77265945830</v>
+        <v>76685260500</v>
       </c>
       <c r="H43" t="n">
-        <v>5918300</v>
+        <v>9254800</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9411199248.477465</v>
+        <v>9340470219.244822</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>74.78</v>
+        <v>71.69</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-40.69</v>
+        <v>-38.14</v>
       </c>
       <c r="BD43" t="n">
-        <v>-51.58</v>
+        <v>-49.49</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-86.34</v>
+        <v>-85.75</v>
       </c>
       <c r="BG43" t="n">
-        <v>18</v>
+        <v>23.08</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>41.2</v>
+        <v>39.5</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>41.48</v>
+        <v>41.25</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>40.09</v>
+        <v>39.47</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.699999999999999</v>
+        <v>8.34</v>
       </c>
       <c r="BR43" t="n">
-        <v>40.39</v>
+        <v>41.03</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6458960</v>
+        <v>6532688</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>3.98</v>
+        <v>4.13</v>
       </c>
       <c r="G46" t="n">
-        <v>3972098127</v>
+        <v>4132234444</v>
       </c>
       <c r="H46" t="n">
-        <v>37354700</v>
+        <v>41219100</v>
       </c>
       <c r="I46" t="n">
         <v>1000541644</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.06904257093179718</v>
+        <v>0.07182604270709787</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249156.24</v>
       </c>
       <c r="AM46" t="n">
-        <v>3894213850</v>
+        <v>4051210239.215686</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.28</v>
+        <v>3.41</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>1.61</v>
+        <v>-2.09</v>
       </c>
       <c r="BD46" t="n">
-        <v>-17.04</v>
+        <v>-20.05</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.37</v>
+        <v>-89.76000000000001</v>
       </c>
       <c r="BG46" t="n">
-        <v>85.39</v>
+        <v>78.66</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>3.98</v>
+        <v>4.13</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.08</v>
+        <v>4.16</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>3.89</v>
+        <v>3.85</v>
       </c>
       <c r="BQ46" t="n">
-        <v>8.699999999999999</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="BR46" t="n">
-        <v>3.93</v>
+        <v>3.99</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>17474723</v>
+        <v>18378000</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>8.9</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="G47" t="n">
-        <v>3106519946</v>
+        <v>3149333408</v>
       </c>
       <c r="H47" t="n">
-        <v>10900</v>
+        <v>8000</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7325531445867058</v>
+        <v>0.7426490515063208</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>550801408.8652482</v>
+        <v>558392448.2269504</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>11.69</v>
+        <v>11.86</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,19 +11304,19 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>61.5</v>
+        <v>59.17</v>
       </c>
       <c r="BD47" t="n">
-        <v>31.86</v>
+        <v>29.97</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-83.61</v>
+        <v>-83.84999999999999</v>
       </c>
       <c r="BG47" t="n">
-        <v>-3.15</v>
+        <v>-4.54</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
@@ -11325,7 +11325,7 @@
         <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>8.9</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11334,7 +11334,7 @@
         <v>1.29</v>
       </c>
       <c r="BM47" t="n">
-        <v>8.949999999999999</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="BN47" t="n">
         <v>9.25</v>
@@ -11343,19 +11343,19 @@
         <v>7.2</v>
       </c>
       <c r="BP47" t="n">
-        <v>8.880000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="BQ47" t="n">
-        <v>6.88</v>
+        <v>6.98</v>
       </c>
       <c r="BR47" t="n">
-        <v>8.93</v>
+        <v>8.9</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>12645</v>
+        <v>12707</v>
       </c>
     </row>
     <row r="48">
@@ -11388,10 +11388,10 @@
         <v>9.02</v>
       </c>
       <c r="G48" t="n">
-        <v>3106519946</v>
+        <v>3149333408</v>
       </c>
       <c r="H48" t="n">
-        <v>1400</v>
+        <v>2000</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>1.993056529453528</v>
+        <v>2.020524452232354</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>543097892.6573427</v>
+        <v>550582763.6363636</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11564,7 +11564,7 @@
         <v>1.29</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.050000000000001</v>
+        <v>9.06</v>
       </c>
       <c r="BN48" t="n">
         <v>9.48</v>
@@ -11573,19 +11573,19 @@
         <v>7.21</v>
       </c>
       <c r="BP48" t="n">
-        <v>8.92</v>
+        <v>9</v>
       </c>
       <c r="BQ48" t="n">
         <v>6.97</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.050000000000001</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2689</v>
+        <v>2702</v>
       </c>
     </row>
     <row r="49">
@@ -11621,7 +11621,7 @@
         <v>996908218</v>
       </c>
       <c r="H49" t="n">
-        <v>6900</v>
+        <v>0</v>
       </c>
       <c r="I49" t="n">
         <v>11540870</v>
@@ -11815,7 +11815,7 @@
         <v>0.54</v>
       </c>
       <c r="BT49" t="n">
-        <v>143</v>
+        <v>373</v>
       </c>
     </row>
     <row r="50">
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>33.9</v>
+        <v>34.5</v>
       </c>
       <c r="G50" t="n">
-        <v>933292214</v>
+        <v>967124900</v>
       </c>
       <c r="H50" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9441996948109511</v>
+        <v>0.9784277868454088</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>318529765.8703071</v>
+        <v>330076757.6791809</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>74.75</v>
+        <v>76.06999999999999</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,19 +11994,19 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>147.43</v>
+        <v>143.12</v>
       </c>
       <c r="BD50" t="n">
-        <v>102.02</v>
+        <v>98.51000000000001</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-72.81999999999999</v>
+        <v>-73.29000000000001</v>
       </c>
       <c r="BG50" t="n">
-        <v>-9.94</v>
+        <v>-11.51</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
@@ -12015,7 +12015,7 @@
         <v>0</v>
       </c>
       <c r="BJ50" t="n">
-        <v>33.9</v>
+        <v>34.5</v>
       </c>
       <c r="BK50" t="n">
         <v>7.34</v>
@@ -12024,22 +12024,22 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>33.9</v>
+        <v>34.5</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
       </c>
       <c r="BO50" t="n">
-        <v>22.89</v>
+        <v>23.5</v>
       </c>
       <c r="BP50" t="n">
-        <v>33.9</v>
+        <v>34.5</v>
       </c>
       <c r="BQ50" t="n">
-        <v>4.46</v>
+        <v>4.54</v>
       </c>
       <c r="BR50" t="n">
-        <v>33.9</v>
+        <v>34.5</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.58</v>
+        <v>6.7</v>
       </c>
       <c r="G53" t="n">
-        <v>869986533</v>
+        <v>916911053</v>
       </c>
       <c r="H53" t="n">
-        <v>89500</v>
+        <v>51100</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.260062829764276</v>
+        <v>2.38196398505093</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>44319232.45033113</v>
+        <v>46709681.76260825</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-40.11</v>
+        <v>-41.18</v>
       </c>
       <c r="BD53" t="n">
-        <v>-51.1</v>
+        <v>-51.98</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.59</v>
+        <v>-95.67</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6.58</v>
+        <v>6.7</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.09</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.74</v>
+        <v>6.78</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,10 +12711,10 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>6.47</v>
+        <v>6.53</v>
       </c>
       <c r="BQ53" t="n">
-        <v>77.12</v>
+        <v>78.53</v>
       </c>
       <c r="BR53" t="n">
         <v>6.53</v>
@@ -12723,7 +12723,7 @@
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>42567</v>
+        <v>44010</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>10.02</v>
+        <v>10.18</v>
       </c>
       <c r="G54" t="n">
-        <v>2405012533</v>
+        <v>2374098231</v>
       </c>
       <c r="H54" t="n">
-        <v>344400</v>
+        <v>364200</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.349913285895204</v>
+        <v>1.332561348463959</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>329003082.4897401</v>
+        <v>324774039.8084816</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>15.95</v>
+        <v>16.2</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,19 +12902,19 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>49.78</v>
+        <v>47.42</v>
       </c>
       <c r="BD54" t="n">
-        <v>22.29</v>
+        <v>20.37</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-90.19</v>
+        <v>-90.34</v>
       </c>
       <c r="BG54" t="n">
-        <v>-34.97</v>
+        <v>-35.99</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
@@ -12923,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>10.02</v>
+        <v>10.18</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>10.05</v>
+        <v>10.18</v>
       </c>
       <c r="BN54" t="n">
         <v>11.75</v>
@@ -12941,19 +12941,19 @@
         <v>8.279999999999999</v>
       </c>
       <c r="BP54" t="n">
-        <v>9.74</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="BQ54" t="n">
-        <v>9.99</v>
+        <v>10.15</v>
       </c>
       <c r="BR54" t="n">
-        <v>9.880000000000001</v>
+        <v>10</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>276570</v>
+        <v>279180</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>51.95</v>
+        <v>51.03</v>
       </c>
       <c r="G55" t="n">
-        <v>6648812643</v>
+        <v>6579775784</v>
       </c>
       <c r="H55" t="n">
-        <v>1800</v>
+        <v>5300</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1.026384909777839</v>
+        <v>1.015727609880742</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>334447316.0462777</v>
+        <v>330974637.0221328</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>54.63</v>
+        <v>53.67</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>20.72</v>
+        <v>22.9</v>
       </c>
       <c r="BD55" t="n">
-        <v>-1.43</v>
+        <v>0.34</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-81.95</v>
+        <v>-81.62</v>
       </c>
       <c r="BG55" t="n">
-        <v>-69.05</v>
+        <v>-68.5</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>51.95</v>
+        <v>51.03</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>51.95</v>
+        <v>51.86</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>34.46</v>
       </c>
       <c r="BP55" t="n">
-        <v>51.31</v>
+        <v>51.03</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.39</v>
+        <v>7.26</v>
       </c>
       <c r="BR55" t="n">
-        <v>51.31</v>
+        <v>51.5</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>7116</v>
+        <v>6564</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>60.33</v>
+        <v>58.72</v>
       </c>
       <c r="G56" t="n">
-        <v>6648812643</v>
+        <v>6579775784</v>
       </c>
       <c r="H56" t="n">
-        <v>24500</v>
+        <v>23000</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.174384309904036</v>
+        <v>2.151806945933237</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>276572905.2828619</v>
+        <v>273701155.7404326</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>57.62</v>
+        <v>56.08</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>3.95</v>
+        <v>6.8</v>
       </c>
       <c r="BD56" t="n">
-        <v>-15.12</v>
+        <v>-12.8</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-84.45999999999999</v>
+        <v>-84.03</v>
       </c>
       <c r="BG56" t="n">
-        <v>-70.7</v>
+        <v>-69.90000000000001</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>60.33</v>
+        <v>58.72</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,28 +13392,28 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>62.59</v>
+        <v>61.25</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
       </c>
       <c r="BO56" t="n">
-        <v>45.75</v>
+        <v>46.08</v>
       </c>
       <c r="BP56" t="n">
-        <v>60.1</v>
+        <v>58.72</v>
       </c>
       <c r="BQ56" t="n">
-        <v>8.58</v>
+        <v>8.35</v>
       </c>
       <c r="BR56" t="n">
-        <v>61.5</v>
+        <v>61.25</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>33210</v>
+        <v>32888</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6.06</v>
+        <v>6.09</v>
       </c>
       <c r="G57" t="n">
-        <v>1407439834</v>
+        <v>1424195255</v>
       </c>
       <c r="H57" t="n">
-        <v>1683600</v>
+        <v>960500</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4212845444522087</v>
+        <v>0.4262998919879031</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>105268499.1772625</v>
+        <v>106521709.4240838</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>9.24</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>116.69</v>
+        <v>115.62</v>
       </c>
       <c r="BD57" t="n">
-        <v>76.93000000000001</v>
+        <v>76.05</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-81.39</v>
+        <v>-81.48999999999999</v>
       </c>
       <c r="BG57" t="n">
-        <v>3.36</v>
+        <v>2.86</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>6.06</v>
+        <v>6.09</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,28 +13622,28 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>6.06</v>
+        <v>6.11</v>
       </c>
       <c r="BN57" t="n">
-        <v>6.08</v>
+        <v>6.11</v>
       </c>
       <c r="BO57" t="n">
         <v>3.39</v>
       </c>
       <c r="BP57" t="n">
-        <v>5.75</v>
+        <v>5.96</v>
       </c>
       <c r="BQ57" t="n">
-        <v>5.85</v>
+        <v>5.88</v>
       </c>
       <c r="BR57" t="n">
-        <v>5.8</v>
+        <v>5.99</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1235809</v>
+        <v>1266570</v>
       </c>
     </row>
     <row r="58">
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>374.25</v>
+        <v>376.6</v>
       </c>
       <c r="G60" t="n">
-        <v>167937576</v>
+        <v>171258852</v>
       </c>
       <c r="H60" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.56149427809238</v>
+        <v>12.80992104751274</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-24624278.0058651</v>
+        <v>-25111268.62170088</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2151.94</v>
+        <v>2165.45</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,19 +14282,19 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>209.21</v>
+        <v>207.28</v>
       </c>
       <c r="BD60" t="n">
-        <v>152.47</v>
+        <v>150.89</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-38.25</v>
+        <v>-38.64</v>
       </c>
       <c r="BG60" t="n">
-        <v>94.52</v>
+        <v>93.3</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>374.25</v>
+        <v>376.6</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14312,7 +14312,7 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>376.99</v>
+        <v>377</v>
       </c>
       <c r="BN60" t="n">
         <v>405</v>
@@ -14321,19 +14321,19 @@
         <v>306.27</v>
       </c>
       <c r="BP60" t="n">
-        <v>373</v>
+        <v>371.25</v>
       </c>
       <c r="BQ60" t="n">
-        <v>2.86</v>
+        <v>2.88</v>
       </c>
       <c r="BR60" t="n">
-        <v>376.99</v>
+        <v>377</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
       </c>
       <c r="BT60" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="61">
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>26.21</v>
+        <v>26.27</v>
       </c>
       <c r="G61" t="n">
-        <v>2226361194</v>
+        <v>2248932444</v>
       </c>
       <c r="H61" t="n">
-        <v>711500</v>
+        <v>369800</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.180715780090424</v>
+        <v>1.192686088916857</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>174753625.9026687</v>
+        <v>176525309.5761381</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>33.02</v>
+        <v>33.1</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-17.96</v>
+        <v>-18.14</v>
       </c>
       <c r="BD61" t="n">
-        <v>-33.01</v>
+        <v>-33.16</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-90.37</v>
+        <v>-90.40000000000001</v>
       </c>
       <c r="BG61" t="n">
-        <v>-55.15</v>
+        <v>-55.25</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>26.21</v>
+        <v>26.27</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>26.41</v>
+        <v>26.54</v>
       </c>
       <c r="BN61" t="n">
         <v>28.25</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>25.29</v>
+        <v>25.91</v>
       </c>
       <c r="BQ61" t="n">
-        <v>14.08</v>
+        <v>14.11</v>
       </c>
       <c r="BR61" t="n">
-        <v>25.56</v>
+        <v>26.05</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>466568</v>
+        <v>480755</v>
       </c>
     </row>
     <row r="62">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.35</v>
+        <v>1.34</v>
       </c>
       <c r="G63" t="n">
-        <v>349063566</v>
+        <v>349083006</v>
       </c>
       <c r="H63" t="n">
-        <v>19700</v>
+        <v>200</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.4293301723642919</v>
+        <v>0.429354082561069</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>198331571.5909091</v>
+        <v>198342617.0454545</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-78.58</v>
+        <v>-78.42</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.35</v>
+        <v>1.34</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.35</v>
+        <v>1.34</v>
       </c>
       <c r="BN63" t="n">
         <v>1.54</v>
@@ -15011,19 +15011,19 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.35</v>
+        <v>1.34</v>
       </c>
       <c r="BQ63" t="n">
-        <v>5.17</v>
+        <v>5.13</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.35</v>
+        <v>1.34</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>14493</v>
+        <v>15137</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>60.45</v>
+        <v>60.82</v>
       </c>
       <c r="G64" t="n">
-        <v>234216490006</v>
+        <v>234645444242</v>
       </c>
       <c r="H64" t="n">
-        <v>11044700</v>
+        <v>7839100</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>67153304617.71185</v>
+        <v>67276292091.72118</v>
       </c>
       <c r="AL64" t="n">
-        <v>18722341327.41806</v>
+        <v>18756630235.17186</v>
       </c>
       <c r="AM64" t="n">
-        <v>20856321460.90828</v>
+        <v>20894518632.41318</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>24.18</v>
+        <v>24.33</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,19 +15202,19 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-21.03</v>
+        <v>-21.51</v>
       </c>
       <c r="BD64" t="n">
-        <v>-35.52</v>
+        <v>-35.91</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-88.93000000000001</v>
+        <v>-88.98999999999999</v>
       </c>
       <c r="BG64" t="n">
-        <v>-82.8</v>
+        <v>-82.90000000000001</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
@@ -15223,7 +15223,7 @@
         <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>60.45</v>
+        <v>60.82</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>61.1</v>
+        <v>61.07</v>
       </c>
       <c r="BN64" t="n">
         <v>64.72</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>58.39</v>
+        <v>60.33</v>
       </c>
       <c r="BQ64" t="n">
-        <v>38.5</v>
+        <v>38.74</v>
       </c>
       <c r="BR64" t="n">
-        <v>58.71</v>
+        <v>61.02</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>12088805</v>
+        <v>12253994</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>23.8</v>
+        <v>23.69</v>
       </c>
       <c r="G65" t="n">
-        <v>234216490006</v>
+        <v>234645444242</v>
       </c>
       <c r="H65" t="n">
-        <v>6000</v>
+        <v>7900</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.662404484384867</v>
+        <v>5.672774857493353</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>17544306367.49064</v>
+        <v>17576437770.93633</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>8.01</v>
+        <v>7.98</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-33.15</v>
+        <v>-32.84</v>
       </c>
       <c r="BD65" t="n">
-        <v>-45.42</v>
+        <v>-45.17</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-90.62</v>
+        <v>-90.58</v>
       </c>
       <c r="BG65" t="n">
-        <v>-85.44</v>
+        <v>-85.37</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>23.8</v>
+        <v>23.69</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>23.8</v>
+        <v>23.9</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>23.43</v>
+        <v>23.44</v>
       </c>
       <c r="BQ65" t="n">
-        <v>15.16</v>
+        <v>15.09</v>
       </c>
       <c r="BR65" t="n">
-        <v>23.8</v>
+        <v>23.89</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>11985</v>
+        <v>11943</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>20.01</v>
+        <v>19.76</v>
       </c>
       <c r="G66" t="n">
-        <v>234216490006</v>
+        <v>234645444242</v>
       </c>
       <c r="H66" t="n">
-        <v>4500</v>
+        <v>2000</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>13.90440585811686</v>
+        <v>13.92987098993464</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>21005963229.23767</v>
+        <v>21044434461.16592</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>8.039999999999999</v>
+        <v>7.94</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-20.49</v>
+        <v>-19.49</v>
       </c>
       <c r="BD66" t="n">
-        <v>-35.08</v>
+        <v>-34.26</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-88.84999999999999</v>
+        <v>-88.70999999999999</v>
       </c>
       <c r="BG66" t="n">
-        <v>-82.68000000000001</v>
+        <v>-82.45999999999999</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>20.01</v>
+        <v>19.76</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>20.59</v>
+        <v>20.2</v>
       </c>
       <c r="BN66" t="n">
         <v>21.16</v>
@@ -15701,19 +15701,19 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>19.97</v>
+        <v>19.55</v>
       </c>
       <c r="BQ66" t="n">
-        <v>12.74</v>
+        <v>12.59</v>
       </c>
       <c r="BR66" t="n">
-        <v>20.05</v>
+        <v>19.57</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>6961</v>
+        <v>7070</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>19.21</v>
+        <v>19.23</v>
       </c>
       <c r="G68" t="n">
-        <v>8255366240</v>
+        <v>8419842135</v>
       </c>
       <c r="H68" t="n">
-        <v>25700</v>
+        <v>18400</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>572494191.4008322</v>
+        <v>583900286.7545077</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>35.54</v>
+        <v>35.58</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,10 +16122,10 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>36.4</v>
+        <v>36.26</v>
       </c>
       <c r="BD68" t="n">
-        <v>11.37</v>
+        <v>11.26</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
@@ -16134,7 +16134,7 @@
         <v>-93.55</v>
       </c>
       <c r="BG68" t="n">
-        <v>229.25</v>
+        <v>228.91</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>19.21</v>
+        <v>19.23</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>19.39</v>
+        <v>19.33</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,19 +16161,19 @@
         <v>15.07</v>
       </c>
       <c r="BP68" t="n">
-        <v>19</v>
+        <v>19.1</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.92</v>
+        <v>12.93</v>
       </c>
       <c r="BR68" t="n">
-        <v>19.39</v>
+        <v>19.33</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>32260</v>
+        <v>32337</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>22.38</v>
+        <v>22.54</v>
       </c>
       <c r="G69" t="n">
-        <v>8255366240</v>
+        <v>8419842135</v>
       </c>
       <c r="H69" t="n">
-        <v>2726600</v>
+        <v>1582700</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>491390847.6190476</v>
+        <v>501181079.4642857</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>39.13</v>
+        <v>39.41</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>17.08</v>
+        <v>16.25</v>
       </c>
       <c r="BD69" t="n">
-        <v>-4.4</v>
+        <v>-5.08</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-94.45999999999999</v>
+        <v>-94.5</v>
       </c>
       <c r="BG69" t="n">
-        <v>210.93</v>
+        <v>208.73</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>22.38</v>
+        <v>22.54</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,28 +16382,28 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>22.59</v>
+        <v>22.61</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
       </c>
       <c r="BO69" t="n">
-        <v>16.6</v>
+        <v>16.71</v>
       </c>
       <c r="BP69" t="n">
-        <v>22.14</v>
+        <v>22.26</v>
       </c>
       <c r="BQ69" t="n">
-        <v>15.05</v>
+        <v>15.16</v>
       </c>
       <c r="BR69" t="n">
-        <v>22.24</v>
+        <v>22.47</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>1859817</v>
+        <v>1918823</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>18.81</v>
+        <v>18.29</v>
       </c>
       <c r="G70" t="n">
-        <v>8819719075</v>
+        <v>8496751613</v>
       </c>
       <c r="H70" t="n">
-        <v>3735000</v>
+        <v>2814000</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6961245075529993</v>
+        <v>0.6706332687132415</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2910798374.587459</v>
+        <v>2804208453.135314</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.16</v>
+        <v>2.1</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,19 +16582,19 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-55.08</v>
+        <v>-53.8</v>
       </c>
       <c r="BD70" t="n">
-        <v>-63.32</v>
+        <v>-62.28</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
       </c>
       <c r="BF70" t="n">
-        <v>-99.36</v>
+        <v>-99.34</v>
       </c>
       <c r="BG70" t="n">
-        <v>-94.31</v>
+        <v>-94.15000000000001</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>18.81</v>
+        <v>18.29</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>19.04</v>
+        <v>18.64</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>18.53</v>
+        <v>18.29</v>
       </c>
       <c r="BQ70" t="n">
-        <v>188.65</v>
+        <v>183.43</v>
       </c>
       <c r="BR70" t="n">
-        <v>18.53</v>
+        <v>18.5</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>6219960</v>
+        <v>6063490</v>
       </c>
     </row>
     <row r="71">

</xml_diff>